<commit_message>
Atualização automática 2026-03-02 09:52:06.406174
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46080.70622685185</v>
+        <v>46083.37527777778</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46080.73770833333</v>
+        <v>46083.38605324074</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46080.68978009259</v>
+        <v>46083.40001157407</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46080.72899305556</v>
+        <v>46083.37709490741</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
         <v>1</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>46080.72792824074</v>
+        <v>46080.88524305556</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46080.7062037037</v>
+        <v>46083.36973379629</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
         <v>1</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>46080.70592592593</v>
+        <v>46080.93313657407</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1382,7 +1382,7 @@
         <v>2</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>46080.7094212963</v>
+        <v>46080.86283564815</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46080.70561342593</v>
+        <v>46083.39371527778</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1510,7 +1510,7 @@
         <v>2</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>46080.73059027778</v>
+        <v>46083.38149305555</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46080.65475694444</v>
+        <v>46083.40207175926</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46080.71113425926</v>
+        <v>46083.39827546296</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1763,7 +1763,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46080.70501157407</v>
+        <v>46083.38108796296</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1905,11 +1905,6 @@
           <t>AUDITORIO</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>10.69.3.146</t>
-        </is>
-      </c>
       <c r="D23" t="n">
         <v>2018</v>
       </c>
@@ -1950,7 +1945,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46080.61047453704</v>
+        <v>46083.22623842592</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2009,7 +2004,7 @@
         <v>1</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>46080.50407407407</v>
+        <v>46083.16126157407</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2065,7 +2060,7 @@
         </is>
       </c>
       <c r="N25" s="3" t="n">
-        <v>46080.39040509259</v>
+        <v>46083.16996527778</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2183,7 +2178,7 @@
         <v>1</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46080.50165509259</v>
+        <v>46083.1434837963</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2244,7 +2239,7 @@
         </is>
       </c>
       <c r="N28" s="3" t="n">
-        <v>46078.73241898148</v>
+        <v>46083.38260416667</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -6570,7 +6565,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46080.67180555555</v>
+        <v>46083.38186342592</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6639,7 +6634,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46080.71556712963</v>
+        <v>46080.79733796296</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6658,6 +6653,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>10.69.3.93</t>
+        </is>
+      </c>
       <c r="D97" t="n">
         <v>2025</v>
       </c>
@@ -6703,7 +6703,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46080.71765046296</v>
+        <v>46083.40333333334</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6767,7 +6767,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46080.68881944445</v>
+        <v>46083.36736111111</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6836,7 +6836,7 @@
         <v>1</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46080.7337962963</v>
+        <v>46081.58810185185</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
         <v>2</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46080.70234953704</v>
+        <v>46083.38962962963</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6974,7 +6974,7 @@
         <v>1</v>
       </c>
       <c r="N101" s="3" t="n">
-        <v>46080.7233449074</v>
+        <v>46083.40013888889</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -7112,7 +7112,7 @@
         <v>2</v>
       </c>
       <c r="N103" s="3" t="n">
-        <v>46080.70444444445</v>
+        <v>46083.39050925926</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -7369,7 +7369,7 @@
         <v>1</v>
       </c>
       <c r="N107" s="3" t="n">
-        <v>46079.65697916667</v>
+        <v>46083.37668981482</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -7507,7 +7507,7 @@
         <v>1</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46080.72489583334</v>
+        <v>46083.39693287037</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7576,7 +7576,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46080.72483796296</v>
+        <v>46083.39693287037</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7645,7 +7645,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46080.71645833334</v>
+        <v>46083.37052083333</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7714,7 +7714,7 @@
         <v>2</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46080.70658564815</v>
+        <v>46083.39858796296</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7783,7 +7783,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46080.72392361111</v>
+        <v>46083.39363425926</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7852,7 +7852,7 @@
         <v>1</v>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46080.72119212963</v>
+        <v>46083.37153935185</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7918,7 +7918,7 @@
         </is>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46080.68064814815</v>
+        <v>46083.37663194445</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7987,7 +7987,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46080.68903935186</v>
+        <v>46083.38702546297</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8006,6 +8006,11 @@
           <t>DP</t>
         </is>
       </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>10.69.3.23</t>
+        </is>
+      </c>
       <c r="D117" t="n">
         <v>2025</v>
       </c>
@@ -8051,7 +8056,7 @@
         <v>1</v>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46080.70883101852</v>
+        <v>46083.40143518519</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8117,7 +8122,7 @@
         </is>
       </c>
       <c r="N118" s="3" t="n">
-        <v>46080.69048611111</v>
+        <v>46083.37429398148</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -8255,7 +8260,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46080.71517361111</v>
+        <v>46083.39744212963</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8324,7 +8329,7 @@
         <v>1</v>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46080.71342592593</v>
+        <v>46081.56248842592</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8390,7 +8395,7 @@
         </is>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46080.715</v>
+        <v>46083.39796296296</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8459,7 +8464,7 @@
         <v>2</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46080.72591435185</v>
+        <v>46083.27993055555</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8528,7 +8533,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46080.72495370371</v>
+        <v>46083.40447916667</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8597,7 +8602,7 @@
         <v>1</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46080.73165509259</v>
+        <v>46083.3908912037</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8666,7 +8671,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46080.70289351852</v>
+        <v>46081.5318287037</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8735,7 +8740,7 @@
         <v>2</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46080.73563657407</v>
+        <v>46083.39143518519</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8804,7 +8809,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46080.6821412037</v>
+        <v>46083.40206018519</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8873,7 +8878,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46080.70576388889</v>
+        <v>46081.63077546296</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -8905,7 +8910,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Microsoft Windows 11 Pro</t>
+          <t>Windows</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -8942,7 +8947,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46080.65162037037</v>
+        <v>46083.37271990741</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9006,7 +9011,7 @@
         <v>1</v>
       </c>
       <c r="N131" s="3" t="n">
-        <v>46080.66407407408</v>
+        <v>46083.38194444445</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -9203,7 +9208,7 @@
         <v>1</v>
       </c>
       <c r="N134" s="3" t="n">
-        <v>46080.5740625</v>
+        <v>46081.60379629629</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -9267,7 +9272,7 @@
         <v>1</v>
       </c>
       <c r="N135" s="3" t="n">
-        <v>46080.73708333333</v>
+        <v>46081.60099537037</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -9458,7 +9463,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46080.7143287037</v>
+        <v>46083.37601851852</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9522,7 +9527,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46080.70793981481</v>
+        <v>46083.37900462963</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9586,7 +9591,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46080.73418981482</v>
+        <v>46081.5971412037</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9650,7 +9655,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46080.72565972222</v>
+        <v>46083.37694444445</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9714,7 +9719,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46080.73232638889</v>
+        <v>46083.39814814815</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9778,7 +9783,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46079.79195601852</v>
+        <v>46083.38372685185</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9842,7 +9847,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46080.72837962963</v>
+        <v>46081.58719907407</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9906,7 +9911,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46080.73259259259</v>
+        <v>46083.38153935185</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9970,7 +9975,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46080.70055555556</v>
+        <v>46083.37847222222</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10034,7 +10039,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46080.72015046296</v>
+        <v>46081.59994212963</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10098,7 +10103,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46080.72857638889</v>
+        <v>46083.37789351852</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10162,7 +10167,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46080.70193287037</v>
+        <v>46083.38362268519</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10226,7 +10231,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46080.73216435185</v>
+        <v>46081.84983796296</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10290,7 +10295,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46080.73047453703</v>
+        <v>46083.37761574074</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10354,7 +10359,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46080.73289351852</v>
+        <v>46083.38886574074</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10373,6 +10378,11 @@
           <t>OPERACAO 7.1</t>
         </is>
       </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>10.69.5.21</t>
+        </is>
+      </c>
       <c r="D153" t="n">
         <v>2018</v>
       </c>
@@ -10413,7 +10423,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46079.87296296296</v>
+        <v>46083.38559027778</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10477,7 +10487,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46080.73444444445</v>
+        <v>46083.37755787037</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10541,7 +10551,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46080.73128472222</v>
+        <v>46083.38436342592</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10605,7 +10615,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46080.69834490741</v>
+        <v>46080.81335648148</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10669,7 +10679,7 @@
         <v>1</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>46080.5724537037</v>
+        <v>46083.38212962963</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -10733,7 +10743,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46080.73016203703</v>
+        <v>46083.36474537037</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10797,7 +10807,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46080.70040509259</v>
+        <v>46083.37556712963</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10861,7 +10871,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46080.70798611111</v>
+        <v>46083.37605324074</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10925,7 +10935,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46080.73342592592</v>
+        <v>46083.37467592592</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -10989,7 +10999,7 @@
         <v>1</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46080.70929398148</v>
+        <v>46083.37278935185</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11117,7 +11127,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46080.71997685185</v>
+        <v>46083.3955324074</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11181,7 +11191,7 @@
         <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46080.56491898148</v>
+        <v>46083.40359953704</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11245,7 +11255,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46080.61219907407</v>
+        <v>46083.37292824074</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11309,7 +11319,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46080.59599537037</v>
+        <v>46083.40298611111</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11373,7 +11383,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46080.55756944444</v>
+        <v>46083.39625</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11437,7 +11447,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46080.70202546296</v>
+        <v>46083.38010416667</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11501,7 +11511,7 @@
         <v>2</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46080.72527777778</v>
+        <v>46083.38280092592</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11565,7 +11575,7 @@
         <v>1</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46080.56064814814</v>
+        <v>46083.40086805556</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11629,7 +11639,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46080.64740740741</v>
+        <v>46081.29152777778</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11693,7 +11703,7 @@
         <v>1</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46080.7253125</v>
+        <v>46083.37211805556</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11757,7 +11767,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46080.57200231482</v>
+        <v>46083.37331018518</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11821,7 +11831,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46080.72491898148</v>
+        <v>46083.38180555555</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11885,7 +11895,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46080.70550925926</v>
+        <v>46080.78006944444</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11949,7 +11959,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46080.69650462963</v>
+        <v>46081.52849537037</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12013,7 +12023,7 @@
         <v>2</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46080.70347222222</v>
+        <v>46083.40362268518</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12077,7 +12087,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46080.70797453704</v>
+        <v>46083.37747685185</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12141,7 +12151,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46080.73609953704</v>
+        <v>46083.37731481482</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12205,7 +12215,7 @@
         <v>1</v>
       </c>
       <c r="N181" s="3" t="n">
-        <v>46079.86542824074</v>
+        <v>46083.39814814815</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
@@ -12333,7 +12343,7 @@
         <v>1</v>
       </c>
       <c r="N183" s="3" t="n">
-        <v>46080.69935185185</v>
+        <v>46081.60625</v>
       </c>
       <c r="O183" t="inlineStr">
         <is>
@@ -12402,7 +12412,7 @@
         <v>2</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46080.70799768518</v>
+        <v>46083.37998842593</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12466,7 +12476,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46079.82648148148</v>
+        <v>46081.37590277778</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12530,7 +12540,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46080.60023148148</v>
+        <v>46081.37732638889</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12594,7 +12604,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46080.7100462963</v>
+        <v>46083.39762731481</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12658,7 +12668,7 @@
         <v>1</v>
       </c>
       <c r="N188" s="3" t="n">
-        <v>46080.48842592593</v>
+        <v>46083.39923611111</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
@@ -12744,6 +12754,11 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>10.69.5.59</t>
+        </is>
+      </c>
       <c r="D190" t="n">
         <v>2015</v>
       </c>
@@ -12781,7 +12796,7 @@
         </is>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46080.71196759259</v>
+        <v>46083.3934375</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12845,7 +12860,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46080.7084837963</v>
+        <v>46083.37872685185</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12909,7 +12924,7 @@
         <v>1</v>
       </c>
       <c r="N192" s="3" t="n">
-        <v>46080.71560185185</v>
+        <v>46083.40439814814</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
@@ -13034,7 +13049,7 @@
         <v>2</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46080.55902777778</v>
+        <v>46083.40412037037</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13098,7 +13113,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46080.70313657408</v>
+        <v>46083.37106481481</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13162,7 +13177,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46080.70790509259</v>
+        <v>46083.39400462963</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13226,7 +13241,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46080.70378472222</v>
+        <v>46083.38978009259</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13290,7 +13305,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46080.73332175926</v>
+        <v>46083.39280092593</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13354,7 +13369,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46080.72146990741</v>
+        <v>46083.39635416667</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13418,7 +13433,7 @@
         <v>1</v>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46080.73277777778</v>
+        <v>46083.40439814814</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13479,7 +13494,7 @@
         </is>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46080.71288194445</v>
+        <v>46081.60105324074</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13543,7 +13558,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46080.71694444444</v>
+        <v>46083.37413194445</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13607,7 +13622,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46080.73456018518</v>
+        <v>46083.39777777778</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13671,7 +13686,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46080.73109953704</v>
+        <v>46081.58994212963</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13735,7 +13750,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46080.72067129629</v>
+        <v>46083.37643518519</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13799,7 +13814,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46080.73501157408</v>
+        <v>46083.39299768519</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13863,7 +13878,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46080.73173611111</v>
+        <v>46083.40020833333</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13927,7 +13942,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46080.57481481481</v>
+        <v>46083.39748842592</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -13991,7 +14006,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46080.70480324074</v>
+        <v>46083.40002314815</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14055,7 +14070,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46080.72105324074</v>
+        <v>46083.40479166667</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14119,7 +14134,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46080.70155092593</v>
+        <v>46083.38034722222</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14183,7 +14198,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46080.71762731481</v>
+        <v>46083.38030092593</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14247,7 +14262,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46080.7065625</v>
+        <v>46083.37788194444</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14311,7 +14326,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46080.71466435185</v>
+        <v>46083.37681712963</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14375,7 +14390,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46080.71866898148</v>
+        <v>46083.38506944444</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14439,7 +14454,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46080.71372685185</v>
+        <v>46083.40157407407</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14458,11 +14473,6 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
-      <c r="C217" t="inlineStr">
-        <is>
-          <t>10.69.5.85</t>
-        </is>
-      </c>
       <c r="D217" t="n">
         <v>2017</v>
       </c>
@@ -14503,7 +14513,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46080.7375</v>
+        <v>46083.38002314815</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14567,7 +14577,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46080.72359953704</v>
+        <v>46083.38348379629</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14631,7 +14641,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46080.73417824074</v>
+        <v>46083.38543981482</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14700,7 +14710,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46080.71976851852</v>
+        <v>46083.38469907407</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14764,7 +14774,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46080.70052083334</v>
+        <v>46083.37788194444</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14828,7 +14838,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46080.73560185185</v>
+        <v>46083.38506944444</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14892,7 +14902,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46080.7293287037</v>
+        <v>46083.40039351852</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14956,7 +14966,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46080.71967592592</v>
+        <v>46081.46488425926</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15020,7 +15030,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46079.82745370371</v>
+        <v>46081.37142361111</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15084,7 +15094,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46080.71939814815</v>
+        <v>46083.40136574074</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15148,7 +15158,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46080.71240740741</v>
+        <v>46081.5990625</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15212,7 +15222,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46080.73627314815</v>
+        <v>46083.40072916666</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15276,7 +15286,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46080.55005787037</v>
+        <v>46083.38762731481</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15340,7 +15350,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46080.70516203704</v>
+        <v>46083.4027199074</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15404,7 +15414,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46080.73565972222</v>
+        <v>46083.39063657408</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15468,7 +15478,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46080.73290509259</v>
+        <v>46083.36997685185</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15532,7 +15542,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46080.72672453704</v>
+        <v>46083.37453703704</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15596,7 +15606,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46080.70543981482</v>
+        <v>46083.40439814814</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15660,7 +15670,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46080.70927083334</v>
+        <v>46083.38736111111</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15724,7 +15734,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46080.70577546296</v>
+        <v>46083.40193287037</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15852,7 +15862,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46080.70150462963</v>
+        <v>46083.38327546296</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15916,7 +15926,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46080.72047453704</v>
+        <v>46083.38950231481</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -15980,7 +15990,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46080.7078125</v>
+        <v>46083.40040509259</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16044,7 +16054,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46080.70758101852</v>
+        <v>46081.56407407407</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16108,7 +16118,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46080.73600694445</v>
+        <v>46083.3785300926</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16172,7 +16182,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46080.67122685185</v>
+        <v>46083.39803240741</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16231,7 +16241,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46080.23087962963</v>
+        <v>46083.12707175926</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16295,7 +16305,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46080.70635416666</v>
+        <v>46083.40189814815</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16359,7 +16369,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46080.73402777778</v>
+        <v>46083.39136574074</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16423,7 +16433,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46080.709375</v>
+        <v>46081.60538194444</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16487,7 +16497,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46080.70929398148</v>
+        <v>46081.59859953704</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16551,7 +16561,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46079.75825231482</v>
+        <v>46083.39855324074</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16570,11 +16580,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C250" t="inlineStr">
-        <is>
-          <t>10.69.5.118</t>
-        </is>
-      </c>
       <c r="D250" t="n">
         <v>2017</v>
       </c>
@@ -16615,7 +16620,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46080.73658564815</v>
+        <v>46083.39784722222</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16679,7 +16684,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46080.71563657407</v>
+        <v>46083.39895833333</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16743,7 +16748,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46080.7049537037</v>
+        <v>46081.59356481482</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16807,7 +16812,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46080.6999074074</v>
+        <v>46083.38966435185</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16865,7 +16870,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46080.70893518518</v>
+        <v>46083.3983912037</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16929,7 +16934,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46080.71915509259</v>
+        <v>46083.39869212963</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -16993,7 +16998,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46080.71219907407</v>
+        <v>46083.38950231481</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17057,7 +17062,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46080.71725694444</v>
+        <v>46083.40335648148</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17121,7 +17126,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46080.71673611111</v>
+        <v>46083.38244212963</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17185,7 +17190,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46080.70047453704</v>
+        <v>46081.38613425926</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17249,7 +17254,7 @@
         <v>1</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46080.60126157408</v>
+        <v>46083.36489583334</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17313,7 +17318,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46080.71167824074</v>
+        <v>46083.40145833333</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17377,7 +17382,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46080.73739583333</v>
+        <v>46083.39061342592</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17441,7 +17446,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46080.72732638889</v>
+        <v>46083.38122685185</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17505,7 +17510,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46080.70329861111</v>
+        <v>46083.4018287037</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17569,7 +17574,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46080.7137037037</v>
+        <v>46083.38542824074</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17633,7 +17638,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46080.7033912037</v>
+        <v>46083.40096064815</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17697,7 +17702,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46080.73524305555</v>
+        <v>46083.39949074074</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17761,7 +17766,7 @@
         <v>1</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46080.71549768518</v>
+        <v>46081.60807870371</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17825,7 +17830,7 @@
         <v>1</v>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46080.72547453704</v>
+        <v>46081.61785879629</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17886,7 +17891,7 @@
         </is>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46080.70121527778</v>
+        <v>46083.37460648148</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -17950,7 +17955,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46080.08175925926</v>
+        <v>46081.29568287037</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -18014,7 +18019,7 @@
         <v>1</v>
       </c>
       <c r="N272" s="3" t="n">
-        <v>46080.65876157407</v>
+        <v>46083.38991898148</v>
       </c>
       <c r="O272" t="inlineStr">
         <is>
@@ -18078,7 +18083,7 @@
         <v>2</v>
       </c>
       <c r="N273" s="3" t="n">
-        <v>46080.6541087963</v>
+        <v>46081.58387731481</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -18334,7 +18339,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46080.70896990741</v>
+        <v>46080.86256944444</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18398,7 +18403,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46080.54747685185</v>
+        <v>46083.40425925926</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18462,7 +18467,7 @@
         <v>1</v>
       </c>
       <c r="N279" s="3" t="n">
-        <v>46080.53621527777</v>
+        <v>46083.40175925926</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -18526,7 +18531,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46080.56951388889</v>
+        <v>46083.38608796296</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18590,7 +18595,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46080.56284722222</v>
+        <v>46083.40166666666</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18609,6 +18614,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>10.69.5.151</t>
+        </is>
+      </c>
       <c r="D282" t="n">
         <v>2017</v>
       </c>
@@ -18649,7 +18659,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46080.70571759259</v>
+        <v>46083.39819444445</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18713,7 +18723,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46080.56560185185</v>
+        <v>46083.39061342592</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18777,7 +18787,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46080.70614583333</v>
+        <v>46083.39412037037</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18841,7 +18851,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46080.73055555556</v>
+        <v>46083.37212962963</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18860,6 +18870,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>10.69.5.155</t>
+        </is>
+      </c>
       <c r="D286" t="n">
         <v>2019</v>
       </c>
@@ -18900,7 +18915,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46080.59967592593</v>
+        <v>46083.35678240741</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18964,7 +18979,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46080.57688657408</v>
+        <v>46083.37887731481</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19028,7 +19043,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46080.54546296296</v>
+        <v>46083.39965277778</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19092,7 +19107,7 @@
         <v>1</v>
       </c>
       <c r="N289" s="3" t="n">
-        <v>46080.57341435185</v>
+        <v>46083.39951388889</v>
       </c>
       <c r="O289" t="inlineStr">
         <is>
@@ -19886,7 +19901,7 @@
         <v>1</v>
       </c>
       <c r="N302" s="3" t="n">
-        <v>46080.73355324074</v>
+        <v>46083.38498842593</v>
       </c>
       <c r="O302" t="inlineStr">
         <is>
@@ -21002,7 +21017,7 @@
         </is>
       </c>
       <c r="N320" s="3" t="n">
-        <v>46080.72577546296</v>
+        <v>46083.40133101852</v>
       </c>
       <c r="O320" t="inlineStr">
         <is>
@@ -21727,7 +21742,7 @@
         <v>1</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46080.71975694445</v>
+        <v>46083.38795138889</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21791,7 +21806,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46080.71267361111</v>
+        <v>46083.38449074074</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21855,7 +21870,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46080.71724537037</v>
+        <v>46083.38957175926</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21919,7 +21934,7 @@
         <v>2</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46080.70806712963</v>
+        <v>46083.39796296296</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21983,7 +21998,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46080.70563657407</v>
+        <v>46083.3806712963</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22047,7 +22062,7 @@
         <v>1</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46080.71649305556</v>
+        <v>46083.36667824074</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22111,7 +22126,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46080.71361111111</v>
+        <v>46083.40239583333</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22175,7 +22190,7 @@
         <v>2</v>
       </c>
       <c r="N339" s="3" t="n">
-        <v>46080.73273148148</v>
+        <v>46083.38565972223</v>
       </c>
       <c r="O339" t="inlineStr">
         <is>
@@ -22239,7 +22254,7 @@
         <v>1</v>
       </c>
       <c r="N340" s="3" t="n">
-        <v>46077.57763888889</v>
+        <v>46081.49881944444</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -22303,7 +22318,7 @@
         <v>2</v>
       </c>
       <c r="N341" s="3" t="n">
-        <v>46080.54791666667</v>
+        <v>46083.38724537037</v>
       </c>
       <c r="O341" t="inlineStr">
         <is>
@@ -22367,7 +22382,7 @@
         <v>2</v>
       </c>
       <c r="N342" s="3" t="n">
-        <v>46080.58256944444</v>
+        <v>46083.37887731481</v>
       </c>
       <c r="O342" t="inlineStr">
         <is>
@@ -22684,7 +22699,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46080.63840277777</v>
+        <v>46081.5865162037</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22748,7 +22763,7 @@
         <v>1</v>
       </c>
       <c r="N348" s="3" t="n">
-        <v>46080.70405092592</v>
+        <v>46080.7421875</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -22831,11 +22846,6 @@
           <t>OPERACAO 9.1</t>
         </is>
       </c>
-      <c r="C350" t="inlineStr">
-        <is>
-          <t>10.69.5.244</t>
-        </is>
-      </c>
       <c r="D350" t="n">
         <v>2014</v>
       </c>
@@ -23190,7 +23200,7 @@
         <v>1</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46080.70574074074</v>
+        <v>46080.74091435185</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23505,7 +23515,7 @@
         <v>2</v>
       </c>
       <c r="N360" s="3" t="n">
-        <v>46080.70782407407</v>
+        <v>46080.8618287037</v>
       </c>
       <c r="O360" t="inlineStr">
         <is>
@@ -23818,7 +23828,7 @@
         <v>1</v>
       </c>
       <c r="N365" s="3" t="n">
-        <v>46080.68246527778</v>
+        <v>46083.38070601852</v>
       </c>
       <c r="O365" t="inlineStr">
         <is>
@@ -23884,7 +23894,7 @@
         </is>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46080.72945601852</v>
+        <v>46083.38340277778</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
@@ -24010,7 +24020,7 @@
         </is>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46080.73319444444</v>
+        <v>46083.39820601852</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24029,11 +24039,6 @@
           <t>RH</t>
         </is>
       </c>
-      <c r="C369" t="inlineStr">
-        <is>
-          <t>10.69.3.13</t>
-        </is>
-      </c>
       <c r="D369" t="n">
         <v>2025</v>
       </c>
@@ -24076,7 +24081,7 @@
         </is>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46080.72767361111</v>
+        <v>46083.39616898148</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24145,7 +24150,7 @@
         <v>1</v>
       </c>
       <c r="N370" s="3" t="n">
-        <v>46079.78256944445</v>
+        <v>46083.36677083333</v>
       </c>
       <c r="O370" t="inlineStr">
         <is>
@@ -24352,7 +24357,7 @@
         <v>1</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46080.48386574074</v>
+        <v>46083.37754629629</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24421,7 +24426,7 @@
         <v>1</v>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46080.70642361111</v>
+        <v>46083.38230324074</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24487,7 +24492,7 @@
         </is>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46080.72482638889</v>
+        <v>46083.40090277778</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24506,11 +24511,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C376" t="inlineStr">
-        <is>
-          <t>10.69.3.72</t>
-        </is>
-      </c>
       <c r="D376" t="n">
         <v>2025</v>
       </c>
@@ -24556,7 +24556,7 @@
         <v>1</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46080.72820601852</v>
+        <v>46083.3753125</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -24625,7 +24625,7 @@
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46080.71266203704</v>
+        <v>46083.39449074074</v>
       </c>
       <c r="O377" t="inlineStr">
         <is>
@@ -24694,7 +24694,7 @@
         <v>2</v>
       </c>
       <c r="N378" s="3" t="n">
-        <v>46080.70809027777</v>
+        <v>46083.37761574074</v>
       </c>
       <c r="O378" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-02 11:52:05.590652
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46083.37527777778</v>
+        <v>46083.45109953704</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46083.38605324074</v>
+        <v>46083.46630787037</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46083.40001157407</v>
+        <v>46083.47232638889</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46083.37709490741</v>
+        <v>46083.45248842592</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46083.36973379629</v>
+        <v>46083.48675925926</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
         <v>1</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>46080.93313657407</v>
+        <v>46083.48105324074</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1382,7 +1382,7 @@
         <v>2</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>46080.86283564815</v>
+        <v>46083.47202546296</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46083.39371527778</v>
+        <v>46083.46743055555</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1510,7 +1510,7 @@
         <v>2</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>46083.38149305555</v>
+        <v>46083.46228009259</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46083.40207175926</v>
+        <v>46083.48002314815</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46083.39827546296</v>
+        <v>46083.47206018519</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1763,7 +1763,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46083.38108796296</v>
+        <v>46083.46305555556</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1945,7 +1945,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46083.22623842592</v>
+        <v>46083.47342592593</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2004,7 +2004,7 @@
         <v>1</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>46083.16126157407</v>
+        <v>46083.47077546296</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2138,6 +2138,11 @@
           <t>AUDITORIO</t>
         </is>
       </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>10.69.3.151</t>
+        </is>
+      </c>
       <c r="D27" t="n">
         <v>2019</v>
       </c>
@@ -2178,7 +2183,7 @@
         <v>1</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46083.1434837963</v>
+        <v>46083.48655092593</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2239,7 +2244,7 @@
         </is>
       </c>
       <c r="N28" s="3" t="n">
-        <v>46083.38260416667</v>
+        <v>46083.46189814815</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -6565,7 +6570,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46083.38186342592</v>
+        <v>46083.45717592593</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6634,7 +6639,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46080.79733796296</v>
+        <v>46083.46807870371</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6703,7 +6708,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46083.40333333334</v>
+        <v>46083.48081018519</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6767,7 +6772,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46083.36736111111</v>
+        <v>46083.48034722222</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6836,7 +6841,7 @@
         <v>1</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46081.58810185185</v>
+        <v>46083.48259259259</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6905,7 +6910,7 @@
         <v>2</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46083.38962962963</v>
+        <v>46083.46832175926</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6974,7 +6979,7 @@
         <v>1</v>
       </c>
       <c r="N101" s="3" t="n">
-        <v>46083.40013888889</v>
+        <v>46083.48170138889</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -7112,7 +7117,7 @@
         <v>2</v>
       </c>
       <c r="N103" s="3" t="n">
-        <v>46083.39050925926</v>
+        <v>46083.46755787037</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -7369,7 +7374,7 @@
         <v>1</v>
       </c>
       <c r="N107" s="3" t="n">
-        <v>46083.37668981482</v>
+        <v>46083.45731481481</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -7507,7 +7512,7 @@
         <v>1</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46083.39693287037</v>
+        <v>46083.47347222222</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7576,7 +7581,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46083.39693287037</v>
+        <v>46083.47645833333</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7645,7 +7650,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46083.37052083333</v>
+        <v>46083.45234953704</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7714,7 +7719,7 @@
         <v>2</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46083.39858796296</v>
+        <v>46083.47554398148</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7783,7 +7788,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46083.39363425926</v>
+        <v>46083.47680555555</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7852,7 +7857,7 @@
         <v>1</v>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46083.37153935185</v>
+        <v>46083.48486111111</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7918,7 +7923,7 @@
         </is>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46083.37663194445</v>
+        <v>46083.45010416667</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7987,7 +7992,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46083.38702546297</v>
+        <v>46083.46612268518</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8056,7 +8061,7 @@
         <v>1</v>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46083.40143518519</v>
+        <v>46083.47858796296</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8122,7 +8127,7 @@
         </is>
       </c>
       <c r="N118" s="3" t="n">
-        <v>46083.37429398148</v>
+        <v>46083.4509837963</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -8260,7 +8265,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46083.39744212963</v>
+        <v>46083.47489583334</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8395,7 +8400,7 @@
         </is>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46083.39796296296</v>
+        <v>46083.47453703704</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8464,7 +8469,7 @@
         <v>2</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46083.27993055555</v>
+        <v>46083.46135416667</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8533,7 +8538,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46083.40447916667</v>
+        <v>46083.48027777778</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8602,7 +8607,7 @@
         <v>1</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46083.3908912037</v>
+        <v>46083.46978009259</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8671,7 +8676,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46081.5318287037</v>
+        <v>46083.45767361111</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8740,7 +8745,7 @@
         <v>2</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46083.39143518519</v>
+        <v>46083.47090277778</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8809,7 +8814,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46083.40206018519</v>
+        <v>46083.47969907407</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8947,7 +8952,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46083.37271990741</v>
+        <v>46083.47067129629</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9011,7 +9016,7 @@
         <v>1</v>
       </c>
       <c r="N131" s="3" t="n">
-        <v>46083.38194444445</v>
+        <v>46083.45921296296</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -9463,7 +9468,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46083.37601851852</v>
+        <v>46083.47012731482</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9527,7 +9532,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46083.37900462963</v>
+        <v>46083.4816087963</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9655,7 +9660,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46083.37694444445</v>
+        <v>46083.45575231482</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9719,7 +9724,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46083.39814814815</v>
+        <v>46083.47912037037</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9783,7 +9788,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46083.38372685185</v>
+        <v>46083.47265046297</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9847,7 +9852,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46081.58719907407</v>
+        <v>46083.48078703704</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9911,7 +9916,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46083.38153935185</v>
+        <v>46083.47329861111</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9975,7 +9980,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46083.37847222222</v>
+        <v>46083.46267361111</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10039,7 +10044,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46081.59994212963</v>
+        <v>46083.48024305556</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10103,7 +10108,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46083.37789351852</v>
+        <v>46083.45395833333</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10167,7 +10172,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46083.38362268519</v>
+        <v>46083.45763888889</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10295,7 +10300,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46083.37761574074</v>
+        <v>46083.45768518518</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10359,7 +10364,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46083.38886574074</v>
+        <v>46083.46550925926</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10423,7 +10428,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46083.38559027778</v>
+        <v>46083.46270833333</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10487,7 +10492,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46083.37755787037</v>
+        <v>46083.46053240741</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10551,7 +10556,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46083.38436342592</v>
+        <v>46083.46204861111</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10679,7 +10684,7 @@
         <v>1</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>46083.38212962963</v>
+        <v>46083.45804398148</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -10743,7 +10748,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46083.36474537037</v>
+        <v>46083.48771990741</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10807,7 +10812,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46083.37556712963</v>
+        <v>46083.45554398148</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10871,7 +10876,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46083.37605324074</v>
+        <v>46083.41800925926</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10935,7 +10940,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46083.37467592592</v>
+        <v>46083.48622685186</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -10999,7 +11004,7 @@
         <v>1</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46083.37278935185</v>
+        <v>46083.48690972223</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11127,7 +11132,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46083.3955324074</v>
+        <v>46083.45256944445</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11191,7 +11196,7 @@
         <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46083.40359953704</v>
+        <v>46083.47783564815</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11255,7 +11260,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46083.37292824074</v>
+        <v>46083.45508101852</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11319,7 +11324,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46083.40298611111</v>
+        <v>46083.47989583333</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11383,7 +11388,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46083.39625</v>
+        <v>46083.45849537037</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11447,7 +11452,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46083.38010416667</v>
+        <v>46083.45473379629</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11511,7 +11516,7 @@
         <v>2</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46083.38280092592</v>
+        <v>46083.4787037037</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11575,7 +11580,7 @@
         <v>1</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46083.40086805556</v>
+        <v>46083.47246527778</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11639,7 +11644,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46081.29152777778</v>
+        <v>46083.45615740741</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11703,7 +11708,7 @@
         <v>1</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46083.37211805556</v>
+        <v>46083.45126157408</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11767,7 +11772,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46083.37331018518</v>
+        <v>46083.45201388889</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11831,7 +11836,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46083.38180555555</v>
+        <v>46083.46388888889</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11895,7 +11900,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46080.78006944444</v>
+        <v>46083.45938657408</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -12023,7 +12028,7 @@
         <v>2</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46083.40362268518</v>
+        <v>46083.48092592593</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12087,7 +12092,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46083.37747685185</v>
+        <v>46083.45118055555</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12151,7 +12156,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46083.37731481482</v>
+        <v>46083.45590277778</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12215,7 +12220,7 @@
         <v>1</v>
       </c>
       <c r="N181" s="3" t="n">
-        <v>46083.39814814815</v>
+        <v>46083.4737037037</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
@@ -12412,7 +12417,7 @@
         <v>2</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46083.37998842593</v>
+        <v>46083.46085648148</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12540,7 +12545,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46081.37732638889</v>
+        <v>46083.48527777778</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12604,7 +12609,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46083.39762731481</v>
+        <v>46083.46237268519</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12754,11 +12759,6 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
-      <c r="C190" t="inlineStr">
-        <is>
-          <t>10.69.5.59</t>
-        </is>
-      </c>
       <c r="D190" t="n">
         <v>2015</v>
       </c>
@@ -12796,7 +12796,7 @@
         </is>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46083.3934375</v>
+        <v>46083.46603009259</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12860,7 +12860,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46083.37872685185</v>
+        <v>46083.4846412037</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12924,7 +12924,7 @@
         <v>1</v>
       </c>
       <c r="N192" s="3" t="n">
-        <v>46083.40439814814</v>
+        <v>46083.46822916667</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
@@ -13049,7 +13049,7 @@
         <v>2</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46083.40412037037</v>
+        <v>46083.47581018518</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13113,7 +13113,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46083.37106481481</v>
+        <v>46083.44994212963</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13177,7 +13177,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46083.39400462963</v>
+        <v>46083.48446759259</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13241,7 +13241,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46083.38978009259</v>
+        <v>46083.46597222222</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13305,7 +13305,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46083.39280092593</v>
+        <v>46083.48665509259</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13369,7 +13369,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46083.39635416667</v>
+        <v>46083.48503472222</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13433,7 +13433,7 @@
         <v>1</v>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46083.40439814814</v>
+        <v>46083.4793287037</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13558,7 +13558,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46083.37413194445</v>
+        <v>46083.45159722222</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13622,7 +13622,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46083.39777777778</v>
+        <v>46083.46668981481</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13750,7 +13750,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46083.37643518519</v>
+        <v>46083.48538194445</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13814,7 +13814,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46083.39299768519</v>
+        <v>46083.47518518518</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13878,7 +13878,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46083.40020833333</v>
+        <v>46083.48559027778</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13942,7 +13942,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46083.39748842592</v>
+        <v>46083.48748842593</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14006,7 +14006,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46083.40002314815</v>
+        <v>46083.4865625</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14070,7 +14070,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46083.40479166667</v>
+        <v>46083.48425925926</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14134,7 +14134,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46083.38034722222</v>
+        <v>46083.45939814814</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14198,7 +14198,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46083.38030092593</v>
+        <v>46083.45439814815</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14262,7 +14262,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46083.37788194444</v>
+        <v>46083.45872685185</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14326,7 +14326,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46083.37681712963</v>
+        <v>46083.45556712963</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14390,7 +14390,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46083.38506944444</v>
+        <v>46083.45809027777</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14454,7 +14454,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46083.40157407407</v>
+        <v>46083.4828125</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14513,7 +14513,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46083.38002314815</v>
+        <v>46083.46002314815</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14577,7 +14577,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46083.38348379629</v>
+        <v>46083.46283564815</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14710,7 +14710,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46083.38469907407</v>
+        <v>46083.45947916667</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14774,7 +14774,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46083.37788194444</v>
+        <v>46083.45923611111</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14838,7 +14838,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46083.38506944444</v>
+        <v>46083.46395833333</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14902,7 +14902,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46083.40039351852</v>
+        <v>46083.47387731481</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -15030,7 +15030,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46081.37142361111</v>
+        <v>46083.44922453703</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15094,7 +15094,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46083.40136574074</v>
+        <v>46083.48498842592</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15222,7 +15222,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46083.40072916666</v>
+        <v>46083.45575231482</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15286,7 +15286,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46083.38762731481</v>
+        <v>46083.47046296296</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15350,7 +15350,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46083.4027199074</v>
+        <v>46083.48119212963</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15414,7 +15414,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46083.39063657408</v>
+        <v>46083.46991898148</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15478,7 +15478,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46083.36997685185</v>
+        <v>46083.485625</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15542,7 +15542,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46083.37453703704</v>
+        <v>46083.45850694444</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15606,7 +15606,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46083.40439814814</v>
+        <v>46083.47975694444</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15670,7 +15670,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46083.38736111111</v>
+        <v>46083.46850694445</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15734,7 +15734,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46083.40193287037</v>
+        <v>46083.48054398148</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15798,7 +15798,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46079.36840277778</v>
+        <v>46083.4871875</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15862,7 +15862,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46083.38327546296</v>
+        <v>46083.47596064815</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15926,7 +15926,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46083.38950231481</v>
+        <v>46083.48064814815</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -15990,7 +15990,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46083.40040509259</v>
+        <v>46083.48549768519</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16118,7 +16118,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46083.3785300926</v>
+        <v>46083.45414351852</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16182,7 +16182,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46083.39803240741</v>
+        <v>46083.47803240741</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16305,7 +16305,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46083.40189814815</v>
+        <v>46083.45965277778</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16369,7 +16369,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46083.39136574074</v>
+        <v>46083.47234953703</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16433,7 +16433,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46081.60538194444</v>
+        <v>46083.48239583334</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16497,7 +16497,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46081.59859953704</v>
+        <v>46083.48245370371</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16561,7 +16561,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46083.39855324074</v>
+        <v>46083.4843287037</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16620,7 +16620,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46083.39784722222</v>
+        <v>46083.47626157408</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16684,7 +16684,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46083.39895833333</v>
+        <v>46083.48538194445</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16812,7 +16812,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46083.38966435185</v>
+        <v>46083.48519675926</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16870,7 +16870,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46083.3983912037</v>
+        <v>46083.47664351852</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16934,7 +16934,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46083.39869212963</v>
+        <v>46083.48570601852</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -16998,7 +16998,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46083.38950231481</v>
+        <v>46083.45616898148</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17062,7 +17062,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46083.40335648148</v>
+        <v>46083.48532407408</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17126,7 +17126,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46083.38244212963</v>
+        <v>46083.48449074074</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17190,7 +17190,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46081.38613425926</v>
+        <v>46083.46590277777</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17254,7 +17254,7 @@
         <v>1</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46083.36489583334</v>
+        <v>46083.48599537037</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17318,7 +17318,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46083.40145833333</v>
+        <v>46083.45221064815</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17382,7 +17382,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46083.39061342592</v>
+        <v>46083.46686342593</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17446,7 +17446,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46083.38122685185</v>
+        <v>46083.45505787037</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17510,7 +17510,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46083.4018287037</v>
+        <v>46083.48453703704</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17574,7 +17574,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46083.38542824074</v>
+        <v>46083.46137731482</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17638,7 +17638,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46083.40096064815</v>
+        <v>46083.47773148148</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17702,7 +17702,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46083.39949074074</v>
+        <v>46083.48579861111</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17766,7 +17766,7 @@
         <v>1</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46081.60807870371</v>
+        <v>46083.48555555556</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17830,7 +17830,7 @@
         <v>1</v>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46081.61785879629</v>
+        <v>46083.47581018518</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17891,7 +17891,7 @@
         </is>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46083.37460648148</v>
+        <v>46083.45570601852</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -17955,7 +17955,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46081.29568287037</v>
+        <v>46083.47642361111</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -18019,7 +18019,7 @@
         <v>1</v>
       </c>
       <c r="N272" s="3" t="n">
-        <v>46083.38991898148</v>
+        <v>46083.46381944444</v>
       </c>
       <c r="O272" t="inlineStr">
         <is>
@@ -18083,7 +18083,7 @@
         <v>2</v>
       </c>
       <c r="N273" s="3" t="n">
-        <v>46081.58387731481</v>
+        <v>46083.48023148148</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -18339,7 +18339,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46080.86256944444</v>
+        <v>46083.48449074074</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18403,7 +18403,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46083.40425925926</v>
+        <v>46083.47967592593</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18467,7 +18467,7 @@
         <v>1</v>
       </c>
       <c r="N279" s="3" t="n">
-        <v>46083.40175925926</v>
+        <v>46083.4815625</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -18531,7 +18531,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46083.38608796296</v>
+        <v>46083.47760416667</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18595,7 +18595,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46083.40166666666</v>
+        <v>46083.47528935185</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18659,7 +18659,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46083.39819444445</v>
+        <v>46083.4853125</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18723,7 +18723,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46083.39061342592</v>
+        <v>46083.48658564815</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18787,7 +18787,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46083.39412037037</v>
+        <v>46083.47018518519</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18851,7 +18851,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46083.37212962963</v>
+        <v>46083.45542824074</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18870,11 +18870,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C286" t="inlineStr">
-        <is>
-          <t>10.69.5.155</t>
-        </is>
-      </c>
       <c r="D286" t="n">
         <v>2019</v>
       </c>
@@ -18915,7 +18910,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46083.35678240741</v>
+        <v>46083.46097222222</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18979,7 +18974,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46083.37887731481</v>
+        <v>46083.45896990741</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19043,7 +19038,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46083.39965277778</v>
+        <v>46083.48280092593</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19107,7 +19102,7 @@
         <v>1</v>
       </c>
       <c r="N289" s="3" t="n">
-        <v>46083.39951388889</v>
+        <v>46083.46714120371</v>
       </c>
       <c r="O289" t="inlineStr">
         <is>
@@ -19901,7 +19896,7 @@
         <v>1</v>
       </c>
       <c r="N302" s="3" t="n">
-        <v>46083.38498842593</v>
+        <v>46083.46466435185</v>
       </c>
       <c r="O302" t="inlineStr">
         <is>
@@ -21017,7 +21012,7 @@
         </is>
       </c>
       <c r="N320" s="3" t="n">
-        <v>46083.40133101852</v>
+        <v>46083.47706018519</v>
       </c>
       <c r="O320" t="inlineStr">
         <is>
@@ -21742,7 +21737,7 @@
         <v>1</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46083.38795138889</v>
+        <v>46083.4721412037</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21806,7 +21801,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46083.38449074074</v>
+        <v>46083.46534722222</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21870,7 +21865,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46083.38957175926</v>
+        <v>46083.46828703704</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21934,7 +21929,7 @@
         <v>2</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46083.39796296296</v>
+        <v>46083.47987268519</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21998,7 +21993,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46083.3806712963</v>
+        <v>46083.45638888889</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22062,7 +22057,7 @@
         <v>1</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46083.36667824074</v>
+        <v>46083.45041666667</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22126,7 +22121,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46083.40239583333</v>
+        <v>46083.48094907407</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22190,7 +22185,7 @@
         <v>2</v>
       </c>
       <c r="N339" s="3" t="n">
-        <v>46083.38565972223</v>
+        <v>46083.46653935185</v>
       </c>
       <c r="O339" t="inlineStr">
         <is>
@@ -22254,7 +22249,7 @@
         <v>1</v>
       </c>
       <c r="N340" s="3" t="n">
-        <v>46081.49881944444</v>
+        <v>46083.46653935185</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -22318,7 +22313,7 @@
         <v>2</v>
       </c>
       <c r="N341" s="3" t="n">
-        <v>46083.38724537037</v>
+        <v>46083.46350694444</v>
       </c>
       <c r="O341" t="inlineStr">
         <is>
@@ -22382,7 +22377,7 @@
         <v>2</v>
       </c>
       <c r="N342" s="3" t="n">
-        <v>46083.37887731481</v>
+        <v>46083.45814814815</v>
       </c>
       <c r="O342" t="inlineStr">
         <is>
@@ -22699,7 +22694,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46081.5865162037</v>
+        <v>46083.48540509259</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22763,7 +22758,7 @@
         <v>1</v>
       </c>
       <c r="N348" s="3" t="n">
-        <v>46080.7421875</v>
+        <v>46083.4868287037</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -22827,7 +22822,7 @@
         <v>1</v>
       </c>
       <c r="N349" s="3" t="n">
-        <v>46080.71203703704</v>
+        <v>46083.4815162037</v>
       </c>
       <c r="O349" t="inlineStr">
         <is>
@@ -22846,6 +22841,11 @@
           <t>OPERACAO 9.1</t>
         </is>
       </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>10.69.5.244</t>
+        </is>
+      </c>
       <c r="D350" t="n">
         <v>2014</v>
       </c>
@@ -22886,7 +22886,7 @@
         <v>1</v>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46080.72943287037</v>
+        <v>46083.46655092593</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -22950,7 +22950,7 @@
         <v>1</v>
       </c>
       <c r="N351" s="3" t="n">
-        <v>46080.70388888889</v>
+        <v>46083.4878125</v>
       </c>
       <c r="O351" t="inlineStr">
         <is>
@@ -23014,7 +23014,7 @@
         <v>1</v>
       </c>
       <c r="N352" s="3" t="n">
-        <v>46080.70270833333</v>
+        <v>46083.48471064815</v>
       </c>
       <c r="O352" t="inlineStr">
         <is>
@@ -23075,7 +23075,7 @@
         </is>
       </c>
       <c r="N353" s="3" t="n">
-        <v>46080.70700231481</v>
+        <v>46083.47951388889</v>
       </c>
       <c r="O353" t="inlineStr">
         <is>
@@ -23200,7 +23200,7 @@
         <v>1</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46080.74091435185</v>
+        <v>46083.48368055555</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23264,7 +23264,7 @@
         <v>1</v>
       </c>
       <c r="N356" s="3" t="n">
-        <v>46080.7109375</v>
+        <v>46083.48166666667</v>
       </c>
       <c r="O356" t="inlineStr">
         <is>
@@ -23328,7 +23328,7 @@
         <v>1</v>
       </c>
       <c r="N357" s="3" t="n">
-        <v>46080.70726851852</v>
+        <v>46083.48263888889</v>
       </c>
       <c r="O357" t="inlineStr">
         <is>
@@ -23451,7 +23451,7 @@
         <v>2</v>
       </c>
       <c r="N359" s="3" t="n">
-        <v>46080.7069675926</v>
+        <v>46083.48140046297</v>
       </c>
       <c r="O359" t="inlineStr">
         <is>
@@ -23515,7 +23515,7 @@
         <v>2</v>
       </c>
       <c r="N360" s="3" t="n">
-        <v>46080.8618287037</v>
+        <v>46083.48318287037</v>
       </c>
       <c r="O360" t="inlineStr">
         <is>
@@ -23579,7 +23579,7 @@
         <v>1</v>
       </c>
       <c r="N361" s="3" t="n">
-        <v>46078.59190972222</v>
+        <v>46083.48659722223</v>
       </c>
       <c r="O361" t="inlineStr">
         <is>
@@ -23640,7 +23640,7 @@
         </is>
       </c>
       <c r="N362" s="3" t="n">
-        <v>46078.57268518519</v>
+        <v>46083.44710648148</v>
       </c>
       <c r="O362" t="inlineStr">
         <is>
@@ -23828,7 +23828,7 @@
         <v>1</v>
       </c>
       <c r="N365" s="3" t="n">
-        <v>46083.38070601852</v>
+        <v>46083.45606481482</v>
       </c>
       <c r="O365" t="inlineStr">
         <is>
@@ -23894,7 +23894,7 @@
         </is>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46083.38340277778</v>
+        <v>46083.45694444444</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
@@ -24020,7 +24020,7 @@
         </is>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46083.39820601852</v>
+        <v>46083.47282407407</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24081,7 +24081,7 @@
         </is>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46083.39616898148</v>
+        <v>46083.47217592593</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24150,7 +24150,7 @@
         <v>1</v>
       </c>
       <c r="N370" s="3" t="n">
-        <v>46083.36677083333</v>
+        <v>46083.44734953704</v>
       </c>
       <c r="O370" t="inlineStr">
         <is>
@@ -24357,7 +24357,7 @@
         <v>1</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46083.37754629629</v>
+        <v>46083.46134259259</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24426,7 +24426,7 @@
         <v>1</v>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46083.38230324074</v>
+        <v>46083.46246527778</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24492,7 +24492,7 @@
         </is>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46083.40090277778</v>
+        <v>46083.473125</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24556,7 +24556,7 @@
         <v>1</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46083.3753125</v>
+        <v>46083.45583333333</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -24625,7 +24625,7 @@
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46083.39449074074</v>
+        <v>46083.47702546296</v>
       </c>
       <c r="O377" t="inlineStr">
         <is>
@@ -24694,7 +24694,7 @@
         <v>2</v>
       </c>
       <c r="N378" s="3" t="n">
-        <v>46083.37761574074</v>
+        <v>46083.4570949074</v>
       </c>
       <c r="O378" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-02 15:52:05.210943
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46083.56918981481</v>
+        <v>46083.64827546296</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46083.54047453704</v>
+        <v>46083.62157407407</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>1</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46083.55497685185</v>
+        <v>46083.63289351852</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46083.52912037037</v>
+        <v>46083.64351851852</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46083.55996527777</v>
+        <v>46083.64274305556</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
         <v>1</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>46083.55962962963</v>
+        <v>46083.64268518519</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1382,7 +1382,7 @@
         <v>2</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>46083.54825231482</v>
+        <v>46083.62454861111</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46083.54990740741</v>
+        <v>46083.62681712963</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1510,7 +1510,7 @@
         <v>2</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>46083.54351851852</v>
+        <v>46083.62244212963</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46083.55915509259</v>
+        <v>46083.63726851852</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46083.55260416667</v>
+        <v>46083.63482638889</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1763,7 +1763,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46083.54425925926</v>
+        <v>46083.62328703704</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1827,7 +1827,7 @@
         <v>1</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>46083.55579861111</v>
+        <v>46083.63702546297</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -1945,7 +1945,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46083.54895833333</v>
+        <v>46083.62525462963</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2004,7 +2004,7 @@
         <v>1</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>46083.54675925926</v>
+        <v>46083.62354166667</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2060,7 +2060,7 @@
         </is>
       </c>
       <c r="N25" s="3" t="n">
-        <v>46083.16996527778</v>
+        <v>46083.60783564814</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2138,11 +2138,6 @@
           <t>AUDITORIO</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>10.69.3.151</t>
-        </is>
-      </c>
       <c r="D27" t="n">
         <v>2019</v>
       </c>
@@ -2183,7 +2178,7 @@
         <v>1</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46083.56804398148</v>
+        <v>46083.60547453703</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2244,7 +2239,7 @@
         </is>
       </c>
       <c r="N28" s="3" t="n">
-        <v>46083.54082175926</v>
+        <v>46083.65369212963</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -6570,7 +6565,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46083.53414351852</v>
+        <v>46083.61366898148</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6639,7 +6634,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46083.55203703704</v>
+        <v>46083.62834490741</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6703,7 +6698,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46083.55609953704</v>
+        <v>46083.63606481482</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6722,11 +6717,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>10.69.3.94</t>
-        </is>
-      </c>
       <c r="D98" t="n">
         <v>2025</v>
       </c>
@@ -6772,7 +6762,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46083.55887731481</v>
+        <v>46083.64167824074</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6841,7 +6831,7 @@
         <v>1</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46083.55950231481</v>
+        <v>46083.63601851852</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6910,7 +6900,7 @@
         <v>2</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46083.54868055556</v>
+        <v>46083.62866898148</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6979,7 +6969,7 @@
         <v>1</v>
       </c>
       <c r="N101" s="3" t="n">
-        <v>46083.55881944444</v>
+        <v>46083.63912037037</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -7117,7 +7107,7 @@
         <v>2</v>
       </c>
       <c r="N103" s="3" t="n">
-        <v>46083.54115740741</v>
+        <v>46083.61645833333</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -7244,7 +7234,7 @@
         </is>
       </c>
       <c r="N105" s="3" t="n">
-        <v>46083.53202546296</v>
+        <v>46083.61646990741</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
@@ -7374,7 +7364,7 @@
         <v>1</v>
       </c>
       <c r="N107" s="3" t="n">
-        <v>46083.57001157408</v>
+        <v>46083.64925925926</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -7512,7 +7502,7 @@
         <v>1</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46083.54788194445</v>
+        <v>46083.62241898148</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7581,7 +7571,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46083.55050925926</v>
+        <v>46083.62952546297</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7650,7 +7640,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46083.5690625</v>
+        <v>46083.64917824074</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7719,7 +7709,7 @@
         <v>2</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46083.55728009259</v>
+        <v>46083.64027777778</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7788,7 +7778,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46083.55974537037</v>
+        <v>46083.63564814815</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7857,7 +7847,7 @@
         <v>1</v>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46083.56407407407</v>
+        <v>46083.6409375</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7923,7 +7913,7 @@
         </is>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46083.53076388889</v>
+        <v>46083.65079861111</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7992,7 +7982,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46083.548125</v>
+        <v>46083.62996527777</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8056,7 +8046,7 @@
         <v>1</v>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46083.55689814815</v>
+        <v>46083.63543981482</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8122,7 +8112,7 @@
         </is>
       </c>
       <c r="N118" s="3" t="n">
-        <v>46083.56763888889</v>
+        <v>46083.64563657407</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -8260,7 +8250,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46083.55271990741</v>
+        <v>46083.62815972222</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8329,7 +8319,7 @@
         <v>1</v>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46083.54563657408</v>
+        <v>46083.654375</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8395,7 +8385,7 @@
         </is>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46083.55269675926</v>
+        <v>46083.63017361111</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8464,7 +8454,7 @@
         <v>2</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46083.54076388889</v>
+        <v>46083.62113425926</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8533,7 +8523,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46083.55755787037</v>
+        <v>46083.63208333333</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8602,7 +8592,7 @@
         <v>1</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46083.54938657407</v>
+        <v>46083.62645833333</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8671,7 +8661,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46083.56831018518</v>
+        <v>46083.65130787037</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8740,7 +8730,7 @@
         <v>2</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46083.54526620371</v>
+        <v>46083.62311342593</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8809,7 +8799,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46083.55567129629</v>
+        <v>46083.6321875</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8947,7 +8937,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46083.56105324074</v>
+        <v>46083.64935185185</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9011,7 +9001,7 @@
         <v>1</v>
       </c>
       <c r="N131" s="3" t="n">
-        <v>46083.53196759259</v>
+        <v>46083.64822916667</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -9144,7 +9134,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46080.56614583333</v>
+        <v>46083.62354166667</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9208,7 +9198,7 @@
         <v>1</v>
       </c>
       <c r="N134" s="3" t="n">
-        <v>46081.60379629629</v>
+        <v>46083.61991898148</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -9272,7 +9262,7 @@
         <v>1</v>
       </c>
       <c r="N135" s="3" t="n">
-        <v>46081.60099537037</v>
+        <v>46083.63270833333</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -9463,7 +9453,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46083.54905092593</v>
+        <v>46083.62744212963</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9527,7 +9517,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46083.55626157407</v>
+        <v>46083.61802083333</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9591,7 +9581,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46081.5971412037</v>
+        <v>46083.61818287037</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9655,7 +9645,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46083.56648148148</v>
+        <v>46083.64263888889</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9719,7 +9709,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46083.56222222222</v>
+        <v>46083.63454861111</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9783,7 +9773,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46083.54902777778</v>
+        <v>46083.63127314814</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9847,7 +9837,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46083.56353009259</v>
+        <v>46083.63987268518</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9911,7 +9901,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46083.54954861111</v>
+        <v>46083.6515625</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9975,7 +9965,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46083.54210648148</v>
+        <v>46083.61875</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10039,7 +10029,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46083.55824074074</v>
+        <v>46083.63528935185</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10103,7 +10093,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46083.56842592593</v>
+        <v>46083.64747685185</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10167,7 +10157,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46083.56886574074</v>
+        <v>46083.64253472222</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10231,7 +10221,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46081.84983796296</v>
+        <v>46083.62334490741</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10295,7 +10285,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46083.53861111111</v>
+        <v>46083.61993055556</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10359,7 +10349,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46083.54528935185</v>
+        <v>46083.63221064815</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10378,6 +10368,11 @@
           <t>OPERACAO 7.1</t>
         </is>
       </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>10.69.5.21</t>
+        </is>
+      </c>
       <c r="D153" t="n">
         <v>2018</v>
       </c>
@@ -10418,7 +10413,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46083.53929398148</v>
+        <v>46083.64587962963</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10482,7 +10477,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46083.53342592593</v>
+        <v>46083.58376157407</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10546,7 +10541,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46083.53804398148</v>
+        <v>46083.64994212963</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10610,7 +10605,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46080.81335648148</v>
+        <v>46083.63701388889</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10674,7 +10669,7 @@
         <v>1</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>46083.53690972222</v>
+        <v>46083.64099537037</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -10738,7 +10733,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46083.56578703703</v>
+        <v>46083.64461805556</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10802,7 +10797,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46083.56385416666</v>
+        <v>46083.64075231482</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10866,7 +10861,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46083.41800925926</v>
+        <v>46083.62144675926</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10930,7 +10925,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46083.56309027778</v>
+        <v>46083.6215162037</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -10994,7 +10989,7 @@
         <v>1</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46083.56423611111</v>
+        <v>46083.61887731482</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11122,7 +11117,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46083.57072916667</v>
+        <v>46083.64513888889</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11250,7 +11245,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46083.53341435185</v>
+        <v>46083.60706018518</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11314,7 +11309,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46083.55519675926</v>
+        <v>46083.59142361111</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11442,7 +11437,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46083.56972222222</v>
+        <v>46083.65333333334</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11634,7 +11629,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46083.56668981481</v>
+        <v>46083.6434375</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11698,7 +11693,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46083.56194444445</v>
+        <v>46083.6396875</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11762,7 +11757,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46083.53202546296</v>
+        <v>46083.57162037037</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11826,7 +11821,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46083.53854166667</v>
+        <v>46083.61597222222</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11890,7 +11885,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46083.54060185186</v>
+        <v>46083.6533912037</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11954,7 +11949,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46083.53942129629</v>
+        <v>46083.61659722222</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12018,7 +12013,7 @@
         <v>2</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46083.55484953704</v>
+        <v>46083.63509259259</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12082,7 +12077,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46083.5346875</v>
+        <v>46083.63703703704</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12146,7 +12141,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46083.53857638889</v>
+        <v>46083.62166666667</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12210,7 +12205,7 @@
         <v>1</v>
       </c>
       <c r="N181" s="3" t="n">
-        <v>46083.54834490741</v>
+        <v>46083.62457175926</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
@@ -12407,7 +12402,7 @@
         <v>2</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46083.53834490741</v>
+        <v>46083.61615740741</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12535,7 +12530,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46083.56493055556</v>
+        <v>46083.60189814815</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12599,7 +12594,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46083.56423611111</v>
+        <v>46083.64149305555</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12791,7 +12786,7 @@
         </is>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46083.54035879629</v>
+        <v>46083.62052083333</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12855,7 +12850,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46083.56825231481</v>
+        <v>46083.64626157407</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12919,7 +12914,7 @@
         <v>1</v>
       </c>
       <c r="N192" s="3" t="n">
-        <v>46083.54177083333</v>
+        <v>46083.61987268519</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
@@ -13044,7 +13039,7 @@
         <v>2</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46083.55328703704</v>
+        <v>46083.62077546296</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13108,7 +13103,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46083.56938657408</v>
+        <v>46083.64942129629</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13172,7 +13167,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46083.56109953704</v>
+        <v>46083.62318287037</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13236,7 +13231,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46083.46597222222</v>
+        <v>46083.62760416666</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13300,7 +13295,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46083.56561342593</v>
+        <v>46083.63877314814</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13364,7 +13359,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46083.55883101852</v>
+        <v>46083.6241087963</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13428,7 +13423,7 @@
         <v>1</v>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46083.55365740741</v>
+        <v>46083.62644675926</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13553,7 +13548,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46083.57033564815</v>
+        <v>46083.64743055555</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13617,7 +13612,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46083.54167824074</v>
+        <v>46083.62196759259</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13745,7 +13740,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46083.53666666667</v>
+        <v>46083.61678240741</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13809,7 +13804,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46083.55402777778</v>
+        <v>46083.61844907407</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13873,7 +13868,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46083.56778935185</v>
+        <v>46083.62094907407</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13937,7 +13932,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46083.56952546296</v>
+        <v>46083.64297453704</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14001,7 +13996,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46083.56548611111</v>
+        <v>46083.62043981482</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14065,7 +14060,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46083.56622685185</v>
+        <v>46083.64709490741</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14129,7 +14124,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46083.53681712963</v>
+        <v>46083.61787037037</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14193,7 +14188,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46083.56474537037</v>
+        <v>46083.63204861111</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14257,7 +14252,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46083.56453703704</v>
+        <v>46083.640625</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14321,7 +14316,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46083.53815972222</v>
+        <v>46083.65145833333</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14385,7 +14380,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46083.53466435185</v>
+        <v>46083.64803240741</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14449,7 +14444,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46083.5660300926</v>
+        <v>46083.641875</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14468,11 +14463,6 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
-      <c r="C217" t="inlineStr">
-        <is>
-          <t>10.69.5.85</t>
-        </is>
-      </c>
       <c r="D217" t="n">
         <v>2017</v>
       </c>
@@ -14513,7 +14503,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46083.54018518519</v>
+        <v>46083.61790509259</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14577,7 +14567,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46083.538125</v>
+        <v>46083.65231481481</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14641,7 +14631,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46083.38543981482</v>
+        <v>46083.62159722222</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14710,7 +14700,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46083.53827546296</v>
+        <v>46083.615</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14774,7 +14764,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46083.53953703704</v>
+        <v>46083.63358796296</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14838,7 +14828,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46083.5421412037</v>
+        <v>46083.61747685185</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14902,7 +14892,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46083.54936342593</v>
+        <v>46083.64677083334</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14966,7 +14956,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46081.46488425926</v>
+        <v>46083.64513888889</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15030,7 +15020,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46083.56575231482</v>
+        <v>46083.63241898148</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15094,7 +15084,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46083.56255787037</v>
+        <v>46083.60423611111</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15158,7 +15148,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46081.5990625</v>
+        <v>46083.63047453704</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15222,7 +15212,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46083.53686342593</v>
+        <v>46083.64711805555</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15286,7 +15276,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46083.54899305556</v>
+        <v>46083.62565972222</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15350,7 +15340,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46083.56108796296</v>
+        <v>46083.62673611111</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15414,7 +15404,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46083.5708912037</v>
+        <v>46083.62876157407</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15478,7 +15468,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46083.56508101852</v>
+        <v>46083.63350694445</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15542,7 +15532,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46083.53571759259</v>
+        <v>46083.64798611111</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15606,7 +15596,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46083.53915509259</v>
+        <v>46083.62177083334</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15670,7 +15660,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46083.5568287037</v>
+        <v>46083.62956018518</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15734,7 +15724,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46083.56023148148</v>
+        <v>46083.636875</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15798,7 +15788,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46083.55936342593</v>
+        <v>46083.63344907408</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15862,7 +15852,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46083.5508449074</v>
+        <v>46083.63061342593</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15926,7 +15916,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46083.56189814815</v>
+        <v>46083.62972222222</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -15990,7 +15980,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46083.56326388889</v>
+        <v>46083.62248842593</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16054,7 +16044,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46081.56407407407</v>
+        <v>46083.61961805556</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16118,7 +16108,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46083.52980324074</v>
+        <v>46083.64872685185</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16182,7 +16172,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46083.55109953704</v>
+        <v>46083.62876157407</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16201,6 +16191,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>10.69.5.112</t>
+        </is>
+      </c>
       <c r="D244" t="n">
         <v>2019</v>
       </c>
@@ -16241,7 +16236,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46083.12707175926</v>
+        <v>46083.65153935185</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16305,7 +16300,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46083.56923611111</v>
+        <v>46083.64868055555</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16369,7 +16364,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46083.55039351852</v>
+        <v>46083.63427083333</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16433,7 +16428,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46083.55814814815</v>
+        <v>46083.64726851852</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16497,7 +16492,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46083.56038194444</v>
+        <v>46083.63898148148</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16561,7 +16556,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46083.56056712963</v>
+        <v>46083.63420138889</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16580,6 +16575,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>10.69.5.118</t>
+        </is>
+      </c>
       <c r="D250" t="n">
         <v>2017</v>
       </c>
@@ -16620,7 +16620,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46083.55554398148</v>
+        <v>46083.61032407408</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16684,7 +16684,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46083.5690625</v>
+        <v>46083.64758101852</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16748,7 +16748,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46081.59356481482</v>
+        <v>46083.61979166666</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16812,7 +16812,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46083.56731481481</v>
+        <v>46083.62361111111</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16870,7 +16870,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46083.55422453704</v>
+        <v>46083.63630787037</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16934,7 +16934,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46083.56314814815</v>
+        <v>46083.63878472222</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -16998,7 +16998,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46083.55032407407</v>
+        <v>46083.62771990741</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17062,7 +17062,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46083.56270833333</v>
+        <v>46083.63990740741</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17126,7 +17126,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46083.52453703704</v>
+        <v>46083.62386574074</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17190,7 +17190,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46083.54216435185</v>
+        <v>46083.57784722222</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17254,7 +17254,7 @@
         <v>1</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46083.56325231482</v>
+        <v>46083.60016203704</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17278,16 +17278,47 @@
           <t>10.69.5.130</t>
         </is>
       </c>
+      <c r="D261" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E261" t="n">
+        <v>3599</v>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Microsoft Windows 7 Professional</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>BRG037FQMK</t>
+        </is>
+      </c>
       <c r="I261" t="inlineStr">
         <is>
           <t>Intel Core 2 Duo</t>
+        </is>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>4 GB</t>
+        </is>
+      </c>
+      <c r="K261" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>HP Compaq 6000 Pro SFF PC</t>
         </is>
       </c>
       <c r="M261" t="n">
         <v>2</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46083.5459375</v>
+        <v>46083.62707175926</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17351,7 +17382,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46083.54708333333</v>
+        <v>46083.62451388889</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17415,7 +17446,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46083.56840277778</v>
+        <v>46083.63410879629</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17479,7 +17510,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46083.56674768519</v>
+        <v>46083.64269675926</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17543,7 +17574,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46083.54287037037</v>
+        <v>46083.64045138889</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17607,7 +17638,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46083.55542824074</v>
+        <v>46083.63592592593</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17671,7 +17702,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46083.56383101852</v>
+        <v>46083.64336805556</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17695,47 +17726,11 @@
           <t>10.69.5.137</t>
         </is>
       </c>
-      <c r="D268" t="n">
-        <v>2011</v>
-      </c>
-      <c r="E268" t="n">
-        <v>8390</v>
-      </c>
-      <c r="F268" t="inlineStr">
-        <is>
-          <t>Microsoft® Windows Vista™ Business</t>
-        </is>
-      </c>
-      <c r="G268" t="inlineStr">
-        <is>
-          <t>BRG922F9BQ</t>
-        </is>
-      </c>
-      <c r="I268" t="inlineStr">
-        <is>
-          <t>Intel Pentium®</t>
-        </is>
-      </c>
-      <c r="J268" t="inlineStr">
-        <is>
-          <t>3 GB</t>
-        </is>
-      </c>
-      <c r="K268" t="inlineStr">
-        <is>
-          <t>HP</t>
-        </is>
-      </c>
-      <c r="L268" t="inlineStr">
-        <is>
-          <t>HP Compaq dx7400 Brazil SFF PC.</t>
-        </is>
-      </c>
       <c r="M268" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46083.56291666667</v>
+        <v>46083.62393518518</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17799,7 +17794,7 @@
         <v>1</v>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46083.56719907407</v>
+        <v>46083.64204861111</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17860,7 +17855,7 @@
         </is>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46083.5362037037</v>
+        <v>46083.65295138889</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -17988,7 +17983,7 @@
         <v>1</v>
       </c>
       <c r="N272" s="3" t="n">
-        <v>46083.53976851852</v>
+        <v>46083.64542824074</v>
       </c>
       <c r="O272" t="inlineStr">
         <is>
@@ -18013,19 +18008,19 @@
         </is>
       </c>
       <c r="D273" t="n">
-        <v>2013</v>
+        <v>2016</v>
       </c>
       <c r="E273" t="n">
-        <v>3913</v>
+        <v>43374</v>
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>Microsoft® Windows Vista™ Business</t>
+          <t>Microsoft Windows 7 Professional</t>
         </is>
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t>G2XQXG1</t>
+          <t>BRG050GDXM</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
@@ -18040,19 +18035,19 @@
       </c>
       <c r="K273" t="inlineStr">
         <is>
-          <t>Dell Inc.</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="L273" t="inlineStr">
         <is>
-          <t>OptiPlex 755</t>
+          <t>COMPAQ 300B MT</t>
         </is>
       </c>
       <c r="M273" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N273" s="3" t="n">
-        <v>46083.55675925926</v>
+        <v>46083.6438425926</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -18127,7 +18122,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>PA_144</t>
+          <t>PA_145</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -18137,50 +18132,47 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>10.69.5.144</t>
+          <t>10.69.5.145</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>2019</v>
+        <v>2013</v>
       </c>
       <c r="E275" t="n">
-        <v>73645</v>
+        <v>3995</v>
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>Microsoft Windows 8.1 Pro</t>
+          <t>Microsoft® Windows Vista™ Business</t>
         </is>
       </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t>BRJ523SGGJ</t>
+          <t>866YLJ1</t>
         </is>
       </c>
       <c r="I275" t="inlineStr">
         <is>
-          <t>Intel Core i5</t>
+          <t>Intel Core 2 Duo</t>
         </is>
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>4 GB</t>
+          <t>2 GB</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Dell Inc.</t>
         </is>
       </c>
       <c r="L275" t="inlineStr">
         <is>
-          <t>HP 402 G1 SFF Business PC</t>
-        </is>
-      </c>
-      <c r="M275" t="n">
-        <v>1</v>
+          <t>OptiPlex 755</t>
+        </is>
       </c>
       <c r="N275" s="3" t="n">
-        <v>46057.48512731482</v>
+        <v>46083.60475694444</v>
       </c>
       <c r="O275" t="inlineStr">
         <is>
@@ -18205,19 +18197,19 @@
         </is>
       </c>
       <c r="D276" t="n">
-        <v>2016</v>
+        <v>2013</v>
       </c>
       <c r="E276" t="n">
-        <v>43374</v>
+        <v>3913</v>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>Microsoft Windows 7 Professional</t>
+          <t>Microsoft® Windows Vista™ Business</t>
         </is>
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t>BRG050GDXM</t>
+          <t>G2XQXG1</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
@@ -18232,19 +18224,19 @@
       </c>
       <c r="K276" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Dell Inc.</t>
         </is>
       </c>
       <c r="L276" t="inlineStr">
         <is>
-          <t>COMPAQ 300B MT</t>
+          <t>OptiPlex 755</t>
         </is>
       </c>
       <c r="M276" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N276" s="3" t="n">
-        <v>46083.5633912037</v>
+        <v>46083.63725694444</v>
       </c>
       <c r="O276" t="inlineStr">
         <is>
@@ -18308,7 +18300,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46083.47967592593</v>
+        <v>46083.58732638889</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18372,7 +18364,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46083.55787037037</v>
+        <v>46083.63924768518</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18500,7 +18492,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46083.54231481482</v>
+        <v>46083.61954861111</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18519,11 +18511,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C281" t="inlineStr">
-        <is>
-          <t>10.69.5.151</t>
-        </is>
-      </c>
       <c r="D281" t="n">
         <v>2017</v>
       </c>
@@ -18628,7 +18615,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46083.56738425926</v>
+        <v>46083.63380787037</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18692,7 +18679,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46083.5427662037</v>
+        <v>46083.6196875</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18756,7 +18743,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46083.53641203704</v>
+        <v>46083.65054398148</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18815,7 +18802,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46083.53586805556</v>
+        <v>46083.57696759259</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18879,7 +18866,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46083.53439814815</v>
+        <v>46083.614375</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18943,7 +18930,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46083.53512731481</v>
+        <v>46083.57546296297</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19007,7 +18994,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46083.55015046296</v>
+        <v>46083.63113425926</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19801,7 +19788,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46083.54177083333</v>
+        <v>46083.61678240741</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20917,7 +20904,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46083.55502314815</v>
+        <v>46083.6359375</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21642,7 +21629,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46083.5497337963</v>
+        <v>46083.63071759259</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21706,7 +21693,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46083.54328703704</v>
+        <v>46083.62244212963</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21770,7 +21757,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46083.54868055556</v>
+        <v>46083.63053240741</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21834,7 +21821,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46083.55744212963</v>
+        <v>46083.63127314814</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21898,7 +21885,7 @@
         <v>1</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46083.57028935185</v>
+        <v>46083.64622685185</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21962,7 +21949,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46083.53484953703</v>
+        <v>46083.61630787037</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22026,7 +22013,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46083.55659722222</v>
+        <v>46083.63027777777</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22090,7 +22077,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46083.53877314815</v>
+        <v>46083.61820601852</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22154,7 +22141,7 @@
         <v>1</v>
       </c>
       <c r="N339" s="3" t="n">
-        <v>46083.54589120371</v>
+        <v>46083.58224537037</v>
       </c>
       <c r="O339" t="inlineStr">
         <is>
@@ -22218,7 +22205,7 @@
         <v>2</v>
       </c>
       <c r="N340" s="3" t="n">
-        <v>46083.54432870371</v>
+        <v>46083.57987268519</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -22599,7 +22586,7 @@
         <v>1</v>
       </c>
       <c r="N346" s="3" t="n">
-        <v>46083.56262731482</v>
+        <v>46083.59797453704</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -22663,7 +22650,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46083.5616087963</v>
+        <v>46083.59905092593</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22727,7 +22714,7 @@
         <v>1</v>
       </c>
       <c r="N348" s="3" t="n">
-        <v>46083.56168981481</v>
+        <v>46083.60413194444</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -22786,7 +22773,7 @@
         <v>1</v>
       </c>
       <c r="N349" s="3" t="n">
-        <v>46083.53971064815</v>
+        <v>46083.57994212963</v>
       </c>
       <c r="O349" t="inlineStr">
         <is>
@@ -22850,7 +22837,7 @@
         <v>1</v>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46083.53127314815</v>
+        <v>46083.57173611111</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -22914,7 +22901,7 @@
         <v>1</v>
       </c>
       <c r="N351" s="3" t="n">
-        <v>46083.56363425926</v>
+        <v>46083.60268518519</v>
       </c>
       <c r="O351" t="inlineStr">
         <is>
@@ -22975,7 +22962,7 @@
         </is>
       </c>
       <c r="N352" s="3" t="n">
-        <v>46083.55767361111</v>
+        <v>46083.59739583333</v>
       </c>
       <c r="O352" t="inlineStr">
         <is>
@@ -23100,7 +23087,7 @@
         <v>1</v>
       </c>
       <c r="N354" s="3" t="n">
-        <v>46083.55420138889</v>
+        <v>46083.59190972222</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -23164,7 +23151,7 @@
         <v>1</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46083.55403935185</v>
+        <v>46083.59245370371</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23228,7 +23215,7 @@
         <v>1</v>
       </c>
       <c r="N356" s="3" t="n">
-        <v>46083.55674768519</v>
+        <v>46083.59840277778</v>
       </c>
       <c r="O356" t="inlineStr">
         <is>
@@ -23351,7 +23338,7 @@
         <v>2</v>
       </c>
       <c r="N358" s="3" t="n">
-        <v>46083.55814814815</v>
+        <v>46083.59804398148</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -23415,7 +23402,7 @@
         <v>2</v>
       </c>
       <c r="N359" s="3" t="n">
-        <v>46083.56371527778</v>
+        <v>46083.60714120371</v>
       </c>
       <c r="O359" t="inlineStr">
         <is>
@@ -23479,7 +23466,7 @@
         <v>1</v>
       </c>
       <c r="N360" s="3" t="n">
-        <v>46083.56481481482</v>
+        <v>46083.60237268519</v>
       </c>
       <c r="O360" t="inlineStr">
         <is>
@@ -23728,7 +23715,7 @@
         <v>1</v>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46083.57113425926</v>
+        <v>46083.64332175926</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23794,7 +23781,7 @@
         </is>
       </c>
       <c r="N365" s="3" t="n">
-        <v>46083.53606481481</v>
+        <v>46083.65340277777</v>
       </c>
       <c r="O365" t="inlineStr">
         <is>
@@ -23920,7 +23907,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46083.55055555556</v>
+        <v>46083.62974537037</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -23986,7 +23973,7 @@
         </is>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46083.56675925926</v>
+        <v>46083.64145833333</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24055,7 +24042,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46083.56980324074</v>
+        <v>46083.64633101852</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24124,7 +24111,7 @@
         <v>1</v>
       </c>
       <c r="N370" s="3" t="n">
-        <v>46083.56604166667</v>
+        <v>46083.64136574074</v>
       </c>
       <c r="O370" t="inlineStr">
         <is>
@@ -24262,7 +24249,7 @@
         <v>1</v>
       </c>
       <c r="N372" s="3" t="n">
-        <v>46083.53954861111</v>
+        <v>46083.58019675926</v>
       </c>
       <c r="O372" t="inlineStr">
         <is>
@@ -24331,7 +24318,7 @@
         <v>1</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46083.54190972223</v>
+        <v>46083.62460648148</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24397,7 +24384,7 @@
         </is>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46083.54856481482</v>
+        <v>46083.62207175926</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24416,6 +24403,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>10.69.3.72</t>
+        </is>
+      </c>
       <c r="D375" t="n">
         <v>2025</v>
       </c>
@@ -24461,7 +24453,7 @@
         <v>1</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46083.53305555556</v>
+        <v>46083.65024305556</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24530,7 +24522,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46083.55510416667</v>
+        <v>46083.63119212963</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -24599,7 +24591,7 @@
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46083.53444444444</v>
+        <v>46083.65084490741</v>
       </c>
       <c r="O377" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-02 17:52:05.024523
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46083.64827546296</v>
+        <v>46083.72732638889</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46083.62157407407</v>
+        <v>46083.69627314815</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>1</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46083.63289351852</v>
+        <v>46083.71427083333</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46083.64274305556</v>
+        <v>46083.72459490741</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
         <v>1</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>46083.64268518519</v>
+        <v>46083.71815972222</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1382,7 +1382,7 @@
         <v>2</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>46083.62454861111</v>
+        <v>46083.70063657407</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46083.62681712963</v>
+        <v>46083.70901620371</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1510,7 +1510,7 @@
         <v>2</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>46083.62244212963</v>
+        <v>46083.70163194444</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46083.63726851852</v>
+        <v>46083.71019675926</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46083.63482638889</v>
+        <v>46083.70993055555</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1763,7 +1763,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46083.62328703704</v>
+        <v>46083.70271990741</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1827,7 +1827,7 @@
         <v>1</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>46083.63702546297</v>
+        <v>46083.67512731482</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -1945,7 +1945,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46083.62525462963</v>
+        <v>46083.70532407407</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2004,7 +2004,7 @@
         <v>1</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>46083.62354166667</v>
+        <v>46083.70152777778</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2060,7 +2060,7 @@
         </is>
       </c>
       <c r="N25" s="3" t="n">
-        <v>46083.60783564814</v>
+        <v>46083.70596064815</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2138,6 +2138,11 @@
           <t>AUDITORIO</t>
         </is>
       </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>10.69.3.151</t>
+        </is>
+      </c>
       <c r="D27" t="n">
         <v>2019</v>
       </c>
@@ -2178,7 +2183,7 @@
         <v>1</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46083.60547453703</v>
+        <v>46083.72892361111</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2239,7 +2244,7 @@
         </is>
       </c>
       <c r="N28" s="3" t="n">
-        <v>46083.65369212963</v>
+        <v>46083.7340625</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -6565,7 +6570,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46083.61366898148</v>
+        <v>46083.69085648148</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6634,7 +6639,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46083.62834490741</v>
+        <v>46083.7112037037</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6698,7 +6703,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46083.63606481482</v>
+        <v>46083.70965277778</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6762,7 +6767,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46083.64167824074</v>
+        <v>46083.67771990741</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6831,7 +6836,7 @@
         <v>1</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46083.63601851852</v>
+        <v>46083.71034722222</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6900,7 +6905,7 @@
         <v>2</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46083.62866898148</v>
+        <v>46083.70572916666</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6969,7 +6974,7 @@
         <v>1</v>
       </c>
       <c r="N101" s="3" t="n">
-        <v>46083.63912037037</v>
+        <v>46083.71619212963</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -7107,7 +7112,7 @@
         <v>2</v>
       </c>
       <c r="N103" s="3" t="n">
-        <v>46083.61645833333</v>
+        <v>46083.7353125</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -7364,7 +7369,7 @@
         <v>1</v>
       </c>
       <c r="N107" s="3" t="n">
-        <v>46083.64925925926</v>
+        <v>46083.68545138889</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -7502,7 +7507,7 @@
         <v>1</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46083.62241898148</v>
+        <v>46083.69700231482</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7571,7 +7576,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46083.62952546297</v>
+        <v>46083.71101851852</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7640,7 +7645,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46083.64917824074</v>
+        <v>46083.72892361111</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7709,7 +7714,7 @@
         <v>2</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46083.64027777778</v>
+        <v>46083.72168981482</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7778,7 +7783,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46083.63564814815</v>
+        <v>46083.71619212963</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7847,7 +7852,7 @@
         <v>1</v>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46083.6409375</v>
+        <v>46083.71591435185</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7913,7 +7918,7 @@
         </is>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46083.65079861111</v>
+        <v>46083.69258101852</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7982,7 +7987,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46083.62996527777</v>
+        <v>46083.70832175926</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8046,7 +8051,7 @@
         <v>1</v>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46083.63543981482</v>
+        <v>46083.67403935185</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8112,7 +8117,7 @@
         </is>
       </c>
       <c r="N118" s="3" t="n">
-        <v>46083.64563657407</v>
+        <v>46083.68240740741</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -8250,7 +8255,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46083.62815972222</v>
+        <v>46083.66435185185</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8319,7 +8324,7 @@
         <v>1</v>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46083.654375</v>
+        <v>46083.73399305555</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8385,7 +8390,7 @@
         </is>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46083.63017361111</v>
+        <v>46083.71195601852</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8454,7 +8459,7 @@
         <v>2</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46083.62113425926</v>
+        <v>46083.70278935185</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8523,7 +8528,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46083.63208333333</v>
+        <v>46083.71390046296</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8592,7 +8597,7 @@
         <v>1</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46083.62645833333</v>
+        <v>46083.70766203704</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8661,7 +8666,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46083.65130787037</v>
+        <v>46083.72841435186</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8730,7 +8735,7 @@
         <v>2</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46083.62311342593</v>
+        <v>46083.73427083333</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8799,7 +8804,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46083.6321875</v>
+        <v>46083.70872685185</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -9001,7 +9006,7 @@
         <v>1</v>
       </c>
       <c r="N131" s="3" t="n">
-        <v>46083.64822916667</v>
+        <v>46083.68626157408</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -9134,7 +9139,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46083.62354166667</v>
+        <v>46083.7340625</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9198,7 +9203,7 @@
         <v>1</v>
       </c>
       <c r="N134" s="3" t="n">
-        <v>46083.61991898148</v>
+        <v>46083.72700231482</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -9262,7 +9267,7 @@
         <v>1</v>
       </c>
       <c r="N135" s="3" t="n">
-        <v>46083.63270833333</v>
+        <v>46083.72935185185</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -9453,7 +9458,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46083.62744212963</v>
+        <v>46083.70478009259</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9517,7 +9522,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46083.61802083333</v>
+        <v>46083.73574074074</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9581,7 +9586,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46083.61818287037</v>
+        <v>46083.73584490741</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9645,7 +9650,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46083.64263888889</v>
+        <v>46083.71518518519</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9709,7 +9714,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46083.63454861111</v>
+        <v>46083.71234953704</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9773,7 +9778,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46083.63127314814</v>
+        <v>46083.70833333334</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9837,7 +9842,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46083.63987268518</v>
+        <v>46083.71268518519</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9901,7 +9906,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46083.6515625</v>
+        <v>46083.72685185185</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9965,7 +9970,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46083.61875</v>
+        <v>46083.72446759259</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10029,7 +10034,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46083.63528935185</v>
+        <v>46083.71918981482</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10093,7 +10098,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46083.64747685185</v>
+        <v>46083.72412037037</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10157,7 +10162,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46083.64253472222</v>
+        <v>46083.71575231481</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10221,7 +10226,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46083.62334490741</v>
+        <v>46083.69945601852</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10285,7 +10290,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46083.61993055556</v>
+        <v>46083.73417824074</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10349,7 +10354,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46083.63221064815</v>
+        <v>46083.70527777778</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10368,11 +10373,6 @@
           <t>OPERACAO 7.1</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>10.69.5.21</t>
-        </is>
-      </c>
       <c r="D153" t="n">
         <v>2018</v>
       </c>
@@ -10413,7 +10413,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46083.64587962963</v>
+        <v>46083.72038194445</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10477,7 +10477,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46083.58376157407</v>
+        <v>46083.69789351852</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10541,7 +10541,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46083.64994212963</v>
+        <v>46083.73212962963</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10605,7 +10605,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46083.63701388889</v>
+        <v>46083.7078125</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10669,7 +10669,7 @@
         <v>1</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>46083.64099537037</v>
+        <v>46083.72836805556</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -10733,7 +10733,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46083.64461805556</v>
+        <v>46083.68221064815</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10797,7 +10797,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46083.64075231482</v>
+        <v>46083.71767361111</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10861,7 +10861,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46083.62144675926</v>
+        <v>46083.73636574074</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10925,7 +10925,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46083.6215162037</v>
+        <v>46083.72542824074</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -10989,7 +10989,7 @@
         <v>1</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46083.61887731482</v>
+        <v>46083.72547453704</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11117,7 +11117,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46083.64513888889</v>
+        <v>46083.72313657407</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11178,10 +11178,10 @@
         </is>
       </c>
       <c r="M165" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46083.5490162037</v>
+        <v>46083.70201388889</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11437,7 +11437,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46083.65333333334</v>
+        <v>46083.73318287037</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11629,7 +11629,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46083.6434375</v>
+        <v>46083.71983796296</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11693,7 +11693,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46083.6396875</v>
+        <v>46083.72195601852</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11821,7 +11821,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46083.61597222222</v>
+        <v>46083.73246527778</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11949,7 +11949,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46083.61659722222</v>
+        <v>46083.70140046296</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12013,7 +12013,7 @@
         <v>2</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46083.63509259259</v>
+        <v>46083.71114583333</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12077,7 +12077,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46083.63703703704</v>
+        <v>46083.72620370371</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12141,7 +12141,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46083.62166666667</v>
+        <v>46083.73425925926</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12205,7 +12205,7 @@
         <v>1</v>
       </c>
       <c r="N181" s="3" t="n">
-        <v>46083.62457175926</v>
+        <v>46083.72331018518</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
@@ -12402,7 +12402,7 @@
         <v>2</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46083.61615740741</v>
+        <v>46083.73196759259</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12594,7 +12594,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46083.64149305555</v>
+        <v>46083.72077546296</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12786,7 +12786,7 @@
         </is>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46083.62052083333</v>
+        <v>46083.72383101852</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12850,7 +12850,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46083.64626157407</v>
+        <v>46083.72721064815</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12914,7 +12914,7 @@
         <v>1</v>
       </c>
       <c r="N192" s="3" t="n">
-        <v>46083.61987268519</v>
+        <v>46083.73101851852</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
@@ -13103,7 +13103,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46083.64942129629</v>
+        <v>46083.72282407407</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13167,7 +13167,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46083.62318287037</v>
+        <v>46083.70224537037</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13231,7 +13231,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46083.62760416666</v>
+        <v>46083.70525462963</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13295,7 +13295,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46083.63877314814</v>
+        <v>46083.72038194445</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13359,7 +13359,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46083.6241087963</v>
+        <v>46083.70072916667</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13423,7 +13423,7 @@
         <v>1</v>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46083.62644675926</v>
+        <v>46083.70248842592</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13548,7 +13548,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46083.64743055555</v>
+        <v>46083.72349537037</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13612,7 +13612,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46083.62196759259</v>
+        <v>46083.73070601852</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13740,7 +13740,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46083.61678240741</v>
+        <v>46083.73490740741</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13804,7 +13804,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46083.61844907407</v>
+        <v>46083.73002314815</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13868,7 +13868,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46083.62094907407</v>
+        <v>46083.73537037037</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13932,7 +13932,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46083.64297453704</v>
+        <v>46083.73013888889</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -13996,7 +13996,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46083.62043981482</v>
+        <v>46083.73083333333</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14060,7 +14060,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46083.64709490741</v>
+        <v>46083.72045138889</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14124,7 +14124,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46083.61787037037</v>
+        <v>46083.73247685185</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14188,7 +14188,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46083.63204861111</v>
+        <v>46083.70912037037</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14252,7 +14252,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46083.640625</v>
+        <v>46083.71547453704</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14316,7 +14316,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46083.65145833333</v>
+        <v>46083.72814814815</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14380,7 +14380,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46083.64803240741</v>
+        <v>46083.72371527777</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14444,7 +14444,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46083.641875</v>
+        <v>46083.71353009259</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14463,6 +14463,11 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>10.69.5.85</t>
+        </is>
+      </c>
       <c r="D217" t="n">
         <v>2017</v>
       </c>
@@ -14503,7 +14508,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46083.61790509259</v>
+        <v>46083.73123842593</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14567,7 +14572,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46083.65231481481</v>
+        <v>46083.72677083333</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14631,7 +14636,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46083.62159722222</v>
+        <v>46083.73140046297</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14700,7 +14705,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46083.615</v>
+        <v>46083.73631944445</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14764,7 +14769,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46083.63358796296</v>
+        <v>46083.72114583333</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14828,7 +14833,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46083.61747685185</v>
+        <v>46083.73515046296</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14892,7 +14897,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46083.64677083334</v>
+        <v>46083.72702546296</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14956,7 +14961,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46083.64513888889</v>
+        <v>46083.70412037037</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15020,7 +15025,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46083.63241898148</v>
+        <v>46083.72814814815</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15148,7 +15153,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46083.63047453704</v>
+        <v>46083.71026620371</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15212,7 +15217,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46083.64711805555</v>
+        <v>46083.72424768518</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15276,7 +15281,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46083.62565972222</v>
+        <v>46083.70344907408</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15340,7 +15345,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46083.62673611111</v>
+        <v>46083.70901620371</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15404,7 +15409,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46083.62876157407</v>
+        <v>46083.72927083333</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15468,7 +15473,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46083.63350694445</v>
+        <v>46083.71130787037</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15532,7 +15537,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46083.64798611111</v>
+        <v>46083.72125</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15596,7 +15601,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46083.62177083334</v>
+        <v>46083.7331712963</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15660,7 +15665,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46083.62956018518</v>
+        <v>46083.70847222222</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15724,7 +15729,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46083.636875</v>
+        <v>46083.70976851852</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15788,7 +15793,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46083.63344907408</v>
+        <v>46083.70553240741</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15852,7 +15857,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46083.63061342593</v>
+        <v>46083.70834490741</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15916,7 +15921,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46083.62972222222</v>
+        <v>46083.70423611111</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -15980,7 +15985,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46083.62248842593</v>
+        <v>46083.72622685185</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16044,7 +16049,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46083.61961805556</v>
+        <v>46083.73260416667</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16108,7 +16113,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46083.64872685185</v>
+        <v>46083.72909722223</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16172,7 +16177,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46083.62876157407</v>
+        <v>46083.70425925926</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16191,11 +16196,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C244" t="inlineStr">
-        <is>
-          <t>10.69.5.112</t>
-        </is>
-      </c>
       <c r="D244" t="n">
         <v>2019</v>
       </c>
@@ -16236,7 +16236,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46083.65153935185</v>
+        <v>46083.72125</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16300,7 +16300,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46083.64868055555</v>
+        <v>46083.72638888889</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16364,7 +16364,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46083.63427083333</v>
+        <v>46083.71601851852</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16428,7 +16428,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46083.64726851852</v>
+        <v>46083.71434027778</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16492,7 +16492,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46083.63898148148</v>
+        <v>46083.70130787037</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16556,7 +16556,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46083.63420138889</v>
+        <v>46083.72697916667</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16684,7 +16684,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46083.64758101852</v>
+        <v>46083.72222222222</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16748,7 +16748,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46083.61979166666</v>
+        <v>46083.72765046296</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16812,7 +16812,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46083.62361111111</v>
+        <v>46083.70789351852</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16870,7 +16870,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46083.63630787037</v>
+        <v>46083.72357638889</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16934,7 +16934,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46083.63878472222</v>
+        <v>46083.71126157408</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -16998,7 +16998,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46083.62771990741</v>
+        <v>46083.72777777778</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17062,7 +17062,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46083.63990740741</v>
+        <v>46083.71354166666</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17126,7 +17126,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46083.62386574074</v>
+        <v>46083.72344907407</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17318,7 +17318,7 @@
         <v>2</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46083.62707175926</v>
+        <v>46083.70436342592</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17382,7 +17382,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46083.62451388889</v>
+        <v>46083.72855324074</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17446,7 +17446,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46083.63410879629</v>
+        <v>46083.70768518518</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17510,7 +17510,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46083.64269675926</v>
+        <v>46083.71542824074</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17574,7 +17574,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46083.64045138889</v>
+        <v>46083.71708333334</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17638,7 +17638,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46083.63592592593</v>
+        <v>46083.73424768518</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17702,7 +17702,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46083.64336805556</v>
+        <v>46083.71803240741</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17730,7 +17730,7 @@
         <v>2</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46083.62393518518</v>
+        <v>46083.69875</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17794,7 +17794,7 @@
         <v>1</v>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46083.64204861111</v>
+        <v>46083.70810185185</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17855,7 +17855,7 @@
         </is>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46083.65295138889</v>
+        <v>46083.72770833333</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -17919,7 +17919,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46083.56170138889</v>
+        <v>46083.66699074074</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -18047,7 +18047,7 @@
         <v>1</v>
       </c>
       <c r="N273" s="3" t="n">
-        <v>46083.6438425926</v>
+        <v>46083.71763888889</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -18068,23 +18068,23 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>10.69.5.143</t>
+          <t>10.69.5.147</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>2016</v>
+        <v>2012</v>
       </c>
       <c r="E274" t="n">
-        <v>43374</v>
+        <v>2956</v>
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>Microsoft Windows 7 Professional</t>
+          <t>Microsoft® Windows Vista™ Business</t>
         </is>
       </c>
       <c r="G274" t="inlineStr">
         <is>
-          <t>BRG132F1WZ</t>
+          <t>B2XQXG1</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
@@ -18099,19 +18099,16 @@
       </c>
       <c r="K274" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Dell Inc.</t>
         </is>
       </c>
       <c r="L274" t="inlineStr">
         <is>
-          <t>COMPAQ 300B MT</t>
-        </is>
-      </c>
-      <c r="M274" t="n">
-        <v>1</v>
+          <t>OptiPlex 755</t>
+        </is>
       </c>
       <c r="N274" s="3" t="n">
-        <v>46032.86671296296</v>
+        <v>46083.67244212963</v>
       </c>
       <c r="O274" t="inlineStr">
         <is>
@@ -18261,19 +18258,19 @@
         </is>
       </c>
       <c r="D277" t="n">
-        <v>2012</v>
+        <v>2016</v>
       </c>
       <c r="E277" t="n">
-        <v>2956</v>
+        <v>43374</v>
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>Microsoft® Windows Vista™ Business</t>
+          <t>Microsoft Windows 7 Professional</t>
         </is>
       </c>
       <c r="G277" t="inlineStr">
         <is>
-          <t>B2XQXG1</t>
+          <t>BRG132F1WZ</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
@@ -18288,19 +18285,19 @@
       </c>
       <c r="K277" t="inlineStr">
         <is>
-          <t>Dell Inc.</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="L277" t="inlineStr">
         <is>
-          <t>OptiPlex 755</t>
+          <t>COMPAQ 300B MT</t>
         </is>
       </c>
       <c r="M277" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46083.58732638889</v>
+        <v>46083.72848379629</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18364,7 +18361,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46083.63924768518</v>
+        <v>46083.72231481481</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18492,7 +18489,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46083.61954861111</v>
+        <v>46083.73494212963</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18615,7 +18612,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46083.63380787037</v>
+        <v>46083.70991898148</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18679,7 +18676,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46083.6196875</v>
+        <v>46083.72295138889</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18743,7 +18740,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46083.65054398148</v>
+        <v>46083.72576388889</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18866,7 +18863,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46083.614375</v>
+        <v>46083.65564814815</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18994,7 +18991,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46083.63113425926</v>
+        <v>46083.70315972222</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19788,7 +19785,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46083.61678240741</v>
+        <v>46083.73559027778</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20904,7 +20901,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46083.6359375</v>
+        <v>46083.71268518519</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21629,7 +21626,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46083.63071759259</v>
+        <v>46083.70618055556</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21693,7 +21690,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46083.62244212963</v>
+        <v>46083.73686342593</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21757,7 +21754,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46083.63053240741</v>
+        <v>46083.70586805556</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21821,7 +21818,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46083.63127314814</v>
+        <v>46083.7130787037</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21885,7 +21882,7 @@
         <v>1</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46083.64622685185</v>
+        <v>46083.68388888889</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21949,7 +21946,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46083.61630787037</v>
+        <v>46083.72972222222</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22013,7 +22010,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46083.63027777777</v>
+        <v>46083.70523148148</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22077,7 +22074,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46083.61820601852</v>
+        <v>46083.69986111111</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -23715,7 +23712,7 @@
         <v>1</v>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46083.64332175926</v>
+        <v>46083.71135416667</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23781,7 +23778,7 @@
         </is>
       </c>
       <c r="N365" s="3" t="n">
-        <v>46083.65340277777</v>
+        <v>46083.73180555556</v>
       </c>
       <c r="O365" t="inlineStr">
         <is>
@@ -23907,7 +23904,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46083.62974537037</v>
+        <v>46083.70922453704</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -23973,7 +23970,7 @@
         </is>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46083.64145833333</v>
+        <v>46083.67690972222</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24042,7 +24039,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46083.64633101852</v>
+        <v>46083.72453703704</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24111,7 +24108,7 @@
         <v>1</v>
       </c>
       <c r="N370" s="3" t="n">
-        <v>46083.64136574074</v>
+        <v>46083.67902777778</v>
       </c>
       <c r="O370" t="inlineStr">
         <is>
@@ -24318,7 +24315,7 @@
         <v>1</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46083.62460648148</v>
+        <v>46083.70039351852</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24384,7 +24381,7 @@
         </is>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46083.62207175926</v>
+        <v>46083.70434027778</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24453,7 +24450,7 @@
         <v>1</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46083.65024305556</v>
+        <v>46083.73392361111</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24522,7 +24519,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46083.63119212963</v>
+        <v>46083.70908564814</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -24591,7 +24588,7 @@
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46083.65084490741</v>
+        <v>46083.72869212963</v>
       </c>
       <c r="O377" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-03 07:52:03.753723
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46083.72732638889</v>
+        <v>46084.30418981481</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46083.69627314815</v>
+        <v>46084.28547453704</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46083.72459490741</v>
+        <v>46084.30827546296</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1382,7 +1382,7 @@
         <v>2</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>46083.70063657407</v>
+        <v>46083.73962962963</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46083.70901620371</v>
+        <v>46084.31751157407</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1510,7 +1510,7 @@
         <v>2</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>46083.70163194444</v>
+        <v>46084.29590277778</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46083.71019675926</v>
+        <v>46084.28484953703</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46083.70993055555</v>
+        <v>46083.7947337963</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1763,7 +1763,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46083.70271990741</v>
+        <v>46084.31332175926</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1945,7 +1945,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46083.70532407407</v>
+        <v>46084.10149305555</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2004,7 +2004,7 @@
         <v>1</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>46083.70152777778</v>
+        <v>46084.10829861111</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2060,7 +2060,7 @@
         </is>
       </c>
       <c r="N25" s="3" t="n">
-        <v>46083.70596064815</v>
+        <v>46084.18665509259</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2138,11 +2138,6 @@
           <t>AUDITORIO</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>10.69.3.151</t>
-        </is>
-      </c>
       <c r="D27" t="n">
         <v>2019</v>
       </c>
@@ -2183,7 +2178,7 @@
         <v>1</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46083.72892361111</v>
+        <v>46084.14333333333</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6639,7 +6634,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46083.7112037037</v>
+        <v>46083.83415509259</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6836,7 +6831,7 @@
         <v>1</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46083.71034722222</v>
+        <v>46083.74866898148</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6905,7 +6900,7 @@
         <v>2</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46083.70572916666</v>
+        <v>46084.28646990741</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6974,7 +6969,7 @@
         <v>1</v>
       </c>
       <c r="N101" s="3" t="n">
-        <v>46083.71619212963</v>
+        <v>46084.29193287037</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -7112,7 +7107,7 @@
         <v>2</v>
       </c>
       <c r="N103" s="3" t="n">
-        <v>46083.7353125</v>
+        <v>46083.81203703704</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -7507,7 +7502,7 @@
         <v>1</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46083.69700231482</v>
+        <v>46084.29267361111</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7576,7 +7571,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46083.71101851852</v>
+        <v>46084.29212962963</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7645,7 +7640,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46083.72892361111</v>
+        <v>46083.7694675926</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7714,7 +7709,7 @@
         <v>2</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46083.72168981482</v>
+        <v>46084.30996527777</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7783,7 +7778,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46083.71619212963</v>
+        <v>46084.29958333333</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7852,7 +7847,7 @@
         <v>1</v>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46083.71591435185</v>
+        <v>46084.30059027778</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -8006,6 +8001,11 @@
           <t>DP</t>
         </is>
       </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>10.69.3.23</t>
+        </is>
+      </c>
       <c r="D117" t="n">
         <v>2025</v>
       </c>
@@ -8051,7 +8051,7 @@
         <v>1</v>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46083.67403935185</v>
+        <v>46084.31523148148</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8255,7 +8255,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46083.66435185185</v>
+        <v>46084.30854166667</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8324,7 +8324,7 @@
         <v>1</v>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46083.73399305555</v>
+        <v>46083.8484375</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8459,7 +8459,7 @@
         <v>2</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46083.70278935185</v>
+        <v>46084.28221064815</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8528,7 +8528,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46083.71390046296</v>
+        <v>46084.31199074074</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8597,7 +8597,7 @@
         <v>1</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46083.70766203704</v>
+        <v>46084.29881944445</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8666,7 +8666,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46083.72841435186</v>
+        <v>46083.76520833333</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8735,7 +8735,7 @@
         <v>2</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46083.73427083333</v>
+        <v>46084.2930324074</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -9139,7 +9139,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46083.7340625</v>
+        <v>46083.8080787037</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9203,7 +9203,7 @@
         <v>1</v>
       </c>
       <c r="N134" s="3" t="n">
-        <v>46083.72700231482</v>
+        <v>46083.80149305556</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -9267,7 +9267,7 @@
         <v>1</v>
       </c>
       <c r="N135" s="3" t="n">
-        <v>46083.72935185185</v>
+        <v>46083.8014699074</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -9458,7 +9458,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46083.70478009259</v>
+        <v>46083.81773148148</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9522,7 +9522,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46083.73574074074</v>
+        <v>46083.81221064815</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9586,7 +9586,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46083.73584490741</v>
+        <v>46083.81528935185</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9650,7 +9650,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46083.71518518519</v>
+        <v>46083.82701388889</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9714,7 +9714,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46083.71234953704</v>
+        <v>46083.79152777778</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9778,7 +9778,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46083.70833333334</v>
+        <v>46083.82107638889</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9842,7 +9842,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46083.71268518519</v>
+        <v>46083.78980324074</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9906,7 +9906,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46083.72685185185</v>
+        <v>46083.84038194444</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9970,7 +9970,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46083.72446759259</v>
+        <v>46083.80175925926</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10034,7 +10034,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46083.71918981482</v>
+        <v>46083.79483796296</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10098,7 +10098,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46083.72412037037</v>
+        <v>46083.79743055555</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10162,7 +10162,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46083.71575231481</v>
+        <v>46083.86951388889</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10226,7 +10226,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46083.69945601852</v>
+        <v>46083.81940972222</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10290,7 +10290,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46083.73417824074</v>
+        <v>46083.81020833334</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10354,7 +10354,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46083.70527777778</v>
+        <v>46083.8221412037</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10373,6 +10373,11 @@
           <t>OPERACAO 7.1</t>
         </is>
       </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>10.69.5.21</t>
+        </is>
+      </c>
       <c r="D153" t="n">
         <v>2018</v>
       </c>
@@ -10413,7 +10418,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46083.72038194445</v>
+        <v>46084.31927083333</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10477,7 +10482,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46083.69789351852</v>
+        <v>46083.82023148148</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10541,7 +10546,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46083.73212962963</v>
+        <v>46083.80534722222</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10605,7 +10610,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46083.7078125</v>
+        <v>46083.82736111111</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10669,7 +10674,7 @@
         <v>1</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>46083.72836805556</v>
+        <v>46083.80753472223</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -10797,7 +10802,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46083.71767361111</v>
+        <v>46083.87065972222</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10861,7 +10866,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46083.73636574074</v>
+        <v>46084.31010416667</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10925,7 +10930,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46083.72542824074</v>
+        <v>46084.3068287037</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -10989,7 +10994,7 @@
         <v>1</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46083.72547453704</v>
+        <v>46083.80217592593</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11114,10 +11119,10 @@
         </is>
       </c>
       <c r="M164" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46083.72313657407</v>
+        <v>46084.29053240741</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11181,7 +11186,7 @@
         <v>1</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46083.70201388889</v>
+        <v>46084.28898148148</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11373,7 +11378,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46083.56975694445</v>
+        <v>46084.31366898148</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11434,10 +11439,10 @@
         </is>
       </c>
       <c r="M169" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46083.73318287037</v>
+        <v>46084.28637731481</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11629,7 +11634,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46083.71983796296</v>
+        <v>46083.77778935185</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11690,10 +11695,10 @@
         </is>
       </c>
       <c r="M173" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46083.72195601852</v>
+        <v>46084.29957175926</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11757,7 +11762,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46083.57162037037</v>
+        <v>46084.31548611111</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11821,7 +11826,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46083.73246527778</v>
+        <v>46084.29391203704</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11949,7 +11954,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46083.70140046296</v>
+        <v>46083.74231481482</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12013,7 +12018,7 @@
         <v>2</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46083.71114583333</v>
+        <v>46084.28680555556</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12077,7 +12082,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46083.72620370371</v>
+        <v>46083.80946759259</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12141,7 +12146,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46083.73425925926</v>
+        <v>46083.80761574074</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12205,7 +12210,7 @@
         <v>1</v>
       </c>
       <c r="N181" s="3" t="n">
-        <v>46083.72331018518</v>
+        <v>46083.80201388889</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
@@ -12402,7 +12407,7 @@
         <v>2</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46083.73196759259</v>
+        <v>46084.31738425926</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12530,7 +12535,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46083.60189814815</v>
+        <v>46084.22221064815</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12594,7 +12599,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46083.72077546296</v>
+        <v>46083.83796296296</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12786,7 +12791,7 @@
         </is>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46083.72383101852</v>
+        <v>46083.80347222222</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12850,7 +12855,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46083.72721064815</v>
+        <v>46083.79954861111</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12914,7 +12919,7 @@
         <v>1</v>
       </c>
       <c r="N192" s="3" t="n">
-        <v>46083.73101851852</v>
+        <v>46083.80466435185</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
@@ -13039,7 +13044,7 @@
         <v>2</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46083.62077546296</v>
+        <v>46084.2702199074</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13103,7 +13108,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46083.72282407407</v>
+        <v>46083.83723379629</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13167,7 +13172,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46083.70224537037</v>
+        <v>46083.82203703704</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13231,7 +13236,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46083.70525462963</v>
+        <v>46083.86458333334</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13295,7 +13300,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46083.72038194445</v>
+        <v>46083.84304398148</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13359,7 +13364,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46083.70072916667</v>
+        <v>46083.81674768519</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13423,7 +13428,7 @@
         <v>1</v>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46083.70248842592</v>
+        <v>46083.85864583333</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13548,7 +13553,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46083.72349537037</v>
+        <v>46083.8021875</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13612,7 +13617,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46083.73070601852</v>
+        <v>46083.80875</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13740,7 +13745,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46083.73490740741</v>
+        <v>46083.81480324074</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13804,7 +13809,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46083.73002314815</v>
+        <v>46083.80962962963</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13868,7 +13873,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46083.73537037037</v>
+        <v>46083.80962962963</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13932,7 +13937,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46083.73013888889</v>
+        <v>46083.80857638889</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -13996,7 +14001,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46083.73083333333</v>
+        <v>46083.80688657407</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14060,7 +14065,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46083.72045138889</v>
+        <v>46083.83802083333</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14124,7 +14129,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46083.73247685185</v>
+        <v>46084.32047453704</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14188,7 +14193,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46083.70912037037</v>
+        <v>46083.79277777778</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14252,7 +14257,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46083.71547453704</v>
+        <v>46083.87391203704</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14316,7 +14321,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46083.72814814815</v>
+        <v>46083.80144675926</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14380,7 +14385,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46083.72371527777</v>
+        <v>46083.79869212963</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14444,7 +14449,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46083.71353009259</v>
+        <v>46083.82762731481</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14463,11 +14468,6 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
-      <c r="C217" t="inlineStr">
-        <is>
-          <t>10.69.5.85</t>
-        </is>
-      </c>
       <c r="D217" t="n">
         <v>2017</v>
       </c>
@@ -14508,7 +14508,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46083.73123842593</v>
+        <v>46083.8052662037</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14572,7 +14572,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46083.72677083333</v>
+        <v>46084.30439814815</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14636,7 +14636,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46083.73140046297</v>
+        <v>46083.8080787037</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14705,7 +14705,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46083.73631944445</v>
+        <v>46083.85549768519</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14769,7 +14769,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46083.72114583333</v>
+        <v>46083.79398148148</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14833,7 +14833,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46083.73515046296</v>
+        <v>46083.81090277778</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14897,7 +14897,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46083.72702546296</v>
+        <v>46083.80289351852</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14961,7 +14961,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46083.70412037037</v>
+        <v>46083.82248842593</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15025,7 +15025,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46083.72814814815</v>
+        <v>46083.80341435185</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15153,7 +15153,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46083.71026620371</v>
+        <v>46083.82641203704</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15217,7 +15217,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46083.72424768518</v>
+        <v>46083.80224537037</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15281,7 +15281,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46083.70344907408</v>
+        <v>46083.81699074074</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15345,7 +15345,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46083.70901620371</v>
+        <v>46083.82431712963</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15409,7 +15409,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46083.72927083333</v>
+        <v>46083.81099537037</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15473,7 +15473,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46083.71130787037</v>
+        <v>46083.82859953704</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15537,7 +15537,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46083.72125</v>
+        <v>46084.3082175926</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15601,7 +15601,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46083.7331712963</v>
+        <v>46083.81302083333</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15665,7 +15665,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46083.70847222222</v>
+        <v>46083.79207175926</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15729,7 +15729,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46083.70976851852</v>
+        <v>46083.82371527778</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15793,7 +15793,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46083.70553240741</v>
+        <v>46083.82596064815</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15857,7 +15857,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46083.70834490741</v>
+        <v>46083.82121527778</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15921,7 +15921,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46083.70423611111</v>
+        <v>46083.82461805556</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -15985,7 +15985,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46083.72622685185</v>
+        <v>46083.80311342593</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16049,7 +16049,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46083.73260416667</v>
+        <v>46083.81465277778</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16113,7 +16113,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46083.72909722223</v>
+        <v>46083.80471064815</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16177,7 +16177,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46083.70425925926</v>
+        <v>46083.82346064815</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16196,6 +16196,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>10.69.5.112</t>
+        </is>
+      </c>
       <c r="D244" t="n">
         <v>2019</v>
       </c>
@@ -16236,7 +16241,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46083.72125</v>
+        <v>46084.22336805556</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16300,7 +16305,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46083.72638888889</v>
+        <v>46083.80362268518</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16364,7 +16369,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46083.71601851852</v>
+        <v>46083.79613425926</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16428,7 +16433,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46083.71434027778</v>
+        <v>46083.8490625</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16492,7 +16497,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46083.70130787037</v>
+        <v>46083.82275462963</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16556,7 +16561,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46083.72697916667</v>
+        <v>46083.79930555556</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16620,7 +16625,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46083.61032407408</v>
+        <v>46083.81512731482</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16684,7 +16689,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46083.72222222222</v>
+        <v>46083.79752314815</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16748,7 +16753,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46083.72765046296</v>
+        <v>46083.80550925926</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16812,7 +16817,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46083.70789351852</v>
+        <v>46083.82759259259</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16870,7 +16875,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46083.72357638889</v>
+        <v>46083.79585648148</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16934,7 +16939,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46083.71126157408</v>
+        <v>46084.30733796296</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -16998,7 +17003,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46083.72777777778</v>
+        <v>46083.80766203703</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17062,7 +17067,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46083.71354166666</v>
+        <v>46083.82917824074</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17126,7 +17131,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46083.72344907407</v>
+        <v>46083.80334490741</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17318,7 +17323,7 @@
         <v>2</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46083.70436342592</v>
+        <v>46083.81766203704</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17382,7 +17387,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46083.72855324074</v>
+        <v>46083.80528935185</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17446,7 +17451,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46083.70768518518</v>
+        <v>46084.31863425926</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17510,7 +17515,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46083.71542824074</v>
+        <v>46083.79763888889</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17574,7 +17579,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46083.71708333334</v>
+        <v>46083.7930787037</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17638,7 +17643,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46083.73424768518</v>
+        <v>46083.80930555556</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17702,7 +17707,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46083.71803240741</v>
+        <v>46083.79447916667</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17730,7 +17735,7 @@
         <v>2</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46083.69875</v>
+        <v>46083.7766087963</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17794,7 +17799,7 @@
         <v>1</v>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46083.70810185185</v>
+        <v>46083.82607638889</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17855,7 +17860,7 @@
         </is>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46083.72770833333</v>
+        <v>46084.31092592593</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -17919,7 +17924,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46083.66699074074</v>
+        <v>46084.30424768518</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -18047,7 +18052,7 @@
         <v>1</v>
       </c>
       <c r="N273" s="3" t="n">
-        <v>46083.71763888889</v>
+        <v>46083.86868055556</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -18294,10 +18299,10 @@
         </is>
       </c>
       <c r="M277" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46083.72848379629</v>
+        <v>46084.31946759259</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18361,7 +18366,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46083.72231481481</v>
+        <v>46084.29840277778</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18489,7 +18494,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46083.73494212963</v>
+        <v>46083.85100694445</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18612,7 +18617,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46083.70991898148</v>
+        <v>46083.82590277777</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18676,7 +18681,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46083.72295138889</v>
+        <v>46083.87239583334</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18740,7 +18745,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46083.72576388889</v>
+        <v>46083.80342592593</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18799,7 +18804,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46083.57696759259</v>
+        <v>46084.19300925926</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18863,7 +18868,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46083.65564814815</v>
+        <v>46084.24326388889</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18991,7 +18996,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46083.70315972222</v>
+        <v>46083.85875</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19785,7 +19790,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46083.73559027778</v>
+        <v>46084.31916666667</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20901,7 +20906,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46083.71268518519</v>
+        <v>46084.295</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21626,7 +21631,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46083.70618055556</v>
+        <v>46083.78344907407</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21690,7 +21695,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46083.73686342593</v>
+        <v>46084.2846412037</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21754,7 +21759,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46083.70586805556</v>
+        <v>46084.28498842593</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21818,7 +21823,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46083.7130787037</v>
+        <v>46084.28475694444</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21882,7 +21887,7 @@
         <v>1</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46083.68388888889</v>
+        <v>46084.28434027778</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21946,7 +21951,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46083.72972222222</v>
+        <v>46084.2852662037</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22010,7 +22015,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46083.70523148148</v>
+        <v>46083.78145833333</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22074,7 +22079,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46083.69986111111</v>
+        <v>46084.31541666666</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22266,7 +22271,7 @@
         <v>2</v>
       </c>
       <c r="N341" s="3" t="n">
-        <v>46083.56980324074</v>
+        <v>46084.29648148148</v>
       </c>
       <c r="O341" t="inlineStr">
         <is>
@@ -23778,7 +23783,7 @@
         </is>
       </c>
       <c r="N365" s="3" t="n">
-        <v>46083.73180555556</v>
+        <v>46084.30540509259</v>
       </c>
       <c r="O365" t="inlineStr">
         <is>
@@ -23923,11 +23928,6 @@
           <t>RH</t>
         </is>
       </c>
-      <c r="C368" t="inlineStr">
-        <is>
-          <t>10.69.3.13</t>
-        </is>
-      </c>
       <c r="D368" t="n">
         <v>2025</v>
       </c>
@@ -24039,7 +24039,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46083.72453703704</v>
+        <v>46084.30673611111</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24315,7 +24315,7 @@
         <v>1</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46083.70039351852</v>
+        <v>46083.74173611111</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24381,7 +24381,7 @@
         </is>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46083.70434027778</v>
+        <v>46084.31881944444</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24450,7 +24450,7 @@
         <v>1</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46083.73392361111</v>
+        <v>46083.81094907408</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24519,7 +24519,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46083.70908564814</v>
+        <v>46083.74791666667</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -24588,7 +24588,7 @@
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46083.72869212963</v>
+        <v>46084.30924768518</v>
       </c>
       <c r="O377" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-03 09:52:05.264454
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46084.30418981481</v>
+        <v>46084.38317129629</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46084.28547453704</v>
+        <v>46084.40255787037</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>1</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46083.71427083333</v>
+        <v>46084.40043981482</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46083.64351851852</v>
+        <v>46084.37159722222</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46084.30827546296</v>
+        <v>46084.3878587963</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46084.31751157407</v>
+        <v>46084.39876157408</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1510,7 +1510,7 @@
         <v>2</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>46084.29590277778</v>
+        <v>46084.37489583333</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46084.28484953703</v>
+        <v>46084.39865740741</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46083.7947337963</v>
+        <v>46084.40065972223</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1699,7 +1699,7 @@
         </is>
       </c>
       <c r="N19" s="3" t="n">
-        <v>45995.65027777778</v>
+        <v>46084.40447916667</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1763,7 +1763,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46084.31332175926</v>
+        <v>46084.39351851852</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -6565,7 +6565,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46083.69085648148</v>
+        <v>46084.39771990741</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6653,6 +6653,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>10.69.3.93</t>
+        </is>
+      </c>
       <c r="D97" t="n">
         <v>2025</v>
       </c>
@@ -6698,7 +6703,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46083.70965277778</v>
+        <v>46084.37287037037</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6762,7 +6767,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46083.67771990741</v>
+        <v>46084.36756944445</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6831,7 +6836,7 @@
         <v>1</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46083.74866898148</v>
+        <v>46084.37560185185</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6900,7 +6905,7 @@
         <v>2</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46084.28646990741</v>
+        <v>46084.40212962963</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6969,7 +6974,7 @@
         <v>1</v>
       </c>
       <c r="N101" s="3" t="n">
-        <v>46084.29193287037</v>
+        <v>46084.36840277778</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -7107,7 +7112,7 @@
         <v>2</v>
       </c>
       <c r="N103" s="3" t="n">
-        <v>46083.81203703704</v>
+        <v>46084.38550925926</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -7364,7 +7369,7 @@
         <v>1</v>
       </c>
       <c r="N107" s="3" t="n">
-        <v>46083.68545138889</v>
+        <v>46084.37907407407</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -7502,7 +7507,7 @@
         <v>1</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46084.29267361111</v>
+        <v>46084.3741087963</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7571,7 +7576,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46084.29212962963</v>
+        <v>46084.3712962963</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7640,7 +7645,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46083.7694675926</v>
+        <v>46084.36873842592</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7709,7 +7714,7 @@
         <v>2</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46084.30996527777</v>
+        <v>46084.39400462963</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7778,7 +7783,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46084.29958333333</v>
+        <v>46084.37175925926</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7847,7 +7852,7 @@
         <v>1</v>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46084.30059027778</v>
+        <v>46084.38185185185</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7913,7 +7918,7 @@
         </is>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46083.69258101852</v>
+        <v>46084.37668981482</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7982,7 +7987,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46083.70832175926</v>
+        <v>46084.4033912037</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8001,11 +8006,6 @@
           <t>DP</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>10.69.3.23</t>
-        </is>
-      </c>
       <c r="D117" t="n">
         <v>2025</v>
       </c>
@@ -8051,7 +8051,7 @@
         <v>1</v>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46084.31523148148</v>
+        <v>46084.39614583334</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8117,7 +8117,7 @@
         </is>
       </c>
       <c r="N118" s="3" t="n">
-        <v>46083.68240740741</v>
+        <v>46084.37339120371</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -8255,7 +8255,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46084.30854166667</v>
+        <v>46084.38349537037</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8324,7 +8324,7 @@
         <v>1</v>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46083.8484375</v>
+        <v>46084.39947916667</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8390,7 +8390,7 @@
         </is>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46083.71195601852</v>
+        <v>46084.39674768518</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8528,7 +8528,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46084.31199074074</v>
+        <v>46084.39277777778</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8597,7 +8597,7 @@
         <v>1</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46084.29881944445</v>
+        <v>46084.37782407407</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8666,7 +8666,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46083.76520833333</v>
+        <v>46084.36984953703</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8735,7 +8735,7 @@
         <v>2</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46084.2930324074</v>
+        <v>46084.36975694444</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8804,7 +8804,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46083.70872685185</v>
+        <v>46084.39956018519</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8905,7 +8905,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Microsoft Windows 11 Pro</t>
+          <t>Windows</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -8942,7 +8942,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46083.64935185185</v>
+        <v>46084.36686342592</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9006,7 +9006,7 @@
         <v>1</v>
       </c>
       <c r="N131" s="3" t="n">
-        <v>46083.68626157408</v>
+        <v>46084.37074074074</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -9139,7 +9139,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46083.8080787037</v>
+        <v>46084.37824074074</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9458,7 +9458,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46083.81773148148</v>
+        <v>46084.37166666667</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9586,7 +9586,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46083.81528935185</v>
+        <v>46084.39728009259</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9650,7 +9650,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46083.82701388889</v>
+        <v>46084.37081018519</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9714,7 +9714,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46083.79152777778</v>
+        <v>46084.39696759259</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9778,7 +9778,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46083.82107638889</v>
+        <v>46084.36958333333</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9842,7 +9842,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46083.78980324074</v>
+        <v>46084.38451388889</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9906,7 +9906,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46083.84038194444</v>
+        <v>46084.395</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9970,7 +9970,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46083.80175925926</v>
+        <v>46084.37546296296</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10034,7 +10034,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46083.79483796296</v>
+        <v>46084.37552083333</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10098,7 +10098,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46083.79743055555</v>
+        <v>46084.38929398148</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10162,7 +10162,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46083.86951388889</v>
+        <v>46084.37179398148</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10226,7 +10226,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46083.81940972222</v>
+        <v>46084.38063657407</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10290,7 +10290,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46083.81020833334</v>
+        <v>46084.38135416667</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10354,7 +10354,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46083.8221412037</v>
+        <v>46084.38663194444</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10418,7 +10418,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46084.31927083333</v>
+        <v>46084.39915509259</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10482,7 +10482,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46083.82023148148</v>
+        <v>46084.4025462963</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10546,7 +10546,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46083.80534722222</v>
+        <v>46084.38120370371</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10610,7 +10610,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46083.82736111111</v>
+        <v>46084.39774305555</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10674,7 +10674,7 @@
         <v>1</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>46083.80753472223</v>
+        <v>46084.37331018518</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -10738,7 +10738,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46083.68221064815</v>
+        <v>46084.37494212963</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10802,7 +10802,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46083.87065972222</v>
+        <v>46084.37290509259</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10866,7 +10866,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46084.31010416667</v>
+        <v>46084.38173611111</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10930,7 +10930,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46084.3068287037</v>
+        <v>46084.38173611111</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -10994,7 +10994,7 @@
         <v>1</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46083.80217592593</v>
+        <v>46084.3782175926</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11119,10 +11119,10 @@
         </is>
       </c>
       <c r="M164" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46084.29053240741</v>
+        <v>46084.37386574074</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11183,10 +11183,10 @@
         </is>
       </c>
       <c r="M165" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46084.28898148148</v>
+        <v>46084.36765046296</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11250,7 +11250,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46083.60706018518</v>
+        <v>46084.39689814814</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11314,7 +11314,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46083.59142361111</v>
+        <v>46084.39369212963</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11378,7 +11378,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46084.31366898148</v>
+        <v>46084.39269675926</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11439,10 +11439,10 @@
         </is>
       </c>
       <c r="M169" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46084.28637731481</v>
+        <v>46084.36775462963</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11506,7 +11506,7 @@
         <v>2</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46083.4787037037</v>
+        <v>46084.39980324074</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11567,10 +11567,10 @@
         </is>
       </c>
       <c r="M171" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46083.54717592592</v>
+        <v>46084.40417824074</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11698,7 +11698,7 @@
         <v>1</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46084.29957175926</v>
+        <v>46084.39270833333</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11762,7 +11762,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46084.31548611111</v>
+        <v>46084.39280092593</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11826,7 +11826,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46084.29391203704</v>
+        <v>46084.37349537037</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -12018,7 +12018,7 @@
         <v>2</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46084.28680555556</v>
+        <v>46084.36739583333</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12082,7 +12082,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46083.80946759259</v>
+        <v>46084.38015046297</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12146,7 +12146,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46083.80761574074</v>
+        <v>46084.40053240741</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12210,7 +12210,7 @@
         <v>1</v>
       </c>
       <c r="N181" s="3" t="n">
-        <v>46083.80201388889</v>
+        <v>46084.38263888889</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
@@ -12407,7 +12407,7 @@
         <v>2</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46084.31738425926</v>
+        <v>46084.39388888889</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12471,7 +12471,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46081.37590277778</v>
+        <v>46084.38715277778</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12535,7 +12535,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46084.22221064815</v>
+        <v>46084.37641203704</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12599,7 +12599,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46083.83796296296</v>
+        <v>46084.38946759259</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12663,7 +12663,7 @@
         <v>1</v>
       </c>
       <c r="N188" s="3" t="n">
-        <v>46083.39923611111</v>
+        <v>46084.39260416666</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
@@ -12749,11 +12749,6 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
-      <c r="C190" t="inlineStr">
-        <is>
-          <t>10.69.5.59</t>
-        </is>
-      </c>
       <c r="D190" t="n">
         <v>2015</v>
       </c>
@@ -12855,7 +12850,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46083.79954861111</v>
+        <v>46084.37543981482</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12919,7 +12914,7 @@
         <v>1</v>
       </c>
       <c r="N192" s="3" t="n">
-        <v>46083.80466435185</v>
+        <v>46084.40319444444</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
@@ -13044,7 +13039,7 @@
         <v>2</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46084.2702199074</v>
+        <v>46084.37980324074</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13108,7 +13103,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46083.83723379629</v>
+        <v>46084.38208333333</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13172,7 +13167,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46083.82203703704</v>
+        <v>46084.38725694444</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13236,7 +13231,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46083.86458333334</v>
+        <v>46084.4009375</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13300,7 +13295,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46083.84304398148</v>
+        <v>46084.39737268518</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13364,7 +13359,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46083.81674768519</v>
+        <v>46084.40123842593</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13553,7 +13548,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46083.8021875</v>
+        <v>46084.37623842592</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13617,7 +13612,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46083.80875</v>
+        <v>46084.37653935186</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13745,7 +13740,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46083.81480324074</v>
+        <v>46084.36822916667</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13809,7 +13804,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46083.80962962963</v>
+        <v>46084.40056712963</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13873,7 +13868,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46083.80962962963</v>
+        <v>46084.39048611111</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13937,7 +13932,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46083.80857638889</v>
+        <v>46084.36810185185</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14001,7 +13996,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46083.80688657407</v>
+        <v>46084.36690972222</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14065,7 +14060,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46083.83802083333</v>
+        <v>46084.38920138889</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14129,7 +14124,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46084.32047453704</v>
+        <v>46084.39905092592</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14193,7 +14188,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46083.79277777778</v>
+        <v>46084.40195601852</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14257,7 +14252,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46083.87391203704</v>
+        <v>46084.38630787037</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14321,7 +14316,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46083.80144675926</v>
+        <v>46084.40170138889</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14449,7 +14444,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46083.82762731481</v>
+        <v>46084.40008101852</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14508,7 +14503,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46083.8052662037</v>
+        <v>46084.39818287037</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14572,7 +14567,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46084.30439814815</v>
+        <v>46084.38317129629</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14636,7 +14631,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46083.8080787037</v>
+        <v>46084.40355324074</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14705,7 +14700,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46083.85549768519</v>
+        <v>46084.36891203704</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14769,7 +14764,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46083.79398148148</v>
+        <v>46084.37917824074</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14833,7 +14828,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46083.81090277778</v>
+        <v>46084.40416666667</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14897,7 +14892,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46083.80289351852</v>
+        <v>46084.39241898148</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14961,7 +14956,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46083.82248842593</v>
+        <v>46084.38871527778</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15025,7 +15020,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46083.80341435185</v>
+        <v>46084.39697916667</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15217,7 +15212,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46083.80224537037</v>
+        <v>46084.37650462963</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15281,7 +15276,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46083.81699074074</v>
+        <v>46084.40407407407</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15345,7 +15340,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46083.82431712963</v>
+        <v>46084.39984953704</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15537,7 +15532,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46084.3082175926</v>
+        <v>46084.38671296297</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15601,7 +15596,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46083.81302083333</v>
+        <v>46084.38575231482</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15665,7 +15660,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46083.79207175926</v>
+        <v>46084.36575231481</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15729,7 +15724,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46083.82371527778</v>
+        <v>46084.40207175926</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15857,7 +15852,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46083.82121527778</v>
+        <v>46084.36619212963</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15921,7 +15916,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46083.82461805556</v>
+        <v>46084.39313657407</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -15985,7 +15980,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46083.80311342593</v>
+        <v>46084.38622685185</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16113,7 +16108,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46083.80471064815</v>
+        <v>46084.4024537037</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16177,7 +16172,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46083.82346064815</v>
+        <v>46084.40094907407</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16196,11 +16191,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C244" t="inlineStr">
-        <is>
-          <t>10.69.5.112</t>
-        </is>
-      </c>
       <c r="D244" t="n">
         <v>2019</v>
       </c>
@@ -16497,7 +16487,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46083.82275462963</v>
+        <v>46084.37299768518</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16561,7 +16551,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46083.79930555556</v>
+        <v>46084.3874074074</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16689,7 +16679,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46083.79752314815</v>
+        <v>46084.39015046296</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16817,7 +16807,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46083.82759259259</v>
+        <v>46084.38758101852</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16875,7 +16865,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46083.79585648148</v>
+        <v>46084.40142361111</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16939,7 +16929,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46084.30733796296</v>
+        <v>46084.38679398148</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -17003,7 +16993,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46083.80766203703</v>
+        <v>46084.40055555556</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17067,7 +17057,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46083.82917824074</v>
+        <v>46084.39890046296</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17131,7 +17121,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46083.80334490741</v>
+        <v>46084.37423611111</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17195,7 +17185,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46083.57784722222</v>
+        <v>46084.32305555556</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17259,7 +17249,7 @@
         <v>1</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46083.60016203704</v>
+        <v>46084.40290509259</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17387,7 +17377,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46083.80528935185</v>
+        <v>46084.37541666667</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17451,7 +17441,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46084.31863425926</v>
+        <v>46084.38899305555</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17515,7 +17505,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46083.79763888889</v>
+        <v>46084.38871527778</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17579,7 +17569,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46083.7930787037</v>
+        <v>46084.40310185185</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17643,7 +17633,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46083.80930555556</v>
+        <v>46084.40018518519</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17707,7 +17697,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46083.79447916667</v>
+        <v>46084.39127314815</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17860,7 +17850,7 @@
         </is>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46084.31092592593</v>
+        <v>46084.39085648148</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -17924,7 +17914,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46084.30424768518</v>
+        <v>46084.37174768518</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -17988,7 +17978,7 @@
         <v>1</v>
       </c>
       <c r="N272" s="3" t="n">
-        <v>46083.64542824074</v>
+        <v>46084.39179398148</v>
       </c>
       <c r="O272" t="inlineStr">
         <is>
@@ -18132,11 +18122,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C275" t="inlineStr">
-        <is>
-          <t>10.69.5.145</t>
-        </is>
-      </c>
       <c r="D275" t="n">
         <v>2013</v>
       </c>
@@ -18302,7 +18287,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46084.31946759259</v>
+        <v>46084.39760416667</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18366,7 +18351,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46084.29840277778</v>
+        <v>46084.37726851852</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18494,7 +18479,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46083.85100694445</v>
+        <v>46084.39119212963</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18617,7 +18602,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46083.82590277777</v>
+        <v>46084.34209490741</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18681,7 +18666,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46083.87239583334</v>
+        <v>46084.38317129629</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18745,7 +18730,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46083.80342592593</v>
+        <v>46084.36872685186</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18764,6 +18749,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>10.69.5.155</t>
+        </is>
+      </c>
       <c r="D285" t="n">
         <v>2019</v>
       </c>
@@ -18804,7 +18794,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46084.19300925926</v>
+        <v>46084.39857638889</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18868,7 +18858,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46084.24326388889</v>
+        <v>46084.39745370371</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18932,7 +18922,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46083.57546296297</v>
+        <v>46084.40054398148</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19790,7 +19780,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46084.31916666667</v>
+        <v>46084.39866898148</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20906,7 +20896,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46084.295</v>
+        <v>46084.37829861111</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21631,7 +21621,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46083.78344907407</v>
+        <v>46084.40119212963</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21695,7 +21685,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46084.2846412037</v>
+        <v>46084.40274305556</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21759,7 +21749,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46084.28498842593</v>
+        <v>46084.40438657408</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21823,7 +21813,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46084.28475694444</v>
+        <v>46084.39600694444</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21887,7 +21877,7 @@
         <v>1</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46084.28434027778</v>
+        <v>46084.4016087963</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21951,7 +21941,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46084.2852662037</v>
+        <v>46084.37049768519</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22015,7 +22005,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46083.78145833333</v>
+        <v>46084.39730324074</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22079,7 +22069,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46084.31541666666</v>
+        <v>46084.38538194444</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22207,7 +22197,7 @@
         <v>2</v>
       </c>
       <c r="N340" s="3" t="n">
-        <v>46083.57987268519</v>
+        <v>46084.37447916667</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -22271,7 +22261,7 @@
         <v>2</v>
       </c>
       <c r="N341" s="3" t="n">
-        <v>46084.29648148148</v>
+        <v>46084.37295138889</v>
       </c>
       <c r="O341" t="inlineStr">
         <is>
@@ -22588,7 +22578,7 @@
         <v>1</v>
       </c>
       <c r="N346" s="3" t="n">
-        <v>46083.59797453704</v>
+        <v>46084.36142361111</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -22716,7 +22706,7 @@
         <v>1</v>
       </c>
       <c r="N348" s="3" t="n">
-        <v>46083.60413194444</v>
+        <v>46084.40400462963</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -22735,6 +22725,11 @@
           <t>OPERACAO 9.1</t>
         </is>
       </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>10.69.5.244</t>
+        </is>
+      </c>
       <c r="D349" t="n">
         <v>2014</v>
       </c>
@@ -22775,7 +22770,7 @@
         <v>1</v>
       </c>
       <c r="N349" s="3" t="n">
-        <v>46083.57994212963</v>
+        <v>46084.40194444444</v>
       </c>
       <c r="O349" t="inlineStr">
         <is>
@@ -22839,7 +22834,7 @@
         <v>1</v>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46083.57173611111</v>
+        <v>46084.39910879629</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -22903,7 +22898,7 @@
         <v>1</v>
       </c>
       <c r="N351" s="3" t="n">
-        <v>46083.60268518519</v>
+        <v>46084.39864583333</v>
       </c>
       <c r="O351" t="inlineStr">
         <is>
@@ -22964,7 +22959,7 @@
         </is>
       </c>
       <c r="N352" s="3" t="n">
-        <v>46083.59739583333</v>
+        <v>46084.36144675926</v>
       </c>
       <c r="O352" t="inlineStr">
         <is>
@@ -23089,7 +23084,7 @@
         <v>1</v>
       </c>
       <c r="N354" s="3" t="n">
-        <v>46083.59190972222</v>
+        <v>46084.40103009259</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -23153,7 +23148,7 @@
         <v>1</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46083.59245370371</v>
+        <v>46084.40265046297</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23217,7 +23212,7 @@
         <v>1</v>
       </c>
       <c r="N356" s="3" t="n">
-        <v>46083.59840277778</v>
+        <v>46084.39940972222</v>
       </c>
       <c r="O356" t="inlineStr">
         <is>
@@ -23236,6 +23231,11 @@
           <t>OPERACAO 9.1</t>
         </is>
       </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>10.69.5.252</t>
+        </is>
+      </c>
       <c r="D357" t="n">
         <v>2012</v>
       </c>
@@ -23276,7 +23276,7 @@
         <v>1</v>
       </c>
       <c r="N357" s="3" t="n">
-        <v>46080.55364583333</v>
+        <v>46084.36210648148</v>
       </c>
       <c r="O357" t="inlineStr">
         <is>
@@ -23340,7 +23340,7 @@
         <v>2</v>
       </c>
       <c r="N358" s="3" t="n">
-        <v>46083.59804398148</v>
+        <v>46084.39716435185</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -23404,7 +23404,7 @@
         <v>2</v>
       </c>
       <c r="N359" s="3" t="n">
-        <v>46083.60714120371</v>
+        <v>46084.40163194444</v>
       </c>
       <c r="O359" t="inlineStr">
         <is>
@@ -23468,7 +23468,7 @@
         <v>1</v>
       </c>
       <c r="N360" s="3" t="n">
-        <v>46083.60237268519</v>
+        <v>46084.40269675926</v>
       </c>
       <c r="O360" t="inlineStr">
         <is>
@@ -23717,7 +23717,7 @@
         <v>1</v>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46083.71135416667</v>
+        <v>46084.36601851852</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23783,7 +23783,7 @@
         </is>
       </c>
       <c r="N365" s="3" t="n">
-        <v>46084.30540509259</v>
+        <v>46084.37921296297</v>
       </c>
       <c r="O365" t="inlineStr">
         <is>
@@ -23909,7 +23909,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46083.70922453704</v>
+        <v>46084.36986111111</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -23928,6 +23928,11 @@
           <t>RH</t>
         </is>
       </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>10.69.3.13</t>
+        </is>
+      </c>
       <c r="D368" t="n">
         <v>2025</v>
       </c>
@@ -23970,7 +23975,7 @@
         </is>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46083.67690972222</v>
+        <v>46084.40091435185</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24039,7 +24044,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46084.30673611111</v>
+        <v>46084.38461805556</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24315,7 +24320,7 @@
         <v>1</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46083.74173611111</v>
+        <v>46084.38796296297</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24381,7 +24386,7 @@
         </is>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46084.31881944444</v>
+        <v>46084.39703703704</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24400,11 +24405,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C375" t="inlineStr">
-        <is>
-          <t>10.69.3.72</t>
-        </is>
-      </c>
       <c r="D375" t="n">
         <v>2025</v>
       </c>
@@ -24519,7 +24519,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46083.74791666667</v>
+        <v>46084.38780092593</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -24588,7 +24588,7 @@
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46084.30924768518</v>
+        <v>46084.38886574074</v>
       </c>
       <c r="O377" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-03 11:52:05.622324
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q377"/>
+  <dimension ref="A1:Q376"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25.2" customWidth="1" min="1" max="1"/>
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46084.38317129629</v>
+        <v>46084.45994212963</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46084.40255787037</v>
+        <v>46084.47519675926</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -734,10 +734,10 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46084.40043981482</v>
+        <v>46084.4811574074</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46084.37159722222</v>
+        <v>46084.48472222222</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46084.3878587963</v>
+        <v>46084.46375</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46084.39876157408</v>
+        <v>46084.47619212963</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1510,7 +1510,7 @@
         <v>2</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>46084.37489583333</v>
+        <v>46084.4481712963</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46084.39865740741</v>
+        <v>46084.47521990741</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46084.40065972223</v>
+        <v>46084.47832175926</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1699,7 +1699,7 @@
         </is>
       </c>
       <c r="N19" s="3" t="n">
-        <v>46084.40447916667</v>
+        <v>46084.4794675926</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1763,7 +1763,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46084.39351851852</v>
+        <v>46084.46835648148</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -6565,7 +6565,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46084.39771990741</v>
+        <v>46084.47893518519</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6634,7 +6634,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46083.83415509259</v>
+        <v>46084.47924768519</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6653,11 +6653,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>10.69.3.93</t>
-        </is>
-      </c>
       <c r="D97" t="n">
         <v>2025</v>
       </c>
@@ -6703,7 +6698,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46084.37287037037</v>
+        <v>46084.45207175926</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6722,6 +6717,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>10.69.3.94</t>
+        </is>
+      </c>
       <c r="D98" t="n">
         <v>2025</v>
       </c>
@@ -6767,7 +6767,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46084.36756944445</v>
+        <v>46084.48283564814</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6836,7 +6836,7 @@
         <v>1</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46084.37560185185</v>
+        <v>46084.45454861111</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
         <v>2</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46084.40212962963</v>
+        <v>46084.4808449074</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6974,7 +6974,7 @@
         <v>1</v>
       </c>
       <c r="N101" s="3" t="n">
-        <v>46084.36840277778</v>
+        <v>46084.48162037037</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -7112,7 +7112,7 @@
         <v>2</v>
       </c>
       <c r="N103" s="3" t="n">
-        <v>46084.38550925926</v>
+        <v>46084.46283564815</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -7239,7 +7239,7 @@
         </is>
       </c>
       <c r="N105" s="3" t="n">
-        <v>46083.61646990741</v>
+        <v>46084.48403935185</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
@@ -7369,7 +7369,7 @@
         <v>1</v>
       </c>
       <c r="N107" s="3" t="n">
-        <v>46084.37907407407</v>
+        <v>46084.45972222222</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -7507,7 +7507,7 @@
         <v>1</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46084.3741087963</v>
+        <v>46084.45159722222</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7576,7 +7576,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46084.3712962963</v>
+        <v>46084.4844212963</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7645,7 +7645,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46084.36873842592</v>
+        <v>46084.44476851852</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7714,7 +7714,7 @@
         <v>2</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46084.39400462963</v>
+        <v>46084.47618055555</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7783,7 +7783,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46084.37175925926</v>
+        <v>46084.45440972222</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7852,7 +7852,7 @@
         <v>1</v>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46084.38185185185</v>
+        <v>46084.45828703704</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7918,7 +7918,7 @@
         </is>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46084.37668981482</v>
+        <v>46084.45491898148</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7987,7 +7987,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46084.4033912037</v>
+        <v>46084.48050925926</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8051,7 +8051,7 @@
         <v>1</v>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46084.39614583334</v>
+        <v>46084.47493055555</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8117,7 +8117,7 @@
         </is>
       </c>
       <c r="N118" s="3" t="n">
-        <v>46084.37339120371</v>
+        <v>46084.44725694445</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -8255,7 +8255,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46084.38349537037</v>
+        <v>46084.45695601852</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8324,7 +8324,7 @@
         <v>1</v>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46084.39947916667</v>
+        <v>46084.47373842593</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8390,7 +8390,7 @@
         </is>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46084.39674768518</v>
+        <v>46084.46833333333</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8459,7 +8459,7 @@
         <v>2</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46084.28221064815</v>
+        <v>46084.4584375</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8528,7 +8528,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46084.39277777778</v>
+        <v>46084.46836805555</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8597,7 +8597,7 @@
         <v>1</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46084.37782407407</v>
+        <v>46084.45269675926</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8666,7 +8666,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46084.36984953703</v>
+        <v>46084.48770833333</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8735,7 +8735,7 @@
         <v>2</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46084.36975694444</v>
+        <v>46084.48043981481</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8804,7 +8804,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46084.39956018519</v>
+        <v>46084.48003472222</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8905,7 +8905,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Windows</t>
+          <t>Microsoft Windows 11 Pro</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -8942,7 +8942,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46084.36686342592</v>
+        <v>46084.45802083334</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9006,7 +9006,7 @@
         <v>1</v>
       </c>
       <c r="N131" s="3" t="n">
-        <v>46084.37074074074</v>
+        <v>46084.44813657407</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -9139,7 +9139,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46084.37824074074</v>
+        <v>46084.45487268519</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9458,7 +9458,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46084.37166666667</v>
+        <v>46084.4492824074</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9586,7 +9586,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46084.39728009259</v>
+        <v>46084.47428240741</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9650,7 +9650,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46084.37081018519</v>
+        <v>46084.48243055555</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9714,7 +9714,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46084.39696759259</v>
+        <v>46084.47712962963</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9778,7 +9778,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46084.36958333333</v>
+        <v>46084.48739583333</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9842,7 +9842,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46084.38451388889</v>
+        <v>46084.46358796296</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9906,7 +9906,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46084.395</v>
+        <v>46084.47497685185</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9970,7 +9970,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46084.37546296296</v>
+        <v>46084.45216435185</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10034,7 +10034,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46084.37552083333</v>
+        <v>46084.44846064815</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10098,7 +10098,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46084.38929398148</v>
+        <v>46084.46325231482</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10162,7 +10162,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46084.37179398148</v>
+        <v>46084.44732638889</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10226,7 +10226,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46084.38063657407</v>
+        <v>46084.45579861111</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10290,7 +10290,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46084.38135416667</v>
+        <v>46084.45974537037</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10354,7 +10354,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46084.38663194444</v>
+        <v>46084.46193287037</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10418,7 +10418,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46084.39915509259</v>
+        <v>46084.47471064814</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10482,7 +10482,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46084.4025462963</v>
+        <v>46084.47917824074</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10546,7 +10546,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46084.38120370371</v>
+        <v>46084.45664351852</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10610,7 +10610,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46084.39774305555</v>
+        <v>46084.47655092592</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10674,7 +10674,7 @@
         <v>1</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>46084.37331018518</v>
+        <v>46084.44763888889</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -10738,7 +10738,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46084.37494212963</v>
+        <v>46084.449375</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10802,7 +10802,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46084.37290509259</v>
+        <v>46084.45290509259</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10866,7 +10866,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46084.38173611111</v>
+        <v>46084.45821759259</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10930,7 +10930,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46084.38173611111</v>
+        <v>46084.45631944444</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -10994,7 +10994,7 @@
         <v>1</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46084.3782175926</v>
+        <v>46084.45520833333</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11122,7 +11122,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46084.37386574074</v>
+        <v>46084.44950231481</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11186,7 +11186,7 @@
         <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46084.36765046296</v>
+        <v>46084.47953703703</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11250,7 +11250,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46084.39689814814</v>
+        <v>46084.47702546296</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11314,7 +11314,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46084.39369212963</v>
+        <v>46084.46769675926</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11378,7 +11378,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46084.39269675926</v>
+        <v>46084.47059027778</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11442,7 +11442,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46084.36775462963</v>
+        <v>46084.48133101852</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11506,7 +11506,7 @@
         <v>2</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46084.39980324074</v>
+        <v>46084.47875</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11570,7 +11570,7 @@
         <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46084.40417824074</v>
+        <v>46084.48459490741</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11698,7 +11698,7 @@
         <v>1</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46084.39270833333</v>
+        <v>46084.47363425926</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11762,7 +11762,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46084.39280092593</v>
+        <v>46084.46461805556</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11826,7 +11826,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46084.37349537037</v>
+        <v>46084.44706018519</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11890,7 +11890,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46083.6533912037</v>
+        <v>46084.45681712963</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -12018,7 +12018,7 @@
         <v>2</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46084.36739583333</v>
+        <v>46084.48237268518</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12082,7 +12082,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46084.38015046297</v>
+        <v>46084.46047453704</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12146,7 +12146,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46084.40053240741</v>
+        <v>46084.47841435186</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12210,7 +12210,7 @@
         <v>1</v>
       </c>
       <c r="N181" s="3" t="n">
-        <v>46084.38263888889</v>
+        <v>46084.46228009259</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
@@ -12407,7 +12407,7 @@
         <v>2</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46084.39388888889</v>
+        <v>46084.47127314815</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12471,7 +12471,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46084.38715277778</v>
+        <v>46084.46628472222</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12535,7 +12535,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46084.37641203704</v>
+        <v>46084.45608796296</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12599,7 +12599,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46084.38946759259</v>
+        <v>46084.46347222223</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12663,7 +12663,7 @@
         <v>1</v>
       </c>
       <c r="N188" s="3" t="n">
-        <v>46084.39260416666</v>
+        <v>46084.4747337963</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
@@ -12850,7 +12850,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46084.37543981482</v>
+        <v>46084.45084490741</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12914,7 +12914,7 @@
         <v>1</v>
       </c>
       <c r="N192" s="3" t="n">
-        <v>46084.40319444444</v>
+        <v>46084.4844212963</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
@@ -13039,7 +13039,7 @@
         <v>2</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46084.37980324074</v>
+        <v>46084.45653935185</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13103,7 +13103,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46084.38208333333</v>
+        <v>46084.45587962963</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13167,7 +13167,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46084.38725694444</v>
+        <v>46084.46653935185</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13231,7 +13231,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46084.4009375</v>
+        <v>46084.47310185185</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13295,7 +13295,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46084.39737268518</v>
+        <v>46084.47495370371</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13359,7 +13359,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46084.40123842593</v>
+        <v>46084.47648148148</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13548,7 +13548,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46084.37623842592</v>
+        <v>46084.45348379629</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13612,7 +13612,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46084.37653935186</v>
+        <v>46084.44756944444</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13740,7 +13740,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46084.36822916667</v>
+        <v>46084.44983796297</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13804,7 +13804,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46084.40056712963</v>
+        <v>46084.47857638889</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13868,7 +13868,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46084.39048611111</v>
+        <v>46084.46678240741</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13932,7 +13932,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46084.36810185185</v>
+        <v>46084.4687037037</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -13996,7 +13996,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46084.36690972222</v>
+        <v>46084.48320601852</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14060,7 +14060,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46084.38920138889</v>
+        <v>46084.46751157408</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14124,7 +14124,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46084.39905092592</v>
+        <v>46084.47591435185</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14188,7 +14188,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46084.40195601852</v>
+        <v>46084.48230324074</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14252,7 +14252,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46084.38630787037</v>
+        <v>46084.463125</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14316,7 +14316,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46084.40170138889</v>
+        <v>46084.47792824074</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14444,7 +14444,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46084.40008101852</v>
+        <v>46084.47603009259</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14503,7 +14503,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46084.39818287037</v>
+        <v>46084.47431712963</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14567,7 +14567,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46084.38317129629</v>
+        <v>46084.45945601852</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14631,7 +14631,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46084.40355324074</v>
+        <v>46084.47719907408</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14700,7 +14700,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46084.36891203704</v>
+        <v>46084.45107638889</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14764,7 +14764,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46084.37917824074</v>
+        <v>46084.4587962963</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14828,7 +14828,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46084.40416666667</v>
+        <v>46084.48608796296</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14892,7 +14892,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46084.39241898148</v>
+        <v>46084.46483796297</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14956,7 +14956,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46084.38871527778</v>
+        <v>46084.48034722222</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15020,7 +15020,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46084.39697916667</v>
+        <v>46084.47553240741</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15044,47 +15044,11 @@
           <t>10.69.5.94</t>
         </is>
       </c>
-      <c r="D226" t="n">
-        <v>2011</v>
-      </c>
-      <c r="E226" t="n">
-        <v>8390</v>
-      </c>
-      <c r="F226" t="inlineStr">
-        <is>
-          <t>Microsoft® Windows Vista™ Business</t>
-        </is>
-      </c>
-      <c r="G226" t="inlineStr">
-        <is>
-          <t>BRG827F584</t>
-        </is>
-      </c>
-      <c r="I226" t="inlineStr">
-        <is>
-          <t>Intel</t>
-        </is>
-      </c>
-      <c r="J226" t="inlineStr">
-        <is>
-          <t>2 GB</t>
-        </is>
-      </c>
-      <c r="K226" t="inlineStr">
-        <is>
-          <t>HP</t>
-        </is>
-      </c>
-      <c r="L226" t="inlineStr">
-        <is>
-          <t>HP Compaq dx7400 Brazil SFF PC.</t>
-        </is>
-      </c>
       <c r="M226" t="n">
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46083.60423611111</v>
+        <v>46084.47436342593</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15212,7 +15176,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46084.37650462963</v>
+        <v>46084.45503472222</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15276,7 +15240,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46084.40407407407</v>
+        <v>46084.4609837963</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15340,7 +15304,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46084.39984953704</v>
+        <v>46084.48142361111</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15532,7 +15496,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46084.38671296297</v>
+        <v>46084.46380787037</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15596,7 +15560,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46084.38575231482</v>
+        <v>46084.46497685185</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15660,7 +15624,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46084.36575231481</v>
+        <v>46084.48364583333</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15724,7 +15688,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46084.40207175926</v>
+        <v>46084.47865740741</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15852,7 +15816,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46084.36619212963</v>
+        <v>46084.48350694445</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15916,7 +15880,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46084.39313657407</v>
+        <v>46084.46675925926</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -15980,7 +15944,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46084.38622685185</v>
+        <v>46084.48310185185</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16044,7 +16008,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46083.81465277778</v>
+        <v>46084.48255787037</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16108,7 +16072,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46084.4024537037</v>
+        <v>46084.48081018519</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16172,7 +16136,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46084.40094907407</v>
+        <v>46084.4765162037</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16487,7 +16451,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46084.37299768518</v>
+        <v>46084.45193287037</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16551,7 +16515,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46084.3874074074</v>
+        <v>46084.46100694445</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16570,11 +16534,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C250" t="inlineStr">
-        <is>
-          <t>10.69.5.118</t>
-        </is>
-      </c>
       <c r="D250" t="n">
         <v>2017</v>
       </c>
@@ -16679,7 +16638,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46084.39015046296</v>
+        <v>46084.46832175926</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16807,7 +16766,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46084.38758101852</v>
+        <v>46084.46350694444</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16865,7 +16824,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46084.40142361111</v>
+        <v>46084.48052083333</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16929,7 +16888,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46084.38679398148</v>
+        <v>46084.4649537037</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -16993,7 +16952,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46084.40055555556</v>
+        <v>46084.46600694444</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17057,7 +17016,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46084.39890046296</v>
+        <v>46084.47856481482</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17121,7 +17080,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46084.37423611111</v>
+        <v>46084.4540625</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17185,7 +17144,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46084.32305555556</v>
+        <v>46084.47333333334</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17249,7 +17208,7 @@
         <v>1</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46084.40290509259</v>
+        <v>46084.48427083333</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17377,7 +17336,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46084.37541666667</v>
+        <v>46084.45271990741</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17441,7 +17400,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46084.38899305555</v>
+        <v>46084.46149305555</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17505,7 +17464,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46084.38871527778</v>
+        <v>46084.46987268519</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17569,7 +17528,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46084.40310185185</v>
+        <v>46084.47915509259</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17633,7 +17592,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46084.40018518519</v>
+        <v>46084.47922453703</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17697,7 +17656,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46084.39127314815</v>
+        <v>46084.47260416667</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17725,7 +17684,7 @@
         <v>2</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46083.7766087963</v>
+        <v>46084.4190625</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17789,7 +17748,7 @@
         <v>1</v>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46083.82607638889</v>
+        <v>46084.4705787037</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17850,7 +17809,7 @@
         </is>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46084.39085648148</v>
+        <v>46084.48637731482</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -17914,7 +17873,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46084.37174768518</v>
+        <v>46084.48377314815</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -17978,7 +17937,7 @@
         <v>1</v>
       </c>
       <c r="N272" s="3" t="n">
-        <v>46084.39179398148</v>
+        <v>46084.46541666667</v>
       </c>
       <c r="O272" t="inlineStr">
         <is>
@@ -18287,7 +18246,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46084.39760416667</v>
+        <v>46084.47275462963</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18351,7 +18310,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46084.37726851852</v>
+        <v>46084.45394675926</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18376,46 +18335,46 @@
         </is>
       </c>
       <c r="D279" t="n">
-        <v>2013</v>
+        <v>2014</v>
       </c>
       <c r="E279" t="n">
-        <v>22943</v>
+        <v>3507</v>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>Microsoft® Windows Vista™ Business</t>
+          <t>Microsoft Windows 7 Professional</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
         <is>
-          <t>L1BFDCZ</t>
+          <t>BRG037G51X</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
         <is>
-          <t>Intel Core 2 Duo</t>
+          <t>Intel Core 2 Quad</t>
         </is>
       </c>
       <c r="J279" t="inlineStr">
         <is>
-          <t>2 GB</t>
+          <t>4 GB</t>
         </is>
       </c>
       <c r="K279" t="inlineStr">
         <is>
-          <t>LENOVO</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="L279" t="inlineStr">
         <is>
-          <t>ThinkCentre M58p</t>
+          <t>HP Compaq 6000 Pro SFF PC</t>
         </is>
       </c>
       <c r="M279" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N279" s="3" t="n">
-        <v>46083.47760416667</v>
+        <v>46084.47466435185</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -18479,7 +18438,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46084.39119212963</v>
+        <v>46084.47033564815</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18602,7 +18561,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46084.34209490741</v>
+        <v>46084.4569212963</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18666,7 +18625,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46084.38317129629</v>
+        <v>46084.46337962963</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18730,7 +18689,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46084.36872685186</v>
+        <v>46084.48361111111</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18794,7 +18753,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46084.39857638889</v>
+        <v>46084.47478009259</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18858,7 +18817,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46084.39745370371</v>
+        <v>46084.47407407407</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18922,7 +18881,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46084.40054398148</v>
+        <v>46084.47958333333</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -18986,7 +18945,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46083.85875</v>
+        <v>46084.45835648148</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19780,7 +19739,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46084.39866898148</v>
+        <v>46084.47283564815</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20896,7 +20855,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46084.37829861111</v>
+        <v>46084.45710648148</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21621,7 +21580,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46084.40119212963</v>
+        <v>46084.4819212963</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21685,7 +21644,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46084.40274305556</v>
+        <v>46084.47818287037</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21749,7 +21708,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46084.40438657408</v>
+        <v>46084.47960648148</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21813,7 +21772,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46084.39600694444</v>
+        <v>46084.47329861111</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21877,7 +21836,7 @@
         <v>1</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46084.4016087963</v>
+        <v>46084.47589120371</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21941,7 +21900,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46084.37049768519</v>
+        <v>46084.45230324074</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22005,7 +21964,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46084.39730324074</v>
+        <v>46084.47204861111</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22069,7 +22028,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46084.38538194444</v>
+        <v>46084.46637731481</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22197,7 +22156,7 @@
         <v>2</v>
       </c>
       <c r="N340" s="3" t="n">
-        <v>46084.37447916667</v>
+        <v>46084.45181712963</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -22261,7 +22220,7 @@
         <v>2</v>
       </c>
       <c r="N341" s="3" t="n">
-        <v>46084.37295138889</v>
+        <v>46084.45305555555</v>
       </c>
       <c r="O341" t="inlineStr">
         <is>
@@ -22280,6 +22239,11 @@
           <t>OPERACAO 9.1</t>
         </is>
       </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>10.69.5.237</t>
+        </is>
+      </c>
       <c r="D342" t="n">
         <v>2017</v>
       </c>
@@ -22322,7 +22286,7 @@
         </is>
       </c>
       <c r="N342" s="3" t="n">
-        <v>46079.42385416666</v>
+        <v>46084.45726851852</v>
       </c>
       <c r="O342" t="inlineStr">
         <is>
@@ -22578,7 +22542,7 @@
         <v>1</v>
       </c>
       <c r="N346" s="3" t="n">
-        <v>46084.36142361111</v>
+        <v>46084.48739583333</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -22642,7 +22606,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46083.59905092593</v>
+        <v>46084.45409722222</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22706,7 +22670,7 @@
         <v>1</v>
       </c>
       <c r="N348" s="3" t="n">
-        <v>46084.40400462963</v>
+        <v>46084.47803240741</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -22731,46 +22695,43 @@
         </is>
       </c>
       <c r="D349" t="n">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="E349" t="n">
-        <v>3507</v>
+        <v>22943</v>
       </c>
       <c r="F349" t="inlineStr">
         <is>
-          <t>Microsoft Windows 7 Professional</t>
+          <t>Microsoft® Windows Vista™ Business</t>
         </is>
       </c>
       <c r="G349" t="inlineStr">
         <is>
-          <t>BRG037G51X</t>
+          <t>L1BFDCZ</t>
         </is>
       </c>
       <c r="I349" t="inlineStr">
         <is>
-          <t>Intel Core 2 Quad</t>
+          <t>Intel Core 2 Duo</t>
         </is>
       </c>
       <c r="J349" t="inlineStr">
         <is>
-          <t>4 GB</t>
+          <t>2 GB</t>
         </is>
       </c>
       <c r="K349" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>LENOVO</t>
         </is>
       </c>
       <c r="L349" t="inlineStr">
         <is>
-          <t>HP Compaq 6000 Pro SFF PC</t>
-        </is>
-      </c>
-      <c r="M349" t="n">
-        <v>1</v>
+          <t>ThinkCentre M58p</t>
+        </is>
       </c>
       <c r="N349" s="3" t="n">
-        <v>46084.40194444444</v>
+        <v>46084.45179398148</v>
       </c>
       <c r="O349" t="inlineStr">
         <is>
@@ -22834,7 +22795,7 @@
         <v>1</v>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46084.39910879629</v>
+        <v>46084.47752314815</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -22898,7 +22859,7 @@
         <v>1</v>
       </c>
       <c r="N351" s="3" t="n">
-        <v>46084.39864583333</v>
+        <v>46084.47392361111</v>
       </c>
       <c r="O351" t="inlineStr">
         <is>
@@ -22909,7 +22870,7 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>PA_247</t>
+          <t>PA_248</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
@@ -22919,7 +22880,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>10.69.5.247</t>
+          <t>10.69.5.248</t>
         </is>
       </c>
       <c r="D352" t="n">
@@ -22935,7 +22896,7 @@
       </c>
       <c r="G352" t="inlineStr">
         <is>
-          <t>BRJ525SZ0B</t>
+          <t>BRJ523SG7Z</t>
         </is>
       </c>
       <c r="I352" t="inlineStr">
@@ -22945,7 +22906,7 @@
       </c>
       <c r="J352" t="inlineStr">
         <is>
-          <t>8 GB</t>
+          <t>6 GB</t>
         </is>
       </c>
       <c r="K352" t="inlineStr">
@@ -22959,7 +22920,7 @@
         </is>
       </c>
       <c r="N352" s="3" t="n">
-        <v>46084.36144675926</v>
+        <v>46080.51325231481</v>
       </c>
       <c r="O352" t="inlineStr">
         <is>
@@ -22970,7 +22931,7 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>PA_248</t>
+          <t>PA_249</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
@@ -22980,23 +22941,23 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>10.69.5.248</t>
+          <t>10.69.5.249</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="E353" t="n">
-        <v>73645</v>
+        <v>51040</v>
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>Microsoft Windows 8.1 Pro</t>
+          <t>Microsoft Windows 7 Professional</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
         <is>
-          <t>BRJ523SG7Z</t>
+          <t>BRG311F8KL</t>
         </is>
       </c>
       <c r="I353" t="inlineStr">
@@ -23006,7 +22967,7 @@
       </c>
       <c r="J353" t="inlineStr">
         <is>
-          <t>6 GB</t>
+          <t>4 GB</t>
         </is>
       </c>
       <c r="K353" t="inlineStr">
@@ -23016,11 +22977,14 @@
       </c>
       <c r="L353" t="inlineStr">
         <is>
-          <t>HP 402 G1 SFF Business PC</t>
-        </is>
+          <t>HP Compaq Pro 4300 SFF Brazil PC</t>
+        </is>
+      </c>
+      <c r="M353" t="n">
+        <v>1</v>
       </c>
       <c r="N353" s="3" t="n">
-        <v>46080.51325231481</v>
+        <v>46084.47817129629</v>
       </c>
       <c r="O353" t="inlineStr">
         <is>
@@ -23031,7 +22995,7 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>PA_249</t>
+          <t>PA_250</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
@@ -23041,14 +23005,14 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>10.69.5.249</t>
+          <t>10.69.5.250</t>
         </is>
       </c>
       <c r="D354" t="n">
         <v>2016</v>
       </c>
       <c r="E354" t="n">
-        <v>51040</v>
+        <v>43374</v>
       </c>
       <c r="F354" t="inlineStr">
         <is>
@@ -23057,12 +23021,12 @@
       </c>
       <c r="G354" t="inlineStr">
         <is>
-          <t>BRG311F8KL</t>
+          <t>BRG103F99B</t>
         </is>
       </c>
       <c r="I354" t="inlineStr">
         <is>
-          <t>Intel Core i5</t>
+          <t>Intel Core 2 Duo</t>
         </is>
       </c>
       <c r="J354" t="inlineStr">
@@ -23077,14 +23041,14 @@
       </c>
       <c r="L354" t="inlineStr">
         <is>
-          <t>HP Compaq Pro 4300 SFF Brazil PC</t>
+          <t>COMPAQ 300B MT</t>
         </is>
       </c>
       <c r="M354" t="n">
         <v>1</v>
       </c>
       <c r="N354" s="3" t="n">
-        <v>46084.40103009259</v>
+        <v>46084.48047453703</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -23095,7 +23059,7 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>PA_250</t>
+          <t>PA_251</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
@@ -23105,14 +23069,14 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>10.69.5.250</t>
+          <t>10.69.5.251</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="E355" t="n">
-        <v>43374</v>
+        <v>59162</v>
       </c>
       <c r="F355" t="inlineStr">
         <is>
@@ -23121,12 +23085,12 @@
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t>BRG103F99B</t>
+          <t>BRG319F89N</t>
         </is>
       </c>
       <c r="I355" t="inlineStr">
         <is>
-          <t>Intel Core 2 Duo</t>
+          <t>Intel Core i3</t>
         </is>
       </c>
       <c r="J355" t="inlineStr">
@@ -23141,14 +23105,14 @@
       </c>
       <c r="L355" t="inlineStr">
         <is>
-          <t>COMPAQ 300B MT</t>
+          <t>HP Compaq Pro 4300 SFF Brazil PC</t>
         </is>
       </c>
       <c r="M355" t="n">
         <v>1</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46084.40265046297</v>
+        <v>46084.47532407408</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23159,7 +23123,7 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>PA_251</t>
+          <t>PA_252</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
@@ -23169,50 +23133,50 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>10.69.5.251</t>
+          <t>10.69.5.252</t>
         </is>
       </c>
       <c r="D356" t="n">
-        <v>2017</v>
+        <v>2012</v>
       </c>
       <c r="E356" t="n">
-        <v>59162</v>
+        <v>2956</v>
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t>Microsoft Windows 7 Professional</t>
+          <t>Microsoft® Windows Vista™ Business</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
         <is>
-          <t>BRG319F89N</t>
+          <t>J5L1JJ1</t>
         </is>
       </c>
       <c r="I356" t="inlineStr">
         <is>
-          <t>Intel Core i3</t>
+          <t>Intel Core 2 Duo</t>
         </is>
       </c>
       <c r="J356" t="inlineStr">
         <is>
-          <t>4 GB</t>
+          <t>2 GB</t>
         </is>
       </c>
       <c r="K356" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Dell Inc.</t>
         </is>
       </c>
       <c r="L356" t="inlineStr">
         <is>
-          <t>HP Compaq Pro 4300 SFF Brazil PC</t>
+          <t>OptiPlex 755</t>
         </is>
       </c>
       <c r="M356" t="n">
         <v>1</v>
       </c>
       <c r="N356" s="3" t="n">
-        <v>46084.39940972222</v>
+        <v>46084.36210648148</v>
       </c>
       <c r="O356" t="inlineStr">
         <is>
@@ -23223,7 +23187,7 @@
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>PA_252</t>
+          <t>PA_253</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
@@ -23233,50 +23197,50 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>10.69.5.252</t>
+          <t>10.69.5.253</t>
         </is>
       </c>
       <c r="D357" t="n">
-        <v>2012</v>
+        <v>2019</v>
       </c>
       <c r="E357" t="n">
-        <v>2956</v>
+        <v>73645</v>
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t>Microsoft® Windows Vista™ Business</t>
+          <t>Microsoft Windows 8.1 Pro</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
         <is>
-          <t>J5L1JJ1</t>
+          <t>BRJ430FZQN</t>
         </is>
       </c>
       <c r="I357" t="inlineStr">
         <is>
-          <t>Intel Core 2 Duo</t>
+          <t>Intel Core i5</t>
         </is>
       </c>
       <c r="J357" t="inlineStr">
         <is>
-          <t>2 GB</t>
+          <t>4 GB</t>
         </is>
       </c>
       <c r="K357" t="inlineStr">
         <is>
-          <t>Dell Inc.</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="L357" t="inlineStr">
         <is>
-          <t>OptiPlex 755</t>
+          <t>HP 402 G1 SFF Business PC</t>
         </is>
       </c>
       <c r="M357" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N357" s="3" t="n">
-        <v>46084.36210648148</v>
+        <v>46084.47333333334</v>
       </c>
       <c r="O357" t="inlineStr">
         <is>
@@ -23287,7 +23251,7 @@
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>PA_253</t>
+          <t>PA_254</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
@@ -23297,33 +23261,33 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>10.69.5.253</t>
+          <t>10.69.5.254</t>
         </is>
       </c>
       <c r="D358" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="E358" t="n">
-        <v>73645</v>
+        <v>43374</v>
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t>Microsoft Windows 8.1 Pro</t>
+          <t>Microsoft Windows 7 Professional</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
         <is>
-          <t>BRJ430FZQN</t>
+          <t>BRG103F9NQ</t>
         </is>
       </c>
       <c r="I358" t="inlineStr">
         <is>
-          <t>Intel Core i5</t>
+          <t>Intel Core 2 Duo</t>
         </is>
       </c>
       <c r="J358" t="inlineStr">
         <is>
-          <t>4 GB</t>
+          <t>2 GB</t>
         </is>
       </c>
       <c r="K358" t="inlineStr">
@@ -23333,14 +23297,14 @@
       </c>
       <c r="L358" t="inlineStr">
         <is>
-          <t>HP 402 G1 SFF Business PC</t>
+          <t>COMPAQ 300B MT</t>
         </is>
       </c>
       <c r="M358" t="n">
         <v>2</v>
       </c>
       <c r="N358" s="3" t="n">
-        <v>46084.39716435185</v>
+        <v>46084.47502314814</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -23351,7 +23315,7 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>PA_254</t>
+          <t>PA_255</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
@@ -23361,14 +23325,14 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>10.69.5.254</t>
+          <t>10.69.2.11</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>2016</v>
+        <v>2012</v>
       </c>
       <c r="E359" t="n">
-        <v>43374</v>
+        <v>98086</v>
       </c>
       <c r="F359" t="inlineStr">
         <is>
@@ -23377,17 +23341,17 @@
       </c>
       <c r="G359" t="inlineStr">
         <is>
-          <t>BRG103F9NQ</t>
+          <t>BRG232F74W</t>
         </is>
       </c>
       <c r="I359" t="inlineStr">
         <is>
-          <t>Intel Core 2 Duo</t>
+          <t>Intel Core i3</t>
         </is>
       </c>
       <c r="J359" t="inlineStr">
         <is>
-          <t>2 GB</t>
+          <t>4 GB</t>
         </is>
       </c>
       <c r="K359" t="inlineStr">
@@ -23397,14 +23361,14 @@
       </c>
       <c r="L359" t="inlineStr">
         <is>
-          <t>COMPAQ 300B MT</t>
+          <t>HP Pro 3410 Series</t>
         </is>
       </c>
       <c r="M359" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N359" s="3" t="n">
-        <v>46084.40163194444</v>
+        <v>46084.47483796296</v>
       </c>
       <c r="O359" t="inlineStr">
         <is>
@@ -23415,7 +23379,7 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>PA_255</t>
+          <t>PA_256</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
@@ -23425,50 +23389,47 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>10.69.2.11</t>
+          <t>10.69.5.9</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="E360" t="n">
-        <v>98086</v>
+        <v>22943</v>
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t>Microsoft Windows 7 Professional</t>
+          <t>Microsoft® Windows Vista™ Business</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
         <is>
-          <t>BRG232F74W</t>
+          <t>GCCKZL1</t>
         </is>
       </c>
       <c r="I360" t="inlineStr">
         <is>
-          <t>Intel Core i3</t>
+          <t>Intel Core 2 Duo</t>
         </is>
       </c>
       <c r="J360" t="inlineStr">
         <is>
-          <t>4 GB</t>
+          <t>2 GB</t>
         </is>
       </c>
       <c r="K360" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Dell Inc.</t>
         </is>
       </c>
       <c r="L360" t="inlineStr">
         <is>
-          <t>HP Pro 3410 Series</t>
-        </is>
-      </c>
-      <c r="M360" t="n">
-        <v>1</v>
+          <t>OptiPlex 360</t>
+        </is>
       </c>
       <c r="N360" s="3" t="n">
-        <v>46084.40269675926</v>
+        <v>46083.44710648148</v>
       </c>
       <c r="O360" t="inlineStr">
         <is>
@@ -23479,7 +23440,7 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>PA_256</t>
+          <t>PA_257</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
@@ -23489,14 +23450,14 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>10.69.5.9</t>
+          <t>10.69.5.218</t>
         </is>
       </c>
       <c r="D361" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="E361" t="n">
-        <v>22943</v>
+        <v>2956</v>
       </c>
       <c r="F361" t="inlineStr">
         <is>
@@ -23505,7 +23466,7 @@
       </c>
       <c r="G361" t="inlineStr">
         <is>
-          <t>GCCKZL1</t>
+          <t>G1XQXG1</t>
         </is>
       </c>
       <c r="I361" t="inlineStr">
@@ -23525,11 +23486,11 @@
       </c>
       <c r="L361" t="inlineStr">
         <is>
-          <t>OptiPlex 360</t>
+          <t>OptiPlex 755</t>
         </is>
       </c>
       <c r="N361" s="3" t="n">
-        <v>46083.44710648148</v>
+        <v>46049.60199074074</v>
       </c>
       <c r="O361" t="inlineStr">
         <is>
@@ -23540,7 +23501,7 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>PA_257</t>
+          <t>PA_258</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
@@ -23550,14 +23511,14 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>10.69.5.218</t>
+          <t>10.69.5.222</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="E362" t="n">
-        <v>2956</v>
+        <v>3913</v>
       </c>
       <c r="F362" t="inlineStr">
         <is>
@@ -23566,7 +23527,7 @@
       </c>
       <c r="G362" t="inlineStr">
         <is>
-          <t>G1XQXG1</t>
+          <t>4KPSZD1</t>
         </is>
       </c>
       <c r="I362" t="inlineStr">
@@ -23586,11 +23547,14 @@
       </c>
       <c r="L362" t="inlineStr">
         <is>
-          <t>OptiPlex 755</t>
-        </is>
+          <t>OptiPlex 745</t>
+        </is>
+      </c>
+      <c r="M362" t="n">
+        <v>2</v>
       </c>
       <c r="N362" s="3" t="n">
-        <v>46049.60199074074</v>
+        <v>46072.39605324074</v>
       </c>
       <c r="O362" t="inlineStr">
         <is>
@@ -23601,60 +23565,59 @@
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>PA_258</t>
+          <t>RECEPCAO</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>OPERACAO 9.1</t>
+          <t>ADM/FIN</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>10.69.5.222</t>
-        </is>
-      </c>
-      <c r="D363" t="n">
-        <v>2013</v>
-      </c>
-      <c r="E363" t="n">
-        <v>3913</v>
+          <t>10.69.3.9</t>
+        </is>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t>Microsoft® Windows Vista™ Business</t>
+          <t>Microsoft Windows 11 Pro</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
         <is>
-          <t>4KPSZD1</t>
+          <t>BRJ846Z6GZ</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>Microsoft Office Home and Business 2016 - pt-br</t>
         </is>
       </c>
       <c r="I363" t="inlineStr">
         <is>
-          <t>Intel Core 2 Duo</t>
+          <t>Intel Core i5</t>
         </is>
       </c>
       <c r="J363" t="inlineStr">
         <is>
-          <t>2 GB</t>
+          <t>8 GB</t>
         </is>
       </c>
       <c r="K363" t="inlineStr">
         <is>
-          <t>Dell Inc.</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="L363" t="inlineStr">
         <is>
-          <t>OptiPlex 745</t>
+          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
         </is>
       </c>
       <c r="M363" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N363" s="3" t="n">
-        <v>46072.39605324074</v>
+        <v>46084.48445601852</v>
       </c>
       <c r="O363" t="inlineStr">
         <is>
@@ -23665,18 +23628,24 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>RECEPCAO</t>
+          <t>RESERVA_GERENTE</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>ADM/FIN</t>
+          <t>RESERVA</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>10.69.3.9</t>
-        </is>
+          <t>10.69.2.13</t>
+        </is>
+      </c>
+      <c r="D364" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E364" t="n">
+        <v>26919</v>
       </c>
       <c r="F364" t="inlineStr">
         <is>
@@ -23685,7 +23654,7 @@
       </c>
       <c r="G364" t="inlineStr">
         <is>
-          <t>BRJ846Z6GZ</t>
+          <t>928FPZ2</t>
         </is>
       </c>
       <c r="H364" t="inlineStr">
@@ -23705,19 +23674,16 @@
       </c>
       <c r="K364" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Dell Inc.</t>
         </is>
       </c>
       <c r="L364" t="inlineStr">
         <is>
-          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
-        </is>
-      </c>
-      <c r="M364" t="n">
-        <v>1</v>
+          <t>OptiPlex 3070</t>
+        </is>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46084.36601851852</v>
+        <v>46084.45631944444</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23728,73 +23694,67 @@
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>RESERVA_GERENTE</t>
+          <t>RH_NOTEBOOK</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>RESERVA</t>
+          <t>RH</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>10.69.2.13</t>
-        </is>
-      </c>
-      <c r="D365" t="n">
-        <v>2025</v>
-      </c>
-      <c r="E365" t="n">
-        <v>26919</v>
+          <t>10.69.2.12</t>
+        </is>
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>Microsoft Windows 11 Pro</t>
+          <t>Microsoft Windows 7 Professional</t>
         </is>
       </c>
       <c r="G365" t="inlineStr">
         <is>
-          <t>928FPZ2</t>
-        </is>
-      </c>
-      <c r="H365" t="inlineStr">
-        <is>
-          <t>Microsoft Office Home and Business 2016 - pt-br</t>
+          <t>BRG050GHBZ</t>
         </is>
       </c>
       <c r="I365" t="inlineStr">
         <is>
-          <t>Intel Core i5</t>
+          <t>Intel Core 2 Duo</t>
         </is>
       </c>
       <c r="J365" t="inlineStr">
         <is>
-          <t>8 GB</t>
+          <t>4 GB</t>
         </is>
       </c>
       <c r="K365" t="inlineStr">
         <is>
-          <t>Dell Inc.</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="L365" t="inlineStr">
         <is>
-          <t>OptiPlex 3070</t>
+          <t>HP 420</t>
         </is>
       </c>
       <c r="N365" s="3" t="n">
-        <v>46084.37921296297</v>
+        <v>46002.58769675926</v>
       </c>
       <c r="O365" t="inlineStr">
         <is>
           <t>Ativo</t>
+        </is>
+      </c>
+      <c r="P365" t="inlineStr">
+        <is>
+          <t>RH.03</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>RH_NOTEBOOK</t>
+          <t>RH01</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
@@ -23804,27 +23764,38 @@
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>10.69.2.12</t>
-        </is>
+          <t>10.69.3.11</t>
+        </is>
+      </c>
+      <c r="D366" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E366" t="n">
+        <v>28733</v>
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t>Microsoft Windows 7 Professional</t>
+          <t>Microsoft Windows 11 Pro</t>
         </is>
       </c>
       <c r="G366" t="inlineStr">
         <is>
-          <t>BRG050GHBZ</t>
+          <t>BRJ0057VPH</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>Microsoft Office Standard 2013</t>
         </is>
       </c>
       <c r="I366" t="inlineStr">
         <is>
-          <t>Intel Core 2 Duo</t>
+          <t>Intel Core i5</t>
         </is>
       </c>
       <c r="J366" t="inlineStr">
         <is>
-          <t>4 GB</t>
+          <t>8 GB</t>
         </is>
       </c>
       <c r="K366" t="inlineStr">
@@ -23834,27 +23805,22 @@
       </c>
       <c r="L366" t="inlineStr">
         <is>
-          <t>HP 420</t>
+          <t>HP ProDesk 400 G5 SFF</t>
         </is>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46002.58769675926</v>
+        <v>46084.48251157408</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
           <t>Ativo</t>
-        </is>
-      </c>
-      <c r="P366" t="inlineStr">
-        <is>
-          <t>RH.03</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>RH01</t>
+          <t>RH03</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
@@ -23864,7 +23830,7 @@
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>10.69.3.11</t>
+          <t>10.69.3.13</t>
         </is>
       </c>
       <c r="D367" t="n">
@@ -23880,12 +23846,12 @@
       </c>
       <c r="G367" t="inlineStr">
         <is>
-          <t>BRJ0057VPH</t>
+          <t>BRJ9364TK8</t>
         </is>
       </c>
       <c r="H367" t="inlineStr">
         <is>
-          <t>Microsoft Office Standard 2013</t>
+          <t>Microsoft Office Home and Business 2019 - pt-br</t>
         </is>
       </c>
       <c r="I367" t="inlineStr">
@@ -23909,7 +23875,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46084.36986111111</v>
+        <v>46084.48055555556</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -23920,7 +23886,7 @@
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>RH03</t>
+          <t>RH04</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
@@ -23930,7 +23896,7 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>10.69.3.13</t>
+          <t>10.69.3.14</t>
         </is>
       </c>
       <c r="D368" t="n">
@@ -23946,12 +23912,12 @@
       </c>
       <c r="G368" t="inlineStr">
         <is>
-          <t>BRJ9364TK8</t>
+          <t>BRJ0057VRJ</t>
         </is>
       </c>
       <c r="H368" t="inlineStr">
         <is>
-          <t>Microsoft Office Home and Business 2019 - pt-br</t>
+          <t>Microsoft Office Standard 2013</t>
         </is>
       </c>
       <c r="I368" t="inlineStr">
@@ -23974,8 +23940,11 @@
           <t>HP ProDesk 400 G5 SFF</t>
         </is>
       </c>
+      <c r="M368" t="n">
+        <v>1</v>
+      </c>
       <c r="N368" s="3" t="n">
-        <v>46084.40091435185</v>
+        <v>46084.46662037037</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -23986,7 +23955,7 @@
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>RH04</t>
+          <t>RH05</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
@@ -23996,7 +23965,7 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>10.69.3.14</t>
+          <t>10.69.3.30</t>
         </is>
       </c>
       <c r="D369" t="n">
@@ -24012,7 +23981,7 @@
       </c>
       <c r="G369" t="inlineStr">
         <is>
-          <t>BRJ0057VRJ</t>
+          <t>BRJ843Y4ML</t>
         </is>
       </c>
       <c r="H369" t="inlineStr">
@@ -24037,14 +24006,14 @@
       </c>
       <c r="L369" t="inlineStr">
         <is>
-          <t>HP ProDesk 400 G5 SFF</t>
+          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
         </is>
       </c>
       <c r="M369" t="n">
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46084.38461805556</v>
+        <v>46084.48318287037</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24055,7 +24024,7 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>RH05</t>
+          <t>RH06</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
@@ -24065,7 +24034,7 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>10.69.3.30</t>
+          <t>10.69.3.16</t>
         </is>
       </c>
       <c r="D370" t="n">
@@ -24076,17 +24045,17 @@
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t>Microsoft Windows 11 Pro</t>
+          <t>Windows</t>
         </is>
       </c>
       <c r="G370" t="inlineStr">
         <is>
-          <t>BRJ843Y4ML</t>
+          <t>BRJ0057VPD</t>
         </is>
       </c>
       <c r="H370" t="inlineStr">
         <is>
-          <t>Microsoft Office Standard 2013</t>
+          <t>Microsoft Office Home and Business 2021 - pt-br</t>
         </is>
       </c>
       <c r="I370" t="inlineStr">
@@ -24106,14 +24075,14 @@
       </c>
       <c r="L370" t="inlineStr">
         <is>
-          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
+          <t>HP ProDesk 400 G5 SFF</t>
         </is>
       </c>
       <c r="M370" t="n">
         <v>1</v>
       </c>
       <c r="N370" s="3" t="n">
-        <v>46083.67902777778</v>
+        <v>46076.49737268518</v>
       </c>
       <c r="O370" t="inlineStr">
         <is>
@@ -24124,17 +24093,17 @@
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>RH06</t>
+          <t>saladereuniao</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>RH</t>
+          <t>ADM/FIN</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>10.69.3.16</t>
+          <t>10.69.2.197</t>
         </is>
       </c>
       <c r="D371" t="n">
@@ -24145,12 +24114,12 @@
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t>Windows</t>
+          <t>Microsoft Windows 11 Pro</t>
         </is>
       </c>
       <c r="G371" t="inlineStr">
         <is>
-          <t>BRJ0057VPD</t>
+          <t>BRJ846Z5SX</t>
         </is>
       </c>
       <c r="H371" t="inlineStr">
@@ -24175,14 +24144,14 @@
       </c>
       <c r="L371" t="inlineStr">
         <is>
-          <t>HP ProDesk 400 G5 SFF</t>
+          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
         </is>
       </c>
       <c r="M371" t="n">
         <v>1</v>
       </c>
       <c r="N371" s="3" t="n">
-        <v>46076.49737268518</v>
+        <v>46084.45818287037</v>
       </c>
       <c r="O371" t="inlineStr">
         <is>
@@ -24193,24 +24162,24 @@
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>saladereuniao</t>
+          <t>SANDRA</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>ADM/FIN</t>
+          <t>DIRETORIA</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>10.69.2.197</t>
+          <t>10.69.3.100</t>
         </is>
       </c>
       <c r="D372" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="E372" t="n">
-        <v>28733</v>
+        <v>70623</v>
       </c>
       <c r="F372" t="inlineStr">
         <is>
@@ -24219,7 +24188,7 @@
       </c>
       <c r="G372" t="inlineStr">
         <is>
-          <t>BRJ846Z5SX</t>
+          <t>BRJ208VH2D</t>
         </is>
       </c>
       <c r="H372" t="inlineStr">
@@ -24234,7 +24203,7 @@
       </c>
       <c r="J372" t="inlineStr">
         <is>
-          <t>8 GB</t>
+          <t>16 GB</t>
         </is>
       </c>
       <c r="K372" t="inlineStr">
@@ -24244,14 +24213,14 @@
       </c>
       <c r="L372" t="inlineStr">
         <is>
-          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
+          <t>HP ProDesk 400 G6 Desktop Mini PC</t>
         </is>
       </c>
       <c r="M372" t="n">
         <v>1</v>
       </c>
       <c r="N372" s="3" t="n">
-        <v>46083.58019675926</v>
+        <v>46084.4653587963</v>
       </c>
       <c r="O372" t="inlineStr">
         <is>
@@ -24262,24 +24231,24 @@
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>SANDRA</t>
+          <t>SANTACASA_C01</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>DIRETORIA</t>
+          <t>COORDENACAO</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>10.69.3.100</t>
+          <t>10.69.3.71</t>
         </is>
       </c>
       <c r="D373" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="E373" t="n">
-        <v>70623</v>
+        <v>26919</v>
       </c>
       <c r="F373" t="inlineStr">
         <is>
@@ -24288,12 +24257,12 @@
       </c>
       <c r="G373" t="inlineStr">
         <is>
-          <t>BRJ208VH2D</t>
+          <t>92QLPZ2</t>
         </is>
       </c>
       <c r="H373" t="inlineStr">
         <is>
-          <t>Microsoft Office Home and Business 2021 - pt-br</t>
+          <t>Microsoft Office Home and Business 2016 - pt-br</t>
         </is>
       </c>
       <c r="I373" t="inlineStr">
@@ -24303,24 +24272,21 @@
       </c>
       <c r="J373" t="inlineStr">
         <is>
-          <t>16 GB</t>
+          <t>8 GB</t>
         </is>
       </c>
       <c r="K373" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Dell Inc.</t>
         </is>
       </c>
       <c r="L373" t="inlineStr">
         <is>
-          <t>HP ProDesk 400 G6 Desktop Mini PC</t>
-        </is>
-      </c>
-      <c r="M373" t="n">
-        <v>1</v>
+          <t>OptiPlex 3070</t>
+        </is>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46084.38796296297</v>
+        <v>46084.47947916666</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24331,24 +24297,19 @@
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>SANTACASA_C01</t>
+          <t>SANTACASA_C02</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
           <t>COORDENACAO</t>
-        </is>
-      </c>
-      <c r="C374" t="inlineStr">
-        <is>
-          <t>10.69.3.71</t>
         </is>
       </c>
       <c r="D374" t="n">
         <v>2025</v>
       </c>
       <c r="E374" t="n">
-        <v>26919</v>
+        <v>28733</v>
       </c>
       <c r="F374" t="inlineStr">
         <is>
@@ -24357,12 +24318,12 @@
       </c>
       <c r="G374" t="inlineStr">
         <is>
-          <t>92QLPZ2</t>
+          <t>BRJ843Y6NF</t>
         </is>
       </c>
       <c r="H374" t="inlineStr">
         <is>
-          <t>Microsoft Office Home and Business 2016 - pt-br</t>
+          <t>Microsoft Office Standard 2013</t>
         </is>
       </c>
       <c r="I374" t="inlineStr">
@@ -24377,16 +24338,19 @@
       </c>
       <c r="K374" t="inlineStr">
         <is>
-          <t>Dell Inc.</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="L374" t="inlineStr">
         <is>
-          <t>OptiPlex 3070</t>
-        </is>
+          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
+        </is>
+      </c>
+      <c r="M374" t="n">
+        <v>1</v>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46084.39703703704</v>
+        <v>46084.45347222222</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24397,19 +24361,24 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>SANTACASA_C02</t>
+          <t>SANTACASA_C03</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
           <t>COORDENACAO</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>10.69.3.85</t>
         </is>
       </c>
       <c r="D375" t="n">
         <v>2025</v>
       </c>
       <c r="E375" t="n">
-        <v>28733</v>
+        <v>26383</v>
       </c>
       <c r="F375" t="inlineStr">
         <is>
@@ -24418,12 +24387,12 @@
       </c>
       <c r="G375" t="inlineStr">
         <is>
-          <t>BRJ843Y6NF</t>
+          <t>PE08KTZD</t>
         </is>
       </c>
       <c r="H375" t="inlineStr">
         <is>
-          <t>Microsoft Office Standard 2013</t>
+          <t>Microsoft Office Home and Business 2016 - pt-br</t>
         </is>
       </c>
       <c r="I375" t="inlineStr">
@@ -24438,19 +24407,19 @@
       </c>
       <c r="K375" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>LENOVO</t>
         </is>
       </c>
       <c r="L375" t="inlineStr">
         <is>
-          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
+          <t>11EE0010BO</t>
         </is>
       </c>
       <c r="M375" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46083.81094907408</v>
+        <v>46084.46340277778</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24461,38 +24430,38 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>SANTACASA_C03</t>
+          <t>SIRLENE</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>COORDENACAO</t>
+          <t>GERENCIA</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>10.69.3.85</t>
+          <t>10.69.3.60</t>
         </is>
       </c>
       <c r="D376" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="E376" t="n">
-        <v>26383</v>
+        <v>184</v>
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t>Microsoft Windows 11 Pro</t>
+          <t>Microsoft Windows 10 Pro</t>
         </is>
       </c>
       <c r="G376" t="inlineStr">
         <is>
-          <t>PE08KTZD</t>
+          <t>CKL22H2</t>
         </is>
       </c>
       <c r="H376" t="inlineStr">
         <is>
-          <t>Microsoft Office Home and Business 2016 - pt-br</t>
+          <t>Microsoft Office Home and Business 2021 - pt-br</t>
         </is>
       </c>
       <c r="I376" t="inlineStr">
@@ -24507,90 +24476,21 @@
       </c>
       <c r="K376" t="inlineStr">
         <is>
-          <t>LENOVO</t>
+          <t>Dell Inc.</t>
         </is>
       </c>
       <c r="L376" t="inlineStr">
         <is>
-          <t>11EE0010BO</t>
+          <t>OptiPlex 3040</t>
         </is>
       </c>
       <c r="M376" t="n">
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46084.38780092593</v>
+        <v>46084.46862268518</v>
       </c>
       <c r="O376" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-    </row>
-    <row r="377">
-      <c r="A377" t="inlineStr">
-        <is>
-          <t>SIRLENE</t>
-        </is>
-      </c>
-      <c r="B377" t="inlineStr">
-        <is>
-          <t>GERENCIA</t>
-        </is>
-      </c>
-      <c r="C377" t="inlineStr">
-        <is>
-          <t>10.69.3.60</t>
-        </is>
-      </c>
-      <c r="D377" t="n">
-        <v>2024</v>
-      </c>
-      <c r="E377" t="n">
-        <v>184</v>
-      </c>
-      <c r="F377" t="inlineStr">
-        <is>
-          <t>Microsoft Windows 10 Pro</t>
-        </is>
-      </c>
-      <c r="G377" t="inlineStr">
-        <is>
-          <t>CKL22H2</t>
-        </is>
-      </c>
-      <c r="H377" t="inlineStr">
-        <is>
-          <t>Microsoft Office Home and Business 2021 - pt-br</t>
-        </is>
-      </c>
-      <c r="I377" t="inlineStr">
-        <is>
-          <t>Intel Core i5</t>
-        </is>
-      </c>
-      <c r="J377" t="inlineStr">
-        <is>
-          <t>8 GB</t>
-        </is>
-      </c>
-      <c r="K377" t="inlineStr">
-        <is>
-          <t>Dell Inc.</t>
-        </is>
-      </c>
-      <c r="L377" t="inlineStr">
-        <is>
-          <t>OptiPlex 3040</t>
-        </is>
-      </c>
-      <c r="M377" t="n">
-        <v>2</v>
-      </c>
-      <c r="N377" s="3" t="n">
-        <v>46084.38886574074</v>
-      </c>
-      <c r="O377" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-03 13:52:04.586273
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -434,7 +434,7 @@
   <cols>
     <col width="25.2" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="15.6" customWidth="1" min="3" max="3"/>
+    <col width="32.4" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="10.8" customWidth="1" min="5" max="5"/>
     <col width="50.4" customWidth="1" min="6" max="6"/>
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46084.45994212963</v>
+        <v>46084.53626157407</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46084.47519675926</v>
+        <v>46084.55636574074</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46084.4811574074</v>
+        <v>46084.56199074074</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46084.48472222222</v>
+        <v>46084.56451388889</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1003,7 +1003,7 @@
         <v>1</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>46064.45694444444</v>
+        <v>46084.53652777777</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46084.46375</v>
+        <v>46084.53892361111</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
         <v>1</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>46083.71815972222</v>
+        <v>46084.54775462963</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1382,7 +1382,7 @@
         <v>2</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>46083.73962962963</v>
+        <v>46084.55350694444</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46084.47619212963</v>
+        <v>46084.55378472222</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1510,7 +1510,7 @@
         <v>2</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>46084.4481712963</v>
+        <v>46084.56775462963</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46084.47521990741</v>
+        <v>46084.55902777778</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46084.47832175926</v>
+        <v>46084.55412037037</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1699,7 +1699,7 @@
         </is>
       </c>
       <c r="N19" s="3" t="n">
-        <v>46084.4794675926</v>
+        <v>46084.55335648148</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1763,7 +1763,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46084.46835648148</v>
+        <v>46084.54769675926</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1827,7 +1827,7 @@
         <v>1</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>46083.67512731482</v>
+        <v>46084.555625</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -1905,6 +1905,11 @@
           <t>AUDITORIO</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>10.69.3.146</t>
+        </is>
+      </c>
       <c r="D23" t="n">
         <v>2018</v>
       </c>
@@ -1945,7 +1950,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46084.10149305555</v>
+        <v>46084.55353009259</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2199,7 +2204,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>10.69.3.199</t>
+          <t>fe80::6712:ea57:4fc5:9afc</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -2239,7 +2244,7 @@
         </is>
       </c>
       <c r="N28" s="3" t="n">
-        <v>46083.7340625</v>
+        <v>46084.54215277778</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -6565,7 +6570,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46084.47893518519</v>
+        <v>46084.55263888889</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6634,7 +6639,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46084.47924768519</v>
+        <v>46084.56196759259</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6698,7 +6703,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46084.45207175926</v>
+        <v>46084.52936342593</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6717,11 +6722,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>10.69.3.94</t>
-        </is>
-      </c>
       <c r="D98" t="n">
         <v>2025</v>
       </c>
@@ -6767,7 +6767,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46084.48283564814</v>
+        <v>46084.55922453704</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6836,7 +6836,7 @@
         <v>1</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46084.45454861111</v>
+        <v>46084.53045138889</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
         <v>2</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46084.4808449074</v>
+        <v>46084.55679398148</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6974,7 +6974,7 @@
         <v>1</v>
       </c>
       <c r="N101" s="3" t="n">
-        <v>46084.48162037037</v>
+        <v>46084.56135416667</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -7112,7 +7112,7 @@
         <v>2</v>
       </c>
       <c r="N103" s="3" t="n">
-        <v>46084.46283564815</v>
+        <v>46084.54328703704</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -7239,7 +7239,7 @@
         </is>
       </c>
       <c r="N105" s="3" t="n">
-        <v>46084.48403935185</v>
+        <v>46084.52150462963</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
@@ -7369,7 +7369,7 @@
         <v>1</v>
       </c>
       <c r="N107" s="3" t="n">
-        <v>46084.45972222222</v>
+        <v>46084.5347800926</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -7507,7 +7507,7 @@
         <v>1</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46084.45159722222</v>
+        <v>46084.53240740741</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7576,7 +7576,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46084.4844212963</v>
+        <v>46084.56248842592</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7645,7 +7645,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46084.44476851852</v>
+        <v>46084.56856481481</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7714,7 +7714,7 @@
         <v>2</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46084.47618055555</v>
+        <v>46084.5525462963</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7783,7 +7783,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46084.45440972222</v>
+        <v>46084.5350462963</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7852,7 +7852,7 @@
         <v>1</v>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46084.45828703704</v>
+        <v>46084.53219907408</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7918,7 +7918,7 @@
         </is>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46084.45491898148</v>
+        <v>46084.5375462963</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7987,7 +7987,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46084.48050925926</v>
+        <v>46084.55615740741</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8006,6 +8006,11 @@
           <t>DP</t>
         </is>
       </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>10.69.3.23</t>
+        </is>
+      </c>
       <c r="D117" t="n">
         <v>2025</v>
       </c>
@@ -8051,7 +8056,7 @@
         <v>1</v>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46084.47493055555</v>
+        <v>46084.55233796296</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8117,7 +8122,7 @@
         </is>
       </c>
       <c r="N118" s="3" t="n">
-        <v>46084.44725694445</v>
+        <v>46084.56768518518</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -8255,7 +8260,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46084.45695601852</v>
+        <v>46084.56672453704</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8324,7 +8329,7 @@
         <v>1</v>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46084.47373842593</v>
+        <v>46084.53263888889</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8390,7 +8395,7 @@
         </is>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46084.46833333333</v>
+        <v>46084.54884259259</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8459,7 +8464,7 @@
         <v>2</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46084.4584375</v>
+        <v>46084.53327546296</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8528,7 +8533,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46084.46836805555</v>
+        <v>46084.54887731482</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8597,7 +8602,7 @@
         <v>1</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46084.45269675926</v>
+        <v>46084.57045138889</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8666,7 +8671,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46084.48770833333</v>
+        <v>46084.56605324074</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8735,7 +8740,7 @@
         <v>2</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46084.48043981481</v>
+        <v>46084.5575462963</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8804,7 +8809,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46084.48003472222</v>
+        <v>46084.55532407408</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8905,7 +8910,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Microsoft Windows 11 Pro</t>
+          <t>Windows</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -8942,7 +8947,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46084.45802083334</v>
+        <v>46084.55239583334</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -8961,6 +8966,11 @@
           <t>ADM/FIN</t>
         </is>
       </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>10.69.3.6</t>
+        </is>
+      </c>
       <c r="D131" t="n">
         <v>2025</v>
       </c>
@@ -9006,7 +9016,7 @@
         <v>1</v>
       </c>
       <c r="N131" s="3" t="n">
-        <v>46084.44813657407</v>
+        <v>46084.57</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -9139,7 +9149,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46084.45487268519</v>
+        <v>46084.56994212963</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9458,7 +9468,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46084.4492824074</v>
+        <v>46084.56916666667</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9586,7 +9596,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46084.47428240741</v>
+        <v>46084.55423611111</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9650,7 +9660,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46084.48243055555</v>
+        <v>46084.55796296296</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9714,7 +9724,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46084.47712962963</v>
+        <v>46084.55511574074</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9778,7 +9788,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46084.48739583333</v>
+        <v>46084.56487268519</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9842,7 +9852,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46084.46358796296</v>
+        <v>46084.53789351852</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9906,7 +9916,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46084.47497685185</v>
+        <v>46084.55695601852</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9970,7 +9980,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46084.45216435185</v>
+        <v>46084.57061342592</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10034,7 +10044,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46084.44846064815</v>
+        <v>46084.56730324074</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10098,7 +10108,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46084.46325231482</v>
+        <v>46084.53902777778</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10162,7 +10172,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46084.44732638889</v>
+        <v>46084.5612962963</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10226,7 +10236,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46084.45579861111</v>
+        <v>46084.56896990741</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10290,7 +10300,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46084.45974537037</v>
+        <v>46084.54097222222</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10354,7 +10364,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46084.46193287037</v>
+        <v>46084.54043981482</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10373,11 +10383,6 @@
           <t>OPERACAO 7.1</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>10.69.5.21</t>
-        </is>
-      </c>
       <c r="D153" t="n">
         <v>2018</v>
       </c>
@@ -10482,7 +10487,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46084.47917824074</v>
+        <v>46084.55800925926</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10546,7 +10551,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46084.45664351852</v>
+        <v>46084.56533564815</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10610,7 +10615,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46084.47655092592</v>
+        <v>46084.55778935185</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10674,7 +10679,7 @@
         <v>1</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>46084.44763888889</v>
+        <v>46084.56699074074</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -10738,7 +10743,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46084.449375</v>
+        <v>46084.48856481481</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10802,7 +10807,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46084.45290509259</v>
+        <v>46084.56940972222</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10866,7 +10871,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46084.45821759259</v>
+        <v>46084.54199074074</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10930,7 +10935,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46084.45631944444</v>
+        <v>46084.53627314815</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -10994,7 +10999,7 @@
         <v>1</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46084.45520833333</v>
+        <v>46084.53744212963</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11122,7 +11127,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46084.44950231481</v>
+        <v>46084.56982638889</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11186,7 +11191,7 @@
         <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46084.47953703703</v>
+        <v>46084.55234953704</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11250,7 +11255,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46084.47702546296</v>
+        <v>46084.55423611111</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11314,7 +11319,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46084.46769675926</v>
+        <v>46084.54571759259</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11378,7 +11383,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46084.47059027778</v>
+        <v>46084.54394675926</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11442,7 +11447,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46084.48133101852</v>
+        <v>46084.55652777778</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11506,7 +11511,7 @@
         <v>2</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46084.47875</v>
+        <v>46084.5577662037</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11570,7 +11575,7 @@
         <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46084.48459490741</v>
+        <v>46084.56268518518</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11634,7 +11639,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46083.77778935185</v>
+        <v>46084.54392361111</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11698,7 +11703,7 @@
         <v>1</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46084.47363425926</v>
+        <v>46084.54900462963</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11762,7 +11767,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46084.46461805556</v>
+        <v>46084.54391203704</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11826,7 +11831,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46084.44706018519</v>
+        <v>46084.56537037037</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11890,7 +11895,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46084.45681712963</v>
+        <v>46084.53811342592</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11954,7 +11959,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46083.74231481482</v>
+        <v>46084.54244212963</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12018,7 +12023,7 @@
         <v>2</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46084.48237268518</v>
+        <v>46084.55725694444</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12082,7 +12087,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46084.46047453704</v>
+        <v>46084.53576388889</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12146,7 +12151,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46084.47841435186</v>
+        <v>46084.55798611111</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12210,7 +12215,7 @@
         <v>1</v>
       </c>
       <c r="N181" s="3" t="n">
-        <v>46084.46228009259</v>
+        <v>46084.54640046296</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
@@ -12407,7 +12412,7 @@
         <v>2</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46084.47127314815</v>
+        <v>46084.54423611111</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12471,7 +12476,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46084.46628472222</v>
+        <v>46084.54170138889</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12535,7 +12540,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46084.45608796296</v>
+        <v>46084.53438657407</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12599,7 +12604,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46084.46347222223</v>
+        <v>46084.53822916667</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12663,7 +12668,7 @@
         <v>1</v>
       </c>
       <c r="N188" s="3" t="n">
-        <v>46084.4747337963</v>
+        <v>46084.55128472222</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
@@ -12850,7 +12855,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46084.45084490741</v>
+        <v>46084.56435185186</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12914,7 +12919,7 @@
         <v>1</v>
       </c>
       <c r="N192" s="3" t="n">
-        <v>46084.4844212963</v>
+        <v>46084.5571412037</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
@@ -13039,7 +13044,7 @@
         <v>2</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46084.45653935185</v>
+        <v>46084.5365625</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13103,7 +13108,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46084.45587962963</v>
+        <v>46084.56443287037</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13167,7 +13172,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46084.46653935185</v>
+        <v>46084.54377314815</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13231,7 +13236,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46084.47310185185</v>
+        <v>46084.55396990741</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13295,7 +13300,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46084.47495370371</v>
+        <v>46084.54920138889</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13359,7 +13364,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46084.47648148148</v>
+        <v>46084.55096064815</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13548,7 +13553,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46084.45348379629</v>
+        <v>46084.5674074074</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13612,7 +13617,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46084.44756944444</v>
+        <v>46084.56818287037</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13740,7 +13745,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46084.44983796297</v>
+        <v>46084.56289351852</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13804,7 +13809,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46084.47857638889</v>
+        <v>46084.55335648148</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13868,7 +13873,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46084.46678240741</v>
+        <v>46084.5324537037</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13932,7 +13937,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46084.4687037037</v>
+        <v>46084.54785879629</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -13996,7 +14001,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46084.48320601852</v>
+        <v>46084.56724537037</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14060,7 +14065,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46084.46751157408</v>
+        <v>46084.55126157407</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14124,7 +14129,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46084.47591435185</v>
+        <v>46084.5490625</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14188,7 +14193,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46084.48230324074</v>
+        <v>46084.56410879629</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14252,7 +14257,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46084.463125</v>
+        <v>46084.54432870371</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14316,7 +14321,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46084.47792824074</v>
+        <v>46084.55881944444</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14444,7 +14449,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46084.47603009259</v>
+        <v>46084.55565972222</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14463,6 +14468,11 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>10.69.5.85</t>
+        </is>
+      </c>
       <c r="D217" t="n">
         <v>2017</v>
       </c>
@@ -14503,7 +14513,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46084.47431712963</v>
+        <v>46084.55231481481</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14567,7 +14577,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46084.45945601852</v>
+        <v>46084.53875</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14631,7 +14641,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46084.47719907408</v>
+        <v>46084.55243055556</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14700,7 +14710,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46084.45107638889</v>
+        <v>46084.56266203704</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14764,7 +14774,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46084.4587962963</v>
+        <v>46084.5427662037</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14828,7 +14838,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46084.48608796296</v>
+        <v>46084.56898148148</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14892,7 +14902,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46084.46483796297</v>
+        <v>46084.5403125</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14956,7 +14966,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46084.48034722222</v>
+        <v>46084.56023148148</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15020,7 +15030,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46084.47553240741</v>
+        <v>46084.55552083333</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15048,7 +15058,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46084.47436342593</v>
+        <v>46084.49026620371</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15176,7 +15186,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46084.45503472222</v>
+        <v>46084.53568287037</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15240,7 +15250,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46084.4609837963</v>
+        <v>46084.53940972222</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15304,7 +15314,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46084.48142361111</v>
+        <v>46084.56112268518</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15432,7 +15442,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46083.82859953704</v>
+        <v>46084.54666666667</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15496,7 +15506,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46084.46380787037</v>
+        <v>46084.54428240741</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15560,7 +15570,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46084.46497685185</v>
+        <v>46084.54100694445</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15624,7 +15634,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46084.48364583333</v>
+        <v>46084.5619212963</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15688,7 +15698,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46084.47865740741</v>
+        <v>46084.56092592593</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15752,7 +15762,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46083.82596064815</v>
+        <v>46084.54099537037</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15816,7 +15826,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46084.48350694445</v>
+        <v>46084.56083333334</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15880,7 +15890,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46084.46675925926</v>
+        <v>46084.53917824074</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -15944,7 +15954,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46084.48310185185</v>
+        <v>46084.55976851852</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16008,7 +16018,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46084.48255787037</v>
+        <v>46084.56504629629</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16072,7 +16082,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46084.48081018519</v>
+        <v>46084.55603009259</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16136,7 +16146,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46084.4765162037</v>
+        <v>46084.55357638889</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16451,7 +16461,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46084.45193287037</v>
+        <v>46084.56609953703</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16515,7 +16525,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46084.46100694445</v>
+        <v>46084.53804398148</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16638,7 +16648,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46084.46832175926</v>
+        <v>46084.54769675926</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16766,7 +16776,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46084.46350694444</v>
+        <v>46084.5433912037</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16824,7 +16834,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46084.48052083333</v>
+        <v>46084.55612268519</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16888,7 +16898,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46084.4649537037</v>
+        <v>46084.54491898148</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -16952,7 +16962,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46084.46600694444</v>
+        <v>46084.54293981481</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17016,7 +17026,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46084.47856481482</v>
+        <v>46084.5609375</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17080,7 +17090,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46084.4540625</v>
+        <v>46084.56975694445</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17144,7 +17154,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46084.47333333334</v>
+        <v>46084.54552083334</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17208,7 +17218,7 @@
         <v>1</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46084.48427083333</v>
+        <v>46084.56056712963</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17336,7 +17346,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46084.45271990741</v>
+        <v>46084.5355324074</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17400,7 +17410,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46084.46149305555</v>
+        <v>46084.53746527778</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17464,7 +17474,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46084.46987268519</v>
+        <v>46084.55083333333</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17528,7 +17538,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46084.47915509259</v>
+        <v>46084.55238425926</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17592,7 +17602,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46084.47922453703</v>
+        <v>46084.55293981481</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17656,7 +17666,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46084.47260416667</v>
+        <v>46084.55721064815</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17748,7 +17758,7 @@
         <v>1</v>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46084.4705787037</v>
+        <v>46084.55180555556</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17809,7 +17819,7 @@
         </is>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46084.48637731482</v>
+        <v>46084.56614583333</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -17937,7 +17947,7 @@
         <v>1</v>
       </c>
       <c r="N272" s="3" t="n">
-        <v>46084.46541666667</v>
+        <v>46084.5427199074</v>
       </c>
       <c r="O272" t="inlineStr">
         <is>
@@ -18246,7 +18256,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46084.47275462963</v>
+        <v>46084.55559027778</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18310,7 +18320,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46084.45394675926</v>
+        <v>46084.53206018519</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18374,7 +18384,7 @@
         <v>2</v>
       </c>
       <c r="N279" s="3" t="n">
-        <v>46084.47466435185</v>
+        <v>46084.54678240741</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -18438,7 +18448,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46084.47033564815</v>
+        <v>46084.55424768518</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18561,7 +18571,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46084.4569212963</v>
+        <v>46084.57105324074</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18625,7 +18635,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46084.46337962963</v>
+        <v>46084.54371527778</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18689,7 +18699,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46084.48361111111</v>
+        <v>46084.56181712963</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18708,11 +18718,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C285" t="inlineStr">
-        <is>
-          <t>10.69.5.155</t>
-        </is>
-      </c>
       <c r="D285" t="n">
         <v>2019</v>
       </c>
@@ -18753,7 +18758,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46084.47478009259</v>
+        <v>46084.54824074074</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18817,7 +18822,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46084.47407407407</v>
+        <v>46084.55267361111</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18881,7 +18886,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46084.47958333333</v>
+        <v>46084.55917824074</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -18945,7 +18950,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46084.45835648148</v>
+        <v>46084.53555555556</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19739,7 +19744,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46084.47283564815</v>
+        <v>46084.55357638889</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20855,7 +20860,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46084.45710648148</v>
+        <v>46084.5352662037</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21580,7 +21585,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46084.4819212963</v>
+        <v>46084.55762731482</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21644,7 +21649,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46084.47818287037</v>
+        <v>46084.55891203704</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21708,7 +21713,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46084.47960648148</v>
+        <v>46084.56314814815</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21772,7 +21777,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46084.47329861111</v>
+        <v>46084.54748842592</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21836,7 +21841,7 @@
         <v>1</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46084.47589120371</v>
+        <v>46084.54813657407</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21900,7 +21905,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46084.45230324074</v>
+        <v>46084.53277777778</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -21964,7 +21969,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46084.47204861111</v>
+        <v>46084.54849537037</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22028,7 +22033,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46084.46637731481</v>
+        <v>46084.54984953703</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22092,7 +22097,7 @@
         <v>1</v>
       </c>
       <c r="N339" s="3" t="n">
-        <v>46083.58224537037</v>
+        <v>46084.54840277778</v>
       </c>
       <c r="O339" t="inlineStr">
         <is>
@@ -22156,7 +22161,7 @@
         <v>2</v>
       </c>
       <c r="N340" s="3" t="n">
-        <v>46084.45181712963</v>
+        <v>46084.5294212963</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -22220,7 +22225,7 @@
         <v>2</v>
       </c>
       <c r="N341" s="3" t="n">
-        <v>46084.45305555555</v>
+        <v>46084.56861111111</v>
       </c>
       <c r="O341" t="inlineStr">
         <is>
@@ -22542,7 +22547,7 @@
         <v>1</v>
       </c>
       <c r="N346" s="3" t="n">
-        <v>46084.48739583333</v>
+        <v>46084.56123842593</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -22606,7 +22611,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46084.45409722222</v>
+        <v>46084.53428240741</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22670,7 +22675,7 @@
         <v>1</v>
       </c>
       <c r="N348" s="3" t="n">
-        <v>46084.47803240741</v>
+        <v>46084.55392361111</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -22795,7 +22800,7 @@
         <v>1</v>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46084.47752314815</v>
+        <v>46084.55452546296</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -22859,7 +22864,7 @@
         <v>1</v>
       </c>
       <c r="N351" s="3" t="n">
-        <v>46084.47392361111</v>
+        <v>46084.55200231481</v>
       </c>
       <c r="O351" t="inlineStr">
         <is>
@@ -22984,7 +22989,7 @@
         <v>1</v>
       </c>
       <c r="N353" s="3" t="n">
-        <v>46084.47817129629</v>
+        <v>46084.55304398148</v>
       </c>
       <c r="O353" t="inlineStr">
         <is>
@@ -23048,7 +23053,7 @@
         <v>1</v>
       </c>
       <c r="N354" s="3" t="n">
-        <v>46084.48047453703</v>
+        <v>46084.55783564815</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -23112,7 +23117,7 @@
         <v>1</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46084.47532407408</v>
+        <v>46084.55162037037</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23240,7 +23245,7 @@
         <v>2</v>
       </c>
       <c r="N357" s="3" t="n">
-        <v>46084.47333333334</v>
+        <v>46084.5502662037</v>
       </c>
       <c r="O357" t="inlineStr">
         <is>
@@ -23304,7 +23309,7 @@
         <v>2</v>
       </c>
       <c r="N358" s="3" t="n">
-        <v>46084.47502314814</v>
+        <v>46084.55349537037</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -23368,7 +23373,7 @@
         <v>1</v>
       </c>
       <c r="N359" s="3" t="n">
-        <v>46084.47483796296</v>
+        <v>46084.55512731482</v>
       </c>
       <c r="O359" t="inlineStr">
         <is>
@@ -23617,7 +23622,7 @@
         <v>1</v>
       </c>
       <c r="N363" s="3" t="n">
-        <v>46084.48445601852</v>
+        <v>46084.56158564815</v>
       </c>
       <c r="O363" t="inlineStr">
         <is>
@@ -23683,7 +23688,7 @@
         </is>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46084.45631944444</v>
+        <v>46084.5359837963</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23809,7 +23814,7 @@
         </is>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46084.48251157408</v>
+        <v>46084.56054398148</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
@@ -23828,11 +23833,6 @@
           <t>RH</t>
         </is>
       </c>
-      <c r="C367" t="inlineStr">
-        <is>
-          <t>10.69.3.13</t>
-        </is>
-      </c>
       <c r="D367" t="n">
         <v>2025</v>
       </c>
@@ -23875,7 +23875,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46084.48055555556</v>
+        <v>46084.51951388889</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -23944,7 +23944,7 @@
         <v>1</v>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46084.46662037037</v>
+        <v>46084.54471064815</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24013,7 +24013,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46084.48318287037</v>
+        <v>46084.55831018519</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24220,7 +24220,7 @@
         <v>1</v>
       </c>
       <c r="N372" s="3" t="n">
-        <v>46084.4653587963</v>
+        <v>46084.54274305556</v>
       </c>
       <c r="O372" t="inlineStr">
         <is>
@@ -24286,7 +24286,7 @@
         </is>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46084.47947916666</v>
+        <v>46084.55614583333</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24350,7 +24350,7 @@
         <v>1</v>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46084.45347222222</v>
+        <v>46084.56418981482</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24419,7 +24419,7 @@
         <v>2</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46084.46340277778</v>
+        <v>46084.53665509259</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24488,7 +24488,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46084.46862268518</v>
+        <v>46084.54549768518</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-03 15:52:05.171878
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -434,7 +434,7 @@
   <cols>
     <col width="25.2" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="32.4" customWidth="1" min="3" max="3"/>
+    <col width="15.6" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="10.8" customWidth="1" min="5" max="5"/>
     <col width="50.4" customWidth="1" min="6" max="6"/>
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46084.53626157407</v>
+        <v>46084.65179398148</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46084.55636574074</v>
+        <v>46084.63797453704</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46084.56199074074</v>
+        <v>46084.63909722222</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46084.56451388889</v>
+        <v>46084.64165509259</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1003,7 +1003,7 @@
         <v>1</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>46084.53652777777</v>
+        <v>46084.57743055555</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46084.53892361111</v>
+        <v>46084.64947916667</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
         <v>1</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>46084.54775462963</v>
+        <v>46084.62491898148</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1382,7 +1382,7 @@
         <v>2</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>46084.55350694444</v>
+        <v>46084.63409722222</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46084.55378472222</v>
+        <v>46084.63269675926</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1510,7 +1510,7 @@
         <v>2</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>46084.56775462963</v>
+        <v>46084.64627314815</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46084.55902777778</v>
+        <v>46084.6403587963</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46084.55412037037</v>
+        <v>46084.6340625</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1699,7 +1699,7 @@
         </is>
       </c>
       <c r="N19" s="3" t="n">
-        <v>46084.55335648148</v>
+        <v>46084.62535879629</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1763,7 +1763,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46084.54769675926</v>
+        <v>46084.62231481481</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1827,7 +1827,7 @@
         <v>1</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>46084.555625</v>
+        <v>46084.59372685185</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -1950,7 +1950,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46084.55353009259</v>
+        <v>46084.63277777778</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2009,7 +2009,7 @@
         <v>1</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>46084.10829861111</v>
+        <v>46084.62636574074</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>fe80::6712:ea57:4fc5:9afc</t>
+          <t>10.69.3.199</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -2244,7 +2244,7 @@
         </is>
       </c>
       <c r="N28" s="3" t="n">
-        <v>46084.54215277778</v>
+        <v>46084.62449074074</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -6570,7 +6570,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46084.55263888889</v>
+        <v>46084.63271990741</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6639,7 +6639,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46084.56196759259</v>
+        <v>46084.64145833333</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6658,6 +6658,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>10.69.3.93</t>
+        </is>
+      </c>
       <c r="D97" t="n">
         <v>2025</v>
       </c>
@@ -6703,7 +6708,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46084.52936342593</v>
+        <v>46084.64672453704</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6767,7 +6772,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46084.55922453704</v>
+        <v>46084.6396875</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6836,7 +6841,7 @@
         <v>1</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46084.53045138889</v>
+        <v>46084.64777777778</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6905,7 +6910,7 @@
         <v>2</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46084.55679398148</v>
+        <v>46084.63572916666</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6974,7 +6979,7 @@
         <v>1</v>
       </c>
       <c r="N101" s="3" t="n">
-        <v>46084.56135416667</v>
+        <v>46084.63706018519</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -7112,7 +7117,7 @@
         <v>2</v>
       </c>
       <c r="N103" s="3" t="n">
-        <v>46084.54328703704</v>
+        <v>46084.61751157408</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -7239,7 +7244,7 @@
         </is>
       </c>
       <c r="N105" s="3" t="n">
-        <v>46084.52150462963</v>
+        <v>46084.63201388889</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
@@ -7369,7 +7374,7 @@
         <v>1</v>
       </c>
       <c r="N107" s="3" t="n">
-        <v>46084.5347800926</v>
+        <v>46084.65407407407</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -7507,7 +7512,7 @@
         <v>1</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46084.53240740741</v>
+        <v>46084.61236111111</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7576,7 +7581,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46084.56248842592</v>
+        <v>46084.64046296296</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7645,7 +7650,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46084.56856481481</v>
+        <v>46084.64497685185</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7714,7 +7719,7 @@
         <v>2</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46084.5525462963</v>
+        <v>46084.63141203704</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7783,7 +7788,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46084.5350462963</v>
+        <v>46084.64796296296</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7852,7 +7857,7 @@
         <v>1</v>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46084.53219907408</v>
+        <v>46084.64582175926</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7918,7 +7923,7 @@
         </is>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46084.5375462963</v>
+        <v>46084.61297453703</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7987,7 +7992,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46084.55615740741</v>
+        <v>46084.63143518518</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8006,11 +8011,6 @@
           <t>DP</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>10.69.3.23</t>
-        </is>
-      </c>
       <c r="D117" t="n">
         <v>2025</v>
       </c>
@@ -8056,7 +8056,7 @@
         <v>1</v>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46084.55233796296</v>
+        <v>46084.62761574074</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8122,7 +8122,7 @@
         </is>
       </c>
       <c r="N118" s="3" t="n">
-        <v>46084.56768518518</v>
+        <v>46084.64030092592</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -8260,7 +8260,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46084.56672453704</v>
+        <v>46084.62788194444</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8329,7 +8329,7 @@
         <v>1</v>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46084.53263888889</v>
+        <v>46084.64578703704</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8395,7 +8395,7 @@
         </is>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46084.54884259259</v>
+        <v>46084.63053240741</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8464,7 +8464,7 @@
         <v>2</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46084.53327546296</v>
+        <v>46084.65108796296</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8533,7 +8533,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46084.54887731482</v>
+        <v>46084.63321759259</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8602,7 +8602,7 @@
         <v>1</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46084.57045138889</v>
+        <v>46084.65189814815</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8671,7 +8671,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46084.56605324074</v>
+        <v>46084.64219907407</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8740,7 +8740,7 @@
         <v>2</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46084.5575462963</v>
+        <v>46084.6330787037</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8809,7 +8809,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46084.55532407408</v>
+        <v>46084.63263888889</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8910,7 +8910,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Windows</t>
+          <t>Microsoft Windows 11 Pro</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -8947,7 +8947,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46084.55239583334</v>
+        <v>46084.65101851852</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -8966,11 +8966,6 @@
           <t>ADM/FIN</t>
         </is>
       </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>10.69.3.6</t>
-        </is>
-      </c>
       <c r="D131" t="n">
         <v>2025</v>
       </c>
@@ -9016,7 +9011,7 @@
         <v>1</v>
       </c>
       <c r="N131" s="3" t="n">
-        <v>46084.57</v>
+        <v>46084.64260416666</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -9149,7 +9144,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46084.56994212963</v>
+        <v>46084.61319444444</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9213,7 +9208,7 @@
         <v>1</v>
       </c>
       <c r="N134" s="3" t="n">
-        <v>46083.80149305556</v>
+        <v>46084.62380787037</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -9277,7 +9272,7 @@
         <v>1</v>
       </c>
       <c r="N135" s="3" t="n">
-        <v>46083.8014699074</v>
+        <v>46084.64950231482</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -9468,7 +9463,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46084.56916666667</v>
+        <v>46084.648125</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9532,7 +9527,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46083.81221064815</v>
+        <v>46084.62300925926</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9596,7 +9591,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46084.55423611111</v>
+        <v>46084.63474537037</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9660,7 +9655,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46084.55796296296</v>
+        <v>46084.64946759259</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9724,7 +9719,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46084.55511574074</v>
+        <v>46084.64946759259</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9788,7 +9783,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46084.56487268519</v>
+        <v>46084.64383101852</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9852,7 +9847,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46084.53789351852</v>
+        <v>46084.6499537037</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9916,7 +9911,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46084.55695601852</v>
+        <v>46084.61871527778</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9980,7 +9975,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46084.57061342592</v>
+        <v>46084.62738425926</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10044,7 +10039,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46084.56730324074</v>
+        <v>46084.64734953704</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10108,7 +10103,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46084.53902777778</v>
+        <v>46084.61670138889</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10172,7 +10167,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46084.5612962963</v>
+        <v>46084.63712962963</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10236,7 +10231,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46084.56896990741</v>
+        <v>46084.64741898148</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10300,7 +10295,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46084.54097222222</v>
+        <v>46084.62207175926</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10364,7 +10359,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46084.54043981482</v>
+        <v>46084.6315625</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10383,6 +10378,11 @@
           <t>OPERACAO 7.1</t>
         </is>
       </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>10.69.5.21</t>
+        </is>
+      </c>
       <c r="D153" t="n">
         <v>2018</v>
       </c>
@@ -10423,7 +10423,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46084.47471064814</v>
+        <v>46084.64226851852</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10487,7 +10487,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46084.55800925926</v>
+        <v>46084.62347222222</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10551,7 +10551,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46084.56533564815</v>
+        <v>46084.64686342593</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10807,7 +10807,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46084.56940972222</v>
+        <v>46084.57736111111</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10871,7 +10871,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46084.54199074074</v>
+        <v>46084.6215162037</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10935,7 +10935,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46084.53627314815</v>
+        <v>46084.5746875</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -10999,7 +10999,7 @@
         <v>1</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46084.53744212963</v>
+        <v>46084.6221412037</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11127,7 +11127,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46084.56982638889</v>
+        <v>46084.64280092593</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11191,7 +11191,7 @@
         <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46084.55234953704</v>
+        <v>46084.5908912037</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11255,7 +11255,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46084.55423611111</v>
+        <v>46084.59501157407</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11319,7 +11319,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46084.54571759259</v>
+        <v>46084.58628472222</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11447,7 +11447,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46084.55652777778</v>
+        <v>46084.63078703704</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11511,7 +11511,7 @@
         <v>2</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46084.5577662037</v>
+        <v>46084.63541666666</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11639,7 +11639,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46084.54392361111</v>
+        <v>46084.62689814815</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11703,7 +11703,7 @@
         <v>1</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46084.54900462963</v>
+        <v>46084.62752314815</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11831,7 +11831,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46084.56537037037</v>
+        <v>46084.63898148148</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11895,7 +11895,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46084.53811342592</v>
+        <v>46084.64018518518</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11959,7 +11959,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46084.54244212963</v>
+        <v>46084.62738425926</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12023,7 +12023,7 @@
         <v>2</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46084.55725694444</v>
+        <v>46084.6378125</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12087,7 +12087,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46084.53576388889</v>
+        <v>46084.62989583334</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12151,7 +12151,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46084.55798611111</v>
+        <v>46084.62489583333</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12215,7 +12215,7 @@
         <v>1</v>
       </c>
       <c r="N181" s="3" t="n">
-        <v>46084.54640046296</v>
+        <v>46084.64025462963</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
@@ -12279,7 +12279,7 @@
         <v>1</v>
       </c>
       <c r="N182" s="3" t="n">
-        <v>46066.87270833334</v>
+        <v>46084.64131944445</v>
       </c>
       <c r="O182" t="inlineStr">
         <is>
@@ -12412,7 +12412,7 @@
         <v>2</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46084.54423611111</v>
+        <v>46084.62633101852</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12476,7 +12476,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46084.54170138889</v>
+        <v>46084.61855324074</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12540,7 +12540,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46084.53438657407</v>
+        <v>46084.5819675926</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12604,7 +12604,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46084.53822916667</v>
+        <v>46084.65358796297</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12668,7 +12668,7 @@
         <v>1</v>
       </c>
       <c r="N188" s="3" t="n">
-        <v>46084.55128472222</v>
+        <v>46084.61840277778</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
@@ -12855,7 +12855,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46084.56435185186</v>
+        <v>46084.62164351852</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12919,7 +12919,7 @@
         <v>1</v>
       </c>
       <c r="N192" s="3" t="n">
-        <v>46084.5571412037</v>
+        <v>46084.63074074074</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
@@ -13044,7 +13044,7 @@
         <v>2</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46084.5365625</v>
+        <v>46084.65336805556</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13108,7 +13108,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46084.56443287037</v>
+        <v>46084.64105324074</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13172,7 +13172,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46084.54377314815</v>
+        <v>46084.61965277778</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13236,7 +13236,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46084.55396990741</v>
+        <v>46084.63496527778</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13300,7 +13300,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46084.54920138889</v>
+        <v>46084.62413194445</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13364,7 +13364,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46084.55096064815</v>
+        <v>46084.62016203703</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13553,7 +13553,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46084.5674074074</v>
+        <v>46084.63253472222</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13617,7 +13617,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46084.56818287037</v>
+        <v>46084.62857638889</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13681,7 +13681,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46081.58994212963</v>
+        <v>46084.62711805556</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13745,7 +13745,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46084.56289351852</v>
+        <v>46084.62112268519</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13809,7 +13809,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46084.55335648148</v>
+        <v>46084.6294212963</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13873,7 +13873,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46084.5324537037</v>
+        <v>46084.62268518518</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13937,7 +13937,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46084.54785879629</v>
+        <v>46084.64899305555</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14001,7 +14001,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46084.56724537037</v>
+        <v>46084.65116898148</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14065,7 +14065,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46084.55126157407</v>
+        <v>46084.62732638889</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14129,7 +14129,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46084.5490625</v>
+        <v>46084.61996527778</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14193,7 +14193,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46084.56410879629</v>
+        <v>46084.64239583333</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14257,7 +14257,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46084.54432870371</v>
+        <v>46084.61876157407</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14321,7 +14321,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46084.55881944444</v>
+        <v>46084.63050925926</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14449,7 +14449,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46084.55565972222</v>
+        <v>46084.6156712963</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14468,11 +14468,6 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
-      <c r="C217" t="inlineStr">
-        <is>
-          <t>10.69.5.85</t>
-        </is>
-      </c>
       <c r="D217" t="n">
         <v>2017</v>
       </c>
@@ -14513,7 +14508,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46084.55231481481</v>
+        <v>46084.62876157407</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14577,7 +14572,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46084.53875</v>
+        <v>46084.61866898148</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14641,7 +14636,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46084.55243055556</v>
+        <v>46084.62195601852</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14710,7 +14705,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46084.56266203704</v>
+        <v>46084.64231481482</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14774,7 +14769,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46084.5427662037</v>
+        <v>46084.63615740741</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14838,7 +14833,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46084.56898148148</v>
+        <v>46084.61805555555</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14902,7 +14897,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46084.5403125</v>
+        <v>46084.61509259259</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14966,7 +14961,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46084.56023148148</v>
+        <v>46084.63180555555</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15030,7 +15025,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46084.55552083333</v>
+        <v>46084.63333333333</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15186,7 +15181,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46084.53568287037</v>
+        <v>46084.65284722222</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15250,7 +15245,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46084.53940972222</v>
+        <v>46084.63142361111</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15314,7 +15309,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46084.56112268518</v>
+        <v>46084.62784722223</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15378,7 +15373,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46083.81099537037</v>
+        <v>46084.63090277778</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15442,7 +15437,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46084.54666666667</v>
+        <v>46084.62681712963</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15506,7 +15501,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46084.54428240741</v>
+        <v>46084.64859953704</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15570,7 +15565,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46084.54100694445</v>
+        <v>46084.64997685186</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15634,7 +15629,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46084.5619212963</v>
+        <v>46084.6525</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15698,7 +15693,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46084.56092592593</v>
+        <v>46084.64855324074</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15762,7 +15757,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46084.54099537037</v>
+        <v>46084.62131944444</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15826,7 +15821,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46084.56083333334</v>
+        <v>46084.64678240741</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15954,7 +15949,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46084.55976851852</v>
+        <v>46084.64821759259</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16018,7 +16013,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46084.56504629629</v>
+        <v>46084.63822916667</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16082,7 +16077,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46084.55603009259</v>
+        <v>46084.57545138889</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16146,7 +16141,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46084.55357638889</v>
+        <v>46084.62407407408</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16269,7 +16264,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46083.80362268518</v>
+        <v>46084.65033564815</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16333,7 +16328,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46083.79613425926</v>
+        <v>46084.64703703704</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16397,7 +16392,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46083.8490625</v>
+        <v>46084.62497685185</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16461,7 +16456,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46084.56609953703</v>
+        <v>46084.64971064815</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16525,7 +16520,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46084.53804398148</v>
+        <v>46084.65206018519</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16544,6 +16539,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>10.69.5.118</t>
+        </is>
+      </c>
       <c r="D250" t="n">
         <v>2017</v>
       </c>
@@ -16584,7 +16584,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46083.81512731482</v>
+        <v>46084.64976851852</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16648,7 +16648,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46084.54769675926</v>
+        <v>46084.65074074074</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16712,7 +16712,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46083.80550925926</v>
+        <v>46084.64748842592</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16776,7 +16776,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46084.5433912037</v>
+        <v>46084.65086805556</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16834,7 +16834,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46084.55612268519</v>
+        <v>46084.63016203704</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16898,7 +16898,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46084.54491898148</v>
+        <v>46084.57303240741</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -16962,7 +16962,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46084.54293981481</v>
+        <v>46084.64739583333</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17026,7 +17026,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46084.5609375</v>
+        <v>46084.65105324074</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17090,7 +17090,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46084.56975694445</v>
+        <v>46084.64224537037</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17154,7 +17154,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46084.54552083334</v>
+        <v>46084.62381944444</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17218,7 +17218,7 @@
         <v>1</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46084.56056712963</v>
+        <v>46084.61356481481</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17282,7 +17282,7 @@
         <v>2</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46083.81766203704</v>
+        <v>46084.64952546296</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17346,7 +17346,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46084.5355324074</v>
+        <v>46084.64403935185</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17410,7 +17410,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46084.53746527778</v>
+        <v>46084.62637731482</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17474,7 +17474,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46084.55083333333</v>
+        <v>46084.64634259259</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17538,7 +17538,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46084.55238425926</v>
+        <v>46084.64802083333</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17602,7 +17602,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46084.55293981481</v>
+        <v>46084.63054398148</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17666,7 +17666,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46084.55721064815</v>
+        <v>46084.65321759259</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17691,10 +17691,10 @@
         </is>
       </c>
       <c r="M268" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46084.4190625</v>
+        <v>46084.62229166667</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17758,7 +17758,7 @@
         <v>1</v>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46084.55180555556</v>
+        <v>46084.65399305556</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17819,7 +17819,7 @@
         </is>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46084.56614583333</v>
+        <v>46084.64287037037</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -17883,7 +17883,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46084.48377314815</v>
+        <v>46084.58141203703</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -17947,7 +17947,7 @@
         <v>1</v>
       </c>
       <c r="N272" s="3" t="n">
-        <v>46084.5427199074</v>
+        <v>46084.62925925926</v>
       </c>
       <c r="O272" t="inlineStr">
         <is>
@@ -18256,7 +18256,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46084.55559027778</v>
+        <v>46084.5759375</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18320,7 +18320,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46084.53206018519</v>
+        <v>46084.57668981481</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18384,7 +18384,7 @@
         <v>2</v>
       </c>
       <c r="N279" s="3" t="n">
-        <v>46084.54678240741</v>
+        <v>46084.62021990741</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -18571,7 +18571,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46084.57105324074</v>
+        <v>46084.62394675926</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18635,7 +18635,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46084.54371527778</v>
+        <v>46084.62640046296</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18699,7 +18699,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46084.56181712963</v>
+        <v>46084.64993055556</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18758,7 +18758,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46084.54824074074</v>
+        <v>46084.58883101852</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18822,7 +18822,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46084.55267361111</v>
+        <v>46084.5887037037</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18950,7 +18950,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46084.53555555556</v>
+        <v>46084.64913194445</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19744,7 +19744,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46084.55357638889</v>
+        <v>46084.63288194445</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20860,7 +20860,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46084.5352662037</v>
+        <v>46084.65055555556</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21585,7 +21585,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46084.55762731482</v>
+        <v>46084.63954861111</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21649,7 +21649,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46084.55891203704</v>
+        <v>46084.61785879629</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21713,7 +21713,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46084.56314814815</v>
+        <v>46084.63962962963</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21777,7 +21777,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46084.54748842592</v>
+        <v>46084.62284722222</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21841,7 +21841,7 @@
         <v>1</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46084.54813657407</v>
+        <v>46084.62634259259</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21905,7 +21905,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46084.53277777778</v>
+        <v>46084.61844907407</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -21969,7 +21969,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46084.54849537037</v>
+        <v>46084.62469907408</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22033,7 +22033,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46084.54984953703</v>
+        <v>46084.63118055555</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22161,7 +22161,7 @@
         <v>2</v>
       </c>
       <c r="N340" s="3" t="n">
-        <v>46084.5294212963</v>
+        <v>46084.5715162037</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -22225,7 +22225,7 @@
         <v>2</v>
       </c>
       <c r="N341" s="3" t="n">
-        <v>46084.56861111111</v>
+        <v>46084.64104166667</v>
       </c>
       <c r="O341" t="inlineStr">
         <is>
@@ -22244,11 +22244,6 @@
           <t>OPERACAO 9.1</t>
         </is>
       </c>
-      <c r="C342" t="inlineStr">
-        <is>
-          <t>10.69.5.237</t>
-        </is>
-      </c>
       <c r="D342" t="n">
         <v>2017</v>
       </c>
@@ -22547,7 +22542,7 @@
         <v>1</v>
       </c>
       <c r="N346" s="3" t="n">
-        <v>46084.56123842593</v>
+        <v>46084.59944444444</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -22611,7 +22606,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46084.53428240741</v>
+        <v>46084.57184027778</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22675,7 +22670,7 @@
         <v>1</v>
       </c>
       <c r="N348" s="3" t="n">
-        <v>46084.55392361111</v>
+        <v>46084.59509259259</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -22800,7 +22795,7 @@
         <v>1</v>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46084.55452546296</v>
+        <v>46084.59063657407</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -22864,7 +22859,7 @@
         <v>1</v>
       </c>
       <c r="N351" s="3" t="n">
-        <v>46084.55200231481</v>
+        <v>46084.5928587963</v>
       </c>
       <c r="O351" t="inlineStr">
         <is>
@@ -22989,7 +22984,7 @@
         <v>1</v>
       </c>
       <c r="N353" s="3" t="n">
-        <v>46084.55304398148</v>
+        <v>46084.59024305556</v>
       </c>
       <c r="O353" t="inlineStr">
         <is>
@@ -23053,7 +23048,7 @@
         <v>1</v>
       </c>
       <c r="N354" s="3" t="n">
-        <v>46084.55783564815</v>
+        <v>46084.59422453704</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -23117,7 +23112,7 @@
         <v>1</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46084.55162037037</v>
+        <v>46084.58819444444</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23245,7 +23240,7 @@
         <v>2</v>
       </c>
       <c r="N357" s="3" t="n">
-        <v>46084.5502662037</v>
+        <v>46084.58700231482</v>
       </c>
       <c r="O357" t="inlineStr">
         <is>
@@ -23309,7 +23304,7 @@
         <v>2</v>
       </c>
       <c r="N358" s="3" t="n">
-        <v>46084.55349537037</v>
+        <v>46084.59506944445</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -23373,7 +23368,7 @@
         <v>1</v>
       </c>
       <c r="N359" s="3" t="n">
-        <v>46084.55512731482</v>
+        <v>46084.59331018518</v>
       </c>
       <c r="O359" t="inlineStr">
         <is>
@@ -23622,7 +23617,7 @@
         <v>1</v>
       </c>
       <c r="N363" s="3" t="n">
-        <v>46084.56158564815</v>
+        <v>46084.6366087963</v>
       </c>
       <c r="O363" t="inlineStr">
         <is>
@@ -23688,7 +23683,7 @@
         </is>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46084.5359837963</v>
+        <v>46084.61320601852</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23814,7 +23809,7 @@
         </is>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46084.56054398148</v>
+        <v>46084.63787037037</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
@@ -23833,6 +23828,11 @@
           <t>RH</t>
         </is>
       </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>10.69.3.13</t>
+        </is>
+      </c>
       <c r="D367" t="n">
         <v>2025</v>
       </c>
@@ -23875,7 +23875,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46084.51951388889</v>
+        <v>46084.64761574074</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -23944,7 +23944,7 @@
         <v>1</v>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46084.54471064815</v>
+        <v>46084.61666666667</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24013,7 +24013,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46084.55831018519</v>
+        <v>46084.64164351852</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24151,7 +24151,7 @@
         <v>1</v>
       </c>
       <c r="N371" s="3" t="n">
-        <v>46084.45818287037</v>
+        <v>46084.61623842592</v>
       </c>
       <c r="O371" t="inlineStr">
         <is>
@@ -24220,7 +24220,7 @@
         <v>1</v>
       </c>
       <c r="N372" s="3" t="n">
-        <v>46084.54274305556</v>
+        <v>46084.61542824074</v>
       </c>
       <c r="O372" t="inlineStr">
         <is>
@@ -24286,7 +24286,7 @@
         </is>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46084.55614583333</v>
+        <v>46084.63716435185</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24350,7 +24350,7 @@
         <v>1</v>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46084.56418981482</v>
+        <v>46084.64211805556</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24419,7 +24419,7 @@
         <v>2</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46084.53665509259</v>
+        <v>46084.64980324074</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24488,7 +24488,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46084.54549768518</v>
+        <v>46084.62356481481</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-03 17:52:05.374925
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46084.65179398148</v>
+        <v>46084.7340625</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46084.63797453704</v>
+        <v>46084.71994212963</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46084.63909722222</v>
+        <v>46084.7158449074</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46084.64165509259</v>
+        <v>46084.71923611111</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46084.64947916667</v>
+        <v>46084.72803240741</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
         <v>1</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>46084.62491898148</v>
+        <v>46084.70671296296</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1382,7 +1382,7 @@
         <v>2</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>46084.63409722222</v>
+        <v>46084.71085648148</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46084.63269675926</v>
+        <v>46084.71350694444</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1510,7 +1510,7 @@
         <v>2</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>46084.64627314815</v>
+        <v>46084.72297453704</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46084.6403587963</v>
+        <v>46084.71782407408</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46084.6340625</v>
+        <v>46084.71778935185</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1699,7 +1699,7 @@
         </is>
       </c>
       <c r="N19" s="3" t="n">
-        <v>46084.62535879629</v>
+        <v>46084.73636574074</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1763,7 +1763,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46084.62231481481</v>
+        <v>46084.70476851852</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1950,7 +1950,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46084.63277777778</v>
+        <v>46084.71334490741</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2009,7 +2009,7 @@
         <v>1</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>46084.62636574074</v>
+        <v>46084.70435185185</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2065,7 +2065,7 @@
         </is>
       </c>
       <c r="N25" s="3" t="n">
-        <v>46084.18665509259</v>
+        <v>46084.70383101852</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
         <v>1</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46084.14333333333</v>
+        <v>46084.69106481481</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2244,7 +2244,7 @@
         </is>
       </c>
       <c r="N28" s="3" t="n">
-        <v>46084.62449074074</v>
+        <v>46084.6993287037</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -6570,7 +6570,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46084.63271990741</v>
+        <v>46084.70987268518</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6639,7 +6639,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46084.64145833333</v>
+        <v>46084.71987268519</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6658,11 +6658,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>10.69.3.93</t>
-        </is>
-      </c>
       <c r="D97" t="n">
         <v>2025</v>
       </c>
@@ -6708,7 +6703,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46084.64672453704</v>
+        <v>46084.68247685185</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6772,7 +6767,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46084.6396875</v>
+        <v>46084.68141203704</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6841,7 +6836,7 @@
         <v>1</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46084.64777777778</v>
+        <v>46084.68824074074</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6910,7 +6905,7 @@
         <v>2</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46084.63572916666</v>
+        <v>46084.70936342593</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6979,7 +6974,7 @@
         <v>1</v>
       </c>
       <c r="N101" s="3" t="n">
-        <v>46084.63706018519</v>
+        <v>46084.71241898148</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -7117,7 +7112,7 @@
         <v>2</v>
       </c>
       <c r="N103" s="3" t="n">
-        <v>46084.61751157408</v>
+        <v>46084.69996527778</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -7244,7 +7239,7 @@
         </is>
       </c>
       <c r="N105" s="3" t="n">
-        <v>46084.63201388889</v>
+        <v>46084.67271990741</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
@@ -7374,7 +7369,7 @@
         <v>1</v>
       </c>
       <c r="N107" s="3" t="n">
-        <v>46084.65407407407</v>
+        <v>46084.69407407408</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -7512,7 +7507,7 @@
         <v>1</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46084.61236111111</v>
+        <v>46084.73256944444</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7581,7 +7576,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46084.64046296296</v>
+        <v>46084.71604166667</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7650,7 +7645,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46084.64497685185</v>
+        <v>46084.71994212963</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7719,7 +7714,7 @@
         <v>2</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46084.63141203704</v>
+        <v>46084.71425925926</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7788,7 +7783,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46084.64796296296</v>
+        <v>46084.7231712963</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7857,7 +7852,7 @@
         <v>1</v>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46084.64582175926</v>
+        <v>46084.72351851852</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7923,7 +7918,7 @@
         </is>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46084.61297453703</v>
+        <v>46084.69607638889</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7992,7 +7987,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46084.63143518518</v>
+        <v>46084.70402777778</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8056,7 +8051,7 @@
         <v>1</v>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46084.62761574074</v>
+        <v>46084.66930555556</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8122,7 +8117,7 @@
         </is>
       </c>
       <c r="N118" s="3" t="n">
-        <v>46084.64030092592</v>
+        <v>46084.68075231482</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -8260,7 +8255,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46084.62788194444</v>
+        <v>46084.70650462963</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8329,7 +8324,7 @@
         <v>1</v>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46084.64578703704</v>
+        <v>46084.72274305556</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8395,7 +8390,7 @@
         </is>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46084.63053240741</v>
+        <v>46084.70891203704</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8464,7 +8459,7 @@
         <v>2</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46084.65108796296</v>
+        <v>46084.6883912037</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8533,7 +8528,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46084.63321759259</v>
+        <v>46084.7121412037</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8602,7 +8597,7 @@
         <v>1</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46084.65189814815</v>
+        <v>46084.73438657408</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8671,7 +8666,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46084.64219907407</v>
+        <v>46084.71928240741</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8740,7 +8735,7 @@
         <v>2</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46084.6330787037</v>
+        <v>46084.71221064815</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8809,7 +8804,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46084.63263888889</v>
+        <v>46084.7084375</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -9011,7 +9006,7 @@
         <v>1</v>
       </c>
       <c r="N131" s="3" t="n">
-        <v>46084.64260416666</v>
+        <v>46084.68109953704</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -9144,7 +9139,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46084.61319444444</v>
+        <v>46084.73178240741</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9208,7 +9203,7 @@
         <v>1</v>
       </c>
       <c r="N134" s="3" t="n">
-        <v>46084.62380787037</v>
+        <v>46084.73511574074</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -9272,7 +9267,7 @@
         <v>1</v>
       </c>
       <c r="N135" s="3" t="n">
-        <v>46084.64950231482</v>
+        <v>46084.72638888889</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -9463,7 +9458,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46084.648125</v>
+        <v>46084.70020833334</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9527,7 +9522,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46084.62300925926</v>
+        <v>46084.70015046297</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9591,7 +9586,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46084.63474537037</v>
+        <v>46084.73678240741</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9655,7 +9650,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46084.64946759259</v>
+        <v>46084.72983796296</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9719,7 +9714,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46084.64946759259</v>
+        <v>46084.70268518518</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9783,7 +9778,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46084.64383101852</v>
+        <v>46084.71349537037</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9847,7 +9842,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46084.6499537037</v>
+        <v>46084.72646990741</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9911,7 +9906,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46084.61871527778</v>
+        <v>46084.73363425926</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9975,7 +9970,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46084.62738425926</v>
+        <v>46084.73542824074</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10039,7 +10034,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46084.64734953704</v>
+        <v>46084.72069444445</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10103,7 +10098,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46084.61670138889</v>
+        <v>46084.73320601852</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10167,7 +10162,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46084.63712962963</v>
+        <v>46084.71077546296</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10231,7 +10226,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46084.64741898148</v>
+        <v>46084.72341435185</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10295,7 +10290,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46084.62207175926</v>
+        <v>46084.73681712963</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10359,7 +10354,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46084.6315625</v>
+        <v>46084.70447916666</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10378,11 +10373,6 @@
           <t>OPERACAO 7.1</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>10.69.5.21</t>
-        </is>
-      </c>
       <c r="D153" t="n">
         <v>2018</v>
       </c>
@@ -10487,7 +10477,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46084.62347222222</v>
+        <v>46084.70134259259</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10551,7 +10541,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46084.64686342593</v>
+        <v>46084.72561342592</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10871,7 +10861,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46084.6215162037</v>
+        <v>46084.73623842592</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10999,7 +10989,7 @@
         <v>1</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46084.6221412037</v>
+        <v>46084.69914351852</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11127,7 +11117,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46084.64280092593</v>
+        <v>46084.7236574074</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11447,7 +11437,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46084.63078703704</v>
+        <v>46084.7130787037</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11511,7 +11501,7 @@
         <v>2</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46084.63541666666</v>
+        <v>46084.71605324074</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11639,7 +11629,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46084.62689814815</v>
+        <v>46084.70344907408</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11703,7 +11693,7 @@
         <v>1</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46084.62752314815</v>
+        <v>46084.70138888889</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11831,7 +11821,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46084.63898148148</v>
+        <v>46084.71407407407</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11895,7 +11885,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46084.64018518518</v>
+        <v>46084.655</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11959,7 +11949,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46084.62738425926</v>
+        <v>46084.70141203704</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12023,7 +12013,7 @@
         <v>2</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46084.6378125</v>
+        <v>46084.72828703704</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12087,7 +12077,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46084.62989583334</v>
+        <v>46084.70319444445</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12151,7 +12141,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46084.62489583333</v>
+        <v>46084.70153935185</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12215,7 +12205,7 @@
         <v>1</v>
       </c>
       <c r="N181" s="3" t="n">
-        <v>46084.64025462963</v>
+        <v>46084.73599537037</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
@@ -12279,7 +12269,7 @@
         <v>1</v>
       </c>
       <c r="N182" s="3" t="n">
-        <v>46084.64131944445</v>
+        <v>46084.71942129629</v>
       </c>
       <c r="O182" t="inlineStr">
         <is>
@@ -12412,7 +12402,7 @@
         <v>2</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46084.62633101852</v>
+        <v>46084.70131944444</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12476,7 +12466,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46084.61855324074</v>
+        <v>46084.70056712963</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12604,7 +12594,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46084.65358796297</v>
+        <v>46084.73300925926</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12668,7 +12658,7 @@
         <v>1</v>
       </c>
       <c r="N188" s="3" t="n">
-        <v>46084.61840277778</v>
+        <v>46084.72922453703</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
@@ -12791,7 +12781,7 @@
         </is>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46083.80347222222</v>
+        <v>46084.70726851852</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12855,7 +12845,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46084.62164351852</v>
+        <v>46084.70711805556</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12919,7 +12909,7 @@
         <v>1</v>
       </c>
       <c r="N192" s="3" t="n">
-        <v>46084.63074074074</v>
+        <v>46084.7062962963</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
@@ -13044,7 +13034,7 @@
         <v>2</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46084.65336805556</v>
+        <v>46084.68956018519</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13108,7 +13098,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46084.64105324074</v>
+        <v>46084.7190162037</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13172,7 +13162,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46084.61965277778</v>
+        <v>46084.7322337963</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13236,7 +13226,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46084.63496527778</v>
+        <v>46084.70831018518</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13300,7 +13290,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46084.62413194445</v>
+        <v>46084.70055555556</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13364,7 +13354,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46084.62016203703</v>
+        <v>46084.69864583333</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13553,7 +13543,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46084.63253472222</v>
+        <v>46084.70137731481</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13617,7 +13607,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46084.62857638889</v>
+        <v>46084.70065972222</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13681,7 +13671,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46084.62711805556</v>
+        <v>46084.71023148148</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13745,7 +13735,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46084.62112268519</v>
+        <v>46084.69863425926</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13809,7 +13799,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46084.6294212963</v>
+        <v>46084.73719907407</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13873,7 +13863,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46084.62268518518</v>
+        <v>46084.7359375</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13937,7 +13927,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46084.64899305555</v>
+        <v>46084.70202546296</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14001,7 +13991,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46084.65116898148</v>
+        <v>46084.73460648148</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14065,7 +14055,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46084.62732638889</v>
+        <v>46084.70429398148</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14129,7 +14119,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46084.61996527778</v>
+        <v>46084.73490740741</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14193,7 +14183,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46084.64239583333</v>
+        <v>46084.73600694445</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14257,7 +14247,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46084.61876157407</v>
+        <v>46084.73681712963</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14321,7 +14311,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46084.63050925926</v>
+        <v>46084.70428240741</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14449,7 +14439,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46084.6156712963</v>
+        <v>46084.70471064815</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14468,6 +14458,11 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>10.69.5.85</t>
+        </is>
+      </c>
       <c r="D217" t="n">
         <v>2017</v>
       </c>
@@ -14508,7 +14503,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46084.62876157407</v>
+        <v>46084.70576388889</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14572,7 +14567,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46084.61866898148</v>
+        <v>46084.73538194445</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14636,7 +14631,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46084.62195601852</v>
+        <v>46084.73686342593</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14705,7 +14700,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46084.64231481482</v>
+        <v>46084.71702546296</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14769,7 +14764,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46084.63615740741</v>
+        <v>46084.71858796296</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14833,7 +14828,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46084.61805555555</v>
+        <v>46084.71498842593</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14897,7 +14892,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46084.61509259259</v>
+        <v>46084.73202546296</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14961,7 +14956,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46084.63180555555</v>
+        <v>46084.71864583333</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15025,7 +15020,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46084.63333333333</v>
+        <v>46084.71616898148</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15117,7 +15112,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46083.82641203704</v>
+        <v>46084.71645833334</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15181,7 +15176,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46084.65284722222</v>
+        <v>46084.72597222222</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15245,7 +15240,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46084.63142361111</v>
+        <v>46084.70770833334</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15309,7 +15304,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46084.62784722223</v>
+        <v>46084.70957175926</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15373,7 +15368,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46084.63090277778</v>
+        <v>46084.73361111111</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15437,7 +15432,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46084.62681712963</v>
+        <v>46084.7012962963</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15501,7 +15496,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46084.64859953704</v>
+        <v>46084.72809027778</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15565,7 +15560,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46084.64997685186</v>
+        <v>46084.71321759259</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15629,7 +15624,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46084.6525</v>
+        <v>46084.72913194444</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15693,7 +15688,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46084.64855324074</v>
+        <v>46084.72696759259</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15757,7 +15752,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46084.62131944444</v>
+        <v>46084.70409722222</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15821,7 +15816,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46084.64678240741</v>
+        <v>46084.71928240741</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15949,7 +15944,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46084.64821759259</v>
+        <v>46084.70136574074</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16013,7 +16008,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46084.63822916667</v>
+        <v>46084.71707175926</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16077,7 +16072,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46084.57545138889</v>
+        <v>46084.71057870371</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16141,7 +16136,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46084.62407407408</v>
+        <v>46084.69780092593</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16264,7 +16259,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46084.65033564815</v>
+        <v>46084.73391203704</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16328,7 +16323,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46084.64703703704</v>
+        <v>46084.70244212963</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16456,7 +16451,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46084.64971064815</v>
+        <v>46084.7003125</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16520,7 +16515,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46084.65206018519</v>
+        <v>46084.73631944445</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16584,7 +16579,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46084.64976851852</v>
+        <v>46084.70366898148</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16648,7 +16643,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46084.65074074074</v>
+        <v>46084.70032407407</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16712,7 +16707,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46084.64748842592</v>
+        <v>46084.70291666667</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16776,7 +16771,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46084.65086805556</v>
+        <v>46084.72864583333</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16834,7 +16829,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46084.63016203704</v>
+        <v>46084.70232638889</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16962,7 +16957,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46084.64739583333</v>
+        <v>46084.69696759259</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17026,7 +17021,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46084.65105324074</v>
+        <v>46084.73625</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17090,7 +17085,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46084.64224537037</v>
+        <v>46084.73101851852</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17154,7 +17149,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46084.62381944444</v>
+        <v>46084.73603009259</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17282,7 +17277,7 @@
         <v>2</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46084.64952546296</v>
+        <v>46084.72785879629</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17346,7 +17341,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46084.64403935185</v>
+        <v>46084.72780092592</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17410,7 +17405,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46084.62637731482</v>
+        <v>46084.70733796297</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17474,7 +17469,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46084.64634259259</v>
+        <v>46084.73739583333</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17538,7 +17533,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46084.64802083333</v>
+        <v>46084.72688657408</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17602,7 +17597,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46084.63054398148</v>
+        <v>46084.70686342593</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17666,7 +17661,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46084.65321759259</v>
+        <v>46084.7322337963</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17694,7 +17689,7 @@
         <v>1</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46084.62229166667</v>
+        <v>46084.70123842593</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17758,7 +17753,7 @@
         <v>1</v>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46084.65399305556</v>
+        <v>46084.73265046296</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17819,7 +17814,7 @@
         </is>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46084.64287037037</v>
+        <v>46084.72300925926</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -17947,7 +17942,7 @@
         <v>1</v>
       </c>
       <c r="N272" s="3" t="n">
-        <v>46084.62925925926</v>
+        <v>46084.70734953704</v>
       </c>
       <c r="O272" t="inlineStr">
         <is>
@@ -18384,7 +18379,7 @@
         <v>2</v>
       </c>
       <c r="N279" s="3" t="n">
-        <v>46084.62021990741</v>
+        <v>46084.73751157407</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -18571,7 +18566,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46084.62394675926</v>
+        <v>46084.70259259259</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18635,7 +18630,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46084.62640046296</v>
+        <v>46084.70274305555</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18699,7 +18694,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46084.64993055556</v>
+        <v>46084.70267361111</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18950,7 +18945,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46084.64913194445</v>
+        <v>46084.72401620371</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19744,7 +19739,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46084.63288194445</v>
+        <v>46084.70533564815</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20860,7 +20855,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46084.65055555556</v>
+        <v>46084.72553240741</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21585,7 +21580,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46084.63954861111</v>
+        <v>46084.71914351852</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21649,7 +21644,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46084.61785879629</v>
+        <v>46084.73435185185</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21713,7 +21708,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46084.63962962963</v>
+        <v>46084.72421296296</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21777,7 +21772,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46084.62284722222</v>
+        <v>46084.70204861111</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21841,7 +21836,7 @@
         <v>1</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46084.62634259259</v>
+        <v>46084.70373842592</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21905,7 +21900,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46084.61844907407</v>
+        <v>46084.69863425926</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -21969,7 +21964,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46084.62469907408</v>
+        <v>46084.70438657407</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22033,7 +22028,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46084.63118055555</v>
+        <v>46084.71006944445</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22225,7 +22220,7 @@
         <v>2</v>
       </c>
       <c r="N341" s="3" t="n">
-        <v>46084.64104166667</v>
+        <v>46084.72238425926</v>
       </c>
       <c r="O341" t="inlineStr">
         <is>
@@ -23617,7 +23612,7 @@
         <v>1</v>
       </c>
       <c r="N363" s="3" t="n">
-        <v>46084.6366087963</v>
+        <v>46084.67568287037</v>
       </c>
       <c r="O363" t="inlineStr">
         <is>
@@ -23683,7 +23678,7 @@
         </is>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46084.61320601852</v>
+        <v>46084.73378472222</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23809,7 +23804,7 @@
         </is>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46084.63787037037</v>
+        <v>46084.67604166667</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
@@ -23875,7 +23870,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46084.64761574074</v>
+        <v>46084.68877314815</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -23944,7 +23939,7 @@
         <v>1</v>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46084.61666666667</v>
+        <v>46084.73568287037</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24013,7 +24008,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46084.64164351852</v>
+        <v>46084.71726851852</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24220,7 +24215,7 @@
         <v>1</v>
       </c>
       <c r="N372" s="3" t="n">
-        <v>46084.61542824074</v>
+        <v>46084.73314814815</v>
       </c>
       <c r="O372" t="inlineStr">
         <is>
@@ -24286,7 +24281,7 @@
         </is>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46084.63716435185</v>
+        <v>46084.71969907408</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24305,6 +24300,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>10.69.3.72</t>
+        </is>
+      </c>
       <c r="D374" t="n">
         <v>2025</v>
       </c>
@@ -24350,7 +24350,7 @@
         <v>1</v>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46084.64211805556</v>
+        <v>46084.72045138889</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24419,7 +24419,7 @@
         <v>2</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46084.64980324074</v>
+        <v>46084.68560185185</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24488,7 +24488,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46084.62356481481</v>
+        <v>46084.73591435186</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-04 07:52:04.794822
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46084.7340625</v>
+        <v>46085.3125462963</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46084.71994212963</v>
+        <v>46085.29917824074</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46084.72803240741</v>
+        <v>46085.310625</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46084.71350694444</v>
+        <v>46085.29418981481</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46084.71782407408</v>
+        <v>46085.30907407407</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46084.71778935185</v>
+        <v>46085.01159722222</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1698,8 +1698,11 @@
           <t>HP ProDesk 400 G4 SFF</t>
         </is>
       </c>
+      <c r="M19" t="n">
+        <v>1</v>
+      </c>
       <c r="N19" s="3" t="n">
-        <v>46084.73636574074</v>
+        <v>46085.30429398148</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1763,7 +1766,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46084.70476851852</v>
+        <v>46085.28655092593</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1827,7 +1830,7 @@
         <v>1</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>46084.59372685185</v>
+        <v>46084.74195601852</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -1905,11 +1908,6 @@
           <t>AUDITORIO</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>10.69.3.146</t>
-        </is>
-      </c>
       <c r="D23" t="n">
         <v>2018</v>
       </c>
@@ -1950,7 +1948,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46084.71334490741</v>
+        <v>46085.12164351852</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2009,7 +2007,7 @@
         <v>1</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>46084.70435185185</v>
+        <v>46085.1834837963</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2065,7 +2063,7 @@
         </is>
       </c>
       <c r="N25" s="3" t="n">
-        <v>46084.70383101852</v>
+        <v>46085.21767361111</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2183,7 +2181,7 @@
         <v>1</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46084.69106481481</v>
+        <v>46085.23695601852</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2244,7 +2242,7 @@
         </is>
       </c>
       <c r="N28" s="3" t="n">
-        <v>46084.6993287037</v>
+        <v>46084.74120370371</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -6639,7 +6637,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46084.71987268519</v>
+        <v>46084.79939814815</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6905,7 +6903,7 @@
         <v>2</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46084.70936342593</v>
+        <v>46085.30033564815</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6974,7 +6972,7 @@
         <v>1</v>
       </c>
       <c r="N101" s="3" t="n">
-        <v>46084.71241898148</v>
+        <v>46085.29677083333</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -7112,7 +7110,7 @@
         <v>2</v>
       </c>
       <c r="N103" s="3" t="n">
-        <v>46084.69996527778</v>
+        <v>46085.30434027778</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -7507,7 +7505,7 @@
         <v>1</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46084.73256944444</v>
+        <v>46085.2837037037</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7576,7 +7574,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46084.71604166667</v>
+        <v>46085.29756944445</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7645,7 +7643,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46084.71994212963</v>
+        <v>46085.01371527778</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7714,7 +7712,7 @@
         <v>2</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46084.71425925926</v>
+        <v>46085.29252314815</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7783,7 +7781,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46084.7231712963</v>
+        <v>46085.31100694444</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7852,7 +7850,7 @@
         <v>1</v>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46084.72351851852</v>
+        <v>46085.28453703703</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -8255,7 +8253,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46084.70650462963</v>
+        <v>46085.31106481481</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8324,7 +8322,7 @@
         <v>1</v>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46084.72274305556</v>
+        <v>46084.83710648148</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8459,7 +8457,7 @@
         <v>2</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46084.6883912037</v>
+        <v>46084.85376157407</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8528,7 +8526,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46084.7121412037</v>
+        <v>46085.30335648148</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8597,7 +8595,7 @@
         <v>1</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46084.73438657408</v>
+        <v>46085.30803240741</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8666,7 +8664,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46084.71928240741</v>
+        <v>46084.75626157408</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8735,7 +8733,7 @@
         <v>2</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46084.71221064815</v>
+        <v>46085.28711805555</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8804,7 +8802,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46084.7084375</v>
+        <v>46085.30443287037</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8942,7 +8940,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46084.65101851852</v>
+        <v>46084.92917824074</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9139,7 +9137,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46084.73178240741</v>
+        <v>46084.80613425926</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9203,7 +9201,7 @@
         <v>1</v>
       </c>
       <c r="N134" s="3" t="n">
-        <v>46084.73511574074</v>
+        <v>46084.81542824074</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -9267,7 +9265,7 @@
         <v>1</v>
       </c>
       <c r="N135" s="3" t="n">
-        <v>46084.72638888889</v>
+        <v>46084.80681712963</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -9458,7 +9456,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46084.70020833334</v>
+        <v>46084.81663194444</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9522,7 +9520,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46084.70015046297</v>
+        <v>46084.81265046296</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9586,7 +9584,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46084.73678240741</v>
+        <v>46084.81913194444</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9650,7 +9648,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46084.72983796296</v>
+        <v>46084.81008101852</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9714,7 +9712,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46084.70268518518</v>
+        <v>46084.82069444445</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9778,7 +9776,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46084.71349537037</v>
+        <v>46084.82730324074</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9842,7 +9840,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46084.72646990741</v>
+        <v>46085.32063657408</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9906,7 +9904,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46084.73363425926</v>
+        <v>46084.81273148148</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9970,7 +9968,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46084.73542824074</v>
+        <v>46084.81199074074</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10034,7 +10032,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46084.72069444445</v>
+        <v>46084.80200231481</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10098,7 +10096,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46084.73320601852</v>
+        <v>46084.81372685185</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10162,7 +10160,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46084.71077546296</v>
+        <v>46084.87166666667</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10226,7 +10224,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46084.72341435185</v>
+        <v>46084.83793981482</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10290,7 +10288,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46084.73681712963</v>
+        <v>46084.80939814815</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10354,7 +10352,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46084.70447916666</v>
+        <v>46084.81796296296</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10477,7 +10475,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46084.70134259259</v>
+        <v>46084.82065972222</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10541,7 +10539,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46084.72561342592</v>
+        <v>46084.80572916667</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10605,7 +10603,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46084.55778935185</v>
+        <v>46085.31283564815</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10797,7 +10795,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46084.57736111111</v>
+        <v>46085.31574074074</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10861,7 +10859,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46084.73623842592</v>
+        <v>46084.81574074074</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10989,7 +10987,7 @@
         <v>1</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46084.69914351852</v>
+        <v>46084.82180555556</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11114,10 +11112,10 @@
         </is>
       </c>
       <c r="M164" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46084.7236574074</v>
+        <v>46085.28658564815</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11178,10 +11176,10 @@
         </is>
       </c>
       <c r="M165" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46084.5908912037</v>
+        <v>46085.28603009259</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11437,7 +11435,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46084.7130787037</v>
+        <v>46085.28792824074</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11501,7 +11499,7 @@
         <v>2</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46084.71605324074</v>
+        <v>46084.75481481481</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11629,7 +11627,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46084.70344907408</v>
+        <v>46085.31050925926</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11693,7 +11691,7 @@
         <v>1</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46084.70138888889</v>
+        <v>46085.28960648148</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11821,7 +11819,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46084.71407407407</v>
+        <v>46085.29671296296</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11949,7 +11947,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46084.70141203704</v>
+        <v>46084.73935185185</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12013,7 +12011,7 @@
         <v>2</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46084.72828703704</v>
+        <v>46085.30575231482</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12077,7 +12075,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46084.70319444445</v>
+        <v>46085.31658564815</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12141,7 +12139,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46084.70153935185</v>
+        <v>46085.31553240741</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12205,7 +12203,7 @@
         <v>1</v>
       </c>
       <c r="N181" s="3" t="n">
-        <v>46084.73599537037</v>
+        <v>46084.81405092592</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
@@ -12269,7 +12267,7 @@
         <v>1</v>
       </c>
       <c r="N182" s="3" t="n">
-        <v>46084.71942129629</v>
+        <v>46084.83988425926</v>
       </c>
       <c r="O182" t="inlineStr">
         <is>
@@ -12402,7 +12400,7 @@
         <v>2</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46084.70131944444</v>
+        <v>46085.29689814815</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12466,7 +12464,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46084.70056712963</v>
+        <v>46084.85907407408</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12530,7 +12528,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46084.5819675926</v>
+        <v>46085.10956018518</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12594,7 +12592,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46084.73300925926</v>
+        <v>46085.30211805556</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12658,7 +12656,7 @@
         <v>1</v>
       </c>
       <c r="N188" s="3" t="n">
-        <v>46084.72922453703</v>
+        <v>46085.30408564815</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
@@ -12781,7 +12779,7 @@
         </is>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46084.70726851852</v>
+        <v>46084.82450231481</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12845,7 +12843,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46084.70711805556</v>
+        <v>46084.82268518519</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12909,7 +12907,7 @@
         <v>1</v>
       </c>
       <c r="N192" s="3" t="n">
-        <v>46084.7062962963</v>
+        <v>46085.31737268518</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
@@ -13034,7 +13032,7 @@
         <v>2</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46084.68956018519</v>
+        <v>46084.92119212963</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13098,7 +13096,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46084.7190162037</v>
+        <v>46084.79570601852</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13162,7 +13160,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46084.7322337963</v>
+        <v>46084.81165509259</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13226,7 +13224,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46084.70831018518</v>
+        <v>46084.86335648148</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13290,7 +13288,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46084.70055555556</v>
+        <v>46084.78153935185</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13354,7 +13352,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46084.69864583333</v>
+        <v>46084.81290509259</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13543,7 +13541,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46084.70137731481</v>
+        <v>46084.81636574074</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13607,7 +13605,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46084.70065972222</v>
+        <v>46084.81444444445</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13671,7 +13669,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46084.71023148148</v>
+        <v>46084.82799768518</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13735,7 +13733,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46084.69863425926</v>
+        <v>46084.81918981481</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13799,7 +13797,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46084.73719907407</v>
+        <v>46084.81486111111</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13863,7 +13861,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46084.7359375</v>
+        <v>46084.81097222222</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13927,7 +13925,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46084.70202546296</v>
+        <v>46084.81940972222</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -13991,7 +13989,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46084.73460648148</v>
+        <v>46084.8125462963</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14055,7 +14053,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46084.70429398148</v>
+        <v>46084.85944444445</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14119,7 +14117,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46084.73490740741</v>
+        <v>46085.31115740741</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14183,7 +14181,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46084.73600694445</v>
+        <v>46084.79677083333</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14247,7 +14245,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46084.73681712963</v>
+        <v>46084.77603009259</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14311,7 +14309,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46084.70428240741</v>
+        <v>46085.28641203704</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14439,7 +14437,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46084.70471064815</v>
+        <v>46084.82215277778</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14503,7 +14501,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46084.70576388889</v>
+        <v>46084.81962962963</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14567,7 +14565,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46084.73538194445</v>
+        <v>46084.77405092592</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14631,7 +14629,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46084.73686342593</v>
+        <v>46084.77278935185</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14700,7 +14698,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46084.71702546296</v>
+        <v>46084.75381944444</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14764,7 +14762,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46084.71858796296</v>
+        <v>46084.79633101852</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14828,7 +14826,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46084.71498842593</v>
+        <v>46084.87027777778</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14892,7 +14890,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46084.73202546296</v>
+        <v>46084.8091087963</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14956,7 +14954,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46084.71864583333</v>
+        <v>46084.79832175926</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15020,7 +15018,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46084.71616898148</v>
+        <v>46084.79524305555</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15112,7 +15110,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46084.71645833334</v>
+        <v>46084.86769675926</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15176,7 +15174,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46084.72597222222</v>
+        <v>46084.80356481481</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15240,7 +15238,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46084.70770833334</v>
+        <v>46084.82365740741</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15304,7 +15302,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46084.70957175926</v>
+        <v>46085.32025462963</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15368,7 +15366,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46084.73361111111</v>
+        <v>46084.8115625</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15432,7 +15430,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46084.7012962963</v>
+        <v>46084.82123842592</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15496,7 +15494,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46084.72809027778</v>
+        <v>46084.80726851852</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15560,7 +15558,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46084.71321759259</v>
+        <v>46084.82922453704</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15624,7 +15622,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46084.72913194444</v>
+        <v>46084.76984953704</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15688,7 +15686,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46084.72696759259</v>
+        <v>46084.76861111111</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15752,7 +15750,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46084.70409722222</v>
+        <v>46084.78313657407</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15816,7 +15814,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46084.71928240741</v>
+        <v>46084.79648148148</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15944,7 +15942,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46084.70136574074</v>
+        <v>46084.81277777778</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16008,7 +16006,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46084.71707175926</v>
+        <v>46084.86973379629</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16136,7 +16134,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46084.69780092593</v>
+        <v>46084.80471064815</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16155,6 +16153,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>10.69.5.112</t>
+        </is>
+      </c>
       <c r="D244" t="n">
         <v>2019</v>
       </c>
@@ -16195,7 +16198,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46084.22336805556</v>
+        <v>46085.26280092593</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16259,7 +16262,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46084.73391203704</v>
+        <v>46084.81222222222</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16323,7 +16326,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46084.70244212963</v>
+        <v>46084.82435185185</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16451,7 +16454,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46084.7003125</v>
+        <v>46084.81915509259</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16515,7 +16518,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46084.73631944445</v>
+        <v>46085.32072916667</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16579,7 +16582,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46084.70366898148</v>
+        <v>46085.32045138889</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16643,7 +16646,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46084.70032407407</v>
+        <v>46085.32072916667</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16707,7 +16710,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46084.70291666667</v>
+        <v>46085.32070601852</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16771,7 +16774,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46084.72864583333</v>
+        <v>46085.31559027778</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16829,7 +16832,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46084.70232638889</v>
+        <v>46085.31554398148</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16893,7 +16896,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46084.57303240741</v>
+        <v>46085.31518518519</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -16957,7 +16960,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46084.69696759259</v>
+        <v>46085.31555555556</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17021,7 +17024,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46084.73625</v>
+        <v>46085.31605324074</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17085,7 +17088,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46084.73101851852</v>
+        <v>46084.80836805556</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17149,7 +17152,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46084.73603009259</v>
+        <v>46085.31915509259</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17213,7 +17216,7 @@
         <v>1</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46084.61356481481</v>
+        <v>46085.31600694444</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17277,7 +17280,7 @@
         <v>2</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46084.72785879629</v>
+        <v>46084.80190972222</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17341,7 +17344,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46084.72780092592</v>
+        <v>46084.80199074074</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17405,7 +17408,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46084.70733796297</v>
+        <v>46084.82236111111</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17469,7 +17472,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46084.73739583333</v>
+        <v>46084.81611111111</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17533,7 +17536,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46084.72688657408</v>
+        <v>46084.80579861111</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17597,7 +17600,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46084.70686342593</v>
+        <v>46084.85935185185</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17661,7 +17664,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46084.7322337963</v>
+        <v>46084.80972222222</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17689,7 +17692,7 @@
         <v>1</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46084.70123842593</v>
+        <v>46084.7815162037</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17753,7 +17756,7 @@
         <v>1</v>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46084.73265046296</v>
+        <v>46084.81061342593</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17814,7 +17817,7 @@
         </is>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46084.72300925926</v>
+        <v>46085.31078703704</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -17878,7 +17881,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46084.58141203703</v>
+        <v>46085.09553240741</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -17942,7 +17945,7 @@
         <v>1</v>
       </c>
       <c r="N272" s="3" t="n">
-        <v>46084.70734953704</v>
+        <v>46084.82542824074</v>
       </c>
       <c r="O272" t="inlineStr">
         <is>
@@ -18315,7 +18318,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46084.57668981481</v>
+        <v>46085.30277777778</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18379,7 +18382,7 @@
         <v>2</v>
       </c>
       <c r="N279" s="3" t="n">
-        <v>46084.73751157407</v>
+        <v>46084.85930555555</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -18566,7 +18569,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46084.70259259259</v>
+        <v>46084.82059027778</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18630,7 +18633,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46084.70274305555</v>
+        <v>46084.81574074074</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18694,7 +18697,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46084.70267361111</v>
+        <v>46084.81486111111</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18753,7 +18756,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46084.58883101852</v>
+        <v>46085.11266203703</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18817,7 +18820,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46084.5887037037</v>
+        <v>46085.13469907407</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18881,7 +18884,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46084.55917824074</v>
+        <v>46085.31564814815</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -18945,7 +18948,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46084.72401620371</v>
+        <v>46084.84157407407</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19739,7 +19742,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46084.70533564815</v>
+        <v>46085.29853009259</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20855,7 +20858,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46084.72553240741</v>
+        <v>46085.31021990741</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21644,7 +21647,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46084.73435185185</v>
+        <v>46085.28693287037</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21708,7 +21711,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46084.72421296296</v>
+        <v>46085.28792824074</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21772,7 +21775,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46084.70204861111</v>
+        <v>46085.28710648148</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21836,7 +21839,7 @@
         <v>1</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46084.70373842592</v>
+        <v>46085.29605324074</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21900,7 +21903,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46084.69863425926</v>
+        <v>46085.28725694444</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -21964,7 +21967,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46084.70438657407</v>
+        <v>46085.28715277778</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22028,7 +22031,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46084.71006944445</v>
+        <v>46085.29231481482</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22220,7 +22223,7 @@
         <v>2</v>
       </c>
       <c r="N341" s="3" t="n">
-        <v>46084.72238425926</v>
+        <v>46085.30392361111</v>
       </c>
       <c r="O341" t="inlineStr">
         <is>
@@ -23678,7 +23681,7 @@
         </is>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46084.73378472222</v>
+        <v>46085.31840277778</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23804,7 +23807,7 @@
         </is>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46084.67604166667</v>
+        <v>46085.32060185185</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
@@ -23939,7 +23942,7 @@
         <v>1</v>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46084.73568287037</v>
+        <v>46085.31896990741</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24008,7 +24011,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46084.71726851852</v>
+        <v>46085.29189814815</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24281,7 +24284,7 @@
         </is>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46084.71969907408</v>
+        <v>46085.29534722222</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24350,7 +24353,7 @@
         <v>1</v>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46084.72045138889</v>
+        <v>46084.79833333333</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24419,7 +24422,7 @@
         <v>2</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46084.68560185185</v>
+        <v>46085.3172337963</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24488,7 +24491,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46084.73591435186</v>
+        <v>46085.3170949074</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-04 09:52:05.499620
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46085.3125462963</v>
+        <v>46085.38731481481</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46085.29917824074</v>
+        <v>46085.37306712963</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46084.7158449074</v>
+        <v>46085.3909375</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46084.71923611111</v>
+        <v>46085.36627314815</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46085.310625</v>
+        <v>46085.39146990741</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46085.29418981481</v>
+        <v>46085.37457175926</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46085.30907407407</v>
+        <v>46085.38403935185</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46085.01159722222</v>
+        <v>46085.4044212963</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1678,6 +1678,11 @@
           <t>BRJ748LCMY</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Microsoft Office Standard 2013</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>Intel Core i5</t>
@@ -1702,7 +1707,7 @@
         <v>1</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>46085.30429398148</v>
+        <v>46085.38184027778</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1766,7 +1771,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46085.28655092593</v>
+        <v>46085.39890046296</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -6568,7 +6573,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46084.70987268518</v>
+        <v>46085.3984837963</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6656,6 +6661,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>10.69.3.93</t>
+        </is>
+      </c>
       <c r="D97" t="n">
         <v>2025</v>
       </c>
@@ -6701,7 +6711,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46084.68247685185</v>
+        <v>46085.39797453704</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6834,7 +6844,7 @@
         <v>1</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46084.68824074074</v>
+        <v>46085.38689814815</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6903,7 +6913,7 @@
         <v>2</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46085.30033564815</v>
+        <v>46085.38328703704</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6972,7 +6982,7 @@
         <v>1</v>
       </c>
       <c r="N101" s="3" t="n">
-        <v>46085.29677083333</v>
+        <v>46085.37409722222</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -7110,7 +7120,7 @@
         <v>2</v>
       </c>
       <c r="N103" s="3" t="n">
-        <v>46085.30434027778</v>
+        <v>46085.38104166667</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -7367,7 +7377,7 @@
         <v>1</v>
       </c>
       <c r="N107" s="3" t="n">
-        <v>46084.69407407408</v>
+        <v>46085.37313657408</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -7505,7 +7515,7 @@
         <v>1</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46085.2837037037</v>
+        <v>46085.36427083334</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7574,7 +7584,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46085.29756944445</v>
+        <v>46085.3747337963</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7643,7 +7653,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46085.01371527778</v>
+        <v>46085.37996527777</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7712,7 +7722,7 @@
         <v>2</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46085.29252314815</v>
+        <v>46085.37673611111</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7781,7 +7791,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46085.31100694444</v>
+        <v>46085.39090277778</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7850,7 +7860,7 @@
         <v>1</v>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46085.28453703703</v>
+        <v>46085.39939814815</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7916,7 +7926,7 @@
         </is>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46084.69607638889</v>
+        <v>46085.38157407408</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7985,7 +7995,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46084.70402777778</v>
+        <v>46085.37252314815</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8049,7 +8059,7 @@
         <v>1</v>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46084.66930555556</v>
+        <v>46085.36538194444</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8115,7 +8125,7 @@
         </is>
       </c>
       <c r="N118" s="3" t="n">
-        <v>46084.68075231482</v>
+        <v>46085.37939814815</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -8253,7 +8263,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46085.31106481481</v>
+        <v>46085.39150462963</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8388,7 +8398,7 @@
         </is>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46084.70891203704</v>
+        <v>46085.37375</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8526,7 +8536,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46085.30335648148</v>
+        <v>46085.38311342592</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8595,7 +8605,7 @@
         <v>1</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46085.30803240741</v>
+        <v>46085.38410879629</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8664,7 +8674,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46084.75626157408</v>
+        <v>46085.38239583333</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8733,7 +8743,7 @@
         <v>2</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46085.28711805555</v>
+        <v>46085.39871527778</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8802,7 +8812,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46085.30443287037</v>
+        <v>46085.38106481481</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8871,7 +8881,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46081.63077546296</v>
+        <v>46085.37274305556</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -9004,7 +9014,7 @@
         <v>1</v>
       </c>
       <c r="N131" s="3" t="n">
-        <v>46084.68109953704</v>
+        <v>46085.38537037037</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -9201,7 +9211,7 @@
         <v>1</v>
       </c>
       <c r="N134" s="3" t="n">
-        <v>46084.81542824074</v>
+        <v>46085.37296296296</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -9456,7 +9466,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46084.81663194444</v>
+        <v>46085.37711805556</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9648,7 +9658,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46084.81008101852</v>
+        <v>46085.36497685185</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9712,7 +9722,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46084.82069444445</v>
+        <v>46085.37613425926</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9776,7 +9786,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46084.82730324074</v>
+        <v>46085.37666666666</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9840,7 +9850,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46085.32063657408</v>
+        <v>46085.39590277777</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9904,7 +9914,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46084.81273148148</v>
+        <v>46085.37509259259</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9968,7 +9978,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46084.81199074074</v>
+        <v>46085.36604166667</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10032,7 +10042,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46084.80200231481</v>
+        <v>46085.39394675926</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10096,7 +10106,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46084.81372685185</v>
+        <v>46085.38582175926</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10160,7 +10170,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46084.87166666667</v>
+        <v>46085.37581018519</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10224,7 +10234,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46084.83793981482</v>
+        <v>46085.38037037037</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10288,7 +10298,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46084.80939814815</v>
+        <v>46085.37833333333</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10352,7 +10362,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46084.81796296296</v>
+        <v>46085.3771875</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10475,7 +10485,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46084.82065972222</v>
+        <v>46085.36856481482</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10539,7 +10549,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46084.80572916667</v>
+        <v>46085.37017361111</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10603,7 +10613,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46085.31283564815</v>
+        <v>46085.39233796296</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10667,7 +10677,7 @@
         <v>1</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>46084.56699074074</v>
+        <v>46085.37024305556</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -10731,7 +10741,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46084.48856481481</v>
+        <v>46085.36972222223</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10795,7 +10805,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46085.31574074074</v>
+        <v>46085.39327546296</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10859,7 +10869,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46084.81574074074</v>
+        <v>46085.37086805556</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10923,7 +10933,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46084.5746875</v>
+        <v>46085.37612268519</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -10987,7 +10997,7 @@
         <v>1</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46084.82180555556</v>
+        <v>46085.37686342592</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11051,7 +11061,7 @@
         <v>2</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46079.55581018519</v>
+        <v>46085.33334490741</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11112,10 +11122,10 @@
         </is>
       </c>
       <c r="M164" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46085.28658564815</v>
+        <v>46085.39973379629</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11176,10 +11186,10 @@
         </is>
       </c>
       <c r="M165" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46085.28603009259</v>
+        <v>46085.40079861111</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11243,7 +11253,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46084.59501157407</v>
+        <v>46085.37339120371</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11307,7 +11317,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46084.58628472222</v>
+        <v>46085.36719907408</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11371,7 +11381,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46084.54394675926</v>
+        <v>46085.3678125</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11435,7 +11445,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46085.28792824074</v>
+        <v>46085.39971064815</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11499,7 +11509,7 @@
         <v>2</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46084.75481481481</v>
+        <v>46085.36356481481</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11560,10 +11570,10 @@
         </is>
       </c>
       <c r="M171" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46084.56268518518</v>
+        <v>46085.36994212963</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11688,10 +11698,10 @@
         </is>
       </c>
       <c r="M173" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46085.28960648148</v>
+        <v>46085.37086805556</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11755,7 +11765,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46084.54391203704</v>
+        <v>46085.37001157407</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11819,7 +11829,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46085.29671296296</v>
+        <v>46085.36817129629</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -12011,7 +12021,7 @@
         <v>2</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46085.30575231482</v>
+        <v>46085.3768287037</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12075,7 +12085,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46085.31658564815</v>
+        <v>46085.39201388889</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12139,7 +12149,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46085.31553240741</v>
+        <v>46085.38697916667</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12400,7 +12410,7 @@
         <v>2</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46085.29689814815</v>
+        <v>46085.37300925926</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12528,7 +12538,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46085.10956018518</v>
+        <v>46085.34899305556</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12592,7 +12602,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46085.30211805556</v>
+        <v>46085.38361111111</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12656,7 +12666,7 @@
         <v>1</v>
       </c>
       <c r="N188" s="3" t="n">
-        <v>46085.30408564815</v>
+        <v>46085.38134259259</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
@@ -12742,6 +12752,11 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>10.69.5.59</t>
+        </is>
+      </c>
       <c r="D190" t="n">
         <v>2015</v>
       </c>
@@ -12779,7 +12794,7 @@
         </is>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46084.82450231481</v>
+        <v>46085.38929398148</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12843,7 +12858,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46084.82268518519</v>
+        <v>46085.39484953704</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12907,7 +12922,7 @@
         <v>1</v>
       </c>
       <c r="N192" s="3" t="n">
-        <v>46085.31737268518</v>
+        <v>46085.39746527778</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
@@ -13032,7 +13047,7 @@
         <v>2</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46084.92119212963</v>
+        <v>46085.38453703704</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13096,7 +13111,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46084.79570601852</v>
+        <v>46085.38813657407</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13160,7 +13175,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46084.81165509259</v>
+        <v>46085.37743055556</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13224,7 +13239,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46084.86335648148</v>
+        <v>46085.38818287037</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13288,7 +13303,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46084.78153935185</v>
+        <v>46085.36961805556</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13352,7 +13367,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46084.81290509259</v>
+        <v>46085.39048611111</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13541,7 +13556,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46084.81636574074</v>
+        <v>46085.37369212963</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13605,7 +13620,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46084.81444444445</v>
+        <v>46085.38291666667</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13669,7 +13684,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46084.82799768518</v>
+        <v>46085.3872337963</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13733,7 +13748,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46084.81918981481</v>
+        <v>46085.36693287037</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13797,7 +13812,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46084.81486111111</v>
+        <v>46085.39599537037</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13861,7 +13876,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46084.81097222222</v>
+        <v>46085.40325231481</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13925,7 +13940,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46084.81940972222</v>
+        <v>46085.38457175926</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -13989,7 +14004,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46084.8125462963</v>
+        <v>46085.37939814815</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14053,7 +14068,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46084.85944444445</v>
+        <v>46085.37394675926</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14117,7 +14132,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46085.31115740741</v>
+        <v>46085.38875</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14181,7 +14196,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46084.79677083333</v>
+        <v>46085.37271990741</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14245,7 +14260,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46084.77603009259</v>
+        <v>46085.38989583333</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14309,7 +14324,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46085.28641203704</v>
+        <v>46085.32649305555</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14437,7 +14452,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46084.82215277778</v>
+        <v>46085.37486111111</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14501,7 +14516,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46084.81962962963</v>
+        <v>46085.37586805555</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14565,7 +14580,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46084.77405092592</v>
+        <v>46085.37207175926</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14629,7 +14644,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46084.77278935185</v>
+        <v>46085.39956018519</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14698,7 +14713,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46084.75381944444</v>
+        <v>46085.37145833333</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14762,7 +14777,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46084.79633101852</v>
+        <v>46085.37144675926</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14826,7 +14841,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46084.87027777778</v>
+        <v>46085.38333333333</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14954,7 +14969,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46084.79832175926</v>
+        <v>46085.38181712963</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15018,7 +15033,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46084.79524305555</v>
+        <v>46085.36686342592</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15174,7 +15189,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46084.80356481481</v>
+        <v>46085.38082175926</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15238,7 +15253,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46084.82365740741</v>
+        <v>46085.40123842593</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15302,7 +15317,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46085.32025462963</v>
+        <v>46085.39646990741</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15366,7 +15381,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46084.8115625</v>
+        <v>46085.39118055555</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15430,7 +15445,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46084.82123842592</v>
+        <v>46085.36945601852</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15494,7 +15509,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46084.80726851852</v>
+        <v>46085.37436342592</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15558,7 +15573,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46084.82922453704</v>
+        <v>46085.38288194445</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15622,7 +15637,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46084.76984953704</v>
+        <v>46085.3699537037</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15686,7 +15701,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46084.76861111111</v>
+        <v>46085.38930555555</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15750,7 +15765,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46084.78313657407</v>
+        <v>46085.3699537037</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15814,7 +15829,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46084.79648148148</v>
+        <v>46085.38697916667</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15878,7 +15893,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46084.53917824074</v>
+        <v>46085.37069444444</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -15942,7 +15957,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46084.81277777778</v>
+        <v>46085.37309027778</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16070,7 +16085,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46084.71057870371</v>
+        <v>46085.40040509259</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16134,7 +16149,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46084.80471064815</v>
+        <v>46085.38100694444</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16153,11 +16168,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C244" t="inlineStr">
-        <is>
-          <t>10.69.5.112</t>
-        </is>
-      </c>
       <c r="D244" t="n">
         <v>2019</v>
       </c>
@@ -16262,7 +16272,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46084.81222222222</v>
+        <v>46085.39841435185</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16326,7 +16336,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46084.82435185185</v>
+        <v>46085.39942129629</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16390,7 +16400,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46084.62497685185</v>
+        <v>46085.40049768519</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16454,7 +16464,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46084.81915509259</v>
+        <v>46085.37971064815</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16518,7 +16528,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46085.32072916667</v>
+        <v>46085.39980324074</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16582,7 +16592,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46085.32045138889</v>
+        <v>46085.39946759259</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16646,7 +16656,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46085.32072916667</v>
+        <v>46085.39891203704</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16710,7 +16720,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46085.32070601852</v>
+        <v>46085.40157407407</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16774,7 +16784,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46085.31559027778</v>
+        <v>46085.39523148148</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16832,7 +16842,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46085.31554398148</v>
+        <v>46085.39219907407</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16896,7 +16906,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46085.31518518519</v>
+        <v>46085.39604166667</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -16960,7 +16970,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46085.31555555556</v>
+        <v>46085.39351851852</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17024,7 +17034,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46085.31605324074</v>
+        <v>46085.39335648148</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17088,7 +17098,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46084.80836805556</v>
+        <v>46085.39840277778</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17152,7 +17162,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46085.31915509259</v>
+        <v>46085.39126157408</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17216,7 +17226,7 @@
         <v>1</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46085.31600694444</v>
+        <v>46085.39809027778</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17344,7 +17354,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46084.80199074074</v>
+        <v>46085.3787962963</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17408,7 +17418,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46084.82236111111</v>
+        <v>46085.37296296296</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17472,7 +17482,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46084.81611111111</v>
+        <v>46085.37842592593</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17536,7 +17546,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46084.80579861111</v>
+        <v>46085.36871527778</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17600,7 +17610,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46084.85935185185</v>
+        <v>46085.36858796296</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17664,7 +17674,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46084.80972222222</v>
+        <v>46085.37315972222</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17817,7 +17827,7 @@
         </is>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46085.31078703704</v>
+        <v>46085.3927662037</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -17945,7 +17955,7 @@
         <v>1</v>
       </c>
       <c r="N272" s="3" t="n">
-        <v>46084.82542824074</v>
+        <v>46085.38119212963</v>
       </c>
       <c r="O272" t="inlineStr">
         <is>
@@ -18254,7 +18264,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46084.5759375</v>
+        <v>46085.40193287037</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18318,7 +18328,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46085.30277777778</v>
+        <v>46085.38519675926</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18337,11 +18347,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C279" t="inlineStr">
-        <is>
-          <t>10.69.5.149</t>
-        </is>
-      </c>
       <c r="D279" t="n">
         <v>2014</v>
       </c>
@@ -18382,7 +18387,7 @@
         <v>2</v>
       </c>
       <c r="N279" s="3" t="n">
-        <v>46084.85930555555</v>
+        <v>46085.38045138889</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -18446,7 +18451,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46084.55424768518</v>
+        <v>46085.3771875</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18505,7 +18510,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46083.55935185185</v>
+        <v>46085.38430555556</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18569,7 +18574,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46084.82059027778</v>
+        <v>46085.40086805556</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18633,7 +18638,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46084.81574074074</v>
+        <v>46085.37141203704</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18697,7 +18702,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46084.81486111111</v>
+        <v>46085.37112268519</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18716,6 +18721,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>10.69.5.155</t>
+        </is>
+      </c>
       <c r="D285" t="n">
         <v>2019</v>
       </c>
@@ -18756,7 +18766,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46085.11266203703</v>
+        <v>46085.39684027778</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18820,7 +18830,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46085.13469907407</v>
+        <v>46085.37947916667</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18884,7 +18894,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46085.31564814815</v>
+        <v>46085.39148148148</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19742,7 +19752,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46085.29853009259</v>
+        <v>46085.37489583333</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20858,7 +20868,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46085.31021990741</v>
+        <v>46085.38627314815</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21583,7 +21593,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46084.71914351852</v>
+        <v>46085.3783912037</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21647,7 +21657,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46085.28693287037</v>
+        <v>46085.39655092593</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21711,7 +21721,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46085.28792824074</v>
+        <v>46085.40267361111</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21775,7 +21785,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46085.28710648148</v>
+        <v>46085.36879629629</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21839,7 +21849,7 @@
         <v>1</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46085.29605324074</v>
+        <v>46085.37380787037</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21903,7 +21913,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46085.28725694444</v>
+        <v>46085.39925925926</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -21967,7 +21977,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46085.28715277778</v>
+        <v>46085.40325231481</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22031,7 +22041,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46085.29231481482</v>
+        <v>46085.40415509259</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22159,7 +22169,7 @@
         <v>2</v>
       </c>
       <c r="N340" s="3" t="n">
-        <v>46084.5715162037</v>
+        <v>46085.37563657408</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -22223,7 +22233,7 @@
         <v>2</v>
       </c>
       <c r="N341" s="3" t="n">
-        <v>46085.30392361111</v>
+        <v>46085.3822337963</v>
       </c>
       <c r="O341" t="inlineStr">
         <is>
@@ -23366,7 +23376,7 @@
         <v>1</v>
       </c>
       <c r="N359" s="3" t="n">
-        <v>46084.59331018518</v>
+        <v>46085.40148148148</v>
       </c>
       <c r="O359" t="inlineStr">
         <is>
@@ -23427,7 +23437,7 @@
         </is>
       </c>
       <c r="N360" s="3" t="n">
-        <v>46083.44710648148</v>
+        <v>46085.40222222222</v>
       </c>
       <c r="O360" t="inlineStr">
         <is>
@@ -23615,7 +23625,7 @@
         <v>1</v>
       </c>
       <c r="N363" s="3" t="n">
-        <v>46084.67568287037</v>
+        <v>46085.37054398148</v>
       </c>
       <c r="O363" t="inlineStr">
         <is>
@@ -23681,7 +23691,7 @@
         </is>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46085.31840277778</v>
+        <v>46085.39601851852</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23807,7 +23817,7 @@
         </is>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46085.32060185185</v>
+        <v>46085.39763888889</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
@@ -23873,7 +23883,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46084.68877314815</v>
+        <v>46085.36576388889</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -23942,7 +23952,7 @@
         <v>1</v>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46085.31896990741</v>
+        <v>46085.40300925926</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24011,7 +24021,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46085.29189814815</v>
+        <v>46085.3712037037</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24218,7 +24228,7 @@
         <v>1</v>
       </c>
       <c r="N372" s="3" t="n">
-        <v>46084.73314814815</v>
+        <v>46085.38895833334</v>
       </c>
       <c r="O372" t="inlineStr">
         <is>
@@ -24284,7 +24294,7 @@
         </is>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46085.29534722222</v>
+        <v>46085.37695601852</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24303,11 +24313,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C374" t="inlineStr">
-        <is>
-          <t>10.69.3.72</t>
-        </is>
-      </c>
       <c r="D374" t="n">
         <v>2025</v>
       </c>
@@ -24422,7 +24427,7 @@
         <v>2</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46085.3172337963</v>
+        <v>46085.39334490741</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24491,7 +24496,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46085.3170949074</v>
+        <v>46085.39123842592</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-04 13:52:05.826634
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46085.46488425926</v>
+        <v>46085.54202546296</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46085.48524305555</v>
+        <v>46085.55907407407</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46085.46355324074</v>
+        <v>46085.54042824074</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46085.47763888889</v>
+        <v>46085.55296296296</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46085.46792824074</v>
+        <v>46085.54520833334</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46085.45295138889</v>
+        <v>46085.56363425926</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46085.45815972222</v>
+        <v>46085.53581018518</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46085.47969907407</v>
+        <v>46085.55818287037</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1702,7 +1702,7 @@
         <v>1</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>46085.48226851852</v>
+        <v>46085.55665509259</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1766,7 +1766,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46084.74195601852</v>
+        <v>46085.53465277778</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>46085.12164351852</v>
+        <v>46085.52607638889</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -1903,6 +1903,11 @@
           <t>AUDITORIO</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>10.69.3.150</t>
+        </is>
+      </c>
       <c r="D23" t="n">
         <v>2019</v>
       </c>
@@ -1943,7 +1948,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46085.1834837963</v>
+        <v>46085.56290509259</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2117,7 +2122,7 @@
         <v>1</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>46085.23695601852</v>
+        <v>46085.53730324074</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2178,7 +2183,7 @@
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46084.74120370371</v>
+        <v>46085.54146990741</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6504,7 +6509,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46085.4803125</v>
+        <v>46085.55564814815</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6573,7 +6578,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46085.46465277778</v>
+        <v>46085.54346064815</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6642,7 +6647,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46085.47550925926</v>
+        <v>46085.55334490741</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6706,7 +6711,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46085.46381944444</v>
+        <v>46085.53996527778</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6775,7 +6780,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46085.46127314815</v>
+        <v>46085.53510416667</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6844,7 +6849,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46085.46061342592</v>
+        <v>46085.53795138889</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6913,7 +6918,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46085.45157407408</v>
+        <v>46085.55913194444</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -7051,7 +7056,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46085.45304398148</v>
+        <v>46085.53225694445</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7181,7 +7186,7 @@
         <v>1</v>
       </c>
       <c r="N104" s="3" t="n">
-        <v>46085.44678240741</v>
+        <v>46085.55344907408</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
@@ -7311,7 +7316,7 @@
         <v>1</v>
       </c>
       <c r="N106" s="3" t="n">
-        <v>46085.45245370371</v>
+        <v>46085.56348379629</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -7449,7 +7454,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46085.48753472222</v>
+        <v>46085.56413194445</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7518,7 +7523,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46085.45289351852</v>
+        <v>46085.56978009259</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7587,7 +7592,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46085.46172453704</v>
+        <v>46085.54903935185</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7656,7 +7661,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46085.45677083333</v>
+        <v>46085.53377314815</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7725,7 +7730,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46085.46574074074</v>
+        <v>46085.54418981481</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7794,7 +7799,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46085.479375</v>
+        <v>46085.55833333333</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7860,7 +7865,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46085.45540509259</v>
+        <v>46085.53607638889</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7929,7 +7934,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46085.48591435186</v>
+        <v>46085.56214120371</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7948,11 +7953,6 @@
           <t>DP</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>10.69.3.23</t>
-        </is>
-      </c>
       <c r="D116" t="n">
         <v>2025</v>
       </c>
@@ -7998,7 +7998,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46085.48405092592</v>
+        <v>46085.5592824074</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8064,7 +8064,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46085.45604166666</v>
+        <v>46085.57053240741</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8202,7 +8202,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46085.47372685185</v>
+        <v>46085.54891203704</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8271,7 +8271,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46085.47318287037</v>
+        <v>46085.5546875</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8337,7 +8337,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46085.44927083333</v>
+        <v>46085.56591435185</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8406,7 +8406,7 @@
         <v>2</v>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46085.46949074074</v>
+        <v>46085.54672453704</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8475,7 +8475,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46085.46094907408</v>
+        <v>46085.53734953704</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8544,7 +8544,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46085.45805555556</v>
+        <v>46085.56849537037</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8613,7 +8613,7 @@
         <v>2</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46085.45922453704</v>
+        <v>46085.53444444444</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8682,7 +8682,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46085.4759837963</v>
+        <v>46085.55207175926</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8751,7 +8751,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46085.4621875</v>
+        <v>46085.57017361111</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8820,7 +8820,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46085.48743055556</v>
+        <v>46085.56247685185</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8953,7 +8953,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46085.46736111111</v>
+        <v>46085.54496527778</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9150,7 +9150,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46085.45224537037</v>
+        <v>46085.53261574074</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9405,7 +9405,7 @@
         <v>1</v>
       </c>
       <c r="N137" s="3" t="n">
-        <v>46085.48755787037</v>
+        <v>46085.56505787037</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -9597,7 +9597,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46085.48373842592</v>
+        <v>46085.56167824074</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9661,7 +9661,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46085.45474537037</v>
+        <v>46085.53033564815</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9725,7 +9725,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46085.45186342593</v>
+        <v>46085.56773148148</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9789,7 +9789,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46085.47614583333</v>
+        <v>46085.5507175926</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9853,7 +9853,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46085.48615740741</v>
+        <v>46085.56096064814</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9917,7 +9917,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46085.48283564814</v>
+        <v>46085.56248842592</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9981,7 +9981,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46085.47321759259</v>
+        <v>46085.5553125</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10045,7 +10045,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46085.4571875</v>
+        <v>46085.53033564815</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10109,7 +10109,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46085.45844907407</v>
+        <v>46085.53605324074</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10173,7 +10173,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46085.45466435186</v>
+        <v>46085.53803240741</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10237,7 +10237,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46085.45214120371</v>
+        <v>46085.53291666666</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10301,7 +10301,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46085.45151620371</v>
+        <v>46085.56891203704</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10424,7 +10424,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46085.48320601852</v>
+        <v>46085.56454861111</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10488,7 +10488,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46085.48303240741</v>
+        <v>46085.56085648148</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10552,7 +10552,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46085.47146990741</v>
+        <v>46085.54344907407</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10616,7 +10616,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46085.44899305556</v>
+        <v>46085.5330787037</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10680,7 +10680,7 @@
         <v>1</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>46085.4843287037</v>
+        <v>46085.56155092592</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -10744,7 +10744,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46085.47049768519</v>
+        <v>46085.54427083334</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10808,7 +10808,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46085.48229166667</v>
+        <v>46085.5588425926</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10872,7 +10872,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46085.48559027778</v>
+        <v>46085.56414351852</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10936,7 +10936,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46085.45537037037</v>
+        <v>46085.53224537037</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -11064,7 +11064,7 @@
         <v>2</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46085.47709490741</v>
+        <v>46085.55741898148</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11128,7 +11128,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46085.48074074074</v>
+        <v>46085.55899305556</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11192,7 +11192,7 @@
         <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46085.48577546296</v>
+        <v>46085.56633101852</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11256,7 +11256,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46085.48357638889</v>
+        <v>46085.56005787037</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11320,7 +11320,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46085.48393518518</v>
+        <v>46085.5609837963</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11384,7 +11384,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46085.47628472222</v>
+        <v>46085.5552662037</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11448,7 +11448,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46085.47855324074</v>
+        <v>46085.5583912037</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11512,7 +11512,7 @@
         <v>1</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46085.4852662037</v>
+        <v>46085.56376157407</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11576,7 +11576,7 @@
         <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46085.31050925926</v>
+        <v>46085.54606481481</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11640,7 +11640,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46085.48634259259</v>
+        <v>46085.56425925926</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11704,7 +11704,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46085.48045138889</v>
+        <v>46085.55576388889</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11768,7 +11768,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46085.48376157408</v>
+        <v>46085.56381944445</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11832,7 +11832,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46085.46077546296</v>
+        <v>46085.53876157408</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11896,7 +11896,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46084.73935185185</v>
+        <v>46085.54247685185</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11960,7 +11960,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46085.44831018519</v>
+        <v>46085.55429398148</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12024,7 +12024,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46085.46836805555</v>
+        <v>46085.55177083334</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12088,7 +12088,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46085.46225694445</v>
+        <v>46085.53905092592</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12349,7 +12349,7 @@
         <v>2</v>
       </c>
       <c r="N183" s="3" t="n">
-        <v>46085.45063657407</v>
+        <v>46085.56880787037</v>
       </c>
       <c r="O183" t="inlineStr">
         <is>
@@ -12477,7 +12477,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46085.46945601852</v>
+        <v>46085.54325231481</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12541,7 +12541,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46085.4656712963</v>
+        <v>46085.54140046296</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12605,7 +12605,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46085.45961805555</v>
+        <v>46085.5333912037</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12691,11 +12691,6 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
-      <c r="C189" t="inlineStr">
-        <is>
-          <t>10.69.5.59</t>
-        </is>
-      </c>
       <c r="D189" t="n">
         <v>2015</v>
       </c>
@@ -12733,7 +12728,7 @@
         </is>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46085.46278935186</v>
+        <v>46085.54357638889</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12797,7 +12792,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46085.47028935186</v>
+        <v>46085.54923611111</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12861,7 +12856,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46085.47950231482</v>
+        <v>46085.56149305555</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12986,7 +12981,7 @@
         <v>2</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46085.46503472222</v>
+        <v>46085.53762731481</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13050,7 +13045,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46085.46231481482</v>
+        <v>46085.54103009259</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13114,7 +13109,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46085.45863425926</v>
+        <v>46085.53576388889</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13178,7 +13173,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46085.46136574074</v>
+        <v>46085.53591435185</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13242,7 +13237,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46085.48457175926</v>
+        <v>46085.55965277777</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13306,7 +13301,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46085.46861111111</v>
+        <v>46085.54526620371</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13370,7 +13365,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46085.46356481482</v>
+        <v>46085.53847222222</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13495,7 +13490,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46085.45655092593</v>
+        <v>46085.53486111111</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13559,7 +13554,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46085.46153935185</v>
+        <v>46085.53664351852</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13623,7 +13618,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46085.46358796296</v>
+        <v>46085.5425462963</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13687,7 +13682,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46085.48668981482</v>
+        <v>46085.56275462963</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13751,7 +13746,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46085.4821875</v>
+        <v>46085.56430555556</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13815,7 +13810,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46085.4718287037</v>
+        <v>46085.55331018518</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13879,7 +13874,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46085.46550925926</v>
+        <v>46085.54253472222</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13943,7 +13938,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46085.45892361111</v>
+        <v>46085.5341550926</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14007,7 +14002,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46085.45436342592</v>
+        <v>46085.56991898148</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14071,7 +14066,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46085.479375</v>
+        <v>46085.56041666667</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14135,7 +14130,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46085.48670138889</v>
+        <v>46085.56207175926</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14199,7 +14194,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46085.46863425926</v>
+        <v>46085.54969907407</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14391,7 +14386,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46085.48633101852</v>
+        <v>46085.56200231481</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14455,7 +14450,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46085.48490740741</v>
+        <v>46085.55780092593</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14519,7 +14514,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46085.48475694445</v>
+        <v>46085.55771990741</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14583,7 +14578,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46085.47273148148</v>
+        <v>46085.54422453704</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14652,7 +14647,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46085.4512962963</v>
+        <v>46085.57087962963</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14716,7 +14711,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46085.48168981481</v>
+        <v>46085.55496527778</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14780,7 +14775,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46085.45686342593</v>
+        <v>46085.53699074074</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14908,7 +14903,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46085.46254629629</v>
+        <v>46085.54078703704</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14972,7 +14967,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46085.48428240741</v>
+        <v>46085.56206018518</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15128,7 +15123,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46085.45851851852</v>
+        <v>46085.53163194445</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15192,7 +15187,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46085.48392361111</v>
+        <v>46085.55576388889</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15256,7 +15251,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46085.47949074074</v>
+        <v>46085.55245370371</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15320,7 +15315,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46085.46717592593</v>
+        <v>46085.54243055556</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15384,7 +15379,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46085.48572916666</v>
+        <v>46085.56171296296</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15448,7 +15443,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46085.45202546296</v>
+        <v>46085.56784722222</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15512,7 +15507,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46085.45782407407</v>
+        <v>46085.53319444445</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15576,7 +15571,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46085.45625</v>
+        <v>46085.53425925926</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15640,7 +15635,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46085.4671875</v>
+        <v>46085.54856481482</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15704,7 +15699,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46085.45099537037</v>
+        <v>46085.56833333334</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15768,7 +15763,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46085.46167824074</v>
+        <v>46085.53869212963</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15832,7 +15827,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46085.45050925926</v>
+        <v>46085.56827546296</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15896,7 +15891,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46085.48450231482</v>
+        <v>46085.56148148148</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -16024,7 +16019,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46085.4800462963</v>
+        <v>46085.55957175926</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16088,7 +16083,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46085.45616898148</v>
+        <v>46085.53704861111</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16211,7 +16206,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46085.47486111111</v>
+        <v>46085.554375</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16275,7 +16270,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46085.47615740741</v>
+        <v>46085.55543981482</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16339,7 +16334,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46085.47888888889</v>
+        <v>46085.56105324074</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16403,7 +16398,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46085.45675925926</v>
+        <v>46085.56597222222</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16467,7 +16462,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46085.44903935185</v>
+        <v>46085.56369212963</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16526,7 +16521,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46085.47266203703</v>
+        <v>46085.54671296296</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16590,7 +16585,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46085.43443287037</v>
+        <v>46085.56451388889</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16654,7 +16649,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46085.47616898148</v>
+        <v>46085.54795138889</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16718,7 +16713,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46085.47371527777</v>
+        <v>46085.55208333334</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16776,7 +16771,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46085.47081018519</v>
+        <v>46085.54910879629</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16840,7 +16835,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46085.47277777778</v>
+        <v>46085.55578703704</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16904,7 +16899,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46085.47618055555</v>
+        <v>46085.55106481481</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -16968,7 +16963,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46085.47488425926</v>
+        <v>46085.55501157408</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17032,7 +17027,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46085.47256944444</v>
+        <v>46085.54958333333</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17096,7 +17091,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46085.46541666667</v>
+        <v>46085.54046296296</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17160,7 +17155,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46085.47412037037</v>
+        <v>46085.55857638889</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17288,7 +17283,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46085.45528935185</v>
+        <v>46085.53434027778</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17352,7 +17347,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46085.45579861111</v>
+        <v>46085.54005787037</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17416,7 +17411,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46085.45896990741</v>
+        <v>46085.5384375</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17480,7 +17475,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46085.4841087963</v>
+        <v>46085.56422453704</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17544,7 +17539,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46085.48614583333</v>
+        <v>46085.5634375</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17608,7 +17603,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46085.45269675926</v>
+        <v>46085.56980324074</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17672,7 +17667,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46085.44836805556</v>
+        <v>46085.56483796296</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17736,7 +17731,7 @@
         <v>1</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46085.48164351852</v>
+        <v>46085.55768518519</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17797,7 +17792,7 @@
         </is>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46085.46856481482</v>
+        <v>46085.55326388889</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17925,7 +17920,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46085.46299768519</v>
+        <v>46085.54412037037</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -18050,7 +18045,7 @@
         </is>
       </c>
       <c r="N273" s="3" t="n">
-        <v>46085.46429398148</v>
+        <v>46085.53635416667</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -18114,7 +18109,7 @@
         <v>1</v>
       </c>
       <c r="N274" s="3" t="n">
-        <v>46085.48234953704</v>
+        <v>46085.56351851852</v>
       </c>
       <c r="O274" t="inlineStr">
         <is>
@@ -18239,7 +18234,7 @@
         <v>2</v>
       </c>
       <c r="N276" s="3" t="n">
-        <v>46083.63725694444</v>
+        <v>46085.56861111111</v>
       </c>
       <c r="O276" t="inlineStr">
         <is>
@@ -18303,7 +18298,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46085.48113425926</v>
+        <v>46085.55493055555</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18367,7 +18362,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46085.46334490741</v>
+        <v>46085.54266203703</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18386,6 +18381,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>10.69.5.149</t>
+        </is>
+      </c>
       <c r="D279" t="n">
         <v>2014</v>
       </c>
@@ -18426,7 +18426,7 @@
         <v>2</v>
       </c>
       <c r="N279" s="3" t="n">
-        <v>46085.46072916667</v>
+        <v>46085.57053240741</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -18490,7 +18490,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46085.45782407407</v>
+        <v>46085.56792824074</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18549,7 +18549,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46085.45861111111</v>
+        <v>46085.53150462963</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18613,7 +18613,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46085.47280092593</v>
+        <v>46085.54644675926</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18677,7 +18677,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46085.46009259259</v>
+        <v>46085.53409722223</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18741,7 +18741,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46085.44751157407</v>
+        <v>46085.56269675926</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18760,11 +18760,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C285" t="inlineStr">
-        <is>
-          <t>10.69.5.155</t>
-        </is>
-      </c>
       <c r="D285" t="n">
         <v>2019</v>
       </c>
@@ -18805,7 +18800,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46085.47215277778</v>
+        <v>46085.5447337963</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18869,7 +18864,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46085.45983796296</v>
+        <v>46085.53614583334</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18933,7 +18928,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46085.47037037037</v>
+        <v>46085.54704861111</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -18997,7 +18992,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46085.46083333333</v>
+        <v>46085.54503472222</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19791,7 +19786,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46085.4499074074</v>
+        <v>46085.56653935185</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20907,7 +20902,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46085.46666666667</v>
+        <v>46085.54546296296</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21632,7 +21627,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46085.45731481481</v>
+        <v>46085.53247685185</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21696,7 +21691,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46085.47401620371</v>
+        <v>46085.5525</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21760,7 +21755,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46085.47998842593</v>
+        <v>46085.55563657408</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21824,7 +21819,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46085.48045138889</v>
+        <v>46085.55188657407</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21888,7 +21883,7 @@
         <v>1</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46085.45090277777</v>
+        <v>46085.56898148148</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21952,7 +21947,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46085.47974537037</v>
+        <v>46085.55792824074</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22016,7 +22011,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46085.48461805555</v>
+        <v>46085.56298611111</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22080,7 +22075,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46085.48775462963</v>
+        <v>46085.56886574074</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22144,7 +22139,7 @@
         <v>1</v>
       </c>
       <c r="N339" s="3" t="n">
-        <v>46084.54840277778</v>
+        <v>46085.54862268519</v>
       </c>
       <c r="O339" t="inlineStr">
         <is>
@@ -22208,7 +22203,7 @@
         <v>2</v>
       </c>
       <c r="N340" s="3" t="n">
-        <v>46085.45284722222</v>
+        <v>46085.56974537037</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -22272,7 +22267,7 @@
         <v>2</v>
       </c>
       <c r="N341" s="3" t="n">
-        <v>46085.45892361111</v>
+        <v>46085.53287037037</v>
       </c>
       <c r="O341" t="inlineStr">
         <is>
@@ -22338,7 +22333,7 @@
         </is>
       </c>
       <c r="N342" s="3" t="n">
-        <v>46085.48449074074</v>
+        <v>46085.55775462963</v>
       </c>
       <c r="O342" t="inlineStr">
         <is>
@@ -22594,7 +22589,7 @@
         <v>1</v>
       </c>
       <c r="N346" s="3" t="n">
-        <v>46085.46608796297</v>
+        <v>46085.54846064815</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -22658,7 +22653,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46085.46341435185</v>
+        <v>46085.54215277778</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22722,7 +22717,7 @@
         <v>1</v>
       </c>
       <c r="N348" s="3" t="n">
-        <v>46085.46792824074</v>
+        <v>46085.54555555555</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -23036,7 +23031,7 @@
         <v>1</v>
       </c>
       <c r="N353" s="3" t="n">
-        <v>46085.48579861111</v>
+        <v>46085.55950231481</v>
       </c>
       <c r="O353" t="inlineStr">
         <is>
@@ -23100,7 +23095,7 @@
         <v>1</v>
       </c>
       <c r="N354" s="3" t="n">
-        <v>46085.45564814815</v>
+        <v>46085.53826388889</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -23164,7 +23159,7 @@
         <v>1</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46085.45016203704</v>
+        <v>46085.56457175926</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23287,7 +23282,7 @@
         <v>2</v>
       </c>
       <c r="N357" s="3" t="n">
-        <v>46085.45777777778</v>
+        <v>46085.53527777778</v>
       </c>
       <c r="O357" t="inlineStr">
         <is>
@@ -23351,7 +23346,7 @@
         <v>2</v>
       </c>
       <c r="N358" s="3" t="n">
-        <v>46085.45243055555</v>
+        <v>46085.52998842593</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -23415,7 +23410,7 @@
         <v>1</v>
       </c>
       <c r="N359" s="3" t="n">
-        <v>46085.47494212963</v>
+        <v>46085.55</v>
       </c>
       <c r="O359" t="inlineStr">
         <is>
@@ -23664,7 +23659,7 @@
         <v>1</v>
       </c>
       <c r="N363" s="3" t="n">
-        <v>46085.47952546296</v>
+        <v>46085.56019675926</v>
       </c>
       <c r="O363" t="inlineStr">
         <is>
@@ -23730,7 +23725,7 @@
         </is>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46085.47243055556</v>
+        <v>46085.55094907407</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23856,7 +23851,7 @@
         </is>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46085.47440972222</v>
+        <v>46085.55019675926</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
@@ -23875,6 +23870,11 @@
           <t>RH</t>
         </is>
       </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>10.69.3.13</t>
+        </is>
+      </c>
       <c r="D367" t="n">
         <v>2025</v>
       </c>
@@ -23917,7 +23917,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46085.48333333333</v>
+        <v>46085.56744212963</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -23986,7 +23986,7 @@
         <v>1</v>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46085.47729166667</v>
+        <v>46085.55761574074</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24055,7 +24055,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46085.48582175926</v>
+        <v>46085.55760416666</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24124,7 +24124,7 @@
         <v>1</v>
       </c>
       <c r="N370" s="3" t="n">
-        <v>46085.46960648148</v>
+        <v>46085.51177083333</v>
       </c>
       <c r="O370" t="inlineStr">
         <is>
@@ -24328,7 +24328,7 @@
         <v>1</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46085.46734953704</v>
+        <v>46085.54847222222</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24394,7 +24394,7 @@
         </is>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46085.45376157408</v>
+        <v>46085.57065972222</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24458,7 +24458,7 @@
         <v>1</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46085.45930555555</v>
+        <v>46085.53672453704</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24527,7 +24527,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46085.47658564815</v>
+        <v>46085.55415509259</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -24596,7 +24596,7 @@
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46085.46582175926</v>
+        <v>46085.54785879629</v>
       </c>
       <c r="O377" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-04 15:52:07.597148
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46085.54202546296</v>
+        <v>46085.62123842593</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46085.55907407407</v>
+        <v>46085.63789351852</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46085.54042824074</v>
+        <v>46085.62150462963</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46085.55296296296</v>
+        <v>46085.6303125</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46085.54520833334</v>
+        <v>46085.61942129629</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46085.56363425926</v>
+        <v>46085.64077546296</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46085.53581018518</v>
+        <v>46085.61732638889</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46085.55818287037</v>
+        <v>46085.63039351852</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1702,7 +1702,7 @@
         <v>1</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>46085.55665509259</v>
+        <v>46085.63917824074</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>46085.52607638889</v>
+        <v>46085.62694444445</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46085.56290509259</v>
+        <v>46085.63791666667</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2122,7 +2122,7 @@
         <v>1</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>46085.53730324074</v>
+        <v>46085.61695601852</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46085.54146990741</v>
+        <v>46085.62</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6509,7 +6509,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46085.55564814815</v>
+        <v>46085.63149305555</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6578,7 +6578,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46085.54346064815</v>
+        <v>46085.62113425926</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6597,11 +6597,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>10.69.3.93</t>
-        </is>
-      </c>
       <c r="D96" t="n">
         <v>2025</v>
       </c>
@@ -6647,7 +6642,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46085.55334490741</v>
+        <v>46085.63018518518</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6711,7 +6706,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46085.53996527778</v>
+        <v>46085.62015046296</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6780,7 +6775,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46085.53510416667</v>
+        <v>46085.61599537037</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6849,7 +6844,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46085.53795138889</v>
+        <v>46085.65331018518</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6918,7 +6913,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46085.55913194444</v>
+        <v>46085.63650462963</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -7056,7 +7051,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46085.53225694445</v>
+        <v>46085.64747685185</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7182,11 +7177,8 @@
           <t>HP ProBook 440 14 inch G9 Notebook PC</t>
         </is>
       </c>
-      <c r="M104" t="n">
-        <v>1</v>
-      </c>
       <c r="N104" s="3" t="n">
-        <v>46085.55344907408</v>
+        <v>46085.59393518518</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
@@ -7316,7 +7308,7 @@
         <v>1</v>
       </c>
       <c r="N106" s="3" t="n">
-        <v>46085.56348379629</v>
+        <v>46085.63619212963</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -7454,7 +7446,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46085.56413194445</v>
+        <v>46085.6466087963</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7523,7 +7515,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46085.56978009259</v>
+        <v>46085.64469907407</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7592,7 +7584,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46085.54903935185</v>
+        <v>46085.62381944444</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7661,7 +7653,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46085.53377314815</v>
+        <v>46085.65069444444</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7730,7 +7722,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46085.54418981481</v>
+        <v>46085.62226851852</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7799,7 +7791,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46085.55833333333</v>
+        <v>46085.63239583333</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7865,7 +7857,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46085.53607638889</v>
+        <v>46085.61451388889</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7934,7 +7926,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46085.56214120371</v>
+        <v>46085.64142361111</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7998,7 +7990,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46085.5592824074</v>
+        <v>46085.63975694445</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8064,7 +8056,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46085.57053240741</v>
+        <v>46085.64814814815</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8202,7 +8194,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46085.54891203704</v>
+        <v>46085.63425925926</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8271,7 +8263,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46085.5546875</v>
+        <v>46085.63377314815</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8337,7 +8329,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46085.56591435185</v>
+        <v>46085.64827546296</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8406,7 +8398,7 @@
         <v>2</v>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46085.54672453704</v>
+        <v>46085.62696759259</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8475,7 +8467,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46085.53734953704</v>
+        <v>46085.6531712963</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8544,7 +8536,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46085.56849537037</v>
+        <v>46085.64790509259</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8613,7 +8605,7 @@
         <v>2</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46085.53444444444</v>
+        <v>46085.65229166667</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8682,7 +8674,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46085.55207175926</v>
+        <v>46085.62912037037</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8751,7 +8743,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46085.57017361111</v>
+        <v>46085.64697916667</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8820,7 +8812,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46085.56247685185</v>
+        <v>46085.6459837963</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8953,7 +8945,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46085.54496527778</v>
+        <v>46085.61662037037</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9086,7 +9078,7 @@
         <v>1</v>
       </c>
       <c r="N132" s="3" t="n">
-        <v>46084.80613425926</v>
+        <v>46085.65390046296</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -9150,7 +9142,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46085.53261574074</v>
+        <v>46085.6250462963</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9214,7 +9206,7 @@
         <v>1</v>
       </c>
       <c r="N134" s="3" t="n">
-        <v>46084.80681712963</v>
+        <v>46085.63438657407</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -9405,7 +9397,7 @@
         <v>1</v>
       </c>
       <c r="N137" s="3" t="n">
-        <v>46085.56505787037</v>
+        <v>46085.64509259259</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -9469,7 +9461,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46084.81265046296</v>
+        <v>46085.6540625</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9533,7 +9525,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46084.81913194444</v>
+        <v>46085.62297453704</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9597,7 +9589,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46085.56167824074</v>
+        <v>46085.64210648148</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9661,7 +9653,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46085.53033564815</v>
+        <v>46085.64761574074</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9725,7 +9717,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46085.56773148148</v>
+        <v>46085.64533564815</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9789,7 +9781,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46085.5507175926</v>
+        <v>46085.63089120371</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9853,7 +9845,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46085.56096064814</v>
+        <v>46085.61726851852</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9917,7 +9909,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46085.56248842592</v>
+        <v>46085.62001157407</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -10045,7 +10037,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46085.53033564815</v>
+        <v>46085.64892361111</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10109,7 +10101,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46085.53605324074</v>
+        <v>46085.6540625</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10173,7 +10165,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46085.53803240741</v>
+        <v>46085.65180555556</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10237,7 +10229,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46085.53291666666</v>
+        <v>46085.64813657408</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10301,7 +10293,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46085.56891203704</v>
+        <v>46085.62280092593</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10424,7 +10416,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46085.56454861111</v>
+        <v>46085.62524305555</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10488,7 +10480,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46085.56085648148</v>
+        <v>46085.63293981482</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10552,7 +10544,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46085.54344907407</v>
+        <v>46085.61849537037</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10616,7 +10608,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46085.5330787037</v>
+        <v>46085.57560185185</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10680,7 +10672,7 @@
         <v>1</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>46085.56155092592</v>
+        <v>46085.6025</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -10744,7 +10736,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46085.54427083334</v>
+        <v>46085.62291666667</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10808,7 +10800,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46085.5588425926</v>
+        <v>46085.63402777778</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10872,7 +10864,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46085.56414351852</v>
+        <v>46085.63211805555</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10936,7 +10928,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46085.53224537037</v>
+        <v>46085.64879629629</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -11064,7 +11056,7 @@
         <v>2</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46085.55741898148</v>
+        <v>46085.62998842593</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11128,7 +11120,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46085.55899305556</v>
+        <v>46085.59677083333</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11192,7 +11184,7 @@
         <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46085.56633101852</v>
+        <v>46085.603125</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11256,7 +11248,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46085.56005787037</v>
+        <v>46085.59586805556</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11384,7 +11376,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46085.5552662037</v>
+        <v>46085.63142361111</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11448,7 +11440,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46085.5583912037</v>
+        <v>46085.62313657408</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11576,7 +11568,7 @@
         <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46085.54606481481</v>
+        <v>46085.62215277777</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11640,7 +11632,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46085.56425925926</v>
+        <v>46085.64153935185</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11704,7 +11696,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46085.55576388889</v>
+        <v>46085.63326388889</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11832,7 +11824,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46085.53876157408</v>
+        <v>46085.61444444444</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11896,7 +11888,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46085.54247685185</v>
+        <v>46085.61582175926</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11960,7 +11952,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46085.55429398148</v>
+        <v>46085.62635416666</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12024,7 +12016,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46085.55177083334</v>
+        <v>46085.62484953704</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12088,7 +12080,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46085.53905092592</v>
+        <v>46085.65237268519</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12152,7 +12144,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46084.81405092592</v>
+        <v>46085.62699074074</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12349,7 +12341,7 @@
         <v>2</v>
       </c>
       <c r="N183" s="3" t="n">
-        <v>46085.56880787037</v>
+        <v>46085.64539351852</v>
       </c>
       <c r="O183" t="inlineStr">
         <is>
@@ -12477,7 +12469,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46085.54325231481</v>
+        <v>46085.63037037037</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12541,7 +12533,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46085.54140046296</v>
+        <v>46085.63194444445</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12605,7 +12597,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46085.5333912037</v>
+        <v>46085.61391203704</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12728,7 +12720,7 @@
         </is>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46085.54357638889</v>
+        <v>46085.62449074074</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12792,7 +12784,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46085.54923611111</v>
+        <v>46085.62590277778</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12856,7 +12848,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46085.56149305555</v>
+        <v>46085.62631944445</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12981,7 +12973,7 @@
         <v>2</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46085.53762731481</v>
+        <v>46085.64833333333</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13045,7 +13037,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46085.54103009259</v>
+        <v>46085.61902777778</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13109,7 +13101,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46085.53576388889</v>
+        <v>46085.61292824074</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13173,7 +13165,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46085.53591435185</v>
+        <v>46085.65166666666</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13301,7 +13293,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46085.54526620371</v>
+        <v>46085.61891203704</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13365,7 +13357,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46085.53847222222</v>
+        <v>46085.63517361111</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13426,7 +13418,7 @@
         </is>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46081.60105324074</v>
+        <v>46085.63079861111</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13490,7 +13482,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46085.53486111111</v>
+        <v>46085.63465277778</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13554,7 +13546,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46085.53664351852</v>
+        <v>46085.62721064815</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13618,7 +13610,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46085.5425462963</v>
+        <v>46085.62511574074</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13682,7 +13674,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46085.56275462963</v>
+        <v>46085.63273148148</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13746,7 +13738,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46085.56430555556</v>
+        <v>46085.6352662037</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13810,7 +13802,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46085.55331018518</v>
+        <v>46085.63018518518</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13874,7 +13866,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46085.54253472222</v>
+        <v>46085.63079861111</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13938,7 +13930,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46085.5341550926</v>
+        <v>46085.61851851852</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14002,7 +13994,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46085.56991898148</v>
+        <v>46085.65225694444</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14066,7 +14058,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46085.56041666667</v>
+        <v>46085.63878472222</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14130,7 +14122,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46085.56207175926</v>
+        <v>46085.62800925926</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14194,7 +14186,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46085.54969907407</v>
+        <v>46085.64836805555</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14258,7 +14250,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46085.32649305555</v>
+        <v>46085.64465277778</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14322,7 +14314,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46083.79869212963</v>
+        <v>46085.64935185185</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14386,7 +14378,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46085.56200231481</v>
+        <v>46085.63813657407</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14450,7 +14442,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46085.55780092593</v>
+        <v>46085.63473379629</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14514,7 +14506,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46085.55771990741</v>
+        <v>46085.64042824074</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14578,7 +14570,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46085.54422453704</v>
+        <v>46085.62479166667</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14647,7 +14639,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46085.57087962963</v>
+        <v>46085.62414351852</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14711,7 +14703,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46085.55496527778</v>
+        <v>46085.62311342593</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14775,7 +14767,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46085.53699074074</v>
+        <v>46085.61760416667</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14839,7 +14831,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46084.8091087963</v>
+        <v>46085.64480324074</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14903,7 +14895,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46085.54078703704</v>
+        <v>46085.63348379629</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14967,7 +14959,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46085.56206018518</v>
+        <v>46085.62699074074</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -14995,7 +14987,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46084.49026620371</v>
+        <v>46085.64210648148</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15059,7 +15051,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46084.86769675926</v>
+        <v>46085.63021990741</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15123,7 +15115,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46085.53163194445</v>
+        <v>46085.64768518518</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15187,7 +15179,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46085.55576388889</v>
+        <v>46085.63300925926</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15251,7 +15243,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46085.55245370371</v>
+        <v>46085.62508101852</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15315,7 +15307,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46085.54243055556</v>
+        <v>46085.62835648148</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15379,7 +15371,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46085.56171296296</v>
+        <v>46085.62174768518</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15443,7 +15435,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46085.56784722222</v>
+        <v>46085.64559027777</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15507,7 +15499,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46085.53319444445</v>
+        <v>46085.62796296296</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15571,7 +15563,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46085.53425925926</v>
+        <v>46085.62834490741</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15635,7 +15627,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46085.54856481482</v>
+        <v>46085.62059027778</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15699,7 +15691,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46085.56833333334</v>
+        <v>46085.64766203704</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15763,7 +15755,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46085.53869212963</v>
+        <v>46085.6250462963</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15827,7 +15819,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46085.56827546296</v>
+        <v>46085.61004629629</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15891,7 +15883,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46085.56148148148</v>
+        <v>46085.64002314815</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -15955,7 +15947,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46084.86973379629</v>
+        <v>46085.62993055556</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16019,7 +16011,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46085.55957175926</v>
+        <v>46085.63427083333</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16083,7 +16075,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46085.53704861111</v>
+        <v>46085.63293981482</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16206,7 +16198,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46085.554375</v>
+        <v>46085.64346064815</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16270,7 +16262,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46085.55543981482</v>
+        <v>46085.63153935185</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16334,7 +16326,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46085.56105324074</v>
+        <v>46085.6427662037</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16398,7 +16390,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46085.56597222222</v>
+        <v>46085.64119212963</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16462,7 +16454,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46085.56369212963</v>
+        <v>46085.63626157407</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16481,6 +16473,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>10.69.5.118</t>
+        </is>
+      </c>
       <c r="D249" t="n">
         <v>2017</v>
       </c>
@@ -16521,7 +16518,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46085.54671296296</v>
+        <v>46085.62292824074</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16585,7 +16582,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46085.56451388889</v>
+        <v>46085.62240740741</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16649,7 +16646,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46085.54795138889</v>
+        <v>46085.62763888889</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16713,7 +16710,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46085.55208333334</v>
+        <v>46085.59743055556</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16771,7 +16768,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46085.54910879629</v>
+        <v>46085.63120370371</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16835,7 +16832,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46085.55578703704</v>
+        <v>46085.65109953703</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16899,7 +16896,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46085.55106481481</v>
+        <v>46085.63475694445</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -16963,7 +16960,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46085.55501157408</v>
+        <v>46085.63185185185</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17027,7 +17024,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46085.54958333333</v>
+        <v>46085.63231481481</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17091,7 +17088,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46085.54046296296</v>
+        <v>46085.598125</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17155,7 +17152,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46085.55857638889</v>
+        <v>46085.59555555556</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17219,7 +17216,7 @@
         <v>2</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46084.80190972222</v>
+        <v>46085.63782407407</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17283,7 +17280,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46085.53434027778</v>
+        <v>46085.65394675926</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17347,7 +17344,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46085.54005787037</v>
+        <v>46085.61991898148</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17411,7 +17408,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46085.5384375</v>
+        <v>46085.62761574074</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17475,7 +17472,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46085.56422453704</v>
+        <v>46085.62555555555</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17539,7 +17536,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46085.5634375</v>
+        <v>46085.64185185185</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17603,7 +17600,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46085.56980324074</v>
+        <v>46085.65289351852</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17667,7 +17664,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46085.56483796296</v>
+        <v>46085.64290509259</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17731,7 +17728,7 @@
         <v>1</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46085.55768518519</v>
+        <v>46085.64084490741</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17792,7 +17789,7 @@
         </is>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46085.55326388889</v>
+        <v>46085.63538194444</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17856,7 +17853,7 @@
         <v>1</v>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46085.09553240741</v>
+        <v>46085.57637731481</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -17920,7 +17917,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46085.54412037037</v>
+        <v>46085.62506944445</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -18045,7 +18042,7 @@
         </is>
       </c>
       <c r="N273" s="3" t="n">
-        <v>46085.53635416667</v>
+        <v>46085.61403935185</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -18109,7 +18106,7 @@
         <v>1</v>
       </c>
       <c r="N274" s="3" t="n">
-        <v>46085.56351851852</v>
+        <v>46085.63672453703</v>
       </c>
       <c r="O274" t="inlineStr">
         <is>
@@ -18362,7 +18359,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46085.54266203703</v>
+        <v>46085.57907407408</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18426,7 +18423,7 @@
         <v>2</v>
       </c>
       <c r="N279" s="3" t="n">
-        <v>46085.57053240741</v>
+        <v>46085.62831018519</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -18490,7 +18487,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46085.56792824074</v>
+        <v>46085.57841435185</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18549,7 +18546,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46085.53150462963</v>
+        <v>46085.57290509259</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18613,7 +18610,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46085.54644675926</v>
+        <v>46085.58581018518</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18677,7 +18674,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46085.53409722223</v>
+        <v>46085.65175925926</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18741,7 +18738,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46085.56269675926</v>
+        <v>46085.62760416666</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18800,7 +18797,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46085.5447337963</v>
+        <v>46085.58457175926</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18864,7 +18861,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46085.53614583334</v>
+        <v>46085.61483796296</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18992,7 +18989,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46085.54503472222</v>
+        <v>46085.62202546297</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19786,7 +19783,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46085.56653935185</v>
+        <v>46085.64788194445</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20902,7 +20899,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46085.54546296296</v>
+        <v>46085.61898148148</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21627,7 +21624,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46085.53247685185</v>
+        <v>46085.64829861111</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21691,7 +21688,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46085.5525</v>
+        <v>46085.62974537037</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21755,7 +21752,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46085.55563657408</v>
+        <v>46085.6346875</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21819,7 +21816,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46085.55188657407</v>
+        <v>46085.63048611111</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21883,7 +21880,7 @@
         <v>1</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46085.56898148148</v>
+        <v>46085.64810185185</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21947,7 +21944,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46085.55792824074</v>
+        <v>46085.63469907407</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22011,7 +22008,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46085.56298611111</v>
+        <v>46085.64354166666</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22075,7 +22072,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46085.56886574074</v>
+        <v>46085.64810185185</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22139,7 +22136,7 @@
         <v>1</v>
       </c>
       <c r="N339" s="3" t="n">
-        <v>46085.54862268519</v>
+        <v>46085.58538194445</v>
       </c>
       <c r="O339" t="inlineStr">
         <is>
@@ -22267,7 +22264,7 @@
         <v>2</v>
       </c>
       <c r="N341" s="3" t="n">
-        <v>46085.53287037037</v>
+        <v>46085.57246527778</v>
       </c>
       <c r="O341" t="inlineStr">
         <is>
@@ -22286,11 +22283,6 @@
           <t>OPERACAO 9.1</t>
         </is>
       </c>
-      <c r="C342" t="inlineStr">
-        <is>
-          <t>10.69.5.237</t>
-        </is>
-      </c>
       <c r="D342" t="n">
         <v>2017</v>
       </c>
@@ -22333,7 +22325,7 @@
         </is>
       </c>
       <c r="N342" s="3" t="n">
-        <v>46085.55775462963</v>
+        <v>46085.59991898148</v>
       </c>
       <c r="O342" t="inlineStr">
         <is>
@@ -22589,7 +22581,7 @@
         <v>1</v>
       </c>
       <c r="N346" s="3" t="n">
-        <v>46085.54846064815</v>
+        <v>46085.5897800926</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -22653,7 +22645,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46085.54215277778</v>
+        <v>46085.58230324074</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22717,7 +22709,7 @@
         <v>1</v>
       </c>
       <c r="N348" s="3" t="n">
-        <v>46085.54555555555</v>
+        <v>46085.58729166666</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -23031,7 +23023,7 @@
         <v>1</v>
       </c>
       <c r="N353" s="3" t="n">
-        <v>46085.55950231481</v>
+        <v>46085.60005787037</v>
       </c>
       <c r="O353" t="inlineStr">
         <is>
@@ -23095,7 +23087,7 @@
         <v>1</v>
       </c>
       <c r="N354" s="3" t="n">
-        <v>46085.53826388889</v>
+        <v>46085.57380787037</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -23159,7 +23151,7 @@
         <v>1</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46085.56457175926</v>
+        <v>46085.60575231481</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23282,7 +23274,7 @@
         <v>2</v>
       </c>
       <c r="N357" s="3" t="n">
-        <v>46085.53527777778</v>
+        <v>46085.575</v>
       </c>
       <c r="O357" t="inlineStr">
         <is>
@@ -23346,7 +23338,7 @@
         <v>2</v>
       </c>
       <c r="N358" s="3" t="n">
-        <v>46085.52998842593</v>
+        <v>46085.61003472222</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -23410,7 +23402,7 @@
         <v>1</v>
       </c>
       <c r="N359" s="3" t="n">
-        <v>46085.55</v>
+        <v>46085.59136574074</v>
       </c>
       <c r="O359" t="inlineStr">
         <is>
@@ -23659,7 +23651,7 @@
         <v>1</v>
       </c>
       <c r="N363" s="3" t="n">
-        <v>46085.56019675926</v>
+        <v>46085.63637731481</v>
       </c>
       <c r="O363" t="inlineStr">
         <is>
@@ -23851,7 +23843,7 @@
         </is>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46085.55019675926</v>
+        <v>46085.63165509259</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
@@ -23917,7 +23909,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46085.56744212963</v>
+        <v>46085.64142361111</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -23986,7 +23978,7 @@
         <v>1</v>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46085.55761574074</v>
+        <v>46085.63322916667</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24055,7 +24047,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46085.55760416666</v>
+        <v>46085.63648148148</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24124,7 +24116,7 @@
         <v>1</v>
       </c>
       <c r="N370" s="3" t="n">
-        <v>46085.51177083333</v>
+        <v>46085.57601851852</v>
       </c>
       <c r="O370" t="inlineStr">
         <is>
@@ -24258,8 +24250,11 @@
           <t>HP ProDesk 400 G5 SFF (Brazil)</t>
         </is>
       </c>
+      <c r="M372" t="n">
+        <v>1</v>
+      </c>
       <c r="N372" s="3" t="n">
-        <v>46084.61623842592</v>
+        <v>46085.61537037037</v>
       </c>
       <c r="O372" t="inlineStr">
         <is>
@@ -24328,7 +24323,7 @@
         <v>1</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46085.54847222222</v>
+        <v>46085.62398148148</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24394,7 +24389,7 @@
         </is>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46085.57065972222</v>
+        <v>46085.64805555555</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24413,6 +24408,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>10.69.3.72</t>
+        </is>
+      </c>
       <c r="D375" t="n">
         <v>2025</v>
       </c>
@@ -24458,7 +24458,7 @@
         <v>1</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46085.53672453704</v>
+        <v>46085.6525462963</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24527,7 +24527,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46085.55415509259</v>
+        <v>46085.62616898148</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -24596,7 +24596,7 @@
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46085.54785879629</v>
+        <v>46085.62660879629</v>
       </c>
       <c r="O377" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-04 17:52:04.564492
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46085.62123842593</v>
+        <v>46085.70050925926</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46085.63789351852</v>
+        <v>46085.6749537037</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46085.62150462963</v>
+        <v>46085.69936342593</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46085.6303125</v>
+        <v>46085.70461805556</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46085.61942129629</v>
+        <v>46085.73425925926</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46085.64077546296</v>
+        <v>46085.71910879629</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46085.61732638889</v>
+        <v>46085.73716435185</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46085.63039351852</v>
+        <v>46085.70717592593</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1702,7 +1702,7 @@
         <v>1</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>46085.63917824074</v>
+        <v>46085.71967592592</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1766,7 +1766,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46085.53465277778</v>
+        <v>46085.73266203704</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1844,6 +1844,11 @@
           <t>AUDITORIO</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>10.69.3.146</t>
+        </is>
+      </c>
       <c r="D22" t="n">
         <v>2018</v>
       </c>
@@ -1884,7 +1889,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>46085.62694444445</v>
+        <v>46085.71766203704</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -1903,11 +1908,6 @@
           <t>AUDITORIO</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>10.69.3.150</t>
-        </is>
-      </c>
       <c r="D23" t="n">
         <v>2019</v>
       </c>
@@ -1948,7 +1948,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46085.63791666667</v>
+        <v>46085.71467592593</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46085.62</v>
+        <v>46085.69731481482</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6509,7 +6509,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46085.63149305555</v>
+        <v>46085.71253472222</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6578,7 +6578,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46085.62113425926</v>
+        <v>46085.70060185185</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6642,7 +6642,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46085.63018518518</v>
+        <v>46085.7075462963</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6661,6 +6661,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>10.69.3.94</t>
+        </is>
+      </c>
       <c r="D97" t="n">
         <v>2025</v>
       </c>
@@ -6706,7 +6711,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46085.62015046296</v>
+        <v>46085.73667824074</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6775,7 +6780,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46085.61599537037</v>
+        <v>46085.69483796296</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6844,7 +6849,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46085.65331018518</v>
+        <v>46085.73212962963</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6913,7 +6918,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46085.63650462963</v>
+        <v>46085.71142361111</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -7051,7 +7056,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46085.64747685185</v>
+        <v>46085.72237268519</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7308,7 +7313,7 @@
         <v>1</v>
       </c>
       <c r="N106" s="3" t="n">
-        <v>46085.63619212963</v>
+        <v>46085.67232638889</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -7446,7 +7451,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46085.6466087963</v>
+        <v>46085.72298611111</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7515,7 +7520,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46085.64469907407</v>
+        <v>46085.72274305556</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7584,7 +7589,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46085.62381944444</v>
+        <v>46085.70056712963</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7653,7 +7658,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46085.65069444444</v>
+        <v>46085.72881944444</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7722,7 +7727,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46085.62226851852</v>
+        <v>46085.70186342593</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7791,7 +7796,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46085.63239583333</v>
+        <v>46085.71254629629</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7857,7 +7862,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46085.61451388889</v>
+        <v>46085.73488425926</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7926,7 +7931,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46085.64142361111</v>
+        <v>46085.68173611111</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7945,6 +7950,11 @@
           <t>DP</t>
         </is>
       </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>10.69.3.23</t>
+        </is>
+      </c>
       <c r="D116" t="n">
         <v>2025</v>
       </c>
@@ -7990,7 +8000,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46085.63975694445</v>
+        <v>46085.67766203704</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8056,7 +8066,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46085.64814814815</v>
+        <v>46085.68864583333</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8194,7 +8204,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46085.63425925926</v>
+        <v>46085.67530092593</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8263,7 +8273,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46085.63377314815</v>
+        <v>46085.71229166666</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8329,7 +8339,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46085.64827546296</v>
+        <v>46085.6836574074</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8398,7 +8408,7 @@
         <v>2</v>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46085.62696759259</v>
+        <v>46085.70680555556</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8467,7 +8477,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46085.6531712963</v>
+        <v>46085.7311574074</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8536,7 +8546,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46085.64790509259</v>
+        <v>46085.72425925926</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8674,7 +8684,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46085.62912037037</v>
+        <v>46085.70788194444</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8743,7 +8753,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46085.64697916667</v>
+        <v>46085.68497685185</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8812,7 +8822,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46085.6459837963</v>
+        <v>46085.68760416667</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8945,7 +8955,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46085.61662037037</v>
+        <v>46085.69841435185</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9078,7 +9088,7 @@
         <v>1</v>
       </c>
       <c r="N132" s="3" t="n">
-        <v>46085.65390046296</v>
+        <v>46085.73224537037</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -9142,7 +9152,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46085.6250462963</v>
+        <v>46085.70248842592</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9206,7 +9216,7 @@
         <v>1</v>
       </c>
       <c r="N134" s="3" t="n">
-        <v>46085.63438657407</v>
+        <v>46085.70763888889</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -9397,7 +9407,7 @@
         <v>1</v>
       </c>
       <c r="N137" s="3" t="n">
-        <v>46085.64509259259</v>
+        <v>46085.72079861111</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -9461,7 +9471,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46085.6540625</v>
+        <v>46085.7184375</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9525,7 +9535,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46085.62297453704</v>
+        <v>46085.70165509259</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9589,7 +9599,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46085.64210648148</v>
+        <v>46085.71903935185</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9653,7 +9663,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46085.64761574074</v>
+        <v>46085.72380787037</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9717,7 +9727,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46085.64533564815</v>
+        <v>46085.72184027778</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9781,7 +9791,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46085.63089120371</v>
+        <v>46085.70356481482</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9845,7 +9855,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46085.61726851852</v>
+        <v>46085.69739583333</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9909,7 +9919,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46085.62001157407</v>
+        <v>46085.7003587963</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9973,7 +9983,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46085.5553125</v>
+        <v>46085.73314814815</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10037,7 +10047,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46085.64892361111</v>
+        <v>46085.72341435185</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10101,7 +10111,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46085.6540625</v>
+        <v>46085.72863425926</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10165,7 +10175,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46085.65180555556</v>
+        <v>46085.73158564815</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10229,7 +10239,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46085.64813657408</v>
+        <v>46085.7229050926</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10293,7 +10303,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46085.62280092593</v>
+        <v>46085.69824074074</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10416,7 +10426,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46085.62524305555</v>
+        <v>46085.70259259259</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10480,7 +10490,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46085.63293981482</v>
+        <v>46085.70716435185</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10736,7 +10746,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46085.62291666667</v>
+        <v>46085.73491898148</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10800,7 +10810,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46085.63402777778</v>
+        <v>46085.71118055555</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10864,7 +10874,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46085.63211805555</v>
+        <v>46085.71289351852</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10928,7 +10938,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46085.64879629629</v>
+        <v>46085.72765046296</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -11056,7 +11066,7 @@
         <v>2</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46085.62998842593</v>
+        <v>46085.70638888889</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11376,7 +11386,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46085.63142361111</v>
+        <v>46085.7074074074</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11440,7 +11450,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46085.62313657408</v>
+        <v>46085.69922453703</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11568,7 +11578,7 @@
         <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46085.62215277777</v>
+        <v>46085.73430555555</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11632,7 +11642,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46085.64153935185</v>
+        <v>46085.72125</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11696,7 +11706,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46085.63326388889</v>
+        <v>46085.70825231481</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11824,7 +11834,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46085.61444444444</v>
+        <v>46085.65648148148</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11888,7 +11898,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46085.61582175926</v>
+        <v>46085.73752314815</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11952,7 +11962,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46085.62635416666</v>
+        <v>46085.70324074074</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12016,7 +12026,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46085.62484953704</v>
+        <v>46085.70167824074</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12080,7 +12090,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46085.65237268519</v>
+        <v>46085.73232638889</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12144,7 +12154,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46085.62699074074</v>
+        <v>46085.70869212963</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12341,7 +12351,7 @@
         <v>2</v>
       </c>
       <c r="N183" s="3" t="n">
-        <v>46085.64539351852</v>
+        <v>46085.72532407408</v>
       </c>
       <c r="O183" t="inlineStr">
         <is>
@@ -12469,7 +12479,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46085.63037037037</v>
+        <v>46085.70818287037</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12533,7 +12543,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46085.63194444445</v>
+        <v>46085.7069675926</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12597,7 +12607,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46085.61391203704</v>
+        <v>46085.69630787037</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12683,6 +12693,11 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>10.69.5.59</t>
+        </is>
+      </c>
       <c r="D189" t="n">
         <v>2015</v>
       </c>
@@ -12720,7 +12735,7 @@
         </is>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46085.62449074074</v>
+        <v>46085.73719907407</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12784,7 +12799,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46085.62590277778</v>
+        <v>46085.69954861111</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12848,7 +12863,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46085.62631944445</v>
+        <v>46085.69976851852</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12973,7 +12988,7 @@
         <v>2</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46085.64833333333</v>
+        <v>46085.72739583333</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13037,7 +13052,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46085.61902777778</v>
+        <v>46085.7303125</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13101,7 +13116,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46085.61292824074</v>
+        <v>46085.73090277778</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13165,7 +13180,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46085.65166666666</v>
+        <v>46085.72971064815</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13293,7 +13308,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46085.61891203704</v>
+        <v>46085.73202546296</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13357,7 +13372,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46085.63517361111</v>
+        <v>46085.71100694445</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13418,7 +13433,7 @@
         </is>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46085.63079861111</v>
+        <v>46085.70883101852</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13482,7 +13497,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46085.63465277778</v>
+        <v>46085.71224537037</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13546,7 +13561,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46085.62721064815</v>
+        <v>46085.71519675926</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13610,7 +13625,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46085.62511574074</v>
+        <v>46085.71192129629</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13674,7 +13689,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46085.63273148148</v>
+        <v>46085.7140625</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13738,7 +13753,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46085.6352662037</v>
+        <v>46085.71332175926</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13802,7 +13817,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46085.63018518518</v>
+        <v>46085.7094212963</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13866,7 +13881,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46085.63079861111</v>
+        <v>46085.705</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13930,7 +13945,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46085.61851851852</v>
+        <v>46085.73180555556</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -13994,7 +14009,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46085.65225694444</v>
+        <v>46085.73616898148</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14058,7 +14073,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46085.63878472222</v>
+        <v>46085.7155787037</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14122,7 +14137,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46085.62800925926</v>
+        <v>46085.70372685185</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14186,7 +14201,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46085.64836805555</v>
+        <v>46085.72895833333</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14250,7 +14265,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46085.64465277778</v>
+        <v>46085.71864583333</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14314,7 +14329,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46085.64935185185</v>
+        <v>46085.7297337963</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14378,7 +14393,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46085.63813657407</v>
+        <v>46085.71267361111</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14442,7 +14457,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46085.63473379629</v>
+        <v>46085.71839120371</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14506,7 +14521,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46085.64042824074</v>
+        <v>46085.72255787037</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14570,7 +14585,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46085.62479166667</v>
+        <v>46085.6996412037</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14639,7 +14654,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46085.62414351852</v>
+        <v>46085.70063657407</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14703,7 +14718,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46085.62311342593</v>
+        <v>46085.73393518518</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14767,7 +14782,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46085.61760416667</v>
+        <v>46085.73297453704</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14831,7 +14846,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46085.64480324074</v>
+        <v>46085.72020833333</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14895,7 +14910,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46085.63348379629</v>
+        <v>46085.71009259259</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14959,7 +14974,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46085.62699074074</v>
+        <v>46085.70311342592</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -14987,7 +15002,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46085.64210648148</v>
+        <v>46085.71528935185</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15051,7 +15066,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46085.63021990741</v>
+        <v>46085.70755787037</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15115,7 +15130,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46085.64768518518</v>
+        <v>46085.72064814815</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15179,7 +15194,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46085.63300925926</v>
+        <v>46085.73358796296</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15243,7 +15258,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46085.62508101852</v>
+        <v>46085.70483796296</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15307,7 +15322,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46085.62835648148</v>
+        <v>46085.70578703703</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15371,7 +15386,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46085.62174768518</v>
+        <v>46085.70019675926</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15435,7 +15450,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46085.64559027777</v>
+        <v>46085.72009259259</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15499,7 +15514,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46085.62796296296</v>
+        <v>46085.70136574074</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15563,7 +15578,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46085.62834490741</v>
+        <v>46085.70809027777</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15627,7 +15642,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46085.62059027778</v>
+        <v>46085.73731481482</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15691,7 +15706,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46085.64766203704</v>
+        <v>46085.72505787037</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15755,7 +15770,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46085.6250462963</v>
+        <v>46085.735</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15883,7 +15898,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46085.64002314815</v>
+        <v>46085.71643518518</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -15947,7 +15962,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46085.62993055556</v>
+        <v>46085.70855324074</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16011,7 +16026,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46085.63427083333</v>
+        <v>46085.71254629629</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16075,7 +16090,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46085.63293981482</v>
+        <v>46085.71284722222</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16134,7 +16149,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46085.26280092593</v>
+        <v>46085.71618055556</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16198,7 +16213,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46085.64346064815</v>
+        <v>46085.72072916666</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16262,7 +16277,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46085.63153935185</v>
+        <v>46085.70700231481</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16326,7 +16341,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46085.6427662037</v>
+        <v>46085.72033564815</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16390,7 +16405,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46085.64119212963</v>
+        <v>46085.70965277778</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16454,7 +16469,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46085.63626157407</v>
+        <v>46085.71336805556</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16518,7 +16533,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46085.62292824074</v>
+        <v>46085.70394675926</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16582,7 +16597,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46085.62240740741</v>
+        <v>46085.71738425926</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16646,7 +16661,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46085.62763888889</v>
+        <v>46085.71113425926</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16710,7 +16725,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46085.59743055556</v>
+        <v>46085.71475694444</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16768,7 +16783,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46085.63120370371</v>
+        <v>46085.709375</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16832,7 +16847,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46085.65109953703</v>
+        <v>46085.73068287037</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16896,7 +16911,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46085.63475694445</v>
+        <v>46085.71269675926</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -16960,7 +16975,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46085.63185185185</v>
+        <v>46085.71335648148</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17024,7 +17039,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46085.63231481481</v>
+        <v>46085.72325231481</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17216,7 +17231,7 @@
         <v>2</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46085.63782407407</v>
+        <v>46085.71630787037</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17280,7 +17295,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46085.65394675926</v>
+        <v>46085.73729166666</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17344,7 +17359,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46085.61991898148</v>
+        <v>46085.73299768518</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17408,7 +17423,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46085.62761574074</v>
+        <v>46085.70221064815</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17472,7 +17487,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46085.62555555555</v>
+        <v>46085.70451388889</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17536,7 +17551,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46085.64185185185</v>
+        <v>46085.71907407408</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17600,7 +17615,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46085.65289351852</v>
+        <v>46085.73752314815</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17664,7 +17679,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46085.64290509259</v>
+        <v>46085.71986111111</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17728,7 +17743,7 @@
         <v>1</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46085.64084490741</v>
+        <v>46085.72050925926</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17789,7 +17804,7 @@
         </is>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46085.63538194444</v>
+        <v>46085.71575231481</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17853,7 +17868,7 @@
         <v>1</v>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46085.57637731481</v>
+        <v>46085.72497685185</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -17917,7 +17932,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46085.62506944445</v>
+        <v>46085.70480324074</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -18042,7 +18057,7 @@
         </is>
       </c>
       <c r="N273" s="3" t="n">
-        <v>46085.61403935185</v>
+        <v>46085.7308449074</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -18106,7 +18121,7 @@
         <v>1</v>
       </c>
       <c r="N274" s="3" t="n">
-        <v>46085.63672453703</v>
+        <v>46085.71091435185</v>
       </c>
       <c r="O274" t="inlineStr">
         <is>
@@ -18378,11 +18393,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C279" t="inlineStr">
-        <is>
-          <t>10.69.5.149</t>
-        </is>
-      </c>
       <c r="D279" t="n">
         <v>2014</v>
       </c>
@@ -18423,7 +18433,7 @@
         <v>2</v>
       </c>
       <c r="N279" s="3" t="n">
-        <v>46085.62831018519</v>
+        <v>46085.70078703704</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -18674,7 +18684,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46085.65175925926</v>
+        <v>46085.72631944445</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18738,7 +18748,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46085.62760416666</v>
+        <v>46085.70715277778</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18861,7 +18871,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46085.61483796296</v>
+        <v>46085.73341435185</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18989,7 +18999,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46085.62202546297</v>
+        <v>46085.73733796296</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19783,7 +19793,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46085.64788194445</v>
+        <v>46085.72796296296</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20899,7 +20909,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46085.61898148148</v>
+        <v>46085.7303125</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21624,7 +21634,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46085.64829861111</v>
+        <v>46085.72340277778</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21688,7 +21698,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46085.62974537037</v>
+        <v>46085.71018518518</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21752,7 +21762,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46085.6346875</v>
+        <v>46085.71355324074</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21816,7 +21826,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46085.63048611111</v>
+        <v>46085.71163194445</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21880,7 +21890,7 @@
         <v>1</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46085.64810185185</v>
+        <v>46085.6875462963</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21944,7 +21954,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46085.63469907407</v>
+        <v>46085.71163194445</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22008,7 +22018,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46085.64354166666</v>
+        <v>46085.7241087963</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22072,7 +22082,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46085.64810185185</v>
+        <v>46085.72849537037</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -23651,7 +23661,7 @@
         <v>1</v>
       </c>
       <c r="N363" s="3" t="n">
-        <v>46085.63637731481</v>
+        <v>46085.6718287037</v>
       </c>
       <c r="O363" t="inlineStr">
         <is>
@@ -23843,7 +23853,7 @@
         </is>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46085.63165509259</v>
+        <v>46085.70670138889</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
@@ -23862,11 +23872,6 @@
           <t>RH</t>
         </is>
       </c>
-      <c r="C367" t="inlineStr">
-        <is>
-          <t>10.69.3.13</t>
-        </is>
-      </c>
       <c r="D367" t="n">
         <v>2025</v>
       </c>
@@ -23909,7 +23914,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46085.64142361111</v>
+        <v>46085.67704861111</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -23978,7 +23983,7 @@
         <v>1</v>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46085.63322916667</v>
+        <v>46085.7053125</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24047,7 +24052,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46085.63648148148</v>
+        <v>46085.6772337963</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24323,7 +24328,7 @@
         <v>1</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46085.62398148148</v>
+        <v>46085.70153935185</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24389,7 +24394,7 @@
         </is>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46085.64805555555</v>
+        <v>46085.72375</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24408,11 +24413,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C375" t="inlineStr">
-        <is>
-          <t>10.69.3.72</t>
-        </is>
-      </c>
       <c r="D375" t="n">
         <v>2025</v>
       </c>
@@ -24458,7 +24458,7 @@
         <v>1</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46085.6525462963</v>
+        <v>46085.73032407407</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24527,7 +24527,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46085.62616898148</v>
+        <v>46085.70646990741</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -24596,7 +24596,7 @@
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46085.62660879629</v>
+        <v>46085.70697916667</v>
       </c>
       <c r="O377" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-05 07:52:04.792428
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -434,7 +434,7 @@
   <cols>
     <col width="25.2" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="15.6" customWidth="1" min="3" max="3"/>
+    <col width="32.4" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="10.8" customWidth="1" min="5" max="5"/>
     <col width="50.4" customWidth="1" min="6" max="6"/>
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46085.70050925926</v>
+        <v>46086.31189814815</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46085.73425925926</v>
+        <v>46086.29811342592</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46085.71910879629</v>
+        <v>46086.30407407408</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46085.73716435185</v>
+        <v>46086.28376157407</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46085.70717592593</v>
+        <v>46086.29634259259</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1702,7 +1702,7 @@
         <v>1</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>46085.71967592592</v>
+        <v>46086.30377314815</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1844,11 +1844,6 @@
           <t>AUDITORIO</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>10.69.3.146</t>
-        </is>
-      </c>
       <c r="D22" t="n">
         <v>2018</v>
       </c>
@@ -1889,7 +1884,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>46085.71766203704</v>
+        <v>46086.16684027778</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -1948,7 +1943,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46085.71467592593</v>
+        <v>46086.13231481481</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2004,7 +1999,7 @@
         </is>
       </c>
       <c r="N24" s="3" t="n">
-        <v>46085.21767361111</v>
+        <v>46086.18418981481</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2122,7 +2117,7 @@
         <v>1</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>46085.61695601852</v>
+        <v>46086.18706018518</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2183,7 +2178,7 @@
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46085.69731481482</v>
+        <v>46085.73777777778</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6578,7 +6573,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46085.70060185185</v>
+        <v>46085.82043981482</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6711,7 +6706,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46085.73667824074</v>
+        <v>46085.81972222222</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6849,7 +6844,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46085.73212962963</v>
+        <v>46086.31811342593</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -7056,7 +7051,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46085.72237268519</v>
+        <v>46085.79913194444</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7451,7 +7446,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46085.72298611111</v>
+        <v>46086.3041087963</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7520,7 +7515,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46085.72274305556</v>
+        <v>46086.31641203703</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7589,7 +7584,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46085.70056712963</v>
+        <v>46086.2852662037</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7658,7 +7653,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46085.72881944444</v>
+        <v>46086.30168981481</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7727,7 +7722,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46085.70186342593</v>
+        <v>46086.28731481481</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7796,7 +7791,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46085.71254629629</v>
+        <v>46086.3078125</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7862,7 +7857,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46085.73488425926</v>
+        <v>46086.30872685185</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7950,11 +7945,6 @@
           <t>DP</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>10.69.3.23</t>
-        </is>
-      </c>
       <c r="D116" t="n">
         <v>2025</v>
       </c>
@@ -8225,7 +8215,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>10.69.3.98</t>
+          <t>fe80::3df5:59e9:a13f:475e</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -8273,7 +8263,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46085.71229166666</v>
+        <v>46086.28118055555</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8408,7 +8398,7 @@
         <v>2</v>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46085.70680555556</v>
+        <v>46085.82665509259</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8477,7 +8467,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46085.7311574074</v>
+        <v>46086.30555555555</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8546,7 +8536,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46085.72425925926</v>
+        <v>46086.30699074074</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8684,7 +8674,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46085.70788194444</v>
+        <v>46086.0124074074</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8753,7 +8743,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46085.68497685185</v>
+        <v>46086.3174537037</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8955,7 +8945,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46085.69841435185</v>
+        <v>46085.7397337963</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9088,7 +9078,7 @@
         <v>1</v>
       </c>
       <c r="N132" s="3" t="n">
-        <v>46085.73224537037</v>
+        <v>46085.81108796296</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -9152,7 +9142,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46085.70248842592</v>
+        <v>46085.8197337963</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9216,7 +9206,7 @@
         <v>1</v>
       </c>
       <c r="N134" s="3" t="n">
-        <v>46085.70763888889</v>
+        <v>46085.82491898148</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -9407,7 +9397,7 @@
         <v>1</v>
       </c>
       <c r="N137" s="3" t="n">
-        <v>46085.72079861111</v>
+        <v>46085.79796296296</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -9471,7 +9461,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46085.7184375</v>
+        <v>46085.79331018519</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9535,7 +9525,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46085.70165509259</v>
+        <v>46085.81833333334</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9599,7 +9589,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46085.71903935185</v>
+        <v>46085.79444444444</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9663,7 +9653,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46085.72380787037</v>
+        <v>46085.79899305556</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9727,7 +9717,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46085.72184027778</v>
+        <v>46085.79775462963</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9791,7 +9781,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46085.70356481482</v>
+        <v>46085.82048611111</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9919,7 +9909,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46085.7003587963</v>
+        <v>46085.82650462963</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9983,7 +9973,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46085.73314814815</v>
+        <v>46085.85682870371</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10047,7 +10037,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46085.72341435185</v>
+        <v>46085.80381944445</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10111,7 +10101,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46085.72863425926</v>
+        <v>46085.84038194444</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10175,7 +10165,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46085.73158564815</v>
+        <v>46085.84305555555</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10239,7 +10229,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46085.7229050926</v>
+        <v>46085.80010416666</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10303,7 +10293,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46085.69824074074</v>
+        <v>46085.81259259259</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10426,7 +10416,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46085.70259259259</v>
+        <v>46085.81927083333</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10490,7 +10480,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46085.70716435185</v>
+        <v>46085.81774305556</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10554,7 +10544,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46085.61849537037</v>
+        <v>46086.30815972222</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10746,7 +10736,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46085.73491898148</v>
+        <v>46086.30636574074</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10810,7 +10800,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46085.71118055555</v>
+        <v>46086.30791666666</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10874,7 +10864,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46085.71289351852</v>
+        <v>46085.86633101852</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10938,7 +10928,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46085.72765046296</v>
+        <v>46085.80440972222</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -11066,7 +11056,7 @@
         <v>2</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46085.70638888889</v>
+        <v>46086.2862962963</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11127,10 +11117,10 @@
         </is>
       </c>
       <c r="M164" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46085.59677083333</v>
+        <v>46086.28998842592</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11322,7 +11312,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46085.5609837963</v>
+        <v>46086.31085648148</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11383,10 +11373,10 @@
         </is>
       </c>
       <c r="M168" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46085.7074074074</v>
+        <v>46086.28731481481</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11450,7 +11440,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46085.69922453703</v>
+        <v>46085.77782407407</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11578,7 +11568,7 @@
         <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46085.73430555555</v>
+        <v>46085.76966435185</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11639,10 +11629,10 @@
         </is>
       </c>
       <c r="M172" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46085.72125</v>
+        <v>46086.28625</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11706,7 +11696,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46085.70825231481</v>
+        <v>46086.31583333333</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11770,7 +11760,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46085.56381944445</v>
+        <v>46086.30042824074</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11962,7 +11952,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46085.70324074074</v>
+        <v>46086.2840162037</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12026,7 +12016,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46085.70167824074</v>
+        <v>46085.81563657407</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12090,7 +12080,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46085.73232638889</v>
+        <v>46085.81025462963</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12154,7 +12144,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46085.70869212963</v>
+        <v>46085.82769675926</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12351,7 +12341,7 @@
         <v>2</v>
       </c>
       <c r="N183" s="3" t="n">
-        <v>46085.72532407408</v>
+        <v>46085.80945601852</v>
       </c>
       <c r="O183" t="inlineStr">
         <is>
@@ -12479,7 +12469,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46085.70818287037</v>
+        <v>46085.80268518518</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12543,7 +12533,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46085.7069675926</v>
+        <v>46085.82383101852</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12693,11 +12683,6 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
-      <c r="C189" t="inlineStr">
-        <is>
-          <t>10.69.5.59</t>
-        </is>
-      </c>
       <c r="D189" t="n">
         <v>2015</v>
       </c>
@@ -12735,7 +12720,7 @@
         </is>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46085.73719907407</v>
+        <v>46085.81462962963</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12799,7 +12784,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46085.69954861111</v>
+        <v>46085.81200231481</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12863,7 +12848,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46085.69976851852</v>
+        <v>46085.81407407407</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12988,7 +12973,7 @@
         <v>2</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46085.72739583333</v>
+        <v>46086.3015625</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13052,7 +13037,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46085.7303125</v>
+        <v>46085.80498842592</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13116,7 +13101,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46085.73090277778</v>
+        <v>46085.80768518519</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13180,7 +13165,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46085.72971064815</v>
+        <v>46085.84046296297</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13308,7 +13293,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46085.73202546296</v>
+        <v>46085.81040509259</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13372,7 +13357,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46085.71100694445</v>
+        <v>46085.82506944444</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13433,7 +13418,7 @@
         </is>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46085.70883101852</v>
+        <v>46085.82528935185</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13497,7 +13482,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46085.71224537037</v>
+        <v>46085.79383101852</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13561,7 +13546,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46085.71519675926</v>
+        <v>46085.79126157407</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13625,7 +13610,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46085.71192129629</v>
+        <v>46085.7903125</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13689,7 +13674,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46085.7140625</v>
+        <v>46085.79150462963</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13753,7 +13738,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46085.71332175926</v>
+        <v>46085.82641203704</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13817,7 +13802,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46085.7094212963</v>
+        <v>46085.82814814815</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13881,7 +13866,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46085.705</v>
+        <v>46085.82481481481</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13945,7 +13930,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46085.73180555556</v>
+        <v>46085.80986111111</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14009,7 +13994,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46085.73616898148</v>
+        <v>46085.81422453704</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14073,7 +14058,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46085.7155787037</v>
+        <v>46085.79266203703</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14137,7 +14122,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46085.70372685185</v>
+        <v>46085.82039351852</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14201,7 +14186,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46085.72895833333</v>
+        <v>46085.8058912037</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14265,7 +14250,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46085.71864583333</v>
+        <v>46085.79451388889</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14329,7 +14314,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46085.7297337963</v>
+        <v>46085.80710648148</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14393,7 +14378,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46085.71267361111</v>
+        <v>46085.82489583334</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14457,7 +14442,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46085.71839120371</v>
+        <v>46085.79701388889</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14521,7 +14506,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46085.72255787037</v>
+        <v>46085.80313657408</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14585,7 +14570,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46085.6996412037</v>
+        <v>46085.81866898148</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14654,7 +14639,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46085.70063657407</v>
+        <v>46085.82170138889</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14718,7 +14703,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46085.73393518518</v>
+        <v>46085.81055555555</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14782,7 +14767,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46085.73297453704</v>
+        <v>46085.81202546296</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14846,7 +14831,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46085.72020833333</v>
+        <v>46085.79569444444</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14910,7 +14895,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46085.71009259259</v>
+        <v>46085.82674768518</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14974,7 +14959,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46085.70311342592</v>
+        <v>46085.8172337963</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15002,7 +14987,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46085.71528935185</v>
+        <v>46085.79258101852</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15066,7 +15051,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46085.70755787037</v>
+        <v>46085.82489583334</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15130,7 +15115,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46085.72064814815</v>
+        <v>46085.79924768519</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15194,7 +15179,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46085.73358796296</v>
+        <v>46085.81381944445</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15258,7 +15243,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46085.70483796296</v>
+        <v>46086.3191087963</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15322,7 +15307,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46085.70578703703</v>
+        <v>46085.82028935185</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15386,7 +15371,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46085.70019675926</v>
+        <v>46085.81546296296</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15450,7 +15435,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46085.72009259259</v>
+        <v>46085.79754629629</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15514,7 +15499,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46085.70136574074</v>
+        <v>46085.8184375</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15578,7 +15563,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46085.70809027777</v>
+        <v>46085.82219907407</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15642,7 +15627,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46085.73731481482</v>
+        <v>46085.81569444444</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15706,7 +15691,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46085.72505787037</v>
+        <v>46085.80333333334</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15770,7 +15755,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46085.735</v>
+        <v>46085.8156712963</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15898,7 +15883,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46085.71643518518</v>
+        <v>46085.82884259259</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -15962,7 +15947,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46085.70855324074</v>
+        <v>46085.82322916666</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16026,7 +16011,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46085.71254629629</v>
+        <v>46085.82479166667</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16090,7 +16075,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46085.71284722222</v>
+        <v>46085.82793981482</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16109,6 +16094,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>10.69.5.112</t>
+        </is>
+      </c>
       <c r="D243" t="n">
         <v>2019</v>
       </c>
@@ -16149,7 +16139,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46085.71618055556</v>
+        <v>46086.30890046297</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16213,7 +16203,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46085.72072916666</v>
+        <v>46086.31018518518</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16277,7 +16267,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46085.70700231481</v>
+        <v>46086.31068287037</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16341,7 +16331,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46085.72033564815</v>
+        <v>46085.80152777778</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16405,7 +16395,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46085.70965277778</v>
+        <v>46086.30935185185</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16469,7 +16459,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46085.71336805556</v>
+        <v>46086.30949074074</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16533,7 +16523,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46085.70394675926</v>
+        <v>46086.30943287037</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16597,7 +16587,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46085.71738425926</v>
+        <v>46086.30997685185</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16661,7 +16651,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46085.71113425926</v>
+        <v>46086.30987268518</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16725,7 +16715,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46085.71475694444</v>
+        <v>46085.79512731481</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16783,7 +16773,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46085.709375</v>
+        <v>46085.82708333333</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16847,7 +16837,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46085.73068287037</v>
+        <v>46085.80891203704</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16911,7 +16901,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46085.71269675926</v>
+        <v>46085.78909722222</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -16975,7 +16965,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46085.71335648148</v>
+        <v>46085.82856481482</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17039,7 +17029,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46085.72325231481</v>
+        <v>46085.83268518518</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17231,7 +17221,7 @@
         <v>2</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46085.71630787037</v>
+        <v>46085.79364583334</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17295,7 +17285,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46085.73729166666</v>
+        <v>46085.81765046297</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17359,7 +17349,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46085.73299768518</v>
+        <v>46086.31778935185</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17423,7 +17413,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46085.70221064815</v>
+        <v>46085.81559027778</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17487,7 +17477,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46085.70451388889</v>
+        <v>46085.82016203704</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17551,7 +17541,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46085.71907407408</v>
+        <v>46085.83751157407</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17615,7 +17605,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46085.73752314815</v>
+        <v>46085.81086805555</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17743,7 +17733,7 @@
         <v>1</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46085.72050925926</v>
+        <v>46085.793125</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17804,7 +17794,7 @@
         </is>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46085.71575231481</v>
+        <v>46086.31225694445</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17868,7 +17858,7 @@
         <v>1</v>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46085.72497685185</v>
+        <v>46086.11908564815</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -17932,7 +17922,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46085.70480324074</v>
+        <v>46086.32050925926</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -18057,7 +18047,7 @@
         </is>
       </c>
       <c r="N273" s="3" t="n">
-        <v>46085.7308449074</v>
+        <v>46086.30993055556</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -18121,7 +18111,7 @@
         <v>1</v>
       </c>
       <c r="N274" s="3" t="n">
-        <v>46085.71091435185</v>
+        <v>46085.86240740741</v>
       </c>
       <c r="O274" t="inlineStr">
         <is>
@@ -18374,7 +18364,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46085.57907407408</v>
+        <v>46086.31916666667</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18393,6 +18383,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>10.69.5.149</t>
+        </is>
+      </c>
       <c r="D279" t="n">
         <v>2014</v>
       </c>
@@ -18433,7 +18428,7 @@
         <v>2</v>
       </c>
       <c r="N279" s="3" t="n">
-        <v>46085.70078703704</v>
+        <v>46085.82259259259</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -18620,7 +18615,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46085.58581018518</v>
+        <v>46086.31890046296</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18684,7 +18679,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46085.72631944445</v>
+        <v>46085.87144675926</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18748,7 +18743,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46085.70715277778</v>
+        <v>46085.82577546296</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18807,7 +18802,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46085.58457175926</v>
+        <v>46086.20561342593</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18871,7 +18866,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46085.73341435185</v>
+        <v>46085.81243055555</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18935,7 +18930,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46085.54704861111</v>
+        <v>46086.31693287037</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -18999,7 +18994,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46085.73733796296</v>
+        <v>46085.85211805555</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19793,7 +19788,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46085.72796296296</v>
+        <v>46086.3127662037</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20909,7 +20904,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46085.7303125</v>
+        <v>46086.31637731481</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21634,7 +21629,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46085.72340277778</v>
+        <v>46086.28171296296</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21698,7 +21693,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46085.71018518518</v>
+        <v>46086.31944444445</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21762,7 +21757,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46085.71355324074</v>
+        <v>46086.28230324074</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21826,7 +21821,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46085.71163194445</v>
+        <v>46086.28180555555</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21887,10 +21882,10 @@
         </is>
       </c>
       <c r="M335" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46085.6875462963</v>
+        <v>46086.29824074074</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21954,7 +21949,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46085.71163194445</v>
+        <v>46086.281875</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22018,7 +22013,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46085.7241087963</v>
+        <v>46086.31903935185</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22082,7 +22077,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46085.72849537037</v>
+        <v>46086.31047453704</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -23872,6 +23867,11 @@
           <t>RH</t>
         </is>
       </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>10.69.3.13</t>
+        </is>
+      </c>
       <c r="D367" t="n">
         <v>2025</v>
       </c>
@@ -23914,7 +23914,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46085.67704861111</v>
+        <v>46086.29527777778</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -23983,7 +23983,7 @@
         <v>1</v>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46085.7053125</v>
+        <v>46086.30815972222</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24328,7 +24328,7 @@
         <v>1</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46085.70153935185</v>
+        <v>46085.73892361111</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24394,7 +24394,7 @@
         </is>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46085.72375</v>
+        <v>46086.30686342593</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24458,7 +24458,7 @@
         <v>1</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46085.73032407407</v>
+        <v>46085.81159722222</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24527,7 +24527,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46085.70646990741</v>
+        <v>46085.78506944444</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -24596,7 +24596,7 @@
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46085.70697916667</v>
+        <v>46086.30560185185</v>
       </c>
       <c r="O377" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-05 09:52:08.325985
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q377"/>
+  <dimension ref="A1:Q378"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25.2" customWidth="1" min="1" max="1"/>
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46086.31189814815</v>
+        <v>46086.39331018519</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46085.6749537037</v>
+        <v>46086.39651620371</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46085.69936342593</v>
+        <v>46086.39417824074</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46085.70461805556</v>
+        <v>46086.37658564815</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46086.29811342592</v>
+        <v>46086.37372685185</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46086.30407407408</v>
+        <v>46086.38474537037</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46086.28376157407</v>
+        <v>46086.40094907407</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46086.29634259259</v>
+        <v>46086.3782175926</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1702,7 +1702,7 @@
         <v>1</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>46086.30377314815</v>
+        <v>46086.38354166667</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1844,6 +1844,11 @@
           <t>AUDITORIO</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>10.69.3.146</t>
+        </is>
+      </c>
       <c r="D22" t="n">
         <v>2018</v>
       </c>
@@ -1884,7 +1889,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>46086.16684027778</v>
+        <v>46086.38715277778</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -6504,7 +6509,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46085.71253472222</v>
+        <v>46086.40284722222</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6656,11 +6661,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>10.69.3.94</t>
-        </is>
-      </c>
       <c r="D97" t="n">
         <v>2025</v>
       </c>
@@ -6706,7 +6706,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46085.81972222222</v>
+        <v>46086.38972222222</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6775,7 +6775,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46085.69483796296</v>
+        <v>46086.38306712963</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6844,7 +6844,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46086.31811342593</v>
+        <v>46086.40141203703</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6913,7 +6913,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46085.71142361111</v>
+        <v>46086.37782407407</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -7308,7 +7308,7 @@
         <v>1</v>
       </c>
       <c r="N106" s="3" t="n">
-        <v>46085.67232638889</v>
+        <v>46086.36996527778</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -7446,7 +7446,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46086.3041087963</v>
+        <v>46086.37863425926</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7515,7 +7515,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46086.31641203703</v>
+        <v>46086.39784722222</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7584,7 +7584,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46086.2852662037</v>
+        <v>46086.36831018519</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7653,7 +7653,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46086.30168981481</v>
+        <v>46086.38293981482</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7722,7 +7722,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46086.28731481481</v>
+        <v>46086.40136574074</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7791,7 +7791,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46086.3078125</v>
+        <v>46086.39009259259</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7857,7 +7857,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46086.30872685185</v>
+        <v>46086.38819444444</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7926,7 +7926,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46085.68173611111</v>
+        <v>46086.39872685185</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7945,6 +7945,11 @@
           <t>DP</t>
         </is>
       </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>10.69.3.23</t>
+        </is>
+      </c>
       <c r="D116" t="n">
         <v>2025</v>
       </c>
@@ -7990,7 +7995,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46085.67766203704</v>
+        <v>46086.40329861111</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8056,7 +8061,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46085.68864583333</v>
+        <v>46086.37034722222</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8194,7 +8199,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46085.67530092593</v>
+        <v>46086.38538194444</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8329,7 +8334,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46085.6836574074</v>
+        <v>46086.37353009259</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8467,7 +8472,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46086.30555555555</v>
+        <v>46086.38405092592</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8536,7 +8541,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46086.30699074074</v>
+        <v>46086.38666666667</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8743,7 +8748,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46086.3174537037</v>
+        <v>46086.39893518519</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8812,7 +8817,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46085.68760416667</v>
+        <v>46086.37872685185</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8881,7 +8886,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46084.92917824074</v>
+        <v>46086.37692129629</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -8900,6 +8905,11 @@
           <t>ADM/FIN</t>
         </is>
       </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>10.69.3.6</t>
+        </is>
+      </c>
       <c r="D130" t="n">
         <v>2025</v>
       </c>
@@ -8945,7 +8955,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46085.7397337963</v>
+        <v>46086.39230324074</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9078,7 +9088,7 @@
         <v>1</v>
       </c>
       <c r="N132" s="3" t="n">
-        <v>46085.81108796296</v>
+        <v>46086.37386574074</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -9397,7 +9407,7 @@
         <v>1</v>
       </c>
       <c r="N137" s="3" t="n">
-        <v>46085.79796296296</v>
+        <v>46086.38385416667</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -9589,7 +9599,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46085.79444444444</v>
+        <v>46086.3634837963</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9653,7 +9663,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46085.79899305556</v>
+        <v>46086.39488425926</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9717,7 +9727,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46085.79775462963</v>
+        <v>46086.40315972222</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9781,7 +9791,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46085.82048611111</v>
+        <v>46086.4037962963</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9845,7 +9855,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46085.69739583333</v>
+        <v>46086.39163194445</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9909,7 +9919,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46085.82650462963</v>
+        <v>46086.36521990741</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9973,7 +9983,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46085.85682870371</v>
+        <v>46086.40070601852</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10037,7 +10047,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46085.80381944445</v>
+        <v>46086.38041666667</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10101,7 +10111,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46085.84038194444</v>
+        <v>46086.38905092593</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10165,7 +10175,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46085.84305555555</v>
+        <v>46086.38391203704</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10229,7 +10239,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46085.80010416666</v>
+        <v>46086.38950231481</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10293,7 +10303,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46085.81259259259</v>
+        <v>46086.38180555555</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10352,7 +10362,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46084.64226851852</v>
+        <v>46086.32950231482</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10416,7 +10426,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46085.81927083333</v>
+        <v>46086.36651620371</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10480,7 +10490,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46085.81774305556</v>
+        <v>46086.37810185185</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10544,7 +10554,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46086.30815972222</v>
+        <v>46086.38533564815</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10608,7 +10618,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46085.57560185185</v>
+        <v>46086.36865740741</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10736,7 +10746,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46086.30636574074</v>
+        <v>46086.38480324074</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10800,7 +10810,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46086.30791666666</v>
+        <v>46086.38445601852</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10864,7 +10874,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46085.86633101852</v>
+        <v>46086.37545138889</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10928,7 +10938,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46085.80440972222</v>
+        <v>46086.37180555556</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -10992,7 +11002,7 @@
         <v>2</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46085.33334490741</v>
+        <v>46086.36907407407</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11056,7 +11066,7 @@
         <v>2</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46086.2862962963</v>
+        <v>46086.40212962963</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11117,10 +11127,10 @@
         </is>
       </c>
       <c r="M164" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46086.28998842592</v>
+        <v>46086.3675</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11184,7 +11194,7 @@
         <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46085.603125</v>
+        <v>46086.38680555556</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11248,7 +11258,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46085.59586805556</v>
+        <v>46086.36831018519</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11312,7 +11322,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46086.31085648148</v>
+        <v>46086.39112268519</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11373,10 +11383,10 @@
         </is>
       </c>
       <c r="M168" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46086.28731481481</v>
+        <v>46086.36736111111</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11440,7 +11450,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46085.77782407407</v>
+        <v>46086.36918981482</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11501,10 +11511,10 @@
         </is>
       </c>
       <c r="M170" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46085.56376157407</v>
+        <v>46086.36613425926</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11632,7 +11642,7 @@
         <v>1</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46086.28625</v>
+        <v>46086.3653587963</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11696,7 +11706,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46086.31583333333</v>
+        <v>46086.39128472222</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11760,7 +11770,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46086.30042824074</v>
+        <v>46086.38056712963</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11952,7 +11962,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46086.2840162037</v>
+        <v>46086.39571759259</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12016,7 +12026,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46085.81563657407</v>
+        <v>46086.37681712963</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12080,7 +12090,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46085.81025462963</v>
+        <v>46086.37944444444</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12533,7 +12543,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46085.82383101852</v>
+        <v>46086.40305555556</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12597,7 +12607,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46085.69630787037</v>
+        <v>46086.39873842592</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12683,6 +12693,11 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>10.69.5.59</t>
+        </is>
+      </c>
       <c r="D189" t="n">
         <v>2015</v>
       </c>
@@ -12720,7 +12735,7 @@
         </is>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46085.81462962963</v>
+        <v>46086.37740740741</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12784,7 +12799,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46085.81200231481</v>
+        <v>46086.39013888889</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12848,7 +12863,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46085.81407407407</v>
+        <v>46086.40193287037</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12973,7 +12988,7 @@
         <v>2</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46086.3015625</v>
+        <v>46086.38114583334</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13037,7 +13052,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46085.80498842592</v>
+        <v>46086.39678240741</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13101,7 +13116,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46085.80768518519</v>
+        <v>46086.36760416667</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13229,7 +13244,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46085.55965277777</v>
+        <v>46086.38783564815</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13293,7 +13308,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46085.81040509259</v>
+        <v>46086.39252314815</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13357,7 +13372,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46085.82506944444</v>
+        <v>46086.36905092592</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13482,7 +13497,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46085.79383101852</v>
+        <v>46086.37502314815</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13546,7 +13561,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46085.79126157407</v>
+        <v>46086.37431712963</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13610,7 +13625,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46085.7903125</v>
+        <v>46086.40159722222</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13674,7 +13689,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46085.79150462963</v>
+        <v>46086.36267361111</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13738,7 +13753,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46085.82641203704</v>
+        <v>46086.3653587963</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13802,7 +13817,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46085.82814814815</v>
+        <v>46086.40056712963</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13866,7 +13881,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46085.82481481481</v>
+        <v>46086.3778587963</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13930,7 +13945,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46085.80986111111</v>
+        <v>46086.37548611111</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -13994,7 +14009,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46085.81422453704</v>
+        <v>46086.37436342592</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14058,7 +14073,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46085.79266203703</v>
+        <v>46086.37579861111</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14122,7 +14137,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46085.82039351852</v>
+        <v>46086.37462962963</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14186,7 +14201,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46085.8058912037</v>
+        <v>46086.38460648148</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14250,7 +14265,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46085.79451388889</v>
+        <v>46086.37756944444</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14378,7 +14393,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46085.82489583334</v>
+        <v>46086.37563657408</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14442,7 +14457,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46085.79701388889</v>
+        <v>46086.37804398148</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14506,7 +14521,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46085.80313657408</v>
+        <v>46086.37637731482</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14570,7 +14585,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46085.81866898148</v>
+        <v>46086.36542824074</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14639,7 +14654,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46085.82170138889</v>
+        <v>46086.37532407408</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14703,7 +14718,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46085.81055555555</v>
+        <v>46086.38393518519</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14767,7 +14782,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46085.81202546296</v>
+        <v>46086.3816087963</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14959,7 +14974,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46085.8172337963</v>
+        <v>46086.40224537037</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -14983,6 +14998,42 @@
           <t>10.69.5.94</t>
         </is>
       </c>
+      <c r="D225" t="n">
+        <v>2019</v>
+      </c>
+      <c r="E225" t="n">
+        <v>73645</v>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>Microsoft Windows 8.1 Pro</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>BRJ525SZ0B</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>Intel Core i5</t>
+        </is>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>8 GB</t>
+        </is>
+      </c>
+      <c r="K225" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>HP 402 G1 SFF Business PC</t>
+        </is>
+      </c>
       <c r="M225" t="n">
         <v>1</v>
       </c>
@@ -15051,7 +15102,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46085.82489583334</v>
+        <v>46086.37131944444</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15115,7 +15166,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46085.79924768519</v>
+        <v>46086.37519675926</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15179,7 +15230,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46085.81381944445</v>
+        <v>46086.39850694445</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15243,7 +15294,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46086.3191087963</v>
+        <v>46086.39563657407</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15307,7 +15358,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46085.82028935185</v>
+        <v>46086.36827546296</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15371,7 +15422,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46085.81546296296</v>
+        <v>46086.3869212963</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15435,7 +15486,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46085.79754629629</v>
+        <v>46086.37006944444</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15499,7 +15550,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46085.8184375</v>
+        <v>46086.40354166667</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15563,7 +15614,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46085.82219907407</v>
+        <v>46086.37576388889</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15627,7 +15678,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46085.81569444444</v>
+        <v>46086.38116898148</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15691,7 +15742,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46085.80333333334</v>
+        <v>46086.39325231482</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15755,7 +15806,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46085.8156712963</v>
+        <v>46086.37673611111</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15819,7 +15870,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46085.61004629629</v>
+        <v>46086.37275462963</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15883,7 +15934,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46085.82884259259</v>
+        <v>46086.37424768518</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -16011,7 +16062,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46085.82479166667</v>
+        <v>46086.36282407407</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16075,7 +16126,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46085.82793981482</v>
+        <v>46086.3744212963</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16094,11 +16145,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C243" t="inlineStr">
-        <is>
-          <t>10.69.5.112</t>
-        </is>
-      </c>
       <c r="D243" t="n">
         <v>2019</v>
       </c>
@@ -16139,7 +16185,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46086.30890046297</v>
+        <v>46086.34685185185</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16267,7 +16313,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46086.31068287037</v>
+        <v>46086.3753125</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16331,7 +16377,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46085.80152777778</v>
+        <v>46086.36740740741</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16395,7 +16441,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46086.30935185185</v>
+        <v>46086.38730324074</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16459,7 +16505,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46086.30949074074</v>
+        <v>46086.38521990741</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16523,7 +16569,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46086.30943287037</v>
+        <v>46086.3849537037</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16587,7 +16633,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46086.30997685185</v>
+        <v>46086.38659722222</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16651,7 +16697,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46086.30987268518</v>
+        <v>46086.38626157407</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16715,7 +16761,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46085.79512731481</v>
+        <v>46086.40398148148</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16773,7 +16819,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46085.82708333333</v>
+        <v>46086.40047453704</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16837,7 +16883,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46085.80891203704</v>
+        <v>46086.38297453704</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16901,7 +16947,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46085.78909722222</v>
+        <v>46086.36715277778</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -16965,7 +17011,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46085.82856481482</v>
+        <v>46086.3671875</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17029,7 +17075,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46085.83268518518</v>
+        <v>46086.40369212963</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17093,7 +17139,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46085.598125</v>
+        <v>46086.32549768518</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17157,7 +17203,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46085.59555555556</v>
+        <v>46086.39956018519</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17285,7 +17331,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46085.81765046297</v>
+        <v>46086.38427083333</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17349,7 +17395,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46086.31778935185</v>
+        <v>46086.39978009259</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17413,7 +17459,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46085.81559027778</v>
+        <v>46086.37892361111</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17477,7 +17523,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46085.82016203704</v>
+        <v>46086.36898148148</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17541,7 +17587,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46085.83751157407</v>
+        <v>46086.37188657407</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17605,7 +17651,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46085.81086805555</v>
+        <v>46086.36939814815</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17794,7 +17840,7 @@
         </is>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46086.31225694445</v>
+        <v>46086.39587962963</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17922,7 +17968,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46086.32050925926</v>
+        <v>46086.39542824074</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -18047,7 +18093,7 @@
         </is>
       </c>
       <c r="N273" s="3" t="n">
-        <v>46086.30993055556</v>
+        <v>46086.38736111111</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -18130,11 +18176,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C275" t="inlineStr">
-        <is>
-          <t>10.69.5.145</t>
-        </is>
-      </c>
       <c r="D275" t="n">
         <v>2013</v>
       </c>
@@ -18300,7 +18341,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46085.55493055555</v>
+        <v>46086.40219907407</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18364,7 +18405,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46086.31916666667</v>
+        <v>46086.39631944444</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18383,11 +18424,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C279" t="inlineStr">
-        <is>
-          <t>10.69.5.149</t>
-        </is>
-      </c>
       <c r="D279" t="n">
         <v>2014</v>
       </c>
@@ -18492,7 +18528,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46085.57841435185</v>
+        <v>46086.37677083333</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18551,7 +18587,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46085.57290509259</v>
+        <v>46086.37296296296</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18615,7 +18651,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46086.31890046296</v>
+        <v>46086.39950231482</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18679,7 +18715,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46085.87144675926</v>
+        <v>46086.37445601852</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18743,7 +18779,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46085.82577546296</v>
+        <v>46086.36570601852</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18802,7 +18838,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46086.20561342593</v>
+        <v>46086.37398148148</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18866,7 +18902,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46085.81243055555</v>
+        <v>46086.37695601852</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18930,7 +18966,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46086.31693287037</v>
+        <v>46086.39809027778</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19788,7 +19824,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46086.3127662037</v>
+        <v>46086.389375</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20904,7 +20940,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46086.31637731481</v>
+        <v>46086.39420138889</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21629,7 +21665,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46086.28171296296</v>
+        <v>46086.40112268519</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21693,7 +21729,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46086.31944444445</v>
+        <v>46086.39383101852</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21757,7 +21793,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46086.28230324074</v>
+        <v>46086.39548611111</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21821,7 +21857,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46086.28180555555</v>
+        <v>46086.39841435185</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21885,7 +21921,7 @@
         <v>2</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46086.29824074074</v>
+        <v>46086.37752314815</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21949,7 +21985,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46086.281875</v>
+        <v>46086.40157407407</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22013,7 +22049,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46086.31903935185</v>
+        <v>46086.40071759259</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22077,7 +22113,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46086.31047453704</v>
+        <v>46086.39075231482</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22205,7 +22241,7 @@
         <v>2</v>
       </c>
       <c r="N340" s="3" t="n">
-        <v>46085.56974537037</v>
+        <v>46086.33009259259</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -22586,7 +22622,7 @@
         <v>1</v>
       </c>
       <c r="N346" s="3" t="n">
-        <v>46085.5897800926</v>
+        <v>46086.37422453704</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -22650,7 +22686,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46085.58230324074</v>
+        <v>46086.37491898148</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22714,7 +22750,7 @@
         <v>1</v>
       </c>
       <c r="N348" s="3" t="n">
-        <v>46085.58729166666</v>
+        <v>46086.37497685185</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -22775,7 +22811,7 @@
         </is>
       </c>
       <c r="N349" s="3" t="n">
-        <v>46085.42546296296</v>
+        <v>46086.37460648148</v>
       </c>
       <c r="O349" t="inlineStr">
         <is>
@@ -22839,7 +22875,7 @@
         <v>1</v>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46085.4259375</v>
+        <v>46086.37583333333</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -22903,7 +22939,7 @@
         <v>1</v>
       </c>
       <c r="N351" s="3" t="n">
-        <v>46084.5928587963</v>
+        <v>46086.37633101852</v>
       </c>
       <c r="O351" t="inlineStr">
         <is>
@@ -22914,7 +22950,7 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>PA_248</t>
+          <t>PA_247</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
@@ -22924,33 +22960,33 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>10.69.5.248</t>
+          <t>10.69.5.247</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>2019</v>
+        <v>2011</v>
       </c>
       <c r="E352" t="n">
-        <v>73645</v>
+        <v>8390</v>
       </c>
       <c r="F352" t="inlineStr">
         <is>
-          <t>Microsoft Windows 8.1 Pro</t>
+          <t>Microsoft® Windows Vista™ Business</t>
         </is>
       </c>
       <c r="G352" t="inlineStr">
         <is>
-          <t>BRJ523SG7Z</t>
+          <t>BRG827F584</t>
         </is>
       </c>
       <c r="I352" t="inlineStr">
         <is>
-          <t>Intel Core i5</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="J352" t="inlineStr">
         <is>
-          <t>6 GB</t>
+          <t>2 GB</t>
         </is>
       </c>
       <c r="K352" t="inlineStr">
@@ -22960,11 +22996,11 @@
       </c>
       <c r="L352" t="inlineStr">
         <is>
-          <t>HP 402 G1 SFF Business PC</t>
+          <t>HP Compaq dx7400 Brazil SFF PC.</t>
         </is>
       </c>
       <c r="N352" s="3" t="n">
-        <v>46080.51325231481</v>
+        <v>46086.37414351852</v>
       </c>
       <c r="O352" t="inlineStr">
         <is>
@@ -22975,7 +23011,7 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>PA_249</t>
+          <t>PA_248</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
@@ -22985,23 +23021,23 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>10.69.5.249</t>
+          <t>10.69.5.248</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>2016</v>
+        <v>2019</v>
       </c>
       <c r="E353" t="n">
-        <v>51040</v>
+        <v>73645</v>
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>Microsoft Windows 7 Professional</t>
+          <t>Microsoft Windows 8.1 Pro</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
         <is>
-          <t>BRG311F8KL</t>
+          <t>BRJ523SG7Z</t>
         </is>
       </c>
       <c r="I353" t="inlineStr">
@@ -23011,7 +23047,7 @@
       </c>
       <c r="J353" t="inlineStr">
         <is>
-          <t>4 GB</t>
+          <t>6 GB</t>
         </is>
       </c>
       <c r="K353" t="inlineStr">
@@ -23021,14 +23057,11 @@
       </c>
       <c r="L353" t="inlineStr">
         <is>
-          <t>HP Compaq Pro 4300 SFF Brazil PC</t>
-        </is>
-      </c>
-      <c r="M353" t="n">
-        <v>1</v>
+          <t>HP 402 G1 SFF Business PC</t>
+        </is>
       </c>
       <c r="N353" s="3" t="n">
-        <v>46085.60005787037</v>
+        <v>46080.51325231481</v>
       </c>
       <c r="O353" t="inlineStr">
         <is>
@@ -23039,7 +23072,7 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>PA_250</t>
+          <t>PA_249</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
@@ -23049,14 +23082,14 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>10.69.5.250</t>
+          <t>10.69.5.249</t>
         </is>
       </c>
       <c r="D354" t="n">
         <v>2016</v>
       </c>
       <c r="E354" t="n">
-        <v>43374</v>
+        <v>51040</v>
       </c>
       <c r="F354" t="inlineStr">
         <is>
@@ -23065,12 +23098,12 @@
       </c>
       <c r="G354" t="inlineStr">
         <is>
-          <t>BRG103F99B</t>
+          <t>BRG311F8KL</t>
         </is>
       </c>
       <c r="I354" t="inlineStr">
         <is>
-          <t>Intel Core 2 Duo</t>
+          <t>Intel Core i5</t>
         </is>
       </c>
       <c r="J354" t="inlineStr">
@@ -23085,14 +23118,14 @@
       </c>
       <c r="L354" t="inlineStr">
         <is>
-          <t>COMPAQ 300B MT</t>
+          <t>HP Compaq Pro 4300 SFF Brazil PC</t>
         </is>
       </c>
       <c r="M354" t="n">
         <v>1</v>
       </c>
       <c r="N354" s="3" t="n">
-        <v>46085.57380787037</v>
+        <v>46086.37416666667</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -23103,7 +23136,7 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>PA_251</t>
+          <t>PA_250</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
@@ -23113,14 +23146,14 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>10.69.5.251</t>
+          <t>10.69.5.250</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="E355" t="n">
-        <v>59162</v>
+        <v>43374</v>
       </c>
       <c r="F355" t="inlineStr">
         <is>
@@ -23129,12 +23162,12 @@
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t>BRG319F89N</t>
+          <t>BRG103F99B</t>
         </is>
       </c>
       <c r="I355" t="inlineStr">
         <is>
-          <t>Intel Core i3</t>
+          <t>Intel Core 2 Duo</t>
         </is>
       </c>
       <c r="J355" t="inlineStr">
@@ -23149,14 +23182,14 @@
       </c>
       <c r="L355" t="inlineStr">
         <is>
-          <t>HP Compaq Pro 4300 SFF Brazil PC</t>
+          <t>COMPAQ 300B MT</t>
         </is>
       </c>
       <c r="M355" t="n">
         <v>1</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46085.60575231481</v>
+        <v>46086.37462962963</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23167,7 +23200,7 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>PA_252</t>
+          <t>PA_251</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
@@ -23175,47 +23208,52 @@
           <t>OPERACAO 9.1</t>
         </is>
       </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>10.69.5.251</t>
+        </is>
+      </c>
       <c r="D356" t="n">
-        <v>2012</v>
+        <v>2017</v>
       </c>
       <c r="E356" t="n">
-        <v>2956</v>
+        <v>59162</v>
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t>Microsoft® Windows Vista™ Business</t>
+          <t>Microsoft Windows 7 Professional</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
         <is>
-          <t>J5L1JJ1</t>
+          <t>BRG319F89N</t>
         </is>
       </c>
       <c r="I356" t="inlineStr">
         <is>
-          <t>Intel Core 2 Duo</t>
+          <t>Intel Core i3</t>
         </is>
       </c>
       <c r="J356" t="inlineStr">
         <is>
-          <t>2 GB</t>
+          <t>4 GB</t>
         </is>
       </c>
       <c r="K356" t="inlineStr">
         <is>
-          <t>Dell Inc.</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="L356" t="inlineStr">
         <is>
-          <t>OptiPlex 755</t>
+          <t>HP Compaq Pro 4300 SFF Brazil PC</t>
         </is>
       </c>
       <c r="M356" t="n">
         <v>1</v>
       </c>
       <c r="N356" s="3" t="n">
-        <v>46085.41123842593</v>
+        <v>46086.37435185185</v>
       </c>
       <c r="O356" t="inlineStr">
         <is>
@@ -23226,7 +23264,7 @@
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>PA_253</t>
+          <t>PA_252</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
@@ -23236,50 +23274,50 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>10.69.5.253</t>
+          <t>10.69.5.252</t>
         </is>
       </c>
       <c r="D357" t="n">
-        <v>2019</v>
+        <v>2012</v>
       </c>
       <c r="E357" t="n">
-        <v>73645</v>
+        <v>2956</v>
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t>Microsoft Windows 8.1 Pro</t>
+          <t>Microsoft® Windows Vista™ Business</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
         <is>
-          <t>BRJ430FZQN</t>
+          <t>J5L1JJ1</t>
         </is>
       </c>
       <c r="I357" t="inlineStr">
         <is>
-          <t>Intel Core i5</t>
+          <t>Intel Core 2 Duo</t>
         </is>
       </c>
       <c r="J357" t="inlineStr">
         <is>
-          <t>4 GB</t>
+          <t>2 GB</t>
         </is>
       </c>
       <c r="K357" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Dell Inc.</t>
         </is>
       </c>
       <c r="L357" t="inlineStr">
         <is>
-          <t>HP 402 G1 SFF Business PC</t>
+          <t>OptiPlex 755</t>
         </is>
       </c>
       <c r="M357" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N357" s="3" t="n">
-        <v>46085.575</v>
+        <v>46086.37550925926</v>
       </c>
       <c r="O357" t="inlineStr">
         <is>
@@ -23290,7 +23328,7 @@
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>PA_254</t>
+          <t>PA_253</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
@@ -23300,33 +23338,33 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>10.69.5.254</t>
+          <t>10.69.5.253</t>
         </is>
       </c>
       <c r="D358" t="n">
-        <v>2016</v>
+        <v>2019</v>
       </c>
       <c r="E358" t="n">
-        <v>43374</v>
+        <v>73645</v>
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t>Microsoft Windows 7 Professional</t>
+          <t>Microsoft Windows 8.1 Pro</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
         <is>
-          <t>BRG103F9NQ</t>
+          <t>BRJ430FZQN</t>
         </is>
       </c>
       <c r="I358" t="inlineStr">
         <is>
-          <t>Intel Core 2 Duo</t>
+          <t>Intel Core i5</t>
         </is>
       </c>
       <c r="J358" t="inlineStr">
         <is>
-          <t>2 GB</t>
+          <t>4 GB</t>
         </is>
       </c>
       <c r="K358" t="inlineStr">
@@ -23336,14 +23374,14 @@
       </c>
       <c r="L358" t="inlineStr">
         <is>
-          <t>COMPAQ 300B MT</t>
+          <t>HP 402 G1 SFF Business PC</t>
         </is>
       </c>
       <c r="M358" t="n">
         <v>2</v>
       </c>
       <c r="N358" s="3" t="n">
-        <v>46085.61003472222</v>
+        <v>46086.37525462963</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -23354,7 +23392,7 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>PA_255</t>
+          <t>PA_254</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
@@ -23364,14 +23402,14 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>10.69.2.11</t>
+          <t>10.69.5.254</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>2012</v>
+        <v>2016</v>
       </c>
       <c r="E359" t="n">
-        <v>98086</v>
+        <v>43374</v>
       </c>
       <c r="F359" t="inlineStr">
         <is>
@@ -23380,17 +23418,17 @@
       </c>
       <c r="G359" t="inlineStr">
         <is>
-          <t>BRG232F74W</t>
+          <t>BRG103F9NQ</t>
         </is>
       </c>
       <c r="I359" t="inlineStr">
         <is>
-          <t>Intel Core i3</t>
+          <t>Intel Core 2 Duo</t>
         </is>
       </c>
       <c r="J359" t="inlineStr">
         <is>
-          <t>4 GB</t>
+          <t>2 GB</t>
         </is>
       </c>
       <c r="K359" t="inlineStr">
@@ -23400,14 +23438,14 @@
       </c>
       <c r="L359" t="inlineStr">
         <is>
-          <t>HP Pro 3410 Series</t>
+          <t>COMPAQ 300B MT</t>
         </is>
       </c>
       <c r="M359" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N359" s="3" t="n">
-        <v>46085.59136574074</v>
+        <v>46086.37553240741</v>
       </c>
       <c r="O359" t="inlineStr">
         <is>
@@ -23418,7 +23456,7 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>PA_256</t>
+          <t>PA_255</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
@@ -23428,47 +23466,50 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>10.69.5.9</t>
+          <t>10.69.2.11</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="E360" t="n">
-        <v>22943</v>
+        <v>98086</v>
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t>Microsoft® Windows Vista™ Business</t>
+          <t>Microsoft Windows 7 Professional</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
         <is>
-          <t>GCCKZL1</t>
+          <t>BRG232F74W</t>
         </is>
       </c>
       <c r="I360" t="inlineStr">
         <is>
-          <t>Intel Core 2 Duo</t>
+          <t>Intel Core i3</t>
         </is>
       </c>
       <c r="J360" t="inlineStr">
         <is>
-          <t>2 GB</t>
+          <t>4 GB</t>
         </is>
       </c>
       <c r="K360" t="inlineStr">
         <is>
-          <t>Dell Inc.</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="L360" t="inlineStr">
         <is>
-          <t>OptiPlex 360</t>
-        </is>
+          <t>HP Pro 3410 Series</t>
+        </is>
+      </c>
+      <c r="M360" t="n">
+        <v>1</v>
       </c>
       <c r="N360" s="3" t="n">
-        <v>46085.40222222222</v>
+        <v>46086.37474537037</v>
       </c>
       <c r="O360" t="inlineStr">
         <is>
@@ -23479,7 +23520,7 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>PA_257</t>
+          <t>PA_256</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
@@ -23489,14 +23530,14 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>10.69.5.218</t>
+          <t>10.69.5.9</t>
         </is>
       </c>
       <c r="D361" t="n">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="E361" t="n">
-        <v>2956</v>
+        <v>22943</v>
       </c>
       <c r="F361" t="inlineStr">
         <is>
@@ -23505,7 +23546,7 @@
       </c>
       <c r="G361" t="inlineStr">
         <is>
-          <t>G1XQXG1</t>
+          <t>GCCKZL1</t>
         </is>
       </c>
       <c r="I361" t="inlineStr">
@@ -23525,11 +23566,11 @@
       </c>
       <c r="L361" t="inlineStr">
         <is>
-          <t>OptiPlex 755</t>
+          <t>OptiPlex 360</t>
         </is>
       </c>
       <c r="N361" s="3" t="n">
-        <v>46049.60199074074</v>
+        <v>46085.40222222222</v>
       </c>
       <c r="O361" t="inlineStr">
         <is>
@@ -23540,7 +23581,7 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>PA_258</t>
+          <t>PA_257</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
@@ -23550,14 +23591,14 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>10.69.5.222</t>
+          <t>10.69.5.218</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="E362" t="n">
-        <v>3913</v>
+        <v>2956</v>
       </c>
       <c r="F362" t="inlineStr">
         <is>
@@ -23566,7 +23607,7 @@
       </c>
       <c r="G362" t="inlineStr">
         <is>
-          <t>4KPSZD1</t>
+          <t>G1XQXG1</t>
         </is>
       </c>
       <c r="I362" t="inlineStr">
@@ -23586,14 +23627,11 @@
       </c>
       <c r="L362" t="inlineStr">
         <is>
-          <t>OptiPlex 745</t>
-        </is>
-      </c>
-      <c r="M362" t="n">
-        <v>2</v>
+          <t>OptiPlex 755</t>
+        </is>
       </c>
       <c r="N362" s="3" t="n">
-        <v>46072.39605324074</v>
+        <v>46049.60199074074</v>
       </c>
       <c r="O362" t="inlineStr">
         <is>
@@ -23604,59 +23642,60 @@
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>RECEPCAO</t>
+          <t>PA_258</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>ADM/FIN</t>
+          <t>OPERACAO 9.1</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>10.69.3.9</t>
-        </is>
+          <t>10.69.5.222</t>
+        </is>
+      </c>
+      <c r="D363" t="n">
+        <v>2013</v>
+      </c>
+      <c r="E363" t="n">
+        <v>3913</v>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t>Microsoft Windows 11 Pro</t>
+          <t>Microsoft® Windows Vista™ Business</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
         <is>
-          <t>BRJ846Z6GZ</t>
-        </is>
-      </c>
-      <c r="H363" t="inlineStr">
-        <is>
-          <t>Microsoft Office Home and Business 2016 - pt-br</t>
+          <t>4KPSZD1</t>
         </is>
       </c>
       <c r="I363" t="inlineStr">
         <is>
-          <t>Intel Core i5</t>
+          <t>Intel Core 2 Duo</t>
         </is>
       </c>
       <c r="J363" t="inlineStr">
         <is>
-          <t>8 GB</t>
+          <t>2 GB</t>
         </is>
       </c>
       <c r="K363" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Dell Inc.</t>
         </is>
       </c>
       <c r="L363" t="inlineStr">
         <is>
-          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
+          <t>OptiPlex 745</t>
         </is>
       </c>
       <c r="M363" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N363" s="3" t="n">
-        <v>46085.6718287037</v>
+        <v>46072.39605324074</v>
       </c>
       <c r="O363" t="inlineStr">
         <is>
@@ -23667,24 +23706,18 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>RESERVA_GERENTE</t>
+          <t>RECEPCAO</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>RESERVA</t>
+          <t>ADM/FIN</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>10.69.2.13</t>
-        </is>
-      </c>
-      <c r="D364" t="n">
-        <v>2025</v>
-      </c>
-      <c r="E364" t="n">
-        <v>26919</v>
+          <t>10.69.3.9</t>
+        </is>
       </c>
       <c r="F364" t="inlineStr">
         <is>
@@ -23693,7 +23726,7 @@
       </c>
       <c r="G364" t="inlineStr">
         <is>
-          <t>928FPZ2</t>
+          <t>BRJ846Z6GZ</t>
         </is>
       </c>
       <c r="H364" t="inlineStr">
@@ -23713,16 +23746,19 @@
       </c>
       <c r="K364" t="inlineStr">
         <is>
-          <t>Dell Inc.</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="L364" t="inlineStr">
         <is>
-          <t>OptiPlex 3070</t>
-        </is>
+          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
+        </is>
+      </c>
+      <c r="M364" t="n">
+        <v>1</v>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46085.55094907407</v>
+        <v>46086.39894675926</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23733,67 +23769,73 @@
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>RH_NOTEBOOK</t>
+          <t>RESERVA_GERENTE</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>RH</t>
+          <t>RESERVA</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>10.69.2.12</t>
-        </is>
+          <t>10.69.2.13</t>
+        </is>
+      </c>
+      <c r="D365" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E365" t="n">
+        <v>26919</v>
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>Microsoft Windows 7 Professional</t>
+          <t>Microsoft Windows 11 Pro</t>
         </is>
       </c>
       <c r="G365" t="inlineStr">
         <is>
-          <t>BRG050GHBZ</t>
+          <t>928FPZ2</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>Microsoft Office Home and Business 2016 - pt-br</t>
         </is>
       </c>
       <c r="I365" t="inlineStr">
         <is>
-          <t>Intel Core 2 Duo</t>
+          <t>Intel Core i5</t>
         </is>
       </c>
       <c r="J365" t="inlineStr">
         <is>
-          <t>4 GB</t>
+          <t>8 GB</t>
         </is>
       </c>
       <c r="K365" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Dell Inc.</t>
         </is>
       </c>
       <c r="L365" t="inlineStr">
         <is>
-          <t>HP 420</t>
+          <t>OptiPlex 3070</t>
         </is>
       </c>
       <c r="N365" s="3" t="n">
-        <v>46002.58769675926</v>
+        <v>46085.55094907407</v>
       </c>
       <c r="O365" t="inlineStr">
         <is>
           <t>Ativo</t>
-        </is>
-      </c>
-      <c r="P365" t="inlineStr">
-        <is>
-          <t>RH.03</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>RH01</t>
+          <t>RH_NOTEBOOK</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
@@ -23803,38 +23845,27 @@
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>10.69.3.11</t>
-        </is>
-      </c>
-      <c r="D366" t="n">
-        <v>2025</v>
-      </c>
-      <c r="E366" t="n">
-        <v>28733</v>
+          <t>10.69.2.12</t>
+        </is>
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t>Microsoft Windows 11 Pro</t>
+          <t>Microsoft Windows 7 Professional</t>
         </is>
       </c>
       <c r="G366" t="inlineStr">
         <is>
-          <t>BRJ0057VPH</t>
-        </is>
-      </c>
-      <c r="H366" t="inlineStr">
-        <is>
-          <t>Microsoft Office Standard 2013</t>
+          <t>BRG050GHBZ</t>
         </is>
       </c>
       <c r="I366" t="inlineStr">
         <is>
-          <t>Intel Core i5</t>
+          <t>Intel Core 2 Duo</t>
         </is>
       </c>
       <c r="J366" t="inlineStr">
         <is>
-          <t>8 GB</t>
+          <t>4 GB</t>
         </is>
       </c>
       <c r="K366" t="inlineStr">
@@ -23844,22 +23875,27 @@
       </c>
       <c r="L366" t="inlineStr">
         <is>
-          <t>HP ProDesk 400 G5 SFF</t>
+          <t>HP 420</t>
         </is>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46085.70670138889</v>
+        <v>46002.58769675926</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
           <t>Ativo</t>
+        </is>
+      </c>
+      <c r="P366" t="inlineStr">
+        <is>
+          <t>RH.03</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>RH03</t>
+          <t>RH01</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
@@ -23869,7 +23905,7 @@
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>10.69.3.13</t>
+          <t>10.69.3.11</t>
         </is>
       </c>
       <c r="D367" t="n">
@@ -23885,12 +23921,12 @@
       </c>
       <c r="G367" t="inlineStr">
         <is>
-          <t>BRJ9364TK8</t>
+          <t>BRJ0057VPH</t>
         </is>
       </c>
       <c r="H367" t="inlineStr">
         <is>
-          <t>Microsoft Office Home and Business 2019 - pt-br</t>
+          <t>Microsoft Office Standard 2013</t>
         </is>
       </c>
       <c r="I367" t="inlineStr">
@@ -23914,7 +23950,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46086.29527777778</v>
+        <v>46086.37923611111</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -23925,17 +23961,12 @@
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>RH04</t>
+          <t>RH03</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
           <t>RH</t>
-        </is>
-      </c>
-      <c r="C368" t="inlineStr">
-        <is>
-          <t>10.69.3.14</t>
         </is>
       </c>
       <c r="D368" t="n">
@@ -23951,12 +23982,12 @@
       </c>
       <c r="G368" t="inlineStr">
         <is>
-          <t>BRJ0057VRJ</t>
+          <t>BRJ9364TK8</t>
         </is>
       </c>
       <c r="H368" t="inlineStr">
         <is>
-          <t>Microsoft Office Standard 2013</t>
+          <t>Microsoft Office Home and Business 2019 - pt-br</t>
         </is>
       </c>
       <c r="I368" t="inlineStr">
@@ -23979,11 +24010,8 @@
           <t>HP ProDesk 400 G5 SFF</t>
         </is>
       </c>
-      <c r="M368" t="n">
-        <v>1</v>
-      </c>
       <c r="N368" s="3" t="n">
-        <v>46086.30815972222</v>
+        <v>46086.3721875</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -23994,7 +24022,7 @@
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>RH05</t>
+          <t>RH04</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
@@ -24004,7 +24032,7 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>10.69.3.30</t>
+          <t>10.69.3.14</t>
         </is>
       </c>
       <c r="D369" t="n">
@@ -24020,7 +24048,7 @@
       </c>
       <c r="G369" t="inlineStr">
         <is>
-          <t>BRJ843Y4ML</t>
+          <t>BRJ0057VRJ</t>
         </is>
       </c>
       <c r="H369" t="inlineStr">
@@ -24045,14 +24073,14 @@
       </c>
       <c r="L369" t="inlineStr">
         <is>
-          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
+          <t>HP ProDesk 400 G5 SFF</t>
         </is>
       </c>
       <c r="M369" t="n">
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46085.6772337963</v>
+        <v>46086.38303240741</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24063,7 +24091,7 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>RH05NEW</t>
+          <t>RH05</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
@@ -24073,23 +24101,23 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>10.69.2.8</t>
+          <t>10.69.3.30</t>
         </is>
       </c>
       <c r="D370" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="E370" t="n">
-        <v>25</v>
+        <v>28733</v>
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t>Microsoft Windows 10 Pro</t>
+          <t>Microsoft Windows 11 Pro</t>
         </is>
       </c>
       <c r="G370" t="inlineStr">
         <is>
-          <t>BRJ748LCMY</t>
+          <t>BRJ843Y4ML</t>
         </is>
       </c>
       <c r="H370" t="inlineStr">
@@ -24104,7 +24132,7 @@
       </c>
       <c r="J370" t="inlineStr">
         <is>
-          <t>4 GB</t>
+          <t>8 GB</t>
         </is>
       </c>
       <c r="K370" t="inlineStr">
@@ -24114,14 +24142,14 @@
       </c>
       <c r="L370" t="inlineStr">
         <is>
-          <t>HP ProDesk 400 G4 SFF</t>
+          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
         </is>
       </c>
       <c r="M370" t="n">
         <v>1</v>
       </c>
       <c r="N370" s="3" t="n">
-        <v>46085.57601851852</v>
+        <v>46085.6772337963</v>
       </c>
       <c r="O370" t="inlineStr">
         <is>
@@ -24132,7 +24160,7 @@
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>RH06</t>
+          <t>RH05NEW</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
@@ -24142,28 +24170,28 @@
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>10.69.3.16</t>
+          <t>10.69.2.8</t>
         </is>
       </c>
       <c r="D371" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="E371" t="n">
-        <v>28733</v>
+        <v>25</v>
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t>Windows</t>
+          <t>Microsoft Windows 10 Pro</t>
         </is>
       </c>
       <c r="G371" t="inlineStr">
         <is>
-          <t>BRJ0057VPD</t>
+          <t>BRJ748LCMY</t>
         </is>
       </c>
       <c r="H371" t="inlineStr">
         <is>
-          <t>Microsoft Office Home and Business 2021 - pt-br</t>
+          <t>Microsoft Office Standard 2013</t>
         </is>
       </c>
       <c r="I371" t="inlineStr">
@@ -24173,7 +24201,7 @@
       </c>
       <c r="J371" t="inlineStr">
         <is>
-          <t>8 GB</t>
+          <t>4 GB</t>
         </is>
       </c>
       <c r="K371" t="inlineStr">
@@ -24183,14 +24211,14 @@
       </c>
       <c r="L371" t="inlineStr">
         <is>
-          <t>HP ProDesk 400 G5 SFF</t>
+          <t>HP ProDesk 400 G4 SFF</t>
         </is>
       </c>
       <c r="M371" t="n">
         <v>1</v>
       </c>
       <c r="N371" s="3" t="n">
-        <v>46076.49737268518</v>
+        <v>46085.57601851852</v>
       </c>
       <c r="O371" t="inlineStr">
         <is>
@@ -24201,17 +24229,17 @@
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>saladereuniao</t>
+          <t>RH06</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>ADM/FIN</t>
+          <t>RH</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>10.69.2.197</t>
+          <t>10.69.3.16</t>
         </is>
       </c>
       <c r="D372" t="n">
@@ -24222,12 +24250,12 @@
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t>Microsoft Windows 11 Pro</t>
+          <t>Windows</t>
         </is>
       </c>
       <c r="G372" t="inlineStr">
         <is>
-          <t>BRJ846Z5SX</t>
+          <t>BRJ0057VPD</t>
         </is>
       </c>
       <c r="H372" t="inlineStr">
@@ -24252,14 +24280,14 @@
       </c>
       <c r="L372" t="inlineStr">
         <is>
-          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
+          <t>HP ProDesk 400 G5 SFF</t>
         </is>
       </c>
       <c r="M372" t="n">
         <v>1</v>
       </c>
       <c r="N372" s="3" t="n">
-        <v>46085.61537037037</v>
+        <v>46076.49737268518</v>
       </c>
       <c r="O372" t="inlineStr">
         <is>
@@ -24270,24 +24298,24 @@
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>SANDRA</t>
+          <t>saladereuniao</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>DIRETORIA</t>
+          <t>ADM/FIN</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>10.69.3.100</t>
+          <t>10.69.2.197</t>
         </is>
       </c>
       <c r="D373" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="E373" t="n">
-        <v>70623</v>
+        <v>28733</v>
       </c>
       <c r="F373" t="inlineStr">
         <is>
@@ -24296,7 +24324,7 @@
       </c>
       <c r="G373" t="inlineStr">
         <is>
-          <t>BRJ208VH2D</t>
+          <t>BRJ846Z5SX</t>
         </is>
       </c>
       <c r="H373" t="inlineStr">
@@ -24311,7 +24339,7 @@
       </c>
       <c r="J373" t="inlineStr">
         <is>
-          <t>16 GB</t>
+          <t>8 GB</t>
         </is>
       </c>
       <c r="K373" t="inlineStr">
@@ -24321,14 +24349,14 @@
       </c>
       <c r="L373" t="inlineStr">
         <is>
-          <t>HP ProDesk 400 G6 Desktop Mini PC</t>
+          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
         </is>
       </c>
       <c r="M373" t="n">
         <v>1</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46085.73892361111</v>
+        <v>46085.61537037037</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24339,24 +24367,24 @@
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>SANTACASA_C01</t>
+          <t>SANDRA</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>COORDENACAO</t>
+          <t>DIRETORIA</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>10.69.3.71</t>
+          <t>10.69.3.100</t>
         </is>
       </c>
       <c r="D374" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="E374" t="n">
-        <v>26919</v>
+        <v>70623</v>
       </c>
       <c r="F374" t="inlineStr">
         <is>
@@ -24365,12 +24393,12 @@
       </c>
       <c r="G374" t="inlineStr">
         <is>
-          <t>92QLPZ2</t>
+          <t>BRJ208VH2D</t>
         </is>
       </c>
       <c r="H374" t="inlineStr">
         <is>
-          <t>Microsoft Office Home and Business 2016 - pt-br</t>
+          <t>Microsoft Office Home and Business 2021 - pt-br</t>
         </is>
       </c>
       <c r="I374" t="inlineStr">
@@ -24380,21 +24408,24 @@
       </c>
       <c r="J374" t="inlineStr">
         <is>
-          <t>8 GB</t>
+          <t>16 GB</t>
         </is>
       </c>
       <c r="K374" t="inlineStr">
         <is>
-          <t>Dell Inc.</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="L374" t="inlineStr">
         <is>
-          <t>OptiPlex 3070</t>
-        </is>
+          <t>HP ProDesk 400 G6 Desktop Mini PC</t>
+        </is>
+      </c>
+      <c r="M374" t="n">
+        <v>1</v>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46086.30686342593</v>
+        <v>46086.38814814815</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24405,19 +24436,24 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>SANTACASA_C02</t>
+          <t>SANTACASA_C01</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
           <t>COORDENACAO</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>10.69.3.71</t>
         </is>
       </c>
       <c r="D375" t="n">
         <v>2025</v>
       </c>
       <c r="E375" t="n">
-        <v>28733</v>
+        <v>26919</v>
       </c>
       <c r="F375" t="inlineStr">
         <is>
@@ -24426,12 +24462,12 @@
       </c>
       <c r="G375" t="inlineStr">
         <is>
-          <t>BRJ843Y6NF</t>
+          <t>92QLPZ2</t>
         </is>
       </c>
       <c r="H375" t="inlineStr">
         <is>
-          <t>Microsoft Office Standard 2013</t>
+          <t>Microsoft Office Home and Business 2016 - pt-br</t>
         </is>
       </c>
       <c r="I375" t="inlineStr">
@@ -24446,19 +24482,16 @@
       </c>
       <c r="K375" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Dell Inc.</t>
         </is>
       </c>
       <c r="L375" t="inlineStr">
         <is>
-          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
-        </is>
-      </c>
-      <c r="M375" t="n">
-        <v>1</v>
+          <t>OptiPlex 3070</t>
+        </is>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46085.81159722222</v>
+        <v>46086.38579861111</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24469,24 +24502,19 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>SANTACASA_C03</t>
+          <t>SANTACASA_C02</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
           <t>COORDENACAO</t>
-        </is>
-      </c>
-      <c r="C376" t="inlineStr">
-        <is>
-          <t>10.69.3.85</t>
         </is>
       </c>
       <c r="D376" t="n">
         <v>2025</v>
       </c>
       <c r="E376" t="n">
-        <v>26383</v>
+        <v>28733</v>
       </c>
       <c r="F376" t="inlineStr">
         <is>
@@ -24495,12 +24523,12 @@
       </c>
       <c r="G376" t="inlineStr">
         <is>
-          <t>PE08KTZD</t>
+          <t>BRJ843Y6NF</t>
         </is>
       </c>
       <c r="H376" t="inlineStr">
         <is>
-          <t>Microsoft Office Home and Business 2016 - pt-br</t>
+          <t>Microsoft Office Standard 2013</t>
         </is>
       </c>
       <c r="I376" t="inlineStr">
@@ -24515,19 +24543,19 @@
       </c>
       <c r="K376" t="inlineStr">
         <is>
-          <t>LENOVO</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="L376" t="inlineStr">
         <is>
-          <t>11EE0010BO</t>
+          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
         </is>
       </c>
       <c r="M376" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46085.78506944444</v>
+        <v>46085.81159722222</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -24538,38 +24566,38 @@
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>SIRLENE</t>
+          <t>SANTACASA_C03</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>GERENCIA</t>
+          <t>COORDENACAO</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>10.69.3.60</t>
+          <t>10.69.3.85</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="E377" t="n">
-        <v>184</v>
+        <v>26383</v>
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t>Microsoft Windows 10 Pro</t>
+          <t>Microsoft Windows 11 Pro</t>
         </is>
       </c>
       <c r="G377" t="inlineStr">
         <is>
-          <t>CKL22H2</t>
+          <t>PE08KTZD</t>
         </is>
       </c>
       <c r="H377" t="inlineStr">
         <is>
-          <t>Microsoft Office Home and Business 2021 - pt-br</t>
+          <t>Microsoft Office Home and Business 2016 - pt-br</t>
         </is>
       </c>
       <c r="I377" t="inlineStr">
@@ -24584,21 +24612,90 @@
       </c>
       <c r="K377" t="inlineStr">
         <is>
-          <t>Dell Inc.</t>
+          <t>LENOVO</t>
         </is>
       </c>
       <c r="L377" t="inlineStr">
         <is>
-          <t>OptiPlex 3040</t>
+          <t>11EE0010BO</t>
         </is>
       </c>
       <c r="M377" t="n">
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46086.30560185185</v>
+        <v>46086.374375</v>
       </c>
       <c r="O377" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>SIRLENE</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>GERENCIA</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>10.69.3.60</t>
+        </is>
+      </c>
+      <c r="D378" t="n">
+        <v>2024</v>
+      </c>
+      <c r="E378" t="n">
+        <v>184</v>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>Microsoft Windows 10 Pro</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>CKL22H2</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>Microsoft Office Home and Business 2021 - pt-br</t>
+        </is>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>Intel Core i5</t>
+        </is>
+      </c>
+      <c r="J378" t="inlineStr">
+        <is>
+          <t>8 GB</t>
+        </is>
+      </c>
+      <c r="K378" t="inlineStr">
+        <is>
+          <t>Dell Inc.</t>
+        </is>
+      </c>
+      <c r="L378" t="inlineStr">
+        <is>
+          <t>OptiPlex 3040</t>
+        </is>
+      </c>
+      <c r="M378" t="n">
+        <v>2</v>
+      </c>
+      <c r="N378" s="3" t="n">
+        <v>46086.37909722222</v>
+      </c>
+      <c r="O378" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-05 11:52:05.849179
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q378"/>
+  <dimension ref="A1:Q377"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25.2" customWidth="1" min="1" max="1"/>
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46086.39331018519</v>
+        <v>46086.46652777777</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46086.39651620371</v>
+        <v>46086.47596064815</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46086.39417824074</v>
+        <v>46086.47538194444</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46086.37658564815</v>
+        <v>46086.45210648148</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46086.37372685185</v>
+        <v>46086.48438657408</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46086.38474537037</v>
+        <v>46086.46130787037</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46086.40094907407</v>
+        <v>46086.47638888889</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46086.3782175926</v>
+        <v>46086.45846064815</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1702,7 +1702,7 @@
         <v>1</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>46086.38354166667</v>
+        <v>46086.46201388889</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1766,7 +1766,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46085.73266203704</v>
+        <v>46086.46438657407</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1844,11 +1844,6 @@
           <t>AUDITORIO</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>10.69.3.146</t>
-        </is>
-      </c>
       <c r="D22" t="n">
         <v>2018</v>
       </c>
@@ -2082,6 +2077,11 @@
           <t>AUDITORIO</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>10.69.3.151</t>
+        </is>
+      </c>
       <c r="D26" t="n">
         <v>2019</v>
       </c>
@@ -2122,7 +2122,7 @@
         <v>1</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>46086.18706018518</v>
+        <v>46086.46799768518</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46085.73777777778</v>
+        <v>46086.45563657407</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6509,7 +6509,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46086.40284722222</v>
+        <v>46086.48377314815</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6578,7 +6578,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46085.82043981482</v>
+        <v>46086.47763888889</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6642,7 +6642,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46085.7075462963</v>
+        <v>46086.46075231482</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6706,7 +6706,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46086.38972222222</v>
+        <v>46086.46108796296</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6775,7 +6775,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46086.38306712963</v>
+        <v>46086.4597337963</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6844,7 +6844,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46086.40141203703</v>
+        <v>46086.47921296296</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6913,7 +6913,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46086.37782407407</v>
+        <v>46086.44953703704</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -7308,7 +7308,7 @@
         <v>1</v>
       </c>
       <c r="N106" s="3" t="n">
-        <v>46086.36996527778</v>
+        <v>46086.48730324074</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -7446,7 +7446,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46086.37863425926</v>
+        <v>46086.45457175926</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7515,7 +7515,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46086.39784722222</v>
+        <v>46086.47501157408</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7584,7 +7584,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46086.36831018519</v>
+        <v>46086.48096064815</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7653,7 +7653,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46086.38293981482</v>
+        <v>46086.45567129629</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7722,7 +7722,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46086.40136574074</v>
+        <v>46086.48214120371</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7791,7 +7791,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46086.39009259259</v>
+        <v>46086.46743055555</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7857,7 +7857,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46086.38819444444</v>
+        <v>46086.46832175926</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7926,7 +7926,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46086.39872685185</v>
+        <v>46086.48017361111</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7995,7 +7995,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46086.40329861111</v>
+        <v>46086.48278935185</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8061,7 +8061,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46086.37034722222</v>
+        <v>46086.451875</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8199,7 +8199,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46086.38538194444</v>
+        <v>46086.46931712963</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8334,7 +8334,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46086.37353009259</v>
+        <v>46086.44712962963</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8472,7 +8472,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46086.38405092592</v>
+        <v>46086.46287037037</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8541,7 +8541,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46086.38666666667</v>
+        <v>46086.46935185185</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8610,7 +8610,7 @@
         <v>2</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46085.65229166667</v>
+        <v>46086.4665625</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8748,7 +8748,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46086.39893518519</v>
+        <v>46086.47401620371</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8817,7 +8817,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46086.37872685185</v>
+        <v>46086.4516087963</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8886,7 +8886,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46086.37692129629</v>
+        <v>46086.45138888889</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -8955,7 +8955,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46086.39230324074</v>
+        <v>46086.46967592592</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9088,7 +9088,7 @@
         <v>1</v>
       </c>
       <c r="N132" s="3" t="n">
-        <v>46086.37386574074</v>
+        <v>46086.48734953703</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -9407,7 +9407,7 @@
         <v>1</v>
       </c>
       <c r="N137" s="3" t="n">
-        <v>46086.38385416667</v>
+        <v>46086.46420138889</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -9599,7 +9599,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46086.3634837963</v>
+        <v>46086.48736111111</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9663,7 +9663,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46086.39488425926</v>
+        <v>46086.48607638889</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9727,7 +9727,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46086.40315972222</v>
+        <v>46086.48116898148</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9791,7 +9791,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46086.4037962963</v>
+        <v>46086.4822337963</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9855,7 +9855,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46086.39163194445</v>
+        <v>46086.4693287037</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9919,7 +9919,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46086.36521990741</v>
+        <v>46086.48672453704</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9983,7 +9983,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46086.40070601852</v>
+        <v>46086.48060185185</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10047,7 +10047,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46086.38041666667</v>
+        <v>46086.46024305555</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10111,7 +10111,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46086.38905092593</v>
+        <v>46086.46627314815</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10175,7 +10175,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46086.38391203704</v>
+        <v>46086.46534722222</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10239,7 +10239,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46086.38950231481</v>
+        <v>46086.47047453704</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10303,7 +10303,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46086.38180555555</v>
+        <v>46086.45927083334</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10426,7 +10426,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46086.36651620371</v>
+        <v>46086.48105324074</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10490,7 +10490,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46086.37810185185</v>
+        <v>46086.45704861111</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10554,7 +10554,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46086.38533564815</v>
+        <v>46086.485625</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10618,7 +10618,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46086.36865740741</v>
+        <v>46086.4531712963</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10746,7 +10746,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46086.38480324074</v>
+        <v>46086.46329861111</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10810,7 +10810,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46086.38445601852</v>
+        <v>46086.45902777778</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10874,7 +10874,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46086.37545138889</v>
+        <v>46086.45204861111</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10938,7 +10938,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46086.37180555556</v>
+        <v>46086.44923611111</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -11066,7 +11066,7 @@
         <v>2</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46086.40212962963</v>
+        <v>46086.48075231481</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11130,7 +11130,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46086.3675</v>
+        <v>46086.4852662037</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11194,7 +11194,7 @@
         <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46086.38680555556</v>
+        <v>46086.45913194444</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11258,7 +11258,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46086.36831018519</v>
+        <v>46086.44865740741</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11322,7 +11322,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46086.39112268519</v>
+        <v>46086.47234953703</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11386,7 +11386,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46086.36736111111</v>
+        <v>46086.48077546297</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11450,7 +11450,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46086.36918981482</v>
+        <v>46086.4852662037</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11514,7 +11514,7 @@
         <v>2</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46086.36613425926</v>
+        <v>46086.47979166666</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11642,7 +11642,7 @@
         <v>1</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46086.3653587963</v>
+        <v>46086.44788194444</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11706,7 +11706,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46086.39128472222</v>
+        <v>46086.48649305556</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11770,7 +11770,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46086.38056712963</v>
+        <v>46086.46126157408</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11834,7 +11834,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46085.65648148148</v>
+        <v>46086.45366898148</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11962,7 +11962,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46086.39571759259</v>
+        <v>46086.47534722222</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12026,7 +12026,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46086.37681712963</v>
+        <v>46086.45335648148</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12415,7 +12415,7 @@
         <v>1</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46084.85907407408</v>
+        <v>46086.48731481482</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12479,7 +12479,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46085.80268518518</v>
+        <v>46086.48545138889</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12543,7 +12543,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46086.40305555556</v>
+        <v>46086.48327546296</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12607,7 +12607,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46086.39873842592</v>
+        <v>46086.48667824074</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12735,7 +12735,7 @@
         </is>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46086.37740740741</v>
+        <v>46086.45497685186</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12799,7 +12799,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46086.39013888889</v>
+        <v>46086.4852662037</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12863,7 +12863,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46086.40193287037</v>
+        <v>46086.47489583334</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12988,7 +12988,7 @@
         <v>2</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46086.38114583334</v>
+        <v>46086.45892361111</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13052,7 +13052,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46086.39678240741</v>
+        <v>46086.4775</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13116,7 +13116,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46086.36760416667</v>
+        <v>46086.48744212963</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13180,7 +13180,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46085.84046296297</v>
+        <v>46086.47625</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13244,7 +13244,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46086.38783564815</v>
+        <v>46086.46800925926</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13308,7 +13308,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46086.39252314815</v>
+        <v>46086.48143518518</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13372,7 +13372,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46086.36905092592</v>
+        <v>46086.48605324074</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13433,7 +13433,7 @@
         </is>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46085.82528935185</v>
+        <v>46086.461875</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13497,7 +13497,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46086.37502314815</v>
+        <v>46086.48416666667</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13561,7 +13561,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46086.37431712963</v>
+        <v>46086.48521990741</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13625,7 +13625,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46086.40159722222</v>
+        <v>46086.4809375</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13689,7 +13689,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46086.36267361111</v>
+        <v>46086.48296296296</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13753,7 +13753,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46086.3653587963</v>
+        <v>46086.4811574074</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13817,7 +13817,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46086.40056712963</v>
+        <v>46086.48592592592</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13881,7 +13881,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46086.3778587963</v>
+        <v>46086.48792824074</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13945,7 +13945,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46086.37548611111</v>
+        <v>46086.48673611111</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14009,7 +14009,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46086.37436342592</v>
+        <v>46086.48354166667</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14073,7 +14073,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46086.37579861111</v>
+        <v>46086.45252314815</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14137,7 +14137,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46086.37462962963</v>
+        <v>46086.45130787037</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14201,7 +14201,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46086.38460648148</v>
+        <v>46086.46039351852</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14265,7 +14265,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46086.37756944444</v>
+        <v>46086.45643518519</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14393,7 +14393,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46086.37563657408</v>
+        <v>46086.45061342593</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14457,7 +14457,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46086.37804398148</v>
+        <v>46086.45341435185</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14521,7 +14521,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46086.37637731482</v>
+        <v>46086.45321759259</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14585,7 +14585,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46086.36542824074</v>
+        <v>46086.47951388889</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14654,7 +14654,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46086.37532407408</v>
+        <v>46086.4562037037</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14718,7 +14718,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46086.38393518519</v>
+        <v>46086.46083333333</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14782,7 +14782,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46086.3816087963</v>
+        <v>46086.45542824074</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14974,7 +14974,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46086.40224537037</v>
+        <v>46086.48032407407</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15102,7 +15102,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46086.37131944444</v>
+        <v>46086.45277777778</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15166,7 +15166,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46086.37519675926</v>
+        <v>46086.45018518518</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15230,7 +15230,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46086.39850694445</v>
+        <v>46086.48097222222</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15294,7 +15294,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46086.39563657407</v>
+        <v>46086.48631944445</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15358,7 +15358,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46086.36827546296</v>
+        <v>46086.48681712963</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15422,7 +15422,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46086.3869212963</v>
+        <v>46086.4800925926</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15486,7 +15486,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46086.37006944444</v>
+        <v>46086.48592592592</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15550,7 +15550,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46086.40354166667</v>
+        <v>46086.4724537037</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15614,7 +15614,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46086.37576388889</v>
+        <v>46086.45128472222</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15678,7 +15678,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46086.38116898148</v>
+        <v>46086.46178240741</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15806,7 +15806,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46086.37673611111</v>
+        <v>46086.45151620371</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15870,7 +15870,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46086.37275462963</v>
+        <v>46086.45078703704</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15934,7 +15934,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46086.37424768518</v>
+        <v>46086.4868287037</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -16062,7 +16062,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46086.36282407407</v>
+        <v>46086.48515046296</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16126,7 +16126,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46086.3744212963</v>
+        <v>46086.45065972222</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16313,7 +16313,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46086.3753125</v>
+        <v>46086.45243055555</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16377,7 +16377,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46086.36740740741</v>
+        <v>46086.48556712963</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16441,7 +16441,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46086.38730324074</v>
+        <v>46086.46643518518</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16505,7 +16505,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46086.38521990741</v>
+        <v>46086.46540509259</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16524,11 +16524,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C249" t="inlineStr">
-        <is>
-          <t>10.69.5.118</t>
-        </is>
-      </c>
       <c r="D249" t="n">
         <v>2017</v>
       </c>
@@ -16569,7 +16564,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46086.3849537037</v>
+        <v>46086.45695601852</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16633,7 +16628,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46086.38659722222</v>
+        <v>46086.47061342592</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16697,7 +16692,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46086.38626157407</v>
+        <v>46086.48546296296</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16761,7 +16756,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46086.40398148148</v>
+        <v>46086.48490740741</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16819,7 +16814,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46086.40047453704</v>
+        <v>46086.47336805556</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16883,7 +16878,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46086.38297453704</v>
+        <v>46086.46005787037</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16947,7 +16942,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46086.36715277778</v>
+        <v>46086.48478009259</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -17011,7 +17006,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46086.3671875</v>
+        <v>46086.48712962963</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17075,7 +17070,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46086.40369212963</v>
+        <v>46086.48418981482</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17203,7 +17198,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46086.39956018519</v>
+        <v>46086.47641203704</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17331,7 +17326,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46086.38427083333</v>
+        <v>46086.46162037037</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17395,7 +17390,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46086.39978009259</v>
+        <v>46086.47432870371</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17459,7 +17454,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46086.37892361111</v>
+        <v>46086.48039351852</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17523,7 +17518,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46086.36898148148</v>
+        <v>46086.48795138889</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17587,7 +17582,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46086.37188657407</v>
+        <v>46086.48091435185</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17651,7 +17646,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46086.36939814815</v>
+        <v>46086.48263888889</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17779,7 +17774,7 @@
         <v>1</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46085.793125</v>
+        <v>46086.48427083333</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17840,7 +17835,7 @@
         </is>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46086.39587962963</v>
+        <v>46086.47372685185</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17968,7 +17963,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46086.39542824074</v>
+        <v>46086.47012731482</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -18093,7 +18088,7 @@
         </is>
       </c>
       <c r="N273" s="3" t="n">
-        <v>46086.38736111111</v>
+        <v>46086.46725694444</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -18341,7 +18336,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46086.40219907407</v>
+        <v>46086.47909722223</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18405,7 +18400,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46086.39631944444</v>
+        <v>46086.47094907407</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18528,7 +18523,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46086.37677083333</v>
+        <v>46086.45322916667</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18587,7 +18582,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46086.37296296296</v>
+        <v>46086.45104166667</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18651,7 +18646,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46086.39950231482</v>
+        <v>46086.47237268519</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18715,7 +18710,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46086.37445601852</v>
+        <v>46086.45143518518</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18779,7 +18774,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46086.36570601852</v>
+        <v>46086.48563657407</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18838,7 +18833,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46086.37398148148</v>
+        <v>46086.45297453704</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18902,7 +18897,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46086.37695601852</v>
+        <v>46086.45162037037</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18966,7 +18961,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46086.39809027778</v>
+        <v>46086.48631944445</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19030,7 +19025,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46085.85211805555</v>
+        <v>46086.46020833333</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19824,7 +19819,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46086.389375</v>
+        <v>46086.46232638889</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20940,7 +20935,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46086.39420138889</v>
+        <v>46086.4737962963</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21665,7 +21660,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46086.40112268519</v>
+        <v>46086.48090277778</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21729,7 +21724,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46086.39383101852</v>
+        <v>46086.47077546296</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21793,7 +21788,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46086.39548611111</v>
+        <v>46086.47649305555</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21857,7 +21852,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46086.39841435185</v>
+        <v>46086.47467592593</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21921,7 +21916,7 @@
         <v>2</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46086.37752314815</v>
+        <v>46086.4572800926</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21985,7 +21980,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46086.40157407407</v>
+        <v>46086.4875</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22049,7 +22044,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46086.40071759259</v>
+        <v>46086.476875</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22113,7 +22108,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46086.39075231482</v>
+        <v>46086.46547453704</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22305,7 +22300,7 @@
         <v>2</v>
       </c>
       <c r="N341" s="3" t="n">
-        <v>46085.57246527778</v>
+        <v>46086.47333333334</v>
       </c>
       <c r="O341" t="inlineStr">
         <is>
@@ -22324,6 +22319,11 @@
           <t>OPERACAO 9.1</t>
         </is>
       </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>10.69.5.237</t>
+        </is>
+      </c>
       <c r="D342" t="n">
         <v>2017</v>
       </c>
@@ -22366,7 +22366,7 @@
         </is>
       </c>
       <c r="N342" s="3" t="n">
-        <v>46085.59991898148</v>
+        <v>46086.47072916666</v>
       </c>
       <c r="O342" t="inlineStr">
         <is>
@@ -22622,7 +22622,7 @@
         <v>1</v>
       </c>
       <c r="N346" s="3" t="n">
-        <v>46086.37422453704</v>
+        <v>46086.46128472222</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -22686,7 +22686,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46086.37491898148</v>
+        <v>46086.45493055556</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22750,7 +22750,7 @@
         <v>1</v>
       </c>
       <c r="N348" s="3" t="n">
-        <v>46086.37497685185</v>
+        <v>46086.45190972222</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -22811,7 +22811,7 @@
         </is>
       </c>
       <c r="N349" s="3" t="n">
-        <v>46086.37460648148</v>
+        <v>46086.41283564815</v>
       </c>
       <c r="O349" t="inlineStr">
         <is>
@@ -22875,7 +22875,7 @@
         <v>1</v>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46086.37583333333</v>
+        <v>46086.45523148148</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -22939,7 +22939,7 @@
         <v>1</v>
       </c>
       <c r="N351" s="3" t="n">
-        <v>46086.37633101852</v>
+        <v>46086.45574074074</v>
       </c>
       <c r="O351" t="inlineStr">
         <is>
@@ -23125,7 +23125,7 @@
         <v>1</v>
       </c>
       <c r="N354" s="3" t="n">
-        <v>46086.37416666667</v>
+        <v>46086.45224537037</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -23189,7 +23189,7 @@
         <v>1</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46086.37462962963</v>
+        <v>46086.48635416666</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23253,7 +23253,7 @@
         <v>1</v>
       </c>
       <c r="N356" s="3" t="n">
-        <v>46086.37435185185</v>
+        <v>46086.45384259259</v>
       </c>
       <c r="O356" t="inlineStr">
         <is>
@@ -23381,7 +23381,7 @@
         <v>2</v>
       </c>
       <c r="N358" s="3" t="n">
-        <v>46086.37525462963</v>
+        <v>46086.45366898148</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -23509,7 +23509,7 @@
         <v>1</v>
       </c>
       <c r="N360" s="3" t="n">
-        <v>46086.37474537037</v>
+        <v>46086.45371527778</v>
       </c>
       <c r="O360" t="inlineStr">
         <is>
@@ -23758,7 +23758,7 @@
         <v>1</v>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46086.39894675926</v>
+        <v>46086.47571759259</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23824,7 +23824,7 @@
         </is>
       </c>
       <c r="N365" s="3" t="n">
-        <v>46085.55094907407</v>
+        <v>46086.46056712963</v>
       </c>
       <c r="O365" t="inlineStr">
         <is>
@@ -23950,7 +23950,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46086.37923611111</v>
+        <v>46086.45829861111</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -24011,7 +24011,7 @@
         </is>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46086.3721875</v>
+        <v>46086.45425925926</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24080,7 +24080,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46086.38303240741</v>
+        <v>46086.45896990741</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24099,27 +24099,6 @@
           <t>RH</t>
         </is>
       </c>
-      <c r="C370" t="inlineStr">
-        <is>
-          <t>10.69.3.30</t>
-        </is>
-      </c>
-      <c r="D370" t="n">
-        <v>2025</v>
-      </c>
-      <c r="E370" t="n">
-        <v>28733</v>
-      </c>
-      <c r="F370" t="inlineStr">
-        <is>
-          <t>Microsoft Windows 11 Pro</t>
-        </is>
-      </c>
-      <c r="G370" t="inlineStr">
-        <is>
-          <t>BRJ843Y4ML</t>
-        </is>
-      </c>
       <c r="H370" t="inlineStr">
         <is>
           <t>Microsoft Office Standard 2013</t>
@@ -24130,26 +24109,11 @@
           <t>Intel Core i5</t>
         </is>
       </c>
-      <c r="J370" t="inlineStr">
-        <is>
-          <t>8 GB</t>
-        </is>
-      </c>
-      <c r="K370" t="inlineStr">
-        <is>
-          <t>HP</t>
-        </is>
-      </c>
-      <c r="L370" t="inlineStr">
-        <is>
-          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
-        </is>
-      </c>
       <c r="M370" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N370" s="3" t="n">
-        <v>46085.6772337963</v>
+        <v>46086.45856481481</v>
       </c>
       <c r="O370" t="inlineStr">
         <is>
@@ -24160,7 +24124,7 @@
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>RH05NEW</t>
+          <t>RH06</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
@@ -24170,28 +24134,28 @@
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>10.69.2.8</t>
+          <t>10.69.3.16</t>
         </is>
       </c>
       <c r="D371" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="E371" t="n">
-        <v>25</v>
+        <v>28733</v>
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t>Microsoft Windows 10 Pro</t>
+          <t>Windows</t>
         </is>
       </c>
       <c r="G371" t="inlineStr">
         <is>
-          <t>BRJ748LCMY</t>
+          <t>BRJ0057VPD</t>
         </is>
       </c>
       <c r="H371" t="inlineStr">
         <is>
-          <t>Microsoft Office Standard 2013</t>
+          <t>Microsoft Office Home and Business 2021 - pt-br</t>
         </is>
       </c>
       <c r="I371" t="inlineStr">
@@ -24201,7 +24165,7 @@
       </c>
       <c r="J371" t="inlineStr">
         <is>
-          <t>4 GB</t>
+          <t>8 GB</t>
         </is>
       </c>
       <c r="K371" t="inlineStr">
@@ -24211,14 +24175,14 @@
       </c>
       <c r="L371" t="inlineStr">
         <is>
-          <t>HP ProDesk 400 G4 SFF</t>
+          <t>HP ProDesk 400 G5 SFF</t>
         </is>
       </c>
       <c r="M371" t="n">
         <v>1</v>
       </c>
       <c r="N371" s="3" t="n">
-        <v>46085.57601851852</v>
+        <v>46076.49737268518</v>
       </c>
       <c r="O371" t="inlineStr">
         <is>
@@ -24229,17 +24193,17 @@
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>RH06</t>
+          <t>saladereuniao</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>RH</t>
+          <t>ADM/FIN</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>10.69.3.16</t>
+          <t>10.69.2.197</t>
         </is>
       </c>
       <c r="D372" t="n">
@@ -24250,12 +24214,12 @@
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t>Windows</t>
+          <t>Microsoft Windows 11 Pro</t>
         </is>
       </c>
       <c r="G372" t="inlineStr">
         <is>
-          <t>BRJ0057VPD</t>
+          <t>BRJ846Z5SX</t>
         </is>
       </c>
       <c r="H372" t="inlineStr">
@@ -24280,14 +24244,14 @@
       </c>
       <c r="L372" t="inlineStr">
         <is>
-          <t>HP ProDesk 400 G5 SFF</t>
+          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
         </is>
       </c>
       <c r="M372" t="n">
         <v>1</v>
       </c>
       <c r="N372" s="3" t="n">
-        <v>46076.49737268518</v>
+        <v>46085.61537037037</v>
       </c>
       <c r="O372" t="inlineStr">
         <is>
@@ -24298,24 +24262,24 @@
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>saladereuniao</t>
+          <t>SANDRA</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>ADM/FIN</t>
+          <t>DIRETORIA</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>10.69.2.197</t>
+          <t>10.69.3.100</t>
         </is>
       </c>
       <c r="D373" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="E373" t="n">
-        <v>28733</v>
+        <v>70623</v>
       </c>
       <c r="F373" t="inlineStr">
         <is>
@@ -24324,7 +24288,7 @@
       </c>
       <c r="G373" t="inlineStr">
         <is>
-          <t>BRJ846Z5SX</t>
+          <t>BRJ208VH2D</t>
         </is>
       </c>
       <c r="H373" t="inlineStr">
@@ -24339,7 +24303,7 @@
       </c>
       <c r="J373" t="inlineStr">
         <is>
-          <t>8 GB</t>
+          <t>16 GB</t>
         </is>
       </c>
       <c r="K373" t="inlineStr">
@@ -24349,14 +24313,14 @@
       </c>
       <c r="L373" t="inlineStr">
         <is>
-          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
+          <t>HP ProDesk 400 G6 Desktop Mini PC</t>
         </is>
       </c>
       <c r="M373" t="n">
         <v>1</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46085.61537037037</v>
+        <v>46086.4647337963</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24367,24 +24331,24 @@
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>SANDRA</t>
+          <t>SANTACASA_C01</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>DIRETORIA</t>
+          <t>COORDENACAO</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>10.69.3.100</t>
+          <t>10.69.3.71</t>
         </is>
       </c>
       <c r="D374" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="E374" t="n">
-        <v>70623</v>
+        <v>26919</v>
       </c>
       <c r="F374" t="inlineStr">
         <is>
@@ -24393,12 +24357,12 @@
       </c>
       <c r="G374" t="inlineStr">
         <is>
-          <t>BRJ208VH2D</t>
+          <t>92QLPZ2</t>
         </is>
       </c>
       <c r="H374" t="inlineStr">
         <is>
-          <t>Microsoft Office Home and Business 2021 - pt-br</t>
+          <t>Microsoft Office Home and Business 2016 - pt-br</t>
         </is>
       </c>
       <c r="I374" t="inlineStr">
@@ -24408,24 +24372,21 @@
       </c>
       <c r="J374" t="inlineStr">
         <is>
-          <t>16 GB</t>
+          <t>8 GB</t>
         </is>
       </c>
       <c r="K374" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Dell Inc.</t>
         </is>
       </c>
       <c r="L374" t="inlineStr">
         <is>
-          <t>HP ProDesk 400 G6 Desktop Mini PC</t>
-        </is>
-      </c>
-      <c r="M374" t="n">
-        <v>1</v>
+          <t>OptiPlex 3070</t>
+        </is>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46086.38814814815</v>
+        <v>46086.45899305555</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24436,24 +24397,19 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>SANTACASA_C01</t>
+          <t>SANTACASA_C02</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
           <t>COORDENACAO</t>
-        </is>
-      </c>
-      <c r="C375" t="inlineStr">
-        <is>
-          <t>10.69.3.71</t>
         </is>
       </c>
       <c r="D375" t="n">
         <v>2025</v>
       </c>
       <c r="E375" t="n">
-        <v>26919</v>
+        <v>28733</v>
       </c>
       <c r="F375" t="inlineStr">
         <is>
@@ -24462,12 +24418,12 @@
       </c>
       <c r="G375" t="inlineStr">
         <is>
-          <t>92QLPZ2</t>
+          <t>BRJ843Y6NF</t>
         </is>
       </c>
       <c r="H375" t="inlineStr">
         <is>
-          <t>Microsoft Office Home and Business 2016 - pt-br</t>
+          <t>Microsoft Office Standard 2013</t>
         </is>
       </c>
       <c r="I375" t="inlineStr">
@@ -24482,16 +24438,19 @@
       </c>
       <c r="K375" t="inlineStr">
         <is>
-          <t>Dell Inc.</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="L375" t="inlineStr">
         <is>
-          <t>OptiPlex 3070</t>
-        </is>
+          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
+        </is>
+      </c>
+      <c r="M375" t="n">
+        <v>1</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46086.38579861111</v>
+        <v>46086.46025462963</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24502,19 +24461,24 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>SANTACASA_C02</t>
+          <t>SANTACASA_C03</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
           <t>COORDENACAO</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>10.69.3.85</t>
         </is>
       </c>
       <c r="D376" t="n">
         <v>2025</v>
       </c>
       <c r="E376" t="n">
-        <v>28733</v>
+        <v>26383</v>
       </c>
       <c r="F376" t="inlineStr">
         <is>
@@ -24523,12 +24487,12 @@
       </c>
       <c r="G376" t="inlineStr">
         <is>
-          <t>BRJ843Y6NF</t>
+          <t>PE08KTZD</t>
         </is>
       </c>
       <c r="H376" t="inlineStr">
         <is>
-          <t>Microsoft Office Standard 2013</t>
+          <t>Microsoft Office Home and Business 2016 - pt-br</t>
         </is>
       </c>
       <c r="I376" t="inlineStr">
@@ -24543,19 +24507,19 @@
       </c>
       <c r="K376" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>LENOVO</t>
         </is>
       </c>
       <c r="L376" t="inlineStr">
         <is>
-          <t>HP ProDesk 400 G5 SFF (Brazil)</t>
+          <t>11EE0010BO</t>
         </is>
       </c>
       <c r="M376" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46085.81159722222</v>
+        <v>46086.45298611111</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -24566,38 +24530,38 @@
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>SANTACASA_C03</t>
+          <t>SIRLENE</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>COORDENACAO</t>
+          <t>GERENCIA</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>10.69.3.85</t>
+          <t>10.69.3.60</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="E377" t="n">
-        <v>26383</v>
+        <v>184</v>
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t>Microsoft Windows 11 Pro</t>
+          <t>Microsoft Windows 10 Pro</t>
         </is>
       </c>
       <c r="G377" t="inlineStr">
         <is>
-          <t>PE08KTZD</t>
+          <t>CKL22H2</t>
         </is>
       </c>
       <c r="H377" t="inlineStr">
         <is>
-          <t>Microsoft Office Home and Business 2016 - pt-br</t>
+          <t>Microsoft Office Home and Business 2021 - pt-br</t>
         </is>
       </c>
       <c r="I377" t="inlineStr">
@@ -24612,90 +24576,21 @@
       </c>
       <c r="K377" t="inlineStr">
         <is>
-          <t>LENOVO</t>
+          <t>Dell Inc.</t>
         </is>
       </c>
       <c r="L377" t="inlineStr">
         <is>
-          <t>11EE0010BO</t>
+          <t>OptiPlex 3040</t>
         </is>
       </c>
       <c r="M377" t="n">
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46086.374375</v>
+        <v>46086.45694444444</v>
       </c>
       <c r="O377" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-    </row>
-    <row r="378">
-      <c r="A378" t="inlineStr">
-        <is>
-          <t>SIRLENE</t>
-        </is>
-      </c>
-      <c r="B378" t="inlineStr">
-        <is>
-          <t>GERENCIA</t>
-        </is>
-      </c>
-      <c r="C378" t="inlineStr">
-        <is>
-          <t>10.69.3.60</t>
-        </is>
-      </c>
-      <c r="D378" t="n">
-        <v>2024</v>
-      </c>
-      <c r="E378" t="n">
-        <v>184</v>
-      </c>
-      <c r="F378" t="inlineStr">
-        <is>
-          <t>Microsoft Windows 10 Pro</t>
-        </is>
-      </c>
-      <c r="G378" t="inlineStr">
-        <is>
-          <t>CKL22H2</t>
-        </is>
-      </c>
-      <c r="H378" t="inlineStr">
-        <is>
-          <t>Microsoft Office Home and Business 2021 - pt-br</t>
-        </is>
-      </c>
-      <c r="I378" t="inlineStr">
-        <is>
-          <t>Intel Core i5</t>
-        </is>
-      </c>
-      <c r="J378" t="inlineStr">
-        <is>
-          <t>8 GB</t>
-        </is>
-      </c>
-      <c r="K378" t="inlineStr">
-        <is>
-          <t>Dell Inc.</t>
-        </is>
-      </c>
-      <c r="L378" t="inlineStr">
-        <is>
-          <t>OptiPlex 3040</t>
-        </is>
-      </c>
-      <c r="M378" t="n">
-        <v>2</v>
-      </c>
-      <c r="N378" s="3" t="n">
-        <v>46086.37909722222</v>
-      </c>
-      <c r="O378" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-05 13:52:06.540171
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -434,7 +434,7 @@
   <cols>
     <col width="25.2" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="32.4" customWidth="1" min="3" max="3"/>
+    <col width="15.6" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="10.8" customWidth="1" min="5" max="5"/>
     <col width="50.4" customWidth="1" min="6" max="6"/>
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46086.46652777777</v>
+        <v>46086.54734953704</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46086.47596064815</v>
+        <v>46086.5585300926</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46086.47538194444</v>
+        <v>46086.55202546297</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46086.45210648148</v>
+        <v>46086.56354166667</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46086.48438657408</v>
+        <v>46086.56211805555</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46086.46130787037</v>
+        <v>46086.53922453704</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46086.47638888889</v>
+        <v>46086.55351851852</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46086.45846064815</v>
+        <v>46086.53814814815</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1702,7 +1702,7 @@
         <v>1</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>46086.46201388889</v>
+        <v>46086.54344907407</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1766,7 +1766,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46086.46438657407</v>
+        <v>46086.54491898148</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>46086.38715277778</v>
+        <v>46086.538125</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -1903,6 +1903,11 @@
           <t>AUDITORIO</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>10.69.3.150</t>
+        </is>
+      </c>
       <c r="D23" t="n">
         <v>2019</v>
       </c>
@@ -1943,7 +1948,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46086.13231481481</v>
+        <v>46086.56766203704</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2077,11 +2082,6 @@
           <t>AUDITORIO</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>10.69.3.151</t>
-        </is>
-      </c>
       <c r="D26" t="n">
         <v>2019</v>
       </c>
@@ -2122,7 +2122,7 @@
         <v>1</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>46086.46799768518</v>
+        <v>46086.53834490741</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46086.45563657407</v>
+        <v>46086.53677083334</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6509,7 +6509,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46086.48377314815</v>
+        <v>46086.55824074074</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6578,7 +6578,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46086.47763888889</v>
+        <v>46086.55083333333</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6642,7 +6642,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46086.46075231482</v>
+        <v>46086.54142361111</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6661,6 +6661,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>10.69.3.94</t>
+        </is>
+      </c>
       <c r="D97" t="n">
         <v>2025</v>
       </c>
@@ -6706,7 +6711,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46086.46108796296</v>
+        <v>46086.57056712963</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6775,7 +6780,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46086.4597337963</v>
+        <v>46086.539375</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6844,7 +6849,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46086.47921296296</v>
+        <v>46086.55912037037</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6913,7 +6918,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46086.44953703704</v>
+        <v>46086.56761574074</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -7051,7 +7056,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46085.79913194444</v>
+        <v>46086.54584490741</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7308,7 +7313,7 @@
         <v>1</v>
       </c>
       <c r="N106" s="3" t="n">
-        <v>46086.48730324074</v>
+        <v>46086.56547453703</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -7446,7 +7451,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46086.45457175926</v>
+        <v>46086.56940972222</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7515,7 +7520,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46086.47501157408</v>
+        <v>46086.5525</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7584,7 +7589,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46086.48096064815</v>
+        <v>46086.56043981481</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7653,7 +7658,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46086.45567129629</v>
+        <v>46086.5387962963</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7722,7 +7727,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46086.48214120371</v>
+        <v>46086.55564814815</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7791,7 +7796,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46086.46743055555</v>
+        <v>46086.5429050926</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7857,7 +7862,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46086.46832175926</v>
+        <v>46086.54194444444</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7926,7 +7931,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46086.48017361111</v>
+        <v>46086.55969907407</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7995,7 +8000,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46086.48278935185</v>
+        <v>46086.56939814815</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8061,7 +8066,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46086.451875</v>
+        <v>46086.56751157407</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8199,7 +8204,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46086.46931712963</v>
+        <v>46086.54643518518</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8220,7 +8225,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>fe80::3df5:59e9:a13f:475e</t>
+          <t>10.69.3.98</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -8268,7 +8273,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46086.28118055555</v>
+        <v>46086.56476851852</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8334,7 +8339,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46086.44712962963</v>
+        <v>46086.56537037037</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8403,7 +8408,7 @@
         <v>2</v>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46085.82665509259</v>
+        <v>46086.54609953704</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8472,7 +8477,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46086.46287037037</v>
+        <v>46086.5393287037</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8541,7 +8546,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46086.46935185185</v>
+        <v>46086.54670138889</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8610,7 +8615,7 @@
         <v>2</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46086.4665625</v>
+        <v>46086.54053240741</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8748,7 +8753,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46086.47401620371</v>
+        <v>46086.5471875</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8817,7 +8822,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46086.4516087963</v>
+        <v>46086.53123842592</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8886,7 +8891,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46086.45138888889</v>
+        <v>46086.56780092593</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -8905,11 +8910,6 @@
           <t>ADM/FIN</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>10.69.3.6</t>
-        </is>
-      </c>
       <c r="D130" t="n">
         <v>2025</v>
       </c>
@@ -8955,7 +8955,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46086.46967592592</v>
+        <v>46086.54608796296</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9088,7 +9088,7 @@
         <v>1</v>
       </c>
       <c r="N132" s="3" t="n">
-        <v>46086.48734953703</v>
+        <v>46086.55947916667</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -9407,7 +9407,7 @@
         <v>1</v>
       </c>
       <c r="N137" s="3" t="n">
-        <v>46086.46420138889</v>
+        <v>46086.54079861111</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -9599,7 +9599,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46086.48736111111</v>
+        <v>46086.54980324074</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9663,7 +9663,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46086.48607638889</v>
+        <v>46086.54797453704</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9727,7 +9727,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46086.48116898148</v>
+        <v>46086.55568287037</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9791,7 +9791,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46086.4822337963</v>
+        <v>46086.55782407407</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9855,7 +9855,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46086.4693287037</v>
+        <v>46086.56469907407</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9919,7 +9919,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46086.48672453704</v>
+        <v>46086.56111111111</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9983,7 +9983,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46086.48060185185</v>
+        <v>46086.53880787037</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10047,7 +10047,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46086.46024305555</v>
+        <v>46086.56888888889</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10111,7 +10111,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46086.46627314815</v>
+        <v>46086.54289351852</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10175,7 +10175,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46086.46534722222</v>
+        <v>46086.54293981481</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10239,7 +10239,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46086.47047453704</v>
+        <v>46086.54318287037</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10303,7 +10303,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46086.45927083334</v>
+        <v>46086.53462962963</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10426,7 +10426,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46086.48105324074</v>
+        <v>46086.56045138889</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10490,7 +10490,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46086.45704861111</v>
+        <v>46086.53581018518</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10554,7 +10554,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46086.485625</v>
+        <v>46086.57148148148</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10618,7 +10618,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46086.4531712963</v>
+        <v>46086.53388888889</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10746,7 +10746,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46086.46329861111</v>
+        <v>46086.54481481481</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10810,7 +10810,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46086.45902777778</v>
+        <v>46086.53461805556</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10874,7 +10874,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46086.45204861111</v>
+        <v>46086.53133101852</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10938,7 +10938,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46086.44923611111</v>
+        <v>46086.56592592593</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -11066,7 +11066,7 @@
         <v>2</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46086.48075231481</v>
+        <v>46086.55782407407</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11130,7 +11130,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46086.4852662037</v>
+        <v>46086.56768518518</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11194,7 +11194,7 @@
         <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46086.45913194444</v>
+        <v>46086.53895833333</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11258,7 +11258,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46086.44865740741</v>
+        <v>46086.56899305555</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11322,7 +11322,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46086.47234953703</v>
+        <v>46086.54707175926</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11386,7 +11386,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46086.48077546297</v>
+        <v>46086.55512731482</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11450,7 +11450,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46086.4852662037</v>
+        <v>46086.56517361111</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11511,10 +11511,10 @@
         </is>
       </c>
       <c r="M170" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46086.47979166666</v>
+        <v>46086.55554398148</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11578,7 +11578,7 @@
         <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46085.76966435185</v>
+        <v>46086.54628472222</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11639,10 +11639,10 @@
         </is>
       </c>
       <c r="M172" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46086.44788194444</v>
+        <v>46086.56407407407</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11706,7 +11706,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46086.48649305556</v>
+        <v>46086.56207175926</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11770,7 +11770,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46086.46126157408</v>
+        <v>46086.56138888889</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11834,7 +11834,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46086.45366898148</v>
+        <v>46086.57109953704</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11898,7 +11898,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46085.73752314815</v>
+        <v>46086.54363425926</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11962,7 +11962,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46086.47534722222</v>
+        <v>46086.5466087963</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12026,7 +12026,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46086.45335648148</v>
+        <v>46086.53083333333</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12479,7 +12479,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46086.48545138889</v>
+        <v>46086.48881944444</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12543,7 +12543,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46086.48327546296</v>
+        <v>46086.56497685185</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12607,7 +12607,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46086.48667824074</v>
+        <v>46086.55085648148</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12735,7 +12735,7 @@
         </is>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46086.45497685186</v>
+        <v>46086.56776620371</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12799,7 +12799,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46086.4852662037</v>
+        <v>46086.56270833333</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12863,7 +12863,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46086.47489583334</v>
+        <v>46086.55246527777</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12988,7 +12988,7 @@
         <v>2</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46086.45892361111</v>
+        <v>46086.55278935185</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13052,7 +13052,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46086.4775</v>
+        <v>46086.55434027778</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13116,7 +13116,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46086.48744212963</v>
+        <v>46086.57033564815</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13180,7 +13180,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46086.47625</v>
+        <v>46086.55554398148</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13244,7 +13244,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46086.46800925926</v>
+        <v>46086.5665162037</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13308,7 +13308,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46086.48143518518</v>
+        <v>46086.55810185185</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13372,7 +13372,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46086.48605324074</v>
+        <v>46086.55584490741</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13433,7 +13433,7 @@
         </is>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46086.461875</v>
+        <v>46086.53946759259</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13497,7 +13497,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46086.48416666667</v>
+        <v>46086.56543981482</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13561,7 +13561,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46086.48521990741</v>
+        <v>46086.56703703704</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13625,7 +13625,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46086.4809375</v>
+        <v>46086.56609953703</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13689,7 +13689,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46086.48296296296</v>
+        <v>46086.55907407407</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13753,7 +13753,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46086.4811574074</v>
+        <v>46086.5578125</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13817,7 +13817,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46086.48592592592</v>
+        <v>46086.5540625</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13881,7 +13881,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46086.48792824074</v>
+        <v>46086.55996527777</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13945,7 +13945,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46086.48673611111</v>
+        <v>46086.53344907407</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14009,7 +14009,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46086.48354166667</v>
+        <v>46086.55935185185</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14073,7 +14073,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46086.45252314815</v>
+        <v>46086.56763888889</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14137,7 +14137,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46086.45130787037</v>
+        <v>46086.56561342593</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14201,7 +14201,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46086.46039351852</v>
+        <v>46086.56063657408</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14265,7 +14265,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46086.45643518519</v>
+        <v>46086.53673611111</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14393,7 +14393,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46086.45061342593</v>
+        <v>46086.56427083333</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14457,7 +14457,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46086.45341435185</v>
+        <v>46086.53141203704</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14521,7 +14521,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46086.45321759259</v>
+        <v>46086.55721064815</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14585,7 +14585,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46086.47951388889</v>
+        <v>46086.55291666667</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14654,7 +14654,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46086.4562037037</v>
+        <v>46086.53756944444</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14718,7 +14718,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46086.46083333333</v>
+        <v>46086.54011574074</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14782,7 +14782,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46086.45542824074</v>
+        <v>46086.56412037037</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14974,7 +14974,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46086.48032407407</v>
+        <v>46086.53378472223</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15102,7 +15102,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46086.45277777778</v>
+        <v>46086.54140046296</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15166,7 +15166,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46086.45018518518</v>
+        <v>46086.54310185185</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15230,7 +15230,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46086.48097222222</v>
+        <v>46086.53358796296</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15294,7 +15294,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46086.48631944445</v>
+        <v>46086.56608796296</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15358,7 +15358,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46086.48681712963</v>
+        <v>46086.55567129629</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15422,7 +15422,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46086.4800925926</v>
+        <v>46086.55803240741</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15486,7 +15486,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46086.48592592592</v>
+        <v>46086.55655092592</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15550,7 +15550,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46086.4724537037</v>
+        <v>46086.55728009259</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15614,7 +15614,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46086.45128472222</v>
+        <v>46086.57033564815</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15678,7 +15678,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46086.46178240741</v>
+        <v>46086.53755787037</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15806,7 +15806,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46086.45151620371</v>
+        <v>46086.56685185185</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15870,7 +15870,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46086.45078703704</v>
+        <v>46086.56699074074</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15934,7 +15934,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46086.4868287037</v>
+        <v>46086.55951388889</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -16062,7 +16062,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46086.48515046296</v>
+        <v>46086.56277777778</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16126,7 +16126,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46086.45065972222</v>
+        <v>46086.53465277778</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16313,7 +16313,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46086.45243055555</v>
+        <v>46086.56994212963</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16377,7 +16377,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46086.48556712963</v>
+        <v>46086.53706018518</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16441,7 +16441,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46086.46643518518</v>
+        <v>46086.54010416667</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16505,7 +16505,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46086.46540509259</v>
+        <v>46086.56269675926</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16564,7 +16564,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46086.45695601852</v>
+        <v>46086.55824074074</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16628,7 +16628,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46086.47061342592</v>
+        <v>46086.54458333334</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16692,7 +16692,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46086.48546296296</v>
+        <v>46086.56668981481</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16756,7 +16756,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46086.48490740741</v>
+        <v>46086.55440972222</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16814,7 +16814,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46086.47336805556</v>
+        <v>46086.54768518519</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16878,7 +16878,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46086.46005787037</v>
+        <v>46086.53614583334</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16942,7 +16942,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46086.48478009259</v>
+        <v>46086.54738425926</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -17006,7 +17006,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46086.48712962963</v>
+        <v>46086.56980324074</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17070,7 +17070,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46086.48418981482</v>
+        <v>46086.57131944445</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17198,7 +17198,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46086.47641203704</v>
+        <v>46086.5600462963</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17326,7 +17326,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46086.46162037037</v>
+        <v>46086.54098379629</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17390,7 +17390,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46086.47432870371</v>
+        <v>46086.55172453704</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17454,7 +17454,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46086.48039351852</v>
+        <v>46086.56313657408</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17518,7 +17518,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46086.48795138889</v>
+        <v>46086.55991898148</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17582,7 +17582,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46086.48091435185</v>
+        <v>46086.55612268519</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17646,7 +17646,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46086.48263888889</v>
+        <v>46086.55065972222</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17774,7 +17774,7 @@
         <v>1</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46086.48427083333</v>
+        <v>46086.56993055555</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17835,7 +17835,7 @@
         </is>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46086.47372685185</v>
+        <v>46086.55670138889</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17963,7 +17963,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46086.47012731482</v>
+        <v>46086.54646990741</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -18088,7 +18088,7 @@
         </is>
       </c>
       <c r="N273" s="3" t="n">
-        <v>46086.46725694444</v>
+        <v>46086.54734953704</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -18336,7 +18336,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46086.47909722223</v>
+        <v>46086.53140046296</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18400,7 +18400,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46086.47094907407</v>
+        <v>46086.54560185185</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18523,7 +18523,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46086.45322916667</v>
+        <v>46086.55077546297</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18542,6 +18542,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>10.69.5.151</t>
+        </is>
+      </c>
       <c r="D281" t="n">
         <v>2017</v>
       </c>
@@ -18582,7 +18587,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46086.45104166667</v>
+        <v>46086.570625</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18646,7 +18651,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46086.47237268519</v>
+        <v>46086.5349537037</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18710,7 +18715,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46086.45143518518</v>
+        <v>46086.53375</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18774,7 +18779,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46086.48563657407</v>
+        <v>46086.56354166667</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18833,7 +18838,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46086.45297453704</v>
+        <v>46086.52972222222</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18897,7 +18902,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46086.45162037037</v>
+        <v>46086.56226851852</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18961,7 +18966,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46086.48631944445</v>
+        <v>46086.54943287037</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19025,7 +19030,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46086.46020833333</v>
+        <v>46086.53855324074</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19819,7 +19824,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46086.46232638889</v>
+        <v>46086.54129629629</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20935,7 +20940,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46086.4737962963</v>
+        <v>46086.55199074074</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21660,7 +21665,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46086.48090277778</v>
+        <v>46086.55931712963</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21724,7 +21729,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46086.47077546296</v>
+        <v>46086.54563657408</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21788,7 +21793,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46086.47649305555</v>
+        <v>46086.55033564815</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21852,7 +21857,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46086.47467592593</v>
+        <v>46086.55209490741</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21916,7 +21921,7 @@
         <v>2</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46086.4572800926</v>
+        <v>46086.53636574074</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21980,7 +21985,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46086.4875</v>
+        <v>46086.5565625</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22044,7 +22049,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46086.476875</v>
+        <v>46086.55143518518</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22108,7 +22113,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46086.46547453704</v>
+        <v>46086.54150462963</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22172,7 +22177,7 @@
         <v>1</v>
       </c>
       <c r="N339" s="3" t="n">
-        <v>46085.58538194445</v>
+        <v>46086.55</v>
       </c>
       <c r="O339" t="inlineStr">
         <is>
@@ -22300,7 +22305,7 @@
         <v>2</v>
       </c>
       <c r="N341" s="3" t="n">
-        <v>46086.47333333334</v>
+        <v>46086.5546875</v>
       </c>
       <c r="O341" t="inlineStr">
         <is>
@@ -22319,11 +22324,6 @@
           <t>OPERACAO 9.1</t>
         </is>
       </c>
-      <c r="C342" t="inlineStr">
-        <is>
-          <t>10.69.5.237</t>
-        </is>
-      </c>
       <c r="D342" t="n">
         <v>2017</v>
       </c>
@@ -22366,7 +22366,7 @@
         </is>
       </c>
       <c r="N342" s="3" t="n">
-        <v>46086.47072916666</v>
+        <v>46086.55002314815</v>
       </c>
       <c r="O342" t="inlineStr">
         <is>
@@ -22622,7 +22622,7 @@
         <v>1</v>
       </c>
       <c r="N346" s="3" t="n">
-        <v>46086.46128472222</v>
+        <v>46086.54282407407</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -22686,7 +22686,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46086.45493055556</v>
+        <v>46086.53469907407</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22750,7 +22750,7 @@
         <v>1</v>
       </c>
       <c r="N348" s="3" t="n">
-        <v>46086.45190972222</v>
+        <v>46086.53243055556</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -22875,7 +22875,7 @@
         <v>1</v>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46086.45523148148</v>
+        <v>46086.5347337963</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -22939,7 +22939,7 @@
         <v>1</v>
       </c>
       <c r="N351" s="3" t="n">
-        <v>46086.45574074074</v>
+        <v>46086.53942129629</v>
       </c>
       <c r="O351" t="inlineStr">
         <is>
@@ -23125,7 +23125,7 @@
         <v>1</v>
       </c>
       <c r="N354" s="3" t="n">
-        <v>46086.45224537037</v>
+        <v>46086.53109953704</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -23189,7 +23189,7 @@
         <v>1</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46086.48635416666</v>
+        <v>46086.56251157408</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23253,7 +23253,7 @@
         <v>1</v>
       </c>
       <c r="N356" s="3" t="n">
-        <v>46086.45384259259</v>
+        <v>46086.57060185185</v>
       </c>
       <c r="O356" t="inlineStr">
         <is>
@@ -23381,7 +23381,7 @@
         <v>2</v>
       </c>
       <c r="N358" s="3" t="n">
-        <v>46086.45366898148</v>
+        <v>46086.53559027778</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -23509,7 +23509,7 @@
         <v>1</v>
       </c>
       <c r="N360" s="3" t="n">
-        <v>46086.45371527778</v>
+        <v>46086.5333912037</v>
       </c>
       <c r="O360" t="inlineStr">
         <is>
@@ -23758,7 +23758,7 @@
         <v>1</v>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46086.47571759259</v>
+        <v>46086.55401620371</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23824,7 +23824,7 @@
         </is>
       </c>
       <c r="N365" s="3" t="n">
-        <v>46086.46056712963</v>
+        <v>46086.49859953704</v>
       </c>
       <c r="O365" t="inlineStr">
         <is>
@@ -23950,7 +23950,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46086.45829861111</v>
+        <v>46086.53605324074</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -24080,7 +24080,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46086.45896990741</v>
+        <v>46086.5350925926</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24099,6 +24099,11 @@
           <t>RH</t>
         </is>
       </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>10.69.3.30</t>
+        </is>
+      </c>
       <c r="H370" t="inlineStr">
         <is>
           <t>Microsoft Office Standard 2013</t>
@@ -24113,7 +24118,7 @@
         <v>2</v>
       </c>
       <c r="N370" s="3" t="n">
-        <v>46086.45856481481</v>
+        <v>46086.53611111111</v>
       </c>
       <c r="O370" t="inlineStr">
         <is>
@@ -24320,7 +24325,7 @@
         <v>1</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46086.4647337963</v>
+        <v>46086.54009259259</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24386,7 +24391,7 @@
         </is>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46086.45899305555</v>
+        <v>46086.53696759259</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24450,7 +24455,7 @@
         <v>1</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46086.46025462963</v>
+        <v>46086.53849537037</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24519,7 +24524,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46086.45298611111</v>
+        <v>46086.56872685185</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -24588,7 +24593,7 @@
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46086.45694444444</v>
+        <v>46086.53766203704</v>
       </c>
       <c r="O377" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-05 15:52:05.766352
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46086.54734953704</v>
+        <v>46086.62292824074</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46086.5585300926</v>
+        <v>46086.63348379629</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46086.55202546297</v>
+        <v>46086.62827546296</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46086.56354166667</v>
+        <v>46086.64232638889</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46086.56211805555</v>
+        <v>46086.63391203704</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46086.53922453704</v>
+        <v>46086.61805555555</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46086.55351851852</v>
+        <v>46086.63253472222</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46086.53814814815</v>
+        <v>46086.64976851852</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1702,7 +1702,7 @@
         <v>1</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>46086.54344907407</v>
+        <v>46086.6240625</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1766,7 +1766,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46086.54491898148</v>
+        <v>46086.62108796297</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>46086.538125</v>
+        <v>46086.57885416667</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46086.56766203704</v>
+        <v>46086.64804398148</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2122,7 +2122,7 @@
         <v>1</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>46086.53834490741</v>
+        <v>46086.61798611111</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46086.53677083334</v>
+        <v>46086.62038194444</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6509,7 +6509,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46086.55824074074</v>
+        <v>46086.65357638889</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6578,7 +6578,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46086.55083333333</v>
+        <v>46086.63059027777</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6642,7 +6642,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46086.54142361111</v>
+        <v>46086.62019675926</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6711,7 +6711,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46086.57056712963</v>
+        <v>46086.64849537037</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6780,7 +6780,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46086.539375</v>
+        <v>46086.62085648148</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6849,7 +6849,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46086.55912037037</v>
+        <v>46086.63890046296</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6918,7 +6918,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46086.56761574074</v>
+        <v>46086.64719907408</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -7056,7 +7056,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46086.54584490741</v>
+        <v>46086.62041666666</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7313,7 +7313,7 @@
         <v>1</v>
       </c>
       <c r="N106" s="3" t="n">
-        <v>46086.56547453703</v>
+        <v>46086.64363425926</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -7451,7 +7451,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46086.56940972222</v>
+        <v>46086.64982638889</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7520,7 +7520,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46086.5525</v>
+        <v>46086.63175925926</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7589,7 +7589,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46086.56043981481</v>
+        <v>46086.64012731481</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7658,7 +7658,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46086.5387962963</v>
+        <v>46086.65050925926</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7727,7 +7727,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46086.55564814815</v>
+        <v>46086.64008101852</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7796,7 +7796,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46086.5429050926</v>
+        <v>46086.62225694444</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7862,7 +7862,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46086.54194444444</v>
+        <v>46086.62060185185</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7931,7 +7931,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46086.55969907407</v>
+        <v>46086.63061342593</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -8000,7 +8000,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46086.56939814815</v>
+        <v>46086.64890046296</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8066,7 +8066,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46086.56751157407</v>
+        <v>46086.64194444445</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8204,7 +8204,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46086.54643518518</v>
+        <v>46086.62503472222</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8273,7 +8273,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46086.56476851852</v>
+        <v>46086.64907407408</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8339,7 +8339,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46086.56537037037</v>
+        <v>46086.64605324074</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8408,7 +8408,7 @@
         <v>2</v>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46086.54609953704</v>
+        <v>46086.6240625</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8477,7 +8477,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46086.5393287037</v>
+        <v>46086.65256944444</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8546,7 +8546,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46086.54670138889</v>
+        <v>46086.62321759259</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8615,7 +8615,7 @@
         <v>2</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46086.54053240741</v>
+        <v>46086.61710648148</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8753,7 +8753,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46086.5471875</v>
+        <v>46086.62005787037</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8822,7 +8822,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46086.53123842592</v>
+        <v>46086.65203703703</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8891,7 +8891,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46086.56780092593</v>
+        <v>46086.64722222222</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -8955,7 +8955,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46086.54608796296</v>
+        <v>46086.58516203704</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9088,7 +9088,7 @@
         <v>1</v>
       </c>
       <c r="N132" s="3" t="n">
-        <v>46086.55947916667</v>
+        <v>46086.63030092593</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -9152,7 +9152,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46085.8197337963</v>
+        <v>46086.62606481482</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9216,7 +9216,7 @@
         <v>1</v>
       </c>
       <c r="N134" s="3" t="n">
-        <v>46085.82491898148</v>
+        <v>46086.61770833333</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -9407,7 +9407,7 @@
         <v>1</v>
       </c>
       <c r="N137" s="3" t="n">
-        <v>46086.54079861111</v>
+        <v>46086.61796296296</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -9471,7 +9471,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46085.79331018519</v>
+        <v>46086.62364583334</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9535,7 +9535,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46085.81833333334</v>
+        <v>46086.62584490741</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9599,7 +9599,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46086.54980324074</v>
+        <v>46086.62326388889</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9663,7 +9663,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46086.54797453704</v>
+        <v>46086.64707175926</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9727,7 +9727,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46086.55568287037</v>
+        <v>46086.63158564815</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9791,7 +9791,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46086.55782407407</v>
+        <v>46086.63318287037</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9855,7 +9855,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46086.56469907407</v>
+        <v>46086.62364583334</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9919,7 +9919,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46086.56111111111</v>
+        <v>46086.62401620371</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9983,7 +9983,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46086.53880787037</v>
+        <v>46086.64246527778</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10047,7 +10047,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46086.56888888889</v>
+        <v>46086.64841435185</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10111,7 +10111,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46086.54289351852</v>
+        <v>46086.61893518519</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10239,7 +10239,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46086.54318287037</v>
+        <v>46086.62425925926</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10303,7 +10303,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46086.53462962963</v>
+        <v>46086.63127314814</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10362,7 +10362,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46086.32950231482</v>
+        <v>46086.62116898148</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10426,7 +10426,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46086.56045138889</v>
+        <v>46086.62368055555</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10490,7 +10490,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46086.53581018518</v>
+        <v>46086.65115740741</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10554,7 +10554,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46086.57148148148</v>
+        <v>46086.65168981482</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10618,7 +10618,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46086.53388888889</v>
+        <v>46086.57491898148</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10746,7 +10746,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46086.54481481481</v>
+        <v>46086.61965277778</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10810,7 +10810,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46086.53461805556</v>
+        <v>46086.61603009259</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10874,7 +10874,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46086.53133101852</v>
+        <v>46086.57278935185</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10938,7 +10938,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46086.56592592593</v>
+        <v>46086.62626157407</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -11066,7 +11066,7 @@
         <v>2</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46086.55782407407</v>
+        <v>46086.63715277778</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11130,7 +11130,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46086.56768518518</v>
+        <v>46086.60918981482</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11194,7 +11194,7 @@
         <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46086.53895833333</v>
+        <v>46086.62033564815</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11258,7 +11258,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46086.56899305555</v>
+        <v>46086.60868055555</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11386,7 +11386,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46086.55512731482</v>
+        <v>46086.6363425926</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11450,7 +11450,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46086.56517361111</v>
+        <v>46086.61810185185</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11578,7 +11578,7 @@
         <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46086.54628472222</v>
+        <v>46086.62856481481</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11642,7 +11642,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46086.56407407407</v>
+        <v>46086.64271990741</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11770,7 +11770,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46086.56138888889</v>
+        <v>46086.64317129629</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11834,7 +11834,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46086.57109953704</v>
+        <v>46086.64773148148</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11898,7 +11898,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46086.54363425926</v>
+        <v>46086.62203703704</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11962,7 +11962,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46086.5466087963</v>
+        <v>46086.61998842593</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12026,7 +12026,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46086.53083333333</v>
+        <v>46086.63445601852</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12090,7 +12090,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46086.37944444444</v>
+        <v>46086.6222337963</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12154,7 +12154,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46085.82769675926</v>
+        <v>46086.62366898148</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12479,7 +12479,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46086.48881944444</v>
+        <v>46086.63839120371</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12543,7 +12543,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46086.56497685185</v>
+        <v>46086.64640046296</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12607,7 +12607,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46086.55085648148</v>
+        <v>46086.62726851852</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12735,7 +12735,7 @@
         </is>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46086.56776620371</v>
+        <v>46086.63175925926</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12799,7 +12799,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46086.56270833333</v>
+        <v>46086.64098379629</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12863,7 +12863,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46086.55246527777</v>
+        <v>46086.61967592593</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12988,7 +12988,7 @@
         <v>2</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46086.55278935185</v>
+        <v>46086.58027777778</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13052,7 +13052,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46086.55434027778</v>
+        <v>46086.63425925926</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13116,7 +13116,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46086.57033564815</v>
+        <v>46086.64945601852</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13180,7 +13180,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46086.55554398148</v>
+        <v>46086.6284375</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13244,7 +13244,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46086.5665162037</v>
+        <v>46086.61712962963</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13308,7 +13308,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46086.55810185185</v>
+        <v>46086.62266203704</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13372,7 +13372,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46086.55584490741</v>
+        <v>46086.62221064815</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13433,7 +13433,7 @@
         </is>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46086.53946759259</v>
+        <v>46086.61435185185</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13497,7 +13497,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46086.56543981482</v>
+        <v>46086.64203703704</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13561,7 +13561,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46086.56703703704</v>
+        <v>46086.62202546297</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13625,7 +13625,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46086.56609953703</v>
+        <v>46086.63148148148</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13689,7 +13689,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46086.55907407407</v>
+        <v>46086.63934027778</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13753,7 +13753,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46086.5578125</v>
+        <v>46086.60002314814</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13817,7 +13817,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46086.5540625</v>
+        <v>46086.63071759259</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13881,7 +13881,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46086.55996527777</v>
+        <v>46086.61907407407</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13945,7 +13945,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46086.53344907407</v>
+        <v>46086.6215162037</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14009,7 +14009,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46086.55935185185</v>
+        <v>46086.6364699074</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14073,7 +14073,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46086.56763888889</v>
+        <v>46086.6211574074</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14137,7 +14137,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46086.56561342593</v>
+        <v>46086.64259259259</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14201,7 +14201,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46086.56063657408</v>
+        <v>46086.64300925926</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14265,7 +14265,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46086.53673611111</v>
+        <v>46086.61386574074</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14329,7 +14329,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46085.80710648148</v>
+        <v>46086.64314814815</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14393,7 +14393,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46086.56427083333</v>
+        <v>46086.64166666667</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14457,7 +14457,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46086.53141203704</v>
+        <v>46086.64509259259</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14521,7 +14521,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46086.55721064815</v>
+        <v>46086.6295949074</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14585,7 +14585,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46086.55291666667</v>
+        <v>46086.64335648148</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14654,7 +14654,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46086.53756944444</v>
+        <v>46086.6346412037</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14718,7 +14718,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46086.54011574074</v>
+        <v>46086.61489583334</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14782,7 +14782,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46086.56412037037</v>
+        <v>46086.6412037037</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14910,7 +14910,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46085.82674768518</v>
+        <v>46086.6403587963</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14974,7 +14974,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46086.53378472223</v>
+        <v>46086.6397337963</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15038,7 +15038,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46085.79258101852</v>
+        <v>46086.64273148148</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15102,7 +15102,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46086.54140046296</v>
+        <v>46086.61924768519</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15166,7 +15166,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46086.54310185185</v>
+        <v>46086.62142361111</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15230,7 +15230,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46086.53358796296</v>
+        <v>46086.63552083333</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15294,7 +15294,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46086.56608796296</v>
+        <v>46086.62216435185</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15358,7 +15358,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46086.55567129629</v>
+        <v>46086.62793981482</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15422,7 +15422,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46086.55803240741</v>
+        <v>46086.62101851852</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15486,7 +15486,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46086.55655092592</v>
+        <v>46086.63449074074</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15550,7 +15550,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46086.55728009259</v>
+        <v>46086.6346875</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15614,7 +15614,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46086.57033564815</v>
+        <v>46086.64796296296</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15678,7 +15678,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46086.53755787037</v>
+        <v>46086.64922453704</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15742,7 +15742,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46086.39325231482</v>
+        <v>46086.63444444445</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15806,7 +15806,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46086.56685185185</v>
+        <v>46086.63460648148</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15870,7 +15870,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46086.56699074074</v>
+        <v>46086.63521990741</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15934,7 +15934,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46086.55951388889</v>
+        <v>46086.63064814815</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -15998,7 +15998,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46085.82322916666</v>
+        <v>46086.63387731482</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16062,7 +16062,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46086.56277777778</v>
+        <v>46086.64121527778</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16126,7 +16126,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46086.53465277778</v>
+        <v>46086.65333333334</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16249,7 +16249,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46086.31018518518</v>
+        <v>46086.62921296297</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16313,7 +16313,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46086.56994212963</v>
+        <v>46086.65322916667</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16377,7 +16377,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46086.53706018518</v>
+        <v>46086.64903935185</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16441,7 +16441,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46086.54010416667</v>
+        <v>46086.62208333334</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16505,7 +16505,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46086.56269675926</v>
+        <v>46086.64417824074</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16564,7 +16564,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46086.55824074074</v>
+        <v>46086.63688657407</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16628,7 +16628,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46086.54458333334</v>
+        <v>46086.62525462963</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16692,7 +16692,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46086.56668981481</v>
+        <v>46086.65038194445</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16756,7 +16756,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46086.55440972222</v>
+        <v>46086.62689814815</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16814,7 +16814,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46086.54768518519</v>
+        <v>46086.64251157407</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16878,7 +16878,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46086.53614583334</v>
+        <v>46086.65269675926</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16942,7 +16942,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46086.54738425926</v>
+        <v>46086.62762731482</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -17006,7 +17006,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46086.56980324074</v>
+        <v>46086.64444444444</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17070,7 +17070,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46086.57131944445</v>
+        <v>46086.64767361111</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17134,7 +17134,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46086.32549768518</v>
+        <v>46086.63461805556</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17198,7 +17198,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46086.5600462963</v>
+        <v>46086.60144675926</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17262,7 +17262,7 @@
         <v>2</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46085.79364583334</v>
+        <v>46086.6280787037</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17326,7 +17326,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46086.54098379629</v>
+        <v>46086.65394675926</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17390,7 +17390,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46086.55172453704</v>
+        <v>46086.62688657407</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17454,7 +17454,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46086.56313657408</v>
+        <v>46086.64292824074</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17518,7 +17518,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46086.55991898148</v>
+        <v>46086.63168981481</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17582,7 +17582,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46086.55612268519</v>
+        <v>46086.63131944444</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17646,7 +17646,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46086.55065972222</v>
+        <v>46086.62418981481</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17710,7 +17710,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46085.71986111111</v>
+        <v>46086.63945601852</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17774,7 +17774,7 @@
         <v>1</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46086.56993055555</v>
+        <v>46086.64575231481</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17835,7 +17835,7 @@
         </is>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46086.55670138889</v>
+        <v>46086.63175925926</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17899,7 +17899,7 @@
         <v>1</v>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46086.11908564815</v>
+        <v>46086.59438657408</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -17963,7 +17963,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46086.54646990741</v>
+        <v>46086.62944444444</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -18088,7 +18088,7 @@
         </is>
       </c>
       <c r="N273" s="3" t="n">
-        <v>46086.54734953704</v>
+        <v>46086.62548611111</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -18336,7 +18336,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46086.53140046296</v>
+        <v>46086.57177083333</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18400,7 +18400,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46086.54560185185</v>
+        <v>46086.62020833333</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18587,7 +18587,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46086.570625</v>
+        <v>46086.65070601852</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18651,7 +18651,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46086.5349537037</v>
+        <v>46086.6178125</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18715,7 +18715,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46086.53375</v>
+        <v>46086.61560185185</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18779,7 +18779,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46086.56354166667</v>
+        <v>46086.64155092592</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18838,7 +18838,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46086.52972222222</v>
+        <v>46086.57170138889</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18902,7 +18902,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46086.56226851852</v>
+        <v>46086.64159722222</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -19030,7 +19030,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46086.53855324074</v>
+        <v>46086.64975694445</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19824,7 +19824,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46086.54129629629</v>
+        <v>46086.61756944445</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20940,7 +20940,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46086.55199074074</v>
+        <v>46086.63533564815</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21665,7 +21665,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46086.55931712963</v>
+        <v>46086.63486111111</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21729,7 +21729,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46086.54563657408</v>
+        <v>46086.61876157407</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21793,7 +21793,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46086.55033564815</v>
+        <v>46086.63197916667</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21857,7 +21857,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46086.55209490741</v>
+        <v>46086.62888888889</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21921,7 +21921,7 @@
         <v>2</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46086.53636574074</v>
+        <v>46086.64973379629</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21985,7 +21985,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46086.5565625</v>
+        <v>46086.63869212963</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22049,7 +22049,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46086.55143518518</v>
+        <v>46086.62677083333</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22113,7 +22113,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46086.54150462963</v>
+        <v>46086.62094907407</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22366,7 +22366,7 @@
         </is>
       </c>
       <c r="N342" s="3" t="n">
-        <v>46086.55002314815</v>
+        <v>46086.58853009259</v>
       </c>
       <c r="O342" t="inlineStr">
         <is>
@@ -22622,7 +22622,7 @@
         <v>1</v>
       </c>
       <c r="N346" s="3" t="n">
-        <v>46086.54282407407</v>
+        <v>46086.58059027778</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -22686,7 +22686,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46086.53469907407</v>
+        <v>46086.57520833334</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22750,7 +22750,7 @@
         <v>1</v>
       </c>
       <c r="N348" s="3" t="n">
-        <v>46086.53243055556</v>
+        <v>46086.57438657407</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -22875,7 +22875,7 @@
         <v>1</v>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46086.5347337963</v>
+        <v>46086.57436342593</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -22939,7 +22939,7 @@
         <v>1</v>
       </c>
       <c r="N351" s="3" t="n">
-        <v>46086.53942129629</v>
+        <v>46086.57956018519</v>
       </c>
       <c r="O351" t="inlineStr">
         <is>
@@ -23125,7 +23125,7 @@
         <v>1</v>
       </c>
       <c r="N354" s="3" t="n">
-        <v>46086.53109953704</v>
+        <v>46086.5721875</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -23381,7 +23381,7 @@
         <v>2</v>
       </c>
       <c r="N358" s="3" t="n">
-        <v>46086.53559027778</v>
+        <v>46086.649375</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -23509,7 +23509,7 @@
         <v>1</v>
       </c>
       <c r="N360" s="3" t="n">
-        <v>46086.5333912037</v>
+        <v>46086.57539351852</v>
       </c>
       <c r="O360" t="inlineStr">
         <is>
@@ -23758,7 +23758,7 @@
         <v>1</v>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46086.55401620371</v>
+        <v>46086.63197916667</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23824,7 +23824,7 @@
         </is>
       </c>
       <c r="N365" s="3" t="n">
-        <v>46086.49859953704</v>
+        <v>46086.65172453703</v>
       </c>
       <c r="O365" t="inlineStr">
         <is>
@@ -23950,7 +23950,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46086.53605324074</v>
+        <v>46086.64650462963</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -24011,7 +24011,7 @@
         </is>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46086.45425925926</v>
+        <v>46086.58142361111</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24080,7 +24080,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46086.5350925926</v>
+        <v>46086.61481481481</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24099,16 +24099,6 @@
           <t>RH</t>
         </is>
       </c>
-      <c r="C370" t="inlineStr">
-        <is>
-          <t>10.69.3.30</t>
-        </is>
-      </c>
-      <c r="H370" t="inlineStr">
-        <is>
-          <t>Microsoft Office Standard 2013</t>
-        </is>
-      </c>
       <c r="I370" t="inlineStr">
         <is>
           <t>Intel Core i5</t>
@@ -24118,7 +24108,7 @@
         <v>2</v>
       </c>
       <c r="N370" s="3" t="n">
-        <v>46086.53611111111</v>
+        <v>46086.6280787037</v>
       </c>
       <c r="O370" t="inlineStr">
         <is>
@@ -24256,7 +24246,7 @@
         <v>1</v>
       </c>
       <c r="N372" s="3" t="n">
-        <v>46085.61537037037</v>
+        <v>46086.63756944444</v>
       </c>
       <c r="O372" t="inlineStr">
         <is>
@@ -24325,7 +24315,7 @@
         <v>1</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46086.54009259259</v>
+        <v>46086.65313657407</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24391,7 +24381,7 @@
         </is>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46086.53696759259</v>
+        <v>46086.64837962963</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24455,7 +24445,7 @@
         <v>1</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46086.53849537037</v>
+        <v>46086.61554398148</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24524,7 +24514,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46086.56872685185</v>
+        <v>46086.64222222222</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -24593,7 +24583,7 @@
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46086.53766203704</v>
+        <v>46086.65013888889</v>
       </c>
       <c r="O377" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-06 07:52:04.481876
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46086.62292824074</v>
+        <v>46087.3078125</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46086.62827546296</v>
+        <v>46086.71040509259</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -870,7 +870,7 @@
         <v>1</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>46080.48991898148</v>
+        <v>46086.72121527778</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46086.63391203704</v>
+        <v>46087.2933912037</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46086.61805555555</v>
+        <v>46087.28476851852</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46086.63253472222</v>
+        <v>46087.30774305556</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46086.64976851852</v>
+        <v>46087.28724537037</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1702,7 +1702,7 @@
         <v>1</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>46086.6240625</v>
+        <v>46087.28761574074</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1766,7 +1766,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46086.62108796297</v>
+        <v>46086.74211805555</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>46086.57885416667</v>
+        <v>46087.18209490741</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -1903,11 +1903,6 @@
           <t>AUDITORIO</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>10.69.3.150</t>
-        </is>
-      </c>
       <c r="D23" t="n">
         <v>2019</v>
       </c>
@@ -1948,7 +1943,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46086.64804398148</v>
+        <v>46087.14934027778</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2004,7 +1999,7 @@
         </is>
       </c>
       <c r="N24" s="3" t="n">
-        <v>46086.18418981481</v>
+        <v>46087.15424768518</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2122,7 +2117,7 @@
         <v>1</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>46086.61798611111</v>
+        <v>46087.10924768518</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2183,7 +2178,7 @@
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46086.62038194444</v>
+        <v>46086.69706018519</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6509,7 +6504,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46086.65357638889</v>
+        <v>46086.7349537037</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6578,7 +6573,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46086.63059027777</v>
+        <v>46086.8169212963</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6642,7 +6637,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46086.62019675926</v>
+        <v>46086.768125</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6661,11 +6656,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>10.69.3.94</t>
-        </is>
-      </c>
       <c r="D97" t="n">
         <v>2025</v>
       </c>
@@ -6711,7 +6701,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46086.64849537037</v>
+        <v>46086.68965277778</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6780,7 +6770,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46086.62085648148</v>
+        <v>46086.69511574074</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6849,7 +6839,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46086.63890046296</v>
+        <v>46087.2936574074</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -7056,7 +7046,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46086.62041666666</v>
+        <v>46087.29035879629</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7313,7 +7303,7 @@
         <v>1</v>
       </c>
       <c r="N106" s="3" t="n">
-        <v>46086.64363425926</v>
+        <v>46086.71836805555</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -7451,7 +7441,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46086.64982638889</v>
+        <v>46087.28413194444</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7520,7 +7510,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46086.63175925926</v>
+        <v>46087.30832175926</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7589,7 +7579,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46086.64012731481</v>
+        <v>46087.31451388889</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7658,7 +7648,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46086.65050925926</v>
+        <v>46087.3106712963</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7727,7 +7717,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46086.64008101852</v>
+        <v>46087.30540509259</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7796,7 +7786,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46086.62225694444</v>
+        <v>46087.29465277777</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7862,7 +7852,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46086.62060185185</v>
+        <v>46087.30511574074</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7931,7 +7921,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46086.63061342593</v>
+        <v>46086.70570601852</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -8000,7 +7990,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46086.64890046296</v>
+        <v>46086.72510416667</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8066,7 +8056,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46086.64194444445</v>
+        <v>46086.68137731482</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8204,7 +8194,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46086.62503472222</v>
+        <v>46086.70379629629</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8273,7 +8263,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46086.64907407408</v>
+        <v>46086.84087962963</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8339,7 +8329,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46086.64605324074</v>
+        <v>46086.68203703704</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8408,7 +8398,7 @@
         <v>2</v>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46086.6240625</v>
+        <v>46086.85857638889</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8477,7 +8467,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46086.65256944444</v>
+        <v>46087.28799768518</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8546,7 +8536,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46086.62321759259</v>
+        <v>46087.29621527778</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8615,7 +8605,7 @@
         <v>2</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46086.61710648148</v>
+        <v>46086.77990740741</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8753,7 +8743,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46086.62005787037</v>
+        <v>46086.7009375</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8822,7 +8812,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46086.65203703703</v>
+        <v>46087.31390046296</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8891,7 +8881,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46086.64722222222</v>
+        <v>46086.71900462963</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -9088,7 +9078,7 @@
         <v>1</v>
       </c>
       <c r="N132" s="3" t="n">
-        <v>46086.63030092593</v>
+        <v>46086.78877314815</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -9152,7 +9142,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46086.62606481482</v>
+        <v>46086.85354166666</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9216,7 +9206,7 @@
         <v>1</v>
       </c>
       <c r="N134" s="3" t="n">
-        <v>46086.61770833333</v>
+        <v>46086.81866898148</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -9407,7 +9397,7 @@
         <v>1</v>
       </c>
       <c r="N137" s="3" t="n">
-        <v>46086.61796296296</v>
+        <v>46087.31840277778</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -9471,7 +9461,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46086.62364583334</v>
+        <v>46086.81694444444</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9535,7 +9525,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46086.62584490741</v>
+        <v>46086.81944444445</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9599,7 +9589,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46086.62326388889</v>
+        <v>46087.31744212963</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9663,7 +9653,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46086.64707175926</v>
+        <v>46086.8053125</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9727,7 +9717,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46086.63158564815</v>
+        <v>46087.32023148148</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9791,7 +9781,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46086.63318287037</v>
+        <v>46086.82635416667</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9855,7 +9845,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46086.62364583334</v>
+        <v>46086.81648148148</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9919,7 +9909,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46086.62401620371</v>
+        <v>46086.81909722222</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9983,7 +9973,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46086.64246527778</v>
+        <v>46086.79465277777</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10047,7 +10037,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46086.64841435185</v>
+        <v>46086.80592592592</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10111,7 +10101,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46086.61893518519</v>
+        <v>46086.81122685185</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10239,7 +10229,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46086.62425925926</v>
+        <v>46086.81674768519</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10303,7 +10293,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46086.63127314814</v>
+        <v>46086.81927083333</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10322,6 +10312,11 @@
           <t>OPERACAO 7.1</t>
         </is>
       </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>10.69.5.21</t>
+        </is>
+      </c>
       <c r="D152" t="n">
         <v>2018</v>
       </c>
@@ -10362,7 +10357,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46086.62116898148</v>
+        <v>46086.85846064815</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10426,7 +10421,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46086.62368055555</v>
+        <v>46087.31672453704</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10490,7 +10485,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46086.65115740741</v>
+        <v>46086.80916666667</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10554,7 +10549,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46086.65168981482</v>
+        <v>46087.30976851852</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10746,7 +10741,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46086.61965277778</v>
+        <v>46087.32032407408</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10810,7 +10805,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46086.61603009259</v>
+        <v>46086.81621527778</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10938,7 +10933,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46086.62626157407</v>
+        <v>46086.8278587963</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -11063,10 +11058,10 @@
         </is>
       </c>
       <c r="M163" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46086.63715277778</v>
+        <v>46087.28609953704</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11194,7 +11189,7 @@
         <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46086.62033564815</v>
+        <v>46086.71538194444</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11322,7 +11317,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46086.54707175926</v>
+        <v>46087.31327546296</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11383,10 +11378,10 @@
         </is>
       </c>
       <c r="M168" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46086.6363425926</v>
+        <v>46087.2921875</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11450,7 +11445,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46086.61810185185</v>
+        <v>46086.76868055556</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11578,7 +11573,7 @@
         <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46086.62856481481</v>
+        <v>46086.78569444444</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11639,10 +11634,10 @@
         </is>
       </c>
       <c r="M172" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46086.64271990741</v>
+        <v>46087.29045138889</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11770,7 +11765,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46086.64317129629</v>
+        <v>46087.29403935185</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11898,7 +11893,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46086.62203703704</v>
+        <v>46086.73244212963</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11962,7 +11957,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46086.61998842593</v>
+        <v>46087.31793981481</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12026,7 +12021,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46086.63445601852</v>
+        <v>46087.31475694444</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12090,7 +12085,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46086.6222337963</v>
+        <v>46086.818125</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12154,7 +12149,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46086.62366898148</v>
+        <v>46086.82105324074</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12479,7 +12474,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46086.63839120371</v>
+        <v>46086.83462962963</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12543,7 +12538,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46086.64640046296</v>
+        <v>46087.31510416666</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12607,7 +12602,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46086.62726851852</v>
+        <v>46087.3074537037</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12735,7 +12730,7 @@
         </is>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46086.63175925926</v>
+        <v>46086.82855324074</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12799,7 +12794,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46086.64098379629</v>
+        <v>46086.78903935185</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12863,7 +12858,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46086.61967592593</v>
+        <v>46087.31579861111</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12988,7 +12983,7 @@
         <v>2</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46086.58027777778</v>
+        <v>46086.72362268518</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13052,7 +13047,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46086.63425925926</v>
+        <v>46086.79143518519</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13116,7 +13111,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46086.64945601852</v>
+        <v>46086.80091435185</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13180,7 +13175,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46086.6284375</v>
+        <v>46086.86160879629</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13244,7 +13239,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46086.61712962963</v>
+        <v>46086.80951388889</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13308,7 +13303,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46086.62266203704</v>
+        <v>46086.81528935185</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13372,7 +13367,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46086.62221064815</v>
+        <v>46086.81688657407</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13433,7 +13428,7 @@
         </is>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46086.61435185185</v>
+        <v>46086.80949074074</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13497,7 +13492,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46086.64203703704</v>
+        <v>46086.79574074074</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13561,7 +13556,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46086.62202546297</v>
+        <v>46086.81133101852</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13625,7 +13620,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46086.63148148148</v>
+        <v>46086.7887962963</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13689,7 +13684,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46086.63934027778</v>
+        <v>46086.7956712963</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13817,7 +13812,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46086.63071759259</v>
+        <v>46087.31722222222</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13945,7 +13940,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46086.6215162037</v>
+        <v>46086.81269675926</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14073,7 +14068,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46086.6211574074</v>
+        <v>46086.81516203703</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14137,7 +14132,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46086.64259259259</v>
+        <v>46086.77622685185</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14201,7 +14196,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46086.64300925926</v>
+        <v>46086.80225694444</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14265,7 +14260,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46086.61386574074</v>
+        <v>46086.80946759259</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14329,7 +14324,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46086.64314814815</v>
+        <v>46086.8340625</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14393,7 +14388,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46086.64166666667</v>
+        <v>46086.79976851852</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14412,11 +14407,6 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
-      <c r="C216" t="inlineStr">
-        <is>
-          <t>10.69.5.85</t>
-        </is>
-      </c>
       <c r="D216" t="n">
         <v>2017</v>
       </c>
@@ -14457,7 +14447,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46086.64509259259</v>
+        <v>46086.80613425926</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14521,7 +14511,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46086.6295949074</v>
+        <v>46086.82789351852</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14585,7 +14575,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46086.64335648148</v>
+        <v>46086.80394675926</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14654,7 +14644,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46086.6346412037</v>
+        <v>46086.79326388889</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14718,7 +14708,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46086.61489583334</v>
+        <v>46086.80873842593</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14782,7 +14772,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46086.6412037037</v>
+        <v>46086.83113425926</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14846,7 +14836,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46085.79569444444</v>
+        <v>46086.82976851852</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14910,7 +14900,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46086.6403587963</v>
+        <v>46086.79446759259</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14974,7 +14964,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46086.6397337963</v>
+        <v>46087.31375</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15038,7 +15028,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46086.64273148148</v>
+        <v>46086.83831018519</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15102,7 +15092,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46086.61924768519</v>
+        <v>46086.80550925926</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15166,7 +15156,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46086.62142361111</v>
+        <v>46086.81878472222</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15230,7 +15220,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46086.63552083333</v>
+        <v>46086.79618055555</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15294,7 +15284,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46086.62216435185</v>
+        <v>46086.81694444444</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15358,7 +15348,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46086.62793981482</v>
+        <v>46086.82910879629</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15422,7 +15412,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46086.62101851852</v>
+        <v>46086.81612268519</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15486,7 +15476,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46086.63449074074</v>
+        <v>46086.82118055555</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15550,7 +15540,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46086.6346875</v>
+        <v>46086.83512731481</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15614,7 +15604,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46086.64796296296</v>
+        <v>46086.8021875</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15678,7 +15668,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46086.64922453704</v>
+        <v>46086.80993055556</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15742,7 +15732,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46086.63444444445</v>
+        <v>46086.82879629629</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15806,7 +15796,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46086.63460648148</v>
+        <v>46086.80788194444</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15870,7 +15860,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46086.63521990741</v>
+        <v>46086.83111111111</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15934,7 +15924,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46086.63064814815</v>
+        <v>46086.82240740741</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -15998,7 +15988,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46086.63387731482</v>
+        <v>46086.83282407407</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16062,7 +16052,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46086.64121527778</v>
+        <v>46086.82635416667</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16126,7 +16116,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46086.65333333334</v>
+        <v>46086.79998842593</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16185,7 +16175,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46086.34685185185</v>
+        <v>46087.20488425926</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16249,7 +16239,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46086.62921296297</v>
+        <v>46087.31642361111</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16313,7 +16303,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46086.65322916667</v>
+        <v>46087.31609953703</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16377,7 +16367,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46086.64903935185</v>
+        <v>46086.76759259259</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16441,7 +16431,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46086.62208333334</v>
+        <v>46087.31554398148</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16505,7 +16495,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46086.64417824074</v>
+        <v>46087.31538194444</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16564,7 +16554,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46086.63688657407</v>
+        <v>46087.31534722223</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16628,7 +16618,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46086.62525462963</v>
+        <v>46086.85931712963</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16692,7 +16682,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46086.65038194445</v>
+        <v>46087.31606481481</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16756,7 +16746,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46086.62689814815</v>
+        <v>46086.8238425926</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16814,7 +16804,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46086.64251157407</v>
+        <v>46086.79658564815</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16878,7 +16868,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46086.65269675926</v>
+        <v>46086.81641203703</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16942,7 +16932,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46086.62762731482</v>
+        <v>46086.82048611111</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -17006,7 +16996,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46086.64444444444</v>
+        <v>46086.795</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17070,7 +17060,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46086.64767361111</v>
+        <v>46086.80559027778</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17134,7 +17124,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46086.63461805556</v>
+        <v>46087.29366898148</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17262,7 +17252,7 @@
         <v>2</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46086.6280787037</v>
+        <v>46086.82716435185</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17326,7 +17316,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46086.65394675926</v>
+        <v>46086.80872685185</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17390,7 +17380,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46086.62688657407</v>
+        <v>46086.8212037037</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17454,7 +17444,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46086.64292824074</v>
+        <v>46086.79226851852</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17518,7 +17508,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46086.63168981481</v>
+        <v>46086.82268518519</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17582,7 +17572,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46086.63131944444</v>
+        <v>46086.86368055556</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17646,7 +17636,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46086.62418981481</v>
+        <v>46086.81373842592</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17710,7 +17700,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46086.63945601852</v>
+        <v>46086.78454861111</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17774,7 +17764,7 @@
         <v>1</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46086.64575231481</v>
+        <v>46086.80248842593</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17835,7 +17825,7 @@
         </is>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46086.63175925926</v>
+        <v>46087.29203703703</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17899,7 +17889,7 @@
         <v>1</v>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46086.59438657408</v>
+        <v>46086.83818287037</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -17963,7 +17953,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46086.62944444444</v>
+        <v>46086.81574074074</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -18088,7 +18078,7 @@
         </is>
       </c>
       <c r="N273" s="3" t="n">
-        <v>46086.62548611111</v>
+        <v>46087.30637731482</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -18336,7 +18326,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46086.57177083333</v>
+        <v>46087.31798611111</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18400,7 +18390,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46086.62020833333</v>
+        <v>46087.30451388889</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18587,7 +18577,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46086.65070601852</v>
+        <v>46087.31644675926</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18651,7 +18641,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46086.6178125</v>
+        <v>46086.85040509259</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18715,7 +18705,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46086.61560185185</v>
+        <v>46086.87230324074</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18779,7 +18769,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46086.64155092592</v>
+        <v>46086.80835648148</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18798,6 +18788,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>10.69.5.155</t>
+        </is>
+      </c>
       <c r="D285" t="n">
         <v>2019</v>
       </c>
@@ -18838,7 +18833,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46086.57170138889</v>
+        <v>46087.29601851852</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18902,7 +18897,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46086.64159722222</v>
+        <v>46086.80025462963</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18966,7 +18961,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46086.54943287037</v>
+        <v>46087.31859953704</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19030,7 +19025,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46086.64975694445</v>
+        <v>46086.83997685185</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19824,7 +19819,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46086.61756944445</v>
+        <v>46087.27961805555</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20940,7 +20935,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46086.63533564815</v>
+        <v>46087.32016203704</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21665,7 +21660,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46086.63486111111</v>
+        <v>46087.28293981482</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21729,7 +21724,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46086.61876157407</v>
+        <v>46087.28287037037</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21793,7 +21788,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46086.63197916667</v>
+        <v>46087.28326388889</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21857,7 +21852,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46086.62888888889</v>
+        <v>46087.3184375</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21918,10 +21913,10 @@
         </is>
       </c>
       <c r="M335" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46086.64973379629</v>
+        <v>46087.28369212963</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21985,7 +21980,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46086.63869212963</v>
+        <v>46087.28376157407</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22049,7 +22044,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46086.62677083333</v>
+        <v>46087.28310185186</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22113,7 +22108,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46086.62094907407</v>
+        <v>46087.3168287037</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -23381,7 +23376,7 @@
         <v>2</v>
       </c>
       <c r="N358" s="3" t="n">
-        <v>46086.649375</v>
+        <v>46086.84068287037</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -23758,7 +23753,7 @@
         <v>1</v>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46086.63197916667</v>
+        <v>46086.66841435185</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23824,7 +23819,7 @@
         </is>
       </c>
       <c r="N365" s="3" t="n">
-        <v>46086.65172453703</v>
+        <v>46087.31290509259</v>
       </c>
       <c r="O365" t="inlineStr">
         <is>
@@ -23950,7 +23945,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46086.64650462963</v>
+        <v>46086.68480324074</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -24080,7 +24075,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46086.61481481481</v>
+        <v>46086.73256944444</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24108,7 +24103,7 @@
         <v>2</v>
       </c>
       <c r="N370" s="3" t="n">
-        <v>46086.6280787037</v>
+        <v>46086.66436342592</v>
       </c>
       <c r="O370" t="inlineStr">
         <is>
@@ -24246,7 +24241,7 @@
         <v>1</v>
       </c>
       <c r="N372" s="3" t="n">
-        <v>46086.63756944444</v>
+        <v>46086.71232638889</v>
       </c>
       <c r="O372" t="inlineStr">
         <is>
@@ -24315,7 +24310,7 @@
         <v>1</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46086.65313657407</v>
+        <v>46086.69269675926</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24381,7 +24376,7 @@
         </is>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46086.64837962963</v>
+        <v>46087.3168287037</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24400,6 +24395,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>10.69.3.72</t>
+        </is>
+      </c>
       <c r="D375" t="n">
         <v>2025</v>
       </c>
@@ -24445,7 +24445,7 @@
         <v>1</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46086.61554398148</v>
+        <v>46086.81421296296</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24514,7 +24514,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46086.64222222222</v>
+        <v>46086.71847222222</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -24583,7 +24583,7 @@
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46086.65013888889</v>
+        <v>46087.29871527778</v>
       </c>
       <c r="O377" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-06 09:52:11.466459
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46087.3078125</v>
+        <v>46087.38416666666</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46086.71040509259</v>
+        <v>46087.3703587963</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46086.64232638889</v>
+        <v>46087.38111111111</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46087.2933912037</v>
+        <v>46087.36828703704</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46087.28476851852</v>
+        <v>46087.39678240741</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46087.30774305556</v>
+        <v>46087.38888888889</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46087.28724537037</v>
+        <v>46087.36465277777</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1702,7 +1702,7 @@
         <v>1</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>46087.28761574074</v>
+        <v>46087.36673611111</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -6504,7 +6504,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46086.7349537037</v>
+        <v>46087.40126157407</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6592,6 +6592,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>10.69.3.93</t>
+        </is>
+      </c>
       <c r="D96" t="n">
         <v>2025</v>
       </c>
@@ -6637,7 +6642,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46086.768125</v>
+        <v>46087.37475694445</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6701,7 +6706,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46086.68965277778</v>
+        <v>46087.37383101852</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6770,7 +6775,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46086.69511574074</v>
+        <v>46087.38763888889</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6839,7 +6844,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46087.2936574074</v>
+        <v>46087.40440972222</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -7046,7 +7051,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46087.29035879629</v>
+        <v>46087.36865740741</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7303,7 +7308,7 @@
         <v>1</v>
       </c>
       <c r="N106" s="3" t="n">
-        <v>46086.71836805555</v>
+        <v>46087.38842592593</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -7441,7 +7446,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46087.28413194444</v>
+        <v>46087.40461805555</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7510,7 +7515,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46087.30832175926</v>
+        <v>46087.38730324074</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7579,7 +7584,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46087.31451388889</v>
+        <v>46087.39628472222</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7648,7 +7653,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46087.3106712963</v>
+        <v>46087.39233796296</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7717,7 +7722,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46087.30540509259</v>
+        <v>46087.38491898148</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7786,7 +7791,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46087.29465277777</v>
+        <v>46087.37655092592</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7852,7 +7857,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46087.30511574074</v>
+        <v>46087.38372685185</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7921,7 +7926,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46086.70570601852</v>
+        <v>46087.37491898148</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7990,7 +7995,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46086.72510416667</v>
+        <v>46087.40100694444</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8056,7 +8061,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46086.68137731482</v>
+        <v>46087.37516203704</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8194,7 +8199,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46086.70379629629</v>
+        <v>46087.38467592592</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8329,7 +8334,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46086.68203703704</v>
+        <v>46087.37332175926</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8467,7 +8472,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46087.28799768518</v>
+        <v>46087.37135416667</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8536,7 +8541,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46087.29621527778</v>
+        <v>46087.37262731481</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8743,7 +8748,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46086.7009375</v>
+        <v>46087.38054398148</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8812,7 +8817,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46087.31390046296</v>
+        <v>46087.39179398148</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8881,7 +8886,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46086.71900462963</v>
+        <v>46087.36814814815</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -9078,7 +9083,7 @@
         <v>1</v>
       </c>
       <c r="N132" s="3" t="n">
-        <v>46086.78877314815</v>
+        <v>46087.37167824074</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -9142,7 +9147,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46086.85354166666</v>
+        <v>46087.3706712963</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9206,7 +9211,7 @@
         <v>1</v>
       </c>
       <c r="N134" s="3" t="n">
-        <v>46086.81866898148</v>
+        <v>46087.37144675926</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -9270,7 +9275,7 @@
         <v>1</v>
       </c>
       <c r="N135" s="3" t="n">
-        <v>46066.80446759259</v>
+        <v>46087.39694444444</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -9397,7 +9402,7 @@
         <v>1</v>
       </c>
       <c r="N137" s="3" t="n">
-        <v>46087.31840277778</v>
+        <v>46087.3990625</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -9461,7 +9466,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46086.81694444444</v>
+        <v>46087.39207175926</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9525,7 +9530,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46086.81944444445</v>
+        <v>46087.37490740741</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9589,7 +9594,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46087.31744212963</v>
+        <v>46087.39532407407</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9653,7 +9658,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46086.8053125</v>
+        <v>46087.37988425926</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9717,7 +9722,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46087.32023148148</v>
+        <v>46087.39503472222</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9781,7 +9786,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46086.82635416667</v>
+        <v>46087.37633101852</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9845,7 +9850,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46086.81648148148</v>
+        <v>46087.3777662037</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9909,7 +9914,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46086.81909722222</v>
+        <v>46087.40157407407</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9973,7 +9978,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46086.79465277777</v>
+        <v>46087.37185185185</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10037,7 +10042,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46086.80592592592</v>
+        <v>46087.37361111111</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10101,7 +10106,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46086.81122685185</v>
+        <v>46087.37643518519</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10229,7 +10234,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46086.81674768519</v>
+        <v>46087.39396990741</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10293,7 +10298,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46086.81927083333</v>
+        <v>46087.37798611111</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10312,11 +10317,6 @@
           <t>OPERACAO 7.1</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>10.69.5.21</t>
-        </is>
-      </c>
       <c r="D152" t="n">
         <v>2018</v>
       </c>
@@ -10357,7 +10357,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46086.85846064815</v>
+        <v>46087.39494212963</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10421,7 +10421,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46087.31672453704</v>
+        <v>46087.3918287037</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10485,7 +10485,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46086.80916666667</v>
+        <v>46087.39390046296</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10549,7 +10549,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46087.30976851852</v>
+        <v>46087.38438657407</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10613,7 +10613,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46086.57491898148</v>
+        <v>46087.373125</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10741,7 +10741,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46087.32032407408</v>
+        <v>46087.39358796296</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10805,7 +10805,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46086.81621527778</v>
+        <v>46087.36560185185</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10869,7 +10869,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46086.57278935185</v>
+        <v>46087.37944444444</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10933,7 +10933,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46086.8278587963</v>
+        <v>46087.37658564815</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -10994,10 +10994,10 @@
         </is>
       </c>
       <c r="M162" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46086.36907407407</v>
+        <v>46087.37243055556</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11058,10 +11058,10 @@
         </is>
       </c>
       <c r="M163" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46087.28609953704</v>
+        <v>46087.36447916667</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11125,7 +11125,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46086.60918981482</v>
+        <v>46087.40320601852</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11189,7 +11189,7 @@
         <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46086.71538194444</v>
+        <v>46087.39662037037</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11250,10 +11250,10 @@
         </is>
       </c>
       <c r="M166" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46086.60868055555</v>
+        <v>46087.36939814815</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11317,7 +11317,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46087.31327546296</v>
+        <v>46087.3908912037</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11378,10 +11378,10 @@
         </is>
       </c>
       <c r="M168" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46087.2921875</v>
+        <v>46087.37053240741</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11445,7 +11445,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46086.76868055556</v>
+        <v>46087.36565972222</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11573,7 +11573,7 @@
         <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46086.78569444444</v>
+        <v>46087.38239583333</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11634,10 +11634,10 @@
         </is>
       </c>
       <c r="M172" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46087.29045138889</v>
+        <v>46087.37079861111</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11701,7 +11701,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46086.56207175926</v>
+        <v>46087.38125</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11765,7 +11765,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46087.29403935185</v>
+        <v>46087.37368055555</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11957,7 +11957,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46087.31793981481</v>
+        <v>46087.39665509259</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12021,7 +12021,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46087.31475694444</v>
+        <v>46087.39631944444</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12538,7 +12538,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46087.31510416666</v>
+        <v>46087.39195601852</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12602,7 +12602,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46087.3074537037</v>
+        <v>46087.3853125</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12730,7 +12730,7 @@
         </is>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46086.82855324074</v>
+        <v>46087.38849537037</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12794,7 +12794,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46086.78903935185</v>
+        <v>46087.38729166667</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12858,7 +12858,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46087.31579861111</v>
+        <v>46087.38821759259</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12983,7 +12983,7 @@
         <v>2</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46086.72362268518</v>
+        <v>46087.3791550926</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13047,7 +13047,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46086.79143518519</v>
+        <v>46087.37640046296</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13111,7 +13111,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46086.80091435185</v>
+        <v>46087.38193287037</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13175,7 +13175,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46086.86160879629</v>
+        <v>46087.40444444444</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13239,7 +13239,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46086.80951388889</v>
+        <v>46087.36858796296</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13303,7 +13303,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46086.81528935185</v>
+        <v>46087.38021990741</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13367,7 +13367,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46086.81688657407</v>
+        <v>46087.4019675926</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13492,7 +13492,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46086.79574074074</v>
+        <v>46087.37445601852</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13556,7 +13556,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46086.81133101852</v>
+        <v>46087.3867824074</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13620,7 +13620,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46086.7887962963</v>
+        <v>46087.38120370371</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13684,7 +13684,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46086.7956712963</v>
+        <v>46087.38087962963</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13748,7 +13748,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46086.60002314814</v>
+        <v>46087.40298611111</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13812,7 +13812,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46087.31722222222</v>
+        <v>46087.39248842592</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13876,7 +13876,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46086.61907407407</v>
+        <v>46087.37259259259</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13940,7 +13940,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46086.81269675926</v>
+        <v>46087.40377314815</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14004,7 +14004,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46086.6364699074</v>
+        <v>46087.38534722223</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14068,7 +14068,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46086.81516203703</v>
+        <v>46087.40113425926</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14132,7 +14132,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46086.77622685185</v>
+        <v>46087.4027662037</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14196,7 +14196,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46086.80225694444</v>
+        <v>46087.38010416667</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14260,7 +14260,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46086.80946759259</v>
+        <v>46087.40365740741</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14388,7 +14388,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46086.79976851852</v>
+        <v>46087.3999537037</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14407,6 +14407,11 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>10.69.5.85</t>
+        </is>
+      </c>
       <c r="D216" t="n">
         <v>2017</v>
       </c>
@@ -14447,7 +14452,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46086.80613425926</v>
+        <v>46087.39967592592</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14511,7 +14516,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46086.82789351852</v>
+        <v>46087.36534722222</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14575,7 +14580,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46086.80394675926</v>
+        <v>46087.40401620371</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14644,7 +14649,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46086.79326388889</v>
+        <v>46087.36846064815</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14772,7 +14777,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46086.83113425926</v>
+        <v>46087.38479166666</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14964,7 +14969,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46087.31375</v>
+        <v>46087.39444444444</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15156,7 +15161,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46086.81878472222</v>
+        <v>46087.36356481481</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15220,7 +15225,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46086.79618055555</v>
+        <v>46087.38988425926</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15284,7 +15289,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46086.81694444444</v>
+        <v>46087.40280092593</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15348,7 +15353,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46086.82910879629</v>
+        <v>46087.36461805556</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15412,7 +15417,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46086.81612268519</v>
+        <v>46087.37738425926</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15476,7 +15481,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46086.82118055555</v>
+        <v>46087.37021990741</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15540,7 +15545,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46086.83512731481</v>
+        <v>46087.3702662037</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15604,7 +15609,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46086.8021875</v>
+        <v>46087.4028125</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15668,7 +15673,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46086.80993055556</v>
+        <v>46087.37836805556</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15796,7 +15801,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46086.80788194444</v>
+        <v>46087.39826388889</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15860,7 +15865,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46086.83111111111</v>
+        <v>46087.39295138889</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15924,7 +15929,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46086.82240740741</v>
+        <v>46087.38436342592</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -16052,7 +16057,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46086.82635416667</v>
+        <v>46087.40428240741</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16116,7 +16121,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46086.79998842593</v>
+        <v>46087.37997685185</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16239,7 +16244,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46087.31642361111</v>
+        <v>46087.39688657408</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16303,7 +16308,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46087.31609953703</v>
+        <v>46087.39993055556</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16367,7 +16372,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46086.76759259259</v>
+        <v>46087.3744212963</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16431,7 +16436,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46087.31554398148</v>
+        <v>46087.39680555555</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16495,7 +16500,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46087.31538194444</v>
+        <v>46087.38798611111</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16514,6 +16519,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>10.69.5.118</t>
+        </is>
+      </c>
       <c r="D249" t="n">
         <v>2017</v>
       </c>
@@ -16554,7 +16564,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46087.31534722223</v>
+        <v>46087.3945949074</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16682,7 +16692,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46087.31606481481</v>
+        <v>46087.39958333333</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16746,7 +16756,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46086.8238425926</v>
+        <v>46087.38344907408</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16804,7 +16814,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46086.79658564815</v>
+        <v>46087.36795138889</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16868,7 +16878,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46086.81641203703</v>
+        <v>46087.38969907408</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16932,7 +16942,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46086.82048611111</v>
+        <v>46087.37840277778</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -16996,7 +17006,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46086.795</v>
+        <v>46087.38759259259</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17060,7 +17070,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46086.80559027778</v>
+        <v>46087.38003472222</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17124,7 +17134,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46087.29366898148</v>
+        <v>46087.36954861111</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17188,7 +17198,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46086.60144675926</v>
+        <v>46087.36559027778</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17316,7 +17326,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46086.80872685185</v>
+        <v>46087.36996527778</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17380,7 +17390,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46086.8212037037</v>
+        <v>46087.37479166667</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17444,7 +17454,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46086.79226851852</v>
+        <v>46087.38585648148</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17508,7 +17518,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46086.82268518519</v>
+        <v>46087.39980324074</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17572,7 +17582,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46086.86368055556</v>
+        <v>46087.4041087963</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17636,7 +17646,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46086.81373842592</v>
+        <v>46087.37429398148</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17825,7 +17835,7 @@
         </is>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46087.29203703703</v>
+        <v>46087.37296296296</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17953,7 +17963,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46086.81574074074</v>
+        <v>46087.38063657407</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -18078,7 +18088,7 @@
         </is>
       </c>
       <c r="N273" s="3" t="n">
-        <v>46087.30637731482</v>
+        <v>46087.38224537037</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -18326,7 +18336,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46087.31798611111</v>
+        <v>46087.40185185185</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18390,7 +18400,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46087.30451388889</v>
+        <v>46087.38113425926</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18532,11 +18542,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C281" t="inlineStr">
-        <is>
-          <t>10.69.5.151</t>
-        </is>
-      </c>
       <c r="D281" t="n">
         <v>2017</v>
       </c>
@@ -18577,7 +18582,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46087.31644675926</v>
+        <v>46087.38846064815</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18641,7 +18646,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46086.85040509259</v>
+        <v>46087.3683912037</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18705,7 +18710,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46086.87230324074</v>
+        <v>46087.36471064815</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18769,7 +18774,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46086.80835648148</v>
+        <v>46087.37013888889</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18833,7 +18838,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46087.29601851852</v>
+        <v>46087.37693287037</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18897,7 +18902,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46086.80025462963</v>
+        <v>46087.3934375</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18961,7 +18966,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46087.31859953704</v>
+        <v>46087.39788194445</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19025,7 +19030,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46086.83997685185</v>
+        <v>46087.39915509259</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19819,7 +19824,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46087.27961805555</v>
+        <v>46087.39837962963</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20935,7 +20940,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46087.32016203704</v>
+        <v>46087.3949074074</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21660,7 +21665,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46087.28293981482</v>
+        <v>46087.40221064815</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21724,7 +21729,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46087.28287037037</v>
+        <v>46087.39665509259</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21788,7 +21793,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46087.28326388889</v>
+        <v>46087.40115740741</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21852,7 +21857,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46087.3184375</v>
+        <v>46087.39206018519</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21916,7 +21921,7 @@
         <v>1</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46087.28369212963</v>
+        <v>46087.39609953704</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21980,7 +21985,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46087.28376157407</v>
+        <v>46087.39773148148</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22044,7 +22049,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46087.28310185186</v>
+        <v>46087.39902777778</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22108,7 +22113,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46087.3168287037</v>
+        <v>46087.39799768518</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22361,7 +22366,7 @@
         </is>
       </c>
       <c r="N342" s="3" t="n">
-        <v>46086.58853009259</v>
+        <v>46087.37149305556</v>
       </c>
       <c r="O342" t="inlineStr">
         <is>
@@ -22617,7 +22622,7 @@
         <v>1</v>
       </c>
       <c r="N346" s="3" t="n">
-        <v>46086.58059027778</v>
+        <v>46087.37127314815</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -22681,7 +22686,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46086.57520833334</v>
+        <v>46087.37318287037</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22745,7 +22750,7 @@
         <v>1</v>
       </c>
       <c r="N348" s="3" t="n">
-        <v>46086.57438657407</v>
+        <v>46087.37241898148</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -22806,7 +22811,7 @@
         </is>
       </c>
       <c r="N349" s="3" t="n">
-        <v>46086.41283564815</v>
+        <v>46087.3720949074</v>
       </c>
       <c r="O349" t="inlineStr">
         <is>
@@ -22870,7 +22875,7 @@
         <v>1</v>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46086.57436342593</v>
+        <v>46087.37222222222</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -22934,7 +22939,7 @@
         <v>1</v>
       </c>
       <c r="N351" s="3" t="n">
-        <v>46086.57956018519</v>
+        <v>46087.3731712963</v>
       </c>
       <c r="O351" t="inlineStr">
         <is>
@@ -22995,7 +23000,7 @@
         </is>
       </c>
       <c r="N352" s="3" t="n">
-        <v>46086.37414351852</v>
+        <v>46087.37065972222</v>
       </c>
       <c r="O352" t="inlineStr">
         <is>
@@ -23120,7 +23125,7 @@
         <v>1</v>
       </c>
       <c r="N354" s="3" t="n">
-        <v>46086.5721875</v>
+        <v>46087.37048611111</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -23184,7 +23189,7 @@
         <v>1</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46086.56251157408</v>
+        <v>46087.37094907407</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23248,7 +23253,7 @@
         <v>1</v>
       </c>
       <c r="N356" s="3" t="n">
-        <v>46086.57060185185</v>
+        <v>46087.37065972222</v>
       </c>
       <c r="O356" t="inlineStr">
         <is>
@@ -23312,7 +23317,7 @@
         <v>1</v>
       </c>
       <c r="N357" s="3" t="n">
-        <v>46086.37550925926</v>
+        <v>46087.37417824074</v>
       </c>
       <c r="O357" t="inlineStr">
         <is>
@@ -23376,7 +23381,7 @@
         <v>2</v>
       </c>
       <c r="N358" s="3" t="n">
-        <v>46086.84068287037</v>
+        <v>46087.37418981481</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -23440,7 +23445,7 @@
         <v>2</v>
       </c>
       <c r="N359" s="3" t="n">
-        <v>46086.37553240741</v>
+        <v>46087.37303240741</v>
       </c>
       <c r="O359" t="inlineStr">
         <is>
@@ -23504,7 +23509,7 @@
         <v>1</v>
       </c>
       <c r="N360" s="3" t="n">
-        <v>46086.57539351852</v>
+        <v>46087.4027199074</v>
       </c>
       <c r="O360" t="inlineStr">
         <is>
@@ -23753,7 +23758,7 @@
         <v>1</v>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46086.66841435185</v>
+        <v>46087.38672453703</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23819,7 +23824,7 @@
         </is>
       </c>
       <c r="N365" s="3" t="n">
-        <v>46087.31290509259</v>
+        <v>46087.39091435185</v>
       </c>
       <c r="O365" t="inlineStr">
         <is>
@@ -23945,7 +23950,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46086.68480324074</v>
+        <v>46087.39736111111</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -24006,7 +24011,7 @@
         </is>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46086.58142361111</v>
+        <v>46087.37417824074</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24075,7 +24080,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46086.73256944444</v>
+        <v>46087.37121527778</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24376,7 +24381,7 @@
         </is>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46087.3168287037</v>
+        <v>46087.39609953704</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24395,11 +24400,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C375" t="inlineStr">
-        <is>
-          <t>10.69.3.72</t>
-        </is>
-      </c>
       <c r="D375" t="n">
         <v>2025</v>
       </c>
@@ -24514,7 +24514,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46086.71847222222</v>
+        <v>46087.37947916667</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -24583,7 +24583,7 @@
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46087.29871527778</v>
+        <v>46087.37711805556</v>
       </c>
       <c r="O377" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-06 11:52:06.517843
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46087.38416666666</v>
+        <v>46087.45799768518</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46086.63348379629</v>
+        <v>46087.48329861111</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46087.3703587963</v>
+        <v>46087.45241898148</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46087.38111111111</v>
+        <v>46087.45368055555</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46087.36828703704</v>
+        <v>46087.48252314814</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46087.39678240741</v>
+        <v>46087.47262731481</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46087.38888888889</v>
+        <v>46087.46513888889</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>46087.36465277777</v>
+        <v>46087.44525462963</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1702,7 +1702,7 @@
         <v>1</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>46087.36673611111</v>
+        <v>46087.48444444445</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1766,7 +1766,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46086.74211805555</v>
+        <v>46087.45587962963</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>46087.18209490741</v>
+        <v>46087.45627314815</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -1903,6 +1903,11 @@
           <t>AUDITORIO</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>10.69.3.150</t>
+        </is>
+      </c>
       <c r="D23" t="n">
         <v>2019</v>
       </c>
@@ -1943,7 +1948,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46087.14934027778</v>
+        <v>46087.48642361111</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -1999,7 +2004,7 @@
         </is>
       </c>
       <c r="N24" s="3" t="n">
-        <v>46087.15424768518</v>
+        <v>46087.48625</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2117,7 +2122,7 @@
         <v>1</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>46087.10924768518</v>
+        <v>46087.45443287037</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2178,7 +2183,7 @@
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46086.69706018519</v>
+        <v>46087.45379629629</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6504,7 +6509,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46087.40126157407</v>
+        <v>46087.47347222222</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6573,7 +6578,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46086.8169212963</v>
+        <v>46087.47755787037</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6592,11 +6597,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>10.69.3.93</t>
-        </is>
-      </c>
       <c r="D96" t="n">
         <v>2025</v>
       </c>
@@ -6642,7 +6642,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46087.37475694445</v>
+        <v>46087.45231481481</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6706,7 +6706,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46087.37383101852</v>
+        <v>46087.45188657408</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6775,7 +6775,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46087.38763888889</v>
+        <v>46087.46756944444</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6844,7 +6844,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46087.40440972222</v>
+        <v>46087.48425925926</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6913,7 +6913,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46086.64719907408</v>
+        <v>46087.48472222222</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -7051,7 +7051,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46087.36865740741</v>
+        <v>46087.44966435185</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7308,7 +7308,7 @@
         <v>1</v>
       </c>
       <c r="N106" s="3" t="n">
-        <v>46087.38842592593</v>
+        <v>46087.45986111111</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -7446,7 +7446,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46087.40461805555</v>
+        <v>46087.4796412037</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7515,7 +7515,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46087.38730324074</v>
+        <v>46087.46729166667</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7584,7 +7584,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46087.39628472222</v>
+        <v>46087.47387731481</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7653,7 +7653,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46087.39233796296</v>
+        <v>46087.47137731482</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7722,7 +7722,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46087.38491898148</v>
+        <v>46087.46002314815</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7791,7 +7791,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46087.37655092592</v>
+        <v>46087.45302083333</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7857,7 +7857,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46087.38372685185</v>
+        <v>46087.46206018519</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7926,7 +7926,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46087.37491898148</v>
+        <v>46087.45607638889</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7995,7 +7995,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46087.40100694444</v>
+        <v>46087.47831018519</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8061,7 +8061,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46087.37516203704</v>
+        <v>46087.4528587963</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8199,7 +8199,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46087.38467592592</v>
+        <v>46087.46324074074</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8268,7 +8268,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46086.84087962963</v>
+        <v>46087.45368055555</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8334,7 +8334,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46087.37332175926</v>
+        <v>46087.48605324074</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8403,7 +8403,7 @@
         <v>2</v>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46086.85857638889</v>
+        <v>46087.47637731482</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8472,7 +8472,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46087.37135416667</v>
+        <v>46087.45038194444</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8541,7 +8541,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46087.37262731481</v>
+        <v>46087.48722222223</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8610,7 +8610,7 @@
         <v>2</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46086.77990740741</v>
+        <v>46087.46297453704</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8748,7 +8748,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46087.38054398148</v>
+        <v>46087.45837962963</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8817,7 +8817,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46087.39179398148</v>
+        <v>46087.46973379629</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8886,7 +8886,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46087.36814814815</v>
+        <v>46087.48212962963</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -8905,6 +8905,11 @@
           <t>ADM/FIN</t>
         </is>
       </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>10.69.3.6</t>
+        </is>
+      </c>
       <c r="D130" t="n">
         <v>2025</v>
       </c>
@@ -8950,7 +8955,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46086.58516203704</v>
+        <v>46087.47216435185</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9083,7 +9088,7 @@
         <v>1</v>
       </c>
       <c r="N132" s="3" t="n">
-        <v>46087.37167824074</v>
+        <v>46087.48354166667</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -9147,7 +9152,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46087.3706712963</v>
+        <v>46087.44803240741</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9211,7 +9216,7 @@
         <v>1</v>
       </c>
       <c r="N134" s="3" t="n">
-        <v>46087.37144675926</v>
+        <v>46087.48774305556</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -9275,7 +9280,7 @@
         <v>1</v>
       </c>
       <c r="N135" s="3" t="n">
-        <v>46087.39694444444</v>
+        <v>46087.47877314815</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -9402,7 +9407,7 @@
         <v>1</v>
       </c>
       <c r="N137" s="3" t="n">
-        <v>46087.3990625</v>
+        <v>46087.4802199074</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -9466,7 +9471,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46087.39207175926</v>
+        <v>46087.46758101852</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9530,7 +9535,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46087.37490740741</v>
+        <v>46087.45377314815</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9594,7 +9599,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46087.39532407407</v>
+        <v>46087.47224537037</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9658,7 +9663,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46087.37988425926</v>
+        <v>46087.46145833333</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9722,7 +9727,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46087.39503472222</v>
+        <v>46087.47243055556</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9786,7 +9791,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46087.37633101852</v>
+        <v>46087.45224537037</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9850,7 +9855,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46087.3777662037</v>
+        <v>46087.41553240741</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9914,7 +9919,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46087.40157407407</v>
+        <v>46087.47785879629</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9978,7 +9983,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46087.37185185185</v>
+        <v>46087.45438657407</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10042,7 +10047,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46087.37361111111</v>
+        <v>46087.45253472222</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10106,7 +10111,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46087.37643518519</v>
+        <v>46087.45271990741</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10234,7 +10239,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46087.39396990741</v>
+        <v>46087.47362268518</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10298,7 +10303,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46087.37798611111</v>
+        <v>46087.45533564815</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10357,7 +10362,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46087.39494212963</v>
+        <v>46087.45875</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10421,7 +10426,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46087.3918287037</v>
+        <v>46087.47096064815</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10485,7 +10490,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46087.39390046296</v>
+        <v>46087.46792824074</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10549,7 +10554,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46087.38438657407</v>
+        <v>46087.47822916666</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10613,7 +10618,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46087.373125</v>
+        <v>46087.45247685185</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10741,7 +10746,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46087.39358796296</v>
+        <v>46087.46831018518</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10805,7 +10810,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46087.36560185185</v>
+        <v>46087.44696759259</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10869,7 +10874,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46087.37944444444</v>
+        <v>46087.45425925926</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10933,7 +10938,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46087.37658564815</v>
+        <v>46087.45017361111</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -10997,7 +11002,7 @@
         <v>1</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46087.37243055556</v>
+        <v>46087.44815972223</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11061,7 +11066,7 @@
         <v>2</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46087.36447916667</v>
+        <v>46087.47940972223</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11125,7 +11130,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46087.40320601852</v>
+        <v>46087.47756944445</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11189,7 +11194,7 @@
         <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46087.39662037037</v>
+        <v>46087.47805555556</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11250,10 +11255,10 @@
         </is>
       </c>
       <c r="M166" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46087.36939814815</v>
+        <v>46087.4807175926</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11317,7 +11322,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46087.3908912037</v>
+        <v>46087.47084490741</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11381,7 +11386,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46087.37053240741</v>
+        <v>46087.48744212963</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11445,7 +11450,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46087.36565972222</v>
+        <v>46087.47979166666</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11573,7 +11578,7 @@
         <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46087.38239583333</v>
+        <v>46087.46229166666</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11637,7 +11642,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46087.37079861111</v>
+        <v>46087.48637731482</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11701,7 +11706,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46087.38125</v>
+        <v>46087.46260416666</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11765,7 +11770,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46087.37368055555</v>
+        <v>46087.44780092593</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11829,7 +11834,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46086.64773148148</v>
+        <v>46087.46905092592</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11957,7 +11962,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46087.39665509259</v>
+        <v>46087.47461805555</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12021,7 +12026,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46087.39631944444</v>
+        <v>46087.47519675926</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12538,7 +12543,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46087.39195601852</v>
+        <v>46087.45268518518</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12602,7 +12607,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46087.3853125</v>
+        <v>46087.45751157407</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12730,7 +12735,7 @@
         </is>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46087.38849537037</v>
+        <v>46087.46827546296</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12794,7 +12799,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46087.38729166667</v>
+        <v>46087.46350694444</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12858,7 +12863,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46087.38821759259</v>
+        <v>46087.4705787037</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12983,7 +12988,7 @@
         <v>2</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46087.3791550926</v>
+        <v>46087.45716435185</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13047,7 +13052,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46087.37640046296</v>
+        <v>46087.45077546296</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13111,7 +13116,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46087.38193287037</v>
+        <v>46087.4878125</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13175,7 +13180,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46087.40444444444</v>
+        <v>46087.48210648148</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13239,7 +13244,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46087.36858796296</v>
+        <v>46087.48163194444</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13303,7 +13308,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46087.38021990741</v>
+        <v>46087.48648148148</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13367,7 +13372,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46087.4019675926</v>
+        <v>46087.47016203704</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13492,7 +13497,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46087.37445601852</v>
+        <v>46087.4496412037</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13556,7 +13561,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46087.3867824074</v>
+        <v>46087.46546296297</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13620,7 +13625,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46087.38120370371</v>
+        <v>46087.45666666667</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13684,7 +13689,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46087.38087962963</v>
+        <v>46087.45648148148</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13748,7 +13753,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46087.40298611111</v>
+        <v>46087.48086805556</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13812,7 +13817,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46087.39248842592</v>
+        <v>46087.48550925926</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13876,7 +13881,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46087.37259259259</v>
+        <v>46087.45395833333</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13940,7 +13945,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46087.40377314815</v>
+        <v>46087.48290509259</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14004,7 +14009,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46087.38534722223</v>
+        <v>46087.46211805556</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14068,7 +14073,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46087.40113425926</v>
+        <v>46087.48390046296</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14132,7 +14137,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46087.4027662037</v>
+        <v>46087.48208333334</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14196,7 +14201,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46087.38010416667</v>
+        <v>46087.4530787037</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14260,7 +14265,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46087.40365740741</v>
+        <v>46087.4825462963</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14388,7 +14393,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46087.3999537037</v>
+        <v>46087.48193287037</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14452,7 +14457,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46087.39967592592</v>
+        <v>46087.47913194444</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14516,7 +14521,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46087.36534722222</v>
+        <v>46087.48678240741</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14580,7 +14585,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46087.40401620371</v>
+        <v>46087.48152777777</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14649,7 +14654,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46087.36846064815</v>
+        <v>46087.48765046296</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14713,7 +14718,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46086.80873842593</v>
+        <v>46087.45744212963</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14777,7 +14782,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46087.38479166666</v>
+        <v>46087.46273148148</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14969,7 +14974,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46087.39444444444</v>
+        <v>46087.48540509259</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15161,7 +15166,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46087.36356481481</v>
+        <v>46087.48486111111</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15225,7 +15230,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46087.38988425926</v>
+        <v>46087.46871527778</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15289,7 +15294,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46087.40280092593</v>
+        <v>46087.46708333334</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15353,7 +15358,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46087.36461805556</v>
+        <v>46087.45144675926</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15417,7 +15422,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46087.37738425926</v>
+        <v>46087.48063657407</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15481,7 +15486,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46087.37021990741</v>
+        <v>46087.47898148148</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15545,7 +15550,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46087.3702662037</v>
+        <v>46087.48590277778</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15609,7 +15614,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46087.4028125</v>
+        <v>46087.486875</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15673,7 +15678,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46087.37836805556</v>
+        <v>46087.45797453704</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15801,7 +15806,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46087.39826388889</v>
+        <v>46087.47359953704</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15865,7 +15870,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46087.39295138889</v>
+        <v>46087.46537037037</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15929,7 +15934,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46087.38436342592</v>
+        <v>46087.47836805556</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -16057,7 +16062,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46087.40428240741</v>
+        <v>46087.47741898148</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16121,7 +16126,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46087.37997685185</v>
+        <v>46087.45679398148</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16244,7 +16249,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46087.39688657408</v>
+        <v>46087.47643518518</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16308,7 +16313,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46087.39993055556</v>
+        <v>46087.48197916667</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16372,7 +16377,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46087.3744212963</v>
+        <v>46087.4846875</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16436,7 +16441,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46087.39680555555</v>
+        <v>46087.4733449074</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16500,7 +16505,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46087.38798611111</v>
+        <v>46087.48078703704</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16564,7 +16569,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46087.3945949074</v>
+        <v>46087.47663194445</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16692,7 +16697,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46087.39958333333</v>
+        <v>46087.47820601852</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16756,7 +16761,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46087.38344907408</v>
+        <v>46087.449375</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16814,7 +16819,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46087.36795138889</v>
+        <v>46087.48112268518</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16878,7 +16883,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46087.38969907408</v>
+        <v>46087.48527777778</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16942,7 +16947,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46087.37840277778</v>
+        <v>46087.48299768518</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -17006,7 +17011,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46087.38759259259</v>
+        <v>46087.46489583333</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17070,7 +17075,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46087.38003472222</v>
+        <v>46087.45498842592</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17134,7 +17139,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46087.36954861111</v>
+        <v>46087.48324074074</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17198,7 +17203,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46087.36559027778</v>
+        <v>46087.48210648148</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17326,7 +17331,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46087.36996527778</v>
+        <v>46087.44722222222</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17390,7 +17395,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46087.37479166667</v>
+        <v>46087.48653935185</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17454,7 +17459,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46087.38585648148</v>
+        <v>46087.48324074074</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17518,7 +17523,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46087.39980324074</v>
+        <v>46087.48200231481</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17582,7 +17587,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46087.4041087963</v>
+        <v>46087.48315972222</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17646,7 +17651,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46087.37429398148</v>
+        <v>46087.45196759259</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17710,7 +17715,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46086.78454861111</v>
+        <v>46087.41716435185</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17774,7 +17779,7 @@
         <v>1</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46086.80248842593</v>
+        <v>46087.46677083334</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17835,7 +17840,7 @@
         </is>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46087.37296296296</v>
+        <v>46087.45491898148</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17899,7 +17904,7 @@
         <v>1</v>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46086.83818287037</v>
+        <v>46087.41416666667</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -17963,7 +17968,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46087.38063657407</v>
+        <v>46087.4597337963</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -18088,7 +18093,7 @@
         </is>
       </c>
       <c r="N273" s="3" t="n">
-        <v>46087.38224537037</v>
+        <v>46087.45804398148</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -18336,7 +18341,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46087.40185185185</v>
+        <v>46087.48677083333</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18400,7 +18405,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46087.38113425926</v>
+        <v>46087.46178240741</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18582,7 +18587,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46087.38846064815</v>
+        <v>46087.46670138889</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18646,7 +18651,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46087.3683912037</v>
+        <v>46087.44738425926</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18710,7 +18715,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46087.36471064815</v>
+        <v>46087.48222222222</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18774,7 +18779,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46087.37013888889</v>
+        <v>46087.48733796296</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18793,11 +18798,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C285" t="inlineStr">
-        <is>
-          <t>10.69.5.155</t>
-        </is>
-      </c>
       <c r="D285" t="n">
         <v>2019</v>
       </c>
@@ -18838,7 +18838,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46087.37693287037</v>
+        <v>46087.45231481481</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18902,7 +18902,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46087.3934375</v>
+        <v>46087.48758101852</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18966,7 +18966,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46087.39788194445</v>
+        <v>46087.48039351852</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19030,7 +19030,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46087.39915509259</v>
+        <v>46087.47928240741</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19824,7 +19824,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46087.39837962963</v>
+        <v>46087.47792824074</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20940,7 +20940,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46087.3949074074</v>
+        <v>46087.47034722222</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21665,7 +21665,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46087.40221064815</v>
+        <v>46087.48390046296</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21729,7 +21729,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46087.39665509259</v>
+        <v>46087.47391203704</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21793,7 +21793,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46087.40115740741</v>
+        <v>46087.48387731481</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21857,7 +21857,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46087.39206018519</v>
+        <v>46087.46649305556</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21921,7 +21921,7 @@
         <v>1</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46087.39609953704</v>
+        <v>46087.46965277778</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21985,7 +21985,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46087.39773148148</v>
+        <v>46087.47412037037</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22049,7 +22049,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46087.39902777778</v>
+        <v>46087.46782407408</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22113,7 +22113,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46087.39799768518</v>
+        <v>46087.47702546296</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22622,7 +22622,7 @@
         <v>1</v>
       </c>
       <c r="N346" s="3" t="n">
-        <v>46087.37127314815</v>
+        <v>46087.48049768519</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -22686,7 +22686,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46087.37318287037</v>
+        <v>46087.45586805556</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22750,7 +22750,7 @@
         <v>1</v>
       </c>
       <c r="N348" s="3" t="n">
-        <v>46087.37241898148</v>
+        <v>46087.45260416667</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -22875,7 +22875,7 @@
         <v>1</v>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46087.37222222222</v>
+        <v>46087.45472222222</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -22939,7 +22939,7 @@
         <v>1</v>
       </c>
       <c r="N351" s="3" t="n">
-        <v>46087.3731712963</v>
+        <v>46087.48706018519</v>
       </c>
       <c r="O351" t="inlineStr">
         <is>
@@ -23125,7 +23125,7 @@
         <v>1</v>
       </c>
       <c r="N354" s="3" t="n">
-        <v>46087.37048611111</v>
+        <v>46087.48429398148</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -23189,7 +23189,7 @@
         <v>1</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46087.37094907407</v>
+        <v>46087.48467592592</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23253,7 +23253,7 @@
         <v>1</v>
       </c>
       <c r="N356" s="3" t="n">
-        <v>46087.37065972222</v>
+        <v>46087.48543981482</v>
       </c>
       <c r="O356" t="inlineStr">
         <is>
@@ -23381,7 +23381,7 @@
         <v>2</v>
       </c>
       <c r="N358" s="3" t="n">
-        <v>46087.37418981481</v>
+        <v>46087.45118055555</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -23445,7 +23445,7 @@
         <v>2</v>
       </c>
       <c r="N359" s="3" t="n">
-        <v>46087.37303240741</v>
+        <v>46087.45547453704</v>
       </c>
       <c r="O359" t="inlineStr">
         <is>
@@ -23509,7 +23509,7 @@
         <v>1</v>
       </c>
       <c r="N360" s="3" t="n">
-        <v>46087.4027199074</v>
+        <v>46087.47716435185</v>
       </c>
       <c r="O360" t="inlineStr">
         <is>
@@ -23758,7 +23758,7 @@
         <v>1</v>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46087.38672453703</v>
+        <v>46087.46706018518</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23824,7 +23824,7 @@
         </is>
       </c>
       <c r="N365" s="3" t="n">
-        <v>46087.39091435185</v>
+        <v>46087.46895833333</v>
       </c>
       <c r="O365" t="inlineStr">
         <is>
@@ -23950,7 +23950,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46087.39736111111</v>
+        <v>46087.47791666666</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -24080,7 +24080,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46087.37121527778</v>
+        <v>46087.48518518519</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24108,7 +24108,7 @@
         <v>2</v>
       </c>
       <c r="N370" s="3" t="n">
-        <v>46086.66436342592</v>
+        <v>46087.48193287037</v>
       </c>
       <c r="O370" t="inlineStr">
         <is>
@@ -24381,7 +24381,7 @@
         </is>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46087.39609953704</v>
+        <v>46087.47168981482</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24514,7 +24514,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46087.37947916667</v>
+        <v>46087.454375</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -24583,7 +24583,7 @@
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46087.37711805556</v>
+        <v>46087.4569675926</v>
       </c>
       <c r="O377" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-06 13:52:08.762284
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46087.45799768518</v>
+        <v>46087.54032407407</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46087.48329861111</v>
+        <v>46087.55841435185</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46087.45241898148</v>
+        <v>46087.56822916667</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46087.45368055555</v>
+        <v>46087.56357638889</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -870,7 +870,7 @@
         <v>1</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>46086.72121527778</v>
+        <v>46087.55134259259</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
         <v>1</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>46080.88524305556</v>
+        <v>46087.5434375</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1003,7 +1003,7 @@
         <v>1</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>46084.57743055555</v>
+        <v>46087.54685185185</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1067,7 +1067,7 @@
         <v>1</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>46078.72996527778</v>
+        <v>46087.54733796296</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46087.48252314814</v>
+        <v>46087.56087962963</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
         <v>1</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>46084.70671296296</v>
+        <v>46087.54518518518</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1382,7 +1382,7 @@
         <v>2</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>46084.71085648148</v>
+        <v>46087.5434837963</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46087.47262731481</v>
+        <v>46087.55569444445</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1510,7 +1510,7 @@
         <v>2</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>46084.72297453704</v>
+        <v>46087.54890046296</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46087.46513888889</v>
+        <v>46087.54075231482</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1702,7 +1702,7 @@
         <v>1</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>46087.48444444445</v>
+        <v>46087.56180555555</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1766,7 +1766,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46087.45587962963</v>
+        <v>46087.53493055556</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>46087.45627314815</v>
+        <v>46087.50902777778</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -1903,11 +1903,6 @@
           <t>AUDITORIO</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>10.69.3.150</t>
-        </is>
-      </c>
       <c r="D23" t="n">
         <v>2019</v>
       </c>
@@ -2004,7 +1999,7 @@
         </is>
       </c>
       <c r="N24" s="3" t="n">
-        <v>46087.48625</v>
+        <v>46087.52459490741</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2063,7 +2058,7 @@
         <v>1</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>46064.45631944444</v>
+        <v>46087.50386574074</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2122,7 +2117,7 @@
         <v>1</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>46087.45443287037</v>
+        <v>46087.53324074074</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2183,7 +2178,7 @@
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46087.45379629629</v>
+        <v>46087.5633912037</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6509,7 +6504,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46087.47347222222</v>
+        <v>46087.54825231482</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6578,7 +6573,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46087.47755787037</v>
+        <v>46087.55947916667</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6642,7 +6637,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46087.45231481481</v>
+        <v>46087.53138888889</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6706,7 +6701,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46087.45188657408</v>
+        <v>46087.56637731481</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6775,7 +6770,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46087.46756944444</v>
+        <v>46087.54103009259</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6844,7 +6839,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46087.48425925926</v>
+        <v>46087.56230324074</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6913,7 +6908,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46087.48472222222</v>
+        <v>46087.55622685186</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -7051,7 +7046,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46087.44966435185</v>
+        <v>46087.56797453704</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7308,7 +7303,7 @@
         <v>1</v>
       </c>
       <c r="N106" s="3" t="n">
-        <v>46087.45986111111</v>
+        <v>46087.53865740741</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -7446,7 +7441,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46087.4796412037</v>
+        <v>46087.55811342593</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7515,7 +7510,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46087.46729166667</v>
+        <v>46087.54768518519</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7584,7 +7579,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46087.47387731481</v>
+        <v>46087.55221064815</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7653,7 +7648,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46087.47137731482</v>
+        <v>46087.54953703703</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7722,7 +7717,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46087.46002314815</v>
+        <v>46087.53820601852</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7791,7 +7786,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46087.45302083333</v>
+        <v>46087.56773148148</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7857,7 +7852,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46087.46206018519</v>
+        <v>46087.53451388889</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7926,7 +7921,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46087.45607638889</v>
+        <v>46087.57107638889</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7995,7 +7990,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46087.47831018519</v>
+        <v>46087.57114583333</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8061,7 +8056,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46087.4528587963</v>
+        <v>46087.56746527777</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8199,7 +8194,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46087.46324074074</v>
+        <v>46087.5427662037</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8268,7 +8263,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46087.45368055555</v>
+        <v>46087.56983796296</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8334,7 +8329,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46087.48605324074</v>
+        <v>46087.56180555555</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8403,7 +8398,7 @@
         <v>2</v>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46087.47637731482</v>
+        <v>46087.55480324074</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8472,7 +8467,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46087.45038194444</v>
+        <v>46087.56865740741</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8541,7 +8536,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46087.48722222223</v>
+        <v>46087.5666087963</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8610,7 +8605,7 @@
         <v>2</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46087.46297453704</v>
+        <v>46087.53707175926</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8748,7 +8743,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46087.45837962963</v>
+        <v>46087.53354166666</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8817,7 +8812,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46087.46973379629</v>
+        <v>46087.54670138889</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8886,7 +8881,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46087.48212962963</v>
+        <v>46087.55524305555</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -8905,11 +8900,6 @@
           <t>ADM/FIN</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>10.69.3.6</t>
-        </is>
-      </c>
       <c r="D130" t="n">
         <v>2025</v>
       </c>
@@ -8955,7 +8945,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46087.47216435185</v>
+        <v>46087.55150462963</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9152,7 +9142,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46087.44803240741</v>
+        <v>46087.56673611111</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9216,7 +9206,7 @@
         <v>1</v>
       </c>
       <c r="N134" s="3" t="n">
-        <v>46087.48774305556</v>
+        <v>46087.56570601852</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -9280,7 +9270,7 @@
         <v>1</v>
       </c>
       <c r="N135" s="3" t="n">
-        <v>46087.47877314815</v>
+        <v>46087.5559375</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -9407,7 +9397,7 @@
         <v>1</v>
       </c>
       <c r="N137" s="3" t="n">
-        <v>46087.4802199074</v>
+        <v>46087.55927083334</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -9471,7 +9461,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46087.46758101852</v>
+        <v>46087.55134259259</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9599,7 +9589,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46087.47224537037</v>
+        <v>46087.55278935185</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9663,7 +9653,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46087.46145833333</v>
+        <v>46087.54049768519</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9727,7 +9717,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46087.47243055556</v>
+        <v>46087.55488425926</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9791,7 +9781,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46087.45224537037</v>
+        <v>46087.53498842593</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9919,7 +9909,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46087.47785879629</v>
+        <v>46087.55883101852</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9983,7 +9973,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46087.45438657407</v>
+        <v>46087.53259259259</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10047,7 +10037,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46087.45253472222</v>
+        <v>46087.5671875</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10111,7 +10101,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46087.45271990741</v>
+        <v>46087.53075231481</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10239,7 +10229,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46087.47362268518</v>
+        <v>46087.54649305555</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10303,7 +10293,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46087.45533564815</v>
+        <v>46087.5712037037</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10322,6 +10312,11 @@
           <t>OPERACAO 7.1</t>
         </is>
       </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>10.69.5.21</t>
+        </is>
+      </c>
       <c r="D152" t="n">
         <v>2018</v>
       </c>
@@ -10362,7 +10357,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46087.45875</v>
+        <v>46087.57123842592</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10426,7 +10421,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46087.47096064815</v>
+        <v>46087.54515046296</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10490,7 +10485,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46087.46792824074</v>
+        <v>46087.54748842592</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10554,7 +10549,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46087.47822916666</v>
+        <v>46087.5603587963</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10618,7 +10613,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46087.45247685185</v>
+        <v>46087.53288194445</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10682,7 +10677,7 @@
         <v>1</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>46085.6025</v>
+        <v>46087.56981481481</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -10746,7 +10741,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46087.46831018518</v>
+        <v>46087.54121527778</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10810,7 +10805,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46087.44696759259</v>
+        <v>46087.56519675926</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10874,7 +10869,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46087.45425925926</v>
+        <v>46087.53649305556</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10938,7 +10933,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46087.45017361111</v>
+        <v>46087.5312037037</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -11002,7 +10997,7 @@
         <v>1</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46087.44815972223</v>
+        <v>46087.56321759259</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11063,10 +11058,10 @@
         </is>
       </c>
       <c r="M163" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46087.47940972223</v>
+        <v>46087.55513888889</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11130,7 +11125,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46087.47756944445</v>
+        <v>46087.55186342593</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11194,7 +11189,7 @@
         <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46087.47805555556</v>
+        <v>46087.5578125</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11258,7 +11253,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46087.4807175926</v>
+        <v>46087.55488425926</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11322,7 +11317,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46087.47084490741</v>
+        <v>46087.55251157407</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11386,7 +11381,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46087.48744212963</v>
+        <v>46087.56015046296</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11450,7 +11445,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46087.47979166666</v>
+        <v>46087.5521875</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11514,7 +11509,7 @@
         <v>1</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46086.55554398148</v>
+        <v>46087.54773148148</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11578,7 +11573,7 @@
         <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46087.46229166666</v>
+        <v>46087.53928240741</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11642,7 +11637,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46087.48637731482</v>
+        <v>46087.56465277778</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11706,7 +11701,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46087.46260416666</v>
+        <v>46087.54109953704</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11770,7 +11765,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46087.44780092593</v>
+        <v>46087.56695601852</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11834,7 +11829,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46087.46905092592</v>
+        <v>46087.5399537037</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11898,7 +11893,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46086.73244212963</v>
+        <v>46087.54305555556</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11962,7 +11957,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46087.47461805555</v>
+        <v>46087.55306712963</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12026,7 +12021,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46087.47519675926</v>
+        <v>46087.55358796296</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12543,7 +12538,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46087.45268518518</v>
+        <v>46087.568125</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12607,7 +12602,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46087.45751157407</v>
+        <v>46087.53423611111</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12735,7 +12730,7 @@
         </is>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46087.46827546296</v>
+        <v>46087.55012731482</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12799,7 +12794,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46087.46350694444</v>
+        <v>46087.56959490741</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12863,7 +12858,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46087.4705787037</v>
+        <v>46087.54961805556</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12988,7 +12983,7 @@
         <v>2</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46087.45716435185</v>
+        <v>46087.56983796296</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13052,7 +13047,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46087.45077546296</v>
+        <v>46087.56893518518</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13116,7 +13111,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46087.4878125</v>
+        <v>46087.52959490741</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13180,7 +13175,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46087.48210648148</v>
+        <v>46087.55809027778</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13244,7 +13239,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46087.48163194444</v>
+        <v>46087.56074074074</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13308,7 +13303,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46087.48648148148</v>
+        <v>46087.55924768518</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13372,7 +13367,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46087.47016203704</v>
+        <v>46087.55362268518</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13497,7 +13492,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46087.4496412037</v>
+        <v>46087.56510416666</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13561,7 +13556,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46087.46546296297</v>
+        <v>46087.5436574074</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13625,7 +13620,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46087.45666666667</v>
+        <v>46087.57099537037</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13689,7 +13684,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46087.45648148148</v>
+        <v>46087.57100694445</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13753,7 +13748,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46087.48086805556</v>
+        <v>46087.5587037037</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13817,7 +13812,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46087.48550925926</v>
+        <v>46087.56194444445</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13881,7 +13876,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46087.45395833333</v>
+        <v>46087.56842592593</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13945,7 +13940,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46087.48290509259</v>
+        <v>46087.56019675926</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14009,7 +14004,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46087.46211805556</v>
+        <v>46087.55184027777</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14073,7 +14068,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46087.48390046296</v>
+        <v>46087.564375</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14137,7 +14132,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46087.48208333334</v>
+        <v>46087.55902777778</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14201,7 +14196,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46087.4530787037</v>
+        <v>46087.56956018518</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14265,7 +14260,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46087.4825462963</v>
+        <v>46087.5558912037</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14393,7 +14388,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46087.48193287037</v>
+        <v>46087.55730324074</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14412,11 +14407,6 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
-      <c r="C216" t="inlineStr">
-        <is>
-          <t>10.69.5.85</t>
-        </is>
-      </c>
       <c r="D216" t="n">
         <v>2017</v>
       </c>
@@ -14457,7 +14447,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46087.47913194444</v>
+        <v>46087.55655092592</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14521,7 +14511,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46087.48678240741</v>
+        <v>46087.57010416667</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14585,7 +14575,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46087.48152777777</v>
+        <v>46087.5547337963</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14654,7 +14644,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46087.48765046296</v>
+        <v>46087.56490740741</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14782,7 +14772,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46087.46273148148</v>
+        <v>46087.53725694444</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14974,7 +14964,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46087.48540509259</v>
+        <v>46087.56344907408</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15166,7 +15156,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46087.48486111111</v>
+        <v>46087.56170138889</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15230,7 +15220,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46087.46871527778</v>
+        <v>46087.55</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15294,7 +15284,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46087.46708333334</v>
+        <v>46087.54670138889</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15358,7 +15348,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46087.45144675926</v>
+        <v>46087.55930555556</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15422,7 +15412,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46087.48063657407</v>
+        <v>46087.56121527778</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15486,7 +15476,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46087.47898148148</v>
+        <v>46087.55950231481</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15550,7 +15540,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46087.48590277778</v>
+        <v>46087.53743055555</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15614,7 +15604,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46087.486875</v>
+        <v>46087.56737268518</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15678,7 +15668,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46087.45797453704</v>
+        <v>46087.53586805556</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15806,7 +15796,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46087.47359953704</v>
+        <v>46087.55296296296</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15870,7 +15860,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46087.46537037037</v>
+        <v>46087.54222222222</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15934,7 +15924,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46087.47836805556</v>
+        <v>46087.55726851852</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -16062,7 +16052,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46087.47741898148</v>
+        <v>46087.55548611111</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16126,7 +16116,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46087.45679398148</v>
+        <v>46087.53032407408</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16249,7 +16239,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46087.47643518518</v>
+        <v>46087.5534375</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16313,7 +16303,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46087.48197916667</v>
+        <v>46087.55665509259</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16377,7 +16367,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46087.4846875</v>
+        <v>46087.55700231482</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16441,7 +16431,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46087.4733449074</v>
+        <v>46087.54835648148</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16505,7 +16495,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46087.48078703704</v>
+        <v>46087.55607638889</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16569,7 +16559,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46087.47663194445</v>
+        <v>46087.55453703704</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16697,7 +16687,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46087.47820601852</v>
+        <v>46087.55619212963</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16761,7 +16751,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46087.449375</v>
+        <v>46087.57064814815</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16819,7 +16809,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46087.48112268518</v>
+        <v>46087.5547337963</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16883,7 +16873,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46087.48527777778</v>
+        <v>46087.56151620371</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16947,7 +16937,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46087.48299768518</v>
+        <v>46087.55989583334</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -17011,7 +17001,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46087.46489583333</v>
+        <v>46087.545</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17075,7 +17065,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46087.45498842592</v>
+        <v>46087.55813657407</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17139,7 +17129,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46087.48324074074</v>
+        <v>46087.56165509259</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17203,7 +17193,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46087.48210648148</v>
+        <v>46087.55831018519</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17331,7 +17321,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46087.44722222222</v>
+        <v>46087.56991898148</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17395,7 +17385,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46087.48653935185</v>
+        <v>46087.56480324074</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17459,7 +17449,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46087.48324074074</v>
+        <v>46087.5590162037</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17523,7 +17513,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46087.48200231481</v>
+        <v>46087.55851851852</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17587,7 +17577,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46087.48315972222</v>
+        <v>46087.55847222222</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17651,7 +17641,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46087.45196759259</v>
+        <v>46087.56997685185</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17779,7 +17769,7 @@
         <v>1</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46087.46677083334</v>
+        <v>46087.538125</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17840,7 +17830,7 @@
         </is>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46087.45491898148</v>
+        <v>46087.53672453704</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17968,7 +17958,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46087.4597337963</v>
+        <v>46087.57118055555</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -18093,7 +18083,7 @@
         </is>
       </c>
       <c r="N273" s="3" t="n">
-        <v>46087.45804398148</v>
+        <v>46087.53586805556</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -18341,7 +18331,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46087.48677083333</v>
+        <v>46087.56422453704</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18405,7 +18395,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46087.46178240741</v>
+        <v>46087.53993055555</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18587,7 +18577,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46087.46670138889</v>
+        <v>46087.55027777778</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18651,7 +18641,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46087.44738425926</v>
+        <v>46087.56675925926</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18715,7 +18705,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46087.48222222222</v>
+        <v>46087.5582175926</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18779,7 +18769,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46087.48733796296</v>
+        <v>46087.56019675926</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18798,6 +18788,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>10.69.5.155</t>
+        </is>
+      </c>
       <c r="D285" t="n">
         <v>2019</v>
       </c>
@@ -18838,7 +18833,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46087.45231481481</v>
+        <v>46087.56849537037</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18902,7 +18897,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46087.48758101852</v>
+        <v>46087.56427083333</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18966,7 +18961,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46087.48039351852</v>
+        <v>46087.55752314815</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19030,7 +19025,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46087.47928240741</v>
+        <v>46087.55929398148</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19824,7 +19819,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46087.47792824074</v>
+        <v>46087.55344907408</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20940,7 +20935,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46087.47034722222</v>
+        <v>46087.54945601852</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21665,7 +21660,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46087.48390046296</v>
+        <v>46087.56185185185</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21729,7 +21724,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46087.47391203704</v>
+        <v>46087.55373842592</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21793,7 +21788,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46087.48387731481</v>
+        <v>46087.56267361111</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21857,7 +21852,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46087.46649305556</v>
+        <v>46087.54416666667</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21921,7 +21916,7 @@
         <v>1</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46087.46965277778</v>
+        <v>46087.5483912037</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21985,7 +21980,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46087.47412037037</v>
+        <v>46087.55553240741</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22049,7 +22044,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46087.46782407408</v>
+        <v>46087.54896990741</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22113,7 +22108,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46087.47702546296</v>
+        <v>46087.55892361111</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22241,7 +22236,7 @@
         <v>2</v>
       </c>
       <c r="N340" s="3" t="n">
-        <v>46086.33009259259</v>
+        <v>46087.55576388889</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -22622,7 +22617,7 @@
         <v>1</v>
       </c>
       <c r="N346" s="3" t="n">
-        <v>46087.48049768519</v>
+        <v>46087.56026620371</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -22686,7 +22681,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46087.45586805556</v>
+        <v>46087.53907407408</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22750,7 +22745,7 @@
         <v>1</v>
       </c>
       <c r="N348" s="3" t="n">
-        <v>46087.45260416667</v>
+        <v>46087.56721064815</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -22875,7 +22870,7 @@
         <v>1</v>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46087.45472222222</v>
+        <v>46087.53168981482</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -22939,7 +22934,7 @@
         <v>1</v>
       </c>
       <c r="N351" s="3" t="n">
-        <v>46087.48706018519</v>
+        <v>46087.56494212963</v>
       </c>
       <c r="O351" t="inlineStr">
         <is>
@@ -23125,7 +23120,7 @@
         <v>1</v>
       </c>
       <c r="N354" s="3" t="n">
-        <v>46087.48429398148</v>
+        <v>46087.56409722222</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -23189,7 +23184,7 @@
         <v>1</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46087.48467592592</v>
+        <v>46087.5646412037</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23253,7 +23248,7 @@
         <v>1</v>
       </c>
       <c r="N356" s="3" t="n">
-        <v>46087.48543981482</v>
+        <v>46087.57063657408</v>
       </c>
       <c r="O356" t="inlineStr">
         <is>
@@ -23381,7 +23376,7 @@
         <v>2</v>
       </c>
       <c r="N358" s="3" t="n">
-        <v>46087.45118055555</v>
+        <v>46087.56284722222</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -23445,7 +23440,7 @@
         <v>2</v>
       </c>
       <c r="N359" s="3" t="n">
-        <v>46087.45547453704</v>
+        <v>46087.53648148148</v>
       </c>
       <c r="O359" t="inlineStr">
         <is>
@@ -23509,7 +23504,7 @@
         <v>1</v>
       </c>
       <c r="N360" s="3" t="n">
-        <v>46087.47716435185</v>
+        <v>46087.55847222222</v>
       </c>
       <c r="O360" t="inlineStr">
         <is>
@@ -23758,7 +23753,7 @@
         <v>1</v>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46087.46706018518</v>
+        <v>46087.53986111111</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23824,7 +23819,7 @@
         </is>
       </c>
       <c r="N365" s="3" t="n">
-        <v>46087.46895833333</v>
+        <v>46087.54540509259</v>
       </c>
       <c r="O365" t="inlineStr">
         <is>
@@ -23950,7 +23945,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46087.47791666666</v>
+        <v>46087.55209490741</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -24080,7 +24075,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46087.48518518519</v>
+        <v>46087.56510416666</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24108,7 +24103,7 @@
         <v>2</v>
       </c>
       <c r="N370" s="3" t="n">
-        <v>46087.48193287037</v>
+        <v>46087.5588425926</v>
       </c>
       <c r="O370" t="inlineStr">
         <is>
@@ -24381,7 +24376,7 @@
         </is>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46087.47168981482</v>
+        <v>46087.54680555555</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24400,6 +24395,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>10.69.3.72</t>
+        </is>
+      </c>
       <c r="D375" t="n">
         <v>2025</v>
       </c>
@@ -24445,7 +24445,7 @@
         <v>1</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46086.81421296296</v>
+        <v>46087.56666666667</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24514,7 +24514,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46087.454375</v>
+        <v>46087.53052083333</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -24583,7 +24583,7 @@
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46087.4569675926</v>
+        <v>46087.53530092593</v>
       </c>
       <c r="O377" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-06 15:52:06.025642
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46087.54032407407</v>
+        <v>46087.61965277778</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46087.55841435185</v>
+        <v>46087.63633101852</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46087.56822916667</v>
+        <v>46087.6452662037</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46087.56357638889</v>
+        <v>46087.63997685185</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -870,7 +870,7 @@
         <v>1</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>46087.55134259259</v>
+        <v>46087.62825231482</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
         <v>1</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>46087.5434375</v>
+        <v>46087.6220949074</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1003,7 +1003,7 @@
         <v>1</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>46087.54685185185</v>
+        <v>46087.63587962963</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1067,7 +1067,7 @@
         <v>1</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>46087.54733796296</v>
+        <v>46087.64900462963</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46087.56087962963</v>
+        <v>46087.6390625</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
         <v>1</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>46087.54518518518</v>
+        <v>46087.65341435185</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1382,7 +1382,7 @@
         <v>2</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>46087.5434837963</v>
+        <v>46087.62629629629</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46087.55569444445</v>
+        <v>46087.63126157408</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1510,7 +1510,7 @@
         <v>2</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>46087.54890046296</v>
+        <v>46087.63935185185</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46087.54075231482</v>
+        <v>46087.63364583333</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1702,7 +1702,7 @@
         <v>1</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>46087.56180555555</v>
+        <v>46087.64087962963</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1766,7 +1766,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46087.53493055556</v>
+        <v>46087.64931712963</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>46087.50902777778</v>
+        <v>46087.64267361111</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -1943,7 +1943,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46087.48642361111</v>
+        <v>46087.61283564815</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -1962,6 +1962,11 @@
           <t>AUDITORIO</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>10.69.3.153</t>
+        </is>
+      </c>
       <c r="D24" t="n">
         <v>2019</v>
       </c>
@@ -1999,7 +2004,7 @@
         </is>
       </c>
       <c r="N24" s="3" t="n">
-        <v>46087.52459490741</v>
+        <v>46087.64443287037</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2058,7 +2063,7 @@
         <v>1</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>46087.50386574074</v>
+        <v>46087.57148148148</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2117,7 +2122,7 @@
         <v>1</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>46087.53324074074</v>
+        <v>46087.6135300926</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2178,7 +2183,7 @@
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46087.5633912037</v>
+        <v>46087.6387962963</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6504,7 +6509,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46087.54825231482</v>
+        <v>46087.62803240741</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6573,7 +6578,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46087.55947916667</v>
+        <v>46087.64159722222</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6592,6 +6597,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>10.69.3.93</t>
+        </is>
+      </c>
       <c r="D96" t="n">
         <v>2025</v>
       </c>
@@ -6637,7 +6647,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46087.53138888889</v>
+        <v>46087.64745370371</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6701,7 +6711,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46087.56637731481</v>
+        <v>46087.64226851852</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6770,7 +6780,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46087.54103009259</v>
+        <v>46087.65103009259</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6839,7 +6849,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46087.56230324074</v>
+        <v>46087.64027777778</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6908,7 +6918,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46087.55622685186</v>
+        <v>46087.63549768519</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -7046,7 +7056,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46087.56797453704</v>
+        <v>46087.6475</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7303,7 +7313,7 @@
         <v>1</v>
       </c>
       <c r="N106" s="3" t="n">
-        <v>46087.53865740741</v>
+        <v>46087.65215277778</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -7441,7 +7451,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46087.55811342593</v>
+        <v>46087.63240740741</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7510,7 +7520,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46087.54768518519</v>
+        <v>46087.6271875</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7579,7 +7589,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46087.55221064815</v>
+        <v>46087.63258101852</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7648,7 +7658,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46087.54953703703</v>
+        <v>46087.6325462963</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7717,7 +7727,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46087.53820601852</v>
+        <v>46087.65322916667</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7786,7 +7796,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46087.56773148148</v>
+        <v>46087.64582175926</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7852,7 +7862,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46087.53451388889</v>
+        <v>46087.6472337963</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7921,7 +7931,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46087.57107638889</v>
+        <v>46087.64664351852</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7990,7 +8000,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46087.57114583333</v>
+        <v>46087.65210648148</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8056,7 +8066,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46087.56746527777</v>
+        <v>46087.64703703704</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8194,7 +8204,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46087.5427662037</v>
+        <v>46087.62384259259</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8263,7 +8273,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46087.56983796296</v>
+        <v>46087.65075231482</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8329,7 +8339,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46087.56180555555</v>
+        <v>46087.63334490741</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8398,7 +8408,7 @@
         <v>2</v>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46087.55480324074</v>
+        <v>46087.63038194444</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8467,7 +8477,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46087.56865740741</v>
+        <v>46087.64491898148</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8536,7 +8546,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46087.5666087963</v>
+        <v>46087.63902777778</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8605,7 +8615,7 @@
         <v>2</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46087.53707175926</v>
+        <v>46087.61675925926</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8743,7 +8753,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46087.53354166666</v>
+        <v>46087.64778935185</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8812,7 +8822,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46087.54670138889</v>
+        <v>46087.6215162037</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8881,7 +8891,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46087.55524305555</v>
+        <v>46087.6340625</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -8945,7 +8955,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46087.55150462963</v>
+        <v>46087.63421296296</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9078,7 +9088,7 @@
         <v>1</v>
       </c>
       <c r="N132" s="3" t="n">
-        <v>46087.48354166667</v>
+        <v>46087.62252314815</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -9142,7 +9152,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46087.56673611111</v>
+        <v>46087.64681712963</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9206,7 +9216,7 @@
         <v>1</v>
       </c>
       <c r="N134" s="3" t="n">
-        <v>46087.56570601852</v>
+        <v>46087.63434027778</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -9270,7 +9280,7 @@
         <v>1</v>
       </c>
       <c r="N135" s="3" t="n">
-        <v>46087.5559375</v>
+        <v>46087.63611111111</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -9397,7 +9407,7 @@
         <v>1</v>
       </c>
       <c r="N137" s="3" t="n">
-        <v>46087.55927083334</v>
+        <v>46087.63818287037</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -9461,7 +9471,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46087.55134259259</v>
+        <v>46087.62424768518</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9525,7 +9535,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46087.45377314815</v>
+        <v>46087.6222337963</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9589,7 +9599,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46087.55278935185</v>
+        <v>46087.63423611111</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9653,7 +9663,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46087.54049768519</v>
+        <v>46087.61940972223</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9717,7 +9727,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46087.55488425926</v>
+        <v>46087.62471064815</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9781,7 +9791,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46087.53498842593</v>
+        <v>46087.61658564815</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9845,7 +9855,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46087.41553240741</v>
+        <v>46087.61915509259</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9909,7 +9919,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46087.55883101852</v>
+        <v>46087.62628472222</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9973,7 +9983,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46087.53259259259</v>
+        <v>46087.64859953704</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10037,7 +10047,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46087.5671875</v>
+        <v>46087.64523148148</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10101,7 +10111,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46087.53075231481</v>
+        <v>46087.65027777778</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10229,7 +10239,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46087.54649305555</v>
+        <v>46087.62451388889</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10293,7 +10303,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46087.5712037037</v>
+        <v>46087.61695601852</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10357,7 +10367,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46087.57123842592</v>
+        <v>46087.64877314815</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10485,7 +10495,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46087.54748842592</v>
+        <v>46087.626875</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10549,7 +10559,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46087.5603587963</v>
+        <v>46087.63614583333</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10613,7 +10623,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46087.53288194445</v>
+        <v>46087.57607638889</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10677,7 +10687,7 @@
         <v>1</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>46087.56981481481</v>
+        <v>46087.64806712963</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -10741,7 +10751,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46087.54121527778</v>
+        <v>46087.65193287037</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10805,7 +10815,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46087.56519675926</v>
+        <v>46087.63925925926</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10869,7 +10879,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46087.53649305556</v>
+        <v>46087.57236111111</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10933,7 +10943,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46087.5312037037</v>
+        <v>46087.63122685185</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -10997,7 +11007,7 @@
         <v>1</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46087.56321759259</v>
+        <v>46087.63866898148</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11058,10 +11068,10 @@
         </is>
       </c>
       <c r="M163" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46087.55513888889</v>
+        <v>46087.63604166666</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11125,7 +11135,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46087.55186342593</v>
+        <v>46087.59200231481</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11189,7 +11199,7 @@
         <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46087.5578125</v>
+        <v>46087.63283564815</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11253,7 +11263,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46087.55488425926</v>
+        <v>46087.63553240741</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11381,7 +11391,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46087.56015046296</v>
+        <v>46087.63738425926</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11445,7 +11455,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46087.5521875</v>
+        <v>46087.63449074074</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11509,7 +11519,7 @@
         <v>1</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46087.54773148148</v>
+        <v>46087.62408564815</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11573,7 +11583,7 @@
         <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46087.53928240741</v>
+        <v>46087.57952546296</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11637,7 +11647,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46087.56465277778</v>
+        <v>46087.64424768519</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11765,7 +11775,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46087.56695601852</v>
+        <v>46087.63790509259</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11829,7 +11839,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46087.5399537037</v>
+        <v>46087.65417824074</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11893,7 +11903,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46087.54305555556</v>
+        <v>46087.61675925926</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11957,7 +11967,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46087.55306712963</v>
+        <v>46087.62608796296</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12021,7 +12031,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46087.55358796296</v>
+        <v>46087.62787037037</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12085,7 +12095,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46086.818125</v>
+        <v>46087.62320601852</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12149,7 +12159,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46086.82105324074</v>
+        <v>46087.63972222222</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12474,7 +12484,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46086.83462962963</v>
+        <v>46087.64421296296</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12538,7 +12548,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46087.568125</v>
+        <v>46087.64712962963</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12602,7 +12612,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46087.53423611111</v>
+        <v>46087.64869212963</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12730,7 +12740,7 @@
         </is>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46087.55012731482</v>
+        <v>46087.63216435185</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12794,7 +12804,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46087.56959490741</v>
+        <v>46087.65247685185</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12858,7 +12868,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46087.54961805556</v>
+        <v>46087.63789351852</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -13047,7 +13057,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46087.56893518518</v>
+        <v>46087.64296296296</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13111,7 +13121,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46087.52959490741</v>
+        <v>46087.6466087963</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13175,7 +13185,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46087.55809027778</v>
+        <v>46087.64336805556</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13239,7 +13249,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46087.56074074074</v>
+        <v>46087.62361111111</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13303,7 +13313,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46087.55924768518</v>
+        <v>46087.62290509259</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13367,7 +13377,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46087.55362268518</v>
+        <v>46087.63493055556</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13428,7 +13438,7 @@
         </is>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46086.80949074074</v>
+        <v>46087.65114583333</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13492,7 +13502,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46087.56510416666</v>
+        <v>46087.64141203704</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13556,7 +13566,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46087.5436574074</v>
+        <v>46087.64674768518</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13620,7 +13630,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46087.57099537037</v>
+        <v>46087.63929398148</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13684,7 +13694,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46087.57100694445</v>
+        <v>46087.65381944444</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13748,7 +13758,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46087.5587037037</v>
+        <v>46087.64288194444</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13812,7 +13822,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46087.56194444445</v>
+        <v>46087.64344907407</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13876,7 +13886,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46087.56842592593</v>
+        <v>46087.64363425926</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13940,7 +13950,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46087.56019675926</v>
+        <v>46087.64091435185</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14004,7 +14014,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46087.55184027777</v>
+        <v>46087.62700231482</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14068,7 +14078,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46087.564375</v>
+        <v>46087.62234953704</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14132,7 +14142,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46087.55902777778</v>
+        <v>46087.6325462963</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14196,7 +14206,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46087.56956018518</v>
+        <v>46087.64309027778</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14260,7 +14270,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46087.5558912037</v>
+        <v>46087.640625</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14324,7 +14334,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46086.8340625</v>
+        <v>46087.64201388889</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14388,7 +14398,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46087.55730324074</v>
+        <v>46087.63530092593</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14447,7 +14457,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46087.55655092592</v>
+        <v>46087.63672453703</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14511,7 +14521,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46087.57010416667</v>
+        <v>46087.64603009259</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14575,7 +14585,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46087.5547337963</v>
+        <v>46087.64047453704</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14644,7 +14654,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46087.56490740741</v>
+        <v>46087.64159722222</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14708,7 +14718,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46087.45744212963</v>
+        <v>46087.61464120371</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14772,7 +14782,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46087.53725694444</v>
+        <v>46087.64528935185</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14900,7 +14910,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46086.79446759259</v>
+        <v>46087.63428240741</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14964,7 +14974,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46087.56344907408</v>
+        <v>46087.63653935185</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15028,7 +15038,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46086.83831018519</v>
+        <v>46087.64077546296</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15092,7 +15102,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46086.80550925926</v>
+        <v>46087.64090277778</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15156,7 +15166,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46087.56170138889</v>
+        <v>46087.64082175926</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15220,7 +15230,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46087.55</v>
+        <v>46087.62266203704</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15284,7 +15294,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46087.54670138889</v>
+        <v>46087.62743055556</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15348,7 +15358,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46087.55930555556</v>
+        <v>46087.63539351852</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15412,7 +15422,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46087.56121527778</v>
+        <v>46087.62538194445</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15476,7 +15486,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46087.55950231481</v>
+        <v>46087.63728009259</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15540,7 +15550,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46087.53743055555</v>
+        <v>46087.63693287037</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15604,7 +15614,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46087.56737268518</v>
+        <v>46087.6403125</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15668,7 +15678,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46087.53586805556</v>
+        <v>46087.61538194444</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15732,7 +15742,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46086.82879629629</v>
+        <v>46087.63736111111</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15796,7 +15806,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46087.55296296296</v>
+        <v>46087.63434027778</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15860,7 +15870,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46087.54222222222</v>
+        <v>46087.6374537037</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15924,7 +15934,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46087.55726851852</v>
+        <v>46087.63295138889</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -15988,7 +15998,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46086.83282407407</v>
+        <v>46087.63715277778</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16052,7 +16062,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46087.55548611111</v>
+        <v>46087.63136574074</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16116,7 +16126,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46087.53032407408</v>
+        <v>46087.63802083334</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16239,7 +16249,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46087.5534375</v>
+        <v>46087.63538194444</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16303,7 +16313,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46087.55665509259</v>
+        <v>46087.63150462963</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16367,7 +16377,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46087.55700231482</v>
+        <v>46087.63414351852</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16431,7 +16441,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46087.54835648148</v>
+        <v>46087.62725694444</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16495,7 +16505,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46087.55607638889</v>
+        <v>46087.63305555555</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16559,7 +16569,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46087.55453703704</v>
+        <v>46087.6290162037</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16623,7 +16633,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46086.85931712963</v>
+        <v>46087.62063657407</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16687,7 +16697,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46087.55619212963</v>
+        <v>46087.63546296296</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16751,7 +16761,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46087.57064814815</v>
+        <v>46087.63716435185</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16809,7 +16819,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46087.5547337963</v>
+        <v>46087.63681712963</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16873,7 +16883,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46087.56151620371</v>
+        <v>46087.64069444445</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16937,7 +16947,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46087.55989583334</v>
+        <v>46087.63837962963</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -17001,7 +17011,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46087.545</v>
+        <v>46087.62148148148</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17065,7 +17075,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46087.55813657407</v>
+        <v>46087.64539351852</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17129,7 +17139,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46087.56165509259</v>
+        <v>46087.6346412037</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17193,7 +17203,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46087.55831018519</v>
+        <v>46087.59630787037</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17257,7 +17267,7 @@
         <v>2</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46086.82716435185</v>
+        <v>46087.62413194445</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17321,7 +17331,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46087.56991898148</v>
+        <v>46087.63928240741</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17385,7 +17395,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46087.56480324074</v>
+        <v>46087.64291666666</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17449,7 +17459,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46087.5590162037</v>
+        <v>46087.63813657407</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17513,7 +17523,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46087.55851851852</v>
+        <v>46087.63329861111</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17577,7 +17587,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46087.55847222222</v>
+        <v>46087.63685185185</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17641,7 +17651,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46087.56997685185</v>
+        <v>46087.64886574074</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17705,7 +17715,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46087.41716435185</v>
+        <v>46087.57641203704</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17769,7 +17779,7 @@
         <v>1</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46087.538125</v>
+        <v>46087.63702546297</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17830,7 +17840,7 @@
         </is>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46087.53672453704</v>
+        <v>46087.61456018518</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17958,7 +17968,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46087.57118055555</v>
+        <v>46087.61518518518</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -18083,7 +18093,7 @@
         </is>
       </c>
       <c r="N273" s="3" t="n">
-        <v>46087.53586805556</v>
+        <v>46087.6540625</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -18331,7 +18341,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46087.56422453704</v>
+        <v>46087.63469907407</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18395,7 +18405,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46087.53993055555</v>
+        <v>46087.62219907407</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18577,7 +18587,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46087.55027777778</v>
+        <v>46087.62858796296</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18641,7 +18651,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46087.56675925926</v>
+        <v>46087.64358796296</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18705,7 +18715,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46087.5582175926</v>
+        <v>46087.63805555556</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18769,7 +18779,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46087.56019675926</v>
+        <v>46087.63228009259</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18788,11 +18798,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C285" t="inlineStr">
-        <is>
-          <t>10.69.5.155</t>
-        </is>
-      </c>
       <c r="D285" t="n">
         <v>2019</v>
       </c>
@@ -19025,7 +19030,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46087.55929398148</v>
+        <v>46087.63836805556</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19819,7 +19824,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46087.55344907408</v>
+        <v>46087.62508101852</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20935,7 +20940,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46087.54945601852</v>
+        <v>46087.63081018518</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21660,7 +21665,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46087.56185185185</v>
+        <v>46087.64071759259</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21724,7 +21729,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46087.55373842592</v>
+        <v>46087.63045138889</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21788,7 +21793,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46087.56267361111</v>
+        <v>46087.63626157407</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21852,7 +21857,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46087.54416666667</v>
+        <v>46087.62143518519</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21980,7 +21985,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46087.55553240741</v>
+        <v>46087.63373842592</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22044,7 +22049,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46087.54896990741</v>
+        <v>46087.62028935185</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22108,7 +22113,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46087.55892361111</v>
+        <v>46087.63026620371</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22617,7 +22622,7 @@
         <v>1</v>
       </c>
       <c r="N346" s="3" t="n">
-        <v>46087.56026620371</v>
+        <v>46087.59559027778</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -22681,7 +22686,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46087.53907407408</v>
+        <v>46087.58287037037</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22745,7 +22750,7 @@
         <v>1</v>
       </c>
       <c r="N348" s="3" t="n">
-        <v>46087.56721064815</v>
+        <v>46087.60527777778</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -22870,7 +22875,7 @@
         <v>1</v>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46087.53168981482</v>
+        <v>46087.57554398148</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -22934,7 +22939,7 @@
         <v>1</v>
       </c>
       <c r="N351" s="3" t="n">
-        <v>46087.56494212963</v>
+        <v>46087.60881944445</v>
       </c>
       <c r="O351" t="inlineStr">
         <is>
@@ -23120,7 +23125,7 @@
         <v>1</v>
       </c>
       <c r="N354" s="3" t="n">
-        <v>46087.56409722222</v>
+        <v>46087.60150462963</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -23184,7 +23189,7 @@
         <v>1</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46087.5646412037</v>
+        <v>46087.60498842593</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23376,7 +23381,7 @@
         <v>2</v>
       </c>
       <c r="N358" s="3" t="n">
-        <v>46087.56284722222</v>
+        <v>46087.60486111111</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -23440,7 +23445,7 @@
         <v>2</v>
       </c>
       <c r="N359" s="3" t="n">
-        <v>46087.53648148148</v>
+        <v>46087.57782407408</v>
       </c>
       <c r="O359" t="inlineStr">
         <is>
@@ -23504,7 +23509,7 @@
         <v>1</v>
       </c>
       <c r="N360" s="3" t="n">
-        <v>46087.55847222222</v>
+        <v>46087.59552083333</v>
       </c>
       <c r="O360" t="inlineStr">
         <is>
@@ -23753,7 +23758,7 @@
         <v>1</v>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46087.53986111111</v>
+        <v>46087.64725694444</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23819,7 +23824,7 @@
         </is>
       </c>
       <c r="N365" s="3" t="n">
-        <v>46087.54540509259</v>
+        <v>46087.62270833334</v>
       </c>
       <c r="O365" t="inlineStr">
         <is>
@@ -23945,7 +23950,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46087.55209490741</v>
+        <v>46087.63309027778</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -24006,7 +24011,7 @@
         </is>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46087.37417824074</v>
+        <v>46087.62934027778</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24075,7 +24080,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46087.56510416666</v>
+        <v>46087.63916666667</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24103,7 +24108,7 @@
         <v>2</v>
       </c>
       <c r="N370" s="3" t="n">
-        <v>46087.5588425926</v>
+        <v>46087.63688657407</v>
       </c>
       <c r="O370" t="inlineStr">
         <is>
@@ -24241,7 +24246,7 @@
         <v>1</v>
       </c>
       <c r="N372" s="3" t="n">
-        <v>46086.71232638889</v>
+        <v>46087.62893518519</v>
       </c>
       <c r="O372" t="inlineStr">
         <is>
@@ -24376,7 +24381,7 @@
         </is>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46087.54680555555</v>
+        <v>46087.62596064815</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24395,11 +24400,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C375" t="inlineStr">
-        <is>
-          <t>10.69.3.72</t>
-        </is>
-      </c>
       <c r="D375" t="n">
         <v>2025</v>
       </c>
@@ -24445,7 +24445,7 @@
         <v>1</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46087.56666666667</v>
+        <v>46087.64563657407</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24514,7 +24514,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46087.53052083333</v>
+        <v>46087.65140046296</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -24583,7 +24583,7 @@
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46087.53530092593</v>
+        <v>46087.65325231481</v>
       </c>
       <c r="O377" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-06 17:52:05.855211
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46087.61965277778</v>
+        <v>46087.73710648148</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46087.63633101852</v>
+        <v>46087.69759259259</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46087.6452662037</v>
+        <v>46087.72545138889</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46087.63997685185</v>
+        <v>46087.72302083333</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -870,7 +870,7 @@
         <v>1</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>46087.62825231482</v>
+        <v>46087.70386574074</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
         <v>1</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>46087.6220949074</v>
+        <v>46087.69795138889</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1003,7 +1003,7 @@
         <v>1</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>46087.63587962963</v>
+        <v>46087.71417824074</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1067,7 +1067,7 @@
         <v>1</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>46087.64900462963</v>
+        <v>46087.72385416667</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Microsoft Windows 7 Professional</t>
+          <t>Windows</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1190,7 +1190,7 @@
         <v>1</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>46062.63414351852</v>
+        <v>46087.68027777778</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>46087.6390625</v>
+        <v>46087.71921296296</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
         <v>1</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>46087.65341435185</v>
+        <v>46087.73180555556</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1382,7 +1382,7 @@
         <v>2</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>46087.62629629629</v>
+        <v>46087.6994675926</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46087.63126157408</v>
+        <v>46087.70715277778</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1510,7 +1510,7 @@
         <v>2</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>46087.63935185185</v>
+        <v>46087.71814814815</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>46087.63364583333</v>
+        <v>46087.71222222222</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1702,7 +1702,7 @@
         <v>1</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>46087.64087962963</v>
+        <v>46087.72064814815</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1766,7 +1766,7 @@
         <v>1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>46087.64931712963</v>
+        <v>46087.69016203703</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>46087.64267361111</v>
+        <v>46087.71460648148</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -1943,7 +1943,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46087.61283564815</v>
+        <v>46087.73119212963</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="N24" s="3" t="n">
-        <v>46087.64443287037</v>
+        <v>46087.73737268519</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2122,7 +2122,7 @@
         <v>1</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>46087.6135300926</v>
+        <v>46087.70180555555</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46087.6387962963</v>
+        <v>46087.71592592593</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6509,7 +6509,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46087.62803240741</v>
+        <v>46087.70666666667</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6578,7 +6578,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46087.64159722222</v>
+        <v>46087.71918981482</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6597,11 +6597,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>10.69.3.93</t>
-        </is>
-      </c>
       <c r="D96" t="n">
         <v>2025</v>
       </c>
@@ -6647,7 +6642,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46087.64745370371</v>
+        <v>46087.68878472222</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6711,7 +6706,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46087.64226851852</v>
+        <v>46087.67993055555</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6780,7 +6775,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46087.65103009259</v>
+        <v>46087.68961805556</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6849,7 +6844,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46087.64027777778</v>
+        <v>46087.71994212963</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6918,7 +6913,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46087.63549768519</v>
+        <v>46087.71275462963</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -7056,7 +7051,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46087.6475</v>
+        <v>46087.68898148148</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7451,7 +7446,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46087.63240740741</v>
+        <v>46087.71005787037</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7520,7 +7515,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46087.6271875</v>
+        <v>46087.70512731482</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7589,7 +7584,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46087.63258101852</v>
+        <v>46087.70859953704</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7658,7 +7653,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46087.6325462963</v>
+        <v>46087.67</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7727,7 +7722,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46087.65322916667</v>
+        <v>46087.73318287037</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7796,7 +7791,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46087.64582175926</v>
+        <v>46087.72094907407</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7862,7 +7857,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46087.6472337963</v>
+        <v>46087.68893518519</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7931,7 +7926,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46087.64664351852</v>
+        <v>46087.68431712963</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -8000,7 +7995,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46087.65210648148</v>
+        <v>46087.68974537037</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8066,7 +8061,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46087.64703703704</v>
+        <v>46087.68583333334</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8204,7 +8199,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46087.62384259259</v>
+        <v>46087.70304398148</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8273,7 +8268,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46087.65075231482</v>
+        <v>46087.72896990741</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8339,7 +8334,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46087.63334490741</v>
+        <v>46087.72768518519</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8408,7 +8403,7 @@
         <v>2</v>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46087.63038194444</v>
+        <v>46087.70310185185</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8477,7 +8472,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46087.64491898148</v>
+        <v>46087.72328703704</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8546,7 +8541,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46087.63902777778</v>
+        <v>46087.71267361111</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8615,7 +8610,7 @@
         <v>2</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46087.61675925926</v>
+        <v>46087.73445601852</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8753,7 +8748,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46087.64778935185</v>
+        <v>46087.68458333334</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8822,7 +8817,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46087.6215162037</v>
+        <v>46087.7331712963</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8891,7 +8886,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46087.6340625</v>
+        <v>46087.71310185185</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -8955,7 +8950,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46087.63421296296</v>
+        <v>46087.67005787037</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9088,7 +9083,7 @@
         <v>1</v>
       </c>
       <c r="N132" s="3" t="n">
-        <v>46087.62252314815</v>
+        <v>46087.73434027778</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -9152,7 +9147,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46087.64681712963</v>
+        <v>46087.72619212963</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9216,7 +9211,7 @@
         <v>1</v>
       </c>
       <c r="N134" s="3" t="n">
-        <v>46087.63434027778</v>
+        <v>46087.73508101852</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -9280,7 +9275,7 @@
         <v>1</v>
       </c>
       <c r="N135" s="3" t="n">
-        <v>46087.63611111111</v>
+        <v>46087.71533564815</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -9407,7 +9402,7 @@
         <v>1</v>
       </c>
       <c r="N137" s="3" t="n">
-        <v>46087.63818287037</v>
+        <v>46087.71581018518</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -9471,7 +9466,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46087.62424768518</v>
+        <v>46087.7365162037</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9535,7 +9530,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46087.6222337963</v>
+        <v>46087.69837962963</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9599,7 +9594,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46087.63423611111</v>
+        <v>46087.71070601852</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9663,7 +9658,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46087.61940972223</v>
+        <v>46087.73444444445</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9727,7 +9722,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46087.62471064815</v>
+        <v>46087.69974537037</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9791,7 +9786,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46087.61658564815</v>
+        <v>46087.69857638889</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9855,7 +9850,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46087.61915509259</v>
+        <v>46087.73673611111</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9919,7 +9914,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46087.62628472222</v>
+        <v>46087.70326388889</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9983,7 +9978,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46087.64859953704</v>
+        <v>46087.72910879629</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10047,7 +10042,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46087.64523148148</v>
+        <v>46087.72172453703</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10111,7 +10106,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46087.65027777778</v>
+        <v>46087.72204861111</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10239,7 +10234,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46087.62451388889</v>
+        <v>46087.70431712963</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10303,7 +10298,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46087.61695601852</v>
+        <v>46087.73606481482</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10367,7 +10362,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46087.64877314815</v>
+        <v>46087.72533564815</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10495,7 +10490,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46087.626875</v>
+        <v>46087.70686342593</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10559,7 +10554,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46087.63614583333</v>
+        <v>46087.71893518518</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10687,7 +10682,7 @@
         <v>1</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>46087.64806712963</v>
+        <v>46087.72265046297</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -10751,7 +10746,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46087.65193287037</v>
+        <v>46087.72472222222</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10815,7 +10810,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46087.63925925926</v>
+        <v>46087.71253472222</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10943,7 +10938,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46087.63122685185</v>
+        <v>46087.71283564815</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -11007,7 +11002,7 @@
         <v>1</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46087.63866898148</v>
+        <v>46087.72118055556</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11071,7 +11066,7 @@
         <v>2</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46087.63604166666</v>
+        <v>46087.71371527778</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11263,7 +11258,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46087.63553240741</v>
+        <v>46087.67258101852</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11391,7 +11386,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46087.63738425926</v>
+        <v>46087.70993055555</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11455,7 +11450,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46087.63449074074</v>
+        <v>46087.71189814815</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11519,7 +11514,7 @@
         <v>1</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46087.62408564815</v>
+        <v>46087.70204861111</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11647,7 +11642,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46087.64424768519</v>
+        <v>46087.72540509259</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11775,7 +11770,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46087.63790509259</v>
+        <v>46087.71304398148</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11903,7 +11898,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46087.61675925926</v>
+        <v>46087.73550925926</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11967,7 +11962,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46087.62608796296</v>
+        <v>46087.70506944445</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12031,7 +12026,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46087.62787037037</v>
+        <v>46087.70556712963</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12095,7 +12090,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46087.62320601852</v>
+        <v>46087.70144675926</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12159,7 +12154,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46087.63972222222</v>
+        <v>46087.71542824074</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12484,7 +12479,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46087.64421296296</v>
+        <v>46087.71947916667</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12548,7 +12543,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46087.64712962963</v>
+        <v>46087.72790509259</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12612,7 +12607,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46087.64869212963</v>
+        <v>46087.72721064815</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12740,7 +12735,7 @@
         </is>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46087.63216435185</v>
+        <v>46087.71405092593</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12804,7 +12799,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46087.65247685185</v>
+        <v>46087.72731481482</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12868,7 +12863,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46087.63789351852</v>
+        <v>46087.71246527778</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -13057,7 +13052,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46087.64296296296</v>
+        <v>46087.7158449074</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13121,7 +13116,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46087.6466087963</v>
+        <v>46087.72091435185</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13185,7 +13180,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46087.64336805556</v>
+        <v>46087.71951388889</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13249,7 +13244,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46087.62361111111</v>
+        <v>46087.70222222222</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13313,7 +13308,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46087.62290509259</v>
+        <v>46087.7000462963</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13377,7 +13372,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46087.63493055556</v>
+        <v>46087.70912037037</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13438,7 +13433,7 @@
         </is>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46087.65114583333</v>
+        <v>46087.71328703704</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13502,7 +13497,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46087.64141203704</v>
+        <v>46087.71940972222</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13566,7 +13561,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46087.64674768518</v>
+        <v>46087.72498842593</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13630,7 +13625,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46087.63929398148</v>
+        <v>46087.71241898148</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13694,7 +13689,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46087.65381944444</v>
+        <v>46087.73590277778</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13758,7 +13753,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46087.64288194444</v>
+        <v>46087.72247685185</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13822,7 +13817,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46087.64344907407</v>
+        <v>46087.72416666667</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13950,7 +13945,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46087.64091435185</v>
+        <v>46087.71376157407</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14014,7 +14009,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46087.62700231482</v>
+        <v>46087.70414351852</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14078,7 +14073,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46087.62234953704</v>
+        <v>46087.73555555556</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14142,7 +14137,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46087.6325462963</v>
+        <v>46087.70673611111</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14206,7 +14201,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46087.64309027778</v>
+        <v>46087.72103009259</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14270,7 +14265,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46087.640625</v>
+        <v>46087.71949074074</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14334,7 +14329,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46087.64201388889</v>
+        <v>46087.71894675926</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14398,7 +14393,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46087.63530092593</v>
+        <v>46087.71212962963</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14457,7 +14452,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46087.63672453703</v>
+        <v>46087.71380787037</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14521,7 +14516,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46087.64603009259</v>
+        <v>46087.72438657407</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14585,7 +14580,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46087.64047453704</v>
+        <v>46087.71696759259</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14654,7 +14649,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46087.64159722222</v>
+        <v>46087.70733796297</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14718,7 +14713,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46087.61464120371</v>
+        <v>46087.72949074074</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14782,7 +14777,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46087.64528935185</v>
+        <v>46087.72635416667</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14846,7 +14841,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46086.82976851852</v>
+        <v>46087.70270833333</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14910,7 +14905,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46087.63428240741</v>
+        <v>46087.72971064815</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14974,7 +14969,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46087.63653935185</v>
+        <v>46087.72023148148</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15102,7 +15097,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46087.64090277778</v>
+        <v>46087.71609953704</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15166,7 +15161,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46087.64082175926</v>
+        <v>46087.72056712963</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15230,7 +15225,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46087.62266203704</v>
+        <v>46087.7046875</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15294,7 +15289,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46087.62743055556</v>
+        <v>46087.70430555556</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15358,7 +15353,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46087.63539351852</v>
+        <v>46087.71447916667</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15422,7 +15417,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46087.62538194445</v>
+        <v>46087.70548611111</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15486,7 +15481,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46087.63728009259</v>
+        <v>46087.71394675926</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15550,7 +15545,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46087.63693287037</v>
+        <v>46087.71673611111</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15614,7 +15609,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46087.6403125</v>
+        <v>46087.72085648148</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15678,7 +15673,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46087.61538194444</v>
+        <v>46087.73145833334</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15742,7 +15737,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46087.63736111111</v>
+        <v>46087.72001157407</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15806,7 +15801,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46087.63434027778</v>
+        <v>46087.71019675926</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15870,7 +15865,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46087.6374537037</v>
+        <v>46087.71604166667</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15934,7 +15929,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46087.63295138889</v>
+        <v>46087.70902777778</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -15998,7 +15993,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46087.63715277778</v>
+        <v>46087.71568287037</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16062,7 +16057,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46087.63136574074</v>
+        <v>46087.71130787037</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16126,7 +16121,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46087.63802083334</v>
+        <v>46087.71560185185</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16249,7 +16244,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46087.63538194444</v>
+        <v>46087.71503472222</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16313,7 +16308,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46087.63150462963</v>
+        <v>46087.71284722222</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16377,7 +16372,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46087.63414351852</v>
+        <v>46087.71109953704</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16441,7 +16436,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46087.62725694444</v>
+        <v>46087.70344907408</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16505,7 +16500,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46087.63305555555</v>
+        <v>46087.70541666666</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16524,11 +16519,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C249" t="inlineStr">
-        <is>
-          <t>10.69.5.118</t>
-        </is>
-      </c>
       <c r="D249" t="n">
         <v>2017</v>
       </c>
@@ -16569,7 +16559,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46087.6290162037</v>
+        <v>46087.70439814815</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16633,7 +16623,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46087.62063657407</v>
+        <v>46087.69905092593</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16697,7 +16687,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46087.63546296296</v>
+        <v>46087.71181712963</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16761,7 +16751,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46087.63716435185</v>
+        <v>46087.73028935185</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16819,7 +16809,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46087.63681712963</v>
+        <v>46087.71334490741</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16883,7 +16873,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46087.64069444445</v>
+        <v>46087.72175925926</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16947,7 +16937,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46087.63837962963</v>
+        <v>46087.716875</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -17011,7 +17001,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46087.62148148148</v>
+        <v>46087.69969907407</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17075,7 +17065,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46087.64539351852</v>
+        <v>46087.71959490741</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17139,7 +17129,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46087.6346412037</v>
+        <v>46087.71172453704</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17267,7 +17257,7 @@
         <v>2</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46087.62413194445</v>
+        <v>46087.66247685185</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17331,7 +17321,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46087.63928240741</v>
+        <v>46087.72134259259</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17395,7 +17385,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46087.64291666666</v>
+        <v>46087.71927083333</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17459,7 +17449,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46087.63813657407</v>
+        <v>46087.70952546296</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17523,7 +17513,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46087.63329861111</v>
+        <v>46087.73209490741</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17587,7 +17577,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46087.63685185185</v>
+        <v>46087.67918981481</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17651,7 +17641,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46087.64886574074</v>
+        <v>46087.72723379629</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17715,7 +17705,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46087.57641203704</v>
+        <v>46087.72226851852</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17779,7 +17769,7 @@
         <v>1</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46087.63702546297</v>
+        <v>46087.70690972222</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17840,7 +17830,7 @@
         </is>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46087.61456018518</v>
+        <v>46087.72869212963</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -18093,7 +18083,7 @@
         </is>
       </c>
       <c r="N273" s="3" t="n">
-        <v>46087.6540625</v>
+        <v>46087.73126157407</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -18341,7 +18331,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46087.63469907407</v>
+        <v>46087.67123842592</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18405,7 +18395,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46087.62219907407</v>
+        <v>46087.73780092593</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18547,6 +18537,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>10.69.5.151</t>
+        </is>
+      </c>
       <c r="D281" t="n">
         <v>2017</v>
       </c>
@@ -18587,7 +18582,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46087.62858796296</v>
+        <v>46087.70546296296</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18651,7 +18646,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46087.64358796296</v>
+        <v>46087.720625</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18715,7 +18710,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46087.63805555556</v>
+        <v>46087.71306712963</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18779,7 +18774,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46087.63228009259</v>
+        <v>46087.71277777778</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -19030,7 +19025,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46087.63836805556</v>
+        <v>46087.71620370371</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19824,7 +19819,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46087.62508101852</v>
+        <v>46087.70596064815</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20940,7 +20935,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46087.63081018518</v>
+        <v>46087.71385416666</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21665,7 +21660,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46087.64071759259</v>
+        <v>46087.71634259259</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21729,7 +21724,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46087.63045138889</v>
+        <v>46087.70870370371</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21793,7 +21788,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46087.63626157407</v>
+        <v>46087.71679398148</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21857,7 +21852,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46087.62143518519</v>
+        <v>46087.69950231481</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21985,7 +21980,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46087.63373842592</v>
+        <v>46087.71552083334</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22049,7 +22044,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46087.62028935185</v>
+        <v>46087.73717592593</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22113,7 +22108,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46087.63026620371</v>
+        <v>46087.70980324074</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -23758,7 +23753,7 @@
         <v>1</v>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46087.64725694444</v>
+        <v>46087.68658564815</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23824,7 +23819,7 @@
         </is>
       </c>
       <c r="N365" s="3" t="n">
-        <v>46087.62270833334</v>
+        <v>46087.73768518519</v>
       </c>
       <c r="O365" t="inlineStr">
         <is>
@@ -23950,7 +23945,7 @@
         </is>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46087.63309027778</v>
+        <v>46087.71225694445</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -24011,7 +24006,7 @@
         </is>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46087.62934027778</v>
+        <v>46087.66454861111</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24080,7 +24075,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46087.63916666667</v>
+        <v>46087.71697916667</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24108,7 +24103,7 @@
         <v>2</v>
       </c>
       <c r="N370" s="3" t="n">
-        <v>46087.63688657407</v>
+        <v>46087.67818287037</v>
       </c>
       <c r="O370" t="inlineStr">
         <is>
@@ -24177,7 +24172,7 @@
         <v>1</v>
       </c>
       <c r="N371" s="3" t="n">
-        <v>46076.49737268518</v>
+        <v>46087.67106481481</v>
       </c>
       <c r="O371" t="inlineStr">
         <is>
@@ -24381,7 +24376,7 @@
         </is>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46087.62596064815</v>
+        <v>46087.70216435185</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24400,6 +24395,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>10.69.3.72</t>
+        </is>
+      </c>
       <c r="D375" t="n">
         <v>2025</v>
       </c>
@@ -24445,7 +24445,7 @@
         <v>1</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46087.64563657407</v>
+        <v>46087.72414351852</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24514,7 +24514,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46087.65140046296</v>
+        <v>46087.68934027778</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -24583,7 +24583,7 @@
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46087.65325231481</v>
+        <v>46087.73127314815</v>
       </c>
       <c r="O377" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-09 07:52:06.031910
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46087.73710648148</v>
+        <v>46090.29980324074</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46087.69759259259</v>
+        <v>46087.8165625</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -1382,7 +1382,7 @@
         <v>2</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>46087.6994675926</v>
+        <v>46087.86063657407</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46087.70715277778</v>
+        <v>46090.31267361111</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>46087.71460648148</v>
+        <v>46090.14413194444</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -1943,7 +1943,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46087.73119212963</v>
+        <v>46090.16956018518</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -1962,11 +1962,6 @@
           <t>AUDITORIO</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>10.69.3.153</t>
-        </is>
-      </c>
       <c r="D24" t="n">
         <v>2019</v>
       </c>
@@ -2004,7 +1999,7 @@
         </is>
       </c>
       <c r="N24" s="3" t="n">
-        <v>46087.73737268519</v>
+        <v>46090.13822916667</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2082,6 +2077,11 @@
           <t>AUDITORIO</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>10.69.3.151</t>
+        </is>
+      </c>
       <c r="D26" t="n">
         <v>2019</v>
       </c>
@@ -2122,7 +2122,7 @@
         <v>1</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>46087.70180555555</v>
+        <v>46090.17209490741</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -6578,7 +6578,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46087.71918981482</v>
+        <v>46087.83966435185</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6844,7 +6844,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46087.71994212963</v>
+        <v>46090.30262731481</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6913,7 +6913,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46087.71275462963</v>
+        <v>46088.59695601852</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -7051,7 +7051,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46087.68898148148</v>
+        <v>46088.60329861111</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7446,7 +7446,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46087.71005787037</v>
+        <v>46090.28568287037</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7515,7 +7515,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46087.70512731482</v>
+        <v>46090.32047453704</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7722,7 +7722,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46087.73318287037</v>
+        <v>46090.31591435185</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7791,7 +7791,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46087.72094907407</v>
+        <v>46090.31212962963</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -8199,7 +8199,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46087.70304398148</v>
+        <v>46087.74436342593</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8268,7 +8268,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46087.72896990741</v>
+        <v>46088.61251157407</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8334,7 +8334,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46087.72768518519</v>
+        <v>46090.31922453704</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8403,7 +8403,7 @@
         <v>2</v>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46087.70310185185</v>
+        <v>46087.82344907407</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8472,7 +8472,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46087.72328703704</v>
+        <v>46090.30061342593</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8541,7 +8541,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46087.71267361111</v>
+        <v>46090.29096064815</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8610,7 +8610,7 @@
         <v>2</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46087.73445601852</v>
+        <v>46087.77148148148</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8748,7 +8748,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46087.68458333334</v>
+        <v>46090.30380787037</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8817,7 +8817,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46087.7331712963</v>
+        <v>46090.28020833333</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -9083,7 +9083,7 @@
         <v>1</v>
       </c>
       <c r="N132" s="3" t="n">
-        <v>46087.73434027778</v>
+        <v>46087.81547453703</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -9147,7 +9147,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46087.72619212963</v>
+        <v>46087.8700462963</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9211,7 +9211,7 @@
         <v>1</v>
       </c>
       <c r="N134" s="3" t="n">
-        <v>46087.73508101852</v>
+        <v>46088.5984375</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -9275,7 +9275,7 @@
         <v>1</v>
       </c>
       <c r="N135" s="3" t="n">
-        <v>46087.71533564815</v>
+        <v>46088.59762731481</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -9402,7 +9402,7 @@
         <v>1</v>
       </c>
       <c r="N137" s="3" t="n">
-        <v>46087.71581018518</v>
+        <v>46088.60962962963</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -9466,7 +9466,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46087.7365162037</v>
+        <v>46088.59219907408</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9530,7 +9530,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46087.69837962963</v>
+        <v>46090.29394675926</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9594,7 +9594,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46087.71070601852</v>
+        <v>46088.61628472222</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9658,7 +9658,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46087.73444444445</v>
+        <v>46088.60600694444</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9722,7 +9722,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46087.69974537037</v>
+        <v>46088.60040509259</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9786,7 +9786,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46087.69857638889</v>
+        <v>46088.61736111111</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9850,7 +9850,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46087.73673611111</v>
+        <v>46088.58673611111</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9914,7 +9914,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46087.70326388889</v>
+        <v>46088.86951388889</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9978,7 +9978,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46087.72910879629</v>
+        <v>46088.59783564815</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10042,7 +10042,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46087.72172453703</v>
+        <v>46088.58641203704</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10106,7 +10106,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46087.72204861111</v>
+        <v>46088.51835648148</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10234,7 +10234,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46087.70431712963</v>
+        <v>46088.59010416667</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10298,7 +10298,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46087.73606481482</v>
+        <v>46088.58695601852</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10317,11 +10317,6 @@
           <t>OPERACAO 7.1</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>10.69.5.21</t>
-        </is>
-      </c>
       <c r="D152" t="n">
         <v>2018</v>
       </c>
@@ -10362,7 +10357,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46087.72533564815</v>
+        <v>46088.58136574074</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10426,7 +10421,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46087.54515046296</v>
+        <v>46088.60319444445</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10490,7 +10485,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46087.70686342593</v>
+        <v>46088.53472222222</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10554,7 +10549,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46087.71893518518</v>
+        <v>46090.31887731481</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10618,7 +10613,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46087.57607638889</v>
+        <v>46088.60349537037</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10682,7 +10677,7 @@
         <v>1</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>46087.72265046297</v>
+        <v>46090.29743055555</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -10746,7 +10741,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46087.72472222222</v>
+        <v>46088.60368055556</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10810,7 +10805,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46087.71253472222</v>
+        <v>46090.30939814815</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10874,7 +10869,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46087.57236111111</v>
+        <v>46088.85196759259</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10938,7 +10933,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46087.71283564815</v>
+        <v>46088.58459490741</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -11002,7 +10997,7 @@
         <v>1</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46087.72118055556</v>
+        <v>46090.31887731481</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11063,10 +11058,10 @@
         </is>
       </c>
       <c r="M163" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46087.71371527778</v>
+        <v>46090.28650462963</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11127,10 +11122,10 @@
         </is>
       </c>
       <c r="M164" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46087.59200231481</v>
+        <v>46088.61319444444</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11191,10 +11186,10 @@
         </is>
       </c>
       <c r="M165" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46087.63283564815</v>
+        <v>46088.6059375</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11255,10 +11250,10 @@
         </is>
       </c>
       <c r="M166" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46087.67258101852</v>
+        <v>46088.4655787037</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11319,10 +11314,10 @@
         </is>
       </c>
       <c r="M167" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46087.55251157407</v>
+        <v>46088.58702546296</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11386,7 +11381,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46087.70993055555</v>
+        <v>46090.29378472222</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11450,7 +11445,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46087.71189814815</v>
+        <v>46088.44020833333</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11514,7 +11509,7 @@
         <v>1</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46087.70204861111</v>
+        <v>46088.5199074074</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11578,7 +11573,7 @@
         <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46087.57952546296</v>
+        <v>46088.52197916667</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11642,7 +11637,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46087.72540509259</v>
+        <v>46090.30262731481</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11770,7 +11765,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46087.71304398148</v>
+        <v>46090.29503472222</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11834,7 +11829,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46087.65417824074</v>
+        <v>46088.53381944444</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11898,7 +11893,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46087.73550925926</v>
+        <v>46088.54965277778</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11962,7 +11957,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46087.70506944445</v>
+        <v>46090.28873842592</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12026,7 +12021,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46087.70556712963</v>
+        <v>46088.57225694445</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12090,7 +12085,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46087.70144675926</v>
+        <v>46088.59194444444</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12154,7 +12149,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46087.71542824074</v>
+        <v>46088.58446759259</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12218,7 +12213,7 @@
         <v>1</v>
       </c>
       <c r="N181" s="3" t="n">
-        <v>46084.83988425926</v>
+        <v>46088.45335648148</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
@@ -12415,7 +12410,7 @@
         <v>1</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46086.48731481482</v>
+        <v>46088.60638888889</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12479,7 +12474,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46087.71947916667</v>
+        <v>46088.61560185185</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12543,7 +12538,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46087.72790509259</v>
+        <v>46088.6009375</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12607,7 +12602,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46087.72721064815</v>
+        <v>46088.58944444444</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12735,7 +12730,7 @@
         </is>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46087.71405092593</v>
+        <v>46088.61644675926</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12799,7 +12794,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46087.72731481482</v>
+        <v>46088.58231481481</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12863,7 +12858,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46087.71246527778</v>
+        <v>46090.30956018518</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12988,7 +12983,7 @@
         <v>2</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46087.56983796296</v>
+        <v>46088.58457175926</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13052,7 +13047,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46087.7158449074</v>
+        <v>46088.59546296296</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13116,7 +13111,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46087.72091435185</v>
+        <v>46088.57453703704</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13180,7 +13175,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46087.71951388889</v>
+        <v>46088.36734953704</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13244,7 +13239,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46087.70222222222</v>
+        <v>46088.43388888889</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13308,7 +13303,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46087.7000462963</v>
+        <v>46088.58556712963</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13372,7 +13367,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46087.70912037037</v>
+        <v>46088.58918981482</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13433,7 +13428,7 @@
         </is>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46087.71328703704</v>
+        <v>46088.61820601852</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13497,7 +13492,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46087.71940972222</v>
+        <v>46088.60704861111</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13561,7 +13556,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46087.72498842593</v>
+        <v>46090.2930787037</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13625,7 +13620,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46087.71241898148</v>
+        <v>46088.84238425926</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13689,7 +13684,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46087.73590277778</v>
+        <v>46088.60763888889</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13753,7 +13748,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46087.72247685185</v>
+        <v>46090.29928240741</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13817,7 +13812,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46087.72416666667</v>
+        <v>46088.53893518518</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13881,7 +13876,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46087.64363425926</v>
+        <v>46088.39084490741</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13945,7 +13940,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46087.71376157407</v>
+        <v>46088.60732638889</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14009,7 +14004,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46087.70414351852</v>
+        <v>46088.60747685185</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14073,7 +14068,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46087.73555555556</v>
+        <v>46088.5837962963</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14137,7 +14132,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46087.70673611111</v>
+        <v>46088.5515625</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14201,7 +14196,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46087.72103009259</v>
+        <v>46088.59747685185</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14265,7 +14260,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46087.71949074074</v>
+        <v>46090.29174768519</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14329,7 +14324,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46087.71894675926</v>
+        <v>46088.48796296296</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14393,7 +14388,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46087.71212962963</v>
+        <v>46088.59248842593</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14412,6 +14407,11 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>10.69.5.85</t>
+        </is>
+      </c>
       <c r="D216" t="n">
         <v>2017</v>
       </c>
@@ -14452,7 +14452,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46087.71380787037</v>
+        <v>46088.61150462963</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14516,7 +14516,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46087.72438657407</v>
+        <v>46088.60881944445</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14580,7 +14580,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46087.71696759259</v>
+        <v>46088.5840625</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14649,7 +14649,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46087.70733796297</v>
+        <v>46088.8556712963</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14713,7 +14713,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46087.72949074074</v>
+        <v>46088.62061342593</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14777,7 +14777,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46087.72635416667</v>
+        <v>46088.60734953704</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14841,7 +14841,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46087.70270833333</v>
+        <v>46088.58564814815</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14905,7 +14905,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46087.72971064815</v>
+        <v>46088.61790509259</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14969,7 +14969,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46087.72023148148</v>
+        <v>46088.43309027778</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15033,7 +15033,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46087.64077546296</v>
+        <v>46088.45923611111</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15097,7 +15097,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46087.71609953704</v>
+        <v>46088.60763888889</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15161,7 +15161,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46087.72056712963</v>
+        <v>46088.83965277778</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15225,7 +15225,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46087.7046875</v>
+        <v>46088.60953703704</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15289,7 +15289,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46087.70430555556</v>
+        <v>46090.31701388889</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15353,7 +15353,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46087.71447916667</v>
+        <v>46090.31739583334</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15417,7 +15417,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46087.70548611111</v>
+        <v>46088.55649305556</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15481,7 +15481,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46087.71394675926</v>
+        <v>46088.554375</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15545,7 +15545,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46087.71673611111</v>
+        <v>46088.61326388889</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15609,7 +15609,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46087.72085648148</v>
+        <v>46088.87041666666</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15673,7 +15673,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46087.73145833334</v>
+        <v>46088.49489583333</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15737,7 +15737,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46087.72001157407</v>
+        <v>46090.31053240741</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15801,7 +15801,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46087.71019675926</v>
+        <v>46088.61842592592</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15865,7 +15865,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46087.71604166667</v>
+        <v>46088.60164351852</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15929,7 +15929,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46087.70902777778</v>
+        <v>46088.5824537037</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -15993,7 +15993,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46087.71568287037</v>
+        <v>46088.50724537037</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16057,7 +16057,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46087.71130787037</v>
+        <v>46088.56922453704</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16121,7 +16121,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46087.71560185185</v>
+        <v>46088.59137731481</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16180,7 +16180,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46087.20488425926</v>
+        <v>46090.12857638889</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16244,7 +16244,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46087.71503472222</v>
+        <v>46088.58771990741</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16308,7 +16308,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46087.71284722222</v>
+        <v>46088.55318287037</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16372,7 +16372,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46087.71109953704</v>
+        <v>46088.59403935185</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16436,7 +16436,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46087.70344907408</v>
+        <v>46088.56605324074</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16500,7 +16500,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46087.70541666666</v>
+        <v>46088.5840625</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16519,6 +16519,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>10.69.5.118</t>
+        </is>
+      </c>
       <c r="D249" t="n">
         <v>2017</v>
       </c>
@@ -16559,7 +16564,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46087.70439814815</v>
+        <v>46088.58399305555</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16623,7 +16628,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46087.69905092593</v>
+        <v>46088.5468287037</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16687,7 +16692,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46087.71181712963</v>
+        <v>46088.59533564815</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16751,7 +16756,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46087.73028935185</v>
+        <v>46090.31918981481</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16809,7 +16814,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46087.71334490741</v>
+        <v>46090.31980324074</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16873,7 +16878,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46087.72175925926</v>
+        <v>46090.31901620371</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16937,7 +16942,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46087.716875</v>
+        <v>46090.31956018518</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -17001,7 +17006,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46087.69969907407</v>
+        <v>46090.31952546296</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17065,7 +17070,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46087.71959490741</v>
+        <v>46088.58796296296</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17129,7 +17134,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46087.71172453704</v>
+        <v>46090.28453703703</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17193,7 +17198,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46087.59630787037</v>
+        <v>46090.3200462963</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17257,7 +17262,7 @@
         <v>2</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46087.66247685185</v>
+        <v>46088.59049768518</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17321,7 +17326,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46087.72134259259</v>
+        <v>46088.59612268519</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17385,7 +17390,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46087.71927083333</v>
+        <v>46088.58460648148</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17449,7 +17454,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46087.70952546296</v>
+        <v>46089.88878472222</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17513,7 +17518,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46087.73209490741</v>
+        <v>46088.84206018518</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17577,7 +17582,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46087.67918981481</v>
+        <v>46088.59836805556</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17641,7 +17646,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46087.72723379629</v>
+        <v>46088.6061574074</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17705,7 +17710,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46087.72226851852</v>
+        <v>46088.60243055555</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17769,7 +17774,7 @@
         <v>1</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46087.70690972222</v>
+        <v>46088.86300925926</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17830,7 +17835,7 @@
         </is>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46087.72869212963</v>
+        <v>46090.29003472222</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17958,7 +17963,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46087.61518518518</v>
+        <v>46088.52164351852</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -18083,7 +18088,7 @@
         </is>
       </c>
       <c r="N273" s="3" t="n">
-        <v>46087.73126157407</v>
+        <v>46088.35070601852</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -18331,7 +18336,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46087.67123842592</v>
+        <v>46090.3134375</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18395,7 +18400,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46087.73780092593</v>
+        <v>46088.5422337963</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18454,7 +18459,7 @@
         <v>2</v>
       </c>
       <c r="N279" s="3" t="n">
-        <v>46085.82259259259</v>
+        <v>46088.61597222222</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -18518,7 +18523,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46086.55077546297</v>
+        <v>46088.61046296296</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18537,11 +18542,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C281" t="inlineStr">
-        <is>
-          <t>10.69.5.151</t>
-        </is>
-      </c>
       <c r="D281" t="n">
         <v>2017</v>
       </c>
@@ -18582,7 +18582,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46087.70546296296</v>
+        <v>46088.54785879629</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18646,7 +18646,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46087.720625</v>
+        <v>46088.44447916667</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18710,7 +18710,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46087.71306712963</v>
+        <v>46088.59975694444</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18774,7 +18774,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46087.71277777778</v>
+        <v>46088.60165509259</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18833,7 +18833,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46087.56849537037</v>
+        <v>46088.60002314814</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18897,7 +18897,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46087.56427083333</v>
+        <v>46088.61594907408</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18961,7 +18961,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46087.55752314815</v>
+        <v>46090.3156712963</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19025,7 +19025,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46087.71620370371</v>
+        <v>46088.58370370371</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19819,7 +19819,7 @@
         <v>1</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>46087.70596064815</v>
+        <v>46090.28481481481</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -20935,7 +20935,7 @@
         </is>
       </c>
       <c r="N319" s="3" t="n">
-        <v>46087.71385416666</v>
+        <v>46090.30978009259</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -21660,7 +21660,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46087.71634259259</v>
+        <v>46088.51744212963</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21724,7 +21724,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46087.70870370371</v>
+        <v>46090.31047453704</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21788,7 +21788,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46087.71679398148</v>
+        <v>46090.31702546297</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21852,7 +21852,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46087.69950231481</v>
+        <v>46090.30957175926</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21913,10 +21913,10 @@
         </is>
       </c>
       <c r="M335" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46087.5483912037</v>
+        <v>46090.28642361111</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21980,7 +21980,7 @@
         <v>1</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46087.71552083334</v>
+        <v>46090.29456018518</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22044,7 +22044,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46087.73717592593</v>
+        <v>46090.30912037037</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22108,7 +22108,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46087.70980324074</v>
+        <v>46090.28839120371</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -23819,7 +23819,7 @@
         </is>
       </c>
       <c r="N365" s="3" t="n">
-        <v>46087.73768518519</v>
+        <v>46090.30744212963</v>
       </c>
       <c r="O365" t="inlineStr">
         <is>
@@ -24075,7 +24075,7 @@
         <v>1</v>
       </c>
       <c r="N369" s="3" t="n">
-        <v>46087.71697916667</v>
+        <v>46090.28827546296</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -24376,7 +24376,7 @@
         </is>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46087.70216435185</v>
+        <v>46090.30547453704</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24445,7 +24445,7 @@
         <v>1</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46087.72414351852</v>
+        <v>46087.80133101852</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24583,7 +24583,7 @@
         <v>2</v>
       </c>
       <c r="N377" s="3" t="n">
-        <v>46087.73127314815</v>
+        <v>46090.28010416667</v>
       </c>
       <c r="O377" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-09 11:52:09.383907
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46090.37974537037</v>
+        <v>46090.45412037037</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46090.40284722222</v>
+        <v>46090.47649305555</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46090.37517361111</v>
+        <v>46090.48756944444</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46090.37946759259</v>
+        <v>46090.46172453704</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>46090.3903587963</v>
+        <v>46090.46604166667</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -6504,7 +6504,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46090.39663194444</v>
+        <v>46090.47288194444</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6573,7 +6573,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46087.83966435185</v>
+        <v>46090.4837962963</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6592,6 +6592,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>10.69.3.93</t>
+        </is>
+      </c>
       <c r="D96" t="n">
         <v>2025</v>
       </c>
@@ -6637,7 +6642,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46090.36844907407</v>
+        <v>46090.48045138889</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6656,11 +6661,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>10.69.3.94</t>
-        </is>
-      </c>
       <c r="D97" t="n">
         <v>2025</v>
       </c>
@@ -6706,7 +6706,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46090.37363425926</v>
+        <v>46090.45501157407</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6775,7 +6775,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46087.68961805556</v>
+        <v>46090.46496527778</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6844,7 +6844,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46090.37914351852</v>
+        <v>46090.46071759259</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6913,7 +6913,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46090.39474537037</v>
+        <v>46090.47021990741</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6982,7 +6982,7 @@
         <v>1</v>
       </c>
       <c r="N101" s="3" t="n">
-        <v>46080.71074074074</v>
+        <v>46090.45045138889</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -7051,7 +7051,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46088.60329861111</v>
+        <v>46090.45805555556</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7446,7 +7446,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46090.39832175926</v>
+        <v>46090.47803240741</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7515,7 +7515,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46090.39861111111</v>
+        <v>46090.47464120371</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7584,7 +7584,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46090.38730324074</v>
+        <v>46090.46525462963</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7653,7 +7653,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46090.37655092592</v>
+        <v>46090.45453703704</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7722,7 +7722,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46090.39859953704</v>
+        <v>46090.47391203704</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7791,7 +7791,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46090.39049768518</v>
+        <v>46090.47321759259</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7857,7 +7857,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46090.38151620371</v>
+        <v>46090.45671296296</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7926,7 +7926,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46090.36736111111</v>
+        <v>46090.48581018519</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7995,7 +7995,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46090.36989583333</v>
+        <v>46090.485625</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8061,7 +8061,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46090.36998842593</v>
+        <v>46090.44938657407</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8199,7 +8199,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46090.38668981481</v>
+        <v>46090.46096064815</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8268,7 +8268,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46088.61251157407</v>
+        <v>46090.47129629629</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8334,7 +8334,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46090.39684027778</v>
+        <v>46090.47939814815</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8472,7 +8472,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46090.3750462963</v>
+        <v>46090.45180555555</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8541,7 +8541,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46090.36657407408</v>
+        <v>46090.48523148148</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8679,7 +8679,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46090.39489583333</v>
+        <v>46090.46765046296</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8748,7 +8748,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46090.38628472222</v>
+        <v>46090.46331018519</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8817,7 +8817,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46090.40008101852</v>
+        <v>46090.47284722222</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8886,7 +8886,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46090.38271990741</v>
+        <v>46090.46710648148</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -9083,7 +9083,7 @@
         <v>1</v>
       </c>
       <c r="N132" s="3" t="n">
-        <v>46090.37586805555</v>
+        <v>46090.48788194444</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -9530,7 +9530,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46090.37236111111</v>
+        <v>46090.45436342592</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9594,7 +9594,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46090.37381944444</v>
+        <v>46090.45221064815</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9658,7 +9658,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46090.3834375</v>
+        <v>46090.455</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9722,7 +9722,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46090.37887731481</v>
+        <v>46090.45878472222</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9786,7 +9786,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46090.36759259259</v>
+        <v>46090.4878125</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9850,7 +9850,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46090.39262731482</v>
+        <v>46090.46719907408</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9914,7 +9914,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46090.40001157407</v>
+        <v>46090.47501157408</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9978,7 +9978,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46090.40239583333</v>
+        <v>46090.48126157407</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10106,7 +10106,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46090.37550925926</v>
+        <v>46090.45182870371</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10234,7 +10234,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46090.37564814815</v>
+        <v>46090.45149305555</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10298,7 +10298,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46090.37456018518</v>
+        <v>46090.48530092592</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10362,7 +10362,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46090.39922453704</v>
+        <v>46090.47851851852</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10426,7 +10426,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46090.36951388889</v>
+        <v>46090.45194444444</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10490,7 +10490,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46088.53472222222</v>
+        <v>46090.44793981482</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10554,7 +10554,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46090.39431712963</v>
+        <v>46090.47112268519</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10618,7 +10618,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46090.37207175926</v>
+        <v>46090.45458333333</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10746,7 +10746,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46088.60368055556</v>
+        <v>46090.45100694444</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10810,7 +10810,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46090.38392361111</v>
+        <v>46090.46099537037</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10874,7 +10874,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46090.37930555556</v>
+        <v>46090.45674768519</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10938,7 +10938,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46090.3717824074</v>
+        <v>46090.45303240741</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -11002,7 +11002,7 @@
         <v>1</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46090.39398148148</v>
+        <v>46090.47417824074</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11066,7 +11066,7 @@
         <v>2</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46090.40053240741</v>
+        <v>46090.48076388889</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11130,7 +11130,7 @@
         <v>1</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46088.61319444444</v>
+        <v>46090.48737268519</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11191,10 +11191,10 @@
         </is>
       </c>
       <c r="M165" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46088.6059375</v>
+        <v>46090.45337962963</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11255,10 +11255,10 @@
         </is>
       </c>
       <c r="M166" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46090.37130787037</v>
+        <v>46090.44980324074</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11322,7 +11322,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46090.40260416667</v>
+        <v>46090.47825231482</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11386,7 +11386,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46090.3712962963</v>
+        <v>46090.45114583334</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11450,7 +11450,7 @@
         <v>2</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>46090.37094907407</v>
+        <v>46090.48653935185</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -11511,10 +11511,10 @@
         </is>
       </c>
       <c r="M170" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46090.36553240741</v>
+        <v>46090.48094907407</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11639,10 +11639,10 @@
         </is>
       </c>
       <c r="M172" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46090.38180555555</v>
+        <v>46090.45539351852</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11706,7 +11706,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46090.38394675926</v>
+        <v>46090.46210648148</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11770,7 +11770,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46090.37184027778</v>
+        <v>46090.45342592592</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11834,7 +11834,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46088.53381944444</v>
+        <v>46090.4546412037</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11962,7 +11962,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46090.40002314815</v>
+        <v>46090.47353009259</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12026,7 +12026,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46090.38798611111</v>
+        <v>46090.46694444444</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12154,7 +12154,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="3" t="n">
-        <v>46090.37027777778</v>
+        <v>46090.48471064815</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -12543,7 +12543,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46090.37487268518</v>
+        <v>46090.45043981481</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12607,7 +12607,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="3" t="n">
-        <v>46090.37010416666</v>
+        <v>46090.45006944444</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -12735,7 +12735,7 @@
         </is>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46090.37245370371</v>
+        <v>46090.44832175926</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12799,7 +12799,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46090.37055555556</v>
+        <v>46090.44952546297</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12863,7 +12863,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="3" t="n">
-        <v>46090.38211805555</v>
+        <v>46090.45729166667</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -12988,7 +12988,7 @@
         <v>2</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46090.37215277777</v>
+        <v>46090.45216435185</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13052,7 +13052,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46090.40135416666</v>
+        <v>46090.47405092593</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13116,7 +13116,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46090.38050925926</v>
+        <v>46090.45902777778</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13180,7 +13180,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46090.38657407407</v>
+        <v>46090.46109953704</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13244,7 +13244,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46090.39967592592</v>
+        <v>46090.48063657407</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13372,7 +13372,7 @@
         <v>1</v>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46090.37893518519</v>
+        <v>46090.45289351852</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13497,7 +13497,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46090.37165509259</v>
+        <v>46090.48530092592</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13561,7 +13561,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46090.38435185186</v>
+        <v>46090.46032407408</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13625,7 +13625,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46090.40429398148</v>
+        <v>46090.4825</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13689,7 +13689,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46090.371875</v>
+        <v>46090.44986111111</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13753,7 +13753,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46090.38431712963</v>
+        <v>46090.46289351852</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13817,7 +13817,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46090.36351851852</v>
+        <v>46090.47856481482</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13881,7 +13881,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46090.38331018519</v>
+        <v>46090.46329861111</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13945,7 +13945,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46090.38103009259</v>
+        <v>46090.45568287037</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14009,7 +14009,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46090.37508101852</v>
+        <v>46090.48693287037</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14073,7 +14073,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46090.37689814815</v>
+        <v>46090.45638888889</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14137,7 +14137,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46090.37707175926</v>
+        <v>46090.45810185185</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14201,7 +14201,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46090.38543981482</v>
+        <v>46090.4612037037</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14393,7 +14393,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46090.37921296297</v>
+        <v>46090.45645833333</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14452,7 +14452,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46090.37835648148</v>
+        <v>46090.45173611111</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14516,7 +14516,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46090.378125</v>
+        <v>46090.45069444444</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14649,7 +14649,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46090.37508101852</v>
+        <v>46090.45056712963</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14713,7 +14713,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46090.38070601852</v>
+        <v>46090.46107638889</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14841,7 +14841,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46090.38002314815</v>
+        <v>46090.45951388889</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -15033,7 +15033,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46090.40248842593</v>
+        <v>46090.48190972222</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15097,7 +15097,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46090.39292824074</v>
+        <v>46090.47083333333</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15161,7 +15161,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46090.37194444444</v>
+        <v>46090.47982638889</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15289,7 +15289,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46090.39061342592</v>
+        <v>46090.46731481481</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15353,7 +15353,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46090.36712962963</v>
+        <v>46090.46701388889</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15417,7 +15417,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46090.36988425926</v>
+        <v>46090.48206018518</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15481,7 +15481,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46090.37457175926</v>
+        <v>46090.45085648148</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15545,7 +15545,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46090.40234953703</v>
+        <v>46090.4804050926</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15609,7 +15609,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46090.37608796296</v>
+        <v>46090.45319444445</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15673,7 +15673,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46090.38928240741</v>
+        <v>46090.4609837963</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15737,7 +15737,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46090.38995370371</v>
+        <v>46090.46758101852</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15801,7 +15801,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46090.37258101852</v>
+        <v>46090.48751157407</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15865,7 +15865,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46090.40368055556</v>
+        <v>46090.47623842592</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15929,7 +15929,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46090.37827546296</v>
+        <v>46090.45931712963</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -16057,7 +16057,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46090.37002314815</v>
+        <v>46090.48657407407</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16121,7 +16121,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46090.36946759259</v>
+        <v>46090.44804398148</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16180,7 +16180,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46090.12857638889</v>
+        <v>46090.44866898148</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16244,7 +16244,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46090.40225694444</v>
+        <v>46090.48082175926</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16308,7 +16308,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46090.3656712963</v>
+        <v>46090.4868287037</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16372,7 +16372,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46090.36618055555</v>
+        <v>46090.4471875</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16436,7 +16436,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46090.36708333333</v>
+        <v>46090.4493287037</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16500,7 +16500,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46090.40380787037</v>
+        <v>46090.47744212963</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16519,6 +16519,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>10.69.5.118</t>
+        </is>
+      </c>
       <c r="D249" t="n">
         <v>2017</v>
       </c>
@@ -16559,7 +16564,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46090.36596064815</v>
+        <v>46090.48304398148</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16623,7 +16628,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46090.40324074074</v>
+        <v>46090.48450231482</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16751,7 +16756,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46090.38931712963</v>
+        <v>46090.46971064815</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16809,7 +16814,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46090.39234953704</v>
+        <v>46090.470625</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16873,7 +16878,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46090.40078703704</v>
+        <v>46090.47990740741</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16937,7 +16942,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46090.39976851852</v>
+        <v>46090.4734375</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -17001,7 +17006,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46090.40006944445</v>
+        <v>46090.48413194445</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17065,7 +17070,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46090.38621527778</v>
+        <v>46090.42594907407</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17129,7 +17134,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46090.39996527778</v>
+        <v>46090.47879629629</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17193,7 +17198,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46090.40158564815</v>
+        <v>46090.48262731481</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17257,7 +17262,7 @@
         <v>2</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46090.39957175926</v>
+        <v>46090.48252314814</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17385,7 +17390,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46090.37681712963</v>
+        <v>46090.44974537037</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17449,7 +17454,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46090.39878472222</v>
+        <v>46090.47267361111</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17513,7 +17518,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46090.37135416667</v>
+        <v>46090.48366898148</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17577,7 +17582,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46090.37425925926</v>
+        <v>46090.44895833333</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17641,7 +17646,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46090.37541666667</v>
+        <v>46090.45717592593</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17705,7 +17710,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46090.40260416667</v>
+        <v>46090.48178240741</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17769,7 +17774,7 @@
         <v>1</v>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46088.86300925926</v>
+        <v>46090.45674768519</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17830,7 +17835,7 @@
         </is>
       </c>
       <c r="N269" s="3" t="n">
-        <v>46090.37269675926</v>
+        <v>46090.45261574074</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -17958,7 +17963,7 @@
         <v>1</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>46090.38866898148</v>
+        <v>46090.46354166666</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -18331,7 +18336,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46090.39206018519</v>
+        <v>46090.46824074074</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18395,7 +18400,7 @@
         <v>1</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>46090.39060185185</v>
+        <v>46090.47189814815</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18518,7 +18523,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46090.38333333333</v>
+        <v>46090.46230324074</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18537,11 +18542,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C281" t="inlineStr">
-        <is>
-          <t>10.69.5.151</t>
-        </is>
-      </c>
       <c r="D281" t="n">
         <v>2017</v>
       </c>
@@ -18582,7 +18582,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46090.37954861111</v>
+        <v>46090.45940972222</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18646,7 +18646,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46090.39873842592</v>
+        <v>46090.47476851852</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18710,7 +18710,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46090.37703703704</v>
+        <v>46090.45703703703</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18774,7 +18774,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46090.37979166667</v>
+        <v>46090.45995370371</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18838,7 +18838,7 @@
         <v>1</v>
       </c>
       <c r="N285" s="3" t="n">
-        <v>46090.37280092593</v>
+        <v>46090.44944444444</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -18966,7 +18966,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46090.39056712963</v>
+        <v>46090.47300925926</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19030,7 +19030,7 @@
         <v>1</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>46088.58370370371</v>
+        <v>46090.45885416667</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19463,7 +19463,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>PA_180</t>
+          <t>PA_181</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -19473,28 +19473,28 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>10.69.5.180</t>
+          <t>10.69.5.181</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="E296" t="n">
-        <v>22943</v>
+        <v>2956</v>
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>Microsoft Windows 7 Professional</t>
+          <t>Microsoft® Windows Vista™ Business</t>
         </is>
       </c>
       <c r="G296" t="inlineStr">
         <is>
-          <t>L1BH5GL</t>
+          <t>83FNLJ1</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
         <is>
-          <t>Intel Pentium®</t>
+          <t>Intel Core 2 Duo</t>
         </is>
       </c>
       <c r="J296" t="inlineStr">
@@ -19504,16 +19504,16 @@
       </c>
       <c r="K296" t="inlineStr">
         <is>
-          <t>LENOVO</t>
+          <t>Dell Inc.</t>
         </is>
       </c>
       <c r="L296" t="inlineStr">
         <is>
-          <t>ThinkCentre M58e</t>
+          <t>OptiPlex 755</t>
         </is>
       </c>
       <c r="N296" s="3" t="n">
-        <v>45908.87260416667</v>
+        <v>45937.37885416667</v>
       </c>
       <c r="O296" t="inlineStr">
         <is>
@@ -19524,7 +19524,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>PA_181</t>
+          <t>PA_183</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
@@ -19534,14 +19534,14 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>10.69.5.181</t>
+          <t>10.69.5.183</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="E297" t="n">
-        <v>2956</v>
+        <v>22943</v>
       </c>
       <c r="F297" t="inlineStr">
         <is>
@@ -19550,7 +19550,7 @@
       </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t>83FNLJ1</t>
+          <t>39CKZL1</t>
         </is>
       </c>
       <c r="I297" t="inlineStr">
@@ -19570,11 +19570,11 @@
       </c>
       <c r="L297" t="inlineStr">
         <is>
-          <t>OptiPlex 755</t>
+          <t>OptiPlex 360</t>
         </is>
       </c>
       <c r="N297" s="3" t="n">
-        <v>45937.37885416667</v>
+        <v>45932.63596064815</v>
       </c>
       <c r="O297" t="inlineStr">
         <is>
@@ -19585,7 +19585,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>PA_183</t>
+          <t>PA_184</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
@@ -19595,7 +19595,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>10.69.5.183</t>
+          <t>10.69.5.184</t>
         </is>
       </c>
       <c r="D298" t="n">
@@ -19611,7 +19611,7 @@
       </c>
       <c r="G298" t="inlineStr">
         <is>
-          <t>39CKZL1</t>
+          <t>GGCKZL1</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
@@ -19634,8 +19634,11 @@
           <t>OptiPlex 360</t>
         </is>
       </c>
+      <c r="M298" t="n">
+        <v>1</v>
+      </c>
       <c r="N298" s="3" t="n">
-        <v>45932.63596064815</v>
+        <v>45895.86393518518</v>
       </c>
       <c r="O298" t="inlineStr">
         <is>
@@ -19646,7 +19649,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>PA_184</t>
+          <t>PA_185</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
@@ -19656,14 +19659,14 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>10.69.5.184</t>
+          <t>10.69.5.185</t>
         </is>
       </c>
       <c r="D299" t="n">
         <v>2013</v>
       </c>
       <c r="E299" t="n">
-        <v>22943</v>
+        <v>3885</v>
       </c>
       <c r="F299" t="inlineStr">
         <is>
@@ -19672,7 +19675,7 @@
       </c>
       <c r="G299" t="inlineStr">
         <is>
-          <t>GGCKZL1</t>
+          <t>JW8QYD1</t>
         </is>
       </c>
       <c r="I299" t="inlineStr">
@@ -19692,14 +19695,11 @@
       </c>
       <c r="L299" t="inlineStr">
         <is>
-          <t>OptiPlex 360</t>
-        </is>
-      </c>
-      <c r="M299" t="n">
-        <v>1</v>
+          <t>OptiPlex 745</t>
+        </is>
       </c>
       <c r="N299" s="3" t="n">
-        <v>45895.86393518518</v>
+        <v>45932.62702546296</v>
       </c>
       <c r="O299" t="inlineStr">
         <is>
@@ -19710,7 +19710,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>PA_185</t>
+          <t>PA_186</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
@@ -19720,14 +19720,14 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>10.69.5.185</t>
+          <t>10.69.5.186</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="E300" t="n">
-        <v>3885</v>
+        <v>2956</v>
       </c>
       <c r="F300" t="inlineStr">
         <is>
@@ -19736,7 +19736,7 @@
       </c>
       <c r="G300" t="inlineStr">
         <is>
-          <t>JW8QYD1</t>
+          <t>814ZSG1</t>
         </is>
       </c>
       <c r="I300" t="inlineStr">
@@ -19746,7 +19746,7 @@
       </c>
       <c r="J300" t="inlineStr">
         <is>
-          <t>2 GB</t>
+          <t>4 GB</t>
         </is>
       </c>
       <c r="K300" t="inlineStr">
@@ -19756,11 +19756,14 @@
       </c>
       <c r="L300" t="inlineStr">
         <is>
-          <t>OptiPlex 745</t>
-        </is>
+          <t>OptiPlex 755</t>
+        </is>
+      </c>
+      <c r="M300" t="n">
+        <v>1</v>
       </c>
       <c r="N300" s="3" t="n">
-        <v>45932.62702546296</v>
+        <v>46090.48268518518</v>
       </c>
       <c r="O300" t="inlineStr">
         <is>
@@ -19771,7 +19774,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>PA_186</t>
+          <t>PA_188</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
@@ -19781,14 +19784,14 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>10.69.5.186</t>
+          <t>10.69.5.188</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="E301" t="n">
-        <v>2956</v>
+        <v>3995</v>
       </c>
       <c r="F301" t="inlineStr">
         <is>
@@ -19797,7 +19800,7 @@
       </c>
       <c r="G301" t="inlineStr">
         <is>
-          <t>814ZSG1</t>
+          <t>30KSSF1</t>
         </is>
       </c>
       <c r="I301" t="inlineStr">
@@ -19820,11 +19823,8 @@
           <t>OptiPlex 755</t>
         </is>
       </c>
-      <c r="M301" t="n">
-        <v>1</v>
-      </c>
       <c r="N301" s="3" t="n">
-        <v>46090.40366898148</v>
+        <v>45932.6643287037</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -19835,7 +19835,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>PA_188</t>
+          <t>PA_189</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
@@ -19845,14 +19845,14 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>10.69.5.188</t>
+          <t>10.69.5.189</t>
         </is>
       </c>
       <c r="D302" t="n">
-        <v>2013</v>
+        <v>2011</v>
       </c>
       <c r="E302" t="n">
-        <v>3995</v>
+        <v>7855</v>
       </c>
       <c r="F302" t="inlineStr">
         <is>
@@ -19861,7 +19861,7 @@
       </c>
       <c r="G302" t="inlineStr">
         <is>
-          <t>30KSSF1</t>
+          <t>L1AX8ZK</t>
         </is>
       </c>
       <c r="I302" t="inlineStr">
@@ -19871,21 +19871,21 @@
       </c>
       <c r="J302" t="inlineStr">
         <is>
-          <t>4 GB</t>
+          <t>2 GB</t>
         </is>
       </c>
       <c r="K302" t="inlineStr">
         <is>
-          <t>Dell Inc.</t>
+          <t>LENOVO</t>
         </is>
       </c>
       <c r="L302" t="inlineStr">
         <is>
-          <t>OptiPlex 755</t>
+          <t>ThinkCentre A55</t>
         </is>
       </c>
       <c r="N302" s="3" t="n">
-        <v>45932.6643287037</v>
+        <v>46066.15606481482</v>
       </c>
       <c r="O302" t="inlineStr">
         <is>
@@ -19896,7 +19896,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>PA_189</t>
+          <t>PA_190</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
@@ -19906,7 +19906,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>10.69.5.189</t>
+          <t>10.69.5.190</t>
         </is>
       </c>
       <c r="D303" t="n">
@@ -19922,7 +19922,7 @@
       </c>
       <c r="G303" t="inlineStr">
         <is>
-          <t>L1AX8ZK</t>
+          <t>L1AW6LX</t>
         </is>
       </c>
       <c r="I303" t="inlineStr">
@@ -19945,8 +19945,11 @@
           <t>ThinkCentre A55</t>
         </is>
       </c>
+      <c r="M303" t="n">
+        <v>1</v>
+      </c>
       <c r="N303" s="3" t="n">
-        <v>46066.15606481482</v>
+        <v>46036.83804398148</v>
       </c>
       <c r="O303" t="inlineStr">
         <is>
@@ -19957,7 +19960,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>PA_190</t>
+          <t>PA_191</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
@@ -19967,14 +19970,14 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>10.69.5.190</t>
+          <t>10.69.5.191</t>
         </is>
       </c>
       <c r="D304" t="n">
         <v>2011</v>
       </c>
       <c r="E304" t="n">
-        <v>7855</v>
+        <v>5155</v>
       </c>
       <c r="F304" t="inlineStr">
         <is>
@@ -19983,7 +19986,7 @@
       </c>
       <c r="G304" t="inlineStr">
         <is>
-          <t>L1AW6LX</t>
+          <t>L1AW6TC</t>
         </is>
       </c>
       <c r="I304" t="inlineStr">
@@ -20006,11 +20009,8 @@
           <t>ThinkCentre A55</t>
         </is>
       </c>
-      <c r="M304" t="n">
-        <v>1</v>
-      </c>
       <c r="N304" s="3" t="n">
-        <v>46036.83804398148</v>
+        <v>46022.85438657407</v>
       </c>
       <c r="O304" t="inlineStr">
         <is>
@@ -20021,7 +20021,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>PA_191</t>
+          <t>PA_195</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -20031,14 +20031,14 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>10.69.5.191</t>
+          <t>10.69.5.195</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>2011</v>
+        <v>2013</v>
       </c>
       <c r="E305" t="n">
-        <v>5155</v>
+        <v>22943</v>
       </c>
       <c r="F305" t="inlineStr">
         <is>
@@ -20047,7 +20047,7 @@
       </c>
       <c r="G305" t="inlineStr">
         <is>
-          <t>L1AW6TC</t>
+          <t>9CCKZL1</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
@@ -20062,16 +20062,19 @@
       </c>
       <c r="K305" t="inlineStr">
         <is>
-          <t>LENOVO</t>
+          <t>Dell Inc.</t>
         </is>
       </c>
       <c r="L305" t="inlineStr">
         <is>
-          <t>ThinkCentre A55</t>
-        </is>
+          <t>OptiPlex 360</t>
+        </is>
+      </c>
+      <c r="M305" t="n">
+        <v>1</v>
       </c>
       <c r="N305" s="3" t="n">
-        <v>46022.85438657407</v>
+        <v>46043.58903935185</v>
       </c>
       <c r="O305" t="inlineStr">
         <is>
@@ -20082,7 +20085,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>PA_195</t>
+          <t>PA_196</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -20092,7 +20095,7 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>10.69.5.195</t>
+          <t>10.69.5.196</t>
         </is>
       </c>
       <c r="D306" t="n">
@@ -20108,7 +20111,7 @@
       </c>
       <c r="G306" t="inlineStr">
         <is>
-          <t>9CCKZL1</t>
+          <t>GFCKZL1</t>
         </is>
       </c>
       <c r="I306" t="inlineStr">
@@ -20131,11 +20134,8 @@
           <t>OptiPlex 360</t>
         </is>
       </c>
-      <c r="M306" t="n">
-        <v>1</v>
-      </c>
       <c r="N306" s="3" t="n">
-        <v>46043.58903935185</v>
+        <v>45903.47273148148</v>
       </c>
       <c r="O306" t="inlineStr">
         <is>
@@ -20146,7 +20146,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>PA_196</t>
+          <t>PA_198</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
@@ -20156,14 +20156,14 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>10.69.5.196</t>
+          <t>10.69.5.198</t>
         </is>
       </c>
       <c r="D307" t="n">
         <v>2013</v>
       </c>
       <c r="E307" t="n">
-        <v>22943</v>
+        <v>3885</v>
       </c>
       <c r="F307" t="inlineStr">
         <is>
@@ -20172,7 +20172,7 @@
       </c>
       <c r="G307" t="inlineStr">
         <is>
-          <t>GFCKZL1</t>
+          <t>CCCD1F1</t>
         </is>
       </c>
       <c r="I307" t="inlineStr">
@@ -20182,7 +20182,7 @@
       </c>
       <c r="J307" t="inlineStr">
         <is>
-          <t>2 GB</t>
+          <t>3 GB</t>
         </is>
       </c>
       <c r="K307" t="inlineStr">
@@ -20192,11 +20192,11 @@
       </c>
       <c r="L307" t="inlineStr">
         <is>
-          <t>OptiPlex 360</t>
+          <t>OptiPlex 745</t>
         </is>
       </c>
       <c r="N307" s="3" t="n">
-        <v>45903.47273148148</v>
+        <v>45971.67914351852</v>
       </c>
       <c r="O307" t="inlineStr">
         <is>
@@ -20207,7 +20207,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>PA_198</t>
+          <t>PA_199</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
@@ -20217,14 +20217,14 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>10.69.5.198</t>
+          <t>10.69.5.199</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="E308" t="n">
-        <v>3885</v>
+        <v>2956</v>
       </c>
       <c r="F308" t="inlineStr">
         <is>
@@ -20233,17 +20233,17 @@
       </c>
       <c r="G308" t="inlineStr">
         <is>
-          <t>CCCD1F1</t>
+          <t>53XQXG1</t>
         </is>
       </c>
       <c r="I308" t="inlineStr">
         <is>
-          <t>Intel Core 2 Duo</t>
+          <t>Intel Xeon</t>
         </is>
       </c>
       <c r="J308" t="inlineStr">
         <is>
-          <t>3 GB</t>
+          <t>2 GB</t>
         </is>
       </c>
       <c r="K308" t="inlineStr">
@@ -20253,11 +20253,11 @@
       </c>
       <c r="L308" t="inlineStr">
         <is>
-          <t>OptiPlex 745</t>
+          <t>OptiPlex 755</t>
         </is>
       </c>
       <c r="N308" s="3" t="n">
-        <v>45971.67914351852</v>
+        <v>46046.92365740741</v>
       </c>
       <c r="O308" t="inlineStr">
         <is>
@@ -20268,7 +20268,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>PA_199</t>
+          <t>PA_200</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
@@ -20278,14 +20278,14 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>10.69.5.199</t>
+          <t>10.69.5.201</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="E309" t="n">
-        <v>2956</v>
+        <v>22943</v>
       </c>
       <c r="F309" t="inlineStr">
         <is>
@@ -20294,12 +20294,12 @@
       </c>
       <c r="G309" t="inlineStr">
         <is>
-          <t>53XQXG1</t>
+          <t>GBCKZL1</t>
         </is>
       </c>
       <c r="I309" t="inlineStr">
         <is>
-          <t>Intel Xeon</t>
+          <t>Intel Core 2 Duo</t>
         </is>
       </c>
       <c r="J309" t="inlineStr">
@@ -20314,11 +20314,14 @@
       </c>
       <c r="L309" t="inlineStr">
         <is>
-          <t>OptiPlex 755</t>
-        </is>
+          <t>OptiPlex 360</t>
+        </is>
+      </c>
+      <c r="M309" t="n">
+        <v>2</v>
       </c>
       <c r="N309" s="3" t="n">
-        <v>46046.92365740741</v>
+        <v>46055.8405324074</v>
       </c>
       <c r="O309" t="inlineStr">
         <is>
@@ -20329,7 +20332,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>PA_200</t>
+          <t>PA_201</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
@@ -20346,7 +20349,7 @@
         <v>2013</v>
       </c>
       <c r="E310" t="n">
-        <v>22943</v>
+        <v>3885</v>
       </c>
       <c r="F310" t="inlineStr">
         <is>
@@ -20355,7 +20358,7 @@
       </c>
       <c r="G310" t="inlineStr">
         <is>
-          <t>GBCKZL1</t>
+          <t>2T974F1</t>
         </is>
       </c>
       <c r="I310" t="inlineStr">
@@ -20375,14 +20378,11 @@
       </c>
       <c r="L310" t="inlineStr">
         <is>
-          <t>OptiPlex 360</t>
-        </is>
-      </c>
-      <c r="M310" t="n">
-        <v>2</v>
+          <t>OptiPlex 745</t>
+        </is>
       </c>
       <c r="N310" s="3" t="n">
-        <v>46055.8405324074</v>
+        <v>46056.50774305555</v>
       </c>
       <c r="O310" t="inlineStr">
         <is>
@@ -20393,7 +20393,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>PA_201</t>
+          <t>PA_202</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
@@ -20403,14 +20403,14 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>10.69.5.201</t>
+          <t>10.69.5.202</t>
         </is>
       </c>
       <c r="D311" t="n">
         <v>2013</v>
       </c>
       <c r="E311" t="n">
-        <v>3885</v>
+        <v>22943</v>
       </c>
       <c r="F311" t="inlineStr">
         <is>
@@ -20419,7 +20419,7 @@
       </c>
       <c r="G311" t="inlineStr">
         <is>
-          <t>2T974F1</t>
+          <t>3BCKZL1</t>
         </is>
       </c>
       <c r="I311" t="inlineStr">
@@ -20439,11 +20439,11 @@
       </c>
       <c r="L311" t="inlineStr">
         <is>
-          <t>OptiPlex 745</t>
+          <t>OptiPlex 360</t>
         </is>
       </c>
       <c r="N311" s="3" t="n">
-        <v>46056.50774305555</v>
+        <v>46057.83956018519</v>
       </c>
       <c r="O311" t="inlineStr">
         <is>
@@ -20454,7 +20454,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>PA_202</t>
+          <t>PA_203</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
@@ -20464,14 +20464,14 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>10.69.5.202</t>
+          <t>10.69.5.203</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>2013</v>
+        <v>2011</v>
       </c>
       <c r="E312" t="n">
-        <v>22943</v>
+        <v>8390</v>
       </c>
       <c r="F312" t="inlineStr">
         <is>
@@ -20480,12 +20480,12 @@
       </c>
       <c r="G312" t="inlineStr">
         <is>
-          <t>3BCKZL1</t>
+          <t>BRG820F82L</t>
         </is>
       </c>
       <c r="I312" t="inlineStr">
         <is>
-          <t>Intel Core 2 Duo</t>
+          <t>Intel Pentium®</t>
         </is>
       </c>
       <c r="J312" t="inlineStr">
@@ -20495,16 +20495,16 @@
       </c>
       <c r="K312" t="inlineStr">
         <is>
-          <t>Dell Inc.</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="L312" t="inlineStr">
         <is>
-          <t>OptiPlex 360</t>
+          <t>HP Compaq dx7400 Brazil SFF PC.</t>
         </is>
       </c>
       <c r="N312" s="3" t="n">
-        <v>46057.83956018519</v>
+        <v>46079.04523148148</v>
       </c>
       <c r="O312" t="inlineStr">
         <is>
@@ -20515,7 +20515,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>PA_203</t>
+          <t>PA_204</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
@@ -20525,14 +20525,14 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>10.69.5.203</t>
+          <t>10.69.5.204</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>2011</v>
+        <v>2013</v>
       </c>
       <c r="E313" t="n">
-        <v>8390</v>
+        <v>22943</v>
       </c>
       <c r="F313" t="inlineStr">
         <is>
@@ -20541,12 +20541,12 @@
       </c>
       <c r="G313" t="inlineStr">
         <is>
-          <t>BRG820F82L</t>
+          <t>L1BFDCZ</t>
         </is>
       </c>
       <c r="I313" t="inlineStr">
         <is>
-          <t>Intel Pentium®</t>
+          <t>Intel Core 2 Duo</t>
         </is>
       </c>
       <c r="J313" t="inlineStr">
@@ -20556,16 +20556,19 @@
       </c>
       <c r="K313" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>LENOVO</t>
         </is>
       </c>
       <c r="L313" t="inlineStr">
         <is>
-          <t>HP Compaq dx7400 Brazil SFF PC.</t>
-        </is>
+          <t>ThinkCentre M58p</t>
+        </is>
+      </c>
+      <c r="M313" t="n">
+        <v>1</v>
       </c>
       <c r="N313" s="3" t="n">
-        <v>46079.04523148148</v>
+        <v>46090.45797453704</v>
       </c>
       <c r="O313" t="inlineStr">
         <is>
@@ -20876,7 +20879,7 @@
         </is>
       </c>
       <c r="N318" s="3" t="n">
-        <v>46090.39251157407</v>
+        <v>46090.46810185185</v>
       </c>
       <c r="O318" t="inlineStr">
         <is>
@@ -21601,7 +21604,7 @@
         <v>1</v>
       </c>
       <c r="N330" s="3" t="n">
-        <v>46090.37818287037</v>
+        <v>46090.48766203703</v>
       </c>
       <c r="O330" t="inlineStr">
         <is>
@@ -21665,7 +21668,7 @@
         <v>2</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46090.38280092592</v>
+        <v>46090.4552662037</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21729,7 +21732,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46090.39908564815</v>
+        <v>46090.47467592593</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21793,7 +21796,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46090.38686342593</v>
+        <v>46090.46494212963</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21857,7 +21860,7 @@
         <v>2</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46090.36391203704</v>
+        <v>46090.48212962963</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21921,7 +21924,7 @@
         <v>1</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46090.37328703704</v>
+        <v>46090.45520833333</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21985,7 +21988,7 @@
         <v>2</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46090.38854166667</v>
+        <v>46090.46662037037</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22049,7 +22052,7 @@
         <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46090.40392361111</v>
+        <v>46090.47935185185</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22177,7 +22180,7 @@
         <v>2</v>
       </c>
       <c r="N339" s="3" t="n">
-        <v>46090.37091435185</v>
+        <v>46090.4512962963</v>
       </c>
       <c r="O339" t="inlineStr">
         <is>
@@ -22241,7 +22244,7 @@
         <v>2</v>
       </c>
       <c r="N340" s="3" t="n">
-        <v>46086.5546875</v>
+        <v>46090.46100694445</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -22260,35 +22263,35 @@
           <t>OPERACAO 9.1</t>
         </is>
       </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>10.69.5.237</t>
+        </is>
+      </c>
       <c r="D341" t="n">
-        <v>2017</v>
+        <v>2011</v>
       </c>
       <c r="E341" t="n">
-        <v>54723</v>
+        <v>8390</v>
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t>Microsoft Windows 7 Professional</t>
+          <t>Microsoft® Windows Vista™ Business</t>
         </is>
       </c>
       <c r="G341" t="inlineStr">
         <is>
-          <t>BRG304F8DK</t>
-        </is>
-      </c>
-      <c r="H341" t="inlineStr">
-        <is>
-          <t>Microsoft Office Standard 2007</t>
+          <t>BRG827F584</t>
         </is>
       </c>
       <c r="I341" t="inlineStr">
         <is>
-          <t>Intel Core i3</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="J341" t="inlineStr">
         <is>
-          <t>4 GB</t>
+          <t>2 GB</t>
         </is>
       </c>
       <c r="K341" t="inlineStr">
@@ -22298,20 +22301,15 @@
       </c>
       <c r="L341" t="inlineStr">
         <is>
-          <t>HP Compaq Pro 4300 SFF Brazil PC</t>
+          <t>HP Compaq dx7400 Brazil SFF PC.</t>
         </is>
       </c>
       <c r="N341" s="3" t="n">
-        <v>46087.37149305556</v>
+        <v>46090.46665509259</v>
       </c>
       <c r="O341" t="inlineStr">
         <is>
           <t>Ativo</t>
-        </is>
-      </c>
-      <c r="P341" t="inlineStr">
-        <is>
-          <t>PJ BALEIA</t>
         </is>
       </c>
     </row>
@@ -22371,7 +22369,7 @@
         <v>1</v>
       </c>
       <c r="N342" s="3" t="n">
-        <v>46057.41765046296</v>
+        <v>46090.47693287037</v>
       </c>
       <c r="O342" t="inlineStr">
         <is>
@@ -22558,7 +22556,7 @@
         <v>1</v>
       </c>
       <c r="N345" s="3" t="n">
-        <v>46087.59559027778</v>
+        <v>46090.47086805556</v>
       </c>
       <c r="O345" t="inlineStr">
         <is>
@@ -22622,7 +22620,7 @@
         <v>1</v>
       </c>
       <c r="N346" s="3" t="n">
-        <v>46090.38048611111</v>
+        <v>46090.45559027778</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -22686,7 +22684,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46090.38070601852</v>
+        <v>46090.4555787037</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22710,6 +22708,22 @@
           <t>10.69.5.244</t>
         </is>
       </c>
+      <c r="D348" t="n">
+        <v>2016</v>
+      </c>
+      <c r="E348" t="n">
+        <v>43374</v>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>Microsoft Windows 7 Professional</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>BRG132F1SW</t>
+        </is>
+      </c>
       <c r="I348" t="inlineStr">
         <is>
           <t>Intel Core 2 Duo</t>
@@ -22720,11 +22734,18 @@
           <t>2 GB</t>
         </is>
       </c>
-      <c r="M348" t="n">
-        <v>1</v>
+      <c r="K348" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="L348" t="inlineStr">
+        <is>
+          <t>COMPAQ 300B MT</t>
+        </is>
       </c>
       <c r="N348" s="3" t="n">
-        <v>46090.39174768519</v>
+        <v>46090.47412037037</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -22788,7 +22809,7 @@
         <v>1</v>
       </c>
       <c r="N349" s="3" t="n">
-        <v>46087.57554398148</v>
+        <v>46090.47880787037</v>
       </c>
       <c r="O349" t="inlineStr">
         <is>
@@ -22852,7 +22873,7 @@
         <v>1</v>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46087.60881944445</v>
+        <v>46090.47693287037</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -22871,35 +22892,35 @@
           <t>OPERACAO 9.1</t>
         </is>
       </c>
-      <c r="C351" t="inlineStr">
-        <is>
-          <t>10.69.5.247</t>
-        </is>
-      </c>
       <c r="D351" t="n">
-        <v>2011</v>
+        <v>2017</v>
       </c>
       <c r="E351" t="n">
-        <v>8390</v>
+        <v>54723</v>
       </c>
       <c r="F351" t="inlineStr">
         <is>
-          <t>Microsoft® Windows Vista™ Business</t>
+          <t>Microsoft Windows 7 Professional</t>
         </is>
       </c>
       <c r="G351" t="inlineStr">
         <is>
-          <t>BRG827F584</t>
+          <t>BRG304F8DK</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>Microsoft Office Standard 2007</t>
         </is>
       </c>
       <c r="I351" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Intel Core i3</t>
         </is>
       </c>
       <c r="J351" t="inlineStr">
         <is>
-          <t>2 GB</t>
+          <t>4 GB</t>
         </is>
       </c>
       <c r="K351" t="inlineStr">
@@ -22909,15 +22930,20 @@
       </c>
       <c r="L351" t="inlineStr">
         <is>
-          <t>HP Compaq dx7400 Brazil SFF PC.</t>
+          <t>HP Compaq Pro 4300 SFF Brazil PC</t>
         </is>
       </c>
       <c r="N351" s="3" t="n">
-        <v>46087.37065972222</v>
+        <v>46090.47795138889</v>
       </c>
       <c r="O351" t="inlineStr">
         <is>
           <t>Ativo</t>
+        </is>
+      </c>
+      <c r="P351" t="inlineStr">
+        <is>
+          <t>PJ BALEIA</t>
         </is>
       </c>
     </row>
@@ -22974,7 +23000,7 @@
         </is>
       </c>
       <c r="N352" s="3" t="n">
-        <v>46080.51325231481</v>
+        <v>46090.45616898148</v>
       </c>
       <c r="O352" t="inlineStr">
         <is>
@@ -23038,7 +23064,7 @@
         <v>1</v>
       </c>
       <c r="N353" s="3" t="n">
-        <v>46087.60150462963</v>
+        <v>46090.47436342593</v>
       </c>
       <c r="O353" t="inlineStr">
         <is>
@@ -23102,7 +23128,7 @@
         <v>1</v>
       </c>
       <c r="N354" s="3" t="n">
-        <v>46087.60498842593</v>
+        <v>46090.47526620371</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -23166,7 +23192,7 @@
         <v>1</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46087.57063657408</v>
+        <v>46090.47763888889</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23190,47 +23216,16 @@
           <t>10.69.5.252</t>
         </is>
       </c>
-      <c r="D356" t="n">
-        <v>2012</v>
-      </c>
-      <c r="E356" t="n">
-        <v>2956</v>
-      </c>
-      <c r="F356" t="inlineStr">
-        <is>
-          <t>Microsoft® Windows Vista™ Business</t>
-        </is>
-      </c>
-      <c r="G356" t="inlineStr">
-        <is>
-          <t>J5L1JJ1</t>
-        </is>
-      </c>
-      <c r="I356" t="inlineStr">
-        <is>
-          <t>Intel Core 2 Duo</t>
-        </is>
-      </c>
       <c r="J356" t="inlineStr">
         <is>
           <t>2 GB</t>
-        </is>
-      </c>
-      <c r="K356" t="inlineStr">
-        <is>
-          <t>Dell Inc.</t>
-        </is>
-      </c>
-      <c r="L356" t="inlineStr">
-        <is>
-          <t>OptiPlex 755</t>
         </is>
       </c>
       <c r="M356" t="n">
         <v>1</v>
       </c>
       <c r="N356" s="3" t="n">
-        <v>46087.37417824074</v>
+        <v>46090.48760416666</v>
       </c>
       <c r="O356" t="inlineStr">
         <is>
@@ -23294,7 +23289,7 @@
         <v>2</v>
       </c>
       <c r="N357" s="3" t="n">
-        <v>46087.60486111111</v>
+        <v>46090.47326388889</v>
       </c>
       <c r="O357" t="inlineStr">
         <is>
@@ -23358,7 +23353,7 @@
         <v>2</v>
       </c>
       <c r="N358" s="3" t="n">
-        <v>46087.57782407408</v>
+        <v>46090.47439814815</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -23422,7 +23417,7 @@
         <v>1</v>
       </c>
       <c r="N359" s="3" t="n">
-        <v>46087.59552083333</v>
+        <v>46090.48658564815</v>
       </c>
       <c r="O359" t="inlineStr">
         <is>
@@ -23483,7 +23478,7 @@
         </is>
       </c>
       <c r="N360" s="3" t="n">
-        <v>46085.40222222222</v>
+        <v>46090.47855324074</v>
       </c>
       <c r="O360" t="inlineStr">
         <is>
@@ -23671,7 +23666,7 @@
         <v>1</v>
       </c>
       <c r="N363" s="3" t="n">
-        <v>46090.36526620371</v>
+        <v>46090.4879050926</v>
       </c>
       <c r="O363" t="inlineStr">
         <is>
@@ -23737,7 +23732,7 @@
         </is>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46090.38342592592</v>
+        <v>46090.46115740741</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23863,7 +23858,7 @@
         </is>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46090.40384259259</v>
+        <v>46090.48552083333</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
@@ -23993,7 +23988,7 @@
         <v>1</v>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46090.36905092592</v>
+        <v>46090.47690972222</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24090,7 +24085,7 @@
         <v>1</v>
       </c>
       <c r="N370" s="3" t="n">
-        <v>46090.39989583333</v>
+        <v>46090.47393518518</v>
       </c>
       <c r="O370" t="inlineStr">
         <is>
@@ -24159,7 +24154,7 @@
         <v>1</v>
       </c>
       <c r="N371" s="3" t="n">
-        <v>46090.39804398148</v>
+        <v>46090.43759259259</v>
       </c>
       <c r="O371" t="inlineStr">
         <is>
@@ -24294,7 +24289,7 @@
         </is>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46090.3787962963</v>
+        <v>46090.4562037037</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24358,7 +24353,7 @@
         <v>1</v>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46087.80133101852</v>
+        <v>46090.46071759259</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -24427,7 +24422,7 @@
         <v>2</v>
       </c>
       <c r="N375" s="3" t="n">
-        <v>46090.40108796296</v>
+        <v>46090.47884259259</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -24496,7 +24491,7 @@
         <v>2</v>
       </c>
       <c r="N376" s="3" t="n">
-        <v>46090.39530092593</v>
+        <v>46090.47393518518</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-09 15:52:09.993468
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46090.56883101852</v>
+        <v>46090.64559027777</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46090.54894675926</v>
+        <v>46090.63208333333</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46090.56560185185</v>
+        <v>46090.64517361111</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46090.53915509259</v>
+        <v>46090.653125</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
         <v>1</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>46090.54481481481</v>
+        <v>46090.62236111111</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1190,7 +1190,7 @@
         <v>1</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>46090.54199074074</v>
+        <v>46090.63181712963</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -2178,7 +2178,7 @@
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46090.53849537037</v>
+        <v>46090.61627314815</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6504,7 +6504,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46090.55438657408</v>
+        <v>46090.63471064815</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6573,7 +6573,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46090.55956018518</v>
+        <v>46090.63760416667</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6637,7 +6637,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46090.55641203704</v>
+        <v>46090.62917824074</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6656,11 +6656,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>10.69.3.94</t>
-        </is>
-      </c>
       <c r="D97" t="n">
         <v>2025</v>
       </c>
@@ -6706,7 +6701,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46090.56756944444</v>
+        <v>46090.6441087963</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6775,7 +6770,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46090.54712962963</v>
+        <v>46090.62523148148</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6844,7 +6839,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46090.53734953704</v>
+        <v>46090.65401620371</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6913,7 +6908,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46090.54589120371</v>
+        <v>46090.6528587963</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6982,7 +6977,7 @@
         <v>1</v>
       </c>
       <c r="N101" s="3" t="n">
-        <v>46090.53221064815</v>
+        <v>46090.64703703704</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -7051,7 +7046,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46090.5381712963</v>
+        <v>46090.65203703703</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7446,7 +7441,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46090.55725694444</v>
+        <v>46090.63789351852</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7515,7 +7510,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46090.55399305555</v>
+        <v>46090.63140046296</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7584,7 +7579,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46090.53972222222</v>
+        <v>46090.62186342593</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7653,7 +7648,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46090.53472222222</v>
+        <v>46090.65069444444</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7722,7 +7717,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46090.55592592592</v>
+        <v>46090.6346875</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7791,7 +7786,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46090.55113425926</v>
+        <v>46090.62784722223</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7857,7 +7852,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46090.53609953704</v>
+        <v>46090.61855324074</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7926,7 +7921,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46090.56328703704</v>
+        <v>46090.63763888889</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7995,7 +7990,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46090.5678125</v>
+        <v>46090.64344907407</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8061,7 +8056,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46090.56728009259</v>
+        <v>46090.64159722222</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8199,7 +8194,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46090.53679398148</v>
+        <v>46090.65155092593</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8334,7 +8329,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46090.56232638889</v>
+        <v>46090.6408912037</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8403,7 +8398,7 @@
         <v>2</v>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46090.53627314815</v>
+        <v>46090.64686342593</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8472,7 +8467,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46090.53164351852</v>
+        <v>46090.64859953704</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8541,7 +8536,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46090.56064814814</v>
+        <v>46090.63814814815</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8679,7 +8674,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46090.54542824074</v>
+        <v>46090.61848379629</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8748,7 +8743,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46090.53715277778</v>
+        <v>46090.6522800926</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8817,7 +8812,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46090.55184027777</v>
+        <v>46090.62480324074</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8886,7 +8881,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46090.53931712963</v>
+        <v>46090.64675925926</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -8950,7 +8945,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46087.67005787037</v>
+        <v>46090.63199074074</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9014,7 +9009,7 @@
         <v>1</v>
       </c>
       <c r="N131" s="3" t="n">
-        <v>46090.56435185186</v>
+        <v>46090.62496527778</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -9078,7 +9073,7 @@
         <v>1</v>
       </c>
       <c r="N132" s="3" t="n">
-        <v>46087.8700462963</v>
+        <v>46090.62893518519</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -9142,7 +9137,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46088.5984375</v>
+        <v>46090.6252662037</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9333,7 +9328,7 @@
         <v>1</v>
       </c>
       <c r="N136" s="3" t="n">
-        <v>46088.60962962963</v>
+        <v>46090.62243055556</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -9397,7 +9392,7 @@
         <v>1</v>
       </c>
       <c r="N137" s="3" t="n">
-        <v>46088.59219907408</v>
+        <v>46090.61814814815</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -9461,7 +9456,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46090.5661574074</v>
+        <v>46090.64328703703</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9525,7 +9520,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46090.5690625</v>
+        <v>46090.6521412037</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9589,7 +9584,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46090.56663194444</v>
+        <v>46090.64048611111</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9653,7 +9648,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46090.53728009259</v>
+        <v>46090.62377314815</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9717,7 +9712,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46090.56565972222</v>
+        <v>46090.64152777778</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9781,7 +9776,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46090.54082175926</v>
+        <v>46090.61872685186</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9845,7 +9840,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46090.55585648148</v>
+        <v>46090.61959490741</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9909,7 +9904,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46090.55392361111</v>
+        <v>46090.62576388889</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9973,7 +9968,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46090.35107638889</v>
+        <v>46090.61748842592</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10037,7 +10032,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46090.56766203704</v>
+        <v>46090.64533564815</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10101,7 +10096,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46086.54293981481</v>
+        <v>46090.62456018518</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10165,7 +10160,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46090.56662037037</v>
+        <v>46090.64149305555</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10229,7 +10224,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46090.56050925926</v>
+        <v>46090.63243055555</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10248,11 +10243,6 @@
           <t>OPERACAO 7.1</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>10.69.5.21</t>
-        </is>
-      </c>
       <c r="D151" t="n">
         <v>2018</v>
       </c>
@@ -10293,7 +10283,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46090.55459490741</v>
+        <v>46090.63511574074</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10357,7 +10347,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46090.56777777777</v>
+        <v>46090.62900462963</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10421,7 +10411,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46090.56475694444</v>
+        <v>46090.638125</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10485,7 +10475,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46090.54701388889</v>
+        <v>46090.6225462963</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10549,7 +10539,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46090.53601851852</v>
+        <v>46090.57751157408</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10741,7 +10731,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46090.5372337963</v>
+        <v>46090.65138888889</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10869,7 +10859,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46090.56914351852</v>
+        <v>46090.62674768519</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10997,7 +10987,7 @@
         <v>2</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46090.56313657408</v>
+        <v>46090.6369675926</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11061,7 +11051,7 @@
         <v>2</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46090.56420138889</v>
+        <v>46090.63697916667</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11125,7 +11115,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46090.57053240741</v>
+        <v>46090.64833333333</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11189,7 +11179,7 @@
         <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46090.52903935185</v>
+        <v>46090.64609953704</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11253,7 +11243,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46090.55684027778</v>
+        <v>46090.6193287037</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11317,7 +11307,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46090.56381944445</v>
+        <v>46090.64023148148</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11381,7 +11371,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46090.56798611111</v>
+        <v>46090.64577546297</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11509,7 +11499,7 @@
         <v>2</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46090.5593287037</v>
+        <v>46090.63803240741</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11573,7 +11563,7 @@
         <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46090.57019675926</v>
+        <v>46090.6446412037</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11701,7 +11691,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46090.56844907408</v>
+        <v>46090.64597222222</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11765,7 +11755,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46090.53476851852</v>
+        <v>46090.61678240741</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11829,7 +11819,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46090.53712962963</v>
+        <v>46090.654375</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11893,7 +11883,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46090.55116898148</v>
+        <v>46090.62944444444</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11957,7 +11947,7 @@
         <v>1</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46090.53841435185</v>
+        <v>46090.63055555556</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12021,7 +12011,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46088.59194444444</v>
+        <v>46090.61931712963</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12085,7 +12075,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46090.56604166667</v>
+        <v>46090.64403935185</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12410,7 +12400,7 @@
         <v>1</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46090.37092592593</v>
+        <v>46090.62696759259</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12474,7 +12464,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46090.53195601852</v>
+        <v>46090.6496412037</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12666,7 +12656,7 @@
         </is>
       </c>
       <c r="N188" s="3" t="n">
-        <v>46090.55277777778</v>
+        <v>46090.63974537037</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
@@ -12730,7 +12720,7 @@
         <v>1</v>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46090.56710648148</v>
+        <v>46090.64886574074</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12794,7 +12784,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46090.57083333333</v>
+        <v>46090.64983796296</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12919,7 +12909,7 @@
         <v>2</v>
       </c>
       <c r="N192" s="3" t="n">
-        <v>46090.5678587963</v>
+        <v>46090.64215277778</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
@@ -12983,7 +12973,7 @@
         <v>1</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46090.55811342593</v>
+        <v>46090.62991898148</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13047,7 +13037,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46090.53501157407</v>
+        <v>46090.61734953704</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13111,7 +13101,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46090.53313657407</v>
+        <v>46090.57171296296</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13175,7 +13165,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46090.55399305555</v>
+        <v>46090.62885416667</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13303,7 +13293,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46090.53548611111</v>
+        <v>46090.65395833334</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13364,7 +13354,7 @@
         </is>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46088.61820601852</v>
+        <v>46090.63005787037</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13428,7 +13418,7 @@
         <v>1</v>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46090.56206018518</v>
+        <v>46090.63894675926</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13492,7 +13482,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46090.54106481482</v>
+        <v>46090.63679398148</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13556,7 +13546,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46090.5595949074</v>
+        <v>46090.62967592593</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13620,7 +13610,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46090.56959490741</v>
+        <v>46090.64898148148</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13684,7 +13674,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46090.54160879629</v>
+        <v>46090.6196875</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13748,7 +13738,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46090.55768518519</v>
+        <v>46090.63725694444</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13876,7 +13866,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46090.53076388889</v>
+        <v>46090.62011574074</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13940,7 +13930,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46090.56605324074</v>
+        <v>46090.64390046296</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14004,7 +13994,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46090.53915509259</v>
+        <v>46090.62181712963</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14068,7 +14058,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46090.53885416667</v>
+        <v>46090.61716435185</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14132,7 +14122,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46090.53570601852</v>
+        <v>46090.57773148148</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14324,7 +14314,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46090.53476851852</v>
+        <v>46090.65435185185</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14343,6 +14333,11 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>10.69.5.85</t>
+        </is>
+      </c>
       <c r="D215" t="n">
         <v>2017</v>
       </c>
@@ -14383,7 +14378,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46090.53453703703</v>
+        <v>46090.64363425926</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14447,7 +14442,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46090.56555555556</v>
+        <v>46090.64123842592</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14511,7 +14506,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46088.5840625</v>
+        <v>46090.5862037037</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14580,7 +14575,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46090.52805555556</v>
+        <v>46090.62451388889</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14644,7 +14639,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46090.54067129629</v>
+        <v>46090.62549768519</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14772,7 +14767,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46090.53759259259</v>
+        <v>46090.64726851852</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14900,7 +14895,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46088.43309027778</v>
+        <v>46090.6505787037</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14964,7 +14959,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46090.56428240741</v>
+        <v>46090.61452546297</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15028,7 +15023,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46090.55202546297</v>
+        <v>46090.6278587963</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15092,7 +15087,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46090.55357638889</v>
+        <v>46090.63539351852</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15156,7 +15151,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46090.36811342592</v>
+        <v>46090.62717592593</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15348,7 +15343,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46090.56064814814</v>
+        <v>46090.62568287037</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15412,7 +15407,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46090.56623842593</v>
+        <v>46090.64430555556</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15476,7 +15471,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46090.55643518519</v>
+        <v>46090.63908564814</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15540,7 +15535,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46090.52903935185</v>
+        <v>46090.64060185185</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15604,7 +15599,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46090.53534722222</v>
+        <v>46090.57744212963</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15668,7 +15663,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46090.54305555556</v>
+        <v>46090.62363425926</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15732,7 +15727,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46090.55806712963</v>
+        <v>46090.63512731482</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15860,7 +15855,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46090.53851851852</v>
+        <v>46090.65216435185</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15988,7 +15983,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46090.5690625</v>
+        <v>46090.65033564815</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16052,7 +16047,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46090.56878472222</v>
+        <v>46090.64673611111</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16175,7 +16170,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46090.55417824074</v>
+        <v>46090.62888888889</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16239,7 +16234,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46090.56289351852</v>
+        <v>46090.64265046296</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16303,7 +16298,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46090.56083333334</v>
+        <v>46090.63956018518</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16367,7 +16362,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46090.55945601852</v>
+        <v>46090.64126157408</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16431,7 +16426,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46090.55783564815</v>
+        <v>46090.63493055556</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16450,11 +16445,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C248" t="inlineStr">
-        <is>
-          <t>10.69.5.118</t>
-        </is>
-      </c>
       <c r="D248" t="n">
         <v>2017</v>
       </c>
@@ -16495,7 +16485,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46090.55894675926</v>
+        <v>46090.63291666667</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16559,7 +16549,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46090.56239583333</v>
+        <v>46090.62336805555</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16687,7 +16677,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46090.54782407408</v>
+        <v>46090.62039351852</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16745,7 +16735,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46090.5480787037</v>
+        <v>46090.61615740741</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16809,7 +16799,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46090.55402777778</v>
+        <v>46090.63628472222</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16873,7 +16863,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46090.55681712963</v>
+        <v>46090.63934027778</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16937,7 +16927,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46090.5595949074</v>
+        <v>46090.64236111111</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -17001,7 +16991,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46090.42594907407</v>
+        <v>46090.63674768519</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17065,7 +17055,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46090.55697916666</v>
+        <v>46090.62981481481</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17129,7 +17119,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46090.56420138889</v>
+        <v>46090.60371527778</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17193,7 +17183,7 @@
         <v>2</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46090.55782407407</v>
+        <v>46090.59398148148</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17257,7 +17247,7 @@
         <v>1</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46088.59612268519</v>
+        <v>46090.6282175926</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17321,7 +17311,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46090.5672337963</v>
+        <v>46090.64314814815</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17385,7 +17375,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46090.5471875</v>
+        <v>46090.62571759259</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17449,7 +17439,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46090.56429398148</v>
+        <v>46090.63366898148</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17513,7 +17503,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46090.56015046296</v>
+        <v>46090.63931712963</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17577,7 +17567,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46090.53583333334</v>
+        <v>46090.65174768519</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17641,7 +17631,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46090.55694444444</v>
+        <v>46090.63290509259</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17705,7 +17695,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46090.53269675926</v>
+        <v>46090.64630787037</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17766,7 +17756,7 @@
         </is>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46090.56824074074</v>
+        <v>46090.64577546297</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17894,7 +17884,7 @@
         <v>1</v>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46090.53619212963</v>
+        <v>46090.63755787037</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -18267,7 +18257,7 @@
         <v>1</v>
       </c>
       <c r="N276" s="3" t="n">
-        <v>46090.54557870371</v>
+        <v>46090.62627314815</v>
       </c>
       <c r="O276" t="inlineStr">
         <is>
@@ -18331,7 +18321,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46090.55458333333</v>
+        <v>46090.63334490741</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18454,7 +18444,7 @@
         <v>1</v>
       </c>
       <c r="N279" s="3" t="n">
-        <v>46090.53990740741</v>
+        <v>46090.5778587963</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -18473,6 +18463,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>10.69.5.151</t>
+        </is>
+      </c>
       <c r="D280" t="n">
         <v>2017</v>
       </c>
@@ -18513,7 +18508,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46090.53515046297</v>
+        <v>46090.65142361111</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18577,7 +18572,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46090.55621527778</v>
+        <v>46090.63969907408</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18641,7 +18636,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46090.53678240741</v>
+        <v>46090.61768518519</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18705,7 +18700,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46090.53467592593</v>
+        <v>46090.61336805556</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18961,7 +18956,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46090.54043981482</v>
+        <v>46090.61842592592</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19694,7 +19689,7 @@
         <v>1</v>
       </c>
       <c r="N299" s="3" t="n">
-        <v>46090.56130787037</v>
+        <v>46090.63841435185</v>
       </c>
       <c r="O299" t="inlineStr">
         <is>
@@ -20810,7 +20805,7 @@
         </is>
       </c>
       <c r="N317" s="3" t="n">
-        <v>46090.5425</v>
+        <v>46090.61793981482</v>
       </c>
       <c r="O317" t="inlineStr">
         <is>
@@ -21535,7 +21530,7 @@
         <v>1</v>
       </c>
       <c r="N329" s="3" t="n">
-        <v>46090.56275462963</v>
+        <v>46090.63883101852</v>
       </c>
       <c r="O329" t="inlineStr">
         <is>
@@ -21599,7 +21594,7 @@
         <v>2</v>
       </c>
       <c r="N330" s="3" t="n">
-        <v>46090.53704861111</v>
+        <v>46090.64981481482</v>
       </c>
       <c r="O330" t="inlineStr">
         <is>
@@ -21663,7 +21658,7 @@
         <v>2</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46090.55276620371</v>
+        <v>46090.63159722222</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21727,7 +21722,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46090.54065972222</v>
+        <v>46090.65061342593</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21791,7 +21786,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46090.56043981481</v>
+        <v>46090.64012731481</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21855,7 +21850,7 @@
         <v>1</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46090.53311342592</v>
+        <v>46090.64643518518</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21919,7 +21914,7 @@
         <v>2</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46090.54133101852</v>
+        <v>46090.62445601852</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21983,7 +21978,7 @@
         <v>2</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46090.56077546296</v>
+        <v>46090.63594907407</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22111,7 +22106,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46090.5355787037</v>
+        <v>46090.5733912037</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22175,7 +22170,7 @@
         <v>2</v>
       </c>
       <c r="N339" s="3" t="n">
-        <v>46090.53633101852</v>
+        <v>46090.57268518519</v>
       </c>
       <c r="O339" t="inlineStr">
         <is>
@@ -22236,7 +22231,7 @@
         </is>
       </c>
       <c r="N340" s="3" t="n">
-        <v>46090.54289351852</v>
+        <v>46090.62061342593</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -22423,7 +22418,7 @@
         <v>1</v>
       </c>
       <c r="N343" s="3" t="n">
-        <v>46090.54460648148</v>
+        <v>46090.61981481482</v>
       </c>
       <c r="O343" t="inlineStr">
         <is>
@@ -22487,7 +22482,7 @@
         <v>1</v>
       </c>
       <c r="N344" s="3" t="n">
-        <v>46090.53743055555</v>
+        <v>46090.65255787037</v>
       </c>
       <c r="O344" t="inlineStr">
         <is>
@@ -22551,7 +22546,7 @@
         <v>1</v>
       </c>
       <c r="N345" s="3" t="n">
-        <v>46090.53793981481</v>
+        <v>46090.6362037037</v>
       </c>
       <c r="O345" t="inlineStr">
         <is>
@@ -22612,7 +22607,7 @@
         </is>
       </c>
       <c r="N346" s="3" t="n">
-        <v>46090.54936342593</v>
+        <v>46090.63268518518</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -22676,7 +22671,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46090.55819444444</v>
+        <v>46090.6177662037</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22740,7 +22735,7 @@
         <v>1</v>
       </c>
       <c r="N348" s="3" t="n">
-        <v>46090.55320601852</v>
+        <v>46090.63333333333</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -22801,7 +22796,7 @@
         </is>
       </c>
       <c r="N349" s="3" t="n">
-        <v>46090.51611111111</v>
+        <v>46090.63385416667</v>
       </c>
       <c r="O349" t="inlineStr">
         <is>
@@ -22867,7 +22862,7 @@
         </is>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46090.56947916667</v>
+        <v>46090.64925925926</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -22931,7 +22926,7 @@
         <v>1</v>
       </c>
       <c r="N351" s="3" t="n">
-        <v>46090.55306712963</v>
+        <v>46090.63042824074</v>
       </c>
       <c r="O351" t="inlineStr">
         <is>
@@ -22995,7 +22990,7 @@
         <v>1</v>
       </c>
       <c r="N352" s="3" t="n">
-        <v>46090.55140046297</v>
+        <v>46090.62754629629</v>
       </c>
       <c r="O352" t="inlineStr">
         <is>
@@ -23059,7 +23054,7 @@
         <v>1</v>
       </c>
       <c r="N353" s="3" t="n">
-        <v>46090.55763888889</v>
+        <v>46090.63325231482</v>
       </c>
       <c r="O353" t="inlineStr">
         <is>
@@ -23092,7 +23087,7 @@
         <v>1</v>
       </c>
       <c r="N354" s="3" t="n">
-        <v>46090.56983796296</v>
+        <v>46090.64662037037</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -23156,7 +23151,7 @@
         <v>2</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46090.47326388889</v>
+        <v>46090.62224537037</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23220,7 +23215,7 @@
         <v>2</v>
       </c>
       <c r="N356" s="3" t="n">
-        <v>46090.55099537037</v>
+        <v>46090.63077546296</v>
       </c>
       <c r="O356" t="inlineStr">
         <is>
@@ -23284,7 +23279,7 @@
         <v>1</v>
       </c>
       <c r="N357" s="3" t="n">
-        <v>46090.56100694444</v>
+        <v>46090.6366087963</v>
       </c>
       <c r="O357" t="inlineStr">
         <is>
@@ -23312,7 +23307,7 @@
         <v>1</v>
       </c>
       <c r="N358" s="3" t="n">
-        <v>46090.56059027778</v>
+        <v>46090.64178240741</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -23335,7 +23330,7 @@
         <v>1</v>
       </c>
       <c r="N359" s="3" t="n">
-        <v>46090.49901620371</v>
+        <v>46090.6193287037</v>
       </c>
       <c r="O359" t="inlineStr">
         <is>
@@ -23462,7 +23457,7 @@
         <v>1</v>
       </c>
       <c r="N361" s="3" t="n">
-        <v>46090.5637037037</v>
+        <v>46090.63865740741</v>
       </c>
       <c r="O361" t="inlineStr">
         <is>
@@ -23528,7 +23523,7 @@
         </is>
       </c>
       <c r="N362" s="3" t="n">
-        <v>46090.54042824074</v>
+        <v>46090.65148148148</v>
       </c>
       <c r="O362" t="inlineStr">
         <is>
@@ -23654,7 +23649,7 @@
         </is>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46090.5592824074</v>
+        <v>46090.63778935185</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23784,7 +23779,7 @@
         <v>1</v>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46090.55710648148</v>
+        <v>46090.63236111111</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
@@ -23812,7 +23807,7 @@
         <v>2</v>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46090.55555555555</v>
+        <v>46090.63650462963</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -23881,7 +23876,7 @@
         <v>1</v>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46090.55001157407</v>
+        <v>46090.62971064815</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24085,7 +24080,7 @@
         </is>
       </c>
       <c r="N371" s="3" t="n">
-        <v>46090.56434027778</v>
+        <v>46090.64346064815</v>
       </c>
       <c r="O371" t="inlineStr">
         <is>
@@ -24104,6 +24099,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>10.69.3.72</t>
+        </is>
+      </c>
       <c r="D372" t="n">
         <v>2025</v>
       </c>
@@ -24149,7 +24149,7 @@
         <v>1</v>
       </c>
       <c r="N372" s="3" t="n">
-        <v>46090.5347800926</v>
+        <v>46090.64954861111</v>
       </c>
       <c r="O372" t="inlineStr">
         <is>
@@ -24218,7 +24218,7 @@
         <v>2</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46090.55405092592</v>
+        <v>46090.62883101852</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24287,7 +24287,7 @@
         <v>2</v>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46090.54997685185</v>
+        <v>46090.6275</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-09 17:52:05.496380
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46090.64559027777</v>
+        <v>46090.7208912037</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46090.63208333333</v>
+        <v>46090.71043981481</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46090.64517361111</v>
+        <v>46090.7244212963</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46090.653125</v>
+        <v>46090.724375</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
         <v>1</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>46090.62236111111</v>
+        <v>46090.70019675926</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1190,7 +1190,7 @@
         <v>1</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>46090.63181712963</v>
+        <v>46090.72584490741</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -2178,7 +2178,7 @@
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46090.61627314815</v>
+        <v>46090.73277777778</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6504,7 +6504,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46090.63471064815</v>
+        <v>46090.71146990741</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6573,7 +6573,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46090.63760416667</v>
+        <v>46090.71255787037</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6637,7 +6637,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46090.62917824074</v>
+        <v>46090.70815972222</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6656,6 +6656,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>10.69.3.94</t>
+        </is>
+      </c>
       <c r="D97" t="n">
         <v>2025</v>
       </c>
@@ -6701,7 +6706,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46090.6441087963</v>
+        <v>46090.72395833334</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6770,7 +6775,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46090.62523148148</v>
+        <v>46090.73159722222</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6839,7 +6844,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46090.65401620371</v>
+        <v>46090.72848379629</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6908,7 +6913,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46090.6528587963</v>
+        <v>46090.72636574074</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6977,7 +6982,7 @@
         <v>1</v>
       </c>
       <c r="N101" s="3" t="n">
-        <v>46090.64703703704</v>
+        <v>46090.72416666667</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -7046,7 +7051,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46090.65203703703</v>
+        <v>46090.73282407408</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7441,7 +7446,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46090.63789351852</v>
+        <v>46090.71714120371</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7510,7 +7515,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46090.63140046296</v>
+        <v>46090.70832175926</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7579,7 +7584,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46090.62186342593</v>
+        <v>46090.69998842593</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7648,7 +7653,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46090.65069444444</v>
+        <v>46090.7262962963</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7717,7 +7722,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46090.6346875</v>
+        <v>46090.71447916667</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7786,7 +7791,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46090.62784722223</v>
+        <v>46090.70395833333</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7852,7 +7857,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46090.61855324074</v>
+        <v>46090.73685185185</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7921,7 +7926,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46090.63763888889</v>
+        <v>46090.67440972223</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7990,7 +7995,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46090.64344907407</v>
+        <v>46090.684375</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8056,7 +8061,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46090.64159722222</v>
+        <v>46090.6825</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8194,7 +8199,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46090.65155092593</v>
+        <v>46090.69013888889</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8329,7 +8334,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46090.6408912037</v>
+        <v>46090.67686342593</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8398,7 +8403,7 @@
         <v>2</v>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46090.64686342593</v>
+        <v>46090.72726851852</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8467,7 +8472,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46090.64859953704</v>
+        <v>46090.73302083334</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8536,7 +8541,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46090.63814814815</v>
+        <v>46090.71278935186</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8674,7 +8679,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46090.61848379629</v>
+        <v>46090.73202546296</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8743,7 +8748,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46090.6522800926</v>
+        <v>46090.69086805556</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8812,7 +8817,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46090.62480324074</v>
+        <v>46090.73658564815</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8881,7 +8886,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46090.64675925926</v>
+        <v>46090.72288194444</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -8945,7 +8950,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46090.63199074074</v>
+        <v>46090.70949074074</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9009,7 +9014,7 @@
         <v>1</v>
       </c>
       <c r="N131" s="3" t="n">
-        <v>46090.62496527778</v>
+        <v>46090.70780092593</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -9073,7 +9078,7 @@
         <v>1</v>
       </c>
       <c r="N132" s="3" t="n">
-        <v>46090.62893518519</v>
+        <v>46090.70758101852</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -9137,7 +9142,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46090.6252662037</v>
+        <v>46090.70351851852</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9328,7 +9333,7 @@
         <v>1</v>
       </c>
       <c r="N136" s="3" t="n">
-        <v>46090.62243055556</v>
+        <v>46090.69908564815</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -9392,7 +9397,7 @@
         <v>1</v>
       </c>
       <c r="N137" s="3" t="n">
-        <v>46090.61814814815</v>
+        <v>46090.73475694445</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -9456,7 +9461,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46090.64328703703</v>
+        <v>46090.72033564815</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9520,7 +9525,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46090.6521412037</v>
+        <v>46090.73034722222</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9584,7 +9589,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46090.64048611111</v>
+        <v>46090.71554398148</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9648,7 +9653,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46090.62377314815</v>
+        <v>46090.70430555556</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9712,7 +9717,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46090.64152777778</v>
+        <v>46090.71460648148</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9776,7 +9781,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46090.61872685186</v>
+        <v>46090.73222222222</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9840,7 +9845,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46090.61959490741</v>
+        <v>46090.69914351852</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9904,7 +9909,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46090.62576388889</v>
+        <v>46090.70489583333</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9968,7 +9973,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46090.61748842592</v>
+        <v>46090.73064814815</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10032,7 +10037,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46090.64533564815</v>
+        <v>46090.71935185185</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10096,7 +10101,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46090.62456018518</v>
+        <v>46090.70642361111</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10224,7 +10229,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46090.63243055555</v>
+        <v>46090.70982638889</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10283,7 +10288,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46090.63511574074</v>
+        <v>46090.71547453704</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10347,7 +10352,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46090.62900462963</v>
+        <v>46090.7075</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10411,7 +10416,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46090.638125</v>
+        <v>46090.71189814815</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10475,7 +10480,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46090.6225462963</v>
+        <v>46090.70458333333</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10603,7 +10608,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46090.37709490741</v>
+        <v>46090.73652777778</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10731,7 +10736,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46090.65138888889</v>
+        <v>46090.7274537037</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10859,7 +10864,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46090.62674768519</v>
+        <v>46090.7033912037</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10987,7 +10992,7 @@
         <v>2</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46090.6369675926</v>
+        <v>46090.7144212963</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11051,7 +11056,7 @@
         <v>2</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46090.63697916667</v>
+        <v>46090.71396990741</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11179,7 +11184,7 @@
         <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46090.64609953704</v>
+        <v>46090.72565972222</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11243,7 +11248,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46090.6193287037</v>
+        <v>46090.69738425926</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11307,7 +11312,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46090.64023148148</v>
+        <v>46090.7199537037</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11371,7 +11376,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46090.64577546297</v>
+        <v>46090.7241087963</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11499,7 +11504,7 @@
         <v>2</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46090.63803240741</v>
+        <v>46090.71854166667</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11563,7 +11568,7 @@
         <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46090.6446412037</v>
+        <v>46090.71619212963</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11691,7 +11696,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46090.64597222222</v>
+        <v>46090.72565972222</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11755,7 +11760,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46090.61678240741</v>
+        <v>46090.6577662037</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11883,7 +11888,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46090.62944444444</v>
+        <v>46090.71303240741</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11947,7 +11952,7 @@
         <v>1</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46090.63055555556</v>
+        <v>46090.70820601852</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12011,7 +12016,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46090.61931712963</v>
+        <v>46090.73197916667</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12075,7 +12080,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46090.64403935185</v>
+        <v>46090.72195601852</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12400,7 +12405,7 @@
         <v>1</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46090.62696759259</v>
+        <v>46090.70774305556</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12464,7 +12469,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46090.6496412037</v>
+        <v>46090.73243055555</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12656,7 +12661,7 @@
         </is>
       </c>
       <c r="N188" s="3" t="n">
-        <v>46090.63974537037</v>
+        <v>46090.71673611111</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
@@ -12720,7 +12725,7 @@
         <v>1</v>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46090.64886574074</v>
+        <v>46090.72921296296</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12784,7 +12789,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46090.64983796296</v>
+        <v>46090.72880787037</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12973,7 +12978,7 @@
         <v>1</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46090.62991898148</v>
+        <v>46090.70128472222</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13037,7 +13042,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46090.61734953704</v>
+        <v>46090.69700231482</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13165,7 +13170,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46090.62885416667</v>
+        <v>46090.70969907408</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13293,7 +13298,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46090.65395833334</v>
+        <v>46090.73010416667</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13354,7 +13359,7 @@
         </is>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46090.63005787037</v>
+        <v>46090.71046296296</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13418,7 +13423,7 @@
         <v>1</v>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46090.63894675926</v>
+        <v>46090.71703703704</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13482,7 +13487,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46090.63679398148</v>
+        <v>46090.71844907408</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13546,7 +13551,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46090.62967592593</v>
+        <v>46090.71354166666</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13610,7 +13615,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46090.64898148148</v>
+        <v>46090.72761574074</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13674,7 +13679,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46090.6196875</v>
+        <v>46090.69767361111</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13738,7 +13743,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46090.63725694444</v>
+        <v>46090.72153935185</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13866,7 +13871,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46090.62011574074</v>
+        <v>46090.73368055555</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13930,7 +13935,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46090.64390046296</v>
+        <v>46090.723125</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -13994,7 +13999,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46090.62181712963</v>
+        <v>46090.73653935185</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14058,7 +14063,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46090.61716435185</v>
+        <v>46090.73131944444</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14122,7 +14127,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46090.57773148148</v>
+        <v>46090.71396990741</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14314,7 +14319,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46090.65435185185</v>
+        <v>46090.73134259259</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14378,7 +14383,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46090.64363425926</v>
+        <v>46090.72479166667</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14442,7 +14447,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46090.64123842592</v>
+        <v>46090.71638888889</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14506,7 +14511,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46090.5862037037</v>
+        <v>46090.66652777778</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14575,7 +14580,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46090.62451388889</v>
+        <v>46090.7034375</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14639,7 +14644,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46090.62549768519</v>
+        <v>46090.73387731481</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14767,7 +14772,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46090.64726851852</v>
+        <v>46090.72799768519</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14831,7 +14836,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46088.61790509259</v>
+        <v>46090.72858796296</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14895,7 +14900,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46090.6505787037</v>
+        <v>46090.72425925926</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -15023,7 +15028,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46090.6278587963</v>
+        <v>46090.71173611111</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15087,7 +15092,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46090.63539351852</v>
+        <v>46090.70938657408</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15151,7 +15156,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46090.62717592593</v>
+        <v>46090.70387731482</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15343,7 +15348,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46090.62568287037</v>
+        <v>46090.70677083333</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15407,7 +15412,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46090.64430555556</v>
+        <v>46090.7224074074</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15471,7 +15476,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46090.63908564814</v>
+        <v>46090.72375</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15535,7 +15540,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46090.64060185185</v>
+        <v>46090.71908564815</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15663,7 +15668,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46090.62363425926</v>
+        <v>46090.73337962963</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15855,7 +15860,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46090.65216435185</v>
+        <v>46090.7316087963</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15983,7 +15988,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46090.65033564815</v>
+        <v>46090.7300462963</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16047,7 +16052,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46090.64673611111</v>
+        <v>46090.72515046296</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16170,7 +16175,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46090.62888888889</v>
+        <v>46090.70607638889</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16234,7 +16239,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46090.64265046296</v>
+        <v>46090.72461805555</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16298,7 +16303,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46090.63956018518</v>
+        <v>46090.7219675926</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16362,7 +16367,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46090.64126157408</v>
+        <v>46090.69415509259</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16426,7 +16431,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46090.63493055556</v>
+        <v>46090.71126157408</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16485,7 +16490,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46090.63291666667</v>
+        <v>46090.70988425926</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16549,7 +16554,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46090.62336805555</v>
+        <v>46090.70482638889</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16613,7 +16618,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46090.40372685185</v>
+        <v>46090.72112268519</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16677,7 +16682,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46090.62039351852</v>
+        <v>46090.72445601852</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16735,7 +16740,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46090.61615740741</v>
+        <v>46090.73405092592</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16799,7 +16804,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46090.63628472222</v>
+        <v>46090.71571759259</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16863,7 +16868,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46090.63934027778</v>
+        <v>46090.71519675926</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16927,7 +16932,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46090.64236111111</v>
+        <v>46090.7237037037</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -16991,7 +16996,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46090.63674768519</v>
+        <v>46090.71030092592</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17055,7 +17060,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46090.62981481481</v>
+        <v>46090.71230324074</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17247,7 +17252,7 @@
         <v>1</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46090.6282175926</v>
+        <v>46090.70876157407</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17311,7 +17316,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46090.64314814815</v>
+        <v>46090.72306712963</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17375,7 +17380,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46090.62571759259</v>
+        <v>46090.70614583333</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17439,7 +17444,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46090.63366898148</v>
+        <v>46090.71072916667</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17567,7 +17572,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46090.65174768519</v>
+        <v>46090.73010416667</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17631,7 +17636,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46090.63290509259</v>
+        <v>46090.70945601852</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17695,7 +17700,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46090.64630787037</v>
+        <v>46090.72741898148</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17756,7 +17761,7 @@
         </is>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46090.64577546297</v>
+        <v>46090.72510416667</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -18257,7 +18262,7 @@
         <v>1</v>
       </c>
       <c r="N276" s="3" t="n">
-        <v>46090.62627314815</v>
+        <v>46090.70959490741</v>
       </c>
       <c r="O276" t="inlineStr">
         <is>
@@ -18321,7 +18326,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46090.63334490741</v>
+        <v>46090.71021990741</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18508,7 +18513,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46090.65142361111</v>
+        <v>46090.72686342592</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18572,7 +18577,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46090.63969907408</v>
+        <v>46090.71825231481</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18636,7 +18641,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46090.61768518519</v>
+        <v>46090.73679398148</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18700,7 +18705,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46090.61336805556</v>
+        <v>46090.73369212963</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18956,7 +18961,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46090.61842592592</v>
+        <v>46090.73402777778</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19094,7 +19099,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>10.69.5.170</t>
+          <t>10.69.2.55</t>
         </is>
       </c>
       <c r="D290" t="n">
@@ -19134,7 +19139,7 @@
         </is>
       </c>
       <c r="N290" s="3" t="n">
-        <v>45937.38847222222</v>
+        <v>46090.70981481481</v>
       </c>
       <c r="O290" t="inlineStr">
         <is>
@@ -19689,7 +19694,7 @@
         <v>1</v>
       </c>
       <c r="N299" s="3" t="n">
-        <v>46090.63841435185</v>
+        <v>46090.71451388889</v>
       </c>
       <c r="O299" t="inlineStr">
         <is>
@@ -20805,7 +20810,7 @@
         </is>
       </c>
       <c r="N317" s="3" t="n">
-        <v>46090.61793981482</v>
+        <v>46090.73289351852</v>
       </c>
       <c r="O317" t="inlineStr">
         <is>
@@ -21530,7 +21535,7 @@
         <v>1</v>
       </c>
       <c r="N329" s="3" t="n">
-        <v>46090.63883101852</v>
+        <v>46090.72127314815</v>
       </c>
       <c r="O329" t="inlineStr">
         <is>
@@ -21594,7 +21599,7 @@
         <v>2</v>
       </c>
       <c r="N330" s="3" t="n">
-        <v>46090.64981481482</v>
+        <v>46090.72320601852</v>
       </c>
       <c r="O330" t="inlineStr">
         <is>
@@ -21658,7 +21663,7 @@
         <v>2</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46090.63159722222</v>
+        <v>46090.71038194445</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21722,7 +21727,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46090.65061342593</v>
+        <v>46090.72608796296</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21786,7 +21791,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46090.64012731481</v>
+        <v>46090.67744212963</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21850,7 +21855,7 @@
         <v>1</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46090.64643518518</v>
+        <v>46090.72564814815</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21914,7 +21919,7 @@
         <v>2</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46090.62445601852</v>
+        <v>46090.73385416667</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21978,7 +21983,7 @@
         <v>2</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46090.63594907407</v>
+        <v>46090.71357638889</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22231,7 +22236,7 @@
         </is>
       </c>
       <c r="N340" s="3" t="n">
-        <v>46090.62061342593</v>
+        <v>46090.73674768519</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -22418,7 +22423,7 @@
         <v>1</v>
       </c>
       <c r="N343" s="3" t="n">
-        <v>46090.61981481482</v>
+        <v>46090.73085648148</v>
       </c>
       <c r="O343" t="inlineStr">
         <is>
@@ -22482,7 +22487,7 @@
         <v>1</v>
       </c>
       <c r="N344" s="3" t="n">
-        <v>46090.65255787037</v>
+        <v>46090.7315162037</v>
       </c>
       <c r="O344" t="inlineStr">
         <is>
@@ -22546,7 +22551,7 @@
         <v>1</v>
       </c>
       <c r="N345" s="3" t="n">
-        <v>46090.6362037037</v>
+        <v>46090.71246527778</v>
       </c>
       <c r="O345" t="inlineStr">
         <is>
@@ -22607,7 +22612,7 @@
         </is>
       </c>
       <c r="N346" s="3" t="n">
-        <v>46090.63268518518</v>
+        <v>46090.71013888889</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -22671,7 +22676,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46090.6177662037</v>
+        <v>46090.73429398148</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22735,7 +22740,7 @@
         <v>1</v>
       </c>
       <c r="N348" s="3" t="n">
-        <v>46090.63333333333</v>
+        <v>46090.70952546296</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -22796,7 +22801,7 @@
         </is>
       </c>
       <c r="N349" s="3" t="n">
-        <v>46090.63385416667</v>
+        <v>46090.70934027778</v>
       </c>
       <c r="O349" t="inlineStr">
         <is>
@@ -22862,7 +22867,7 @@
         </is>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46090.64925925926</v>
+        <v>46090.72428240741</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -22926,7 +22931,7 @@
         <v>1</v>
       </c>
       <c r="N351" s="3" t="n">
-        <v>46090.63042824074</v>
+        <v>46090.71317129629</v>
       </c>
       <c r="O351" t="inlineStr">
         <is>
@@ -22990,7 +22995,7 @@
         <v>1</v>
       </c>
       <c r="N352" s="3" t="n">
-        <v>46090.62754629629</v>
+        <v>46090.70506944445</v>
       </c>
       <c r="O352" t="inlineStr">
         <is>
@@ -23054,7 +23059,7 @@
         <v>1</v>
       </c>
       <c r="N353" s="3" t="n">
-        <v>46090.63325231482</v>
+        <v>46090.71192129629</v>
       </c>
       <c r="O353" t="inlineStr">
         <is>
@@ -23087,7 +23092,7 @@
         <v>1</v>
       </c>
       <c r="N354" s="3" t="n">
-        <v>46090.64662037037</v>
+        <v>46090.72910879629</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -23151,7 +23156,7 @@
         <v>2</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46090.62224537037</v>
+        <v>46090.70608796296</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23215,7 +23220,7 @@
         <v>2</v>
       </c>
       <c r="N356" s="3" t="n">
-        <v>46090.63077546296</v>
+        <v>46090.71278935186</v>
       </c>
       <c r="O356" t="inlineStr">
         <is>
@@ -23279,7 +23284,7 @@
         <v>1</v>
       </c>
       <c r="N357" s="3" t="n">
-        <v>46090.6366087963</v>
+        <v>46090.71460648148</v>
       </c>
       <c r="O357" t="inlineStr">
         <is>
@@ -23307,7 +23312,7 @@
         <v>1</v>
       </c>
       <c r="N358" s="3" t="n">
-        <v>46090.64178240741</v>
+        <v>46090.71971064815</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -23330,7 +23335,7 @@
         <v>1</v>
       </c>
       <c r="N359" s="3" t="n">
-        <v>46090.6193287037</v>
+        <v>46090.73712962963</v>
       </c>
       <c r="O359" t="inlineStr">
         <is>
@@ -23457,7 +23462,7 @@
         <v>1</v>
       </c>
       <c r="N361" s="3" t="n">
-        <v>46090.63865740741</v>
+        <v>46090.67503472222</v>
       </c>
       <c r="O361" t="inlineStr">
         <is>
@@ -23523,7 +23528,7 @@
         </is>
       </c>
       <c r="N362" s="3" t="n">
-        <v>46090.65148148148</v>
+        <v>46090.73091435185</v>
       </c>
       <c r="O362" t="inlineStr">
         <is>
@@ -23649,7 +23654,7 @@
         </is>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46090.63778935185</v>
+        <v>46090.67434027778</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23779,7 +23784,7 @@
         <v>1</v>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46090.63236111111</v>
+        <v>46090.70628472222</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
@@ -23807,7 +23812,7 @@
         <v>2</v>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46090.63650462963</v>
+        <v>46090.67349537037</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -23876,7 +23881,7 @@
         <v>1</v>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46090.62971064815</v>
+        <v>46090.66498842592</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24080,7 +24085,7 @@
         </is>
       </c>
       <c r="N371" s="3" t="n">
-        <v>46090.64346064815</v>
+        <v>46090.719375</v>
       </c>
       <c r="O371" t="inlineStr">
         <is>
@@ -24099,11 +24104,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C372" t="inlineStr">
-        <is>
-          <t>10.69.3.72</t>
-        </is>
-      </c>
       <c r="D372" t="n">
         <v>2025</v>
       </c>
@@ -24149,7 +24149,7 @@
         <v>1</v>
       </c>
       <c r="N372" s="3" t="n">
-        <v>46090.64954861111</v>
+        <v>46090.72101851852</v>
       </c>
       <c r="O372" t="inlineStr">
         <is>
@@ -24218,7 +24218,7 @@
         <v>2</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46090.62883101852</v>
+        <v>46090.70787037037</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24287,7 +24287,7 @@
         <v>2</v>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46090.6275</v>
+        <v>46090.71020833333</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-10 07:52:05.220034
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46090.7208912037</v>
+        <v>46091.30716435185</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46090.71043981481</v>
+        <v>46091.2983912037</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46090.7244212963</v>
+        <v>46090.7625</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46090.724375</v>
+        <v>46091.30769675926</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
         <v>1</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>46090.70019675926</v>
+        <v>46091.2818287037</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Windows</t>
+          <t>Microsoft Windows 7 Professional</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1190,7 +1190,7 @@
         <v>1</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>46090.72584490741</v>
+        <v>46091.26743055556</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1943,7 +1943,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46090.54105324074</v>
+        <v>46091.18637731481</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2178,7 +2178,7 @@
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46090.73277777778</v>
+        <v>46091.3140162037</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6573,7 +6573,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46090.71255787037</v>
+        <v>46090.82709490741</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6656,11 +6656,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>10.69.3.94</t>
-        </is>
-      </c>
       <c r="D97" t="n">
         <v>2025</v>
       </c>
@@ -6775,7 +6770,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46090.73159722222</v>
+        <v>46090.77138888889</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6844,7 +6839,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46090.72848379629</v>
+        <v>46091.30961805556</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6913,7 +6908,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46090.72636574074</v>
+        <v>46091.29398148148</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -7051,7 +7046,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46090.73282407408</v>
+        <v>46090.77542824074</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7446,7 +7441,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46090.71714120371</v>
+        <v>46091.29694444445</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7515,7 +7510,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46090.70832175926</v>
+        <v>46091.31166666667</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7653,7 +7648,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46090.7262962963</v>
+        <v>46091.31159722222</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7722,7 +7717,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46090.71447916667</v>
+        <v>46091.29461805556</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7791,7 +7786,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46090.70395833333</v>
+        <v>46091.28936342592</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7857,7 +7852,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46090.73685185185</v>
+        <v>46091.30846064815</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7995,7 +7990,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46090.684375</v>
+        <v>46091.31898148148</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8268,7 +8263,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46090.54766203704</v>
+        <v>46090.82616898148</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8403,7 +8398,7 @@
         <v>2</v>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46090.72726851852</v>
+        <v>46090.84603009259</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8472,7 +8467,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46090.73302083334</v>
+        <v>46091.31226851852</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8541,7 +8536,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46090.71278935186</v>
+        <v>46091.28494212963</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8679,7 +8674,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46090.73202546296</v>
+        <v>46091.30572916667</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8817,7 +8812,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46090.73658564815</v>
+        <v>46091.28334490741</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8886,7 +8881,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46090.72288194444</v>
+        <v>46090.79708333333</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -8950,7 +8945,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46090.70949074074</v>
+        <v>46090.74510416666</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9014,7 +9009,7 @@
         <v>1</v>
       </c>
       <c r="N131" s="3" t="n">
-        <v>46090.70780092593</v>
+        <v>46090.82747685185</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -9078,7 +9073,7 @@
         <v>1</v>
       </c>
       <c r="N132" s="3" t="n">
-        <v>46090.70758101852</v>
+        <v>46090.81717592593</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -9142,7 +9137,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46090.70351851852</v>
+        <v>46090.79936342593</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9333,7 +9328,7 @@
         <v>1</v>
       </c>
       <c r="N136" s="3" t="n">
-        <v>46090.69908564815</v>
+        <v>46090.81172453704</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -9397,7 +9392,7 @@
         <v>1</v>
       </c>
       <c r="N137" s="3" t="n">
-        <v>46090.73475694445</v>
+        <v>46090.81349537037</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -9461,7 +9456,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46090.72033564815</v>
+        <v>46090.79704861111</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9525,7 +9520,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46090.73034722222</v>
+        <v>46090.80644675926</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9589,7 +9584,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46090.71554398148</v>
+        <v>46090.79418981481</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9653,7 +9648,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46090.70430555556</v>
+        <v>46090.81510416666</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9717,7 +9712,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46090.71460648148</v>
+        <v>46090.7941087963</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9781,7 +9776,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46090.73222222222</v>
+        <v>46090.81020833334</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9845,7 +9840,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46090.69914351852</v>
+        <v>46090.81679398148</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9909,7 +9904,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46090.70489583333</v>
+        <v>46090.82053240741</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9973,7 +9968,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46090.73064814815</v>
+        <v>46090.85123842592</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10037,7 +10032,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46090.71935185185</v>
+        <v>46090.79208333333</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10101,7 +10096,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46090.70642361111</v>
+        <v>46090.82105324074</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10229,7 +10224,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46090.70982638889</v>
+        <v>46090.82715277778</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10248,6 +10243,11 @@
           <t>OPERACAO 7.1</t>
         </is>
       </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>10.69.5.85</t>
+        </is>
+      </c>
       <c r="D151" t="n">
         <v>2018</v>
       </c>
@@ -10288,7 +10288,7 @@
         <v>1</v>
       </c>
       <c r="N151" s="3" t="n">
-        <v>46090.71547453704</v>
+        <v>46090.87237268518</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -10352,7 +10352,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46090.7075</v>
+        <v>46090.82177083333</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10416,7 +10416,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46090.71189814815</v>
+        <v>46090.82085648148</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10480,7 +10480,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46090.70458333333</v>
+        <v>46090.82048611111</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10608,7 +10608,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46090.73652777778</v>
+        <v>46091.31403935186</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10736,7 +10736,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46090.7274537037</v>
+        <v>46090.81090277778</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10864,7 +10864,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46090.7033912037</v>
+        <v>46090.81864583334</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10989,10 +10989,10 @@
         </is>
       </c>
       <c r="M162" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46090.7144212963</v>
+        <v>46091.28747685185</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11056,7 +11056,7 @@
         <v>2</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46090.71396990741</v>
+        <v>46090.75048611111</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11312,7 +11312,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46090.7199537037</v>
+        <v>46091.319375</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11376,7 +11376,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46090.7241087963</v>
+        <v>46090.75980324074</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11565,10 +11565,10 @@
         </is>
       </c>
       <c r="M171" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46090.71619212963</v>
+        <v>46091.30586805556</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11696,7 +11696,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46090.72565972222</v>
+        <v>46091.30231481481</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11888,7 +11888,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46090.71303240741</v>
+        <v>46091.28649305556</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11952,7 +11952,7 @@
         <v>1</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46090.70820601852</v>
+        <v>46090.82122685185</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12016,7 +12016,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46090.73197916667</v>
+        <v>46090.80800925926</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12080,7 +12080,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46090.72195601852</v>
+        <v>46090.80582175926</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12405,7 +12405,7 @@
         <v>1</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46090.70774305556</v>
+        <v>46090.82577546296</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12469,7 +12469,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46090.73243055555</v>
+        <v>46091.30021990741</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12661,7 +12661,7 @@
         </is>
       </c>
       <c r="N188" s="3" t="n">
-        <v>46090.71673611111</v>
+        <v>46090.79686342592</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
@@ -12725,7 +12725,7 @@
         <v>1</v>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46090.72921296296</v>
+        <v>46090.80657407407</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12789,7 +12789,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46090.72880787037</v>
+        <v>46091.31800925926</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12978,7 +12978,7 @@
         <v>1</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46090.70128472222</v>
+        <v>46090.8184837963</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13042,7 +13042,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46090.69700231482</v>
+        <v>46090.8562962963</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13170,7 +13170,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46090.70969907408</v>
+        <v>46090.86125</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13298,7 +13298,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46090.73010416667</v>
+        <v>46090.80855324074</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13359,7 +13359,7 @@
         </is>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46090.71046296296</v>
+        <v>46090.82388888889</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13423,7 +13423,7 @@
         <v>1</v>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46090.71703703704</v>
+        <v>46090.7971875</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13487,7 +13487,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46090.71844907408</v>
+        <v>46090.82969907407</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13551,7 +13551,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46090.71354166666</v>
+        <v>46091.31756944444</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13615,7 +13615,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46090.72761574074</v>
+        <v>46090.80270833334</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13679,7 +13679,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46090.69767361111</v>
+        <v>46091.28270833333</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13743,7 +13743,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46090.72153935185</v>
+        <v>46090.7990625</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13871,7 +13871,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46090.73368055555</v>
+        <v>46090.80877314815</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13935,7 +13935,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46090.723125</v>
+        <v>46090.84145833334</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -13999,7 +13999,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46090.73653935185</v>
+        <v>46090.81447916666</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14063,7 +14063,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46090.73131944444</v>
+        <v>46090.81043981481</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14127,7 +14127,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46090.71396990741</v>
+        <v>46090.86604166667</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14319,7 +14319,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46090.73134259259</v>
+        <v>46090.80826388889</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14338,11 +14338,6 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
-      <c r="C215" t="inlineStr">
-        <is>
-          <t>10.69.5.85</t>
-        </is>
-      </c>
       <c r="D215" t="n">
         <v>2017</v>
       </c>
@@ -14383,7 +14378,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46090.72479166667</v>
+        <v>46090.8359837963</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14447,7 +14442,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46090.71638888889</v>
+        <v>46091.28858796296</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14511,7 +14506,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46090.66652777778</v>
+        <v>46091.26158564815</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14580,7 +14575,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46090.7034375</v>
+        <v>46090.82233796296</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14644,7 +14639,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46090.73387731481</v>
+        <v>46090.81008101852</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14772,7 +14767,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46090.72799768519</v>
+        <v>46090.80145833334</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14836,7 +14831,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46090.72858796296</v>
+        <v>46090.84946759259</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14900,7 +14895,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46090.72425925926</v>
+        <v>46090.84013888889</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -14964,7 +14959,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46090.61452546297</v>
+        <v>46091.2377662037</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15028,7 +15023,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46090.71173611111</v>
+        <v>46090.82773148148</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15092,7 +15087,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46090.70938657408</v>
+        <v>46090.78802083333</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15156,7 +15151,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46090.70387731482</v>
+        <v>46090.82256944444</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15220,7 +15215,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46090.54609953704</v>
+        <v>46091.31951388889</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15348,7 +15343,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46090.70677083333</v>
+        <v>46090.82722222222</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15412,7 +15407,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46090.7224074074</v>
+        <v>46090.8009375</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15476,7 +15471,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46090.72375</v>
+        <v>46090.80135416667</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15540,7 +15535,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46090.71908564815</v>
+        <v>46090.84180555555</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15668,7 +15663,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46090.73337962963</v>
+        <v>46091.31357638889</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15860,7 +15855,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46090.7316087963</v>
+        <v>46090.81212962963</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15988,7 +15983,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46090.7300462963</v>
+        <v>46090.80538194445</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16052,7 +16047,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46090.72515046296</v>
+        <v>46090.80076388889</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16071,6 +16066,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>10.69.5.112</t>
+        </is>
+      </c>
       <c r="D242" t="n">
         <v>2019</v>
       </c>
@@ -16111,7 +16111,7 @@
         <v>1</v>
       </c>
       <c r="N242" s="3" t="n">
-        <v>46090.44866898148</v>
+        <v>46091.20150462963</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -16175,7 +16175,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46090.70607638889</v>
+        <v>46090.81695601852</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16239,7 +16239,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46090.72461805555</v>
+        <v>46090.80371527778</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16303,7 +16303,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46090.7219675926</v>
+        <v>46090.79925925926</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16431,7 +16431,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46090.71126157408</v>
+        <v>46090.82715277778</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16490,7 +16490,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46090.70988425926</v>
+        <v>46090.82106481482</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16554,7 +16554,7 @@
         <v>1</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>46090.70482638889</v>
+        <v>46090.78440972222</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -16618,7 +16618,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46090.72112268519</v>
+        <v>46091.32008101852</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16682,7 +16682,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46090.72445601852</v>
+        <v>46091.3165625</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16740,7 +16740,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46090.73405092592</v>
+        <v>46090.81273148148</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16804,7 +16804,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46090.71571759259</v>
+        <v>46091.31601851852</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16868,7 +16868,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46090.71519675926</v>
+        <v>46091.31659722222</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16932,7 +16932,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46090.7237037037</v>
+        <v>46090.81640046297</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -16996,7 +16996,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46090.71030092592</v>
+        <v>46090.82679398148</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17060,7 +17060,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46090.71230324074</v>
+        <v>46091.29612268518</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17252,7 +17252,7 @@
         <v>1</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46090.70876157407</v>
+        <v>46090.82313657407</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17316,7 +17316,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46090.72306712963</v>
+        <v>46090.79819444445</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17380,7 +17380,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46090.70614583333</v>
+        <v>46090.82032407408</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17444,7 +17444,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46090.71072916667</v>
+        <v>46090.82666666667</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17572,7 +17572,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46090.73010416667</v>
+        <v>46090.81144675926</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17636,7 +17636,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46090.70945601852</v>
+        <v>46090.82424768519</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17700,7 +17700,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46090.72741898148</v>
+        <v>46090.80217592593</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17761,7 +17761,7 @@
         </is>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46090.72510416667</v>
+        <v>46091.28130787037</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -18262,7 +18262,7 @@
         <v>1</v>
       </c>
       <c r="N276" s="3" t="n">
-        <v>46090.70959490741</v>
+        <v>46090.78663194444</v>
       </c>
       <c r="O276" t="inlineStr">
         <is>
@@ -18326,7 +18326,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46090.71021990741</v>
+        <v>46091.29998842593</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18513,7 +18513,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46090.72686342592</v>
+        <v>46091.30475694445</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18577,7 +18577,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46090.71825231481</v>
+        <v>46091.31758101852</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18641,7 +18641,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46090.73679398148</v>
+        <v>46090.87267361111</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18705,7 +18705,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46090.73369212963</v>
+        <v>46090.81214120371</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18724,11 +18724,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C284" t="inlineStr">
-        <is>
-          <t>10.69.5.155</t>
-        </is>
-      </c>
       <c r="D284" t="n">
         <v>2019</v>
       </c>
@@ -18769,7 +18764,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46090.56362268519</v>
+        <v>46091.12612268519</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18897,7 +18892,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46090.54790509259</v>
+        <v>46091.31533564815</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18961,7 +18956,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46090.73402777778</v>
+        <v>46090.84643518519</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19139,7 +19134,7 @@
         </is>
       </c>
       <c r="N290" s="3" t="n">
-        <v>46090.70981481481</v>
+        <v>46091.29744212963</v>
       </c>
       <c r="O290" t="inlineStr">
         <is>
@@ -19694,7 +19689,7 @@
         <v>1</v>
       </c>
       <c r="N299" s="3" t="n">
-        <v>46090.71451388889</v>
+        <v>46091.29557870371</v>
       </c>
       <c r="O299" t="inlineStr">
         <is>
@@ -21535,7 +21530,7 @@
         <v>1</v>
       </c>
       <c r="N329" s="3" t="n">
-        <v>46090.72127314815</v>
+        <v>46090.75836805555</v>
       </c>
       <c r="O329" t="inlineStr">
         <is>
@@ -21599,7 +21594,7 @@
         <v>2</v>
       </c>
       <c r="N330" s="3" t="n">
-        <v>46090.72320601852</v>
+        <v>46091.31903935185</v>
       </c>
       <c r="O330" t="inlineStr">
         <is>
@@ -21663,7 +21658,7 @@
         <v>2</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46090.71038194445</v>
+        <v>46091.28393518519</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21727,7 +21722,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46090.72608796296</v>
+        <v>46091.28341435185</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21791,7 +21786,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46090.67744212963</v>
+        <v>46091.28347222223</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21855,7 +21850,7 @@
         <v>1</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46090.72564814815</v>
+        <v>46091.29082175926</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21919,7 +21914,7 @@
         <v>2</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46090.73385416667</v>
+        <v>46090.77055555556</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21983,7 +21978,7 @@
         <v>2</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46090.71357638889</v>
+        <v>46091.2909375</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22236,7 +22231,7 @@
         </is>
       </c>
       <c r="N340" s="3" t="n">
-        <v>46090.73674768519</v>
+        <v>46091.3116087963</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -22801,7 +22796,7 @@
         </is>
       </c>
       <c r="N349" s="3" t="n">
-        <v>46090.70934027778</v>
+        <v>46090.74628472222</v>
       </c>
       <c r="O349" t="inlineStr">
         <is>
@@ -22867,7 +22862,7 @@
         </is>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46090.72428240741</v>
+        <v>46091.30444444445</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -23528,7 +23523,7 @@
         </is>
       </c>
       <c r="N362" s="3" t="n">
-        <v>46090.73091435185</v>
+        <v>46091.3109837963</v>
       </c>
       <c r="O362" t="inlineStr">
         <is>
@@ -23784,7 +23779,7 @@
         <v>1</v>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46090.70628472222</v>
+        <v>46090.74696759259</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
@@ -24085,7 +24080,7 @@
         </is>
       </c>
       <c r="N371" s="3" t="n">
-        <v>46090.719375</v>
+        <v>46091.29601851852</v>
       </c>
       <c r="O371" t="inlineStr">
         <is>
@@ -24104,6 +24099,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>10.69.3.72</t>
+        </is>
+      </c>
       <c r="D372" t="n">
         <v>2025</v>
       </c>
@@ -24149,7 +24149,7 @@
         <v>1</v>
       </c>
       <c r="N372" s="3" t="n">
-        <v>46090.72101851852</v>
+        <v>46090.80238425926</v>
       </c>
       <c r="O372" t="inlineStr">
         <is>
@@ -24287,7 +24287,7 @@
         <v>2</v>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46090.71020833333</v>
+        <v>46091.29577546296</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-10 09:52:06.457513
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46091.30716435185</v>
+        <v>46091.38413194445</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46091.2983912037</v>
+        <v>46091.38047453704</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46090.7625</v>
+        <v>46091.39585648148</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46091.30769675926</v>
+        <v>46091.38664351852</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
         <v>1</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>46091.2818287037</v>
+        <v>46091.3996875</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1190,7 +1190,7 @@
         <v>1</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>46091.26743055556</v>
+        <v>46091.33005787037</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -2178,7 +2178,7 @@
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46091.3140162037</v>
+        <v>46091.38960648148</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6504,7 +6504,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46090.71146990741</v>
+        <v>46091.3721875</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6592,6 +6592,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>10.69.3.93</t>
+        </is>
+      </c>
       <c r="D96" t="n">
         <v>2025</v>
       </c>
@@ -6637,7 +6642,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46090.70815972222</v>
+        <v>46091.40369212963</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6701,7 +6706,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46090.72395833334</v>
+        <v>46091.36950231482</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6770,7 +6775,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46090.77138888889</v>
+        <v>46091.37574074074</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6839,7 +6844,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46091.30961805556</v>
+        <v>46091.38549768519</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6908,7 +6913,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46091.29398148148</v>
+        <v>46091.37432870371</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -7441,7 +7446,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46091.29694444445</v>
+        <v>46091.37930555556</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7510,7 +7515,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46091.31166666667</v>
+        <v>46091.39126157408</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7579,7 +7584,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46090.69998842593</v>
+        <v>46091.3710300926</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7648,7 +7653,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46091.31159722222</v>
+        <v>46091.38686342593</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7717,7 +7722,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46091.29461805556</v>
+        <v>46091.37453703704</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7786,7 +7791,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46091.28936342592</v>
+        <v>46091.40247685185</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7852,7 +7857,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46091.30846064815</v>
+        <v>46091.38608796296</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7921,7 +7926,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46090.67440972223</v>
+        <v>46091.37875</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7990,7 +7995,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46091.31898148148</v>
+        <v>46091.39376157407</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8056,7 +8061,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46090.6825</v>
+        <v>46091.40070601852</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8194,7 +8199,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46090.69013888889</v>
+        <v>46091.38135416667</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8329,7 +8334,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46090.67686342593</v>
+        <v>46091.39883101852</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8467,7 +8472,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46091.31226851852</v>
+        <v>46091.38671296297</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8536,7 +8541,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46091.28494212963</v>
+        <v>46091.40116898148</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8605,7 +8610,7 @@
         <v>2</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46087.77148148148</v>
+        <v>46091.37450231481</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8674,7 +8679,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46091.30572916667</v>
+        <v>46091.38578703703</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8743,7 +8748,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46090.69086805556</v>
+        <v>46091.37094907407</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8812,7 +8817,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46091.28334490741</v>
+        <v>46091.39594907407</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8881,7 +8886,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46090.79708333333</v>
+        <v>46091.37119212963</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -9009,7 +9014,7 @@
         <v>1</v>
       </c>
       <c r="N131" s="3" t="n">
-        <v>46090.82747685185</v>
+        <v>46091.39922453704</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -9328,7 +9333,7 @@
         <v>1</v>
       </c>
       <c r="N136" s="3" t="n">
-        <v>46090.81172453704</v>
+        <v>46091.38291666667</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -9520,7 +9525,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46090.80644675926</v>
+        <v>46091.37829861111</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9584,7 +9589,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46090.79418981481</v>
+        <v>46091.38737268518</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9648,7 +9653,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46090.81510416666</v>
+        <v>46091.38050925926</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9712,7 +9717,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46090.7941087963</v>
+        <v>46091.37800925926</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9776,7 +9781,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46090.81020833334</v>
+        <v>46091.38976851852</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9840,7 +9845,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46090.81679398148</v>
+        <v>46091.37188657407</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9904,7 +9909,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46090.82053240741</v>
+        <v>46091.39884259259</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9968,7 +9973,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46090.85123842592</v>
+        <v>46091.38561342593</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10032,7 +10037,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46090.79208333333</v>
+        <v>46091.38710648148</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10224,7 +10229,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46090.82715277778</v>
+        <v>46091.37731481482</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10243,11 +10248,6 @@
           <t>OPERACAO 7.1</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>10.69.5.85</t>
-        </is>
-      </c>
       <c r="D151" t="n">
         <v>2018</v>
       </c>
@@ -10352,7 +10352,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46090.82177083333</v>
+        <v>46091.37122685185</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10480,7 +10480,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46090.82048611111</v>
+        <v>46091.36431712963</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10544,7 +10544,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46090.57751157408</v>
+        <v>46091.37195601852</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10608,7 +10608,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46091.31403935186</v>
+        <v>46091.39344907407</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10672,7 +10672,7 @@
         <v>1</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>46090.52734953703</v>
+        <v>46091.37946759259</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -10736,7 +10736,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46090.81090277778</v>
+        <v>46091.37126157407</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10800,7 +10800,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46090.56813657407</v>
+        <v>46091.38789351852</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10864,7 +10864,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46090.81864583334</v>
+        <v>46091.37732638889</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10925,10 +10925,10 @@
         </is>
       </c>
       <c r="M161" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46090.55627314815</v>
+        <v>46091.35789351852</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -10989,10 +10989,10 @@
         </is>
       </c>
       <c r="M162" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46091.28747685185</v>
+        <v>46091.36825231482</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11120,7 +11120,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46090.64833333333</v>
+        <v>46091.37152777778</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11181,10 +11181,10 @@
         </is>
       </c>
       <c r="M165" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46090.72565972222</v>
+        <v>46091.37351851852</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11248,7 +11248,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46090.69738425926</v>
+        <v>46091.40390046296</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11312,7 +11312,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46091.319375</v>
+        <v>46091.39545138889</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11376,7 +11376,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46090.75980324074</v>
+        <v>46091.37930555556</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11565,10 +11565,10 @@
         </is>
       </c>
       <c r="M171" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46091.30586805556</v>
+        <v>46091.3863425926</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11632,7 +11632,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46090.53986111111</v>
+        <v>46091.38998842592</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11696,7 +11696,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46091.30231481481</v>
+        <v>46091.38540509259</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11888,7 +11888,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46091.28649305556</v>
+        <v>46091.36443287037</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11952,7 +11952,7 @@
         <v>1</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46090.82122685185</v>
+        <v>46091.36556712963</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12341,7 +12341,7 @@
         <v>1</v>
       </c>
       <c r="N183" s="3" t="n">
-        <v>46088.60638888889</v>
+        <v>46091.36527777778</v>
       </c>
       <c r="O183" t="inlineStr">
         <is>
@@ -12405,7 +12405,7 @@
         <v>1</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46090.82577546296</v>
+        <v>46091.36651620371</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12469,7 +12469,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46091.30021990741</v>
+        <v>46091.36959490741</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12533,7 +12533,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46090.56700231481</v>
+        <v>46091.38211805555</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12661,7 +12661,7 @@
         </is>
       </c>
       <c r="N188" s="3" t="n">
-        <v>46090.79686342592</v>
+        <v>46091.38475694445</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
@@ -12725,7 +12725,7 @@
         <v>1</v>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46090.80657407407</v>
+        <v>46091.39648148148</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12789,7 +12789,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46091.31800925926</v>
+        <v>46091.39354166666</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12914,7 +12914,7 @@
         <v>2</v>
       </c>
       <c r="N192" s="3" t="n">
-        <v>46090.64215277778</v>
+        <v>46091.37446759259</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
@@ -12978,7 +12978,7 @@
         <v>1</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46090.8184837963</v>
+        <v>46091.37728009259</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13042,7 +13042,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46090.8562962963</v>
+        <v>46091.40446759259</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13106,7 +13106,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46090.57171296296</v>
+        <v>46091.37707175926</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13170,7 +13170,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46090.86125</v>
+        <v>46091.36515046296</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13234,7 +13234,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46088.58556712963</v>
+        <v>46091.36805555555</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13423,7 +13423,7 @@
         <v>1</v>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46090.7971875</v>
+        <v>46091.39719907408</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13487,7 +13487,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46090.82969907407</v>
+        <v>46091.38642361111</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13551,7 +13551,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46091.31756944444</v>
+        <v>46091.39642361111</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13615,7 +13615,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46090.80270833334</v>
+        <v>46091.37061342593</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13679,7 +13679,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46091.28270833333</v>
+        <v>46091.4021875</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13743,7 +13743,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46090.7990625</v>
+        <v>46091.36467592593</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13807,7 +13807,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46090.54067129629</v>
+        <v>46091.37828703703</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13871,7 +13871,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46090.80877314815</v>
+        <v>46091.40078703704</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13935,7 +13935,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46090.84145833334</v>
+        <v>46091.38277777778</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -13999,7 +13999,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46090.81447916666</v>
+        <v>46091.3890625</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14063,7 +14063,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46090.81043981481</v>
+        <v>46091.38818287037</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14127,7 +14127,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46090.86604166667</v>
+        <v>46091.39105324074</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14191,7 +14191,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46090.32711805555</v>
+        <v>46091.39104166667</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14255,7 +14255,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46088.48796296296</v>
+        <v>46091.38839120371</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14319,7 +14319,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46090.80826388889</v>
+        <v>46091.39395833333</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14338,6 +14338,11 @@
           <t>OPERACAO 8.1</t>
         </is>
       </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>10.69.5.85</t>
+        </is>
+      </c>
       <c r="D215" t="n">
         <v>2017</v>
       </c>
@@ -14378,7 +14383,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46090.8359837963</v>
+        <v>46091.38870370371</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14442,7 +14447,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46091.28858796296</v>
+        <v>46091.40310185185</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14506,7 +14511,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46091.26158564815</v>
+        <v>46091.37175925926</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14575,7 +14580,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46090.82233796296</v>
+        <v>46091.38142361111</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14639,7 +14644,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46090.81008101852</v>
+        <v>46091.3821875</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14703,7 +14708,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46088.60734953704</v>
+        <v>46091.39038194445</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14767,7 +14772,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46090.80145833334</v>
+        <v>46091.37961805556</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14831,7 +14836,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46090.84946759259</v>
+        <v>46091.36796296296</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14959,7 +14964,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46091.2377662037</v>
+        <v>46091.36611111111</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15023,7 +15028,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46090.82773148148</v>
+        <v>46091.39908564815</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15087,7 +15092,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46090.78802083333</v>
+        <v>46091.36684027778</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15151,7 +15156,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46090.82256944444</v>
+        <v>46091.39215277778</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15215,7 +15220,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46091.31951388889</v>
+        <v>46091.39840277778</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15279,7 +15284,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46090.46701388889</v>
+        <v>46091.37600694445</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15343,7 +15348,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46090.82722222222</v>
+        <v>46091.36783564815</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15407,7 +15412,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46090.8009375</v>
+        <v>46091.38172453704</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15471,7 +15476,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46090.80135416667</v>
+        <v>46091.39039351852</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15599,7 +15604,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46090.57744212963</v>
+        <v>46091.38012731481</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15663,7 +15668,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46091.31357638889</v>
+        <v>46091.39243055556</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15727,7 +15732,7 @@
         <v>1</v>
       </c>
       <c r="N236" s="3" t="n">
-        <v>46090.63512731482</v>
+        <v>46091.34369212963</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -15791,7 +15796,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46090.55576388889</v>
+        <v>46091.39079861111</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15855,7 +15860,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46090.81212962963</v>
+        <v>46091.36538194444</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15983,7 +15988,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46090.80538194445</v>
+        <v>46091.37670138889</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16047,7 +16052,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46090.80076388889</v>
+        <v>46091.37489583333</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16066,11 +16071,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C242" t="inlineStr">
-        <is>
-          <t>10.69.5.112</t>
-        </is>
-      </c>
       <c r="D242" t="n">
         <v>2019</v>
       </c>
@@ -16175,7 +16175,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46090.81695601852</v>
+        <v>46091.40203703703</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16239,7 +16239,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46090.80371527778</v>
+        <v>46091.39828703704</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16303,7 +16303,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46090.79925925926</v>
+        <v>46091.38695601852</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16367,7 +16367,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46090.69415509259</v>
+        <v>46091.38436342592</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16431,7 +16431,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46090.82715277778</v>
+        <v>46091.40449074074</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16450,6 +16450,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>10.69.5.118</t>
+        </is>
+      </c>
       <c r="D248" t="n">
         <v>2017</v>
       </c>
@@ -16490,7 +16495,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46090.82106481482</v>
+        <v>46091.3877662037</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16618,7 +16623,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46091.32008101852</v>
+        <v>46091.39806712963</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16682,7 +16687,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46091.3165625</v>
+        <v>46091.39613425926</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16740,7 +16745,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46090.81273148148</v>
+        <v>46091.37241898148</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16804,7 +16809,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46091.31601851852</v>
+        <v>46091.40368055556</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16868,7 +16873,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46091.31659722222</v>
+        <v>46091.40246527778</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16932,7 +16937,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46090.81640046297</v>
+        <v>46091.37336805555</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -16996,7 +17001,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46090.82679398148</v>
+        <v>46091.39302083333</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17060,7 +17065,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46091.29612268518</v>
+        <v>46091.3768287037</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17124,7 +17129,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46090.60371527778</v>
+        <v>46091.37460648148</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17316,7 +17321,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46090.79819444445</v>
+        <v>46091.40023148148</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17380,7 +17385,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46090.82032407408</v>
+        <v>46091.36902777778</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17444,7 +17449,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46090.82666666667</v>
+        <v>46091.40206018519</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17508,7 +17513,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46090.63931712963</v>
+        <v>46091.37924768519</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17572,7 +17577,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46090.81144675926</v>
+        <v>46091.37487268518</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17761,7 +17766,7 @@
         </is>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46091.28130787037</v>
+        <v>46091.40123842593</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17889,7 +17894,7 @@
         <v>1</v>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46090.63755787037</v>
+        <v>46091.38575231482</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -18262,7 +18267,7 @@
         <v>1</v>
       </c>
       <c r="N276" s="3" t="n">
-        <v>46090.78663194444</v>
+        <v>46091.36653935185</v>
       </c>
       <c r="O276" t="inlineStr">
         <is>
@@ -18326,7 +18331,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46091.29998842593</v>
+        <v>46091.38353009259</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18449,7 +18454,7 @@
         <v>1</v>
       </c>
       <c r="N279" s="3" t="n">
-        <v>46090.5778587963</v>
+        <v>46091.38575231482</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -18468,11 +18473,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C280" t="inlineStr">
-        <is>
-          <t>10.69.5.151</t>
-        </is>
-      </c>
       <c r="D280" t="n">
         <v>2017</v>
       </c>
@@ -18513,7 +18513,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46091.30475694445</v>
+        <v>46091.38179398148</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18577,7 +18577,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46091.31758101852</v>
+        <v>46091.39811342592</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18641,7 +18641,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46090.87267361111</v>
+        <v>46091.4027662037</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18705,7 +18705,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46090.81214120371</v>
+        <v>46091.37783564815</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18724,6 +18724,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>10.69.5.155</t>
+        </is>
+      </c>
       <c r="D284" t="n">
         <v>2019</v>
       </c>
@@ -18764,7 +18769,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46091.12612268519</v>
+        <v>46091.36609953704</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18892,7 +18897,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46091.31533564815</v>
+        <v>46091.36555555555</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -19134,7 +19139,7 @@
         </is>
       </c>
       <c r="N290" s="3" t="n">
-        <v>46091.29744212963</v>
+        <v>46091.37430555555</v>
       </c>
       <c r="O290" t="inlineStr">
         <is>
@@ -19564,7 +19569,7 @@
         <v>1</v>
       </c>
       <c r="N297" s="3" t="n">
-        <v>45895.86393518518</v>
+        <v>46091.40252314815</v>
       </c>
       <c r="O297" t="inlineStr">
         <is>
@@ -19689,7 +19694,7 @@
         <v>1</v>
       </c>
       <c r="N299" s="3" t="n">
-        <v>46091.29557870371</v>
+        <v>46091.37688657407</v>
       </c>
       <c r="O299" t="inlineStr">
         <is>
@@ -20494,7 +20499,7 @@
         <v>1</v>
       </c>
       <c r="N312" s="3" t="n">
-        <v>46090.45797453704</v>
+        <v>46091.37824074074</v>
       </c>
       <c r="O312" t="inlineStr">
         <is>
@@ -21530,7 +21535,7 @@
         <v>1</v>
       </c>
       <c r="N329" s="3" t="n">
-        <v>46090.75836805555</v>
+        <v>46091.40266203704</v>
       </c>
       <c r="O329" t="inlineStr">
         <is>
@@ -21594,7 +21599,7 @@
         <v>2</v>
       </c>
       <c r="N330" s="3" t="n">
-        <v>46091.31903935185</v>
+        <v>46091.40290509259</v>
       </c>
       <c r="O330" t="inlineStr">
         <is>
@@ -21658,7 +21663,7 @@
         <v>2</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46091.28393518519</v>
+        <v>46091.36884259259</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21722,7 +21727,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46091.28341435185</v>
+        <v>46091.40347222222</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21786,7 +21791,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46091.28347222223</v>
+        <v>46091.39510416667</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21850,7 +21855,7 @@
         <v>1</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46091.29082175926</v>
+        <v>46091.37240740741</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21914,7 +21919,7 @@
         <v>2</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46090.77055555556</v>
+        <v>46091.37530092592</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21978,7 +21983,7 @@
         <v>2</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46091.2909375</v>
+        <v>46091.37076388889</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22106,7 +22111,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46090.5733912037</v>
+        <v>46091.37349537037</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22231,7 +22236,7 @@
         </is>
       </c>
       <c r="N340" s="3" t="n">
-        <v>46091.3116087963</v>
+        <v>46091.38570601852</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -22862,7 +22867,7 @@
         </is>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46091.30444444445</v>
+        <v>46091.38141203704</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -23457,7 +23462,7 @@
         <v>1</v>
       </c>
       <c r="N361" s="3" t="n">
-        <v>46090.67503472222</v>
+        <v>46091.36630787037</v>
       </c>
       <c r="O361" t="inlineStr">
         <is>
@@ -23523,7 +23528,7 @@
         </is>
       </c>
       <c r="N362" s="3" t="n">
-        <v>46091.3109837963</v>
+        <v>46091.38306712963</v>
       </c>
       <c r="O362" t="inlineStr">
         <is>
@@ -23649,7 +23654,7 @@
         </is>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46090.67434027778</v>
+        <v>46091.36879629629</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23779,7 +23784,7 @@
         <v>1</v>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46090.74696759259</v>
+        <v>46091.3700925926</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
@@ -23807,7 +23812,7 @@
         <v>2</v>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46090.67349537037</v>
+        <v>46091.37094907407</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -23839,7 +23844,7 @@
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t>Windows</t>
+          <t>Microsoft Windows 11 Pro</t>
         </is>
       </c>
       <c r="G368" t="inlineStr">
@@ -23876,7 +23881,7 @@
         <v>1</v>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46090.66498842592</v>
+        <v>46091.37864583333</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24080,7 +24085,7 @@
         </is>
       </c>
       <c r="N371" s="3" t="n">
-        <v>46091.29601851852</v>
+        <v>46091.3749537037</v>
       </c>
       <c r="O371" t="inlineStr">
         <is>
@@ -24099,11 +24104,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C372" t="inlineStr">
-        <is>
-          <t>10.69.3.72</t>
-        </is>
-      </c>
       <c r="D372" t="n">
         <v>2025</v>
       </c>
@@ -24218,7 +24218,7 @@
         <v>2</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46090.70787037037</v>
+        <v>46091.39199074074</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24287,7 +24287,7 @@
         <v>2</v>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46091.29577546296</v>
+        <v>46091.37211805556</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-10 11:52:05.441410
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46091.38413194445</v>
+        <v>46091.46369212963</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46091.38047453704</v>
+        <v>46091.46114583333</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46091.39585648148</v>
+        <v>46091.47986111111</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46091.38664351852</v>
+        <v>46091.46797453704</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
         <v>1</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>46091.3996875</v>
+        <v>46091.47511574074</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1190,7 +1190,7 @@
         <v>1</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>46091.33005787037</v>
+        <v>46091.48385416667</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -2178,7 +2178,7 @@
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46091.38960648148</v>
+        <v>46091.47332175926</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6504,7 +6504,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46091.3721875</v>
+        <v>46091.44981481481</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6573,7 +6573,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46090.82709490741</v>
+        <v>46091.45435185185</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6592,11 +6592,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>10.69.3.93</t>
-        </is>
-      </c>
       <c r="D96" t="n">
         <v>2025</v>
       </c>
@@ -6642,7 +6637,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46091.40369212963</v>
+        <v>46091.48322916667</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6706,7 +6701,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46091.36950231482</v>
+        <v>46091.44771990741</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6775,7 +6770,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46091.37574074074</v>
+        <v>46091.45234953704</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6844,7 +6839,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46091.38549768519</v>
+        <v>46091.45945601852</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6913,7 +6908,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46091.37432870371</v>
+        <v>46091.4871412037</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -7051,7 +7046,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46090.77542824074</v>
+        <v>46091.46678240741</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7446,7 +7441,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46091.37930555556</v>
+        <v>46091.45722222222</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7515,7 +7510,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46091.39126157408</v>
+        <v>46091.47098379629</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7584,7 +7579,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46091.3710300926</v>
+        <v>46091.44646990741</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7653,7 +7648,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46091.38686342593</v>
+        <v>46091.46883101852</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7722,7 +7717,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46091.37453703704</v>
+        <v>46091.45407407408</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7791,7 +7786,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46091.40247685185</v>
+        <v>46091.48274305555</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7857,7 +7852,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46091.38608796296</v>
+        <v>46091.46746527778</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7926,7 +7921,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46091.37875</v>
+        <v>46091.46118055555</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7995,7 +7990,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46091.39376157407</v>
+        <v>46091.46903935185</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8061,7 +8056,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46091.40070601852</v>
+        <v>46091.47358796297</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8199,7 +8194,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46091.38135416667</v>
+        <v>46091.46296296296</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8268,7 +8263,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46090.82616898148</v>
+        <v>46091.48207175926</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8334,7 +8329,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46091.39883101852</v>
+        <v>46091.47635416667</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8403,7 +8398,7 @@
         <v>2</v>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46090.84603009259</v>
+        <v>46091.48401620371</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8472,7 +8467,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46091.38671296297</v>
+        <v>46091.46603009259</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8541,7 +8536,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46091.40116898148</v>
+        <v>46091.47802083333</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8610,7 +8605,7 @@
         <v>2</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46091.37450231481</v>
+        <v>46091.45321759259</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8679,7 +8674,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46091.38578703703</v>
+        <v>46091.46395833333</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8748,7 +8743,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46091.37094907407</v>
+        <v>46091.48739583333</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8817,7 +8812,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46091.39594907407</v>
+        <v>46091.47376157407</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8886,7 +8881,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46091.37119212963</v>
+        <v>46091.48302083334</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -8905,6 +8900,11 @@
           <t>ADM/FIN</t>
         </is>
       </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>10.69.3.6</t>
+        </is>
+      </c>
       <c r="D130" t="n">
         <v>2025</v>
       </c>
@@ -8950,7 +8950,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46090.74510416666</v>
+        <v>46091.48386574074</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9014,7 +9014,7 @@
         <v>1</v>
       </c>
       <c r="N131" s="3" t="n">
-        <v>46091.39922453704</v>
+        <v>46091.48234953704</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -9333,7 +9333,7 @@
         <v>1</v>
       </c>
       <c r="N136" s="3" t="n">
-        <v>46091.38291666667</v>
+        <v>46091.46390046296</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -9525,7 +9525,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46091.37829861111</v>
+        <v>46091.44984953704</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9589,7 +9589,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46091.38737268518</v>
+        <v>46091.46534722222</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9653,7 +9653,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46091.38050925926</v>
+        <v>46091.45607638889</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9717,7 +9717,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46091.37800925926</v>
+        <v>46091.46028935185</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9781,7 +9781,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46091.38976851852</v>
+        <v>46091.46546296297</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9845,7 +9845,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46091.37188657407</v>
+        <v>46091.45329861111</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9909,7 +9909,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46091.39884259259</v>
+        <v>46091.4727199074</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9973,7 +9973,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46091.38561342593</v>
+        <v>46091.42211805555</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10037,7 +10037,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46091.38710648148</v>
+        <v>46091.46130787037</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10229,7 +10229,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46091.37731481482</v>
+        <v>46091.45222222222</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10352,7 +10352,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46091.37122685185</v>
+        <v>46091.48655092593</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10480,7 +10480,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46091.36431712963</v>
+        <v>46091.48503472222</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10544,7 +10544,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46091.37195601852</v>
+        <v>46091.45207175926</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10608,7 +10608,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46091.39344907407</v>
+        <v>46091.46974537037</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10672,7 +10672,7 @@
         <v>1</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>46091.37946759259</v>
+        <v>46091.46071759259</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -10736,7 +10736,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46091.37126157407</v>
+        <v>46091.48232638889</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10800,7 +10800,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46091.38789351852</v>
+        <v>46091.46599537037</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10864,7 +10864,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46091.37732638889</v>
+        <v>46091.45408564815</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10992,7 +10992,7 @@
         <v>2</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46091.36825231482</v>
+        <v>46091.48663194444</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11120,7 +11120,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46091.37152777778</v>
+        <v>46091.4855787037</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11181,10 +11181,10 @@
         </is>
       </c>
       <c r="M165" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46091.37351851852</v>
+        <v>46091.45199074074</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11248,7 +11248,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46091.40390046296</v>
+        <v>46091.4766087963</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11312,7 +11312,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46091.39545138889</v>
+        <v>46091.47267361111</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11376,7 +11376,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46091.37930555556</v>
+        <v>46091.45429398148</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11568,7 +11568,7 @@
         <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46091.3863425926</v>
+        <v>46091.46534722222</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11632,7 +11632,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46091.38998842592</v>
+        <v>46091.46649305556</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11696,7 +11696,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46091.38540509259</v>
+        <v>46091.46299768519</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11760,7 +11760,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46090.6577662037</v>
+        <v>46091.45403935185</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11888,7 +11888,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46091.36443287037</v>
+        <v>46091.44732638889</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11952,7 +11952,7 @@
         <v>1</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46091.36556712963</v>
+        <v>46091.44869212963</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12341,7 +12341,7 @@
         <v>1</v>
       </c>
       <c r="N183" s="3" t="n">
-        <v>46091.36527777778</v>
+        <v>46091.44810185185</v>
       </c>
       <c r="O183" t="inlineStr">
         <is>
@@ -12405,7 +12405,7 @@
         <v>1</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46091.36651620371</v>
+        <v>46091.45747685185</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12469,7 +12469,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46091.36959490741</v>
+        <v>46091.46010416667</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12533,7 +12533,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46091.38211805555</v>
+        <v>46091.46457175926</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12661,7 +12661,7 @@
         </is>
       </c>
       <c r="N188" s="3" t="n">
-        <v>46091.38475694445</v>
+        <v>46091.46087962963</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
@@ -12725,7 +12725,7 @@
         <v>1</v>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46091.39648148148</v>
+        <v>46091.47086805556</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12789,7 +12789,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46091.39354166666</v>
+        <v>46091.47138888889</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12914,7 +12914,7 @@
         <v>2</v>
       </c>
       <c r="N192" s="3" t="n">
-        <v>46091.37446759259</v>
+        <v>46091.4560300926</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
@@ -12978,7 +12978,7 @@
         <v>1</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46091.37728009259</v>
+        <v>46091.45171296296</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13042,7 +13042,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46091.40446759259</v>
+        <v>46091.45539351852</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13106,7 +13106,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46091.37707175926</v>
+        <v>46091.45471064815</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13170,7 +13170,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46091.36515046296</v>
+        <v>46091.44857638889</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13234,7 +13234,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46091.36805555555</v>
+        <v>46091.460625</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13423,7 +13423,7 @@
         <v>1</v>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46091.39719907408</v>
+        <v>46091.47673611111</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13487,7 +13487,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46091.38642361111</v>
+        <v>46091.46284722222</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13551,7 +13551,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46091.39642361111</v>
+        <v>46091.47273148148</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13615,7 +13615,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46091.37061342593</v>
+        <v>46091.48100694444</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13679,7 +13679,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46091.4021875</v>
+        <v>46091.47805555556</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13743,7 +13743,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46091.36467592593</v>
+        <v>46091.45534722223</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13807,7 +13807,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46091.37828703703</v>
+        <v>46091.45086805556</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13871,7 +13871,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46091.40078703704</v>
+        <v>46091.45556712963</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13935,7 +13935,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46091.38277777778</v>
+        <v>46091.4615162037</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -13999,7 +13999,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46091.3890625</v>
+        <v>46091.46630787037</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14063,7 +14063,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46091.38818287037</v>
+        <v>46091.46461805556</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14127,7 +14127,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46091.39105324074</v>
+        <v>46091.45097222222</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14191,7 +14191,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46091.39104166667</v>
+        <v>46091.46771990741</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14255,7 +14255,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46091.38839120371</v>
+        <v>46091.46575231481</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14319,7 +14319,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46091.39395833333</v>
+        <v>46091.46856481482</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14383,7 +14383,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46091.38870370371</v>
+        <v>46091.46479166667</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14447,7 +14447,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46091.40310185185</v>
+        <v>46091.48121527778</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14511,7 +14511,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46091.37175925926</v>
+        <v>46091.46619212963</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14580,7 +14580,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46091.38142361111</v>
+        <v>46091.46527777778</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14644,7 +14644,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46091.3821875</v>
+        <v>46091.46649305556</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14708,7 +14708,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46091.39038194445</v>
+        <v>46091.47305555556</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14772,7 +14772,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46091.37961805556</v>
+        <v>46091.45702546297</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14836,7 +14836,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46091.36796296296</v>
+        <v>46091.47576388889</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14964,7 +14964,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46091.36611111111</v>
+        <v>46091.45690972222</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15028,7 +15028,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46091.39908564815</v>
+        <v>46091.47892361111</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15092,7 +15092,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46091.36684027778</v>
+        <v>46091.44685185186</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15156,7 +15156,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46091.39215277778</v>
+        <v>46091.46943287037</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15220,7 +15220,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46091.39840277778</v>
+        <v>46091.47892361111</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15284,7 +15284,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46091.37600694445</v>
+        <v>46091.45321759259</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15348,7 +15348,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46091.36783564815</v>
+        <v>46091.45778935185</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15412,7 +15412,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46091.38172453704</v>
+        <v>46091.45900462963</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15476,7 +15476,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46091.39039351852</v>
+        <v>46091.46689814814</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15540,7 +15540,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46090.84180555555</v>
+        <v>46091.45604166666</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15604,7 +15604,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46091.38012731481</v>
+        <v>46091.46221064815</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15668,7 +15668,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46091.39243055556</v>
+        <v>46091.4647800926</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15796,7 +15796,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46091.39079861111</v>
+        <v>46091.46842592592</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15860,7 +15860,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46091.36538194444</v>
+        <v>46091.45655092593</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15924,7 +15924,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46088.50724537037</v>
+        <v>46091.46150462963</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -15988,7 +15988,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46091.37670138889</v>
+        <v>46091.45138888889</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16052,7 +16052,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46091.37489583333</v>
+        <v>46091.48605324074</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16175,7 +16175,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46091.40203703703</v>
+        <v>46091.45646990741</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16239,7 +16239,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46091.39828703704</v>
+        <v>46091.47644675926</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16303,7 +16303,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46091.38695601852</v>
+        <v>46091.46600694444</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16367,7 +16367,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46091.38436342592</v>
+        <v>46091.47222222222</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16431,7 +16431,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46091.40449074074</v>
+        <v>46091.45506944445</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16495,7 +16495,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46091.3877662037</v>
+        <v>46091.4659837963</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16623,7 +16623,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46091.39806712963</v>
+        <v>46091.47912037037</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16687,7 +16687,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46091.39613425926</v>
+        <v>46091.47740740741</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16745,7 +16745,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46091.37241898148</v>
+        <v>46091.46540509259</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16809,7 +16809,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46091.40368055556</v>
+        <v>46091.45568287037</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16873,7 +16873,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46091.40246527778</v>
+        <v>46091.47922453703</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16937,7 +16937,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46091.37336805555</v>
+        <v>46091.48657407407</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -17065,7 +17065,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46091.3768287037</v>
+        <v>46091.45326388889</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17129,7 +17129,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46091.37460648148</v>
+        <v>46091.45855324074</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17321,7 +17321,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46091.40023148148</v>
+        <v>46091.4731712963</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17385,7 +17385,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46091.36902777778</v>
+        <v>46091.4572337963</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17449,7 +17449,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46091.40206018519</v>
+        <v>46091.48074074074</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17513,7 +17513,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46091.37924768519</v>
+        <v>46091.45484953704</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17577,7 +17577,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46091.37487268518</v>
+        <v>46091.45431712963</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17641,7 +17641,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46090.82424768519</v>
+        <v>46091.47135416666</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17705,7 +17705,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46090.80217592593</v>
+        <v>46091.45452546296</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17766,7 +17766,7 @@
         </is>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46091.40123842593</v>
+        <v>46091.47659722222</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17894,7 +17894,7 @@
         <v>1</v>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46091.38575231482</v>
+        <v>46091.4591087963</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -18267,7 +18267,7 @@
         <v>1</v>
       </c>
       <c r="N276" s="3" t="n">
-        <v>46091.36653935185</v>
+        <v>46091.47740740741</v>
       </c>
       <c r="O276" t="inlineStr">
         <is>
@@ -18331,7 +18331,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46091.38353009259</v>
+        <v>46091.46513888889</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18454,7 +18454,7 @@
         <v>1</v>
       </c>
       <c r="N279" s="3" t="n">
-        <v>46091.38575231482</v>
+        <v>46091.46032407408</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -18513,7 +18513,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46091.38179398148</v>
+        <v>46091.45958333334</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18577,7 +18577,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46091.39811342592</v>
+        <v>46091.47244212963</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18641,7 +18641,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46091.4027662037</v>
+        <v>46091.47693287037</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18705,7 +18705,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46091.37783564815</v>
+        <v>46091.46091435185</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18769,7 +18769,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46091.36609953704</v>
+        <v>46091.48783564815</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18897,7 +18897,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46091.36555555555</v>
+        <v>46091.47523148148</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18961,7 +18961,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46090.84643518519</v>
+        <v>46091.45693287037</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19139,7 +19139,7 @@
         </is>
       </c>
       <c r="N290" s="3" t="n">
-        <v>46091.37430555555</v>
+        <v>46091.48706018519</v>
       </c>
       <c r="O290" t="inlineStr">
         <is>
@@ -19569,7 +19569,7 @@
         <v>1</v>
       </c>
       <c r="N297" s="3" t="n">
-        <v>46091.40252314815</v>
+        <v>46091.48170138889</v>
       </c>
       <c r="O297" t="inlineStr">
         <is>
@@ -19694,7 +19694,7 @@
         <v>1</v>
       </c>
       <c r="N299" s="3" t="n">
-        <v>46091.37688657407</v>
+        <v>46091.45600694444</v>
       </c>
       <c r="O299" t="inlineStr">
         <is>
@@ -21535,7 +21535,7 @@
         <v>1</v>
       </c>
       <c r="N329" s="3" t="n">
-        <v>46091.40266203704</v>
+        <v>46091.48137731481</v>
       </c>
       <c r="O329" t="inlineStr">
         <is>
@@ -21599,7 +21599,7 @@
         <v>2</v>
       </c>
       <c r="N330" s="3" t="n">
-        <v>46091.40290509259</v>
+        <v>46091.48600694445</v>
       </c>
       <c r="O330" t="inlineStr">
         <is>
@@ -21663,7 +21663,7 @@
         <v>2</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46091.36884259259</v>
+        <v>46091.48033564815</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21727,7 +21727,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46091.40347222222</v>
+        <v>46091.48268518518</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21791,7 +21791,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46091.39510416667</v>
+        <v>46091.47528935185</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21855,7 +21855,7 @@
         <v>1</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46091.37240740741</v>
+        <v>46091.45902777778</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21919,7 +21919,7 @@
         <v>2</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46091.37530092592</v>
+        <v>46091.4584375</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21983,7 +21983,7 @@
         <v>2</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46091.37076388889</v>
+        <v>46091.44924768519</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22111,7 +22111,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46091.37349537037</v>
+        <v>46091.45185185185</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22175,7 +22175,7 @@
         <v>2</v>
       </c>
       <c r="N339" s="3" t="n">
-        <v>46090.57268518519</v>
+        <v>46091.46513888889</v>
       </c>
       <c r="O339" t="inlineStr">
         <is>
@@ -22236,7 +22236,7 @@
         </is>
       </c>
       <c r="N340" s="3" t="n">
-        <v>46091.38570601852</v>
+        <v>46091.46496527778</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -22867,7 +22867,7 @@
         </is>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46091.38141203704</v>
+        <v>46091.45572916666</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -23462,7 +23462,7 @@
         <v>1</v>
       </c>
       <c r="N361" s="3" t="n">
-        <v>46091.36630787037</v>
+        <v>46091.47975694444</v>
       </c>
       <c r="O361" t="inlineStr">
         <is>
@@ -23528,7 +23528,7 @@
         </is>
       </c>
       <c r="N362" s="3" t="n">
-        <v>46091.38306712963</v>
+        <v>46091.45553240741</v>
       </c>
       <c r="O362" t="inlineStr">
         <is>
@@ -23654,7 +23654,7 @@
         </is>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46091.36879629629</v>
+        <v>46091.48111111111</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23784,7 +23784,7 @@
         <v>1</v>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46091.3700925926</v>
+        <v>46091.48554398148</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
@@ -23812,7 +23812,7 @@
         <v>2</v>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46091.37094907407</v>
+        <v>46091.45859953704</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -23881,7 +23881,7 @@
         <v>1</v>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46091.37864583333</v>
+        <v>46091.45293981482</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24085,7 +24085,7 @@
         </is>
       </c>
       <c r="N371" s="3" t="n">
-        <v>46091.3749537037</v>
+        <v>46091.45234953704</v>
       </c>
       <c r="O371" t="inlineStr">
         <is>
@@ -24149,7 +24149,7 @@
         <v>1</v>
       </c>
       <c r="N372" s="3" t="n">
-        <v>46090.80238425926</v>
+        <v>46091.45506944445</v>
       </c>
       <c r="O372" t="inlineStr">
         <is>
@@ -24218,7 +24218,7 @@
         <v>2</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46091.39199074074</v>
+        <v>46091.47167824074</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24287,7 +24287,7 @@
         <v>2</v>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46091.37211805556</v>
+        <v>46091.45349537037</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-10 13:52:05.644442
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -434,7 +434,7 @@
   <cols>
     <col width="25.2" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="15.6" customWidth="1" min="3" max="3"/>
+    <col width="32.4" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="10.8" customWidth="1" min="5" max="5"/>
     <col width="50.4" customWidth="1" min="6" max="6"/>
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46091.46369212963</v>
+        <v>46091.5453125</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46091.46114583333</v>
+        <v>46091.53520833333</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46091.47986111111</v>
+        <v>46091.56841435185</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46091.46797453704</v>
+        <v>46091.54094907407</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
         <v>1</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>46091.47511574074</v>
+        <v>46091.54641203704</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1943,7 +1943,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46091.18637731481</v>
+        <v>46091.50116898148</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2178,7 +2178,7 @@
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46091.47332175926</v>
+        <v>46091.54615740741</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6504,7 +6504,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46091.44981481481</v>
+        <v>46091.56734953704</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6573,7 +6573,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46091.45435185185</v>
+        <v>46091.5346412037</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6637,7 +6637,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46091.48322916667</v>
+        <v>46091.5588425926</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6656,6 +6656,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>10.69.3.94</t>
+        </is>
+      </c>
       <c r="D97" t="n">
         <v>2025</v>
       </c>
@@ -6701,7 +6706,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46091.44771990741</v>
+        <v>46091.57077546296</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6770,7 +6775,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46091.45234953704</v>
+        <v>46091.53412037037</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6839,7 +6844,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46091.45945601852</v>
+        <v>46091.54143518519</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6908,7 +6913,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46091.4871412037</v>
+        <v>46091.56530092593</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -7046,7 +7051,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46091.46678240741</v>
+        <v>46091.54201388889</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7441,7 +7446,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46091.45722222222</v>
+        <v>46091.53649305556</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7510,7 +7515,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46091.47098379629</v>
+        <v>46091.54628472222</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7579,7 +7584,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46091.44646990741</v>
+        <v>46091.56907407408</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7648,7 +7653,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46091.46883101852</v>
+        <v>46091.54547453704</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7717,7 +7722,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46091.45407407408</v>
+        <v>46091.53613425926</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7786,7 +7791,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46091.48274305555</v>
+        <v>46091.56296296296</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7852,7 +7857,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46091.46746527778</v>
+        <v>46091.54583333333</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7921,7 +7926,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46091.46118055555</v>
+        <v>46091.54019675926</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7990,7 +7995,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46091.46903935185</v>
+        <v>46091.54586805555</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8056,7 +8061,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46091.47358796297</v>
+        <v>46091.54856481482</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8194,7 +8199,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46091.46296296296</v>
+        <v>46091.54413194444</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8263,7 +8268,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46091.48207175926</v>
+        <v>46091.56232638889</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8284,7 +8289,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>10.69.3.81</t>
+          <t>fe80::c253:614c:cc25:dbac</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -8329,7 +8334,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46091.47635416667</v>
+        <v>46091.55653935186</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8398,7 +8403,7 @@
         <v>2</v>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46091.48401620371</v>
+        <v>46091.56732638889</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8467,7 +8472,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46091.46603009259</v>
+        <v>46091.54270833333</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8536,7 +8541,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46091.47802083333</v>
+        <v>46091.55431712963</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8605,7 +8610,7 @@
         <v>2</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46091.45321759259</v>
+        <v>46091.56628472222</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8674,7 +8679,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46091.46395833333</v>
+        <v>46091.54086805556</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8743,7 +8748,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46091.48739583333</v>
+        <v>46091.56482638889</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8812,7 +8817,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46091.47376157407</v>
+        <v>46091.55278935185</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8881,7 +8886,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46091.48302083334</v>
+        <v>46091.56363425926</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -8900,11 +8905,6 @@
           <t>ADM/FIN</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>10.69.3.6</t>
-        </is>
-      </c>
       <c r="D130" t="n">
         <v>2025</v>
       </c>
@@ -8950,7 +8950,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46091.48386574074</v>
+        <v>46091.56010416667</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9014,7 +9014,7 @@
         <v>1</v>
       </c>
       <c r="N131" s="3" t="n">
-        <v>46091.48234953704</v>
+        <v>46091.55965277777</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -9333,7 +9333,7 @@
         <v>1</v>
       </c>
       <c r="N136" s="3" t="n">
-        <v>46091.46390046296</v>
+        <v>46091.53924768518</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -9525,7 +9525,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46091.44984953704</v>
+        <v>46091.54651620371</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9589,7 +9589,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46091.46534722222</v>
+        <v>46091.54460648148</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9653,7 +9653,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46091.45607638889</v>
+        <v>46091.53961805555</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9717,7 +9717,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46091.46028935185</v>
+        <v>46091.53640046297</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9781,7 +9781,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46091.46546296297</v>
+        <v>46091.54100694445</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9845,7 +9845,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46091.45329861111</v>
+        <v>46091.56953703704</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9909,7 +9909,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46091.4727199074</v>
+        <v>46091.54607638889</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -10037,7 +10037,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46091.46130787037</v>
+        <v>46091.54131944444</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10229,7 +10229,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46091.45222222222</v>
+        <v>46091.56831018518</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10352,7 +10352,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46091.48655092593</v>
+        <v>46091.55894675926</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10480,7 +10480,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46091.48503472222</v>
+        <v>46091.56207175926</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10544,7 +10544,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46091.45207175926</v>
+        <v>46091.52915509259</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10608,7 +10608,7 @@
         <v>1</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>46091.46974537037</v>
+        <v>46091.54935185185</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -10672,7 +10672,7 @@
         <v>1</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>46091.46071759259</v>
+        <v>46091.54155092593</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -10736,7 +10736,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46091.48232638889</v>
+        <v>46091.56166666667</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10800,7 +10800,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46091.46599537037</v>
+        <v>46091.54168981482</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10864,7 +10864,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46091.45408564815</v>
+        <v>46091.56677083333</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10928,7 +10928,7 @@
         <v>1</v>
       </c>
       <c r="N161" s="3" t="n">
-        <v>46091.35789351852</v>
+        <v>46091.56011574074</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -10992,7 +10992,7 @@
         <v>2</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46091.48663194444</v>
+        <v>46091.56376157407</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11053,10 +11053,10 @@
         </is>
       </c>
       <c r="M163" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46090.75048611111</v>
+        <v>46091.54478009259</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11120,7 +11120,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46091.4855787037</v>
+        <v>46091.55704861111</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11184,7 +11184,7 @@
         <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46091.45199074074</v>
+        <v>46091.56965277778</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11248,7 +11248,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="3" t="n">
-        <v>46091.4766087963</v>
+        <v>46091.55024305556</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -11312,7 +11312,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46091.47267361111</v>
+        <v>46091.54685185185</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11376,7 +11376,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46091.45429398148</v>
+        <v>46091.53189814815</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11504,7 +11504,7 @@
         <v>2</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46090.71854166667</v>
+        <v>46091.54347222222</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11565,10 +11565,10 @@
         </is>
       </c>
       <c r="M171" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46091.46534722222</v>
+        <v>46091.54309027778</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11632,7 +11632,7 @@
         <v>2</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>46091.46649305556</v>
+        <v>46091.54247685185</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -11696,7 +11696,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46091.46299768519</v>
+        <v>46091.53524305556</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11760,7 +11760,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46091.45403935185</v>
+        <v>46091.56842592593</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11824,7 +11824,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46090.654375</v>
+        <v>46091.54422453704</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11888,7 +11888,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46091.44732638889</v>
+        <v>46091.563125</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11952,7 +11952,7 @@
         <v>1</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46091.44869212963</v>
+        <v>46091.56737268518</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12341,7 +12341,7 @@
         <v>1</v>
       </c>
       <c r="N183" s="3" t="n">
-        <v>46091.44810185185</v>
+        <v>46091.56393518519</v>
       </c>
       <c r="O183" t="inlineStr">
         <is>
@@ -12405,7 +12405,7 @@
         <v>1</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46091.45747685185</v>
+        <v>46091.53273148148</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12469,7 +12469,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46091.46010416667</v>
+        <v>46091.54043981482</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12533,7 +12533,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46091.46457175926</v>
+        <v>46091.54134259259</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12661,7 +12661,7 @@
         </is>
       </c>
       <c r="N188" s="3" t="n">
-        <v>46091.46087962963</v>
+        <v>46091.53605324074</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
@@ -12725,7 +12725,7 @@
         <v>1</v>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46091.47086805556</v>
+        <v>46091.5440162037</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12789,7 +12789,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46091.47138888889</v>
+        <v>46091.55329861111</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12914,7 +12914,7 @@
         <v>2</v>
       </c>
       <c r="N192" s="3" t="n">
-        <v>46091.4560300926</v>
+        <v>46091.53763888889</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
@@ -12978,7 +12978,7 @@
         <v>1</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46091.45171296296</v>
+        <v>46091.56285879629</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13042,7 +13042,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46091.45539351852</v>
+        <v>46091.53510416667</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13106,7 +13106,7 @@
         <v>1</v>
       </c>
       <c r="N195" s="3" t="n">
-        <v>46091.45471064815</v>
+        <v>46091.56694444444</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -13170,7 +13170,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46091.44857638889</v>
+        <v>46091.53180555555</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13234,7 +13234,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46091.460625</v>
+        <v>46091.54027777778</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13423,7 +13423,7 @@
         <v>1</v>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46091.47673611111</v>
+        <v>46091.55502314815</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13487,7 +13487,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46091.46284722222</v>
+        <v>46091.53732638889</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13551,7 +13551,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46091.47273148148</v>
+        <v>46091.55346064815</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13615,7 +13615,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46091.48100694444</v>
+        <v>46091.55775462963</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13679,7 +13679,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46091.47805555556</v>
+        <v>46091.55238425926</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13743,7 +13743,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46091.45534722223</v>
+        <v>46091.53670138889</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13807,7 +13807,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="3" t="n">
-        <v>46091.45086805556</v>
+        <v>46091.49</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -13871,7 +13871,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46091.45556712963</v>
+        <v>46091.56356481482</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13935,7 +13935,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46091.4615162037</v>
+        <v>46091.53824074074</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -13999,7 +13999,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46091.46630787037</v>
+        <v>46091.54766203704</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14063,7 +14063,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46091.46461805556</v>
+        <v>46091.53956018519</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14127,7 +14127,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46091.45097222222</v>
+        <v>46091.56994212963</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14191,7 +14191,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46091.46771990741</v>
+        <v>46091.54569444444</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14255,7 +14255,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46091.46575231481</v>
+        <v>46091.54146990741</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14319,7 +14319,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46091.46856481482</v>
+        <v>46091.54289351852</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14383,7 +14383,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46091.46479166667</v>
+        <v>46091.50074074074</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14447,7 +14447,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46091.48121527778</v>
+        <v>46091.55721064815</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14511,7 +14511,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46091.46619212963</v>
+        <v>46091.545625</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14580,7 +14580,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46091.46527777778</v>
+        <v>46091.54611111111</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14644,7 +14644,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46091.46649305556</v>
+        <v>46091.54239583333</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14708,7 +14708,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46091.47305555556</v>
+        <v>46091.55482638889</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14772,7 +14772,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46091.45702546297</v>
+        <v>46091.53320601852</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14836,7 +14836,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="3" t="n">
-        <v>46091.47576388889</v>
+        <v>46091.5503587963</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -14964,7 +14964,7 @@
         <v>1</v>
       </c>
       <c r="N224" s="3" t="n">
-        <v>46091.45690972222</v>
+        <v>46091.56853009259</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -15028,7 +15028,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46091.47892361111</v>
+        <v>46091.55293981481</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15092,7 +15092,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46091.44685185186</v>
+        <v>46091.56800925926</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15156,7 +15156,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46091.46943287037</v>
+        <v>46091.54487268518</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15220,7 +15220,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46091.47892361111</v>
+        <v>46091.56018518518</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15284,7 +15284,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46091.45321759259</v>
+        <v>46091.56861111111</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15348,7 +15348,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46091.45778935185</v>
+        <v>46091.5375462963</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15412,7 +15412,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46091.45900462963</v>
+        <v>46091.53416666666</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15476,7 +15476,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46091.46689814814</v>
+        <v>46091.5478125</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15540,7 +15540,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46091.45604166666</v>
+        <v>46091.56866898148</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15604,7 +15604,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46091.46221064815</v>
+        <v>46091.53834490741</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15668,7 +15668,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46091.4647800926</v>
+        <v>46091.54068287037</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15796,7 +15796,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46091.46842592592</v>
+        <v>46091.55137731481</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15860,7 +15860,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46091.45655092593</v>
+        <v>46091.53394675926</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15924,7 +15924,7 @@
         <v>1</v>
       </c>
       <c r="N239" s="3" t="n">
-        <v>46091.46150462963</v>
+        <v>46091.50197916666</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -15988,7 +15988,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46091.45138888889</v>
+        <v>46091.56424768519</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16052,7 +16052,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46091.48605324074</v>
+        <v>46091.56197916667</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16175,7 +16175,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46091.45646990741</v>
+        <v>46091.53472222222</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16239,7 +16239,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46091.47644675926</v>
+        <v>46091.55206018518</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16303,7 +16303,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46091.46600694444</v>
+        <v>46091.54486111111</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16367,7 +16367,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46091.47222222222</v>
+        <v>46091.54572916667</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16431,7 +16431,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46091.45506944445</v>
+        <v>46091.53516203703</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16495,7 +16495,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46091.4659837963</v>
+        <v>46091.5421412037</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16623,7 +16623,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46091.47912037037</v>
+        <v>46091.55392361111</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16687,7 +16687,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46091.47740740741</v>
+        <v>46091.5516087963</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16745,7 +16745,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46091.46540509259</v>
+        <v>46091.54010416667</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16809,7 +16809,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46091.45568287037</v>
+        <v>46091.5344212963</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16873,7 +16873,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46091.47922453703</v>
+        <v>46091.56034722222</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16937,7 +16937,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46091.48657407407</v>
+        <v>46091.56133101852</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -17065,7 +17065,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46091.45326388889</v>
+        <v>46091.57018518518</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17129,7 +17129,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46091.45855324074</v>
+        <v>46091.54193287037</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17321,7 +17321,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46091.4731712963</v>
+        <v>46091.55471064815</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17385,7 +17385,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46091.4572337963</v>
+        <v>46091.53056712963</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17449,7 +17449,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46091.48074074074</v>
+        <v>46091.55908564815</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17513,7 +17513,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46091.45484953704</v>
+        <v>46091.5303587963</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17577,7 +17577,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46091.45431712963</v>
+        <v>46091.53197916667</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17641,7 +17641,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46091.47135416666</v>
+        <v>46091.55015046296</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17705,7 +17705,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46091.45452546296</v>
+        <v>46091.56655092593</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17766,7 +17766,7 @@
         </is>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46091.47659722222</v>
+        <v>46091.55370370371</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17894,7 +17894,7 @@
         <v>1</v>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46091.4591087963</v>
+        <v>46091.53880787037</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -18267,7 +18267,7 @@
         <v>1</v>
       </c>
       <c r="N276" s="3" t="n">
-        <v>46091.47740740741</v>
+        <v>46091.55188657407</v>
       </c>
       <c r="O276" t="inlineStr">
         <is>
@@ -18331,7 +18331,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46091.46513888889</v>
+        <v>46091.54219907407</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18454,7 +18454,7 @@
         <v>1</v>
       </c>
       <c r="N279" s="3" t="n">
-        <v>46091.46032407408</v>
+        <v>46091.53612268518</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -18513,7 +18513,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46091.45958333334</v>
+        <v>46091.53915509259</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18577,7 +18577,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46091.47244212963</v>
+        <v>46091.54835648148</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18641,7 +18641,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46091.47693287037</v>
+        <v>46091.55344907408</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18705,7 +18705,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46091.46091435185</v>
+        <v>46091.53841435185</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18769,7 +18769,7 @@
         <v>1</v>
       </c>
       <c r="N284" s="3" t="n">
-        <v>46091.48783564815</v>
+        <v>46091.56341435185</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18897,7 +18897,7 @@
         <v>1</v>
       </c>
       <c r="N286" s="3" t="n">
-        <v>46091.47523148148</v>
+        <v>46091.55574074074</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -18961,7 +18961,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46091.45693287037</v>
+        <v>46091.53480324074</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19139,7 +19139,7 @@
         </is>
       </c>
       <c r="N290" s="3" t="n">
-        <v>46091.48706018519</v>
+        <v>46091.56613425926</v>
       </c>
       <c r="O290" t="inlineStr">
         <is>
@@ -19569,7 +19569,7 @@
         <v>1</v>
       </c>
       <c r="N297" s="3" t="n">
-        <v>46091.48170138889</v>
+        <v>46091.55402777778</v>
       </c>
       <c r="O297" t="inlineStr">
         <is>
@@ -19694,7 +19694,7 @@
         <v>1</v>
       </c>
       <c r="N299" s="3" t="n">
-        <v>46091.45600694444</v>
+        <v>46091.56699074074</v>
       </c>
       <c r="O299" t="inlineStr">
         <is>
@@ -21535,7 +21535,7 @@
         <v>1</v>
       </c>
       <c r="N329" s="3" t="n">
-        <v>46091.48137731481</v>
+        <v>46091.56415509259</v>
       </c>
       <c r="O329" t="inlineStr">
         <is>
@@ -21599,7 +21599,7 @@
         <v>2</v>
       </c>
       <c r="N330" s="3" t="n">
-        <v>46091.48600694445</v>
+        <v>46091.56412037037</v>
       </c>
       <c r="O330" t="inlineStr">
         <is>
@@ -21663,7 +21663,7 @@
         <v>2</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46091.48033564815</v>
+        <v>46091.55696759259</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21727,7 +21727,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46091.48268518518</v>
+        <v>46091.56087962963</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21791,7 +21791,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46091.47528935185</v>
+        <v>46091.54637731481</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21855,7 +21855,7 @@
         <v>1</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46091.45902777778</v>
+        <v>46091.54484953704</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21919,7 +21919,7 @@
         <v>2</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46091.4584375</v>
+        <v>46091.53988425926</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21983,7 +21983,7 @@
         <v>2</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46091.44924768519</v>
+        <v>46091.56626157407</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22044,10 +22044,10 @@
         </is>
       </c>
       <c r="M337" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46090.55195601852</v>
+        <v>46091.56130787037</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22111,7 +22111,7 @@
         <v>2</v>
       </c>
       <c r="N338" s="3" t="n">
-        <v>46091.45185185185</v>
+        <v>46091.56998842592</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -22175,7 +22175,7 @@
         <v>2</v>
       </c>
       <c r="N339" s="3" t="n">
-        <v>46091.46513888889</v>
+        <v>46091.5361574074</v>
       </c>
       <c r="O339" t="inlineStr">
         <is>
@@ -22236,7 +22236,7 @@
         </is>
       </c>
       <c r="N340" s="3" t="n">
-        <v>46091.46496527778</v>
+        <v>46091.54226851852</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -22867,7 +22867,7 @@
         </is>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46091.45572916666</v>
+        <v>46091.56989583333</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -23462,7 +23462,7 @@
         <v>1</v>
       </c>
       <c r="N361" s="3" t="n">
-        <v>46091.47975694444</v>
+        <v>46091.55685185185</v>
       </c>
       <c r="O361" t="inlineStr">
         <is>
@@ -23528,7 +23528,7 @@
         </is>
       </c>
       <c r="N362" s="3" t="n">
-        <v>46091.45553240741</v>
+        <v>46091.53650462963</v>
       </c>
       <c r="O362" t="inlineStr">
         <is>
@@ -23654,7 +23654,7 @@
         </is>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46091.48111111111</v>
+        <v>46091.55773148148</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23784,7 +23784,7 @@
         <v>1</v>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46091.48554398148</v>
+        <v>46091.56077546296</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
@@ -23812,7 +23812,7 @@
         <v>2</v>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46091.45859953704</v>
+        <v>46091.53305555556</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -23881,7 +23881,7 @@
         <v>1</v>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46091.45293981482</v>
+        <v>46091.57097222222</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24085,7 +24085,7 @@
         </is>
       </c>
       <c r="N371" s="3" t="n">
-        <v>46091.45234953704</v>
+        <v>46091.53103009259</v>
       </c>
       <c r="O371" t="inlineStr">
         <is>
@@ -24149,7 +24149,7 @@
         <v>1</v>
       </c>
       <c r="N372" s="3" t="n">
-        <v>46091.45506944445</v>
+        <v>46091.53457175926</v>
       </c>
       <c r="O372" t="inlineStr">
         <is>
@@ -24218,7 +24218,7 @@
         <v>2</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46091.47167824074</v>
+        <v>46091.55059027778</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24287,7 +24287,7 @@
         <v>2</v>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46091.45349537037</v>
+        <v>46091.56847222222</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-10 15:52:10.920986
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -434,7 +434,7 @@
   <cols>
     <col width="25.2" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="32.4" customWidth="1" min="3" max="3"/>
+    <col width="15.6" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="10.8" customWidth="1" min="5" max="5"/>
     <col width="50.4" customWidth="1" min="6" max="6"/>
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46091.5453125</v>
+        <v>46091.6253125</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46091.53520833333</v>
+        <v>46091.65208333333</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46091.56841435185</v>
+        <v>46091.64045138889</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46091.54094907407</v>
+        <v>46091.61862268519</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
         <v>1</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>46091.54641203704</v>
+        <v>46091.62174768518</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Microsoft Windows 7 Professional</t>
+          <t>Windows</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1190,7 +1190,7 @@
         <v>1</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>46091.48385416667</v>
+        <v>46091.5753125</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1962,6 +1962,11 @@
           <t>AUDITORIO</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>10.69.3.153</t>
+        </is>
+      </c>
       <c r="D24" t="n">
         <v>2019</v>
       </c>
@@ -1999,7 +2004,7 @@
         </is>
       </c>
       <c r="N24" s="3" t="n">
-        <v>46090.50244212963</v>
+        <v>46091.60961805555</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2178,7 +2183,7 @@
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46091.54615740741</v>
+        <v>46091.62216435185</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6504,7 +6509,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46091.56734953704</v>
+        <v>46091.64637731481</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6573,7 +6578,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46091.5346412037</v>
+        <v>46091.6180787037</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6637,7 +6642,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46091.5588425926</v>
+        <v>46091.6377199074</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6706,7 +6711,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46091.57077546296</v>
+        <v>46091.64969907407</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6775,7 +6780,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46091.53412037037</v>
+        <v>46091.64759259259</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6844,7 +6849,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46091.54143518519</v>
+        <v>46091.61957175926</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6913,7 +6918,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46091.56530092593</v>
+        <v>46091.64761574074</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6982,7 +6987,7 @@
         <v>1</v>
       </c>
       <c r="N101" s="3" t="n">
-        <v>46090.72416666667</v>
+        <v>46091.61975694444</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -7051,7 +7056,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46091.54201388889</v>
+        <v>46091.62238425926</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7446,7 +7451,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46091.53649305556</v>
+        <v>46091.6159375</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7515,7 +7520,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46091.54628472222</v>
+        <v>46091.62356481481</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7584,7 +7589,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46091.56907407408</v>
+        <v>46091.64443287037</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7653,7 +7658,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46091.54547453704</v>
+        <v>46091.65414351852</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7722,7 +7727,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46091.53613425926</v>
+        <v>46091.64981481482</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7791,7 +7796,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46091.56296296296</v>
+        <v>46091.64181712963</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7857,7 +7862,7 @@
         </is>
       </c>
       <c r="N114" s="3" t="n">
-        <v>46091.54583333333</v>
+        <v>46091.62126157407</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7926,7 +7931,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46091.54019675926</v>
+        <v>46091.61944444444</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7995,7 +8000,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46091.54586805555</v>
+        <v>46091.62253472222</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8061,7 +8066,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46091.54856481482</v>
+        <v>46091.62274305556</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8199,7 +8204,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46091.54413194444</v>
+        <v>46091.62111111111</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8268,7 +8273,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46091.56232638889</v>
+        <v>46091.6366087963</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8289,7 +8294,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>fe80::c253:614c:cc25:dbac</t>
+          <t>10.69.3.81</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -8334,7 +8339,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46091.55653935186</v>
+        <v>46091.6285300926</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8403,7 +8408,7 @@
         <v>2</v>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46091.56732638889</v>
+        <v>46091.63989583333</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8472,7 +8477,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46091.54270833333</v>
+        <v>46091.65429398148</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8541,7 +8546,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46091.55431712963</v>
+        <v>46091.63167824074</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8610,7 +8615,7 @@
         <v>2</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46091.56628472222</v>
+        <v>46091.64142361111</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8679,7 +8684,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46091.54086805556</v>
+        <v>46091.61427083334</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8748,7 +8753,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46091.56482638889</v>
+        <v>46091.64509259259</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8817,7 +8822,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46091.55278935185</v>
+        <v>46091.62784722223</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8886,7 +8891,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46091.56363425926</v>
+        <v>46091.64157407408</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -8950,7 +8955,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46091.56010416667</v>
+        <v>46091.64303240741</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9014,7 +9019,7 @@
         <v>1</v>
       </c>
       <c r="N131" s="3" t="n">
-        <v>46091.55965277777</v>
+        <v>46091.62206018518</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -9078,7 +9083,7 @@
         <v>1</v>
       </c>
       <c r="N132" s="3" t="n">
-        <v>46090.81717592593</v>
+        <v>46091.58313657407</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -9142,7 +9147,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46090.79936342593</v>
+        <v>46091.61983796296</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9333,7 +9338,7 @@
         <v>1</v>
       </c>
       <c r="N136" s="3" t="n">
-        <v>46091.53924768518</v>
+        <v>46091.65243055556</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -9397,7 +9402,7 @@
         <v>1</v>
       </c>
       <c r="N137" s="3" t="n">
-        <v>46090.81349537037</v>
+        <v>46091.6225</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -9461,7 +9466,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46090.79704861111</v>
+        <v>46091.65137731482</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9525,7 +9530,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46091.54651620371</v>
+        <v>46091.62240740741</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9589,7 +9594,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46091.54460648148</v>
+        <v>46091.62449074074</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9653,7 +9658,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46091.53961805555</v>
+        <v>46091.62274305556</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9717,7 +9722,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46091.53640046297</v>
+        <v>46091.64649305555</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9781,7 +9786,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46091.54100694445</v>
+        <v>46091.62086805556</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9845,7 +9850,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46091.56953703704</v>
+        <v>46091.62370370371</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9909,7 +9914,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46091.54607638889</v>
+        <v>46091.64804398148</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9973,7 +9978,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46091.42211805555</v>
+        <v>46091.6209837963</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10037,7 +10042,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46091.54131944444</v>
+        <v>46091.6528125</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10101,7 +10106,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46090.82105324074</v>
+        <v>46091.62368055555</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10165,7 +10170,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46090.64149305555</v>
+        <v>46091.62300925926</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10229,7 +10234,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46091.56831018518</v>
+        <v>46091.64751157408</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10352,7 +10357,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46091.55894675926</v>
+        <v>46091.63981481481</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10416,7 +10421,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46090.82085648148</v>
+        <v>46091.62424768518</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10480,7 +10485,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46091.56207175926</v>
+        <v>46091.63731481481</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10544,7 +10549,7 @@
         <v>1</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>46091.52915509259</v>
+        <v>46091.57142361111</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -10672,7 +10677,7 @@
         <v>1</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>46091.54155092593</v>
+        <v>46091.61717592592</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -10736,7 +10741,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46091.56166666667</v>
+        <v>46091.63915509259</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10800,7 +10805,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46091.54168981482</v>
+        <v>46091.62271990741</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10864,7 +10869,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46091.56677083333</v>
+        <v>46091.62431712963</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10992,7 +10997,7 @@
         <v>2</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46091.56376157407</v>
+        <v>46091.63837962963</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11053,10 +11058,10 @@
         </is>
       </c>
       <c r="M163" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46091.54478009259</v>
+        <v>46091.62303240741</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11120,7 +11125,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="3" t="n">
-        <v>46091.55704861111</v>
+        <v>46091.59893518518</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -11184,7 +11189,7 @@
         <v>2</v>
       </c>
       <c r="N165" s="3" t="n">
-        <v>46091.56965277778</v>
+        <v>46091.605</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -11312,7 +11317,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46091.54685185185</v>
+        <v>46091.62391203704</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11376,7 +11381,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46091.53189814815</v>
+        <v>46091.65043981482</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11504,7 +11509,7 @@
         <v>2</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46091.54347222222</v>
+        <v>46091.62005787037</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11565,10 +11570,10 @@
         </is>
       </c>
       <c r="M171" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46091.54309027778</v>
+        <v>46091.62076388889</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11696,7 +11701,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46091.53524305556</v>
+        <v>46091.61824074074</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11760,7 +11765,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="3" t="n">
-        <v>46091.56842592593</v>
+        <v>46091.6444212963</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -11824,7 +11829,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46091.54422453704</v>
+        <v>46091.62333333334</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11888,7 +11893,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46091.563125</v>
+        <v>46091.63947916667</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11952,7 +11957,7 @@
         <v>1</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46091.56737268518</v>
+        <v>46091.6291087963</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12016,7 +12021,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46090.80800925926</v>
+        <v>46091.62238425926</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12080,7 +12085,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46090.80582175926</v>
+        <v>46091.62402777778</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12341,7 +12346,7 @@
         <v>1</v>
       </c>
       <c r="N183" s="3" t="n">
-        <v>46091.56393518519</v>
+        <v>46091.63849537037</v>
       </c>
       <c r="O183" t="inlineStr">
         <is>
@@ -12405,7 +12410,7 @@
         <v>1</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46091.53273148148</v>
+        <v>46091.65115740741</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12469,7 +12474,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46091.54043981482</v>
+        <v>46091.62380787037</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12533,7 +12538,7 @@
         <v>1</v>
       </c>
       <c r="N186" s="3" t="n">
-        <v>46091.54134259259</v>
+        <v>46091.58236111111</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -12661,7 +12666,7 @@
         </is>
       </c>
       <c r="N188" s="3" t="n">
-        <v>46091.53605324074</v>
+        <v>46091.62310185185</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
@@ -12725,7 +12730,7 @@
         <v>1</v>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46091.5440162037</v>
+        <v>46091.62336805555</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12789,7 +12794,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46091.55329861111</v>
+        <v>46091.62241898148</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12914,7 +12919,7 @@
         <v>2</v>
       </c>
       <c r="N192" s="3" t="n">
-        <v>46091.53763888889</v>
+        <v>46091.58023148148</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
@@ -12978,7 +12983,7 @@
         <v>1</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46091.56285879629</v>
+        <v>46091.64248842592</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13042,7 +13047,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46091.53510416667</v>
+        <v>46091.61616898148</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13170,7 +13175,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46091.53180555555</v>
+        <v>46091.6234837963</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13234,7 +13239,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="3" t="n">
-        <v>46091.54027777778</v>
+        <v>46091.57859953704</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -13298,7 +13303,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46090.80855324074</v>
+        <v>46091.62597222222</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13359,7 +13364,7 @@
         </is>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46090.82388888889</v>
+        <v>46091.6374074074</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13423,7 +13428,7 @@
         <v>1</v>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46091.55502314815</v>
+        <v>46091.64223379629</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13487,7 +13492,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46091.53732638889</v>
+        <v>46091.64954861111</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13551,7 +13556,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46091.55346064815</v>
+        <v>46091.62140046297</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13615,7 +13620,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46091.55775462963</v>
+        <v>46091.63511574074</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13679,7 +13684,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46091.55238425926</v>
+        <v>46091.63061342593</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13743,7 +13748,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46091.53670138889</v>
+        <v>46091.6207175926</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13871,7 +13876,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46091.56356481482</v>
+        <v>46091.62244212963</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13935,7 +13940,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46091.53824074074</v>
+        <v>46091.61525462963</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -13999,7 +14004,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46091.54766203704</v>
+        <v>46091.61863425926</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14063,7 +14068,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46091.53956018519</v>
+        <v>46091.61972222223</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14127,7 +14132,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46091.56994212963</v>
+        <v>46091.62122685185</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14191,7 +14196,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46091.54569444444</v>
+        <v>46091.62341435185</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14255,7 +14260,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46091.54146990741</v>
+        <v>46091.62148148148</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14319,7 +14324,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46091.54289351852</v>
+        <v>46091.62446759259</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14383,7 +14388,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46091.50074074074</v>
+        <v>46091.61680555555</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14447,7 +14452,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46091.55721064815</v>
+        <v>46091.63984953704</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14511,7 +14516,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="3" t="n">
-        <v>46091.545625</v>
+        <v>46091.58400462963</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -14580,7 +14585,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46091.54611111111</v>
+        <v>46091.62594907408</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14644,7 +14649,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="3" t="n">
-        <v>46091.54239583333</v>
+        <v>46091.57959490741</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -14708,7 +14713,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46091.55482638889</v>
+        <v>46091.63680555556</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -14772,7 +14777,7 @@
         <v>1</v>
       </c>
       <c r="N221" s="3" t="n">
-        <v>46091.53320601852</v>
+        <v>46091.57538194444</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -14900,7 +14905,7 @@
         <v>1</v>
       </c>
       <c r="N223" s="3" t="n">
-        <v>46090.84013888889</v>
+        <v>46091.59369212963</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -15028,7 +15033,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46091.55293981481</v>
+        <v>46091.64892361111</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15092,7 +15097,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46091.56800925926</v>
+        <v>46091.64215277778</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15156,7 +15161,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46091.54487268518</v>
+        <v>46091.61785879629</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15220,7 +15225,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46091.56018518518</v>
+        <v>46091.64163194445</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15284,7 +15289,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46091.56861111111</v>
+        <v>46091.64759259259</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15348,7 +15353,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46091.5375462963</v>
+        <v>46091.62650462963</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15412,7 +15417,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46091.53416666666</v>
+        <v>46091.64923611111</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15476,7 +15481,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46091.5478125</v>
+        <v>46091.62873842593</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15540,7 +15545,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46091.56866898148</v>
+        <v>46091.65173611111</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15604,7 +15609,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46091.53834490741</v>
+        <v>46091.62023148148</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15668,7 +15673,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46091.54068287037</v>
+        <v>46091.61813657408</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15796,7 +15801,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46091.55137731481</v>
+        <v>46091.6278587963</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15860,7 +15865,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46091.53394675926</v>
+        <v>46091.6280787037</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15988,7 +15993,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46091.56424768519</v>
+        <v>46091.64160879629</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16052,7 +16057,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46091.56197916667</v>
+        <v>46091.62293981481</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16175,7 +16180,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46091.53472222222</v>
+        <v>46091.6493287037</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16239,7 +16244,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46091.55206018518</v>
+        <v>46091.62510416667</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16303,7 +16308,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46091.54486111111</v>
+        <v>46091.62196759259</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16367,7 +16372,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46091.54572916667</v>
+        <v>46091.62032407407</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16431,7 +16436,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46091.53516203703</v>
+        <v>46091.6522337963</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16450,11 +16455,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C248" t="inlineStr">
-        <is>
-          <t>10.69.5.118</t>
-        </is>
-      </c>
       <c r="D248" t="n">
         <v>2017</v>
       </c>
@@ -16495,7 +16495,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46091.5421412037</v>
+        <v>46091.62076388889</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16623,7 +16623,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46091.55392361111</v>
+        <v>46091.63239583333</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16687,7 +16687,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46091.5516087963</v>
+        <v>46091.62255787037</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16745,7 +16745,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46091.54010416667</v>
+        <v>46091.63030092593</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16809,7 +16809,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46091.5344212963</v>
+        <v>46091.64833333333</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16873,7 +16873,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46091.56034722222</v>
+        <v>46091.63760416667</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16937,7 +16937,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46091.56133101852</v>
+        <v>46091.64378472222</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -17001,7 +17001,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46091.39302083333</v>
+        <v>46091.63923611111</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17065,7 +17065,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46091.57018518518</v>
+        <v>46091.64753472222</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17129,7 +17129,7 @@
         <v>1</v>
       </c>
       <c r="N258" s="3" t="n">
-        <v>46091.54193287037</v>
+        <v>46091.62255787037</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -17257,7 +17257,7 @@
         <v>1</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46090.82313657407</v>
+        <v>46091.62298611111</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17321,7 +17321,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46091.55471064815</v>
+        <v>46091.63282407408</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17385,7 +17385,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46091.53056712963</v>
+        <v>46091.64815972222</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17404,11 +17404,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C263" t="inlineStr">
-        <is>
-          <t>10.69.5.134</t>
-        </is>
-      </c>
       <c r="D263" t="n">
         <v>2017</v>
       </c>
@@ -17449,7 +17444,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46091.55908564815</v>
+        <v>46091.63537037037</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17513,7 +17508,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46091.5303587963</v>
+        <v>46091.64653935185</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17577,7 +17572,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46091.53197916667</v>
+        <v>46091.64996527778</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17641,7 +17636,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="3" t="n">
-        <v>46091.55015046296</v>
+        <v>46091.62657407407</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -17705,7 +17700,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46091.56655092593</v>
+        <v>46091.64037037037</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17766,7 +17761,7 @@
         </is>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46091.55370370371</v>
+        <v>46091.63201388889</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17894,7 +17889,7 @@
         <v>1</v>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46091.53880787037</v>
+        <v>46091.65390046296</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -18267,7 +18262,7 @@
         <v>1</v>
       </c>
       <c r="N276" s="3" t="n">
-        <v>46091.55188657407</v>
+        <v>46091.62549768519</v>
       </c>
       <c r="O276" t="inlineStr">
         <is>
@@ -18331,7 +18326,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46091.54219907407</v>
+        <v>46091.61608796296</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18454,7 +18449,7 @@
         <v>1</v>
       </c>
       <c r="N279" s="3" t="n">
-        <v>46091.53612268518</v>
+        <v>46091.57715277778</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -18513,7 +18508,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46091.53915509259</v>
+        <v>46091.61708333333</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18577,7 +18572,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46091.54835648148</v>
+        <v>46091.62799768519</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18641,7 +18636,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46091.55344907408</v>
+        <v>46091.63604166666</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18705,7 +18700,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46091.53841435185</v>
+        <v>46091.65260416667</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18724,11 +18719,6 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
-      <c r="C284" t="inlineStr">
-        <is>
-          <t>10.69.5.155</t>
-        </is>
-      </c>
       <c r="D284" t="n">
         <v>2019</v>
       </c>
@@ -18961,7 +18951,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46091.53480324074</v>
+        <v>46091.65070601852</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19139,7 +19129,7 @@
         </is>
       </c>
       <c r="N290" s="3" t="n">
-        <v>46091.56613425926</v>
+        <v>46091.6421412037</v>
       </c>
       <c r="O290" t="inlineStr">
         <is>
@@ -19569,7 +19559,7 @@
         <v>1</v>
       </c>
       <c r="N297" s="3" t="n">
-        <v>46091.55402777778</v>
+        <v>46091.63351851852</v>
       </c>
       <c r="O297" t="inlineStr">
         <is>
@@ -19694,7 +19684,7 @@
         <v>1</v>
       </c>
       <c r="N299" s="3" t="n">
-        <v>46091.56699074074</v>
+        <v>46091.64679398148</v>
       </c>
       <c r="O299" t="inlineStr">
         <is>
@@ -21599,7 +21589,7 @@
         <v>2</v>
       </c>
       <c r="N330" s="3" t="n">
-        <v>46091.56412037037</v>
+        <v>46091.64063657408</v>
       </c>
       <c r="O330" t="inlineStr">
         <is>
@@ -21663,7 +21653,7 @@
         <v>2</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46091.55696759259</v>
+        <v>46091.63309027778</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21727,7 +21717,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46091.56087962963</v>
+        <v>46091.63584490741</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21791,7 +21781,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46091.54637731481</v>
+        <v>46091.62887731481</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21855,7 +21845,7 @@
         <v>1</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46091.54484953704</v>
+        <v>46091.6215162037</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21919,7 +21909,7 @@
         <v>2</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46091.53988425926</v>
+        <v>46091.65168981482</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21983,7 +21973,7 @@
         <v>2</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46091.56626157407</v>
+        <v>46091.64107638889</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22044,10 +22034,10 @@
         </is>
       </c>
       <c r="M337" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46091.56130787037</v>
+        <v>46091.63615740741</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22175,7 +22165,7 @@
         <v>2</v>
       </c>
       <c r="N339" s="3" t="n">
-        <v>46091.5361574074</v>
+        <v>46091.57383101852</v>
       </c>
       <c r="O339" t="inlineStr">
         <is>
@@ -22236,7 +22226,7 @@
         </is>
       </c>
       <c r="N340" s="3" t="n">
-        <v>46091.54226851852</v>
+        <v>46091.62291666667</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -22255,6 +22245,11 @@
           <t>OPERACAO 9.1</t>
         </is>
       </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>10.69.5.239</t>
+        </is>
+      </c>
       <c r="D341" t="n">
         <v>2018</v>
       </c>
@@ -22278,7 +22273,7 @@
       </c>
       <c r="J341" t="inlineStr">
         <is>
-          <t>4 GB</t>
+          <t>2 GB</t>
         </is>
       </c>
       <c r="K341" t="inlineStr">
@@ -22295,7 +22290,7 @@
         <v>1</v>
       </c>
       <c r="N341" s="3" t="n">
-        <v>46057.4218287037</v>
+        <v>46091.64876157408</v>
       </c>
       <c r="O341" t="inlineStr">
         <is>
@@ -22356,10 +22351,10 @@
         </is>
       </c>
       <c r="M342" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N342" s="3" t="n">
-        <v>46045.4404050926</v>
+        <v>46091.6540625</v>
       </c>
       <c r="O342" t="inlineStr">
         <is>
@@ -22423,7 +22418,7 @@
         <v>1</v>
       </c>
       <c r="N343" s="3" t="n">
-        <v>46090.73085648148</v>
+        <v>46091.65422453704</v>
       </c>
       <c r="O343" t="inlineStr">
         <is>
@@ -22487,7 +22482,7 @@
         <v>1</v>
       </c>
       <c r="N344" s="3" t="n">
-        <v>46090.7315162037</v>
+        <v>46091.65269675926</v>
       </c>
       <c r="O344" t="inlineStr">
         <is>
@@ -22551,7 +22546,7 @@
         <v>1</v>
       </c>
       <c r="N345" s="3" t="n">
-        <v>46090.71246527778</v>
+        <v>46091.61565972222</v>
       </c>
       <c r="O345" t="inlineStr">
         <is>
@@ -22612,7 +22607,7 @@
         </is>
       </c>
       <c r="N346" s="3" t="n">
-        <v>46090.71013888889</v>
+        <v>46091.65393518518</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -22676,7 +22671,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46090.73429398148</v>
+        <v>46091.61675925926</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22759,6 +22754,11 @@
           <t>OPERACAO 9.1</t>
         </is>
       </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>10.69.5.247</t>
+        </is>
+      </c>
       <c r="D349" t="n">
         <v>2017</v>
       </c>
@@ -22801,7 +22801,7 @@
         </is>
       </c>
       <c r="N349" s="3" t="n">
-        <v>46090.74628472222</v>
+        <v>46091.62501157408</v>
       </c>
       <c r="O349" t="inlineStr">
         <is>
@@ -22867,7 +22867,7 @@
         </is>
       </c>
       <c r="N350" s="3" t="n">
-        <v>46091.56989583333</v>
+        <v>46091.64936342592</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -22931,7 +22931,7 @@
         <v>1</v>
       </c>
       <c r="N351" s="3" t="n">
-        <v>46090.71317129629</v>
+        <v>46091.65210648148</v>
       </c>
       <c r="O351" t="inlineStr">
         <is>
@@ -22995,7 +22995,7 @@
         <v>1</v>
       </c>
       <c r="N352" s="3" t="n">
-        <v>46090.70506944445</v>
+        <v>46091.6515162037</v>
       </c>
       <c r="O352" t="inlineStr">
         <is>
@@ -23059,7 +23059,7 @@
         <v>1</v>
       </c>
       <c r="N353" s="3" t="n">
-        <v>46090.71192129629</v>
+        <v>46091.61635416667</v>
       </c>
       <c r="O353" t="inlineStr">
         <is>
@@ -23092,7 +23092,7 @@
         <v>1</v>
       </c>
       <c r="N354" s="3" t="n">
-        <v>46090.72910879629</v>
+        <v>46091.61354166667</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -23156,7 +23156,7 @@
         <v>2</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46090.70608796296</v>
+        <v>46091.61885416666</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23220,7 +23220,7 @@
         <v>2</v>
       </c>
       <c r="N356" s="3" t="n">
-        <v>46090.71278935186</v>
+        <v>46091.61416666667</v>
       </c>
       <c r="O356" t="inlineStr">
         <is>
@@ -23284,7 +23284,7 @@
         <v>1</v>
       </c>
       <c r="N357" s="3" t="n">
-        <v>46090.71460648148</v>
+        <v>46091.65018518519</v>
       </c>
       <c r="O357" t="inlineStr">
         <is>
@@ -23312,7 +23312,7 @@
         <v>1</v>
       </c>
       <c r="N358" s="3" t="n">
-        <v>46090.71971064815</v>
+        <v>46091.65146990741</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -23335,7 +23335,7 @@
         <v>1</v>
       </c>
       <c r="N359" s="3" t="n">
-        <v>46090.73712962963</v>
+        <v>46091.61271990741</v>
       </c>
       <c r="O359" t="inlineStr">
         <is>
@@ -23462,7 +23462,7 @@
         <v>1</v>
       </c>
       <c r="N361" s="3" t="n">
-        <v>46091.55685185185</v>
+        <v>46091.63599537037</v>
       </c>
       <c r="O361" t="inlineStr">
         <is>
@@ -23528,7 +23528,7 @@
         </is>
       </c>
       <c r="N362" s="3" t="n">
-        <v>46091.53650462963</v>
+        <v>46091.65020833333</v>
       </c>
       <c r="O362" t="inlineStr">
         <is>
@@ -23654,7 +23654,7 @@
         </is>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46091.55773148148</v>
+        <v>46091.63537037037</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23784,7 +23784,7 @@
         <v>1</v>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46091.56077546296</v>
+        <v>46091.63858796296</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
@@ -23812,7 +23812,7 @@
         <v>2</v>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46091.53305555556</v>
+        <v>46091.64909722222</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -23881,7 +23881,7 @@
         <v>1</v>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46091.57097222222</v>
+        <v>46091.64994212963</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24085,7 +24085,7 @@
         </is>
       </c>
       <c r="N371" s="3" t="n">
-        <v>46091.53103009259</v>
+        <v>46091.65043981482</v>
       </c>
       <c r="O371" t="inlineStr">
         <is>
@@ -24149,7 +24149,7 @@
         <v>1</v>
       </c>
       <c r="N372" s="3" t="n">
-        <v>46091.53457175926</v>
+        <v>46091.64752314815</v>
       </c>
       <c r="O372" t="inlineStr">
         <is>
@@ -24218,7 +24218,7 @@
         <v>2</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46091.55059027778</v>
+        <v>46091.62561342592</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24287,7 +24287,7 @@
         <v>2</v>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46091.56847222222</v>
+        <v>46091.64233796296</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-10 17:52:05.603190
</commit_message>
<xml_diff>
--- a/Computadores.xlsx
+++ b/Computadores.xlsx
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>46091.6253125</v>
+        <v>46091.70840277777</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>46091.65208333333</v>
+        <v>46091.73166666667</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>46091.64045138889</v>
+        <v>46091.67689814815</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>46091.61862268519</v>
+        <v>46091.73373842592</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
         <v>1</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>46091.62174768518</v>
+        <v>46091.73638888889</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1903,6 +1903,11 @@
           <t>AUDITORIO</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>10.69.3.150</t>
+        </is>
+      </c>
       <c r="D23" t="n">
         <v>2019</v>
       </c>
@@ -1943,7 +1948,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>46091.50116898148</v>
+        <v>46091.70152777778</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -1962,11 +1967,6 @@
           <t>AUDITORIO</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>10.69.3.153</t>
-        </is>
-      </c>
       <c r="D24" t="n">
         <v>2019</v>
       </c>
@@ -2183,7 +2183,7 @@
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>46091.62216435185</v>
+        <v>46091.70012731481</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6509,7 +6509,7 @@
         <v>1</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>46091.64637731481</v>
+        <v>46091.68409722222</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6578,7 +6578,7 @@
         <v>1</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>46091.6180787037</v>
+        <v>46091.69703703704</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6642,7 +6642,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>46091.6377199074</v>
+        <v>46091.67766203704</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6661,11 +6661,6 @@
           <t>COORDENACAO</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>10.69.3.94</t>
-        </is>
-      </c>
       <c r="D97" t="n">
         <v>2025</v>
       </c>
@@ -6711,7 +6706,7 @@
         <v>1</v>
       </c>
       <c r="N97" s="3" t="n">
-        <v>46091.64969907407</v>
+        <v>46091.69055555556</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6780,7 +6775,7 @@
         <v>1</v>
       </c>
       <c r="N98" s="3" t="n">
-        <v>46091.64759259259</v>
+        <v>46091.68480324074</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6849,7 +6844,7 @@
         <v>2</v>
       </c>
       <c r="N99" s="3" t="n">
-        <v>46091.61957175926</v>
+        <v>46091.69715277778</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6918,7 +6913,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="3" t="n">
-        <v>46091.64761574074</v>
+        <v>46091.68560185185</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6987,7 +6982,7 @@
         <v>1</v>
       </c>
       <c r="N101" s="3" t="n">
-        <v>46091.61975694444</v>
+        <v>46091.66016203703</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -7056,7 +7051,7 @@
         <v>2</v>
       </c>
       <c r="N102" s="3" t="n">
-        <v>46091.62238425926</v>
+        <v>46091.70288194445</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -7451,7 +7446,7 @@
         <v>1</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>46091.6159375</v>
+        <v>46091.73131944444</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -7520,7 +7515,7 @@
         <v>2</v>
       </c>
       <c r="N109" s="3" t="n">
-        <v>46091.62356481481</v>
+        <v>46091.70231481481</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -7589,7 +7584,7 @@
         <v>2</v>
       </c>
       <c r="N110" s="3" t="n">
-        <v>46091.64443287037</v>
+        <v>46091.71813657408</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7658,7 +7653,7 @@
         <v>2</v>
       </c>
       <c r="N111" s="3" t="n">
-        <v>46091.65414351852</v>
+        <v>46091.73168981481</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7727,7 +7722,7 @@
         <v>1</v>
       </c>
       <c r="N112" s="3" t="n">
-        <v>46091.64981481482</v>
+        <v>46091.72712962963</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7796,7 +7791,7 @@
         <v>1</v>
       </c>
       <c r="N113" s="3" t="n">
-        <v>46091.64181712963</v>
+        <v>46091.71888888889</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7931,7 +7926,7 @@
         <v>1</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>46091.61944444444</v>
+        <v>46091.70107638889</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -8000,7 +7995,7 @@
         <v>1</v>
       </c>
       <c r="N116" s="3" t="n">
-        <v>46091.62253472222</v>
+        <v>46091.69655092592</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -8066,7 +8061,7 @@
         </is>
       </c>
       <c r="N117" s="3" t="n">
-        <v>46091.62274305556</v>
+        <v>46091.6978125</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -8204,7 +8199,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>46091.62111111111</v>
+        <v>46091.70369212963</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -8273,7 +8268,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="3" t="n">
-        <v>46091.6366087963</v>
+        <v>46091.71760416667</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -8339,7 +8334,7 @@
         </is>
       </c>
       <c r="N121" s="3" t="n">
-        <v>46091.6285300926</v>
+        <v>46091.70806712963</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -8408,7 +8403,7 @@
         <v>2</v>
       </c>
       <c r="N122" s="3" t="n">
-        <v>46091.63989583333</v>
+        <v>46091.72347222222</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -8477,7 +8472,7 @@
         <v>1</v>
       </c>
       <c r="N123" s="3" t="n">
-        <v>46091.65429398148</v>
+        <v>46091.73371527778</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -8546,7 +8541,7 @@
         <v>1</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>46091.63167824074</v>
+        <v>46091.67120370371</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -8615,7 +8610,7 @@
         <v>2</v>
       </c>
       <c r="N125" s="3" t="n">
-        <v>46091.64142361111</v>
+        <v>46091.68162037037</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -8684,7 +8679,7 @@
         <v>2</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>46091.61427083334</v>
+        <v>46091.72811342592</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -8753,7 +8748,7 @@
         <v>1</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>46091.64509259259</v>
+        <v>46091.68143518519</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -8822,7 +8817,7 @@
         <v>1</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>46091.62784722223</v>
+        <v>46091.70061342593</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -8891,7 +8886,7 @@
         <v>1</v>
       </c>
       <c r="N129" s="3" t="n">
-        <v>46091.64157407408</v>
+        <v>46091.72336805556</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -8955,7 +8950,7 @@
         <v>1</v>
       </c>
       <c r="N130" s="3" t="n">
-        <v>46091.64303240741</v>
+        <v>46091.72091435185</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -9019,7 +9014,7 @@
         <v>1</v>
       </c>
       <c r="N131" s="3" t="n">
-        <v>46091.62206018518</v>
+        <v>46091.704375</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -9147,7 +9142,7 @@
         <v>1</v>
       </c>
       <c r="N133" s="3" t="n">
-        <v>46091.61983796296</v>
+        <v>46091.73453703704</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9338,7 +9333,7 @@
         <v>1</v>
       </c>
       <c r="N136" s="3" t="n">
-        <v>46091.65243055556</v>
+        <v>46091.73052083333</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -9402,7 +9397,7 @@
         <v>1</v>
       </c>
       <c r="N137" s="3" t="n">
-        <v>46091.6225</v>
+        <v>46091.69934027778</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -9466,7 +9461,7 @@
         <v>1</v>
       </c>
       <c r="N138" s="3" t="n">
-        <v>46091.65137731482</v>
+        <v>46091.72555555555</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -9530,7 +9525,7 @@
         <v>1</v>
       </c>
       <c r="N139" s="3" t="n">
-        <v>46091.62240740741</v>
+        <v>46091.70030092593</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -9594,7 +9589,7 @@
         <v>1</v>
       </c>
       <c r="N140" s="3" t="n">
-        <v>46091.62449074074</v>
+        <v>46091.70186342593</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -9658,7 +9653,7 @@
         <v>1</v>
       </c>
       <c r="N141" s="3" t="n">
-        <v>46091.62274305556</v>
+        <v>46091.73716435185</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -9722,7 +9717,7 @@
         <v>1</v>
       </c>
       <c r="N142" s="3" t="n">
-        <v>46091.64649305555</v>
+        <v>46091.72346064815</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -9786,7 +9781,7 @@
         <v>1</v>
       </c>
       <c r="N143" s="3" t="n">
-        <v>46091.62086805556</v>
+        <v>46091.73430555555</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -9850,7 +9845,7 @@
         <v>1</v>
       </c>
       <c r="N144" s="3" t="n">
-        <v>46091.62370370371</v>
+        <v>46091.69829861111</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -9914,7 +9909,7 @@
         <v>1</v>
       </c>
       <c r="N145" s="3" t="n">
-        <v>46091.64804398148</v>
+        <v>46091.72545138889</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -9978,7 +9973,7 @@
         <v>1</v>
       </c>
       <c r="N146" s="3" t="n">
-        <v>46091.6209837963</v>
+        <v>46091.70335648148</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -10042,7 +10037,7 @@
         <v>1</v>
       </c>
       <c r="N147" s="3" t="n">
-        <v>46091.6528125</v>
+        <v>46091.7296875</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -10106,7 +10101,7 @@
         <v>1</v>
       </c>
       <c r="N148" s="3" t="n">
-        <v>46091.62368055555</v>
+        <v>46091.70037037037</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -10170,7 +10165,7 @@
         <v>1</v>
       </c>
       <c r="N149" s="3" t="n">
-        <v>46091.62300925926</v>
+        <v>46091.73300925926</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -10234,7 +10229,7 @@
         <v>1</v>
       </c>
       <c r="N150" s="3" t="n">
-        <v>46091.64751157408</v>
+        <v>46091.72034722222</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -10357,7 +10352,7 @@
         <v>1</v>
       </c>
       <c r="N152" s="3" t="n">
-        <v>46091.63981481481</v>
+        <v>46091.72140046296</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -10421,7 +10416,7 @@
         <v>1</v>
       </c>
       <c r="N153" s="3" t="n">
-        <v>46091.62424768518</v>
+        <v>46091.70084490741</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -10485,7 +10480,7 @@
         <v>1</v>
       </c>
       <c r="N154" s="3" t="n">
-        <v>46091.63731481481</v>
+        <v>46091.71333333333</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -10677,7 +10672,7 @@
         <v>1</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>46091.61717592592</v>
+        <v>46091.73152777777</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -10741,7 +10736,7 @@
         <v>1</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>46091.63915509259</v>
+        <v>46091.71084490741</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -10805,7 +10800,7 @@
         <v>1</v>
       </c>
       <c r="N159" s="3" t="n">
-        <v>46091.62271990741</v>
+        <v>46091.70038194444</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -10869,7 +10864,7 @@
         <v>1</v>
       </c>
       <c r="N160" s="3" t="n">
-        <v>46091.62431712963</v>
+        <v>46091.69775462963</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -10997,7 +10992,7 @@
         <v>2</v>
       </c>
       <c r="N162" s="3" t="n">
-        <v>46091.63837962963</v>
+        <v>46091.71261574074</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -11061,7 +11056,7 @@
         <v>2</v>
       </c>
       <c r="N163" s="3" t="n">
-        <v>46091.62303240741</v>
+        <v>46091.73744212963</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -11317,7 +11312,7 @@
         <v>2</v>
       </c>
       <c r="N167" s="3" t="n">
-        <v>46091.62391203704</v>
+        <v>46091.69858796296</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -11381,7 +11376,7 @@
         <v>2</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>46091.65043981482</v>
+        <v>46091.72741898148</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -11509,7 +11504,7 @@
         <v>2</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>46091.62005787037</v>
+        <v>46091.703125</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -11573,7 +11568,7 @@
         <v>2</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>46091.62076388889</v>
+        <v>46091.73784722222</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -11701,7 +11696,7 @@
         <v>2</v>
       </c>
       <c r="N173" s="3" t="n">
-        <v>46091.61824074074</v>
+        <v>46091.7312962963</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -11829,7 +11824,7 @@
         <v>2</v>
       </c>
       <c r="N175" s="3" t="n">
-        <v>46091.62333333334</v>
+        <v>46091.73793981481</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -11893,7 +11888,7 @@
         <v>2</v>
       </c>
       <c r="N176" s="3" t="n">
-        <v>46091.63947916667</v>
+        <v>46091.71304398148</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -11957,7 +11952,7 @@
         <v>1</v>
       </c>
       <c r="N177" s="3" t="n">
-        <v>46091.6291087963</v>
+        <v>46091.71040509259</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -12021,7 +12016,7 @@
         <v>1</v>
       </c>
       <c r="N178" s="3" t="n">
-        <v>46091.62238425926</v>
+        <v>46091.70122685185</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -12085,7 +12080,7 @@
         <v>1</v>
       </c>
       <c r="N179" s="3" t="n">
-        <v>46091.62402777778</v>
+        <v>46091.73652777778</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -12346,7 +12341,7 @@
         <v>1</v>
       </c>
       <c r="N183" s="3" t="n">
-        <v>46091.63849537037</v>
+        <v>46091.71465277778</v>
       </c>
       <c r="O183" t="inlineStr">
         <is>
@@ -12410,7 +12405,7 @@
         <v>1</v>
       </c>
       <c r="N184" s="3" t="n">
-        <v>46091.65115740741</v>
+        <v>46091.72918981482</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -12474,7 +12469,7 @@
         <v>1</v>
       </c>
       <c r="N185" s="3" t="n">
-        <v>46091.62380787037</v>
+        <v>46091.70248842592</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -12666,7 +12661,7 @@
         </is>
       </c>
       <c r="N188" s="3" t="n">
-        <v>46091.62310185185</v>
+        <v>46091.70231481481</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
@@ -12730,7 +12725,7 @@
         <v>1</v>
       </c>
       <c r="N189" s="3" t="n">
-        <v>46091.62336805555</v>
+        <v>46091.70490740741</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -12794,7 +12789,7 @@
         <v>1</v>
       </c>
       <c r="N190" s="3" t="n">
-        <v>46091.62241898148</v>
+        <v>46091.70207175926</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -12983,7 +12978,7 @@
         <v>1</v>
       </c>
       <c r="N193" s="3" t="n">
-        <v>46091.64248842592</v>
+        <v>46091.72586805555</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -13047,7 +13042,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="3" t="n">
-        <v>46091.61616898148</v>
+        <v>46091.73402777778</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -13175,7 +13170,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="3" t="n">
-        <v>46091.6234837963</v>
+        <v>46091.70336805555</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -13303,7 +13298,7 @@
         <v>1</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>46091.62597222222</v>
+        <v>46091.7021875</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -13364,7 +13359,7 @@
         </is>
       </c>
       <c r="N199" s="3" t="n">
-        <v>46091.6374074074</v>
+        <v>46091.71762731481</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -13428,7 +13423,7 @@
         <v>1</v>
       </c>
       <c r="N200" s="3" t="n">
-        <v>46091.64223379629</v>
+        <v>46091.71909722222</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -13492,7 +13487,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="3" t="n">
-        <v>46091.64954861111</v>
+        <v>46091.73119212963</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -13556,7 +13551,7 @@
         <v>1</v>
       </c>
       <c r="N202" s="3" t="n">
-        <v>46091.62140046297</v>
+        <v>46091.71314814815</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -13620,7 +13615,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="3" t="n">
-        <v>46091.63511574074</v>
+        <v>46091.71331018519</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -13684,7 +13679,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="3" t="n">
-        <v>46091.63061342593</v>
+        <v>46091.70708333333</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -13748,7 +13743,7 @@
         <v>1</v>
       </c>
       <c r="N205" s="3" t="n">
-        <v>46091.6207175926</v>
+        <v>46091.73113425926</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -13876,7 +13871,7 @@
         <v>1</v>
       </c>
       <c r="N207" s="3" t="n">
-        <v>46091.62244212963</v>
+        <v>46091.70120370371</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -13940,7 +13935,7 @@
         <v>1</v>
       </c>
       <c r="N208" s="3" t="n">
-        <v>46091.61525462963</v>
+        <v>46091.72702546296</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -14004,7 +13999,7 @@
         <v>1</v>
       </c>
       <c r="N209" s="3" t="n">
-        <v>46091.61863425926</v>
+        <v>46091.73100694444</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -14068,7 +14063,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="3" t="n">
-        <v>46091.61972222223</v>
+        <v>46091.72825231482</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -14132,7 +14127,7 @@
         <v>1</v>
       </c>
       <c r="N211" s="3" t="n">
-        <v>46091.62122685185</v>
+        <v>46091.73550925926</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -14196,7 +14191,7 @@
         <v>1</v>
       </c>
       <c r="N212" s="3" t="n">
-        <v>46091.62341435185</v>
+        <v>46091.69921296297</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -14260,7 +14255,7 @@
         <v>1</v>
       </c>
       <c r="N213" s="3" t="n">
-        <v>46091.62148148148</v>
+        <v>46091.70195601852</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -14324,7 +14319,7 @@
         <v>1</v>
       </c>
       <c r="N214" s="3" t="n">
-        <v>46091.62446759259</v>
+        <v>46091.73673611111</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -14388,7 +14383,7 @@
         <v>1</v>
       </c>
       <c r="N215" s="3" t="n">
-        <v>46091.61680555555</v>
+        <v>46091.7340625</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -14452,7 +14447,7 @@
         <v>1</v>
       </c>
       <c r="N216" s="3" t="n">
-        <v>46091.63984953704</v>
+        <v>46091.71981481482</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -14585,7 +14580,7 @@
         <v>1</v>
       </c>
       <c r="N218" s="3" t="n">
-        <v>46091.62594907408</v>
+        <v>46091.73768518519</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -14713,7 +14708,7 @@
         <v>1</v>
       </c>
       <c r="N220" s="3" t="n">
-        <v>46091.63680555556</v>
+        <v>46091.7125</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -15033,7 +15028,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="3" t="n">
-        <v>46091.64892361111</v>
+        <v>46091.72868055556</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -15097,7 +15092,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="3" t="n">
-        <v>46091.64215277778</v>
+        <v>46091.72158564815</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -15161,7 +15156,7 @@
         <v>1</v>
       </c>
       <c r="N227" s="3" t="n">
-        <v>46091.61785879629</v>
+        <v>46091.7377662037</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -15225,7 +15220,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="3" t="n">
-        <v>46091.64163194445</v>
+        <v>46091.71851851852</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -15289,7 +15284,7 @@
         <v>1</v>
       </c>
       <c r="N229" s="3" t="n">
-        <v>46091.64759259259</v>
+        <v>46091.72496527778</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -15353,7 +15348,7 @@
         <v>1</v>
       </c>
       <c r="N230" s="3" t="n">
-        <v>46091.62650462963</v>
+        <v>46091.70810185185</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -15417,7 +15412,7 @@
         <v>1</v>
       </c>
       <c r="N231" s="3" t="n">
-        <v>46091.64923611111</v>
+        <v>46091.73048611111</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -15481,7 +15476,7 @@
         <v>1</v>
       </c>
       <c r="N232" s="3" t="n">
-        <v>46091.62873842593</v>
+        <v>46091.72752314815</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -15545,7 +15540,7 @@
         <v>1</v>
       </c>
       <c r="N233" s="3" t="n">
-        <v>46091.65173611111</v>
+        <v>46091.72502314814</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -15609,7 +15604,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="3" t="n">
-        <v>46091.62023148148</v>
+        <v>46091.73608796296</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -15673,7 +15668,7 @@
         <v>1</v>
       </c>
       <c r="N235" s="3" t="n">
-        <v>46091.61813657408</v>
+        <v>46091.73270833334</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -15801,7 +15796,7 @@
         <v>1</v>
       </c>
       <c r="N237" s="3" t="n">
-        <v>46091.6278587963</v>
+        <v>46091.70175925926</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -15865,7 +15860,7 @@
         <v>1</v>
       </c>
       <c r="N238" s="3" t="n">
-        <v>46091.6280787037</v>
+        <v>46091.70584490741</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -15993,7 +15988,7 @@
         <v>1</v>
       </c>
       <c r="N240" s="3" t="n">
-        <v>46091.64160879629</v>
+        <v>46091.71614583334</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -16057,7 +16052,7 @@
         <v>1</v>
       </c>
       <c r="N241" s="3" t="n">
-        <v>46091.62293981481</v>
+        <v>46091.73715277778</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -16180,7 +16175,7 @@
         <v>1</v>
       </c>
       <c r="N243" s="3" t="n">
-        <v>46091.6493287037</v>
+        <v>46091.7237037037</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -16244,7 +16239,7 @@
         <v>1</v>
       </c>
       <c r="N244" s="3" t="n">
-        <v>46091.62510416667</v>
+        <v>46091.70649305556</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -16308,7 +16303,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="3" t="n">
-        <v>46091.62196759259</v>
+        <v>46091.73787037037</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -16372,7 +16367,7 @@
         <v>1</v>
       </c>
       <c r="N246" s="3" t="n">
-        <v>46091.62032407407</v>
+        <v>46091.72320601852</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -16436,7 +16431,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="3" t="n">
-        <v>46091.6522337963</v>
+        <v>46091.72423611111</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -16495,7 +16490,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>46091.62076388889</v>
+        <v>46091.73113425926</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -16623,7 +16618,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>46091.63239583333</v>
+        <v>46091.71303240741</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -16687,7 +16682,7 @@
         <v>1</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>46091.62255787037</v>
+        <v>46091.70246527778</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -16745,7 +16740,7 @@
         <v>1</v>
       </c>
       <c r="N252" s="3" t="n">
-        <v>46091.63030092593</v>
+        <v>46091.70577546296</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -16809,7 +16804,7 @@
         <v>1</v>
       </c>
       <c r="N253" s="3" t="n">
-        <v>46091.64833333333</v>
+        <v>46091.72021990741</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -16873,7 +16868,7 @@
         <v>1</v>
       </c>
       <c r="N254" s="3" t="n">
-        <v>46091.63760416667</v>
+        <v>46091.71202546296</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -16937,7 +16932,7 @@
         <v>1</v>
       </c>
       <c r="N255" s="3" t="n">
-        <v>46091.64378472222</v>
+        <v>46091.72252314815</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -17001,7 +16996,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="3" t="n">
-        <v>46091.63923611111</v>
+        <v>46091.72015046296</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -17065,7 +17060,7 @@
         <v>1</v>
       </c>
       <c r="N257" s="3" t="n">
-        <v>46091.64753472222</v>
+        <v>46091.72672453704</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -17193,7 +17188,7 @@
         <v>2</v>
       </c>
       <c r="N259" s="3" t="n">
-        <v>46090.59398148148</v>
+        <v>46091.73640046296</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -17257,7 +17252,7 @@
         <v>1</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>46091.62298611111</v>
+        <v>46091.70211805555</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -17321,7 +17316,7 @@
         <v>1</v>
       </c>
       <c r="N261" s="3" t="n">
-        <v>46091.63282407408</v>
+        <v>46091.72831018519</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -17385,7 +17380,7 @@
         <v>1</v>
       </c>
       <c r="N262" s="3" t="n">
-        <v>46091.64815972222</v>
+        <v>46091.72186342593</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -17404,6 +17399,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>10.69.5.134</t>
+        </is>
+      </c>
       <c r="D263" t="n">
         <v>2017</v>
       </c>
@@ -17444,7 +17444,7 @@
         <v>1</v>
       </c>
       <c r="N263" s="3" t="n">
-        <v>46091.63537037037</v>
+        <v>46091.71523148148</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -17508,7 +17508,7 @@
         <v>1</v>
       </c>
       <c r="N264" s="3" t="n">
-        <v>46091.64653935185</v>
+        <v>46091.7305324074</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -17572,7 +17572,7 @@
         <v>1</v>
       </c>
       <c r="N265" s="3" t="n">
-        <v>46091.64996527778</v>
+        <v>46091.72435185185</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -17700,7 +17700,7 @@
         <v>1</v>
       </c>
       <c r="N267" s="3" t="n">
-        <v>46091.64037037037</v>
+        <v>46091.71630787037</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -17761,7 +17761,7 @@
         </is>
       </c>
       <c r="N268" s="3" t="n">
-        <v>46091.63201388889</v>
+        <v>46091.70938657408</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -17889,7 +17889,7 @@
         <v>1</v>
       </c>
       <c r="N270" s="3" t="n">
-        <v>46091.65390046296</v>
+        <v>46091.72758101852</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -18262,7 +18262,7 @@
         <v>1</v>
       </c>
       <c r="N276" s="3" t="n">
-        <v>46091.62549768519</v>
+        <v>46091.70383101852</v>
       </c>
       <c r="O276" t="inlineStr">
         <is>
@@ -18326,7 +18326,7 @@
         <v>1</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>46091.61608796296</v>
+        <v>46091.73744212963</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18468,6 +18468,11 @@
           <t>OPERACAO 8.2</t>
         </is>
       </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>10.69.5.151</t>
+        </is>
+      </c>
       <c r="D280" t="n">
         <v>2017</v>
       </c>
@@ -18508,7 +18513,7 @@
         <v>1</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>46091.61708333333</v>
+        <v>46091.73570601852</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -18572,7 +18577,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>46091.62799768519</v>
+        <v>46091.71069444445</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -18636,7 +18641,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>46091.63604166666</v>
+        <v>46091.715625</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -18700,7 +18705,7 @@
         <v>1</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>46091.65260416667</v>
+        <v>46091.72914351852</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18951,7 +18956,7 @@
         <v>1</v>
       </c>
       <c r="N287" s="3" t="n">
-        <v>46091.65070601852</v>
+        <v>46091.72664351852</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -19129,7 +19134,7 @@
         </is>
       </c>
       <c r="N290" s="3" t="n">
-        <v>46091.6421412037</v>
+        <v>46091.72224537037</v>
       </c>
       <c r="O290" t="inlineStr">
         <is>
@@ -19559,7 +19564,7 @@
         <v>1</v>
       </c>
       <c r="N297" s="3" t="n">
-        <v>46091.63351851852</v>
+        <v>46091.71638888889</v>
       </c>
       <c r="O297" t="inlineStr">
         <is>
@@ -19684,7 +19689,7 @@
         <v>1</v>
       </c>
       <c r="N299" s="3" t="n">
-        <v>46091.64679398148</v>
+        <v>46091.72685185185</v>
       </c>
       <c r="O299" t="inlineStr">
         <is>
@@ -21589,7 +21594,7 @@
         <v>2</v>
       </c>
       <c r="N330" s="3" t="n">
-        <v>46091.64063657408</v>
+        <v>46091.71325231482</v>
       </c>
       <c r="O330" t="inlineStr">
         <is>
@@ -21653,7 +21658,7 @@
         <v>2</v>
       </c>
       <c r="N331" s="3" t="n">
-        <v>46091.63309027778</v>
+        <v>46091.7071412037</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -21717,7 +21722,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>46091.63584490741</v>
+        <v>46091.71487268519</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -21781,7 +21786,7 @@
         <v>2</v>
       </c>
       <c r="N333" s="3" t="n">
-        <v>46091.62887731481</v>
+        <v>46091.66609953704</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -21845,7 +21850,7 @@
         <v>1</v>
       </c>
       <c r="N334" s="3" t="n">
-        <v>46091.6215162037</v>
+        <v>46091.70546296296</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -21909,7 +21914,7 @@
         <v>2</v>
       </c>
       <c r="N335" s="3" t="n">
-        <v>46091.65168981482</v>
+        <v>46091.72780092592</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -21973,7 +21978,7 @@
         <v>2</v>
       </c>
       <c r="N336" s="3" t="n">
-        <v>46091.64107638889</v>
+        <v>46091.71921296296</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -22037,7 +22042,7 @@
         <v>1</v>
       </c>
       <c r="N337" s="3" t="n">
-        <v>46091.63615740741</v>
+        <v>46091.71511574074</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -22226,7 +22231,7 @@
         </is>
       </c>
       <c r="N340" s="3" t="n">
-        <v>46091.62291666667</v>
+        <v>46091.69890046296</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -22245,11 +22250,6 @@
           <t>OPERACAO 9.1</t>
         </is>
       </c>
-      <c r="C341" t="inlineStr">
-        <is>
-          <t>10.69.5.239</t>
-        </is>
-      </c>
       <c r="D341" t="n">
         <v>2018</v>
       </c>
@@ -22351,10 +22351,10 @@
         </is>
       </c>
       <c r="M342" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N342" s="3" t="n">
-        <v>46091.6540625</v>
+        <v>46091.66920138889</v>
       </c>
       <c r="O342" t="inlineStr">
         <is>
@@ -22546,7 +22546,7 @@
         <v>1</v>
       </c>
       <c r="N345" s="3" t="n">
-        <v>46091.61565972222</v>
+        <v>46091.73096064815</v>
       </c>
       <c r="O345" t="inlineStr">
         <is>
@@ -22671,7 +22671,7 @@
         <v>1</v>
       </c>
       <c r="N347" s="3" t="n">
-        <v>46091.61675925926</v>
+        <v>46091.67387731482</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -22754,11 +22754,6 @@
           <t>OPERACAO 9.1</t>
         </is>
       </c>
-      <c r="C349" t="inlineStr">
-        <is>
-          <t>10.69.5.247</t>
-        </is>
-      </c>
       <c r="D349" t="n">
         <v>2017</v>
       </c>
@@ -22801,7 +22796,7 @@
         </is>
       </c>
       <c r="N349" s="3" t="n">
-        <v>46091.62501157408</v>
+        <v>46091.66603009259</v>
       </c>
       <c r="O349" t="inlineStr">
         <is>
@@ -23059,7 +23054,7 @@
         <v>1</v>
       </c>
       <c r="N353" s="3" t="n">
-        <v>46091.61635416667</v>
+        <v>46091.65805555556</v>
       </c>
       <c r="O353" t="inlineStr">
         <is>
@@ -23092,7 +23087,7 @@
         <v>1</v>
       </c>
       <c r="N354" s="3" t="n">
-        <v>46091.61354166667</v>
+        <v>46091.65540509259</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -23156,7 +23151,7 @@
         <v>2</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>46091.61885416666</v>
+        <v>46091.65613425926</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -23220,7 +23215,7 @@
         <v>2</v>
       </c>
       <c r="N356" s="3" t="n">
-        <v>46091.61416666667</v>
+        <v>46091.6571412037</v>
       </c>
       <c r="O356" t="inlineStr">
         <is>
@@ -23462,7 +23457,7 @@
         <v>1</v>
       </c>
       <c r="N361" s="3" t="n">
-        <v>46091.63599537037</v>
+        <v>46091.67556712963</v>
       </c>
       <c r="O361" t="inlineStr">
         <is>
@@ -23528,7 +23523,7 @@
         </is>
       </c>
       <c r="N362" s="3" t="n">
-        <v>46091.65020833333</v>
+        <v>46091.72369212963</v>
       </c>
       <c r="O362" t="inlineStr">
         <is>
@@ -23654,7 +23649,7 @@
         </is>
       </c>
       <c r="N364" s="3" t="n">
-        <v>46091.63537037037</v>
+        <v>46091.71302083333</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -23784,7 +23779,7 @@
         <v>1</v>
       </c>
       <c r="N366" s="3" t="n">
-        <v>46091.63858796296</v>
+        <v>46091.71390046296</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
@@ -23812,7 +23807,7 @@
         <v>2</v>
       </c>
       <c r="N367" s="3" t="n">
-        <v>46091.64909722222</v>
+        <v>46091.68930555556</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -23881,7 +23876,7 @@
         <v>1</v>
       </c>
       <c r="N368" s="3" t="n">
-        <v>46091.64994212963</v>
+        <v>46091.68716435185</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -24085,7 +24080,7 @@
         </is>
       </c>
       <c r="N371" s="3" t="n">
-        <v>46091.65043981482</v>
+        <v>46091.7296875</v>
       </c>
       <c r="O371" t="inlineStr">
         <is>
@@ -24104,6 +24099,11 @@
           <t>COORDENACAO</t>
         </is>
       </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>10.69.3.72</t>
+        </is>
+      </c>
       <c r="D372" t="n">
         <v>2025</v>
       </c>
@@ -24149,7 +24149,7 @@
         <v>1</v>
       </c>
       <c r="N372" s="3" t="n">
-        <v>46091.64752314815</v>
+        <v>46091.72520833334</v>
       </c>
       <c r="O372" t="inlineStr">
         <is>
@@ -24218,7 +24218,7 @@
         <v>2</v>
       </c>
       <c r="N373" s="3" t="n">
-        <v>46091.62561342592</v>
+        <v>46091.70109953704</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -24287,7 +24287,7 @@
         <v>2</v>
       </c>
       <c r="N374" s="3" t="n">
-        <v>46091.64233796296</v>
+        <v>46091.72204861111</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>

</xml_diff>